<commit_message>
Atualização automática: 2026-09-17 08:38
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -1572,7 +1572,7 @@
         <v>46268.63953865741</v>
       </c>
       <c r="W2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X2" t="s">
         <v>191</v>
@@ -1649,7 +1649,7 @@
         <v>46266.57730150463</v>
       </c>
       <c r="W3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X3" t="s">
         <v>192</v>
@@ -1726,7 +1726,7 @@
         <v>46266.41668148148</v>
       </c>
       <c r="W4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X4" t="s">
         <v>193</v>
@@ -1803,7 +1803,7 @@
         <v>46267.75233784723</v>
       </c>
       <c r="W5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X5" t="s">
         <v>191</v>
@@ -1877,7 +1877,7 @@
         <v>46267.75233927083</v>
       </c>
       <c r="W6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X6" t="s">
         <v>192</v>
@@ -1951,7 +1951,7 @@
         <v>46267.7523394676</v>
       </c>
       <c r="W7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X7" t="s">
         <v>192</v>
@@ -2025,7 +2025,7 @@
         <v>46267.75234278935</v>
       </c>
       <c r="W8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X8" t="s">
         <v>194</v>
@@ -2099,7 +2099,7 @@
         <v>46267.75234309028</v>
       </c>
       <c r="W9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X9" t="s">
         <v>193</v>
@@ -2173,7 +2173,7 @@
         <v>46267.75234383102</v>
       </c>
       <c r="W10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X10" t="s">
         <v>195</v>
@@ -2247,7 +2247,7 @@
         <v>46267.75234424769</v>
       </c>
       <c r="W11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X11" t="s">
         <v>195</v>
@@ -2321,7 +2321,7 @@
         <v>46267.47365627315</v>
       </c>
       <c r="W12">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="X12" t="s">
         <v>196</v>
@@ -2395,7 +2395,7 @@
         <v>46266.47620831019</v>
       </c>
       <c r="W13">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X13" t="s">
         <v>197</v>
@@ -2469,7 +2469,7 @@
         <v>46267.57586420139</v>
       </c>
       <c r="W14">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X14" t="s">
         <v>198</v>
@@ -2540,7 +2540,7 @@
         <v>46266.44145744213</v>
       </c>
       <c r="W15">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="X15" t="s">
         <v>199</v>
@@ -2608,7 +2608,7 @@
         <v>46266.44156952546</v>
       </c>
       <c r="W16">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="X16" t="s">
         <v>199</v>
@@ -2676,7 +2676,7 @@
         <v>46266.44152346065</v>
       </c>
       <c r="W17">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X17" t="s">
         <v>199</v>
@@ -2750,7 +2750,7 @@
         <v>46269.3962034375</v>
       </c>
       <c r="W18">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X18" t="s">
         <v>200</v>
@@ -2827,7 +2827,7 @@
         <v>46268.54759884259</v>
       </c>
       <c r="W19">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X19" t="s">
         <v>197</v>
@@ -2904,7 +2904,7 @@
         <v>46269.38216940972</v>
       </c>
       <c r="W20">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X20" t="s">
         <v>198</v>
@@ -2981,7 +2981,7 @@
         <v>46269.40844942129</v>
       </c>
       <c r="W21">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X21" t="s">
         <v>196</v>
@@ -3058,7 +3058,7 @@
         <v>46266.37634084491</v>
       </c>
       <c r="W22">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X22" t="s">
         <v>201</v>
@@ -3132,7 +3132,7 @@
         <v>46267.47452163194</v>
       </c>
       <c r="W23">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X23" t="s">
         <v>196</v>
@@ -3206,7 +3206,7 @@
         <v>46267.4745221412</v>
       </c>
       <c r="W24">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X24" t="s">
         <v>196</v>
@@ -3280,7 +3280,7 @@
         <v>46267.47452299768</v>
       </c>
       <c r="W25">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X25" t="s">
         <v>196</v>
@@ -3354,7 +3354,7 @@
         <v>46267.75231010417</v>
       </c>
       <c r="W26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X26" t="s">
         <v>197</v>
@@ -3428,7 +3428,7 @@
         <v>46267.75234059028</v>
       </c>
       <c r="W27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X27" t="s">
         <v>196</v>
@@ -3502,7 +3502,7 @@
         <v>46267.7523409375</v>
       </c>
       <c r="W28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X28" t="s">
         <v>196</v>
@@ -3576,7 +3576,7 @@
         <v>46267.75234170139</v>
       </c>
       <c r="W29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X29" t="s">
         <v>196</v>
@@ -3650,7 +3650,7 @@
         <v>46268.58940019676</v>
       </c>
       <c r="W30">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X30" t="s">
         <v>200</v>
@@ -3727,7 +3727,7 @@
         <v>46268.37896984954</v>
       </c>
       <c r="W31">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X31" t="s">
         <v>192</v>
@@ -3804,7 +3804,7 @@
         <v>46269.71652982639</v>
       </c>
       <c r="W32">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X32" t="s">
         <v>194</v>
@@ -3881,7 +3881,7 @@
         <v>46269.71069613426</v>
       </c>
       <c r="W33">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X33" t="s">
         <v>193</v>
@@ -3958,7 +3958,7 @@
         <v>46267.55838734953</v>
       </c>
       <c r="W34">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X34" t="s">
         <v>197</v>
@@ -4038,7 +4038,7 @@
         <v>46273.59003707176</v>
       </c>
       <c r="W35">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X35" t="s">
         <v>201</v>
@@ -4118,7 +4118,7 @@
         <v>46268.74069754629</v>
       </c>
       <c r="W36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X36" t="s">
         <v>191</v>
@@ -4198,7 +4198,7 @@
         <v>46273.45940115741</v>
       </c>
       <c r="W37">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X37" t="s">
         <v>200</v>
@@ -4275,7 +4275,7 @@
         <v>46267.66088636574</v>
       </c>
       <c r="W38">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X38" t="s">
         <v>197</v>
@@ -4355,7 +4355,7 @@
         <v>46268.45922827546</v>
       </c>
       <c r="W39">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X39" t="s">
         <v>198</v>
@@ -4435,7 +4435,7 @@
         <v>46269.59248078704</v>
       </c>
       <c r="W40">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X40" t="s">
         <v>192</v>
@@ -4515,7 +4515,7 @@
         <v>46269.59224453704</v>
       </c>
       <c r="W41">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X41" t="s">
         <v>192</v>
@@ -4595,7 +4595,7 @@
         <v>46268.5891771875</v>
       </c>
       <c r="W42">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X42" t="s">
         <v>200</v>
@@ -4675,7 +4675,7 @@
         <v>46267.64795916666</v>
       </c>
       <c r="W43">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X43" t="s">
         <v>196</v>
@@ -4755,7 +4755,7 @@
         <v>46267.4478849537</v>
       </c>
       <c r="W44">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X44" t="s">
         <v>194</v>
@@ -4835,7 +4835,7 @@
         <v>46269.59056300926</v>
       </c>
       <c r="W45">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X45" t="s">
         <v>193</v>
@@ -4909,7 +4909,7 @@
         <v>46273.67026252315</v>
       </c>
       <c r="W46">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X46" t="s">
         <v>197</v>
@@ -4983,7 +4983,7 @@
         <v>46269.677524375</v>
       </c>
       <c r="W47">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X47" t="s">
         <v>198</v>
@@ -5057,7 +5057,7 @@
         <v>46269.677525</v>
       </c>
       <c r="W48">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X48" t="s">
         <v>192</v>
@@ -5131,7 +5131,7 @@
         <v>46269.677525625</v>
       </c>
       <c r="W49">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X49" t="s">
         <v>192</v>
@@ -5205,7 +5205,7 @@
         <v>46268.58906282407</v>
       </c>
       <c r="W50">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X50" t="s">
         <v>200</v>
@@ -5279,7 +5279,7 @@
         <v>46267.64761306713</v>
       </c>
       <c r="W51">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X51" t="s">
         <v>196</v>
@@ -5356,7 +5356,7 @@
         <v>46273.64957155092</v>
       </c>
       <c r="W52">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X52" t="s">
         <v>194</v>
@@ -5433,7 +5433,7 @@
         <v>46273.39871140046</v>
       </c>
       <c r="W53">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X53" t="s">
         <v>193</v>
@@ -5510,7 +5510,7 @@
         <v>46267.35832805555</v>
       </c>
       <c r="W54">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X54" t="s">
         <v>198</v>
@@ -5590,7 +5590,7 @@
         <v>46268.71229238426</v>
       </c>
       <c r="W55">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X55" t="s">
         <v>192</v>
@@ -5670,7 +5670,7 @@
         <v>46268.71229297454</v>
       </c>
       <c r="W56">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X56" t="s">
         <v>192</v>
@@ -5750,7 +5750,7 @@
         <v>46267.74532275463</v>
       </c>
       <c r="W57">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X57" t="s">
         <v>200</v>
@@ -5827,7 +5827,7 @@
         <v>46269.60160202546</v>
       </c>
       <c r="W58">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X58" t="s">
         <v>197</v>
@@ -5907,7 +5907,7 @@
         <v>46273.64508760416</v>
       </c>
       <c r="W59">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X59" t="s">
         <v>201</v>
@@ -5987,7 +5987,7 @@
         <v>46268.45926839121</v>
       </c>
       <c r="W60">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X60" t="s">
         <v>198</v>
@@ -6067,7 +6067,7 @@
         <v>46269.59250902777</v>
       </c>
       <c r="W61">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X61" t="s">
         <v>192</v>
@@ -6147,7 +6147,7 @@
         <v>46269.5922865625</v>
       </c>
       <c r="W62">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X62" t="s">
         <v>192</v>
@@ -6227,7 +6227,7 @@
         <v>46268.58922707176</v>
       </c>
       <c r="W63">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X63" t="s">
         <v>200</v>
@@ -6307,7 +6307,7 @@
         <v>46267.64800344907</v>
       </c>
       <c r="W64">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X64" t="s">
         <v>196</v>
@@ -6387,7 +6387,7 @@
         <v>46267.44799793982</v>
       </c>
       <c r="W65">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X65" t="s">
         <v>194</v>
@@ -6467,7 +6467,7 @@
         <v>46269.59070487269</v>
       </c>
       <c r="W66">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X66" t="s">
         <v>193</v>
@@ -6547,7 +6547,7 @@
         <v>46269.49635894676</v>
       </c>
       <c r="W67">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X67" t="s">
         <v>198</v>
@@ -6621,7 +6621,7 @@
         <v>46269.63659284722</v>
       </c>
       <c r="W68">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X68" t="s">
         <v>197</v>
@@ -6695,7 +6695,7 @@
         <v>46273.64532122685</v>
       </c>
       <c r="W69">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X69" t="s">
         <v>201</v>
@@ -6769,7 +6769,7 @@
         <v>46268.45929986111</v>
       </c>
       <c r="W70">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X70" t="s">
         <v>198</v>
@@ -6843,7 +6843,7 @@
         <v>46269.5925421875</v>
       </c>
       <c r="W71">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X71" t="s">
         <v>192</v>
@@ -6917,7 +6917,7 @@
         <v>46269.59231454861</v>
       </c>
       <c r="W72">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X72" t="s">
         <v>192</v>
@@ -6991,7 +6991,7 @@
         <v>46268.58932953704</v>
       </c>
       <c r="W73">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X73" t="s">
         <v>200</v>
@@ -7065,7 +7065,7 @@
         <v>46267.648038125</v>
       </c>
       <c r="W74">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X74" t="s">
         <v>196</v>
@@ -7139,7 +7139,7 @@
         <v>46267.44824061343</v>
       </c>
       <c r="W75">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X75" t="s">
         <v>194</v>
@@ -7213,7 +7213,7 @@
         <v>46269.59082328704</v>
       </c>
       <c r="W76">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X76" t="s">
         <v>193</v>
@@ -7284,7 +7284,7 @@
         <v>46273.63629708334</v>
       </c>
       <c r="W77">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X77" t="s">
         <v>193</v>
@@ -7358,7 +7358,7 @@
         <v>46273.64318633102</v>
       </c>
       <c r="W78">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X78" t="s">
         <v>193</v>
@@ -7432,7 +7432,7 @@
         <v>46273.64880981482</v>
       </c>
       <c r="W79">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X79" t="s">
         <v>193</v>
@@ -7509,7 +7509,7 @@
         <v>46267.72055925926</v>
       </c>
       <c r="W80">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X80" t="s">
         <v>191</v>
@@ -7580,7 +7580,7 @@
         <v>46267.79441380787</v>
       </c>
       <c r="W81">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X81" t="s">
         <v>192</v>
@@ -7654,7 +7654,7 @@
         <v>46267.79441215278</v>
       </c>
       <c r="W82">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X82" t="s">
         <v>193</v>
@@ -7728,7 +7728,7 @@
         <v>46267.7205502662</v>
       </c>
       <c r="W83">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X83" t="s">
         <v>191</v>
@@ -7799,7 +7799,7 @@
         <v>46267.79439748843</v>
       </c>
       <c r="W84">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X84" t="s">
         <v>192</v>
@@ -7870,7 +7870,7 @@
         <v>46267.79440011574</v>
       </c>
       <c r="W85">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X85" t="s">
         <v>194</v>
@@ -7941,7 +7941,7 @@
         <v>46267.79439818287</v>
       </c>
       <c r="W86">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X86" t="s">
         <v>193</v>
@@ -8015,7 +8015,7 @@
         <v>46267.7202693287</v>
       </c>
       <c r="W87">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X87" t="s">
         <v>191</v>
@@ -8086,7 +8086,7 @@
         <v>46267.79409846065</v>
       </c>
       <c r="W88">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X88" t="s">
         <v>192</v>
@@ -8160,7 +8160,7 @@
         <v>46267.79409725694</v>
       </c>
       <c r="W89">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X89" t="s">
         <v>192</v>
@@ -8228,7 +8228,7 @@
         <v>46267.79410239583</v>
       </c>
       <c r="W90">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X90" t="s">
         <v>194</v>
@@ -8296,7 +8296,7 @@
         <v>46267.79409934028</v>
       </c>
       <c r="W91">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X91" t="s">
         <v>193</v>
@@ -8370,7 +8370,7 @@
         <v>46267.72033356482</v>
       </c>
       <c r="W92">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X92" t="s">
         <v>191</v>
@@ -8441,7 +8441,7 @@
         <v>46267.79418105324</v>
       </c>
       <c r="W93">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X93" t="s">
         <v>192</v>
@@ -8515,7 +8515,7 @@
         <v>46267.79418005787</v>
       </c>
       <c r="W94">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X94" t="s">
         <v>192</v>
@@ -8583,7 +8583,7 @@
         <v>46267.79418379629</v>
       </c>
       <c r="W95">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X95" t="s">
         <v>194</v>
@@ -8651,7 +8651,7 @@
         <v>46267.79418283565</v>
       </c>
       <c r="W96">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X96" t="s">
         <v>193</v>
@@ -8725,7 +8725,7 @@
         <v>46267.71937662037</v>
       </c>
       <c r="W97">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X97" t="s">
         <v>191</v>
@@ -8796,7 +8796,7 @@
         <v>46267.79259834491</v>
       </c>
       <c r="W98">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X98" t="s">
         <v>192</v>
@@ -8870,7 +8870,7 @@
         <v>46267.79260170139</v>
       </c>
       <c r="W99">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X99" t="s">
         <v>193</v>
@@ -8947,7 +8947,7 @@
         <v>46268.37621265047</v>
       </c>
       <c r="W100">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X100" t="s">
         <v>195</v>
@@ -9021,7 +9021,7 @@
         <v>46267.79440636574</v>
       </c>
       <c r="W101">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X101" t="s">
         <v>194</v>
@@ -9095,7 +9095,7 @@
         <v>46267.72037954861</v>
       </c>
       <c r="W102">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X102" t="s">
         <v>191</v>
@@ -9166,7 +9166,7 @@
         <v>46267.79424664352</v>
       </c>
       <c r="W103">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X103" t="s">
         <v>192</v>
@@ -9240,7 +9240,7 @@
         <v>46267.79424586806</v>
       </c>
       <c r="W104">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X104" t="s">
         <v>192</v>
@@ -9308,7 +9308,7 @@
         <v>46267.79424864583</v>
       </c>
       <c r="W105">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X105" t="s">
         <v>194</v>
@@ -9376,7 +9376,7 @@
         <v>46267.79424725694</v>
       </c>
       <c r="W106">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X106" t="s">
         <v>193</v>
@@ -9450,7 +9450,7 @@
         <v>46267.79425081018</v>
       </c>
       <c r="W107">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X107" t="s">
         <v>195</v>
@@ -9524,7 +9524,7 @@
         <v>46267.71942916667</v>
       </c>
       <c r="W108">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X108" t="s">
         <v>191</v>
@@ -9595,7 +9595,7 @@
         <v>46267.79268530093</v>
       </c>
       <c r="W109">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X109" t="s">
         <v>194</v>
@@ -9669,7 +9669,7 @@
         <v>46267.79268769676</v>
       </c>
       <c r="W110">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X110" t="s">
         <v>193</v>
@@ -9740,7 +9740,7 @@
         <v>46267.79249748842</v>
       </c>
       <c r="W111">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X111" t="s">
         <v>194</v>
@@ -9814,7 +9814,7 @@
         <v>46267.79249788194</v>
       </c>
       <c r="W112">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X112" t="s">
         <v>193</v>
@@ -9888,7 +9888,7 @@
         <v>46267.71927280092</v>
       </c>
       <c r="W113">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X113" t="s">
         <v>191</v>
@@ -9959,7 +9959,7 @@
         <v>46267.79251079861</v>
       </c>
       <c r="W114">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X114" t="s">
         <v>194</v>
@@ -10033,7 +10033,7 @@
         <v>46267.79251038194</v>
       </c>
       <c r="W115">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X115" t="s">
         <v>193</v>
@@ -10107,7 +10107,7 @@
         <v>46267.72044811342</v>
       </c>
       <c r="W116">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X116" t="s">
         <v>191</v>
@@ -10178,7 +10178,7 @@
         <v>46267.79429737268</v>
       </c>
       <c r="W117">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X117" t="s">
         <v>192</v>
@@ -10252,7 +10252,7 @@
         <v>46267.79429603009</v>
       </c>
       <c r="W118">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X118" t="s">
         <v>192</v>
@@ -10320,7 +10320,7 @@
         <v>46267.79429876158</v>
       </c>
       <c r="W119">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X119" t="s">
         <v>194</v>
@@ -10388,7 +10388,7 @@
         <v>46267.79429826389</v>
       </c>
       <c r="W120">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X120" t="s">
         <v>193</v>
@@ -10462,7 +10462,7 @@
         <v>46267.72050385417</v>
       </c>
       <c r="W121">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X121" t="s">
         <v>191</v>
@@ -10533,7 +10533,7 @@
         <v>46267.79434996528</v>
       </c>
       <c r="W122">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X122" t="s">
         <v>192</v>
@@ -10607,7 +10607,7 @@
         <v>46267.79434864583</v>
       </c>
       <c r="W123">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X123" t="s">
         <v>192</v>
@@ -10675,7 +10675,7 @@
         <v>46267.79435208334</v>
       </c>
       <c r="W124">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X124" t="s">
         <v>194</v>
@@ -10743,7 +10743,7 @@
         <v>46267.79435100695</v>
       </c>
       <c r="W125">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X125" t="s">
         <v>193</v>
@@ -10820,7 +10820,7 @@
         <v>46273.6788224074</v>
       </c>
       <c r="W126">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X126" t="s">
         <v>193</v>
@@ -10900,7 +10900,7 @@
         <v>46273.67943539352</v>
       </c>
       <c r="W127">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X127" t="s">
         <v>193</v>
@@ -10977,7 +10977,7 @@
         <v>46266.37636392361</v>
       </c>
       <c r="W128">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X128" t="s">
         <v>197</v>
@@ -11051,7 +11051,7 @@
         <v>46266.37598834491</v>
       </c>
       <c r="W129">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X129" t="s">
         <v>197</v>
@@ -11128,7 +11128,7 @@
         <v>46268.45899988426</v>
       </c>
       <c r="W130">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X130" t="s">
         <v>198</v>
@@ -11205,7 +11205,7 @@
         <v>46266.45957881944</v>
       </c>
       <c r="W131">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X131" t="s">
         <v>196</v>
@@ -11279,7 +11279,7 @@
         <v>46266.37645462963</v>
       </c>
       <c r="W132">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X132" t="s">
         <v>197</v>
@@ -11353,7 +11353,7 @@
         <v>46266.37649475694</v>
       </c>
       <c r="W133">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X133" t="s">
         <v>197</v>
@@ -11427,7 +11427,7 @@
         <v>46266.37591180555</v>
       </c>
       <c r="W134">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X134" t="s">
         <v>197</v>
@@ -11504,7 +11504,7 @@
         <v>46268.45896508102</v>
       </c>
       <c r="W135">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X135" t="s">
         <v>198</v>
@@ -11581,7 +11581,7 @@
         <v>46266.45946195602</v>
       </c>
       <c r="W136">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X136" t="s">
         <v>196</v>
@@ -11655,7 +11655,7 @@
         <v>46266.37538684028</v>
       </c>
       <c r="W137">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X137" t="s">
         <v>197</v>
@@ -11729,7 +11729,7 @@
         <v>46266.37538506944</v>
       </c>
       <c r="W138">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X138" t="s">
         <v>201</v>
@@ -11806,7 +11806,7 @@
         <v>46268.45881820602</v>
       </c>
       <c r="W139">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X139" t="s">
         <v>198</v>
@@ -11883,7 +11883,7 @@
         <v>46266.45895332176</v>
       </c>
       <c r="W140">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X140" t="s">
         <v>200</v>
@@ -11957,7 +11957,7 @@
         <v>46266.45874105324</v>
       </c>
       <c r="W141">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X141" t="s">
         <v>196</v>
@@ -12031,7 +12031,7 @@
         <v>46266.45873584491</v>
       </c>
       <c r="W142">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X142" t="s">
         <v>196</v>
@@ -12105,7 +12105,7 @@
         <v>46273.6799675</v>
       </c>
       <c r="W143">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X143" t="s">
         <v>196</v>
@@ -12179,7 +12179,7 @@
         <v>46273.55254606481</v>
       </c>
       <c r="W144">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X144" t="s">
         <v>197</v>
@@ -12253,7 +12253,7 @@
         <v>46273.55252126158</v>
       </c>
       <c r="W145">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X145" t="s">
         <v>201</v>
@@ -12327,7 +12327,7 @@
         <v>46273.55254163194</v>
       </c>
       <c r="W146">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X146" t="s">
         <v>198</v>
@@ -12401,7 +12401,7 @@
         <v>46273.5525440162</v>
       </c>
       <c r="W147">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X147" t="s">
         <v>200</v>
@@ -12475,7 +12475,7 @@
         <v>46273.84422141204</v>
       </c>
       <c r="W148">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X148" t="s">
         <v>196</v>
@@ -12549,7 +12549,7 @@
         <v>46273.55254652778</v>
       </c>
       <c r="W149">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X149" t="s">
         <v>196</v>
@@ -12626,7 +12626,7 @@
         <v>46268.45898549769</v>
       </c>
       <c r="W150">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X150" t="s">
         <v>198</v>
@@ -12703,7 +12703,7 @@
         <v>46268.45915543981</v>
       </c>
       <c r="W151">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X151" t="s">
         <v>198</v>
@@ -12777,7 +12777,7 @@
         <v>46273.56305208334</v>
       </c>
       <c r="W152">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X152" t="s">
         <v>196</v>
@@ -12851,7 +12851,7 @@
         <v>46267.44505795139</v>
       </c>
       <c r="W153">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X153" t="s">
         <v>196</v>
@@ -12922,7 +12922,7 @@
         <v>46266.04180934028</v>
       </c>
       <c r="W154">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X154" t="s">
         <v>192</v>
@@ -12996,7 +12996,7 @@
         <v>46266.08343295139</v>
       </c>
       <c r="W155">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X155" t="s">
         <v>196</v>
@@ -13070,7 +13070,7 @@
         <v>46266.08344398148</v>
       </c>
       <c r="W156">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X156" t="s">
         <v>194</v>
@@ -13144,7 +13144,7 @@
         <v>46266.25077376157</v>
       </c>
       <c r="W157">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X157" t="s">
         <v>197</v>
@@ -13218,7 +13218,7 @@
         <v>46266.25004302083</v>
       </c>
       <c r="W158">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X158" t="s">
         <v>201</v>
@@ -13292,7 +13292,7 @@
         <v>46266.25135543982</v>
       </c>
       <c r="W159">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X159" t="s">
         <v>200</v>
@@ -13366,7 +13366,7 @@
         <v>46266.25305</v>
       </c>
       <c r="W160">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="X160" t="s">
         <v>197</v>
@@ -13440,7 +13440,7 @@
         <v>46266.25270034722</v>
       </c>
       <c r="W161">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="X161" t="s">
         <v>201</v>
@@ -13514,7 +13514,7 @@
         <v>46266.25274991898</v>
       </c>
       <c r="W162">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="X162" t="s">
         <v>192</v>
@@ -13588,7 +13588,7 @@
         <v>46266.25364633102</v>
       </c>
       <c r="W163">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="X163" t="s">
         <v>200</v>
@@ -13662,7 +13662,7 @@
         <v>46266.25369826389</v>
       </c>
       <c r="W164">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="X164" t="s">
         <v>193</v>
@@ -13736,7 +13736,7 @@
         <v>46266.25305112269</v>
       </c>
       <c r="W165">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X165" t="s">
         <v>197</v>
@@ -13810,7 +13810,7 @@
         <v>46266.25275173611</v>
       </c>
       <c r="W166">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X166" t="s">
         <v>192</v>
@@ -13884,7 +13884,7 @@
         <v>46266.25364869213</v>
       </c>
       <c r="W167">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X167" t="s">
         <v>196</v>
@@ -13958,7 +13958,7 @@
         <v>46266.25369988426</v>
       </c>
       <c r="W168">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X168" t="s">
         <v>193</v>
@@ -14035,7 +14035,7 @@
         <v>46268.62318445602</v>
       </c>
       <c r="W169">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X169" t="s">
         <v>197</v>
@@ -14112,7 +14112,7 @@
         <v>46268.62319864584</v>
       </c>
       <c r="W170">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X170" t="s">
         <v>201</v>
@@ -14189,7 +14189,7 @@
         <v>46268.62320026621</v>
       </c>
       <c r="W171">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X171" t="s">
         <v>198</v>
@@ -14266,7 +14266,7 @@
         <v>46268.62320177083</v>
       </c>
       <c r="W172">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X172" t="s">
         <v>191</v>
@@ -14343,7 +14343,7 @@
         <v>46268.62320378472</v>
       </c>
       <c r="W173">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X173" t="s">
         <v>192</v>
@@ -14420,7 +14420,7 @@
         <v>46268.62320393518</v>
       </c>
       <c r="W174">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X174" t="s">
         <v>192</v>
@@ -14497,7 +14497,7 @@
         <v>46268.62320697917</v>
       </c>
       <c r="W175">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X175" t="s">
         <v>200</v>
@@ -14574,7 +14574,7 @@
         <v>46268.62320717592</v>
       </c>
       <c r="W176">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X176" t="s">
         <v>196</v>
@@ -14651,7 +14651,7 @@
         <v>46268.62320732639</v>
       </c>
       <c r="W177">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X177" t="s">
         <v>196</v>
@@ -14728,7 +14728,7 @@
         <v>46268.62320810185</v>
       </c>
       <c r="W178">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X178" t="s">
         <v>196</v>
@@ -14805,7 +14805,7 @@
         <v>46268.6232125</v>
       </c>
       <c r="W179">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X179" t="s">
         <v>194</v>
@@ -14882,7 +14882,7 @@
         <v>46268.62321412037</v>
       </c>
       <c r="W180">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X180" t="s">
         <v>193</v>
@@ -14959,7 +14959,7 @@
         <v>46268.6232128125</v>
       </c>
       <c r="W181">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X181" t="s">
         <v>195</v>
@@ -15036,7 +15036,7 @@
         <v>46268.62321296296</v>
       </c>
       <c r="W182">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X182" t="s">
         <v>195</v>
@@ -15110,7 +15110,7 @@
         <v>46269.41908927084</v>
       </c>
       <c r="W183">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X183" t="s">
         <v>197</v>
@@ -15181,7 +15181,7 @@
         <v>46269.41910457176</v>
       </c>
       <c r="W184">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X184" t="s">
         <v>201</v>
@@ -15252,7 +15252,7 @@
         <v>46269.37885223379</v>
       </c>
       <c r="W185">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X185" t="s">
         <v>198</v>
@@ -15323,7 +15323,7 @@
         <v>46269.3782503125</v>
       </c>
       <c r="W186">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X186" t="s">
         <v>191</v>
@@ -15394,7 +15394,7 @@
         <v>46269.41913152778</v>
       </c>
       <c r="W187">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X187" t="s">
         <v>192</v>
@@ -15465,7 +15465,7 @@
         <v>46269.41913775463</v>
       </c>
       <c r="W188">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X188" t="s">
         <v>192</v>
@@ -15536,7 +15536,7 @@
         <v>46268.7596207176</v>
       </c>
       <c r="W189">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X189" t="s">
         <v>197</v>
@@ -15607,7 +15607,7 @@
         <v>46268.75963109954</v>
       </c>
       <c r="W190">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X190" t="s">
         <v>201</v>
@@ -15678,7 +15678,7 @@
         <v>46268.75963225694</v>
       </c>
       <c r="W191">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X191" t="s">
         <v>198</v>
@@ -15749,7 +15749,7 @@
         <v>46268.75963348379</v>
       </c>
       <c r="W192">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X192" t="s">
         <v>191</v>
@@ -15820,7 +15820,7 @@
         <v>46268.75963414352</v>
       </c>
       <c r="W193">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X193" t="s">
         <v>192</v>
@@ -15891,7 +15891,7 @@
         <v>46268.62326365741</v>
       </c>
       <c r="W194">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X194" t="s">
         <v>192</v>
@@ -15962,7 +15962,7 @@
         <v>46268.75963472222</v>
       </c>
       <c r="W195">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X195" t="s">
         <v>200</v>
@@ -16033,7 +16033,7 @@
         <v>46268.75963475694</v>
       </c>
       <c r="W196">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X196" t="s">
         <v>196</v>
@@ -16104,7 +16104,7 @@
         <v>46268.75963506944</v>
       </c>
       <c r="W197">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X197" t="s">
         <v>196</v>
@@ -16175,7 +16175,7 @@
         <v>46268.7596360301</v>
       </c>
       <c r="W198">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X198" t="s">
         <v>196</v>
@@ -16246,7 +16246,7 @@
         <v>46268.62327121528</v>
       </c>
       <c r="W199">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X199" t="s">
         <v>194</v>
@@ -16317,7 +16317,7 @@
         <v>46268.75963931713</v>
       </c>
       <c r="W200">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X200" t="s">
         <v>193</v>
@@ -16388,7 +16388,7 @@
         <v>46268.75963822917</v>
       </c>
       <c r="W201">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X201" t="s">
         <v>195</v>
@@ -16459,7 +16459,7 @@
         <v>46268.75963857639</v>
       </c>
       <c r="W202">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X202" t="s">
         <v>195</v>
@@ -16530,7 +16530,7 @@
         <v>46269.41908901621</v>
       </c>
       <c r="W203">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X203" t="s">
         <v>197</v>
@@ -16601,7 +16601,7 @@
         <v>46269.41910425926</v>
       </c>
       <c r="W204">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X204" t="s">
         <v>201</v>
@@ -16672,7 +16672,7 @@
         <v>46269.37890997685</v>
       </c>
       <c r="W205">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X205" t="s">
         <v>198</v>
@@ -16743,7 +16743,7 @@
         <v>46269.37833320602</v>
       </c>
       <c r="W206">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X206" t="s">
         <v>191</v>
@@ -16814,7 +16814,7 @@
         <v>46269.41913112268</v>
       </c>
       <c r="W207">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X207" t="s">
         <v>192</v>
@@ -16885,7 +16885,7 @@
         <v>46269.41913740741</v>
       </c>
       <c r="W208">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X208" t="s">
         <v>192</v>
@@ -16956,7 +16956,7 @@
         <v>46267.66131466435</v>
       </c>
       <c r="W209">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X209" t="s">
         <v>201</v>
@@ -17030,7 +17030,7 @@
         <v>46266.21595836805</v>
       </c>
       <c r="W210">
-        <v>-40</v>
+        <v>-39</v>
       </c>
       <c r="X210" t="s">
         <v>201</v>
@@ -17104,7 +17104,7 @@
         <v>46266.21572962963</v>
       </c>
       <c r="W211">
-        <v>-40</v>
+        <v>-39</v>
       </c>
       <c r="X211" t="s">
         <v>197</v>
@@ -17178,7 +17178,7 @@
         <v>46266.21550011574</v>
       </c>
       <c r="W212">
-        <v>-40</v>
+        <v>-39</v>
       </c>
       <c r="X212" t="s">
         <v>198</v>
@@ -17252,7 +17252,7 @@
         <v>46266.00006921296</v>
       </c>
       <c r="W213">
-        <v>-40</v>
+        <v>-39</v>
       </c>
       <c r="X213" t="s">
         <v>197</v>
@@ -17323,7 +17323,7 @@
         <v>46266.00006921296</v>
       </c>
       <c r="W214">
-        <v>-40</v>
+        <v>-39</v>
       </c>
       <c r="X214" t="s">
         <v>201</v>
@@ -17391,7 +17391,7 @@
         <v>46269.57097615741</v>
       </c>
       <c r="W215">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X215" t="s">
         <v>198</v>
@@ -17459,7 +17459,7 @@
         <v>46266.00006921296</v>
       </c>
       <c r="W216">
-        <v>-40</v>
+        <v>-39</v>
       </c>
       <c r="X216" t="s">
         <v>198</v>
@@ -17527,7 +17527,7 @@
         <v>46269.46753030093</v>
       </c>
       <c r="W217">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X217" t="s">
         <v>194</v>
@@ -17604,7 +17604,7 @@
         <v>46280.37528408565</v>
       </c>
       <c r="W218">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X218" t="s">
         <v>197</v>
@@ -17681,7 +17681,7 @@
         <v>46281.63558861111</v>
       </c>
       <c r="W219">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X219" t="s">
         <v>192</v>
@@ -17761,7 +17761,7 @@
         <v>46281.6358927662</v>
       </c>
       <c r="W220">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X220" t="s">
         <v>192</v>
@@ -17841,7 +17841,7 @@
         <v>46281.47564895833</v>
       </c>
       <c r="W221">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X221" t="s">
         <v>194</v>
@@ -17921,7 +17921,7 @@
         <v>46279.66710767361</v>
       </c>
       <c r="W222">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X222" t="s">
         <v>196</v>
@@ -18001,7 +18001,7 @@
         <v>46281.68877074074</v>
       </c>
       <c r="W223">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X223" t="s">
         <v>198</v>
@@ -18081,7 +18081,7 @@
         <v>46280.57958537037</v>
       </c>
       <c r="W224">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X224" t="s">
         <v>191</v>
@@ -18161,7 +18161,7 @@
         <v>46281.63570936343</v>
       </c>
       <c r="W225">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X225" t="s">
         <v>192</v>
@@ -18241,7 +18241,7 @@
         <v>46281.63595871528</v>
       </c>
       <c r="W226">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X226" t="s">
         <v>192</v>
@@ -18318,7 +18318,7 @@
         <v>46279.62681744213</v>
       </c>
       <c r="W227">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X227" t="s">
         <v>200</v>
@@ -18392,7 +18392,7 @@
         <v>46279.66707821759</v>
       </c>
       <c r="W228">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X228" t="s">
         <v>196</v>
@@ -18469,7 +18469,7 @@
         <v>46281.68880230324</v>
       </c>
       <c r="W229">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X229" t="s">
         <v>198</v>
@@ -18549,7 +18549,7 @@
         <v>46280.57972293982</v>
       </c>
       <c r="W230">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X230" t="s">
         <v>191</v>
@@ -18629,7 +18629,7 @@
         <v>46281.63575075231</v>
       </c>
       <c r="W231">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X231" t="s">
         <v>192</v>
@@ -18709,7 +18709,7 @@
         <v>46281.63599785879</v>
       </c>
       <c r="W232">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X232" t="s">
         <v>192</v>
@@ -18786,7 +18786,7 @@
         <v>46279.6268503125</v>
       </c>
       <c r="W233">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X233" t="s">
         <v>200</v>
@@ -18860,7 +18860,7 @@
         <v>46279.66698128472</v>
       </c>
       <c r="W234">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="X234" t="s">
         <v>196</v>
@@ -18931,7 +18931,7 @@
         <v>46279.66929922454</v>
       </c>
       <c r="W235">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X235" t="s">
         <v>197</v>
@@ -19008,7 +19008,7 @@
         <v>46280.61353684028</v>
       </c>
       <c r="W236">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X236" t="s">
         <v>201</v>
@@ -19085,7 +19085,7 @@
         <v>46280.61353920139</v>
       </c>
       <c r="W237">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X237" t="s">
         <v>198</v>
@@ -19162,7 +19162,7 @@
         <v>46279.63250563657</v>
       </c>
       <c r="W238">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X238" t="s">
         <v>191</v>
@@ -19239,7 +19239,7 @@
         <v>46280.61354019676</v>
       </c>
       <c r="W239">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X239" t="s">
         <v>192</v>
@@ -19316,7 +19316,7 @@
         <v>46280.6135403125</v>
       </c>
       <c r="W240">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X240" t="s">
         <v>192</v>
@@ -19396,7 +19396,7 @@
         <v>46281.71218414352</v>
       </c>
       <c r="W241">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X241" t="s">
         <v>200</v>
@@ -19473,7 +19473,7 @@
         <v>46281.41576883102</v>
       </c>
       <c r="W242">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X242" t="s">
         <v>196</v>
@@ -19550,7 +19550,7 @@
         <v>46280.43132989584</v>
       </c>
       <c r="W243">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X243" t="s">
         <v>194</v>
@@ -19627,7 +19627,7 @@
         <v>46280.61367623843</v>
       </c>
       <c r="W244">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X244" t="s">
         <v>193</v>
@@ -19704,7 +19704,7 @@
         <v>46274.60593387731</v>
       </c>
       <c r="W245">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X245" t="s">
         <v>197</v>
@@ -19784,7 +19784,7 @@
         <v>46274.47210818287</v>
       </c>
       <c r="W246">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X246" t="s">
         <v>198</v>
@@ -19864,7 +19864,7 @@
         <v>46276.48975401621</v>
       </c>
       <c r="W247">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X247" t="s">
         <v>192</v>
@@ -19944,7 +19944,7 @@
         <v>46279.38429019676</v>
       </c>
       <c r="W248">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X248" t="s">
         <v>192</v>
@@ -20024,7 +20024,7 @@
         <v>46274.48792050926</v>
       </c>
       <c r="W249">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X249" t="s">
         <v>196</v>
@@ -20104,7 +20104,7 @@
         <v>46274.588374375</v>
       </c>
       <c r="W250">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X250" t="s">
         <v>194</v>
@@ -20181,7 +20181,7 @@
         <v>46274.34198912037</v>
       </c>
       <c r="W251">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X251" t="s">
         <v>193</v>
@@ -20252,7 +20252,7 @@
         <v>46279.6693627662</v>
       </c>
       <c r="W252">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X252" t="s">
         <v>197</v>
@@ -20332,7 +20332,7 @@
         <v>46279.5886965625</v>
       </c>
       <c r="W253">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X253" t="s">
         <v>198</v>
@@ -20409,7 +20409,7 @@
         <v>46279.40189383102</v>
       </c>
       <c r="W254">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X254" t="s">
         <v>191</v>
@@ -20489,7 +20489,7 @@
         <v>46279.58878520833</v>
       </c>
       <c r="W255">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X255" t="s">
         <v>192</v>
@@ -20569,7 +20569,7 @@
         <v>46279.58873577546</v>
       </c>
       <c r="W256">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X256" t="s">
         <v>192</v>
@@ -20646,7 +20646,7 @@
         <v>46279.63255</v>
       </c>
       <c r="W257">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X257" t="s">
         <v>200</v>
@@ -20723,7 +20723,7 @@
         <v>46276.63187557871</v>
       </c>
       <c r="W258">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X258" t="s">
         <v>196</v>
@@ -20800,7 +20800,7 @@
         <v>46279.6265846875</v>
       </c>
       <c r="W259">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X259" t="s">
         <v>194</v>
@@ -20877,7 +20877,7 @@
         <v>46279.63255401621</v>
       </c>
       <c r="W260">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X260" t="s">
         <v>193</v>
@@ -20957,7 +20957,7 @@
         <v>46279.66713805556</v>
       </c>
       <c r="W261">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X261" t="s">
         <v>196</v>
@@ -21031,7 +21031,7 @@
         <v>46281.63317659722</v>
       </c>
       <c r="W262">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X262" t="s">
         <v>198</v>
@@ -21105,7 +21105,7 @@
         <v>46275.39631951389</v>
       </c>
       <c r="W263">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X263" t="s">
         <v>192</v>
@@ -21179,7 +21179,7 @@
         <v>46275.39631994213</v>
       </c>
       <c r="W264">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X264" t="s">
         <v>192</v>
@@ -21259,7 +21259,7 @@
         <v>46280.62789608796</v>
       </c>
       <c r="W265">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X265" t="s">
         <v>195</v>
@@ -21339,7 +21339,7 @@
         <v>46280.63189497685</v>
       </c>
       <c r="W266">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X266" t="s">
         <v>195</v>
@@ -21419,7 +21419,7 @@
         <v>46280.72961366898</v>
       </c>
       <c r="W267">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X267" t="s">
         <v>192</v>
@@ -21493,7 +21493,7 @@
         <v>46276.37795540509</v>
       </c>
       <c r="W268">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X268" t="s">
         <v>194</v>
@@ -21570,7 +21570,7 @@
         <v>46276.66923222222</v>
       </c>
       <c r="W269">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X269" t="s">
         <v>191</v>
@@ -21644,7 +21644,7 @@
         <v>46276.40669469907</v>
       </c>
       <c r="W270">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X270" t="s">
         <v>192</v>
@@ -21721,7 +21721,7 @@
         <v>46276.64773491898</v>
       </c>
       <c r="W271">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X271" t="s">
         <v>192</v>
@@ -21798,7 +21798,7 @@
         <v>46276.39101108797</v>
       </c>
       <c r="W272">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X272" t="s">
         <v>194</v>
@@ -21878,7 +21878,7 @@
         <v>46280.40395534722</v>
       </c>
       <c r="W273">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X273" t="s">
         <v>193</v>
@@ -21955,7 +21955,7 @@
         <v>46279.74982357639</v>
       </c>
       <c r="W274">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X274" t="s">
         <v>195</v>
@@ -22035,7 +22035,7 @@
         <v>46276.66651596065</v>
       </c>
       <c r="W275">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X275" t="s">
         <v>195</v>
@@ -22112,7 +22112,7 @@
         <v>46280.66345891204</v>
       </c>
       <c r="W276">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="X276" t="s">
         <v>192</v>
@@ -22186,7 +22186,7 @@
         <v>46274.36843923611</v>
       </c>
       <c r="W277">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X277" t="s">
         <v>192</v>
@@ -22263,7 +22263,7 @@
         <v>46274.66470667824</v>
       </c>
       <c r="W278">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X278" t="s">
         <v>195</v>
@@ -22340,7 +22340,7 @@
         <v>46274.74452168981</v>
       </c>
       <c r="W279">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X279" t="s">
         <v>195</v>
@@ -22420,7 +22420,7 @@
         <v>46274.64801501157</v>
       </c>
       <c r="W280">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X280" t="s">
         <v>191</v>
@@ -22494,7 +22494,7 @@
         <v>46274.36695243056</v>
       </c>
       <c r="W281">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X281" t="s">
         <v>192</v>
@@ -22568,7 +22568,7 @@
         <v>46276.4084265625</v>
       </c>
       <c r="W282">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X282" t="s">
         <v>194</v>
@@ -22645,7 +22645,7 @@
         <v>46274.7274781713</v>
       </c>
       <c r="W283">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X283" t="s">
         <v>195</v>
@@ -22719,7 +22719,7 @@
         <v>46274.74558746528</v>
       </c>
       <c r="W284">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X284" t="s">
         <v>195</v>
@@ -22793,7 +22793,7 @@
         <v>46275.79245582176</v>
       </c>
       <c r="W285">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X285" t="s">
         <v>193</v>
@@ -22867,7 +22867,7 @@
         <v>46280.63707425926</v>
       </c>
       <c r="W286">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X286" t="s">
         <v>192</v>
@@ -22944,7 +22944,7 @@
         <v>46280.38311703704</v>
       </c>
       <c r="W287">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X287" t="s">
         <v>194</v>
@@ -23024,7 +23024,7 @@
         <v>46280.37743127315</v>
       </c>
       <c r="W288">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X288" t="s">
         <v>193</v>
@@ -23104,7 +23104,7 @@
         <v>46280.45035295139</v>
       </c>
       <c r="W289">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X289" t="s">
         <v>198</v>
@@ -23181,7 +23181,7 @@
         <v>46280.59788275463</v>
       </c>
       <c r="W290">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X290" t="s">
         <v>198</v>
@@ -23261,7 +23261,7 @@
         <v>46280.73313407407</v>
       </c>
       <c r="W291">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X291" t="s">
         <v>196</v>
@@ -23338,7 +23338,7 @@
         <v>46276.49596842592</v>
       </c>
       <c r="W292">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X292" t="s">
         <v>197</v>
@@ -23412,7 +23412,7 @@
         <v>46276.53874935185</v>
       </c>
       <c r="W293">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X293" t="s">
         <v>201</v>
@@ -23486,7 +23486,7 @@
         <v>46276.49597027778</v>
       </c>
       <c r="W294">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X294" t="s">
         <v>198</v>
@@ -23560,7 +23560,7 @@
         <v>46276.62604146991</v>
       </c>
       <c r="W295">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X295" t="s">
         <v>200</v>
@@ -23634,7 +23634,7 @@
         <v>46276.68231165509</v>
       </c>
       <c r="W296">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X296" t="s">
         <v>196</v>
@@ -23711,7 +23711,7 @@
         <v>46276.7163278588</v>
       </c>
       <c r="W297">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X297" t="s">
         <v>196</v>
@@ -23788,7 +23788,7 @@
         <v>46276.6823121412</v>
       </c>
       <c r="W298">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X298" t="s">
         <v>196</v>
@@ -23865,7 +23865,7 @@
         <v>46280.69323744213</v>
       </c>
       <c r="W299">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X299" t="s">
         <v>197</v>
@@ -23942,7 +23942,7 @@
         <v>46274.70622837963</v>
       </c>
       <c r="W300">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X300" t="s">
         <v>201</v>
@@ -24016,7 +24016,7 @@
         <v>46275.71996309028</v>
       </c>
       <c r="W301">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X301" t="s">
         <v>200</v>
@@ -24090,7 +24090,7 @@
         <v>46275.54278886574</v>
       </c>
       <c r="W302">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X302" t="s">
         <v>196</v>
@@ -24167,7 +24167,7 @@
         <v>46280.74859975695</v>
       </c>
       <c r="W303">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X303" t="s">
         <v>197</v>
@@ -24244,7 +24244,7 @@
         <v>46275.7000328588</v>
       </c>
       <c r="W304">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X304" t="s">
         <v>201</v>
@@ -24318,7 +24318,7 @@
         <v>46275.72031699074</v>
       </c>
       <c r="W305">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X305" t="s">
         <v>198</v>
@@ -24392,7 +24392,7 @@
         <v>46275.54095912037</v>
       </c>
       <c r="W306">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X306" t="s">
         <v>200</v>
@@ -24466,7 +24466,7 @@
         <v>46275.72225363426</v>
       </c>
       <c r="W307">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X307" t="s">
         <v>196</v>
@@ -24540,7 +24540,7 @@
         <v>46275.7222629051</v>
       </c>
       <c r="W308">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X308" t="s">
         <v>196</v>
@@ -24614,7 +24614,7 @@
         <v>46275.7222709838</v>
       </c>
       <c r="W309">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X309" t="s">
         <v>196</v>
@@ -24691,7 +24691,7 @@
         <v>46274.74837762731</v>
       </c>
       <c r="W310">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X310" t="s">
         <v>197</v>
@@ -24771,7 +24771,7 @@
         <v>46274.74838096065</v>
       </c>
       <c r="W311">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X311" t="s">
         <v>200</v>
@@ -24851,7 +24851,7 @@
         <v>46280.56274502315</v>
       </c>
       <c r="W312">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X312" t="s">
         <v>196</v>
@@ -24928,7 +24928,7 @@
         <v>46274.42878043981</v>
       </c>
       <c r="W313">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X313" t="s">
         <v>197</v>
@@ -25005,7 +25005,7 @@
         <v>46275.40196778935</v>
       </c>
       <c r="W314">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X314" t="s">
         <v>198</v>
@@ -25082,7 +25082,7 @@
         <v>46276.52399603009</v>
       </c>
       <c r="W315">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X315" t="s">
         <v>200</v>
@@ -25159,7 +25159,7 @@
         <v>46276.5240703125</v>
       </c>
       <c r="W316">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X316" t="s">
         <v>196</v>
@@ -25233,7 +25233,7 @@
         <v>46275.4100730787</v>
       </c>
       <c r="W317">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X317" t="s">
         <v>193</v>
@@ -25307,7 +25307,7 @@
         <v>46275.40964188657</v>
       </c>
       <c r="W318">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X318" t="s">
         <v>195</v>
@@ -25381,7 +25381,7 @@
         <v>46275.40964245371</v>
       </c>
       <c r="W319">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X319" t="s">
         <v>195</v>
@@ -25455,7 +25455,7 @@
         <v>46275.45011145833</v>
       </c>
       <c r="W320">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X320" t="s">
         <v>191</v>
@@ -25529,7 +25529,7 @@
         <v>46275.44901016204</v>
       </c>
       <c r="W321">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X321" t="s">
         <v>192</v>
@@ -25603,7 +25603,7 @@
         <v>46276.71732053241</v>
       </c>
       <c r="W322">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X322" t="s">
         <v>200</v>
@@ -25680,7 +25680,7 @@
         <v>46276.71697232639</v>
       </c>
       <c r="W323">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X323" t="s">
         <v>196</v>
@@ -25757,7 +25757,7 @@
         <v>46276.7175884838</v>
       </c>
       <c r="W324">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X324" t="s">
         <v>196</v>
@@ -25834,7 +25834,7 @@
         <v>46276.7175895949</v>
       </c>
       <c r="W325">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X325" t="s">
         <v>196</v>
@@ -25911,7 +25911,7 @@
         <v>46276.71759461806</v>
       </c>
       <c r="W326">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X326" t="s">
         <v>194</v>
@@ -25985,7 +25985,7 @@
         <v>46275.44975668981</v>
       </c>
       <c r="W327">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X327" t="s">
         <v>193</v>
@@ -26059,7 +26059,7 @@
         <v>46275.44933692129</v>
       </c>
       <c r="W328">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X328" t="s">
         <v>195</v>
@@ -26133,7 +26133,7 @@
         <v>46275.44933814815</v>
       </c>
       <c r="W329">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X329" t="s">
         <v>195</v>
@@ -26207,7 +26207,7 @@
         <v>46274.41771849537</v>
       </c>
       <c r="W330">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X330" t="s">
         <v>200</v>
@@ -26278,7 +26278,7 @@
         <v>46274.41775447917</v>
       </c>
       <c r="W331">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X331" t="s">
         <v>196</v>
@@ -26349,7 +26349,7 @@
         <v>46274.41777533565</v>
       </c>
       <c r="W332">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X332" t="s">
         <v>196</v>
@@ -26420,7 +26420,7 @@
         <v>46274.41799166667</v>
       </c>
       <c r="W333">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X333" t="s">
         <v>194</v>
@@ -26491,7 +26491,7 @@
         <v>46274.41800114583</v>
       </c>
       <c r="W334">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X334" t="s">
         <v>193</v>
@@ -26562,7 +26562,7 @@
         <v>46274.41772148148</v>
       </c>
       <c r="W335">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X335" t="s">
         <v>200</v>
@@ -26633,7 +26633,7 @@
         <v>46274.41773631945</v>
       </c>
       <c r="W336">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X336" t="s">
         <v>196</v>
@@ -26704,7 +26704,7 @@
         <v>46274.41777481481</v>
       </c>
       <c r="W337">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X337" t="s">
         <v>196</v>
@@ -26775,7 +26775,7 @@
         <v>46274.41799332176</v>
       </c>
       <c r="W338">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X338" t="s">
         <v>194</v>
@@ -26846,7 +26846,7 @@
         <v>46274.41800085648</v>
       </c>
       <c r="W339">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X339" t="s">
         <v>193</v>
@@ -26917,7 +26917,7 @@
         <v>46275.31737530093</v>
       </c>
       <c r="W340">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X340" t="s">
         <v>197</v>
@@ -26988,7 +26988,7 @@
         <v>46275.31747032407</v>
       </c>
       <c r="W341">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X341" t="s">
         <v>201</v>
@@ -27059,7 +27059,7 @@
         <v>46275.31747981482</v>
       </c>
       <c r="W342">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X342" t="s">
         <v>198</v>
@@ -27130,7 +27130,7 @@
         <v>46275.31748724537</v>
       </c>
       <c r="W343">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X343" t="s">
         <v>191</v>
@@ -27201,7 +27201,7 @@
         <v>46275.31749535879</v>
       </c>
       <c r="W344">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X344" t="s">
         <v>192</v>
@@ -27272,7 +27272,7 @@
         <v>46275.31750491898</v>
       </c>
       <c r="W345">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X345" t="s">
         <v>200</v>
@@ -27343,7 +27343,7 @@
         <v>46275.31750555555</v>
       </c>
       <c r="W346">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X346" t="s">
         <v>196</v>
@@ -27414,7 +27414,7 @@
         <v>46275.31750599537</v>
       </c>
       <c r="W347">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X347" t="s">
         <v>196</v>
@@ -27485,7 +27485,7 @@
         <v>46275.5810894676</v>
       </c>
       <c r="W348">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X348" t="s">
         <v>197</v>
@@ -27559,7 +27559,7 @@
         <v>46275.58158541666</v>
       </c>
       <c r="W349">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X349" t="s">
         <v>198</v>
@@ -27633,7 +27633,7 @@
         <v>46279.70955146991</v>
       </c>
       <c r="W350">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="X350" t="s">
         <v>197</v>
@@ -27707,7 +27707,7 @@
         <v>46276.41675075232</v>
       </c>
       <c r="W351">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X351" t="s">
         <v>192</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-17 15:21
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5544" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5558" uniqueCount="353">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1437,7 +1437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI385"/>
+  <dimension ref="A1:AI386"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -27761,16 +27761,16 @@
     </row>
     <row r="352" spans="1:35">
       <c r="A352">
-        <v>6703</v>
+        <v>6548</v>
       </c>
       <c r="B352" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C352" t="s">
         <v>50</v>
       </c>
       <c r="D352" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E352" t="s">
         <v>54</v>
@@ -27779,13 +27779,13 @@
         <v>56</v>
       </c>
       <c r="G352">
-        <v>1628</v>
+        <v>1697</v>
       </c>
       <c r="H352">
-        <v>1581</v>
+        <v>1650</v>
       </c>
       <c r="I352" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J352" t="s">
         <v>75</v>
@@ -27800,31 +27800,31 @@
         <v>2026</v>
       </c>
       <c r="R352">
-        <v>17955176</v>
+        <v>17968001</v>
       </c>
       <c r="S352" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="T352" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="U352" t="s">
         <v>193</v>
       </c>
       <c r="V352" s="1">
-        <v>46282.42251184028</v>
+        <v>46282.62254486111</v>
       </c>
       <c r="W352">
         <v>-4</v>
       </c>
       <c r="X352" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="AB352">
         <v>0</v>
       </c>
       <c r="AC352" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="AH352" t="s">
         <v>347</v>
@@ -27835,16 +27835,16 @@
     </row>
     <row r="353" spans="1:35">
       <c r="A353">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B353" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C353" t="s">
         <v>50</v>
       </c>
       <c r="D353" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E353" t="s">
         <v>54</v>
@@ -27853,49 +27853,52 @@
         <v>56</v>
       </c>
       <c r="G353">
-        <v>5883</v>
+        <v>1628</v>
       </c>
       <c r="H353">
-        <v>5792</v>
+        <v>1581</v>
       </c>
       <c r="I353" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J353" t="s">
-        <v>125</v>
+        <v>75</v>
       </c>
       <c r="N353" s="1">
         <v>46286</v>
       </c>
       <c r="P353">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q353">
         <v>2026</v>
       </c>
       <c r="R353">
-        <v>17399067</v>
+        <v>17955176</v>
       </c>
       <c r="S353" t="s">
-        <v>171</v>
+        <v>165</v>
+      </c>
+      <c r="T353" t="s">
+        <v>186</v>
       </c>
       <c r="U353" t="s">
         <v>193</v>
       </c>
       <c r="V353" s="1">
-        <v>46282.47420876157</v>
+        <v>46282.42251184028</v>
       </c>
       <c r="W353">
         <v>-4</v>
       </c>
       <c r="X353" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AB353">
         <v>0</v>
       </c>
       <c r="AC353" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="AH353" t="s">
         <v>347</v>
@@ -27924,7 +27927,7 @@
         <v>56</v>
       </c>
       <c r="G354">
-        <v>5884</v>
+        <v>5883</v>
       </c>
       <c r="H354">
         <v>5792</v>
@@ -27933,7 +27936,7 @@
         <v>61</v>
       </c>
       <c r="J354" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N354" s="1">
         <v>46286</v>
@@ -27945,7 +27948,7 @@
         <v>2026</v>
       </c>
       <c r="R354">
-        <v>17399077</v>
+        <v>17399067</v>
       </c>
       <c r="S354" t="s">
         <v>171</v>
@@ -27954,7 +27957,7 @@
         <v>193</v>
       </c>
       <c r="V354" s="1">
-        <v>46282.47437324074</v>
+        <v>46282.47420876157</v>
       </c>
       <c r="W354">
         <v>-4</v>
@@ -27977,16 +27980,16 @@
     </row>
     <row r="355" spans="1:35">
       <c r="A355">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B355" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C355" t="s">
         <v>50</v>
       </c>
       <c r="D355" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E355" t="s">
         <v>54</v>
@@ -27995,23 +27998,20 @@
         <v>56</v>
       </c>
       <c r="G355">
-        <v>5903</v>
+        <v>5884</v>
       </c>
       <c r="H355">
-        <v>5830</v>
+        <v>5792</v>
       </c>
       <c r="I355" t="s">
         <v>61</v>
       </c>
       <c r="J355" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="N355" s="1">
         <v>46286</v>
       </c>
-      <c r="O355" t="s">
-        <v>154</v>
-      </c>
       <c r="P355">
         <v>9</v>
       </c>
@@ -28019,34 +28019,28 @@
         <v>2026</v>
       </c>
       <c r="R355">
-        <v>16962221</v>
+        <v>17399077</v>
       </c>
       <c r="S355" t="s">
-        <v>172</v>
-      </c>
-      <c r="T355" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="U355" t="s">
         <v>193</v>
       </c>
       <c r="V355" s="1">
-        <v>46282.42048836806</v>
+        <v>46282.47437324074</v>
       </c>
       <c r="W355">
         <v>-4</v>
       </c>
       <c r="X355" t="s">
-        <v>205</v>
-      </c>
-      <c r="Y355" t="s">
-        <v>337</v>
+        <v>201</v>
       </c>
       <c r="AB355">
         <v>0</v>
       </c>
       <c r="AC355" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AH355" t="s">
         <v>347</v>
@@ -28075,20 +28069,23 @@
         <v>56</v>
       </c>
       <c r="G356">
+        <v>5903</v>
+      </c>
+      <c r="H356">
         <v>5830</v>
-      </c>
-      <c r="H356">
-        <v>5784</v>
       </c>
       <c r="I356" t="s">
         <v>61</v>
       </c>
       <c r="J356" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N356" s="1">
         <v>46286</v>
       </c>
+      <c r="O356" t="s">
+        <v>154</v>
+      </c>
       <c r="P356">
         <v>9</v>
       </c>
@@ -28096,7 +28093,7 @@
         <v>2026</v>
       </c>
       <c r="R356">
-        <v>16962211</v>
+        <v>16962221</v>
       </c>
       <c r="S356" t="s">
         <v>172</v>
@@ -28108,13 +28105,16 @@
         <v>193</v>
       </c>
       <c r="V356" s="1">
-        <v>46282.42138976852</v>
+        <v>46282.42048836806</v>
       </c>
       <c r="W356">
         <v>-4</v>
       </c>
       <c r="X356" t="s">
         <v>205</v>
+      </c>
+      <c r="Y356" t="s">
+        <v>337</v>
       </c>
       <c r="AB356">
         <v>0</v>
@@ -28149,55 +28149,52 @@
         <v>56</v>
       </c>
       <c r="G357">
-        <v>7025</v>
+        <v>5830</v>
       </c>
       <c r="H357">
-        <v>0</v>
+        <v>5784</v>
       </c>
       <c r="I357" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J357" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="N357" s="1">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="P357">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q357">
         <v>2026</v>
       </c>
       <c r="R357">
-        <v>16962338</v>
+        <v>16962211</v>
       </c>
       <c r="S357" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="T357" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="U357" t="s">
         <v>193</v>
       </c>
       <c r="V357" s="1">
-        <v>46282.54038741898</v>
+        <v>46282.42138976852</v>
       </c>
       <c r="W357">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="X357" t="s">
         <v>205</v>
       </c>
-      <c r="Y357" t="s">
-        <v>338</v>
-      </c>
       <c r="AB357">
         <v>0</v>
       </c>
       <c r="AC357" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="AH357" t="s">
         <v>347</v>
@@ -28208,16 +28205,16 @@
     </row>
     <row r="358" spans="1:35">
       <c r="A358">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B358" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C358" t="s">
         <v>50</v>
       </c>
       <c r="D358" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E358" t="s">
         <v>54</v>
@@ -28226,58 +28223,58 @@
         <v>56</v>
       </c>
       <c r="G358">
-        <v>9086</v>
+        <v>7025</v>
       </c>
       <c r="H358">
         <v>0</v>
       </c>
       <c r="I358" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J358" t="s">
-        <v>144</v>
+        <v>121</v>
       </c>
       <c r="N358" s="1">
-        <v>46282</v>
-      </c>
-      <c r="O358" t="s">
-        <v>155</v>
+        <v>46288</v>
       </c>
       <c r="P358">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q358">
         <v>2026</v>
       </c>
       <c r="R358">
-        <v>17399363</v>
+        <v>16962338</v>
       </c>
       <c r="S358" t="s">
-        <v>181</v>
+        <v>180</v>
+      </c>
+      <c r="T358" t="s">
+        <v>191</v>
       </c>
       <c r="U358" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="V358" s="1">
-        <v>46282.36440621527</v>
+        <v>46282.54038741898</v>
       </c>
       <c r="W358">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="X358" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="Y358" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="AB358">
         <v>0</v>
       </c>
       <c r="AC358" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AH358" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="AI358" t="s">
         <v>352</v>
@@ -28285,16 +28282,16 @@
     </row>
     <row r="359" spans="1:35">
       <c r="A359">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B359" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C359" t="s">
         <v>50</v>
       </c>
       <c r="D359" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E359" t="s">
         <v>54</v>
@@ -28327,7 +28324,7 @@
         <v>2026</v>
       </c>
       <c r="R359">
-        <v>16962380</v>
+        <v>17399363</v>
       </c>
       <c r="S359" t="s">
         <v>181</v>
@@ -28336,13 +28333,13 @@
         <v>194</v>
       </c>
       <c r="V359" s="1">
-        <v>46282.36462596065</v>
+        <v>46282.36440621527</v>
       </c>
       <c r="W359">
         <v>0</v>
       </c>
       <c r="X359" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="Y359" t="s">
         <v>339</v>
@@ -28362,16 +28359,16 @@
     </row>
     <row r="360" spans="1:35">
       <c r="A360">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B360" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C360" t="s">
         <v>50</v>
       </c>
       <c r="D360" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E360" t="s">
         <v>54</v>
@@ -28404,7 +28401,7 @@
         <v>2026</v>
       </c>
       <c r="R360">
-        <v>16976270</v>
+        <v>16962380</v>
       </c>
       <c r="S360" t="s">
         <v>181</v>
@@ -28413,13 +28410,13 @@
         <v>194</v>
       </c>
       <c r="V360" s="1">
-        <v>46282.36464421296</v>
+        <v>46282.36462596065</v>
       </c>
       <c r="W360">
         <v>0</v>
       </c>
       <c r="X360" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="Y360" t="s">
         <v>339</v>
@@ -28439,10 +28436,10 @@
     </row>
     <row r="361" spans="1:35">
       <c r="A361">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B361" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C361" t="s">
         <v>50</v>
@@ -28481,7 +28478,7 @@
         <v>2026</v>
       </c>
       <c r="R361">
-        <v>17222865</v>
+        <v>16976270</v>
       </c>
       <c r="S361" t="s">
         <v>181</v>
@@ -28490,13 +28487,13 @@
         <v>194</v>
       </c>
       <c r="V361" s="1">
-        <v>46282.36467337963</v>
+        <v>46282.36464421296</v>
       </c>
       <c r="W361">
         <v>0</v>
       </c>
       <c r="X361" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="Y361" t="s">
         <v>339</v>
@@ -28516,10 +28513,10 @@
     </row>
     <row r="362" spans="1:35">
       <c r="A362">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B362" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C362" t="s">
         <v>50</v>
@@ -28528,7 +28525,7 @@
         <v>51</v>
       </c>
       <c r="E362" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F362" t="s">
         <v>56</v>
@@ -28558,7 +28555,7 @@
         <v>2026</v>
       </c>
       <c r="R362">
-        <v>17042587</v>
+        <v>17222865</v>
       </c>
       <c r="S362" t="s">
         <v>181</v>
@@ -28567,13 +28564,13 @@
         <v>194</v>
       </c>
       <c r="V362" s="1">
-        <v>46282.36469679398</v>
+        <v>46282.36467337963</v>
       </c>
       <c r="W362">
         <v>0</v>
       </c>
       <c r="X362" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="Y362" t="s">
         <v>339</v>
@@ -28593,16 +28590,16 @@
     </row>
     <row r="363" spans="1:35">
       <c r="A363">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B363" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C363" t="s">
         <v>50</v>
       </c>
       <c r="D363" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E363" t="s">
         <v>55</v>
@@ -28635,7 +28632,7 @@
         <v>2026</v>
       </c>
       <c r="R363">
-        <v>16960074</v>
+        <v>17042587</v>
       </c>
       <c r="S363" t="s">
         <v>181</v>
@@ -28644,7 +28641,7 @@
         <v>194</v>
       </c>
       <c r="V363" s="1">
-        <v>46282.36469869213</v>
+        <v>46282.36469679398</v>
       </c>
       <c r="W363">
         <v>0</v>
@@ -28670,19 +28667,19 @@
     </row>
     <row r="364" spans="1:35">
       <c r="A364">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B364" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C364" t="s">
         <v>50</v>
       </c>
       <c r="D364" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E364" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F364" t="s">
         <v>56</v>
@@ -28712,7 +28709,7 @@
         <v>2026</v>
       </c>
       <c r="R364">
-        <v>17941217</v>
+        <v>16960074</v>
       </c>
       <c r="S364" t="s">
         <v>181</v>
@@ -28721,13 +28718,13 @@
         <v>194</v>
       </c>
       <c r="V364" s="1">
-        <v>46282.36473159722</v>
+        <v>46282.36469869213</v>
       </c>
       <c r="W364">
         <v>0</v>
       </c>
       <c r="X364" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="Y364" t="s">
         <v>339</v>
@@ -28747,16 +28744,16 @@
     </row>
     <row r="365" spans="1:35">
       <c r="A365">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B365" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C365" t="s">
         <v>50</v>
       </c>
       <c r="D365" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E365" t="s">
         <v>54</v>
@@ -28789,7 +28786,7 @@
         <v>2026</v>
       </c>
       <c r="R365">
-        <v>17952444</v>
+        <v>17941217</v>
       </c>
       <c r="S365" t="s">
         <v>181</v>
@@ -28798,13 +28795,13 @@
         <v>194</v>
       </c>
       <c r="V365" s="1">
-        <v>46282.36473394676</v>
+        <v>46282.36473159722</v>
       </c>
       <c r="W365">
         <v>0</v>
       </c>
       <c r="X365" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="Y365" t="s">
         <v>339</v>
@@ -28824,16 +28821,16 @@
     </row>
     <row r="366" spans="1:35">
       <c r="A366">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B366" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C366" t="s">
         <v>50</v>
       </c>
       <c r="D366" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E366" t="s">
         <v>54</v>
@@ -28866,7 +28863,7 @@
         <v>2026</v>
       </c>
       <c r="R366">
-        <v>17952624</v>
+        <v>17952444</v>
       </c>
       <c r="S366" t="s">
         <v>181</v>
@@ -28875,7 +28872,7 @@
         <v>194</v>
       </c>
       <c r="V366" s="1">
-        <v>46282.36473579861</v>
+        <v>46282.36473394676</v>
       </c>
       <c r="W366">
         <v>0</v>
@@ -28901,10 +28898,10 @@
     </row>
     <row r="367" spans="1:35">
       <c r="A367">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B367" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C367" t="s">
         <v>50</v>
@@ -28943,7 +28940,7 @@
         <v>2026</v>
       </c>
       <c r="R367">
-        <v>18056801</v>
+        <v>17952624</v>
       </c>
       <c r="S367" t="s">
         <v>181</v>
@@ -28952,7 +28949,7 @@
         <v>194</v>
       </c>
       <c r="V367" s="1">
-        <v>46282.36475297454</v>
+        <v>46282.36473579861</v>
       </c>
       <c r="W367">
         <v>0</v>
@@ -28978,10 +28975,10 @@
     </row>
     <row r="368" spans="1:35">
       <c r="A368">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B368" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C368" t="s">
         <v>50</v>
@@ -28993,7 +28990,7 @@
         <v>54</v>
       </c>
       <c r="F368" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G368">
         <v>9086</v>
@@ -29020,7 +29017,7 @@
         <v>2026</v>
       </c>
       <c r="R368">
-        <v>18164551</v>
+        <v>18056801</v>
       </c>
       <c r="S368" t="s">
         <v>181</v>
@@ -29029,13 +29026,13 @@
         <v>194</v>
       </c>
       <c r="V368" s="1">
-        <v>46282.36486408565</v>
+        <v>46282.36475297454</v>
       </c>
       <c r="W368">
         <v>0</v>
       </c>
       <c r="X368" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="Y368" t="s">
         <v>339</v>
@@ -29055,16 +29052,16 @@
     </row>
     <row r="369" spans="1:35">
       <c r="A369">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B369" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C369" t="s">
         <v>50</v>
       </c>
       <c r="D369" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E369" t="s">
         <v>54</v>
@@ -29097,7 +29094,7 @@
         <v>2026</v>
       </c>
       <c r="R369">
-        <v>18178187</v>
+        <v>18164551</v>
       </c>
       <c r="S369" t="s">
         <v>181</v>
@@ -29106,16 +29103,16 @@
         <v>194</v>
       </c>
       <c r="V369" s="1">
-        <v>46282.36487561343</v>
+        <v>46282.36486408565</v>
       </c>
       <c r="W369">
         <v>0</v>
       </c>
       <c r="X369" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="Y369" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="AB369">
         <v>0</v>
@@ -29132,16 +29129,16 @@
     </row>
     <row r="370" spans="1:35">
       <c r="A370">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B370" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C370" t="s">
         <v>50</v>
       </c>
       <c r="D370" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E370" t="s">
         <v>54</v>
@@ -29174,7 +29171,7 @@
         <v>2026</v>
       </c>
       <c r="R370">
-        <v>18188774</v>
+        <v>18178187</v>
       </c>
       <c r="S370" t="s">
         <v>181</v>
@@ -29183,16 +29180,16 @@
         <v>194</v>
       </c>
       <c r="V370" s="1">
-        <v>46282.36486778935</v>
+        <v>46282.36487561343</v>
       </c>
       <c r="W370">
         <v>0</v>
       </c>
       <c r="X370" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="Y370" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AB370">
         <v>0</v>
@@ -29209,10 +29206,10 @@
     </row>
     <row r="371" spans="1:35">
       <c r="A371">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B371" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C371" t="s">
         <v>50</v>
@@ -29251,7 +29248,7 @@
         <v>2026</v>
       </c>
       <c r="R371">
-        <v>18188680</v>
+        <v>18188774</v>
       </c>
       <c r="S371" t="s">
         <v>181</v>
@@ -29260,7 +29257,7 @@
         <v>194</v>
       </c>
       <c r="V371" s="1">
-        <v>46282.36486851852</v>
+        <v>46282.36486778935</v>
       </c>
       <c r="W371">
         <v>0</v>
@@ -29286,40 +29283,40 @@
     </row>
     <row r="372" spans="1:35">
       <c r="A372">
-        <v>5417</v>
+        <v>6963</v>
       </c>
       <c r="B372" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C372" t="s">
         <v>50</v>
       </c>
       <c r="D372" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E372" t="s">
         <v>54</v>
       </c>
       <c r="F372" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G372">
-        <v>9088</v>
+        <v>9086</v>
       </c>
       <c r="H372">
         <v>0</v>
       </c>
       <c r="I372" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J372" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N372" s="1">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="O372" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P372">
         <v>9</v>
@@ -29328,31 +29325,31 @@
         <v>2026</v>
       </c>
       <c r="R372">
-        <v>17399383</v>
+        <v>18188680</v>
       </c>
       <c r="S372" t="s">
-        <v>54</v>
+        <v>181</v>
       </c>
       <c r="U372" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="V372" s="1">
-        <v>46282.3651903588</v>
+        <v>46282.36486851852</v>
       </c>
       <c r="W372">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X372" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="Y372" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="AB372">
         <v>0</v>
       </c>
       <c r="AC372" t="s">
-        <v>54</v>
+        <v>181</v>
       </c>
       <c r="AH372" t="s">
         <v>349</v>
@@ -29363,16 +29360,16 @@
     </row>
     <row r="373" spans="1:35">
       <c r="A373">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B373" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C373" t="s">
         <v>50</v>
       </c>
       <c r="D373" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E373" t="s">
         <v>54</v>
@@ -29405,7 +29402,7 @@
         <v>2026</v>
       </c>
       <c r="R373">
-        <v>16962400</v>
+        <v>17399383</v>
       </c>
       <c r="S373" t="s">
         <v>54</v>
@@ -29414,13 +29411,13 @@
         <v>193</v>
       </c>
       <c r="V373" s="1">
-        <v>46282.36525856482</v>
+        <v>46282.3651903588</v>
       </c>
       <c r="W373">
         <v>-1</v>
       </c>
       <c r="X373" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="Y373" t="s">
         <v>341</v>
@@ -29440,16 +29437,16 @@
     </row>
     <row r="374" spans="1:35">
       <c r="A374">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B374" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C374" t="s">
         <v>50</v>
       </c>
       <c r="D374" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E374" t="s">
         <v>54</v>
@@ -29482,7 +29479,7 @@
         <v>2026</v>
       </c>
       <c r="R374">
-        <v>16976290</v>
+        <v>16962400</v>
       </c>
       <c r="S374" t="s">
         <v>54</v>
@@ -29491,13 +29488,13 @@
         <v>193</v>
       </c>
       <c r="V374" s="1">
-        <v>46282.36526855324</v>
+        <v>46282.36525856482</v>
       </c>
       <c r="W374">
         <v>-1</v>
       </c>
       <c r="X374" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="Y374" t="s">
         <v>341</v>
@@ -29517,10 +29514,10 @@
     </row>
     <row r="375" spans="1:35">
       <c r="A375">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B375" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C375" t="s">
         <v>50</v>
@@ -29559,7 +29556,7 @@
         <v>2026</v>
       </c>
       <c r="R375">
-        <v>17222899</v>
+        <v>16976290</v>
       </c>
       <c r="S375" t="s">
         <v>54</v>
@@ -29568,13 +29565,13 @@
         <v>193</v>
       </c>
       <c r="V375" s="1">
-        <v>46282.36527959491</v>
+        <v>46282.36526855324</v>
       </c>
       <c r="W375">
         <v>-1</v>
       </c>
       <c r="X375" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="Y375" t="s">
         <v>341</v>
@@ -29594,10 +29591,10 @@
     </row>
     <row r="376" spans="1:35">
       <c r="A376">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B376" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C376" t="s">
         <v>50</v>
@@ -29606,7 +29603,7 @@
         <v>51</v>
       </c>
       <c r="E376" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F376" t="s">
         <v>56</v>
@@ -29636,22 +29633,22 @@
         <v>2026</v>
       </c>
       <c r="R376">
-        <v>17042627</v>
+        <v>17222899</v>
       </c>
       <c r="S376" t="s">
-        <v>182</v>
+        <v>54</v>
       </c>
       <c r="U376" t="s">
         <v>193</v>
       </c>
       <c r="V376" s="1">
-        <v>46282.36528526621</v>
+        <v>46282.36527959491</v>
       </c>
       <c r="W376">
         <v>-1</v>
       </c>
       <c r="X376" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="Y376" t="s">
         <v>341</v>
@@ -29660,7 +29657,7 @@
         <v>0</v>
       </c>
       <c r="AC376" t="s">
-        <v>182</v>
+        <v>54</v>
       </c>
       <c r="AH376" t="s">
         <v>349</v>
@@ -29671,16 +29668,16 @@
     </row>
     <row r="377" spans="1:35">
       <c r="A377">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B377" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C377" t="s">
         <v>50</v>
       </c>
       <c r="D377" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E377" t="s">
         <v>55</v>
@@ -29713,16 +29710,16 @@
         <v>2026</v>
       </c>
       <c r="R377">
-        <v>16960098</v>
+        <v>17042627</v>
       </c>
       <c r="S377" t="s">
-        <v>55</v>
+        <v>182</v>
       </c>
       <c r="U377" t="s">
         <v>193</v>
       </c>
       <c r="V377" s="1">
-        <v>46282.36528619213</v>
+        <v>46282.36528526621</v>
       </c>
       <c r="W377">
         <v>-1</v>
@@ -29737,7 +29734,7 @@
         <v>0</v>
       </c>
       <c r="AC377" t="s">
-        <v>55</v>
+        <v>182</v>
       </c>
       <c r="AH377" t="s">
         <v>349</v>
@@ -29748,19 +29745,19 @@
     </row>
     <row r="378" spans="1:35">
       <c r="A378">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B378" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C378" t="s">
         <v>50</v>
       </c>
       <c r="D378" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E378" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F378" t="s">
         <v>56</v>
@@ -29790,22 +29787,22 @@
         <v>2026</v>
       </c>
       <c r="R378">
-        <v>17941237</v>
+        <v>16960098</v>
       </c>
       <c r="S378" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="U378" t="s">
         <v>193</v>
       </c>
       <c r="V378" s="1">
-        <v>46282.36529351852</v>
+        <v>46282.36528619213</v>
       </c>
       <c r="W378">
         <v>-1</v>
       </c>
       <c r="X378" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="Y378" t="s">
         <v>341</v>
@@ -29814,7 +29811,7 @@
         <v>0</v>
       </c>
       <c r="AC378" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="AH378" t="s">
         <v>349</v>
@@ -29825,16 +29822,16 @@
     </row>
     <row r="379" spans="1:35">
       <c r="A379">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B379" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C379" t="s">
         <v>50</v>
       </c>
       <c r="D379" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E379" t="s">
         <v>54</v>
@@ -29867,7 +29864,7 @@
         <v>2026</v>
       </c>
       <c r="R379">
-        <v>17952466</v>
+        <v>17941237</v>
       </c>
       <c r="S379" t="s">
         <v>54</v>
@@ -29876,13 +29873,13 @@
         <v>193</v>
       </c>
       <c r="V379" s="1">
-        <v>46282.36529424768</v>
+        <v>46282.36529351852</v>
       </c>
       <c r="W379">
         <v>-1</v>
       </c>
       <c r="X379" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="Y379" t="s">
         <v>341</v>
@@ -29902,16 +29899,16 @@
     </row>
     <row r="380" spans="1:35">
       <c r="A380">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B380" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C380" t="s">
         <v>50</v>
       </c>
       <c r="D380" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E380" t="s">
         <v>54</v>
@@ -29944,7 +29941,7 @@
         <v>2026</v>
       </c>
       <c r="R380">
-        <v>17952646</v>
+        <v>17952466</v>
       </c>
       <c r="S380" t="s">
         <v>54</v>
@@ -29953,7 +29950,7 @@
         <v>193</v>
       </c>
       <c r="V380" s="1">
-        <v>46282.36529490741</v>
+        <v>46282.36529424768</v>
       </c>
       <c r="W380">
         <v>-1</v>
@@ -29979,10 +29976,10 @@
     </row>
     <row r="381" spans="1:35">
       <c r="A381">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B381" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C381" t="s">
         <v>50</v>
@@ -30021,16 +30018,16 @@
         <v>2026</v>
       </c>
       <c r="R381">
-        <v>18056821</v>
+        <v>17952646</v>
       </c>
       <c r="S381" t="s">
-        <v>182</v>
+        <v>54</v>
       </c>
       <c r="U381" t="s">
         <v>193</v>
       </c>
       <c r="V381" s="1">
-        <v>46282.36529869213</v>
+        <v>46282.36529490741</v>
       </c>
       <c r="W381">
         <v>-1</v>
@@ -30045,7 +30042,7 @@
         <v>0</v>
       </c>
       <c r="AC381" t="s">
-        <v>182</v>
+        <v>54</v>
       </c>
       <c r="AH381" t="s">
         <v>349</v>
@@ -30056,10 +30053,10 @@
     </row>
     <row r="382" spans="1:35">
       <c r="A382">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B382" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C382" t="s">
         <v>50</v>
@@ -30071,7 +30068,7 @@
         <v>54</v>
       </c>
       <c r="F382" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G382">
         <v>9088</v>
@@ -30098,22 +30095,22 @@
         <v>2026</v>
       </c>
       <c r="R382">
-        <v>18164565</v>
+        <v>18056821</v>
       </c>
       <c r="S382" t="s">
-        <v>54</v>
+        <v>182</v>
       </c>
       <c r="U382" t="s">
         <v>193</v>
       </c>
       <c r="V382" s="1">
-        <v>46282.36531149306</v>
+        <v>46282.36529869213</v>
       </c>
       <c r="W382">
         <v>-1</v>
       </c>
       <c r="X382" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="Y382" t="s">
         <v>341</v>
@@ -30122,7 +30119,7 @@
         <v>0</v>
       </c>
       <c r="AC382" t="s">
-        <v>54</v>
+        <v>182</v>
       </c>
       <c r="AH382" t="s">
         <v>349</v>
@@ -30133,16 +30130,16 @@
     </row>
     <row r="383" spans="1:35">
       <c r="A383">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B383" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C383" t="s">
         <v>50</v>
       </c>
       <c r="D383" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E383" t="s">
         <v>54</v>
@@ -30175,31 +30172,31 @@
         <v>2026</v>
       </c>
       <c r="R383">
-        <v>18178199</v>
+        <v>18164565</v>
       </c>
       <c r="S383" t="s">
-        <v>182</v>
+        <v>54</v>
       </c>
       <c r="U383" t="s">
         <v>193</v>
       </c>
       <c r="V383" s="1">
-        <v>46282.36531554398</v>
+        <v>46282.36531149306</v>
       </c>
       <c r="W383">
         <v>-1</v>
       </c>
       <c r="X383" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="Y383" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AB383">
         <v>0</v>
       </c>
       <c r="AC383" t="s">
-        <v>182</v>
+        <v>54</v>
       </c>
       <c r="AH383" t="s">
         <v>349</v>
@@ -30210,16 +30207,16 @@
     </row>
     <row r="384" spans="1:35">
       <c r="A384">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B384" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C384" t="s">
         <v>50</v>
       </c>
       <c r="D384" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E384" t="s">
         <v>54</v>
@@ -30252,31 +30249,31 @@
         <v>2026</v>
       </c>
       <c r="R384">
-        <v>18188788</v>
+        <v>18178199</v>
       </c>
       <c r="S384" t="s">
-        <v>54</v>
+        <v>182</v>
       </c>
       <c r="U384" t="s">
         <v>193</v>
       </c>
       <c r="V384" s="1">
-        <v>46282.36531253472</v>
+        <v>46282.36531554398</v>
       </c>
       <c r="W384">
         <v>-1</v>
       </c>
       <c r="X384" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="Y384" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AB384">
         <v>0</v>
       </c>
       <c r="AC384" t="s">
-        <v>54</v>
+        <v>182</v>
       </c>
       <c r="AH384" t="s">
         <v>349</v>
@@ -30287,10 +30284,10 @@
     </row>
     <row r="385" spans="1:35">
       <c r="A385">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B385" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C385" t="s">
         <v>50</v>
@@ -30329,7 +30326,7 @@
         <v>2026</v>
       </c>
       <c r="R385">
-        <v>18188694</v>
+        <v>18188788</v>
       </c>
       <c r="S385" t="s">
         <v>54</v>
@@ -30338,7 +30335,7 @@
         <v>193</v>
       </c>
       <c r="V385" s="1">
-        <v>46282.36531288194</v>
+        <v>46282.36531253472</v>
       </c>
       <c r="W385">
         <v>-1</v>
@@ -30359,6 +30356,83 @@
         <v>349</v>
       </c>
       <c r="AI385" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="386" spans="1:35">
+      <c r="A386">
+        <v>6963</v>
+      </c>
+      <c r="B386" t="s">
+        <v>41</v>
+      </c>
+      <c r="C386" t="s">
+        <v>50</v>
+      </c>
+      <c r="D386" t="s">
+        <v>53</v>
+      </c>
+      <c r="E386" t="s">
+        <v>54</v>
+      </c>
+      <c r="F386" t="s">
+        <v>57</v>
+      </c>
+      <c r="G386">
+        <v>9088</v>
+      </c>
+      <c r="H386">
+        <v>0</v>
+      </c>
+      <c r="I386" t="s">
+        <v>65</v>
+      </c>
+      <c r="J386" t="s">
+        <v>145</v>
+      </c>
+      <c r="N386" s="1">
+        <v>46283</v>
+      </c>
+      <c r="O386" t="s">
+        <v>154</v>
+      </c>
+      <c r="P386">
+        <v>9</v>
+      </c>
+      <c r="Q386">
+        <v>2026</v>
+      </c>
+      <c r="R386">
+        <v>18188694</v>
+      </c>
+      <c r="S386" t="s">
+        <v>54</v>
+      </c>
+      <c r="U386" t="s">
+        <v>193</v>
+      </c>
+      <c r="V386" s="1">
+        <v>46282.36531288194</v>
+      </c>
+      <c r="W386">
+        <v>-1</v>
+      </c>
+      <c r="X386" t="s">
+        <v>199</v>
+      </c>
+      <c r="Y386" t="s">
+        <v>341</v>
+      </c>
+      <c r="AB386">
+        <v>0</v>
+      </c>
+      <c r="AC386" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH386" t="s">
+        <v>349</v>
+      </c>
+      <c r="AI386" t="s">
         <v>352</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-18 11:13
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6008" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6022" uniqueCount="364">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1468,7 +1468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI416"/>
+  <dimension ref="A1:AI417"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -27644,31 +27644,31 @@
     </row>
     <row r="350" spans="1:35">
       <c r="A350">
-        <v>6703</v>
+        <v>6949</v>
       </c>
       <c r="B350" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C350" t="s">
         <v>50</v>
       </c>
       <c r="D350" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E350" t="s">
         <v>54</v>
       </c>
       <c r="F350" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G350">
-        <v>1628</v>
+        <v>1697</v>
       </c>
       <c r="H350">
-        <v>1581</v>
+        <v>1650</v>
       </c>
       <c r="I350" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J350" t="s">
         <v>75</v>
@@ -27683,31 +27683,31 @@
         <v>2026</v>
       </c>
       <c r="R350">
-        <v>17955176</v>
+        <v>18178280</v>
       </c>
       <c r="S350" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="T350" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="U350" t="s">
         <v>198</v>
       </c>
       <c r="V350" s="1">
-        <v>46282.42251184028</v>
+        <v>46283.44840582176</v>
       </c>
       <c r="W350">
         <v>-3</v>
       </c>
       <c r="X350" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="AB350">
         <v>0</v>
       </c>
       <c r="AC350" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="AH350" t="s">
         <v>358</v>
@@ -27718,16 +27718,16 @@
     </row>
     <row r="351" spans="1:35">
       <c r="A351">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B351" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C351" t="s">
         <v>50</v>
       </c>
       <c r="D351" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E351" t="s">
         <v>54</v>
@@ -27736,49 +27736,52 @@
         <v>56</v>
       </c>
       <c r="G351">
-        <v>5883</v>
+        <v>1628</v>
       </c>
       <c r="H351">
-        <v>5792</v>
+        <v>1581</v>
       </c>
       <c r="I351" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J351" t="s">
-        <v>125</v>
+        <v>75</v>
       </c>
       <c r="N351" s="1">
         <v>46286</v>
       </c>
       <c r="P351">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q351">
         <v>2026</v>
       </c>
       <c r="R351">
-        <v>17399067</v>
+        <v>17955176</v>
       </c>
       <c r="S351" t="s">
-        <v>176</v>
+        <v>170</v>
+      </c>
+      <c r="T351" t="s">
+        <v>191</v>
       </c>
       <c r="U351" t="s">
         <v>198</v>
       </c>
       <c r="V351" s="1">
-        <v>46282.47420876157</v>
+        <v>46282.42251184028</v>
       </c>
       <c r="W351">
         <v>-3</v>
       </c>
       <c r="X351" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="AB351">
         <v>0</v>
       </c>
       <c r="AC351" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="AH351" t="s">
         <v>358</v>
@@ -27807,7 +27810,7 @@
         <v>56</v>
       </c>
       <c r="G352">
-        <v>5884</v>
+        <v>5883</v>
       </c>
       <c r="H352">
         <v>5792</v>
@@ -27816,7 +27819,7 @@
         <v>61</v>
       </c>
       <c r="J352" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N352" s="1">
         <v>46286</v>
@@ -27828,7 +27831,7 @@
         <v>2026</v>
       </c>
       <c r="R352">
-        <v>17399077</v>
+        <v>17399067</v>
       </c>
       <c r="S352" t="s">
         <v>176</v>
@@ -27837,7 +27840,7 @@
         <v>198</v>
       </c>
       <c r="V352" s="1">
-        <v>46282.47437324074</v>
+        <v>46282.47420876157</v>
       </c>
       <c r="W352">
         <v>-3</v>
@@ -27860,16 +27863,16 @@
     </row>
     <row r="353" spans="1:35">
       <c r="A353">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B353" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C353" t="s">
         <v>50</v>
       </c>
       <c r="D353" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E353" t="s">
         <v>54</v>
@@ -27878,23 +27881,20 @@
         <v>56</v>
       </c>
       <c r="G353">
-        <v>5903</v>
+        <v>5884</v>
       </c>
       <c r="H353">
-        <v>5830</v>
+        <v>5792</v>
       </c>
       <c r="I353" t="s">
         <v>61</v>
       </c>
       <c r="J353" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="N353" s="1">
         <v>46286</v>
       </c>
-      <c r="O353" t="s">
-        <v>159</v>
-      </c>
       <c r="P353">
         <v>9</v>
       </c>
@@ -27902,34 +27902,28 @@
         <v>2026</v>
       </c>
       <c r="R353">
-        <v>16962221</v>
+        <v>17399077</v>
       </c>
       <c r="S353" t="s">
-        <v>177</v>
-      </c>
-      <c r="T353" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="U353" t="s">
         <v>198</v>
       </c>
       <c r="V353" s="1">
-        <v>46282.42048836806</v>
+        <v>46282.47437324074</v>
       </c>
       <c r="W353">
         <v>-3</v>
       </c>
       <c r="X353" t="s">
-        <v>210</v>
-      </c>
-      <c r="Y353" t="s">
-        <v>339</v>
+        <v>206</v>
       </c>
       <c r="AB353">
         <v>0</v>
       </c>
       <c r="AC353" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AH353" t="s">
         <v>358</v>
@@ -27958,20 +27952,23 @@
         <v>56</v>
       </c>
       <c r="G354">
+        <v>5903</v>
+      </c>
+      <c r="H354">
         <v>5830</v>
-      </c>
-      <c r="H354">
-        <v>5784</v>
       </c>
       <c r="I354" t="s">
         <v>61</v>
       </c>
       <c r="J354" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N354" s="1">
         <v>46286</v>
       </c>
+      <c r="O354" t="s">
+        <v>159</v>
+      </c>
       <c r="P354">
         <v>9</v>
       </c>
@@ -27979,7 +27976,7 @@
         <v>2026</v>
       </c>
       <c r="R354">
-        <v>16962211</v>
+        <v>16962221</v>
       </c>
       <c r="S354" t="s">
         <v>177</v>
@@ -27991,7 +27988,7 @@
         <v>198</v>
       </c>
       <c r="V354" s="1">
-        <v>46282.42138976852</v>
+        <v>46282.42048836806</v>
       </c>
       <c r="W354">
         <v>-3</v>
@@ -27999,6 +27996,9 @@
       <c r="X354" t="s">
         <v>210</v>
       </c>
+      <c r="Y354" t="s">
+        <v>339</v>
+      </c>
       <c r="AB354">
         <v>0</v>
       </c>
@@ -28014,16 +28014,16 @@
     </row>
     <row r="355" spans="1:35">
       <c r="A355">
-        <v>6548</v>
+        <v>6404</v>
       </c>
       <c r="B355" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="C355" t="s">
         <v>50</v>
       </c>
       <c r="D355" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E355" t="s">
         <v>54</v>
@@ -28032,52 +28032,52 @@
         <v>56</v>
       </c>
       <c r="G355">
-        <v>1913</v>
+        <v>5830</v>
       </c>
       <c r="H355">
-        <v>1862</v>
+        <v>5784</v>
       </c>
       <c r="I355" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J355" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="N355" s="1">
         <v>46286</v>
       </c>
       <c r="P355">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q355">
         <v>2026</v>
       </c>
       <c r="R355">
-        <v>17988579</v>
+        <v>16962211</v>
       </c>
       <c r="S355" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="T355" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="U355" t="s">
         <v>198</v>
       </c>
       <c r="V355" s="1">
-        <v>46283.3939177662</v>
+        <v>46282.42138976852</v>
       </c>
       <c r="W355">
         <v>-3</v>
       </c>
       <c r="X355" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="AB355">
         <v>0</v>
       </c>
       <c r="AC355" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="AH355" t="s">
         <v>358</v>
@@ -28088,37 +28088,37 @@
     </row>
     <row r="356" spans="1:35">
       <c r="A356">
-        <v>6628</v>
+        <v>6548</v>
       </c>
       <c r="B356" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C356" t="s">
         <v>50</v>
       </c>
       <c r="D356" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E356" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F356" t="s">
         <v>56</v>
       </c>
       <c r="G356">
-        <v>1879</v>
+        <v>1913</v>
       </c>
       <c r="H356">
-        <v>0</v>
+        <v>1862</v>
       </c>
       <c r="I356" t="s">
         <v>62</v>
       </c>
       <c r="J356" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N356" s="1">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="P356">
         <v>8</v>
@@ -28127,37 +28127,34 @@
         <v>2026</v>
       </c>
       <c r="R356">
-        <v>17988684</v>
+        <v>17988579</v>
       </c>
       <c r="S356" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="T356" t="s">
         <v>195</v>
       </c>
       <c r="U356" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="V356" s="1">
-        <v>46283.41459880787</v>
+        <v>46283.3939177662</v>
       </c>
       <c r="W356">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="X356" t="s">
-        <v>201</v>
-      </c>
-      <c r="Y356" t="s">
-        <v>340</v>
+        <v>200</v>
       </c>
       <c r="AB356">
         <v>0</v>
       </c>
       <c r="AC356" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="AH356" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="AI356" t="s">
         <v>363</v>
@@ -28165,25 +28162,25 @@
     </row>
     <row r="357" spans="1:35">
       <c r="A357">
-        <v>6548</v>
+        <v>6628</v>
       </c>
       <c r="B357" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C357" t="s">
         <v>50</v>
       </c>
       <c r="D357" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E357" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F357" t="s">
         <v>56</v>
       </c>
       <c r="G357">
-        <v>7026</v>
+        <v>1879</v>
       </c>
       <c r="H357">
         <v>0</v>
@@ -28192,10 +28189,10 @@
         <v>62</v>
       </c>
       <c r="J357" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="N357" s="1">
-        <v>46288</v>
+        <v>46283</v>
       </c>
       <c r="P357">
         <v>8</v>
@@ -28204,37 +28201,37 @@
         <v>2026</v>
       </c>
       <c r="R357">
-        <v>18094899</v>
+        <v>17988684</v>
       </c>
       <c r="S357" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="T357" t="s">
         <v>195</v>
       </c>
       <c r="U357" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="V357" s="1">
-        <v>46282.74573174769</v>
+        <v>46283.41459880787</v>
       </c>
       <c r="W357">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="X357" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="Y357" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="AB357">
         <v>0</v>
       </c>
       <c r="AC357" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="AH357" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="AI357" t="s">
         <v>363</v>
@@ -28242,10 +28239,10 @@
     </row>
     <row r="358" spans="1:35">
       <c r="A358">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B358" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C358" t="s">
         <v>50</v>
@@ -28254,7 +28251,7 @@
         <v>51</v>
       </c>
       <c r="E358" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F358" t="s">
         <v>56</v>
@@ -28281,31 +28278,34 @@
         <v>2026</v>
       </c>
       <c r="R358">
-        <v>18048473</v>
+        <v>18094899</v>
       </c>
       <c r="S358" t="s">
-        <v>181</v>
+        <v>180</v>
+      </c>
+      <c r="T358" t="s">
+        <v>195</v>
       </c>
       <c r="U358" t="s">
         <v>198</v>
       </c>
       <c r="V358" s="1">
-        <v>46282.74485532408</v>
+        <v>46282.74573174769</v>
       </c>
       <c r="W358">
         <v>-5</v>
       </c>
       <c r="X358" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Y358" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AB358">
         <v>0</v>
       </c>
       <c r="AC358" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AH358" t="s">
         <v>358</v>
@@ -28316,10 +28316,10 @@
     </row>
     <row r="359" spans="1:35">
       <c r="A359">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B359" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C359" t="s">
         <v>50</v>
@@ -28328,25 +28328,25 @@
         <v>51</v>
       </c>
       <c r="E359" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F359" t="s">
         <v>56</v>
       </c>
       <c r="G359">
-        <v>1914</v>
+        <v>7026</v>
       </c>
       <c r="H359">
-        <v>1862</v>
+        <v>0</v>
       </c>
       <c r="I359" t="s">
         <v>62</v>
       </c>
       <c r="J359" t="s">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="N359" s="1">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="P359">
         <v>8</v>
@@ -28355,31 +28355,31 @@
         <v>2026</v>
       </c>
       <c r="R359">
-        <v>17988591</v>
+        <v>18048473</v>
       </c>
       <c r="S359" t="s">
-        <v>180</v>
-      </c>
-      <c r="T359" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="U359" t="s">
         <v>198</v>
       </c>
       <c r="V359" s="1">
-        <v>46283.39413969908</v>
+        <v>46282.74485532408</v>
       </c>
       <c r="W359">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="X359" t="s">
-        <v>200</v>
+        <v>201</v>
+      </c>
+      <c r="Y359" t="s">
+        <v>342</v>
       </c>
       <c r="AB359">
         <v>0</v>
       </c>
       <c r="AC359" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AH359" t="s">
         <v>358</v>
@@ -28390,10 +28390,10 @@
     </row>
     <row r="360" spans="1:35">
       <c r="A360">
-        <v>6704</v>
+        <v>6548</v>
       </c>
       <c r="B360" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C360" t="s">
         <v>50</v>
@@ -28408,22 +28408,19 @@
         <v>56</v>
       </c>
       <c r="G360">
-        <v>11874</v>
+        <v>1914</v>
       </c>
       <c r="H360">
-        <v>0</v>
+        <v>1862</v>
       </c>
       <c r="I360" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J360" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="N360" s="1">
-        <v>46281</v>
-      </c>
-      <c r="O360" t="s">
-        <v>160</v>
+        <v>46286</v>
       </c>
       <c r="P360">
         <v>8</v>
@@ -28432,37 +28429,34 @@
         <v>2026</v>
       </c>
       <c r="R360">
-        <v>18273589</v>
+        <v>17988591</v>
       </c>
       <c r="S360" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="T360" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="U360" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="V360" s="1">
-        <v>46282.70138376157</v>
+        <v>46283.39413969908</v>
       </c>
       <c r="W360">
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="X360" t="s">
-        <v>205</v>
-      </c>
-      <c r="Y360" t="s">
-        <v>343</v>
+        <v>200</v>
       </c>
       <c r="AB360">
         <v>0</v>
       </c>
       <c r="AC360" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="AH360" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="AI360" t="s">
         <v>363</v>
@@ -28470,16 +28464,16 @@
     </row>
     <row r="361" spans="1:35">
       <c r="A361">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B361" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C361" t="s">
         <v>50</v>
       </c>
       <c r="D361" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E361" t="s">
         <v>54</v>
@@ -28512,7 +28506,7 @@
         <v>2026</v>
       </c>
       <c r="R361">
-        <v>18239293</v>
+        <v>18273589</v>
       </c>
       <c r="S361" t="s">
         <v>185</v>
@@ -28524,7 +28518,7 @@
         <v>197</v>
       </c>
       <c r="V361" s="1">
-        <v>46282.7013840625</v>
+        <v>46282.70138376157</v>
       </c>
       <c r="W361">
         <v>2</v>
@@ -28568,7 +28562,7 @@
         <v>56</v>
       </c>
       <c r="G362">
-        <v>1805</v>
+        <v>11874</v>
       </c>
       <c r="H362">
         <v>0</v>
@@ -28577,10 +28571,13 @@
         <v>63</v>
       </c>
       <c r="J362" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="N362" s="1">
-        <v>46283</v>
+        <v>46281</v>
+      </c>
+      <c r="O362" t="s">
+        <v>160</v>
       </c>
       <c r="P362">
         <v>8</v>
@@ -28589,7 +28586,7 @@
         <v>2026</v>
       </c>
       <c r="R362">
-        <v>17948948</v>
+        <v>18239293</v>
       </c>
       <c r="S362" t="s">
         <v>185</v>
@@ -28598,19 +28595,19 @@
         <v>196</v>
       </c>
       <c r="U362" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="V362" s="1">
-        <v>46283.35452896991</v>
+        <v>46282.7013840625</v>
       </c>
       <c r="W362">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X362" t="s">
         <v>205</v>
       </c>
       <c r="Y362" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="AB362">
         <v>0</v>
@@ -28627,10 +28624,10 @@
     </row>
     <row r="363" spans="1:35">
       <c r="A363">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B363" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C363" t="s">
         <v>50</v>
@@ -28666,7 +28663,7 @@
         <v>2026</v>
       </c>
       <c r="R363">
-        <v>18084966</v>
+        <v>17948948</v>
       </c>
       <c r="S363" t="s">
         <v>185</v>
@@ -28678,7 +28675,7 @@
         <v>199</v>
       </c>
       <c r="V363" s="1">
-        <v>46283.35453171296</v>
+        <v>46283.35452896991</v>
       </c>
       <c r="W363">
         <v>0</v>
@@ -28704,16 +28701,16 @@
     </row>
     <row r="364" spans="1:35">
       <c r="A364">
-        <v>5417</v>
+        <v>6779</v>
       </c>
       <c r="B364" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C364" t="s">
         <v>50</v>
       </c>
       <c r="D364" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E364" t="s">
         <v>54</v>
@@ -28722,7 +28719,7 @@
         <v>56</v>
       </c>
       <c r="G364">
-        <v>7025</v>
+        <v>1805</v>
       </c>
       <c r="H364">
         <v>0</v>
@@ -28731,10 +28728,10 @@
         <v>63</v>
       </c>
       <c r="J364" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="N364" s="1">
-        <v>46288</v>
+        <v>46283</v>
       </c>
       <c r="P364">
         <v>8</v>
@@ -28743,7 +28740,7 @@
         <v>2026</v>
       </c>
       <c r="R364">
-        <v>17399280</v>
+        <v>18084966</v>
       </c>
       <c r="S364" t="s">
         <v>185</v>
@@ -28752,19 +28749,19 @@
         <v>196</v>
       </c>
       <c r="U364" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="V364" s="1">
-        <v>46283.38367943287</v>
+        <v>46283.35453171296</v>
       </c>
       <c r="W364">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="X364" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Y364" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="AB364">
         <v>0</v>
@@ -28773,7 +28770,7 @@
         <v>185</v>
       </c>
       <c r="AH364" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="AI364" t="s">
         <v>363</v>
@@ -28781,16 +28778,16 @@
     </row>
     <row r="365" spans="1:35">
       <c r="A365">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B365" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C365" t="s">
         <v>50</v>
       </c>
       <c r="D365" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E365" t="s">
         <v>54</v>
@@ -28820,7 +28817,7 @@
         <v>2026</v>
       </c>
       <c r="R365">
-        <v>16962338</v>
+        <v>17399280</v>
       </c>
       <c r="S365" t="s">
         <v>185</v>
@@ -28832,16 +28829,16 @@
         <v>198</v>
       </c>
       <c r="V365" s="1">
-        <v>46282.54038741898</v>
+        <v>46283.38367943287</v>
       </c>
       <c r="W365">
         <v>-5</v>
       </c>
       <c r="X365" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="Y365" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="AB365">
         <v>0</v>
@@ -28858,16 +28855,16 @@
     </row>
     <row r="366" spans="1:35">
       <c r="A366">
-        <v>6705</v>
+        <v>6404</v>
       </c>
       <c r="B366" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C366" t="s">
         <v>50</v>
       </c>
       <c r="D366" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E366" t="s">
         <v>54</v>
@@ -28876,22 +28873,19 @@
         <v>56</v>
       </c>
       <c r="G366">
-        <v>7022</v>
+        <v>7025</v>
       </c>
       <c r="H366">
         <v>0</v>
       </c>
       <c r="I366" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J366" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="N366" s="1">
-        <v>46283</v>
-      </c>
-      <c r="O366" t="s">
-        <v>159</v>
+        <v>46288</v>
       </c>
       <c r="P366">
         <v>8</v>
@@ -28900,34 +28894,37 @@
         <v>2026</v>
       </c>
       <c r="R366">
-        <v>17952601</v>
+        <v>16962338</v>
       </c>
       <c r="S366" t="s">
-        <v>186</v>
+        <v>185</v>
+      </c>
+      <c r="T366" t="s">
+        <v>196</v>
       </c>
       <c r="U366" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="V366" s="1">
-        <v>46283.38329579861</v>
+        <v>46282.54038741898</v>
       </c>
       <c r="W366">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="X366" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="Y366" t="s">
-        <v>317</v>
+        <v>346</v>
       </c>
       <c r="AB366">
         <v>0</v>
       </c>
       <c r="AC366" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AH366" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="AI366" t="s">
         <v>363</v>
@@ -28935,16 +28932,16 @@
     </row>
     <row r="367" spans="1:35">
       <c r="A367">
-        <v>5417</v>
+        <v>6705</v>
       </c>
       <c r="B367" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C367" t="s">
         <v>50</v>
       </c>
       <c r="D367" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E367" t="s">
         <v>54</v>
@@ -28953,7 +28950,7 @@
         <v>56</v>
       </c>
       <c r="G367">
-        <v>9086</v>
+        <v>7022</v>
       </c>
       <c r="H367">
         <v>0</v>
@@ -28962,22 +28959,22 @@
         <v>64</v>
       </c>
       <c r="J367" t="s">
-        <v>147</v>
+        <v>115</v>
       </c>
       <c r="N367" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="O367" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="P367">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q367">
         <v>2026</v>
       </c>
       <c r="R367">
-        <v>17399363</v>
+        <v>17952601</v>
       </c>
       <c r="S367" t="s">
         <v>186</v>
@@ -28986,16 +28983,16 @@
         <v>199</v>
       </c>
       <c r="V367" s="1">
-        <v>46282.36440621527</v>
+        <v>46283.38329579861</v>
       </c>
       <c r="W367">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X367" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Y367" t="s">
-        <v>347</v>
+        <v>317</v>
       </c>
       <c r="AB367">
         <v>0</v>
@@ -29004,7 +29001,7 @@
         <v>186</v>
       </c>
       <c r="AH367" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="AI367" t="s">
         <v>363</v>
@@ -29012,16 +29009,16 @@
     </row>
     <row r="368" spans="1:35">
       <c r="A368">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B368" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C368" t="s">
         <v>50</v>
       </c>
       <c r="D368" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E368" t="s">
         <v>54</v>
@@ -29054,7 +29051,7 @@
         <v>2026</v>
       </c>
       <c r="R368">
-        <v>16962380</v>
+        <v>17399363</v>
       </c>
       <c r="S368" t="s">
         <v>186</v>
@@ -29063,13 +29060,13 @@
         <v>199</v>
       </c>
       <c r="V368" s="1">
-        <v>46282.36462596065</v>
+        <v>46282.36440621527</v>
       </c>
       <c r="W368">
         <v>1</v>
       </c>
       <c r="X368" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="Y368" t="s">
         <v>347</v>
@@ -29089,16 +29086,16 @@
     </row>
     <row r="369" spans="1:35">
       <c r="A369">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B369" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C369" t="s">
         <v>50</v>
       </c>
       <c r="D369" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E369" t="s">
         <v>54</v>
@@ -29131,7 +29128,7 @@
         <v>2026</v>
       </c>
       <c r="R369">
-        <v>16976270</v>
+        <v>16962380</v>
       </c>
       <c r="S369" t="s">
         <v>186</v>
@@ -29140,13 +29137,13 @@
         <v>199</v>
       </c>
       <c r="V369" s="1">
-        <v>46282.36464421296</v>
+        <v>46282.36462596065</v>
       </c>
       <c r="W369">
         <v>1</v>
       </c>
       <c r="X369" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="Y369" t="s">
         <v>347</v>
@@ -29166,10 +29163,10 @@
     </row>
     <row r="370" spans="1:35">
       <c r="A370">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B370" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C370" t="s">
         <v>50</v>
@@ -29208,7 +29205,7 @@
         <v>2026</v>
       </c>
       <c r="R370">
-        <v>17222865</v>
+        <v>16976270</v>
       </c>
       <c r="S370" t="s">
         <v>186</v>
@@ -29217,13 +29214,13 @@
         <v>199</v>
       </c>
       <c r="V370" s="1">
-        <v>46282.36467337963</v>
+        <v>46282.36464421296</v>
       </c>
       <c r="W370">
         <v>1</v>
       </c>
       <c r="X370" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="Y370" t="s">
         <v>347</v>
@@ -29243,10 +29240,10 @@
     </row>
     <row r="371" spans="1:35">
       <c r="A371">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B371" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C371" t="s">
         <v>50</v>
@@ -29255,7 +29252,7 @@
         <v>51</v>
       </c>
       <c r="E371" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F371" t="s">
         <v>56</v>
@@ -29285,7 +29282,7 @@
         <v>2026</v>
       </c>
       <c r="R371">
-        <v>17042587</v>
+        <v>17222865</v>
       </c>
       <c r="S371" t="s">
         <v>186</v>
@@ -29294,13 +29291,13 @@
         <v>199</v>
       </c>
       <c r="V371" s="1">
-        <v>46282.36469679398</v>
+        <v>46282.36467337963</v>
       </c>
       <c r="W371">
         <v>1</v>
       </c>
       <c r="X371" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Y371" t="s">
         <v>347</v>
@@ -29320,16 +29317,16 @@
     </row>
     <row r="372" spans="1:35">
       <c r="A372">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B372" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C372" t="s">
         <v>50</v>
       </c>
       <c r="D372" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E372" t="s">
         <v>55</v>
@@ -29362,7 +29359,7 @@
         <v>2026</v>
       </c>
       <c r="R372">
-        <v>16960074</v>
+        <v>17042587</v>
       </c>
       <c r="S372" t="s">
         <v>186</v>
@@ -29371,7 +29368,7 @@
         <v>199</v>
       </c>
       <c r="V372" s="1">
-        <v>46282.36469869213</v>
+        <v>46282.36469679398</v>
       </c>
       <c r="W372">
         <v>1</v>
@@ -29397,19 +29394,19 @@
     </row>
     <row r="373" spans="1:35">
       <c r="A373">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B373" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C373" t="s">
         <v>50</v>
       </c>
       <c r="D373" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E373" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F373" t="s">
         <v>56</v>
@@ -29439,7 +29436,7 @@
         <v>2026</v>
       </c>
       <c r="R373">
-        <v>17941217</v>
+        <v>16960074</v>
       </c>
       <c r="S373" t="s">
         <v>186</v>
@@ -29448,13 +29445,13 @@
         <v>199</v>
       </c>
       <c r="V373" s="1">
-        <v>46282.36473159722</v>
+        <v>46282.36469869213</v>
       </c>
       <c r="W373">
         <v>1</v>
       </c>
       <c r="X373" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="Y373" t="s">
         <v>347</v>
@@ -29474,16 +29471,16 @@
     </row>
     <row r="374" spans="1:35">
       <c r="A374">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B374" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C374" t="s">
         <v>50</v>
       </c>
       <c r="D374" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E374" t="s">
         <v>54</v>
@@ -29516,7 +29513,7 @@
         <v>2026</v>
       </c>
       <c r="R374">
-        <v>17952444</v>
+        <v>17941217</v>
       </c>
       <c r="S374" t="s">
         <v>186</v>
@@ -29525,13 +29522,13 @@
         <v>199</v>
       </c>
       <c r="V374" s="1">
-        <v>46282.36473394676</v>
+        <v>46282.36473159722</v>
       </c>
       <c r="W374">
         <v>1</v>
       </c>
       <c r="X374" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="Y374" t="s">
         <v>347</v>
@@ -29551,16 +29548,16 @@
     </row>
     <row r="375" spans="1:35">
       <c r="A375">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B375" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C375" t="s">
         <v>50</v>
       </c>
       <c r="D375" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E375" t="s">
         <v>54</v>
@@ -29593,7 +29590,7 @@
         <v>2026</v>
       </c>
       <c r="R375">
-        <v>17952624</v>
+        <v>17952444</v>
       </c>
       <c r="S375" t="s">
         <v>186</v>
@@ -29602,7 +29599,7 @@
         <v>199</v>
       </c>
       <c r="V375" s="1">
-        <v>46282.36473579861</v>
+        <v>46282.36473394676</v>
       </c>
       <c r="W375">
         <v>1</v>
@@ -29628,10 +29625,10 @@
     </row>
     <row r="376" spans="1:35">
       <c r="A376">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B376" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C376" t="s">
         <v>50</v>
@@ -29670,7 +29667,7 @@
         <v>2026</v>
       </c>
       <c r="R376">
-        <v>18056801</v>
+        <v>17952624</v>
       </c>
       <c r="S376" t="s">
         <v>186</v>
@@ -29679,7 +29676,7 @@
         <v>199</v>
       </c>
       <c r="V376" s="1">
-        <v>46282.36475297454</v>
+        <v>46282.36473579861</v>
       </c>
       <c r="W376">
         <v>1</v>
@@ -29705,10 +29702,10 @@
     </row>
     <row r="377" spans="1:35">
       <c r="A377">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B377" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C377" t="s">
         <v>50</v>
@@ -29720,7 +29717,7 @@
         <v>54</v>
       </c>
       <c r="F377" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G377">
         <v>9086</v>
@@ -29747,7 +29744,7 @@
         <v>2026</v>
       </c>
       <c r="R377">
-        <v>18164551</v>
+        <v>18056801</v>
       </c>
       <c r="S377" t="s">
         <v>186</v>
@@ -29756,13 +29753,13 @@
         <v>199</v>
       </c>
       <c r="V377" s="1">
-        <v>46282.36486408565</v>
+        <v>46282.36475297454</v>
       </c>
       <c r="W377">
         <v>1</v>
       </c>
       <c r="X377" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="Y377" t="s">
         <v>347</v>
@@ -29782,16 +29779,16 @@
     </row>
     <row r="378" spans="1:35">
       <c r="A378">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B378" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C378" t="s">
         <v>50</v>
       </c>
       <c r="D378" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E378" t="s">
         <v>54</v>
@@ -29824,7 +29821,7 @@
         <v>2026</v>
       </c>
       <c r="R378">
-        <v>18178187</v>
+        <v>18164551</v>
       </c>
       <c r="S378" t="s">
         <v>186</v>
@@ -29833,16 +29830,16 @@
         <v>199</v>
       </c>
       <c r="V378" s="1">
-        <v>46282.36487561343</v>
+        <v>46282.36486408565</v>
       </c>
       <c r="W378">
         <v>1</v>
       </c>
       <c r="X378" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Y378" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="AB378">
         <v>0</v>
@@ -29859,16 +29856,16 @@
     </row>
     <row r="379" spans="1:35">
       <c r="A379">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B379" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C379" t="s">
         <v>50</v>
       </c>
       <c r="D379" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E379" t="s">
         <v>54</v>
@@ -29901,7 +29898,7 @@
         <v>2026</v>
       </c>
       <c r="R379">
-        <v>18188774</v>
+        <v>18178187</v>
       </c>
       <c r="S379" t="s">
         <v>186</v>
@@ -29910,16 +29907,16 @@
         <v>199</v>
       </c>
       <c r="V379" s="1">
-        <v>46282.36486778935</v>
+        <v>46282.36487561343</v>
       </c>
       <c r="W379">
         <v>1</v>
       </c>
       <c r="X379" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="Y379" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="AB379">
         <v>0</v>
@@ -29936,10 +29933,10 @@
     </row>
     <row r="380" spans="1:35">
       <c r="A380">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B380" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C380" t="s">
         <v>50</v>
@@ -29978,7 +29975,7 @@
         <v>2026</v>
       </c>
       <c r="R380">
-        <v>18188680</v>
+        <v>18188774</v>
       </c>
       <c r="S380" t="s">
         <v>186</v>
@@ -29987,7 +29984,7 @@
         <v>199</v>
       </c>
       <c r="V380" s="1">
-        <v>46282.36486851852</v>
+        <v>46282.36486778935</v>
       </c>
       <c r="W380">
         <v>1</v>
@@ -30013,10 +30010,10 @@
     </row>
     <row r="381" spans="1:35">
       <c r="A381">
-        <v>6404</v>
+        <v>6963</v>
       </c>
       <c r="B381" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C381" t="s">
         <v>50</v>
@@ -30028,10 +30025,10 @@
         <v>54</v>
       </c>
       <c r="F381" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G381">
-        <v>940</v>
+        <v>9086</v>
       </c>
       <c r="H381">
         <v>0</v>
@@ -30040,13 +30037,13 @@
         <v>64</v>
       </c>
       <c r="J381" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N381" s="1">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="O381" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P381">
         <v>9</v>
@@ -30055,25 +30052,25 @@
         <v>2026</v>
       </c>
       <c r="R381">
-        <v>16962074</v>
+        <v>18188680</v>
       </c>
       <c r="S381" t="s">
         <v>186</v>
       </c>
       <c r="U381" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="V381" s="1">
-        <v>46282.79619427084</v>
+        <v>46282.36486851852</v>
       </c>
       <c r="W381">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X381" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="Y381" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="AB381">
         <v>0</v>
@@ -30090,16 +30087,16 @@
     </row>
     <row r="382" spans="1:35">
       <c r="A382">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B382" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C382" t="s">
         <v>50</v>
       </c>
       <c r="D382" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E382" t="s">
         <v>54</v>
@@ -30132,7 +30129,7 @@
         <v>2026</v>
       </c>
       <c r="R382">
-        <v>16975871</v>
+        <v>16962074</v>
       </c>
       <c r="S382" t="s">
         <v>186</v>
@@ -30141,13 +30138,13 @@
         <v>198</v>
       </c>
       <c r="V382" s="1">
-        <v>46282.79620872685</v>
+        <v>46282.79619427084</v>
       </c>
       <c r="W382">
         <v>0</v>
       </c>
       <c r="X382" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="Y382" t="s">
         <v>349</v>
@@ -30167,10 +30164,10 @@
     </row>
     <row r="383" spans="1:35">
       <c r="A383">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B383" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C383" t="s">
         <v>50</v>
@@ -30209,7 +30206,7 @@
         <v>2026</v>
       </c>
       <c r="R383">
-        <v>17222366</v>
+        <v>16975871</v>
       </c>
       <c r="S383" t="s">
         <v>186</v>
@@ -30218,13 +30215,13 @@
         <v>198</v>
       </c>
       <c r="V383" s="1">
-        <v>46282.79623825232</v>
+        <v>46282.79620872685</v>
       </c>
       <c r="W383">
         <v>0</v>
       </c>
       <c r="X383" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="Y383" t="s">
         <v>349</v>
@@ -30244,10 +30241,10 @@
     </row>
     <row r="384" spans="1:35">
       <c r="A384">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B384" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C384" t="s">
         <v>50</v>
@@ -30256,7 +30253,7 @@
         <v>51</v>
       </c>
       <c r="E384" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F384" t="s">
         <v>56</v>
@@ -30286,7 +30283,7 @@
         <v>2026</v>
       </c>
       <c r="R384">
-        <v>17042221</v>
+        <v>17222366</v>
       </c>
       <c r="S384" t="s">
         <v>186</v>
@@ -30295,13 +30292,13 @@
         <v>198</v>
       </c>
       <c r="V384" s="1">
-        <v>46282.7962541551</v>
+        <v>46282.79623825232</v>
       </c>
       <c r="W384">
         <v>0</v>
       </c>
       <c r="X384" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Y384" t="s">
         <v>349</v>
@@ -30321,16 +30318,16 @@
     </row>
     <row r="385" spans="1:35">
       <c r="A385">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B385" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C385" t="s">
         <v>50</v>
       </c>
       <c r="D385" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E385" t="s">
         <v>55</v>
@@ -30363,7 +30360,7 @@
         <v>2026</v>
       </c>
       <c r="R385">
-        <v>16959926</v>
+        <v>17042221</v>
       </c>
       <c r="S385" t="s">
         <v>186</v>
@@ -30372,7 +30369,7 @@
         <v>198</v>
       </c>
       <c r="V385" s="1">
-        <v>46282.7962703125</v>
+        <v>46282.7962541551</v>
       </c>
       <c r="W385">
         <v>0</v>
@@ -30398,19 +30395,19 @@
     </row>
     <row r="386" spans="1:35">
       <c r="A386">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B386" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C386" t="s">
         <v>50</v>
       </c>
       <c r="D386" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E386" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F386" t="s">
         <v>56</v>
@@ -30440,7 +30437,7 @@
         <v>2026</v>
       </c>
       <c r="R386">
-        <v>17941112</v>
+        <v>16959926</v>
       </c>
       <c r="S386" t="s">
         <v>186</v>
@@ -30449,13 +30446,13 @@
         <v>198</v>
       </c>
       <c r="V386" s="1">
-        <v>46282.79628381944</v>
+        <v>46282.7962703125</v>
       </c>
       <c r="W386">
         <v>0</v>
       </c>
       <c r="X386" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="Y386" t="s">
         <v>349</v>
@@ -30475,16 +30472,16 @@
     </row>
     <row r="387" spans="1:35">
       <c r="A387">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B387" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C387" t="s">
         <v>50</v>
       </c>
       <c r="D387" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E387" t="s">
         <v>54</v>
@@ -30517,7 +30514,7 @@
         <v>2026</v>
       </c>
       <c r="R387">
-        <v>17952292</v>
+        <v>17941112</v>
       </c>
       <c r="S387" t="s">
         <v>186</v>
@@ -30526,13 +30523,13 @@
         <v>198</v>
       </c>
       <c r="V387" s="1">
-        <v>46282.79630119213</v>
+        <v>46282.79628381944</v>
       </c>
       <c r="W387">
         <v>0</v>
       </c>
       <c r="X387" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="Y387" t="s">
         <v>349</v>
@@ -30552,16 +30549,16 @@
     </row>
     <row r="388" spans="1:35">
       <c r="A388">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B388" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C388" t="s">
         <v>50</v>
       </c>
       <c r="D388" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E388" t="s">
         <v>54</v>
@@ -30594,7 +30591,7 @@
         <v>2026</v>
       </c>
       <c r="R388">
-        <v>17952491</v>
+        <v>17952292</v>
       </c>
       <c r="S388" t="s">
         <v>186</v>
@@ -30603,7 +30600,7 @@
         <v>198</v>
       </c>
       <c r="V388" s="1">
-        <v>46282.79631224537</v>
+        <v>46282.79630119213</v>
       </c>
       <c r="W388">
         <v>0</v>
@@ -30629,10 +30626,10 @@
     </row>
     <row r="389" spans="1:35">
       <c r="A389">
-        <v>6945</v>
+        <v>6705</v>
       </c>
       <c r="B389" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C389" t="s">
         <v>50</v>
@@ -30644,7 +30641,7 @@
         <v>54</v>
       </c>
       <c r="F389" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G389">
         <v>940</v>
@@ -30671,7 +30668,7 @@
         <v>2026</v>
       </c>
       <c r="R389">
-        <v>18164473</v>
+        <v>17952491</v>
       </c>
       <c r="S389" t="s">
         <v>186</v>
@@ -30680,16 +30677,16 @@
         <v>198</v>
       </c>
       <c r="V389" s="1">
-        <v>46282.79637734954</v>
+        <v>46282.79631224537</v>
       </c>
       <c r="W389">
         <v>0</v>
       </c>
       <c r="X389" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="Y389" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AB389">
         <v>0</v>
@@ -30706,16 +30703,16 @@
     </row>
     <row r="390" spans="1:35">
       <c r="A390">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B390" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C390" t="s">
         <v>50</v>
       </c>
       <c r="D390" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E390" t="s">
         <v>54</v>
@@ -30748,7 +30745,7 @@
         <v>2026</v>
       </c>
       <c r="R390">
-        <v>18178120</v>
+        <v>18164473</v>
       </c>
       <c r="S390" t="s">
         <v>186</v>
@@ -30757,13 +30754,13 @@
         <v>198</v>
       </c>
       <c r="V390" s="1">
-        <v>46282.79638922454</v>
+        <v>46282.79637734954</v>
       </c>
       <c r="W390">
         <v>0</v>
       </c>
       <c r="X390" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Y390" t="s">
         <v>350</v>
@@ -30783,10 +30780,10 @@
     </row>
     <row r="391" spans="1:35">
       <c r="A391">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B391" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C391" t="s">
         <v>50</v>
@@ -30798,19 +30795,19 @@
         <v>54</v>
       </c>
       <c r="F391" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G391">
-        <v>9088</v>
+        <v>940</v>
       </c>
       <c r="H391">
         <v>0</v>
       </c>
       <c r="I391" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J391" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="N391" s="1">
         <v>46283</v>
@@ -30825,22 +30822,22 @@
         <v>2026</v>
       </c>
       <c r="R391">
-        <v>17399383</v>
+        <v>18178120</v>
       </c>
       <c r="S391" t="s">
-        <v>54</v>
+        <v>186</v>
       </c>
       <c r="U391" t="s">
         <v>198</v>
       </c>
       <c r="V391" s="1">
-        <v>46282.3651903588</v>
+        <v>46282.79638922454</v>
       </c>
       <c r="W391">
         <v>0</v>
       </c>
       <c r="X391" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="Y391" t="s">
         <v>350</v>
@@ -30849,7 +30846,7 @@
         <v>0</v>
       </c>
       <c r="AC391" t="s">
-        <v>54</v>
+        <v>186</v>
       </c>
       <c r="AH391" t="s">
         <v>360</v>
@@ -30860,16 +30857,16 @@
     </row>
     <row r="392" spans="1:35">
       <c r="A392">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B392" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C392" t="s">
         <v>50</v>
       </c>
       <c r="D392" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E392" t="s">
         <v>54</v>
@@ -30902,7 +30899,7 @@
         <v>2026</v>
       </c>
       <c r="R392">
-        <v>16962400</v>
+        <v>17399383</v>
       </c>
       <c r="S392" t="s">
         <v>54</v>
@@ -30911,13 +30908,13 @@
         <v>198</v>
       </c>
       <c r="V392" s="1">
-        <v>46282.36525856482</v>
+        <v>46282.3651903588</v>
       </c>
       <c r="W392">
         <v>0</v>
       </c>
       <c r="X392" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="Y392" t="s">
         <v>350</v>
@@ -30937,16 +30934,16 @@
     </row>
     <row r="393" spans="1:35">
       <c r="A393">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B393" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C393" t="s">
         <v>50</v>
       </c>
       <c r="D393" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E393" t="s">
         <v>54</v>
@@ -30979,7 +30976,7 @@
         <v>2026</v>
       </c>
       <c r="R393">
-        <v>16976290</v>
+        <v>16962400</v>
       </c>
       <c r="S393" t="s">
         <v>54</v>
@@ -30988,13 +30985,13 @@
         <v>198</v>
       </c>
       <c r="V393" s="1">
-        <v>46282.36526855324</v>
+        <v>46282.36525856482</v>
       </c>
       <c r="W393">
         <v>0</v>
       </c>
       <c r="X393" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="Y393" t="s">
         <v>350</v>
@@ -31014,10 +31011,10 @@
     </row>
     <row r="394" spans="1:35">
       <c r="A394">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B394" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C394" t="s">
         <v>50</v>
@@ -31056,7 +31053,7 @@
         <v>2026</v>
       </c>
       <c r="R394">
-        <v>17222899</v>
+        <v>16976290</v>
       </c>
       <c r="S394" t="s">
         <v>54</v>
@@ -31065,13 +31062,13 @@
         <v>198</v>
       </c>
       <c r="V394" s="1">
-        <v>46282.36527959491</v>
+        <v>46282.36526855324</v>
       </c>
       <c r="W394">
         <v>0</v>
       </c>
       <c r="X394" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="Y394" t="s">
         <v>350</v>
@@ -31091,10 +31088,10 @@
     </row>
     <row r="395" spans="1:35">
       <c r="A395">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B395" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C395" t="s">
         <v>50</v>
@@ -31103,7 +31100,7 @@
         <v>51</v>
       </c>
       <c r="E395" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F395" t="s">
         <v>56</v>
@@ -31133,22 +31130,22 @@
         <v>2026</v>
       </c>
       <c r="R395">
-        <v>17042627</v>
+        <v>17222899</v>
       </c>
       <c r="S395" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="U395" t="s">
         <v>198</v>
       </c>
       <c r="V395" s="1">
-        <v>46282.36528526621</v>
+        <v>46282.36527959491</v>
       </c>
       <c r="W395">
         <v>0</v>
       </c>
       <c r="X395" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Y395" t="s">
         <v>350</v>
@@ -31157,7 +31154,7 @@
         <v>0</v>
       </c>
       <c r="AC395" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="AH395" t="s">
         <v>360</v>
@@ -31168,16 +31165,16 @@
     </row>
     <row r="396" spans="1:35">
       <c r="A396">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B396" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C396" t="s">
         <v>50</v>
       </c>
       <c r="D396" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E396" t="s">
         <v>55</v>
@@ -31210,16 +31207,16 @@
         <v>2026</v>
       </c>
       <c r="R396">
-        <v>16960098</v>
+        <v>17042627</v>
       </c>
       <c r="S396" t="s">
-        <v>55</v>
+        <v>187</v>
       </c>
       <c r="U396" t="s">
         <v>198</v>
       </c>
       <c r="V396" s="1">
-        <v>46282.36528619213</v>
+        <v>46282.36528526621</v>
       </c>
       <c r="W396">
         <v>0</v>
@@ -31234,7 +31231,7 @@
         <v>0</v>
       </c>
       <c r="AC396" t="s">
-        <v>55</v>
+        <v>187</v>
       </c>
       <c r="AH396" t="s">
         <v>360</v>
@@ -31245,19 +31242,19 @@
     </row>
     <row r="397" spans="1:35">
       <c r="A397">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B397" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C397" t="s">
         <v>50</v>
       </c>
       <c r="D397" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E397" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F397" t="s">
         <v>56</v>
@@ -31287,22 +31284,22 @@
         <v>2026</v>
       </c>
       <c r="R397">
-        <v>17941237</v>
+        <v>16960098</v>
       </c>
       <c r="S397" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="U397" t="s">
         <v>198</v>
       </c>
       <c r="V397" s="1">
-        <v>46282.36529351852</v>
+        <v>46282.36528619213</v>
       </c>
       <c r="W397">
         <v>0</v>
       </c>
       <c r="X397" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="Y397" t="s">
         <v>350</v>
@@ -31311,7 +31308,7 @@
         <v>0</v>
       </c>
       <c r="AC397" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="AH397" t="s">
         <v>360</v>
@@ -31322,16 +31319,16 @@
     </row>
     <row r="398" spans="1:35">
       <c r="A398">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B398" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C398" t="s">
         <v>50</v>
       </c>
       <c r="D398" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E398" t="s">
         <v>54</v>
@@ -31364,7 +31361,7 @@
         <v>2026</v>
       </c>
       <c r="R398">
-        <v>17952466</v>
+        <v>17941237</v>
       </c>
       <c r="S398" t="s">
         <v>54</v>
@@ -31373,13 +31370,13 @@
         <v>198</v>
       </c>
       <c r="V398" s="1">
-        <v>46282.36529424768</v>
+        <v>46282.36529351852</v>
       </c>
       <c r="W398">
         <v>0</v>
       </c>
       <c r="X398" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="Y398" t="s">
         <v>350</v>
@@ -31399,16 +31396,16 @@
     </row>
     <row r="399" spans="1:35">
       <c r="A399">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B399" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C399" t="s">
         <v>50</v>
       </c>
       <c r="D399" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E399" t="s">
         <v>54</v>
@@ -31441,7 +31438,7 @@
         <v>2026</v>
       </c>
       <c r="R399">
-        <v>17952646</v>
+        <v>17952466</v>
       </c>
       <c r="S399" t="s">
         <v>54</v>
@@ -31450,7 +31447,7 @@
         <v>198</v>
       </c>
       <c r="V399" s="1">
-        <v>46282.36529490741</v>
+        <v>46282.36529424768</v>
       </c>
       <c r="W399">
         <v>0</v>
@@ -31476,10 +31473,10 @@
     </row>
     <row r="400" spans="1:35">
       <c r="A400">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B400" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C400" t="s">
         <v>50</v>
@@ -31518,16 +31515,16 @@
         <v>2026</v>
       </c>
       <c r="R400">
-        <v>18056821</v>
+        <v>17952646</v>
       </c>
       <c r="S400" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="U400" t="s">
         <v>198</v>
       </c>
       <c r="V400" s="1">
-        <v>46282.36529869213</v>
+        <v>46282.36529490741</v>
       </c>
       <c r="W400">
         <v>0</v>
@@ -31542,7 +31539,7 @@
         <v>0</v>
       </c>
       <c r="AC400" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="AH400" t="s">
         <v>360</v>
@@ -31553,10 +31550,10 @@
     </row>
     <row r="401" spans="1:35">
       <c r="A401">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B401" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C401" t="s">
         <v>50</v>
@@ -31568,7 +31565,7 @@
         <v>54</v>
       </c>
       <c r="F401" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G401">
         <v>9088</v>
@@ -31595,22 +31592,22 @@
         <v>2026</v>
       </c>
       <c r="R401">
-        <v>18164565</v>
+        <v>18056821</v>
       </c>
       <c r="S401" t="s">
-        <v>54</v>
+        <v>187</v>
       </c>
       <c r="U401" t="s">
         <v>198</v>
       </c>
       <c r="V401" s="1">
-        <v>46282.36531149306</v>
+        <v>46282.36529869213</v>
       </c>
       <c r="W401">
         <v>0</v>
       </c>
       <c r="X401" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="Y401" t="s">
         <v>350</v>
@@ -31619,7 +31616,7 @@
         <v>0</v>
       </c>
       <c r="AC401" t="s">
-        <v>54</v>
+        <v>187</v>
       </c>
       <c r="AH401" t="s">
         <v>360</v>
@@ -31630,16 +31627,16 @@
     </row>
     <row r="402" spans="1:35">
       <c r="A402">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B402" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C402" t="s">
         <v>50</v>
       </c>
       <c r="D402" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E402" t="s">
         <v>54</v>
@@ -31672,31 +31669,31 @@
         <v>2026</v>
       </c>
       <c r="R402">
-        <v>18178199</v>
+        <v>18164565</v>
       </c>
       <c r="S402" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="U402" t="s">
         <v>198</v>
       </c>
       <c r="V402" s="1">
-        <v>46282.36531554398</v>
+        <v>46282.36531149306</v>
       </c>
       <c r="W402">
         <v>0</v>
       </c>
       <c r="X402" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Y402" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="AB402">
         <v>0</v>
       </c>
       <c r="AC402" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="AH402" t="s">
         <v>360</v>
@@ -31707,16 +31704,16 @@
     </row>
     <row r="403" spans="1:35">
       <c r="A403">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B403" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C403" t="s">
         <v>50</v>
       </c>
       <c r="D403" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E403" t="s">
         <v>54</v>
@@ -31749,31 +31746,31 @@
         <v>2026</v>
       </c>
       <c r="R403">
-        <v>18188788</v>
+        <v>18178199</v>
       </c>
       <c r="S403" t="s">
-        <v>54</v>
+        <v>187</v>
       </c>
       <c r="U403" t="s">
         <v>198</v>
       </c>
       <c r="V403" s="1">
-        <v>46282.36531253472</v>
+        <v>46282.36531554398</v>
       </c>
       <c r="W403">
         <v>0</v>
       </c>
       <c r="X403" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="Y403" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="AB403">
         <v>0</v>
       </c>
       <c r="AC403" t="s">
-        <v>54</v>
+        <v>187</v>
       </c>
       <c r="AH403" t="s">
         <v>360</v>
@@ -31784,10 +31781,10 @@
     </row>
     <row r="404" spans="1:35">
       <c r="A404">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B404" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C404" t="s">
         <v>50</v>
@@ -31826,7 +31823,7 @@
         <v>2026</v>
       </c>
       <c r="R404">
-        <v>18188694</v>
+        <v>18188788</v>
       </c>
       <c r="S404" t="s">
         <v>54</v>
@@ -31835,7 +31832,7 @@
         <v>198</v>
       </c>
       <c r="V404" s="1">
-        <v>46282.36531288194</v>
+        <v>46282.36531253472</v>
       </c>
       <c r="W404">
         <v>0</v>
@@ -31861,10 +31858,10 @@
     </row>
     <row r="405" spans="1:35">
       <c r="A405">
-        <v>6404</v>
+        <v>6963</v>
       </c>
       <c r="B405" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C405" t="s">
         <v>50</v>
@@ -31876,10 +31873,10 @@
         <v>54</v>
       </c>
       <c r="F405" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G405">
-        <v>6813</v>
+        <v>9088</v>
       </c>
       <c r="H405">
         <v>0</v>
@@ -31888,7 +31885,7 @@
         <v>65</v>
       </c>
       <c r="J405" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="N405" s="1">
         <v>46283</v>
@@ -31903,7 +31900,7 @@
         <v>2026</v>
       </c>
       <c r="R405">
-        <v>16962319</v>
+        <v>18188694</v>
       </c>
       <c r="S405" t="s">
         <v>54</v>
@@ -31912,13 +31909,13 @@
         <v>198</v>
       </c>
       <c r="V405" s="1">
-        <v>46282.79619331018</v>
+        <v>46282.36531288194</v>
       </c>
       <c r="W405">
         <v>0</v>
       </c>
       <c r="X405" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="Y405" t="s">
         <v>350</v>
@@ -31938,16 +31935,16 @@
     </row>
     <row r="406" spans="1:35">
       <c r="A406">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B406" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C406" t="s">
         <v>50</v>
       </c>
       <c r="D406" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E406" t="s">
         <v>54</v>
@@ -31980,7 +31977,7 @@
         <v>2026</v>
       </c>
       <c r="R406">
-        <v>16976198</v>
+        <v>16962319</v>
       </c>
       <c r="S406" t="s">
         <v>54</v>
@@ -31989,13 +31986,13 @@
         <v>198</v>
       </c>
       <c r="V406" s="1">
-        <v>46282.79620888889</v>
+        <v>46282.79619331018</v>
       </c>
       <c r="W406">
         <v>0</v>
       </c>
       <c r="X406" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="Y406" t="s">
         <v>350</v>
@@ -32015,10 +32012,10 @@
     </row>
     <row r="407" spans="1:35">
       <c r="A407">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B407" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C407" t="s">
         <v>50</v>
@@ -32057,7 +32054,7 @@
         <v>2026</v>
       </c>
       <c r="R407">
-        <v>17222763</v>
+        <v>16976198</v>
       </c>
       <c r="S407" t="s">
         <v>54</v>
@@ -32066,13 +32063,13 @@
         <v>198</v>
       </c>
       <c r="V407" s="1">
-        <v>46282.79623803241</v>
+        <v>46282.79620888889</v>
       </c>
       <c r="W407">
         <v>0</v>
       </c>
       <c r="X407" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="Y407" t="s">
         <v>350</v>
@@ -32092,10 +32089,10 @@
     </row>
     <row r="408" spans="1:35">
       <c r="A408">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B408" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C408" t="s">
         <v>50</v>
@@ -32104,7 +32101,7 @@
         <v>51</v>
       </c>
       <c r="E408" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F408" t="s">
         <v>56</v>
@@ -32134,22 +32131,22 @@
         <v>2026</v>
       </c>
       <c r="R408">
-        <v>17042469</v>
+        <v>17222763</v>
       </c>
       <c r="S408" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="U408" t="s">
         <v>198</v>
       </c>
       <c r="V408" s="1">
-        <v>46282.79625384259</v>
+        <v>46282.79623803241</v>
       </c>
       <c r="W408">
         <v>0</v>
       </c>
       <c r="X408" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Y408" t="s">
         <v>350</v>
@@ -32158,7 +32155,7 @@
         <v>0</v>
       </c>
       <c r="AC408" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="AH408" t="s">
         <v>360</v>
@@ -32169,16 +32166,16 @@
     </row>
     <row r="409" spans="1:35">
       <c r="A409">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B409" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C409" t="s">
         <v>50</v>
       </c>
       <c r="D409" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E409" t="s">
         <v>55</v>
@@ -32211,16 +32208,16 @@
         <v>2026</v>
       </c>
       <c r="R409">
-        <v>16960013</v>
+        <v>17042469</v>
       </c>
       <c r="S409" t="s">
-        <v>55</v>
+        <v>187</v>
       </c>
       <c r="U409" t="s">
         <v>198</v>
       </c>
       <c r="V409" s="1">
-        <v>46282.79626969907</v>
+        <v>46282.79625384259</v>
       </c>
       <c r="W409">
         <v>0</v>
@@ -32235,7 +32232,7 @@
         <v>0</v>
       </c>
       <c r="AC409" t="s">
-        <v>55</v>
+        <v>187</v>
       </c>
       <c r="AH409" t="s">
         <v>360</v>
@@ -32246,19 +32243,19 @@
     </row>
     <row r="410" spans="1:35">
       <c r="A410">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B410" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C410" t="s">
         <v>50</v>
       </c>
       <c r="D410" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E410" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F410" t="s">
         <v>56</v>
@@ -32288,22 +32285,22 @@
         <v>2026</v>
       </c>
       <c r="R410">
-        <v>17941197</v>
+        <v>16960013</v>
       </c>
       <c r="S410" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="U410" t="s">
         <v>198</v>
       </c>
       <c r="V410" s="1">
-        <v>46282.79628394676</v>
+        <v>46282.79626969907</v>
       </c>
       <c r="W410">
         <v>0</v>
       </c>
       <c r="X410" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="Y410" t="s">
         <v>350</v>
@@ -32312,7 +32309,7 @@
         <v>0</v>
       </c>
       <c r="AC410" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="AH410" t="s">
         <v>360</v>
@@ -32323,16 +32320,16 @@
     </row>
     <row r="411" spans="1:35">
       <c r="A411">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B411" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C411" t="s">
         <v>50</v>
       </c>
       <c r="D411" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E411" t="s">
         <v>54</v>
@@ -32365,7 +32362,7 @@
         <v>2026</v>
       </c>
       <c r="R411">
-        <v>17952411</v>
+        <v>17941197</v>
       </c>
       <c r="S411" t="s">
         <v>54</v>
@@ -32374,13 +32371,13 @@
         <v>198</v>
       </c>
       <c r="V411" s="1">
-        <v>46282.79630097222</v>
+        <v>46282.79628394676</v>
       </c>
       <c r="W411">
         <v>0</v>
       </c>
       <c r="X411" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="Y411" t="s">
         <v>350</v>
@@ -32400,16 +32397,16 @@
     </row>
     <row r="412" spans="1:35">
       <c r="A412">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B412" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C412" t="s">
         <v>50</v>
       </c>
       <c r="D412" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E412" t="s">
         <v>54</v>
@@ -32442,7 +32439,7 @@
         <v>2026</v>
       </c>
       <c r="R412">
-        <v>17952591</v>
+        <v>17952411</v>
       </c>
       <c r="S412" t="s">
         <v>54</v>
@@ -32451,7 +32448,7 @@
         <v>198</v>
       </c>
       <c r="V412" s="1">
-        <v>46282.79631204861</v>
+        <v>46282.79630097222</v>
       </c>
       <c r="W412">
         <v>0</v>
@@ -32477,10 +32474,10 @@
     </row>
     <row r="413" spans="1:35">
       <c r="A413">
-        <v>6945</v>
+        <v>6705</v>
       </c>
       <c r="B413" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C413" t="s">
         <v>50</v>
@@ -32492,7 +32489,7 @@
         <v>54</v>
       </c>
       <c r="F413" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G413">
         <v>6813</v>
@@ -32519,7 +32516,7 @@
         <v>2026</v>
       </c>
       <c r="R413">
-        <v>18164530</v>
+        <v>17952591</v>
       </c>
       <c r="S413" t="s">
         <v>54</v>
@@ -32528,16 +32525,16 @@
         <v>198</v>
       </c>
       <c r="V413" s="1">
-        <v>46282.79637748843</v>
+        <v>46282.79631204861</v>
       </c>
       <c r="W413">
         <v>0</v>
       </c>
       <c r="X413" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="Y413" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="AB413">
         <v>0</v>
@@ -32554,16 +32551,16 @@
     </row>
     <row r="414" spans="1:35">
       <c r="A414">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B414" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C414" t="s">
         <v>50</v>
       </c>
       <c r="D414" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E414" t="s">
         <v>54</v>
@@ -32596,22 +32593,22 @@
         <v>2026</v>
       </c>
       <c r="R414">
-        <v>18178169</v>
+        <v>18164530</v>
       </c>
       <c r="S414" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="U414" t="s">
         <v>198</v>
       </c>
       <c r="V414" s="1">
-        <v>46282.79638901621</v>
+        <v>46282.79637748843</v>
       </c>
       <c r="W414">
         <v>0</v>
       </c>
       <c r="X414" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Y414" t="s">
         <v>351</v>
@@ -32620,7 +32617,7 @@
         <v>0</v>
       </c>
       <c r="AC414" t="s">
-        <v>187</v>
+        <v>54</v>
       </c>
       <c r="AH414" t="s">
         <v>360</v>
@@ -32631,10 +32628,10 @@
     </row>
     <row r="415" spans="1:35">
       <c r="A415">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B415" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C415" t="s">
         <v>50</v>
@@ -32646,10 +32643,10 @@
         <v>54</v>
       </c>
       <c r="F415" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G415">
-        <v>7027</v>
+        <v>6813</v>
       </c>
       <c r="H415">
         <v>0</v>
@@ -32658,46 +32655,49 @@
         <v>65</v>
       </c>
       <c r="J415" t="s">
-        <v>121</v>
+        <v>150</v>
       </c>
       <c r="N415" s="1">
-        <v>46289</v>
+        <v>46283</v>
+      </c>
+      <c r="O415" t="s">
+        <v>159</v>
       </c>
       <c r="P415">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q415">
         <v>2026</v>
       </c>
       <c r="R415">
-        <v>17399290</v>
+        <v>18178169</v>
       </c>
       <c r="S415" t="s">
-        <v>54</v>
+        <v>187</v>
       </c>
       <c r="U415" t="s">
         <v>198</v>
       </c>
       <c r="V415" s="1">
-        <v>46283.39832862269</v>
+        <v>46282.79638901621</v>
       </c>
       <c r="W415">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="X415" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="Y415" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="AB415">
         <v>0</v>
       </c>
       <c r="AC415" t="s">
-        <v>54</v>
+        <v>187</v>
       </c>
       <c r="AH415" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="AI415" t="s">
         <v>363</v>
@@ -32705,16 +32705,16 @@
     </row>
     <row r="416" spans="1:35">
       <c r="A416">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B416" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C416" t="s">
         <v>50</v>
       </c>
       <c r="D416" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E416" t="s">
         <v>54</v>
@@ -32744,7 +32744,7 @@
         <v>2026</v>
       </c>
       <c r="R416">
-        <v>16962348</v>
+        <v>17399290</v>
       </c>
       <c r="S416" t="s">
         <v>54</v>
@@ -32753,16 +32753,16 @@
         <v>198</v>
       </c>
       <c r="V416" s="1">
-        <v>46282.64018086805</v>
+        <v>46283.39832862269</v>
       </c>
       <c r="W416">
         <v>-6</v>
       </c>
       <c r="X416" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="Y416" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="AB416">
         <v>0</v>
@@ -32774,6 +32774,80 @@
         <v>358</v>
       </c>
       <c r="AI416" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="417" spans="1:35">
+      <c r="A417">
+        <v>6404</v>
+      </c>
+      <c r="B417" t="s">
+        <v>47</v>
+      </c>
+      <c r="C417" t="s">
+        <v>50</v>
+      </c>
+      <c r="D417" t="s">
+        <v>53</v>
+      </c>
+      <c r="E417" t="s">
+        <v>54</v>
+      </c>
+      <c r="F417" t="s">
+        <v>56</v>
+      </c>
+      <c r="G417">
+        <v>7027</v>
+      </c>
+      <c r="H417">
+        <v>0</v>
+      </c>
+      <c r="I417" t="s">
+        <v>65</v>
+      </c>
+      <c r="J417" t="s">
+        <v>121</v>
+      </c>
+      <c r="N417" s="1">
+        <v>46289</v>
+      </c>
+      <c r="P417">
+        <v>8</v>
+      </c>
+      <c r="Q417">
+        <v>2026</v>
+      </c>
+      <c r="R417">
+        <v>16962348</v>
+      </c>
+      <c r="S417" t="s">
+        <v>54</v>
+      </c>
+      <c r="U417" t="s">
+        <v>198</v>
+      </c>
+      <c r="V417" s="1">
+        <v>46282.64018086805</v>
+      </c>
+      <c r="W417">
+        <v>-6</v>
+      </c>
+      <c r="X417" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y417" t="s">
+        <v>353</v>
+      </c>
+      <c r="AB417">
+        <v>0</v>
+      </c>
+      <c r="AC417" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH417" t="s">
+        <v>358</v>
+      </c>
+      <c r="AI417" t="s">
         <v>363</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-24 09:02
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -813,13 +813,13 @@
     <t>BENEFICIO SOCIAL - BOLETOS - Data Comentário: 01/09/2026 14:26</t>
   </si>
   <si>
+    <t>Demissão Por Justa Causa em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:14</t>
+  </si>
+  <si>
+    <t>Demissão Por Justa Causa em 03/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:29</t>
+  </si>
+  <si>
     <t>Pedido de demissão - Desconto de Aviso em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 03/09/2026 16:47</t>
-  </si>
-  <si>
-    <t>Demissão Por Justa Causa em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:14</t>
-  </si>
-  <si>
-    <t>Demissão Por Justa Causa em 03/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:29</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/09/2026 
@@ -7559,13 +7559,13 @@
         <v>2026</v>
       </c>
       <c r="R77">
-        <v>18263044</v>
+        <v>18269524</v>
       </c>
       <c r="U77" t="s">
         <v>220</v>
       </c>
       <c r="V77" s="1">
-        <v>46273.63629708334</v>
+        <v>46273.64318633102</v>
       </c>
       <c r="W77">
         <v>15</v>
@@ -7633,13 +7633,13 @@
         <v>2026</v>
       </c>
       <c r="R78">
-        <v>18269524</v>
+        <v>18269550</v>
       </c>
       <c r="U78" t="s">
         <v>220</v>
       </c>
       <c r="V78" s="1">
-        <v>46273.64318633102</v>
+        <v>46273.64880981482</v>
       </c>
       <c r="W78">
         <v>15</v>
@@ -7707,13 +7707,13 @@
         <v>2026</v>
       </c>
       <c r="R79">
-        <v>18269550</v>
+        <v>18263044</v>
       </c>
       <c r="U79" t="s">
         <v>220</v>
       </c>
       <c r="V79" s="1">
-        <v>46273.64880981482</v>
+        <v>46273.63629708334</v>
       </c>
       <c r="W79">
         <v>15</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-24 13:09
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -816,13 +816,13 @@
     <t>BENEFICIO SOCIAL - BOLETOS - Data Comentário: 01/09/2026 14:26</t>
   </si>
   <si>
+    <t>Pedido de demissão - Desconto de Aviso em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 03/09/2026 16:47</t>
+  </si>
+  <si>
+    <t>Demissão Por Justa Causa em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:14</t>
+  </si>
+  <si>
     <t>Demissão Por Justa Causa em 03/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:29</t>
-  </si>
-  <si>
-    <t>Pedido de demissão - Desconto de Aviso em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 03/09/2026 16:47</t>
-  </si>
-  <si>
-    <t>Demissão Por Justa Causa em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:14</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/09/2026 
@@ -7572,13 +7572,13 @@
         <v>2026</v>
       </c>
       <c r="R77">
-        <v>18269550</v>
+        <v>18263044</v>
       </c>
       <c r="U77" t="s">
         <v>221</v>
       </c>
       <c r="V77" s="1">
-        <v>46273.64880981482</v>
+        <v>46273.63629708334</v>
       </c>
       <c r="W77">
         <v>15</v>
@@ -7646,13 +7646,13 @@
         <v>2026</v>
       </c>
       <c r="R78">
-        <v>18263044</v>
+        <v>18269524</v>
       </c>
       <c r="U78" t="s">
         <v>221</v>
       </c>
       <c r="V78" s="1">
-        <v>46273.63629708334</v>
+        <v>46273.64318633102</v>
       </c>
       <c r="W78">
         <v>15</v>
@@ -7720,13 +7720,13 @@
         <v>2026</v>
       </c>
       <c r="R79">
-        <v>18269524</v>
+        <v>18269550</v>
       </c>
       <c r="U79" t="s">
         <v>221</v>
       </c>
       <c r="V79" s="1">
-        <v>46273.64318633102</v>
+        <v>46273.64880981482</v>
       </c>
       <c r="W79">
         <v>15</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-24 19:37
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -816,13 +816,13 @@
     <t>BENEFICIO SOCIAL - BOLETOS - Data Comentário: 01/09/2026 14:26</t>
   </si>
   <si>
+    <t>Pedido de demissão - Desconto de Aviso em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 03/09/2026 16:47</t>
+  </si>
+  <si>
+    <t>Demissão Por Justa Causa em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:14</t>
+  </si>
+  <si>
     <t>Demissão Por Justa Causa em 03/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:29</t>
-  </si>
-  <si>
-    <t>Pedido de demissão - Desconto de Aviso em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 03/09/2026 16:47</t>
-  </si>
-  <si>
-    <t>Demissão Por Justa Causa em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:14</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/09/2026 
@@ -7569,13 +7569,13 @@
         <v>2026</v>
       </c>
       <c r="R77">
-        <v>18269550</v>
+        <v>18263044</v>
       </c>
       <c r="U77" t="s">
         <v>221</v>
       </c>
       <c r="V77" s="1">
-        <v>46273.64880981482</v>
+        <v>46273.63629708334</v>
       </c>
       <c r="W77">
         <v>15</v>
@@ -7643,13 +7643,13 @@
         <v>2026</v>
       </c>
       <c r="R78">
-        <v>18263044</v>
+        <v>18269524</v>
       </c>
       <c r="U78" t="s">
         <v>221</v>
       </c>
       <c r="V78" s="1">
-        <v>46273.63629708334</v>
+        <v>46273.64318633102</v>
       </c>
       <c r="W78">
         <v>15</v>
@@ -7717,13 +7717,13 @@
         <v>2026</v>
       </c>
       <c r="R79">
-        <v>18269524</v>
+        <v>18269550</v>
       </c>
       <c r="U79" t="s">
         <v>221</v>
       </c>
       <c r="V79" s="1">
-        <v>46273.64318633102</v>
+        <v>46273.64880981482</v>
       </c>
       <c r="W79">
         <v>15</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-25 09:00
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7223" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7219" uniqueCount="433">
   <si>
     <t>CodCliente</t>
   </si>
@@ -816,13 +816,13 @@
     <t>BENEFICIO SOCIAL - BOLETOS - Data Comentário: 01/09/2026 14:26</t>
   </si>
   <si>
+    <t>Demissão Por Justa Causa em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:14</t>
+  </si>
+  <si>
+    <t>Demissão Por Justa Causa em 03/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:29</t>
+  </si>
+  <si>
     <t>Pedido de demissão - Desconto de Aviso em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 03/09/2026 16:47</t>
-  </si>
-  <si>
-    <t>Demissão Por Justa Causa em 02/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:14</t>
-  </si>
-  <si>
-    <t>Demissão Por Justa Causa em 03/09/2026 - Pgto 11/09/2026 - Data Comentário: 08/09/2026 15:29</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/09/2026 
@@ -1851,7 +1851,7 @@
         <v>46268.63953865741</v>
       </c>
       <c r="W2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X2" t="s">
         <v>223</v>
@@ -1928,7 +1928,7 @@
         <v>46266.57730150463</v>
       </c>
       <c r="W3">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X3" t="s">
         <v>224</v>
@@ -2005,7 +2005,7 @@
         <v>46266.41668148148</v>
       </c>
       <c r="W4">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X4" t="s">
         <v>225</v>
@@ -2082,7 +2082,7 @@
         <v>46267.75233784723</v>
       </c>
       <c r="W5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X5" t="s">
         <v>223</v>
@@ -2156,7 +2156,7 @@
         <v>46267.75233927083</v>
       </c>
       <c r="W6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X6" t="s">
         <v>224</v>
@@ -2230,7 +2230,7 @@
         <v>46267.7523394676</v>
       </c>
       <c r="W7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X7" t="s">
         <v>224</v>
@@ -2304,7 +2304,7 @@
         <v>46267.75234278935</v>
       </c>
       <c r="W8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X8" t="s">
         <v>226</v>
@@ -2378,7 +2378,7 @@
         <v>46267.75234309028</v>
       </c>
       <c r="W9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X9" t="s">
         <v>225</v>
@@ -2452,7 +2452,7 @@
         <v>46267.75234383102</v>
       </c>
       <c r="W10">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X10" t="s">
         <v>227</v>
@@ -2526,7 +2526,7 @@
         <v>46267.75234424769</v>
       </c>
       <c r="W11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X11" t="s">
         <v>227</v>
@@ -2600,7 +2600,7 @@
         <v>46267.47365627315</v>
       </c>
       <c r="W12">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X12" t="s">
         <v>228</v>
@@ -2674,7 +2674,7 @@
         <v>46266.47620831019</v>
       </c>
       <c r="W13">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X13" t="s">
         <v>229</v>
@@ -2748,7 +2748,7 @@
         <v>46267.57586420139</v>
       </c>
       <c r="W14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X14" t="s">
         <v>230</v>
@@ -2819,7 +2819,7 @@
         <v>46266.44145744213</v>
       </c>
       <c r="W15">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="X15" t="s">
         <v>231</v>
@@ -2887,7 +2887,7 @@
         <v>46266.44156952546</v>
       </c>
       <c r="W16">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X16" t="s">
         <v>231</v>
@@ -2955,7 +2955,7 @@
         <v>46266.44152346065</v>
       </c>
       <c r="W17">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X17" t="s">
         <v>231</v>
@@ -3029,7 +3029,7 @@
         <v>46269.3962034375</v>
       </c>
       <c r="W18">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X18" t="s">
         <v>232</v>
@@ -3106,7 +3106,7 @@
         <v>46268.54759884259</v>
       </c>
       <c r="W19">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X19" t="s">
         <v>229</v>
@@ -3183,7 +3183,7 @@
         <v>46269.38216940972</v>
       </c>
       <c r="W20">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X20" t="s">
         <v>230</v>
@@ -3260,7 +3260,7 @@
         <v>46269.40844942129</v>
       </c>
       <c r="W21">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X21" t="s">
         <v>228</v>
@@ -3337,7 +3337,7 @@
         <v>46266.37634084491</v>
       </c>
       <c r="W22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X22" t="s">
         <v>233</v>
@@ -3411,7 +3411,7 @@
         <v>46267.47452163194</v>
       </c>
       <c r="W23">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X23" t="s">
         <v>228</v>
@@ -3485,7 +3485,7 @@
         <v>46267.4745221412</v>
       </c>
       <c r="W24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X24" t="s">
         <v>228</v>
@@ -3559,7 +3559,7 @@
         <v>46267.47452299768</v>
       </c>
       <c r="W25">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X25" t="s">
         <v>228</v>
@@ -3633,7 +3633,7 @@
         <v>46267.75231010417</v>
       </c>
       <c r="W26">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X26" t="s">
         <v>229</v>
@@ -3707,7 +3707,7 @@
         <v>46267.75234059028</v>
       </c>
       <c r="W27">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X27" t="s">
         <v>228</v>
@@ -3781,7 +3781,7 @@
         <v>46267.7523409375</v>
       </c>
       <c r="W28">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X28" t="s">
         <v>228</v>
@@ -3855,7 +3855,7 @@
         <v>46267.75234170139</v>
       </c>
       <c r="W29">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X29" t="s">
         <v>228</v>
@@ -3929,7 +3929,7 @@
         <v>46268.58940019676</v>
       </c>
       <c r="W30">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X30" t="s">
         <v>232</v>
@@ -4006,7 +4006,7 @@
         <v>46268.37896984954</v>
       </c>
       <c r="W31">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X31" t="s">
         <v>224</v>
@@ -4083,7 +4083,7 @@
         <v>46269.71652982639</v>
       </c>
       <c r="W32">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X32" t="s">
         <v>226</v>
@@ -4160,7 +4160,7 @@
         <v>46269.71069613426</v>
       </c>
       <c r="W33">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X33" t="s">
         <v>225</v>
@@ -4240,7 +4240,7 @@
         <v>46267.55838734953</v>
       </c>
       <c r="W34">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X34" t="s">
         <v>229</v>
@@ -4320,7 +4320,7 @@
         <v>46273.59003707176</v>
       </c>
       <c r="W35">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X35" t="s">
         <v>233</v>
@@ -4400,7 +4400,7 @@
         <v>46268.74069754629</v>
       </c>
       <c r="W36">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X36" t="s">
         <v>223</v>
@@ -4480,7 +4480,7 @@
         <v>46273.45940115741</v>
       </c>
       <c r="W37">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X37" t="s">
         <v>232</v>
@@ -4560,7 +4560,7 @@
         <v>46267.66088636574</v>
       </c>
       <c r="W38">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X38" t="s">
         <v>229</v>
@@ -4640,7 +4640,7 @@
         <v>46268.45922827546</v>
       </c>
       <c r="W39">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X39" t="s">
         <v>230</v>
@@ -4720,7 +4720,7 @@
         <v>46269.59248078704</v>
       </c>
       <c r="W40">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X40" t="s">
         <v>224</v>
@@ -4800,7 +4800,7 @@
         <v>46269.59224453704</v>
       </c>
       <c r="W41">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X41" t="s">
         <v>224</v>
@@ -4880,7 +4880,7 @@
         <v>46268.5891771875</v>
       </c>
       <c r="W42">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X42" t="s">
         <v>232</v>
@@ -4960,7 +4960,7 @@
         <v>46267.64795916666</v>
       </c>
       <c r="W43">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X43" t="s">
         <v>228</v>
@@ -5040,7 +5040,7 @@
         <v>46267.4478849537</v>
       </c>
       <c r="W44">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X44" t="s">
         <v>226</v>
@@ -5120,7 +5120,7 @@
         <v>46269.59056300926</v>
       </c>
       <c r="W45">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X45" t="s">
         <v>225</v>
@@ -5197,7 +5197,7 @@
         <v>46273.67026252315</v>
       </c>
       <c r="W46">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X46" t="s">
         <v>229</v>
@@ -5271,7 +5271,7 @@
         <v>46269.677524375</v>
       </c>
       <c r="W47">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X47" t="s">
         <v>230</v>
@@ -5345,7 +5345,7 @@
         <v>46269.677525</v>
       </c>
       <c r="W48">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X48" t="s">
         <v>224</v>
@@ -5419,7 +5419,7 @@
         <v>46269.677525625</v>
       </c>
       <c r="W49">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X49" t="s">
         <v>224</v>
@@ -5493,7 +5493,7 @@
         <v>46268.58906282407</v>
       </c>
       <c r="W50">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X50" t="s">
         <v>232</v>
@@ -5567,7 +5567,7 @@
         <v>46267.64761306713</v>
       </c>
       <c r="W51">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X51" t="s">
         <v>228</v>
@@ -5644,7 +5644,7 @@
         <v>46273.64957155092</v>
       </c>
       <c r="W52">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X52" t="s">
         <v>226</v>
@@ -5721,7 +5721,7 @@
         <v>46273.39871140046</v>
       </c>
       <c r="W53">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X53" t="s">
         <v>225</v>
@@ -5798,7 +5798,7 @@
         <v>46267.35832805555</v>
       </c>
       <c r="W54">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X54" t="s">
         <v>230</v>
@@ -5878,7 +5878,7 @@
         <v>46268.71229238426</v>
       </c>
       <c r="W55">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X55" t="s">
         <v>224</v>
@@ -5958,7 +5958,7 @@
         <v>46268.71229297454</v>
       </c>
       <c r="W56">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X56" t="s">
         <v>224</v>
@@ -6038,7 +6038,7 @@
         <v>46267.74532275463</v>
       </c>
       <c r="W57">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X57" t="s">
         <v>232</v>
@@ -6118,7 +6118,7 @@
         <v>46269.60160202546</v>
       </c>
       <c r="W58">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X58" t="s">
         <v>229</v>
@@ -6198,7 +6198,7 @@
         <v>46273.64508760416</v>
       </c>
       <c r="W59">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X59" t="s">
         <v>233</v>
@@ -6278,7 +6278,7 @@
         <v>46268.45926839121</v>
       </c>
       <c r="W60">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X60" t="s">
         <v>230</v>
@@ -6358,7 +6358,7 @@
         <v>46269.59250902777</v>
       </c>
       <c r="W61">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X61" t="s">
         <v>224</v>
@@ -6438,7 +6438,7 @@
         <v>46269.5922865625</v>
       </c>
       <c r="W62">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X62" t="s">
         <v>224</v>
@@ -6518,7 +6518,7 @@
         <v>46268.58922707176</v>
       </c>
       <c r="W63">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X63" t="s">
         <v>232</v>
@@ -6598,7 +6598,7 @@
         <v>46267.64800344907</v>
       </c>
       <c r="W64">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X64" t="s">
         <v>228</v>
@@ -6678,7 +6678,7 @@
         <v>46267.44799793982</v>
       </c>
       <c r="W65">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X65" t="s">
         <v>226</v>
@@ -6758,7 +6758,7 @@
         <v>46269.59070487269</v>
       </c>
       <c r="W66">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X66" t="s">
         <v>225</v>
@@ -6838,7 +6838,7 @@
         <v>46269.49635894676</v>
       </c>
       <c r="W67">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X67" t="s">
         <v>230</v>
@@ -6915,7 +6915,7 @@
         <v>46269.63659284722</v>
       </c>
       <c r="W68">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X68" t="s">
         <v>229</v>
@@ -6989,7 +6989,7 @@
         <v>46273.64532122685</v>
       </c>
       <c r="W69">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X69" t="s">
         <v>233</v>
@@ -7063,7 +7063,7 @@
         <v>46268.45929986111</v>
       </c>
       <c r="W70">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X70" t="s">
         <v>230</v>
@@ -7137,7 +7137,7 @@
         <v>46269.5925421875</v>
       </c>
       <c r="W71">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X71" t="s">
         <v>224</v>
@@ -7211,7 +7211,7 @@
         <v>46269.59231454861</v>
       </c>
       <c r="W72">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X72" t="s">
         <v>224</v>
@@ -7285,7 +7285,7 @@
         <v>46268.58932953704</v>
       </c>
       <c r="W73">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X73" t="s">
         <v>232</v>
@@ -7359,7 +7359,7 @@
         <v>46267.648038125</v>
       </c>
       <c r="W74">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X74" t="s">
         <v>228</v>
@@ -7433,7 +7433,7 @@
         <v>46267.44824061343</v>
       </c>
       <c r="W75">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X75" t="s">
         <v>226</v>
@@ -7507,7 +7507,7 @@
         <v>46269.59082328704</v>
       </c>
       <c r="W76">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X76" t="s">
         <v>225</v>
@@ -7569,16 +7569,16 @@
         <v>2026</v>
       </c>
       <c r="R77">
-        <v>18263044</v>
+        <v>18269524</v>
       </c>
       <c r="U77" t="s">
         <v>221</v>
       </c>
       <c r="V77" s="1">
-        <v>46273.63629708334</v>
+        <v>46273.64318633102</v>
       </c>
       <c r="W77">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X77" t="s">
         <v>225</v>
@@ -7643,16 +7643,16 @@
         <v>2026</v>
       </c>
       <c r="R78">
-        <v>18269524</v>
+        <v>18269550</v>
       </c>
       <c r="U78" t="s">
         <v>221</v>
       </c>
       <c r="V78" s="1">
-        <v>46273.64318633102</v>
+        <v>46273.64880981482</v>
       </c>
       <c r="W78">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X78" t="s">
         <v>225</v>
@@ -7717,16 +7717,16 @@
         <v>2026</v>
       </c>
       <c r="R79">
-        <v>18269550</v>
+        <v>18263044</v>
       </c>
       <c r="U79" t="s">
         <v>221</v>
       </c>
       <c r="V79" s="1">
-        <v>46273.64880981482</v>
+        <v>46273.63629708334</v>
       </c>
       <c r="W79">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X79" t="s">
         <v>225</v>
@@ -7803,7 +7803,7 @@
         <v>46267.72055925926</v>
       </c>
       <c r="W80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X80" t="s">
         <v>223</v>
@@ -7877,7 +7877,7 @@
         <v>46267.79441380787</v>
       </c>
       <c r="W81">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X81" t="s">
         <v>224</v>
@@ -7948,7 +7948,7 @@
         <v>46267.79441215278</v>
       </c>
       <c r="W82">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X82" t="s">
         <v>225</v>
@@ -8022,7 +8022,7 @@
         <v>46267.7205502662</v>
       </c>
       <c r="W83">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X83" t="s">
         <v>223</v>
@@ -8096,7 +8096,7 @@
         <v>46267.79439748843</v>
       </c>
       <c r="W84">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X84" t="s">
         <v>224</v>
@@ -8167,7 +8167,7 @@
         <v>46267.79440011574</v>
       </c>
       <c r="W85">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X85" t="s">
         <v>226</v>
@@ -8238,7 +8238,7 @@
         <v>46267.79439818287</v>
       </c>
       <c r="W86">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X86" t="s">
         <v>225</v>
@@ -8309,7 +8309,7 @@
         <v>46267.7202693287</v>
       </c>
       <c r="W87">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X87" t="s">
         <v>223</v>
@@ -8383,7 +8383,7 @@
         <v>46267.79409846065</v>
       </c>
       <c r="W88">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X88" t="s">
         <v>224</v>
@@ -8457,7 +8457,7 @@
         <v>46267.79409725694</v>
       </c>
       <c r="W89">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X89" t="s">
         <v>224</v>
@@ -8525,7 +8525,7 @@
         <v>46267.79410239583</v>
       </c>
       <c r="W90">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X90" t="s">
         <v>226</v>
@@ -8593,7 +8593,7 @@
         <v>46267.79409934028</v>
       </c>
       <c r="W91">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X91" t="s">
         <v>225</v>
@@ -8664,7 +8664,7 @@
         <v>46267.72033356482</v>
       </c>
       <c r="W92">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X92" t="s">
         <v>223</v>
@@ -8738,7 +8738,7 @@
         <v>46267.79418105324</v>
       </c>
       <c r="W93">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X93" t="s">
         <v>224</v>
@@ -8812,7 +8812,7 @@
         <v>46267.79418005787</v>
       </c>
       <c r="W94">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X94" t="s">
         <v>224</v>
@@ -8880,7 +8880,7 @@
         <v>46267.79418379629</v>
       </c>
       <c r="W95">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X95" t="s">
         <v>226</v>
@@ -8948,7 +8948,7 @@
         <v>46267.79418283565</v>
       </c>
       <c r="W96">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X96" t="s">
         <v>225</v>
@@ -9019,7 +9019,7 @@
         <v>46267.71937662037</v>
       </c>
       <c r="W97">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X97" t="s">
         <v>223</v>
@@ -9093,7 +9093,7 @@
         <v>46267.79259834491</v>
       </c>
       <c r="W98">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X98" t="s">
         <v>224</v>
@@ -9164,7 +9164,7 @@
         <v>46267.79260170139</v>
       </c>
       <c r="W99">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X99" t="s">
         <v>225</v>
@@ -9241,7 +9241,7 @@
         <v>46268.37621265047</v>
       </c>
       <c r="W100">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X100" t="s">
         <v>227</v>
@@ -9318,7 +9318,7 @@
         <v>46267.79440636574</v>
       </c>
       <c r="W101">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X101" t="s">
         <v>226</v>
@@ -9392,7 +9392,7 @@
         <v>46267.72037954861</v>
       </c>
       <c r="W102">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X102" t="s">
         <v>223</v>
@@ -9466,7 +9466,7 @@
         <v>46267.79424664352</v>
       </c>
       <c r="W103">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X103" t="s">
         <v>224</v>
@@ -9540,7 +9540,7 @@
         <v>46267.79424586806</v>
       </c>
       <c r="W104">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X104" t="s">
         <v>224</v>
@@ -9608,7 +9608,7 @@
         <v>46267.79424864583</v>
       </c>
       <c r="W105">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X105" t="s">
         <v>226</v>
@@ -9676,7 +9676,7 @@
         <v>46267.79424725694</v>
       </c>
       <c r="W106">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X106" t="s">
         <v>225</v>
@@ -9747,7 +9747,7 @@
         <v>46267.79425081018</v>
       </c>
       <c r="W107">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X107" t="s">
         <v>227</v>
@@ -9821,7 +9821,7 @@
         <v>46267.71942916667</v>
       </c>
       <c r="W108">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X108" t="s">
         <v>223</v>
@@ -9895,7 +9895,7 @@
         <v>46267.79268530093</v>
       </c>
       <c r="W109">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X109" t="s">
         <v>226</v>
@@ -9966,7 +9966,7 @@
         <v>46267.79268769676</v>
       </c>
       <c r="W110">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X110" t="s">
         <v>225</v>
@@ -10040,7 +10040,7 @@
         <v>46267.79249748842</v>
       </c>
       <c r="W111">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X111" t="s">
         <v>226</v>
@@ -10111,7 +10111,7 @@
         <v>46267.79249788194</v>
       </c>
       <c r="W112">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X112" t="s">
         <v>225</v>
@@ -10185,7 +10185,7 @@
         <v>46267.71927280092</v>
       </c>
       <c r="W113">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X113" t="s">
         <v>223</v>
@@ -10259,7 +10259,7 @@
         <v>46267.79251079861</v>
       </c>
       <c r="W114">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X114" t="s">
         <v>226</v>
@@ -10330,7 +10330,7 @@
         <v>46267.79251038194</v>
       </c>
       <c r="W115">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X115" t="s">
         <v>225</v>
@@ -10404,7 +10404,7 @@
         <v>46267.72044811342</v>
       </c>
       <c r="W116">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X116" t="s">
         <v>223</v>
@@ -10478,7 +10478,7 @@
         <v>46267.79429737268</v>
       </c>
       <c r="W117">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X117" t="s">
         <v>224</v>
@@ -10552,7 +10552,7 @@
         <v>46267.79429603009</v>
       </c>
       <c r="W118">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X118" t="s">
         <v>224</v>
@@ -10620,7 +10620,7 @@
         <v>46267.79429876158</v>
       </c>
       <c r="W119">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X119" t="s">
         <v>226</v>
@@ -10688,7 +10688,7 @@
         <v>46267.79429826389</v>
       </c>
       <c r="W120">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X120" t="s">
         <v>225</v>
@@ -10759,7 +10759,7 @@
         <v>46267.72050385417</v>
       </c>
       <c r="W121">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X121" t="s">
         <v>223</v>
@@ -10833,7 +10833,7 @@
         <v>46267.79434996528</v>
       </c>
       <c r="W122">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X122" t="s">
         <v>224</v>
@@ -10907,7 +10907,7 @@
         <v>46267.79434864583</v>
       </c>
       <c r="W123">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X123" t="s">
         <v>224</v>
@@ -10975,7 +10975,7 @@
         <v>46267.79435208334</v>
       </c>
       <c r="W124">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X124" t="s">
         <v>226</v>
@@ -11043,7 +11043,7 @@
         <v>46267.79435100695</v>
       </c>
       <c r="W125">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X125" t="s">
         <v>225</v>
@@ -11114,7 +11114,7 @@
         <v>46273.6788224074</v>
       </c>
       <c r="W126">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X126" t="s">
         <v>225</v>
@@ -11191,7 +11191,7 @@
         <v>46273.67943539352</v>
       </c>
       <c r="W127">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X127" t="s">
         <v>225</v>
@@ -11268,7 +11268,7 @@
         <v>46266.37636392361</v>
       </c>
       <c r="W128">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X128" t="s">
         <v>229</v>
@@ -11342,7 +11342,7 @@
         <v>46266.37598834491</v>
       </c>
       <c r="W129">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X129" t="s">
         <v>229</v>
@@ -11419,7 +11419,7 @@
         <v>46268.45899988426</v>
       </c>
       <c r="W130">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X130" t="s">
         <v>230</v>
@@ -11496,7 +11496,7 @@
         <v>46266.45957881944</v>
       </c>
       <c r="W131">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X131" t="s">
         <v>228</v>
@@ -11570,7 +11570,7 @@
         <v>46266.37645462963</v>
       </c>
       <c r="W132">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X132" t="s">
         <v>229</v>
@@ -11644,7 +11644,7 @@
         <v>46266.37649475694</v>
       </c>
       <c r="W133">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X133" t="s">
         <v>229</v>
@@ -11718,7 +11718,7 @@
         <v>46266.37591180555</v>
       </c>
       <c r="W134">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X134" t="s">
         <v>229</v>
@@ -11795,7 +11795,7 @@
         <v>46268.45896508102</v>
       </c>
       <c r="W135">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X135" t="s">
         <v>230</v>
@@ -11872,7 +11872,7 @@
         <v>46266.45946195602</v>
       </c>
       <c r="W136">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X136" t="s">
         <v>228</v>
@@ -11946,7 +11946,7 @@
         <v>46266.37538684028</v>
       </c>
       <c r="W137">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X137" t="s">
         <v>229</v>
@@ -12020,7 +12020,7 @@
         <v>46266.37538506944</v>
       </c>
       <c r="W138">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X138" t="s">
         <v>233</v>
@@ -12097,7 +12097,7 @@
         <v>46268.45881820602</v>
       </c>
       <c r="W139">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X139" t="s">
         <v>230</v>
@@ -12174,7 +12174,7 @@
         <v>46266.45895332176</v>
       </c>
       <c r="W140">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X140" t="s">
         <v>232</v>
@@ -12248,7 +12248,7 @@
         <v>46266.45874105324</v>
       </c>
       <c r="W141">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X141" t="s">
         <v>228</v>
@@ -12322,7 +12322,7 @@
         <v>46266.45873584491</v>
       </c>
       <c r="W142">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X142" t="s">
         <v>228</v>
@@ -12396,7 +12396,7 @@
         <v>46273.6799675</v>
       </c>
       <c r="W143">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X143" t="s">
         <v>228</v>
@@ -12470,7 +12470,7 @@
         <v>46273.55254606481</v>
       </c>
       <c r="W144">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X144" t="s">
         <v>229</v>
@@ -12544,7 +12544,7 @@
         <v>46273.55252126158</v>
       </c>
       <c r="W145">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X145" t="s">
         <v>233</v>
@@ -12618,7 +12618,7 @@
         <v>46273.55254163194</v>
       </c>
       <c r="W146">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X146" t="s">
         <v>230</v>
@@ -12692,7 +12692,7 @@
         <v>46273.5525440162</v>
       </c>
       <c r="W147">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X147" t="s">
         <v>232</v>
@@ -12766,7 +12766,7 @@
         <v>46273.84422141204</v>
       </c>
       <c r="W148">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X148" t="s">
         <v>228</v>
@@ -12840,7 +12840,7 @@
         <v>46273.55254652778</v>
       </c>
       <c r="W149">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X149" t="s">
         <v>228</v>
@@ -12917,7 +12917,7 @@
         <v>46268.45898549769</v>
       </c>
       <c r="W150">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="X150" t="s">
         <v>230</v>
@@ -12994,7 +12994,7 @@
         <v>46268.45915543981</v>
       </c>
       <c r="W151">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X151" t="s">
         <v>230</v>
@@ -13068,7 +13068,7 @@
         <v>46273.56305208334</v>
       </c>
       <c r="W152">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X152" t="s">
         <v>228</v>
@@ -13142,7 +13142,7 @@
         <v>46267.44505795139</v>
       </c>
       <c r="W153">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X153" t="s">
         <v>228</v>
@@ -13213,7 +13213,7 @@
         <v>46266.25305112269</v>
       </c>
       <c r="W154">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X154" t="s">
         <v>229</v>
@@ -13287,7 +13287,7 @@
         <v>46266.25275173611</v>
       </c>
       <c r="W155">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X155" t="s">
         <v>224</v>
@@ -13361,7 +13361,7 @@
         <v>46266.25364869213</v>
       </c>
       <c r="W156">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X156" t="s">
         <v>228</v>
@@ -13435,7 +13435,7 @@
         <v>46266.25369988426</v>
       </c>
       <c r="W157">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X157" t="s">
         <v>225</v>
@@ -13512,7 +13512,7 @@
         <v>46268.62318445602</v>
       </c>
       <c r="W158">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X158" t="s">
         <v>229</v>
@@ -13589,7 +13589,7 @@
         <v>46268.62319864584</v>
       </c>
       <c r="W159">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X159" t="s">
         <v>233</v>
@@ -13666,7 +13666,7 @@
         <v>46268.62320026621</v>
       </c>
       <c r="W160">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X160" t="s">
         <v>230</v>
@@ -13743,7 +13743,7 @@
         <v>46268.62320177083</v>
       </c>
       <c r="W161">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X161" t="s">
         <v>223</v>
@@ -13820,7 +13820,7 @@
         <v>46268.62320378472</v>
       </c>
       <c r="W162">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X162" t="s">
         <v>224</v>
@@ -13897,7 +13897,7 @@
         <v>46268.62320393518</v>
       </c>
       <c r="W163">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X163" t="s">
         <v>224</v>
@@ -13974,7 +13974,7 @@
         <v>46268.62320697917</v>
       </c>
       <c r="W164">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X164" t="s">
         <v>232</v>
@@ -14051,7 +14051,7 @@
         <v>46268.62320717592</v>
       </c>
       <c r="W165">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X165" t="s">
         <v>228</v>
@@ -14128,7 +14128,7 @@
         <v>46268.62320732639</v>
       </c>
       <c r="W166">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X166" t="s">
         <v>228</v>
@@ -14205,7 +14205,7 @@
         <v>46268.62320810185</v>
       </c>
       <c r="W167">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X167" t="s">
         <v>228</v>
@@ -14282,7 +14282,7 @@
         <v>46268.6232125</v>
       </c>
       <c r="W168">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X168" t="s">
         <v>226</v>
@@ -14359,7 +14359,7 @@
         <v>46268.62321412037</v>
       </c>
       <c r="W169">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X169" t="s">
         <v>225</v>
@@ -14436,7 +14436,7 @@
         <v>46268.6232128125</v>
       </c>
       <c r="W170">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X170" t="s">
         <v>227</v>
@@ -14513,7 +14513,7 @@
         <v>46268.62321296296</v>
       </c>
       <c r="W171">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X171" t="s">
         <v>227</v>
@@ -14587,7 +14587,7 @@
         <v>46269.41908927084</v>
       </c>
       <c r="W172">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X172" t="s">
         <v>229</v>
@@ -14658,7 +14658,7 @@
         <v>46269.41910457176</v>
       </c>
       <c r="W173">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X173" t="s">
         <v>233</v>
@@ -14729,7 +14729,7 @@
         <v>46269.37885223379</v>
       </c>
       <c r="W174">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X174" t="s">
         <v>230</v>
@@ -14800,7 +14800,7 @@
         <v>46269.3782503125</v>
       </c>
       <c r="W175">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X175" t="s">
         <v>223</v>
@@ -14871,7 +14871,7 @@
         <v>46269.41913152778</v>
       </c>
       <c r="W176">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X176" t="s">
         <v>224</v>
@@ -14942,7 +14942,7 @@
         <v>46269.41913775463</v>
       </c>
       <c r="W177">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X177" t="s">
         <v>224</v>
@@ -15013,7 +15013,7 @@
         <v>46268.7596207176</v>
       </c>
       <c r="W178">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X178" t="s">
         <v>229</v>
@@ -15084,7 +15084,7 @@
         <v>46268.75963109954</v>
       </c>
       <c r="W179">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X179" t="s">
         <v>233</v>
@@ -15155,7 +15155,7 @@
         <v>46268.75963225694</v>
       </c>
       <c r="W180">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X180" t="s">
         <v>230</v>
@@ -15226,7 +15226,7 @@
         <v>46268.75963348379</v>
       </c>
       <c r="W181">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X181" t="s">
         <v>223</v>
@@ -15297,7 +15297,7 @@
         <v>46268.75963414352</v>
       </c>
       <c r="W182">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X182" t="s">
         <v>224</v>
@@ -15368,7 +15368,7 @@
         <v>46268.62326365741</v>
       </c>
       <c r="W183">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X183" t="s">
         <v>224</v>
@@ -15439,7 +15439,7 @@
         <v>46268.75963472222</v>
       </c>
       <c r="W184">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X184" t="s">
         <v>232</v>
@@ -15510,7 +15510,7 @@
         <v>46268.75963475694</v>
       </c>
       <c r="W185">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X185" t="s">
         <v>228</v>
@@ -15581,7 +15581,7 @@
         <v>46268.75963506944</v>
       </c>
       <c r="W186">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X186" t="s">
         <v>228</v>
@@ -15652,7 +15652,7 @@
         <v>46268.7596360301</v>
       </c>
       <c r="W187">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X187" t="s">
         <v>228</v>
@@ -15723,7 +15723,7 @@
         <v>46268.62327121528</v>
       </c>
       <c r="W188">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X188" t="s">
         <v>226</v>
@@ -15794,7 +15794,7 @@
         <v>46268.75963931713</v>
       </c>
       <c r="W189">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X189" t="s">
         <v>225</v>
@@ -15865,7 +15865,7 @@
         <v>46268.75963822917</v>
       </c>
       <c r="W190">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X190" t="s">
         <v>227</v>
@@ -15936,7 +15936,7 @@
         <v>46268.75963857639</v>
       </c>
       <c r="W191">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X191" t="s">
         <v>227</v>
@@ -16007,7 +16007,7 @@
         <v>46269.41908901621</v>
       </c>
       <c r="W192">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X192" t="s">
         <v>229</v>
@@ -16078,7 +16078,7 @@
         <v>46269.41910425926</v>
       </c>
       <c r="W193">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X193" t="s">
         <v>233</v>
@@ -16149,7 +16149,7 @@
         <v>46269.37890997685</v>
       </c>
       <c r="W194">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X194" t="s">
         <v>230</v>
@@ -16220,7 +16220,7 @@
         <v>46269.37833320602</v>
       </c>
       <c r="W195">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X195" t="s">
         <v>223</v>
@@ -16291,7 +16291,7 @@
         <v>46269.41913112268</v>
       </c>
       <c r="W196">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X196" t="s">
         <v>224</v>
@@ -16362,7 +16362,7 @@
         <v>46269.41913740741</v>
       </c>
       <c r="W197">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X197" t="s">
         <v>224</v>
@@ -16433,7 +16433,7 @@
         <v>46267.66131466435</v>
       </c>
       <c r="W198">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X198" t="s">
         <v>233</v>
@@ -16507,7 +16507,7 @@
         <v>46266.21595836805</v>
       </c>
       <c r="W199">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="X199" t="s">
         <v>233</v>
@@ -16581,7 +16581,7 @@
         <v>46266.21572962963</v>
       </c>
       <c r="W200">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="X200" t="s">
         <v>229</v>
@@ -16655,7 +16655,7 @@
         <v>46266.21550011574</v>
       </c>
       <c r="W201">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="X201" t="s">
         <v>230</v>
@@ -16729,7 +16729,7 @@
         <v>46266.00006921296</v>
       </c>
       <c r="W202">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="X202" t="s">
         <v>229</v>
@@ -16800,7 +16800,7 @@
         <v>46266.00006921296</v>
       </c>
       <c r="W203">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="X203" t="s">
         <v>233</v>
@@ -16868,7 +16868,7 @@
         <v>46269.57097615741</v>
       </c>
       <c r="W204">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X204" t="s">
         <v>230</v>
@@ -16936,7 +16936,7 @@
         <v>46266.00006921296</v>
       </c>
       <c r="W205">
-        <v>-32</v>
+        <v>-31</v>
       </c>
       <c r="X205" t="s">
         <v>230</v>
@@ -17004,7 +17004,7 @@
         <v>46269.46753030093</v>
       </c>
       <c r="W206">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X206" t="s">
         <v>226</v>
@@ -17081,7 +17081,7 @@
         <v>46280.37528408565</v>
       </c>
       <c r="W207">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X207" t="s">
         <v>229</v>
@@ -17158,7 +17158,7 @@
         <v>46281.63558861111</v>
       </c>
       <c r="W208">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X208" t="s">
         <v>224</v>
@@ -17238,7 +17238,7 @@
         <v>46281.6358927662</v>
       </c>
       <c r="W209">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X209" t="s">
         <v>224</v>
@@ -17318,7 +17318,7 @@
         <v>46281.47564895833</v>
       </c>
       <c r="W210">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X210" t="s">
         <v>226</v>
@@ -17398,7 +17398,7 @@
         <v>46279.66710767361</v>
       </c>
       <c r="W211">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X211" t="s">
         <v>228</v>
@@ -17478,7 +17478,7 @@
         <v>46281.68877074074</v>
       </c>
       <c r="W212">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X212" t="s">
         <v>230</v>
@@ -17558,7 +17558,7 @@
         <v>46280.57958537037</v>
       </c>
       <c r="W213">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X213" t="s">
         <v>223</v>
@@ -17638,7 +17638,7 @@
         <v>46281.63570936343</v>
       </c>
       <c r="W214">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X214" t="s">
         <v>224</v>
@@ -17718,7 +17718,7 @@
         <v>46281.63595871528</v>
       </c>
       <c r="W215">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X215" t="s">
         <v>224</v>
@@ -17795,7 +17795,7 @@
         <v>46279.62681744213</v>
       </c>
       <c r="W216">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X216" t="s">
         <v>232</v>
@@ -17869,7 +17869,7 @@
         <v>46279.66707821759</v>
       </c>
       <c r="W217">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X217" t="s">
         <v>228</v>
@@ -17946,7 +17946,7 @@
         <v>46281.68880230324</v>
       </c>
       <c r="W218">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X218" t="s">
         <v>230</v>
@@ -18026,7 +18026,7 @@
         <v>46280.57972293982</v>
       </c>
       <c r="W219">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X219" t="s">
         <v>223</v>
@@ -18106,7 +18106,7 @@
         <v>46281.63575075231</v>
       </c>
       <c r="W220">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X220" t="s">
         <v>224</v>
@@ -18186,7 +18186,7 @@
         <v>46281.63599785879</v>
       </c>
       <c r="W221">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X221" t="s">
         <v>224</v>
@@ -18263,7 +18263,7 @@
         <v>46279.6268503125</v>
       </c>
       <c r="W222">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X222" t="s">
         <v>232</v>
@@ -18337,7 +18337,7 @@
         <v>46279.66698128472</v>
       </c>
       <c r="W223">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X223" t="s">
         <v>228</v>
@@ -18411,7 +18411,7 @@
         <v>46279.66929922454</v>
       </c>
       <c r="W224">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X224" t="s">
         <v>229</v>
@@ -18488,7 +18488,7 @@
         <v>46280.61353684028</v>
       </c>
       <c r="W225">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X225" t="s">
         <v>233</v>
@@ -18565,7 +18565,7 @@
         <v>46280.61353920139</v>
       </c>
       <c r="W226">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X226" t="s">
         <v>230</v>
@@ -18642,7 +18642,7 @@
         <v>46279.63250563657</v>
       </c>
       <c r="W227">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X227" t="s">
         <v>223</v>
@@ -18719,7 +18719,7 @@
         <v>46280.61354019676</v>
       </c>
       <c r="W228">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X228" t="s">
         <v>224</v>
@@ -18796,7 +18796,7 @@
         <v>46280.6135403125</v>
       </c>
       <c r="W229">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X229" t="s">
         <v>224</v>
@@ -18876,7 +18876,7 @@
         <v>46281.71218414352</v>
       </c>
       <c r="W230">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X230" t="s">
         <v>232</v>
@@ -18953,7 +18953,7 @@
         <v>46281.41576883102</v>
       </c>
       <c r="W231">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X231" t="s">
         <v>228</v>
@@ -19030,7 +19030,7 @@
         <v>46280.43132989584</v>
       </c>
       <c r="W232">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X232" t="s">
         <v>226</v>
@@ -19107,7 +19107,7 @@
         <v>46280.61367623843</v>
       </c>
       <c r="W233">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X233" t="s">
         <v>225</v>
@@ -19187,7 +19187,7 @@
         <v>46274.60593387731</v>
       </c>
       <c r="W234">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X234" t="s">
         <v>229</v>
@@ -19267,7 +19267,7 @@
         <v>46274.47210818287</v>
       </c>
       <c r="W235">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X235" t="s">
         <v>230</v>
@@ -19347,7 +19347,7 @@
         <v>46276.48975401621</v>
       </c>
       <c r="W236">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X236" t="s">
         <v>224</v>
@@ -19427,7 +19427,7 @@
         <v>46279.38429019676</v>
       </c>
       <c r="W237">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X237" t="s">
         <v>224</v>
@@ -19507,7 +19507,7 @@
         <v>46274.48792050926</v>
       </c>
       <c r="W238">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X238" t="s">
         <v>228</v>
@@ -19587,7 +19587,7 @@
         <v>46274.588374375</v>
       </c>
       <c r="W239">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X239" t="s">
         <v>226</v>
@@ -19664,7 +19664,7 @@
         <v>46274.34198912037</v>
       </c>
       <c r="W240">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X240" t="s">
         <v>225</v>
@@ -19738,7 +19738,7 @@
         <v>46279.6693627662</v>
       </c>
       <c r="W241">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X241" t="s">
         <v>229</v>
@@ -19818,7 +19818,7 @@
         <v>46279.5886965625</v>
       </c>
       <c r="W242">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X242" t="s">
         <v>230</v>
@@ -19895,7 +19895,7 @@
         <v>46279.40189383102</v>
       </c>
       <c r="W243">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X243" t="s">
         <v>223</v>
@@ -19975,7 +19975,7 @@
         <v>46279.58878520833</v>
       </c>
       <c r="W244">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X244" t="s">
         <v>224</v>
@@ -20055,7 +20055,7 @@
         <v>46279.58873577546</v>
       </c>
       <c r="W245">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X245" t="s">
         <v>224</v>
@@ -20132,7 +20132,7 @@
         <v>46279.63255</v>
       </c>
       <c r="W246">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X246" t="s">
         <v>232</v>
@@ -20209,7 +20209,7 @@
         <v>46276.63187557871</v>
       </c>
       <c r="W247">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X247" t="s">
         <v>228</v>
@@ -20286,7 +20286,7 @@
         <v>46279.6265846875</v>
       </c>
       <c r="W248">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X248" t="s">
         <v>226</v>
@@ -20363,7 +20363,7 @@
         <v>46279.63255401621</v>
       </c>
       <c r="W249">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X249" t="s">
         <v>225</v>
@@ -20443,7 +20443,7 @@
         <v>46279.66713805556</v>
       </c>
       <c r="W250">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X250" t="s">
         <v>228</v>
@@ -20517,7 +20517,7 @@
         <v>46281.63317659722</v>
       </c>
       <c r="W251">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X251" t="s">
         <v>230</v>
@@ -20591,7 +20591,7 @@
         <v>46275.39631951389</v>
       </c>
       <c r="W252">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X252" t="s">
         <v>224</v>
@@ -20665,7 +20665,7 @@
         <v>46275.39631994213</v>
       </c>
       <c r="W253">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X253" t="s">
         <v>224</v>
@@ -20745,7 +20745,7 @@
         <v>46280.62789608796</v>
       </c>
       <c r="W254">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X254" t="s">
         <v>227</v>
@@ -20825,7 +20825,7 @@
         <v>46280.63189497685</v>
       </c>
       <c r="W255">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X255" t="s">
         <v>227</v>
@@ -20905,7 +20905,7 @@
         <v>46280.72961366898</v>
       </c>
       <c r="W256">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X256" t="s">
         <v>224</v>
@@ -20982,7 +20982,7 @@
         <v>46276.37795540509</v>
       </c>
       <c r="W257">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X257" t="s">
         <v>226</v>
@@ -21059,7 +21059,7 @@
         <v>46276.66923222222</v>
       </c>
       <c r="W258">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X258" t="s">
         <v>223</v>
@@ -21136,7 +21136,7 @@
         <v>46276.40669469907</v>
       </c>
       <c r="W259">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X259" t="s">
         <v>224</v>
@@ -21213,7 +21213,7 @@
         <v>46276.64773491898</v>
       </c>
       <c r="W260">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X260" t="s">
         <v>224</v>
@@ -21293,7 +21293,7 @@
         <v>46276.39101108797</v>
       </c>
       <c r="W261">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X261" t="s">
         <v>226</v>
@@ -21370,7 +21370,7 @@
         <v>46280.40395534722</v>
       </c>
       <c r="W262">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X262" t="s">
         <v>225</v>
@@ -21447,7 +21447,7 @@
         <v>46279.74982357639</v>
       </c>
       <c r="W263">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X263" t="s">
         <v>227</v>
@@ -21527,7 +21527,7 @@
         <v>46276.66651596065</v>
       </c>
       <c r="W264">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X264" t="s">
         <v>227</v>
@@ -21604,7 +21604,7 @@
         <v>46280.66345891204</v>
       </c>
       <c r="W265">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X265" t="s">
         <v>224</v>
@@ -21681,7 +21681,7 @@
         <v>46274.36843923611</v>
       </c>
       <c r="W266">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X266" t="s">
         <v>224</v>
@@ -21758,7 +21758,7 @@
         <v>46274.66470667824</v>
       </c>
       <c r="W267">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X267" t="s">
         <v>227</v>
@@ -21835,7 +21835,7 @@
         <v>46274.74452168981</v>
       </c>
       <c r="W268">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X268" t="s">
         <v>227</v>
@@ -21915,7 +21915,7 @@
         <v>46274.64801501157</v>
       </c>
       <c r="W269">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X269" t="s">
         <v>223</v>
@@ -21992,7 +21992,7 @@
         <v>46274.36695243056</v>
       </c>
       <c r="W270">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X270" t="s">
         <v>224</v>
@@ -22069,7 +22069,7 @@
         <v>46276.4084265625</v>
       </c>
       <c r="W271">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X271" t="s">
         <v>226</v>
@@ -22146,7 +22146,7 @@
         <v>46274.7274781713</v>
       </c>
       <c r="W272">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X272" t="s">
         <v>227</v>
@@ -22220,7 +22220,7 @@
         <v>46274.74558746528</v>
       </c>
       <c r="W273">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X273" t="s">
         <v>227</v>
@@ -22291,7 +22291,7 @@
         <v>46275.79245582176</v>
       </c>
       <c r="W274">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X274" t="s">
         <v>225</v>
@@ -22368,7 +22368,7 @@
         <v>46280.63707425926</v>
       </c>
       <c r="W275">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X275" t="s">
         <v>224</v>
@@ -22448,7 +22448,7 @@
         <v>46280.38311703704</v>
       </c>
       <c r="W276">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X276" t="s">
         <v>226</v>
@@ -22525,7 +22525,7 @@
         <v>46280.37743127315</v>
       </c>
       <c r="W277">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X277" t="s">
         <v>225</v>
@@ -22605,7 +22605,7 @@
         <v>46280.45035295139</v>
       </c>
       <c r="W278">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X278" t="s">
         <v>230</v>
@@ -22682,7 +22682,7 @@
         <v>46280.59788275463</v>
       </c>
       <c r="W279">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X279" t="s">
         <v>230</v>
@@ -22762,7 +22762,7 @@
         <v>46280.73313407407</v>
       </c>
       <c r="W280">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X280" t="s">
         <v>228</v>
@@ -22839,7 +22839,7 @@
         <v>46276.49596842592</v>
       </c>
       <c r="W281">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X281" t="s">
         <v>229</v>
@@ -22913,7 +22913,7 @@
         <v>46276.53874935185</v>
       </c>
       <c r="W282">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X282" t="s">
         <v>233</v>
@@ -22987,7 +22987,7 @@
         <v>46276.49597027778</v>
       </c>
       <c r="W283">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X283" t="s">
         <v>230</v>
@@ -23061,7 +23061,7 @@
         <v>46276.62604146991</v>
       </c>
       <c r="W284">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X284" t="s">
         <v>232</v>
@@ -23135,7 +23135,7 @@
         <v>46276.68231165509</v>
       </c>
       <c r="W285">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X285" t="s">
         <v>228</v>
@@ -23212,7 +23212,7 @@
         <v>46276.7163278588</v>
       </c>
       <c r="W286">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X286" t="s">
         <v>228</v>
@@ -23289,7 +23289,7 @@
         <v>46276.6823121412</v>
       </c>
       <c r="W287">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X287" t="s">
         <v>228</v>
@@ -23366,7 +23366,7 @@
         <v>46280.69323744213</v>
       </c>
       <c r="W288">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X288" t="s">
         <v>229</v>
@@ -23443,7 +23443,7 @@
         <v>46274.70622837963</v>
       </c>
       <c r="W289">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X289" t="s">
         <v>233</v>
@@ -23517,7 +23517,7 @@
         <v>46275.71996309028</v>
       </c>
       <c r="W290">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X290" t="s">
         <v>232</v>
@@ -23591,7 +23591,7 @@
         <v>46275.54278886574</v>
       </c>
       <c r="W291">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X291" t="s">
         <v>228</v>
@@ -23668,7 +23668,7 @@
         <v>46280.74859975695</v>
       </c>
       <c r="W292">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X292" t="s">
         <v>229</v>
@@ -23745,7 +23745,7 @@
         <v>46275.7000328588</v>
       </c>
       <c r="W293">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X293" t="s">
         <v>233</v>
@@ -23819,7 +23819,7 @@
         <v>46275.72031699074</v>
       </c>
       <c r="W294">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X294" t="s">
         <v>230</v>
@@ -23893,7 +23893,7 @@
         <v>46275.54095912037</v>
       </c>
       <c r="W295">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X295" t="s">
         <v>232</v>
@@ -23967,7 +23967,7 @@
         <v>46275.72225363426</v>
       </c>
       <c r="W296">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X296" t="s">
         <v>228</v>
@@ -24041,7 +24041,7 @@
         <v>46275.7222629051</v>
       </c>
       <c r="W297">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X297" t="s">
         <v>228</v>
@@ -24115,7 +24115,7 @@
         <v>46275.7222709838</v>
       </c>
       <c r="W298">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X298" t="s">
         <v>228</v>
@@ -24192,7 +24192,7 @@
         <v>46274.74837762731</v>
       </c>
       <c r="W299">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X299" t="s">
         <v>229</v>
@@ -24272,7 +24272,7 @@
         <v>46274.74838096065</v>
       </c>
       <c r="W300">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X300" t="s">
         <v>232</v>
@@ -24352,7 +24352,7 @@
         <v>46280.56274502315</v>
       </c>
       <c r="W301">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X301" t="s">
         <v>228</v>
@@ -24429,7 +24429,7 @@
         <v>46274.42878043981</v>
       </c>
       <c r="W302">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X302" t="s">
         <v>229</v>
@@ -24506,7 +24506,7 @@
         <v>46275.40196778935</v>
       </c>
       <c r="W303">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X303" t="s">
         <v>230</v>
@@ -24583,7 +24583,7 @@
         <v>46276.52399603009</v>
       </c>
       <c r="W304">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X304" t="s">
         <v>232</v>
@@ -24660,7 +24660,7 @@
         <v>46276.5240703125</v>
       </c>
       <c r="W305">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X305" t="s">
         <v>228</v>
@@ -24734,7 +24734,7 @@
         <v>46275.4100730787</v>
       </c>
       <c r="W306">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X306" t="s">
         <v>225</v>
@@ -24808,7 +24808,7 @@
         <v>46275.40964188657</v>
       </c>
       <c r="W307">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X307" t="s">
         <v>227</v>
@@ -24882,7 +24882,7 @@
         <v>46275.40964245371</v>
       </c>
       <c r="W308">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X308" t="s">
         <v>227</v>
@@ -24956,7 +24956,7 @@
         <v>46275.45011145833</v>
       </c>
       <c r="W309">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X309" t="s">
         <v>223</v>
@@ -25030,7 +25030,7 @@
         <v>46275.44901016204</v>
       </c>
       <c r="W310">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X310" t="s">
         <v>224</v>
@@ -25104,7 +25104,7 @@
         <v>46276.71732053241</v>
       </c>
       <c r="W311">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X311" t="s">
         <v>232</v>
@@ -25181,7 +25181,7 @@
         <v>46276.71697232639</v>
       </c>
       <c r="W312">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X312" t="s">
         <v>228</v>
@@ -25258,7 +25258,7 @@
         <v>46276.7175884838</v>
       </c>
       <c r="W313">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X313" t="s">
         <v>228</v>
@@ -25335,7 +25335,7 @@
         <v>46276.7175895949</v>
       </c>
       <c r="W314">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X314" t="s">
         <v>228</v>
@@ -25412,7 +25412,7 @@
         <v>46276.71759461806</v>
       </c>
       <c r="W315">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X315" t="s">
         <v>226</v>
@@ -25486,7 +25486,7 @@
         <v>46275.44975668981</v>
       </c>
       <c r="W316">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X316" t="s">
         <v>225</v>
@@ -25560,7 +25560,7 @@
         <v>46275.44933692129</v>
       </c>
       <c r="W317">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X317" t="s">
         <v>227</v>
@@ -25634,7 +25634,7 @@
         <v>46275.44933814815</v>
       </c>
       <c r="W318">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X318" t="s">
         <v>227</v>
@@ -25708,7 +25708,7 @@
         <v>46274.41771849537</v>
       </c>
       <c r="W319">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X319" t="s">
         <v>232</v>
@@ -25779,7 +25779,7 @@
         <v>46274.41775447917</v>
       </c>
       <c r="W320">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X320" t="s">
         <v>228</v>
@@ -25850,7 +25850,7 @@
         <v>46274.41777533565</v>
       </c>
       <c r="W321">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X321" t="s">
         <v>228</v>
@@ -25921,7 +25921,7 @@
         <v>46274.41799166667</v>
       </c>
       <c r="W322">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X322" t="s">
         <v>226</v>
@@ -25992,7 +25992,7 @@
         <v>46274.41800114583</v>
       </c>
       <c r="W323">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X323" t="s">
         <v>225</v>
@@ -26063,7 +26063,7 @@
         <v>46274.41772148148</v>
       </c>
       <c r="W324">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X324" t="s">
         <v>232</v>
@@ -26134,7 +26134,7 @@
         <v>46274.41773631945</v>
       </c>
       <c r="W325">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X325" t="s">
         <v>228</v>
@@ -26205,7 +26205,7 @@
         <v>46274.41777481481</v>
       </c>
       <c r="W326">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X326" t="s">
         <v>228</v>
@@ -26276,7 +26276,7 @@
         <v>46274.41799332176</v>
       </c>
       <c r="W327">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X327" t="s">
         <v>226</v>
@@ -26347,7 +26347,7 @@
         <v>46274.41800085648</v>
       </c>
       <c r="W328">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="X328" t="s">
         <v>225</v>
@@ -26418,7 +26418,7 @@
         <v>46275.31737530093</v>
       </c>
       <c r="W329">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X329" t="s">
         <v>229</v>
@@ -26489,7 +26489,7 @@
         <v>46275.31747032407</v>
       </c>
       <c r="W330">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X330" t="s">
         <v>233</v>
@@ -26560,7 +26560,7 @@
         <v>46275.31747981482</v>
       </c>
       <c r="W331">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X331" t="s">
         <v>230</v>
@@ -26631,7 +26631,7 @@
         <v>46275.31748724537</v>
       </c>
       <c r="W332">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X332" t="s">
         <v>223</v>
@@ -26702,7 +26702,7 @@
         <v>46275.31749535879</v>
       </c>
       <c r="W333">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X333" t="s">
         <v>224</v>
@@ -26773,7 +26773,7 @@
         <v>46275.31750491898</v>
       </c>
       <c r="W334">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X334" t="s">
         <v>232</v>
@@ -26844,7 +26844,7 @@
         <v>46275.31750555555</v>
       </c>
       <c r="W335">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X335" t="s">
         <v>228</v>
@@ -26915,7 +26915,7 @@
         <v>46275.31750599537</v>
       </c>
       <c r="W336">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X336" t="s">
         <v>228</v>
@@ -26986,7 +26986,7 @@
         <v>46275.5810894676</v>
       </c>
       <c r="W337">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X337" t="s">
         <v>229</v>
@@ -27060,7 +27060,7 @@
         <v>46275.58158541666</v>
       </c>
       <c r="W338">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="X338" t="s">
         <v>230</v>
@@ -27134,7 +27134,7 @@
         <v>46276.41675075232</v>
       </c>
       <c r="W339">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X339" t="s">
         <v>224</v>
@@ -27214,7 +27214,7 @@
         <v>46288.76065641204</v>
       </c>
       <c r="W340">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X340" t="s">
         <v>224</v>
@@ -27294,7 +27294,7 @@
         <v>46288.7606568287</v>
       </c>
       <c r="W341">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X341" t="s">
         <v>224</v>
@@ -27374,7 +27374,7 @@
         <v>46288.76066791666</v>
       </c>
       <c r="W342">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X342" t="s">
         <v>225</v>
@@ -27454,7 +27454,7 @@
         <v>46289.64172979166</v>
       </c>
       <c r="W343">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X343" t="s">
         <v>224</v>
@@ -27534,7 +27534,7 @@
         <v>46289.56480809028</v>
       </c>
       <c r="W344">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X344" t="s">
         <v>226</v>
@@ -27611,7 +27611,7 @@
         <v>46288.43167056713</v>
       </c>
       <c r="W345">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X345" t="s">
         <v>226</v>
@@ -27688,7 +27688,7 @@
         <v>46282.62254486111</v>
       </c>
       <c r="W346">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X346" t="s">
         <v>223</v>
@@ -27765,7 +27765,7 @@
         <v>46286.64173940972</v>
       </c>
       <c r="W347">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X347" t="s">
         <v>224</v>
@@ -27842,7 +27842,7 @@
         <v>46283.44840582176</v>
       </c>
       <c r="W348">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X348" t="s">
         <v>225</v>
@@ -27919,7 +27919,7 @@
         <v>46287.48052434028</v>
       </c>
       <c r="W349">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X349" t="s">
         <v>229</v>
@@ -27999,7 +27999,7 @@
         <v>46289.41381568287</v>
       </c>
       <c r="W350">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X350" t="s">
         <v>233</v>
@@ -28079,7 +28079,7 @@
         <v>46289.44878592592</v>
       </c>
       <c r="W351">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X351" t="s">
         <v>230</v>
@@ -28159,7 +28159,7 @@
         <v>46289.44878644676</v>
       </c>
       <c r="W352">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X352" t="s">
         <v>232</v>
@@ -28239,7 +28239,7 @@
         <v>46289.64049288195</v>
       </c>
       <c r="W353">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X353" t="s">
         <v>228</v>
@@ -28319,7 +28319,7 @@
         <v>46289.64073386574</v>
       </c>
       <c r="W354">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X354" t="s">
         <v>228</v>
@@ -28399,7 +28399,7 @@
         <v>46287.48083141204</v>
       </c>
       <c r="W355">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X355" t="s">
         <v>229</v>
@@ -28479,7 +28479,7 @@
         <v>46289.40860091435</v>
       </c>
       <c r="W356">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X356" t="s">
         <v>233</v>
@@ -28559,7 +28559,7 @@
         <v>46289.44826453704</v>
       </c>
       <c r="W357">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X357" t="s">
         <v>230</v>
@@ -28639,7 +28639,7 @@
         <v>46289.4482663426</v>
       </c>
       <c r="W358">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X358" t="s">
         <v>232</v>
@@ -28716,7 +28716,7 @@
         <v>46289.57045818287</v>
       </c>
       <c r="W359">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X359" t="s">
         <v>229</v>
@@ -28793,7 +28793,7 @@
         <v>46282.42251184028</v>
       </c>
       <c r="W360">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X360" t="s">
         <v>232</v>
@@ -28867,7 +28867,7 @@
         <v>46282.47420876157</v>
       </c>
       <c r="W361">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X361" t="s">
         <v>229</v>
@@ -28944,7 +28944,7 @@
         <v>46286.7220354051</v>
       </c>
       <c r="W362">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X362" t="s">
         <v>226</v>
@@ -29024,7 +29024,7 @@
         <v>46288.73877236111</v>
       </c>
       <c r="W363">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X363" t="s">
         <v>225</v>
@@ -29101,7 +29101,7 @@
         <v>46282.47437324074</v>
       </c>
       <c r="W364">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X364" t="s">
         <v>229</v>
@@ -29178,7 +29178,7 @@
         <v>46286.7221544213</v>
       </c>
       <c r="W365">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X365" t="s">
         <v>226</v>
@@ -29258,7 +29258,7 @@
         <v>46288.73927210648</v>
       </c>
       <c r="W366">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X366" t="s">
         <v>225</v>
@@ -29335,7 +29335,7 @@
         <v>46288.65462493055</v>
       </c>
       <c r="W367">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="X367" t="s">
         <v>229</v>
@@ -29412,7 +29412,7 @@
         <v>46287.66751398148</v>
       </c>
       <c r="W368">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="X368" t="s">
         <v>230</v>
@@ -29492,7 +29492,7 @@
         <v>46287.46969533565</v>
       </c>
       <c r="W369">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="X369" t="s">
         <v>232</v>
@@ -29572,7 +29572,7 @@
         <v>46286.71510853009</v>
       </c>
       <c r="W370">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X370" t="s">
         <v>229</v>
@@ -29652,7 +29652,7 @@
         <v>46283.59424842593</v>
       </c>
       <c r="W371">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X371" t="s">
         <v>230</v>
@@ -29732,7 +29732,7 @@
         <v>46283.68435655093</v>
       </c>
       <c r="W372">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X372" t="s">
         <v>223</v>
@@ -29812,7 +29812,7 @@
         <v>46283.5942487037</v>
       </c>
       <c r="W373">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X373" t="s">
         <v>224</v>
@@ -29892,7 +29892,7 @@
         <v>46283.59424924768</v>
       </c>
       <c r="W374">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X374" t="s">
         <v>224</v>
@@ -29972,7 +29972,7 @@
         <v>46283.68161918982</v>
       </c>
       <c r="W375">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X375" t="s">
         <v>232</v>
@@ -30052,7 +30052,7 @@
         <v>46286.6489187037</v>
       </c>
       <c r="W376">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X376" t="s">
         <v>228</v>
@@ -30132,7 +30132,7 @@
         <v>46288.38004474537</v>
       </c>
       <c r="W377">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X377" t="s">
         <v>226</v>
@@ -30212,7 +30212,7 @@
         <v>46282.42048836806</v>
       </c>
       <c r="W378">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X378" t="s">
         <v>233</v>
@@ -30289,7 +30289,7 @@
         <v>46282.42138976852</v>
       </c>
       <c r="W379">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X379" t="s">
         <v>233</v>
@@ -30363,7 +30363,7 @@
         <v>46288.65112511574</v>
       </c>
       <c r="W380">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="X380" t="s">
         <v>229</v>
@@ -30440,7 +30440,7 @@
         <v>46287.66967658565</v>
       </c>
       <c r="W381">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="X381" t="s">
         <v>230</v>
@@ -30520,7 +30520,7 @@
         <v>46287.47257043982</v>
       </c>
       <c r="W382">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="X382" t="s">
         <v>232</v>
@@ -30594,7 +30594,7 @@
         <v>46288.72977305556</v>
       </c>
       <c r="W383">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X383" t="s">
         <v>226</v>
@@ -30668,7 +30668,7 @@
         <v>46286.6987844213</v>
       </c>
       <c r="W384">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X384" t="s">
         <v>224</v>
@@ -30735,12 +30735,6 @@
       <c r="R385">
         <v>18283554</v>
       </c>
-      <c r="S385" t="s">
-        <v>194</v>
-      </c>
-      <c r="T385" t="s">
-        <v>214</v>
-      </c>
       <c r="U385" t="s">
         <v>222</v>
       </c>
@@ -30748,7 +30742,7 @@
         <v>46289.40156327546</v>
       </c>
       <c r="W385">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X385" t="s">
         <v>224</v>
@@ -30815,12 +30809,6 @@
       <c r="R386">
         <v>18283548</v>
       </c>
-      <c r="S386" t="s">
-        <v>194</v>
-      </c>
-      <c r="T386" t="s">
-        <v>214</v>
-      </c>
       <c r="U386" t="s">
         <v>222</v>
       </c>
@@ -30828,7 +30816,7 @@
         <v>46289.40156390046</v>
       </c>
       <c r="W386">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X386" t="s">
         <v>224</v>
@@ -30905,7 +30893,7 @@
         <v>46289.4053630787</v>
       </c>
       <c r="W387">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="X387" t="s">
         <v>233</v>
@@ -30979,7 +30967,7 @@
         <v>46289.40503480324</v>
       </c>
       <c r="W388">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="X388" t="s">
         <v>233</v>
@@ -31050,7 +31038,7 @@
         <v>46287.45807677083</v>
       </c>
       <c r="W389">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X389" t="s">
         <v>229</v>
@@ -31130,7 +31118,7 @@
         <v>46286.74096042824</v>
       </c>
       <c r="W390">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X390" t="s">
         <v>225</v>
@@ -31207,7 +31195,7 @@
         <v>46283.3939177662</v>
       </c>
       <c r="W391">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X391" t="s">
         <v>223</v>
@@ -31284,7 +31272,7 @@
         <v>46286.64017539352</v>
       </c>
       <c r="W392">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X392" t="s">
         <v>224</v>
@@ -31361,7 +31349,7 @@
         <v>46286.7204416551</v>
       </c>
       <c r="W393">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X393" t="s">
         <v>225</v>
@@ -31438,7 +31426,7 @@
         <v>46283.66538607639</v>
       </c>
       <c r="W394">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X394" t="s">
         <v>223</v>
@@ -31515,7 +31503,7 @@
         <v>46286.43482986111</v>
       </c>
       <c r="W395">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X395" t="s">
         <v>224</v>
@@ -31589,7 +31577,7 @@
         <v>46286.74368133102</v>
       </c>
       <c r="W396">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X396" t="s">
         <v>225</v>
@@ -31666,7 +31654,7 @@
         <v>46283.41459880787</v>
       </c>
       <c r="W397">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X397" t="s">
         <v>224</v>
@@ -31743,7 +31731,7 @@
         <v>46283.73838344908</v>
       </c>
       <c r="W398">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X398" t="s">
         <v>226</v>
@@ -31820,7 +31808,7 @@
         <v>46286.76327152778</v>
       </c>
       <c r="W399">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X399" t="s">
         <v>227</v>
@@ -31897,7 +31885,7 @@
         <v>46286.76330447917</v>
       </c>
       <c r="W400">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X400" t="s">
         <v>227</v>
@@ -31977,7 +31965,7 @@
         <v>46287.42040790509</v>
       </c>
       <c r="W401">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X401" t="s">
         <v>223</v>
@@ -32054,7 +32042,7 @@
         <v>46283.75381304398</v>
       </c>
       <c r="W402">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X402" t="s">
         <v>224</v>
@@ -32128,7 +32116,7 @@
         <v>46289.70979120371</v>
       </c>
       <c r="W403">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X403" t="s">
         <v>225</v>
@@ -32208,7 +32196,7 @@
         <v>46287.67534456019</v>
       </c>
       <c r="W404">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X404" t="s">
         <v>223</v>
@@ -32285,7 +32273,7 @@
         <v>46289.49194748842</v>
       </c>
       <c r="W405">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X405" t="s">
         <v>224</v>
@@ -32362,7 +32350,7 @@
         <v>46283.39413969908</v>
       </c>
       <c r="W406">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X406" t="s">
         <v>223</v>
@@ -32436,7 +32424,7 @@
         <v>46286.72051887732</v>
       </c>
       <c r="W407">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X407" t="s">
         <v>225</v>
@@ -32516,7 +32504,7 @@
         <v>46283.54620269676</v>
       </c>
       <c r="W408">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X408" t="s">
         <v>229</v>
@@ -32593,7 +32581,7 @@
         <v>46288.58542337963</v>
       </c>
       <c r="W409">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X409" t="s">
         <v>230</v>
@@ -32673,7 +32661,7 @@
         <v>46289.35188425926</v>
       </c>
       <c r="W410">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X410" t="s">
         <v>228</v>
@@ -32753,7 +32741,7 @@
         <v>46287.46001957176</v>
       </c>
       <c r="W411">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X411" t="s">
         <v>229</v>
@@ -32833,7 +32821,7 @@
         <v>46287.46001266204</v>
       </c>
       <c r="W412">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X412" t="s">
         <v>233</v>
@@ -32913,7 +32901,7 @@
         <v>46286.72594498843</v>
       </c>
       <c r="W413">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X413" t="s">
         <v>230</v>
@@ -32993,7 +32981,7 @@
         <v>46282.70138376157</v>
       </c>
       <c r="W414">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X414" t="s">
         <v>228</v>
@@ -33073,7 +33061,7 @@
         <v>46282.7013840625</v>
       </c>
       <c r="W415">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X415" t="s">
         <v>228</v>
@@ -33150,7 +33138,7 @@
         <v>46283.75077045139</v>
       </c>
       <c r="W416">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X416" t="s">
         <v>232</v>
@@ -33230,7 +33218,7 @@
         <v>46286.36164050926</v>
       </c>
       <c r="W417">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X417" t="s">
         <v>228</v>
@@ -33310,7 +33298,7 @@
         <v>46286.36164494213</v>
       </c>
       <c r="W418">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X418" t="s">
         <v>229</v>
@@ -33390,7 +33378,7 @@
         <v>46286.36164826389</v>
       </c>
       <c r="W419">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X419" t="s">
         <v>233</v>
@@ -33467,7 +33455,7 @@
         <v>46283.35452896991</v>
       </c>
       <c r="W420">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X420" t="s">
         <v>228</v>
@@ -33544,7 +33532,7 @@
         <v>46283.35453171296</v>
       </c>
       <c r="W421">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X421" t="s">
         <v>228</v>
@@ -33624,7 +33612,7 @@
         <v>46287.36782538195</v>
       </c>
       <c r="W422">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X422" t="s">
         <v>232</v>
@@ -33704,7 +33692,7 @@
         <v>46287.42044105324</v>
       </c>
       <c r="W423">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X423" t="s">
         <v>233</v>
@@ -33784,7 +33772,7 @@
         <v>46288.49685543981</v>
       </c>
       <c r="W424">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X424" t="s">
         <v>232</v>
@@ -33864,7 +33852,7 @@
         <v>46287.75597989583</v>
       </c>
       <c r="W425">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X425" t="s">
         <v>229</v>
@@ -33944,7 +33932,7 @@
         <v>46288.76876331019</v>
       </c>
       <c r="W426">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X426" t="s">
         <v>228</v>
@@ -34021,7 +34009,7 @@
         <v>46283.38367943287</v>
       </c>
       <c r="W427">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X427" t="s">
         <v>229</v>
@@ -34098,7 +34086,7 @@
         <v>46282.54038741898</v>
       </c>
       <c r="W428">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X428" t="s">
         <v>233</v>
@@ -34175,7 +34163,7 @@
         <v>46283.64213659722</v>
       </c>
       <c r="W429">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X429" t="s">
         <v>224</v>
@@ -34252,7 +34240,7 @@
         <v>46283.65291121528</v>
       </c>
       <c r="W430">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X430" t="s">
         <v>228</v>
@@ -34329,7 +34317,7 @@
         <v>46283.65291194445</v>
       </c>
       <c r="W431">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X431" t="s">
         <v>228</v>
@@ -34406,7 +34394,7 @@
         <v>46286.39955256944</v>
       </c>
       <c r="W432">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X432" t="s">
         <v>226</v>
@@ -34480,7 +34468,7 @@
         <v>46286.42397924769</v>
       </c>
       <c r="W433">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X433" t="s">
         <v>229</v>
@@ -34554,7 +34542,7 @@
         <v>46286.42389136574</v>
       </c>
       <c r="W434">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X434" t="s">
         <v>233</v>
@@ -34631,7 +34619,7 @@
         <v>46283.67999300926</v>
       </c>
       <c r="W435">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X435" t="s">
         <v>224</v>
@@ -34708,7 +34696,7 @@
         <v>46286.42398471065</v>
       </c>
       <c r="W436">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X436" t="s">
         <v>232</v>
@@ -34782,7 +34770,7 @@
         <v>46286.42398568287</v>
       </c>
       <c r="W437">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X437" t="s">
         <v>228</v>
@@ -34859,7 +34847,7 @@
         <v>46283.67625043981</v>
       </c>
       <c r="W438">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X438" t="s">
         <v>226</v>
@@ -34936,7 +34924,7 @@
         <v>46283.38329579861</v>
       </c>
       <c r="W439">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X439" t="s">
         <v>228</v>
@@ -35013,7 +35001,7 @@
         <v>46282.36440621527</v>
       </c>
       <c r="W440">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X440" t="s">
         <v>229</v>
@@ -35090,7 +35078,7 @@
         <v>46282.36462596065</v>
       </c>
       <c r="W441">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X441" t="s">
         <v>233</v>
@@ -35167,7 +35155,7 @@
         <v>46282.36464421296</v>
       </c>
       <c r="W442">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X442" t="s">
         <v>230</v>
@@ -35244,7 +35232,7 @@
         <v>46282.36467337963</v>
       </c>
       <c r="W443">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X443" t="s">
         <v>223</v>
@@ -35321,7 +35309,7 @@
         <v>46282.36469679398</v>
       </c>
       <c r="W444">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X444" t="s">
         <v>224</v>
@@ -35398,7 +35386,7 @@
         <v>46282.36469869213</v>
       </c>
       <c r="W445">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X445" t="s">
         <v>224</v>
@@ -35475,7 +35463,7 @@
         <v>46282.36473159722</v>
       </c>
       <c r="W446">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X446" t="s">
         <v>232</v>
@@ -35552,7 +35540,7 @@
         <v>46282.36473394676</v>
       </c>
       <c r="W447">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X447" t="s">
         <v>228</v>
@@ -35629,7 +35617,7 @@
         <v>46282.36473579861</v>
       </c>
       <c r="W448">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X448" t="s">
         <v>228</v>
@@ -35706,7 +35694,7 @@
         <v>46282.36475297454</v>
       </c>
       <c r="W449">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X449" t="s">
         <v>228</v>
@@ -35783,7 +35771,7 @@
         <v>46282.36486408565</v>
       </c>
       <c r="W450">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X450" t="s">
         <v>226</v>
@@ -35860,7 +35848,7 @@
         <v>46282.36487561343</v>
       </c>
       <c r="W451">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X451" t="s">
         <v>225</v>
@@ -35937,7 +35925,7 @@
         <v>46282.36486778935</v>
       </c>
       <c r="W452">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X452" t="s">
         <v>227</v>
@@ -36014,7 +36002,7 @@
         <v>46282.36486851852</v>
       </c>
       <c r="W453">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X453" t="s">
         <v>227</v>
@@ -36091,7 +36079,7 @@
         <v>46286.45925082176</v>
       </c>
       <c r="W454">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X454" t="s">
         <v>229</v>
@@ -36168,7 +36156,7 @@
         <v>46282.79619427084</v>
       </c>
       <c r="W455">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X455" t="s">
         <v>233</v>
@@ -36245,7 +36233,7 @@
         <v>46282.79620872685</v>
       </c>
       <c r="W456">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X456" t="s">
         <v>230</v>
@@ -36322,7 +36310,7 @@
         <v>46282.79623825232</v>
       </c>
       <c r="W457">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X457" t="s">
         <v>223</v>
@@ -36399,7 +36387,7 @@
         <v>46282.7962541551</v>
       </c>
       <c r="W458">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X458" t="s">
         <v>224</v>
@@ -36476,7 +36464,7 @@
         <v>46282.7962703125</v>
       </c>
       <c r="W459">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X459" t="s">
         <v>224</v>
@@ -36553,7 +36541,7 @@
         <v>46282.79628381944</v>
       </c>
       <c r="W460">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X460" t="s">
         <v>232</v>
@@ -36630,7 +36618,7 @@
         <v>46282.79630119213</v>
       </c>
       <c r="W461">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X461" t="s">
         <v>228</v>
@@ -36707,7 +36695,7 @@
         <v>46282.79631224537</v>
       </c>
       <c r="W462">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X462" t="s">
         <v>228</v>
@@ -36784,7 +36772,7 @@
         <v>46282.79637734954</v>
       </c>
       <c r="W463">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X463" t="s">
         <v>226</v>
@@ -36861,7 +36849,7 @@
         <v>46282.79638922454</v>
       </c>
       <c r="W464">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X464" t="s">
         <v>225</v>
@@ -36938,7 +36926,7 @@
         <v>46282.3651903588</v>
       </c>
       <c r="W465">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X465" t="s">
         <v>229</v>
@@ -37015,7 +37003,7 @@
         <v>46282.36525856482</v>
       </c>
       <c r="W466">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X466" t="s">
         <v>233</v>
@@ -37092,7 +37080,7 @@
         <v>46282.36526855324</v>
       </c>
       <c r="W467">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X467" t="s">
         <v>230</v>
@@ -37169,7 +37157,7 @@
         <v>46282.36527959491</v>
       </c>
       <c r="W468">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X468" t="s">
         <v>223</v>
@@ -37246,7 +37234,7 @@
         <v>46282.36528526621</v>
       </c>
       <c r="W469">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X469" t="s">
         <v>224</v>
@@ -37323,7 +37311,7 @@
         <v>46282.36528619213</v>
       </c>
       <c r="W470">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X470" t="s">
         <v>224</v>
@@ -37400,7 +37388,7 @@
         <v>46282.36529351852</v>
       </c>
       <c r="W471">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X471" t="s">
         <v>232</v>
@@ -37477,7 +37465,7 @@
         <v>46282.36529424768</v>
       </c>
       <c r="W472">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X472" t="s">
         <v>228</v>
@@ -37554,7 +37542,7 @@
         <v>46282.36529490741</v>
       </c>
       <c r="W473">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X473" t="s">
         <v>228</v>
@@ -37631,7 +37619,7 @@
         <v>46282.36529869213</v>
       </c>
       <c r="W474">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X474" t="s">
         <v>228</v>
@@ -37708,7 +37696,7 @@
         <v>46282.36531149306</v>
       </c>
       <c r="W475">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X475" t="s">
         <v>226</v>
@@ -37785,7 +37773,7 @@
         <v>46282.36531554398</v>
       </c>
       <c r="W476">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X476" t="s">
         <v>225</v>
@@ -37862,7 +37850,7 @@
         <v>46282.36531253472</v>
       </c>
       <c r="W477">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X477" t="s">
         <v>227</v>
@@ -37939,7 +37927,7 @@
         <v>46282.36531288194</v>
       </c>
       <c r="W478">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X478" t="s">
         <v>227</v>
@@ -38016,7 +38004,7 @@
         <v>46286.45925106481</v>
       </c>
       <c r="W479">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X479" t="s">
         <v>229</v>
@@ -38093,7 +38081,7 @@
         <v>46282.79619331018</v>
       </c>
       <c r="W480">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X480" t="s">
         <v>233</v>
@@ -38170,7 +38158,7 @@
         <v>46282.79620888889</v>
       </c>
       <c r="W481">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X481" t="s">
         <v>230</v>
@@ -38247,7 +38235,7 @@
         <v>46282.79623803241</v>
       </c>
       <c r="W482">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X482" t="s">
         <v>223</v>
@@ -38324,7 +38312,7 @@
         <v>46282.79625384259</v>
       </c>
       <c r="W483">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X483" t="s">
         <v>224</v>
@@ -38401,7 +38389,7 @@
         <v>46282.79626969907</v>
       </c>
       <c r="W484">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X484" t="s">
         <v>224</v>
@@ -38478,7 +38466,7 @@
         <v>46282.79628394676</v>
       </c>
       <c r="W485">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X485" t="s">
         <v>232</v>
@@ -38555,7 +38543,7 @@
         <v>46282.79630097222</v>
       </c>
       <c r="W486">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X486" t="s">
         <v>228</v>
@@ -38632,7 +38620,7 @@
         <v>46282.79631204861</v>
       </c>
       <c r="W487">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X487" t="s">
         <v>228</v>
@@ -38709,7 +38697,7 @@
         <v>46282.79637748843</v>
       </c>
       <c r="W488">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X488" t="s">
         <v>226</v>
@@ -38786,7 +38774,7 @@
         <v>46282.79638901621</v>
       </c>
       <c r="W489">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X489" t="s">
         <v>225</v>
@@ -38860,7 +38848,7 @@
         <v>46283.39832862269</v>
       </c>
       <c r="W490">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X490" t="s">
         <v>229</v>
@@ -38934,7 +38922,7 @@
         <v>46282.64018086805</v>
       </c>
       <c r="W491">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X491" t="s">
         <v>233</v>
@@ -39008,7 +38996,7 @@
         <v>46287.492834375</v>
       </c>
       <c r="W492">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X492" t="s">
         <v>229</v>
@@ -39082,7 +39070,7 @@
         <v>46287.49337789352</v>
       </c>
       <c r="W493">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X493" t="s">
         <v>227</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-25 10:02
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7219" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7251" uniqueCount="433">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1685,7 +1685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI493"/>
+  <dimension ref="A1:AI495"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -39091,6 +39091,166 @@
         <v>432</v>
       </c>
     </row>
+    <row r="494" spans="1:35">
+      <c r="A494">
+        <v>6962</v>
+      </c>
+      <c r="B494" t="s">
+        <v>40</v>
+      </c>
+      <c r="C494" t="s">
+        <v>50</v>
+      </c>
+      <c r="D494" t="s">
+        <v>53</v>
+      </c>
+      <c r="E494" t="s">
+        <v>54</v>
+      </c>
+      <c r="F494" t="s">
+        <v>57</v>
+      </c>
+      <c r="G494">
+        <v>11516</v>
+      </c>
+      <c r="H494">
+        <v>0</v>
+      </c>
+      <c r="I494" t="s">
+        <v>59</v>
+      </c>
+      <c r="J494" t="s">
+        <v>140</v>
+      </c>
+      <c r="N494" s="1">
+        <v>46290</v>
+      </c>
+      <c r="O494" t="s">
+        <v>177</v>
+      </c>
+      <c r="P494">
+        <v>8</v>
+      </c>
+      <c r="Q494">
+        <v>2026</v>
+      </c>
+      <c r="R494">
+        <v>18187985</v>
+      </c>
+      <c r="S494" t="s">
+        <v>188</v>
+      </c>
+      <c r="T494" t="s">
+        <v>211</v>
+      </c>
+      <c r="U494" t="s">
+        <v>222</v>
+      </c>
+      <c r="V494" s="1">
+        <v>46290.40572291666</v>
+      </c>
+      <c r="W494">
+        <v>0</v>
+      </c>
+      <c r="X494" t="s">
+        <v>227</v>
+      </c>
+      <c r="Y494" t="s">
+        <v>354</v>
+      </c>
+      <c r="AB494">
+        <v>0</v>
+      </c>
+      <c r="AC494" t="s">
+        <v>188</v>
+      </c>
+      <c r="AH494" t="s">
+        <v>428</v>
+      </c>
+      <c r="AI494" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="495" spans="1:35">
+      <c r="A495">
+        <v>6963</v>
+      </c>
+      <c r="B495" t="s">
+        <v>41</v>
+      </c>
+      <c r="C495" t="s">
+        <v>50</v>
+      </c>
+      <c r="D495" t="s">
+        <v>53</v>
+      </c>
+      <c r="E495" t="s">
+        <v>54</v>
+      </c>
+      <c r="F495" t="s">
+        <v>57</v>
+      </c>
+      <c r="G495">
+        <v>11516</v>
+      </c>
+      <c r="H495">
+        <v>0</v>
+      </c>
+      <c r="I495" t="s">
+        <v>59</v>
+      </c>
+      <c r="J495" t="s">
+        <v>140</v>
+      </c>
+      <c r="N495" s="1">
+        <v>46290</v>
+      </c>
+      <c r="O495" t="s">
+        <v>177</v>
+      </c>
+      <c r="P495">
+        <v>8</v>
+      </c>
+      <c r="Q495">
+        <v>2026</v>
+      </c>
+      <c r="R495">
+        <v>18241255</v>
+      </c>
+      <c r="S495" t="s">
+        <v>188</v>
+      </c>
+      <c r="T495" t="s">
+        <v>211</v>
+      </c>
+      <c r="U495" t="s">
+        <v>222</v>
+      </c>
+      <c r="V495" s="1">
+        <v>46290.40597356481</v>
+      </c>
+      <c r="W495">
+        <v>0</v>
+      </c>
+      <c r="X495" t="s">
+        <v>227</v>
+      </c>
+      <c r="Y495" t="s">
+        <v>354</v>
+      </c>
+      <c r="AB495">
+        <v>0</v>
+      </c>
+      <c r="AC495" t="s">
+        <v>188</v>
+      </c>
+      <c r="AH495" t="s">
+        <v>428</v>
+      </c>
+      <c r="AI495" t="s">
+        <v>432</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-25 14:04
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7308" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7392" uniqueCount="437">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1698,7 +1698,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI500"/>
+  <dimension ref="A1:AI506"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -39064,22 +39064,22 @@
     </row>
     <row r="494" spans="1:35">
       <c r="A494">
-        <v>6962</v>
+        <v>6548</v>
       </c>
       <c r="B494" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C494" t="s">
         <v>50</v>
       </c>
       <c r="D494" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E494" t="s">
         <v>54</v>
       </c>
       <c r="F494" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G494">
         <v>6892</v>
@@ -39103,31 +39103,31 @@
         <v>2026</v>
       </c>
       <c r="R494">
-        <v>18187955</v>
+        <v>17968017</v>
       </c>
       <c r="S494" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="T494" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="U494" t="s">
         <v>223</v>
       </c>
       <c r="V494" s="1">
-        <v>46290.481633125</v>
+        <v>46290.56449253472</v>
       </c>
       <c r="W494">
         <v>0</v>
       </c>
       <c r="X494" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="AB494">
         <v>0</v>
       </c>
       <c r="AC494" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="AH494" t="s">
         <v>432</v>
@@ -39138,22 +39138,22 @@
     </row>
     <row r="495" spans="1:35">
       <c r="A495">
-        <v>6963</v>
+        <v>6627</v>
       </c>
       <c r="B495" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C495" t="s">
         <v>50</v>
       </c>
       <c r="D495" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E495" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F495" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G495">
         <v>6892</v>
@@ -39177,10 +39177,10 @@
         <v>2026</v>
       </c>
       <c r="R495">
-        <v>18187893</v>
+        <v>17042486</v>
       </c>
       <c r="S495" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="T495" t="s">
         <v>212</v>
@@ -39189,19 +39189,19 @@
         <v>223</v>
       </c>
       <c r="V495" s="1">
-        <v>46290.48190942129</v>
+        <v>46290.56093913194</v>
       </c>
       <c r="W495">
         <v>0</v>
       </c>
       <c r="X495" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="AB495">
         <v>0</v>
       </c>
       <c r="AC495" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="AH495" t="s">
         <v>432</v>
@@ -39212,16 +39212,16 @@
     </row>
     <row r="496" spans="1:35">
       <c r="A496">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B496" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C496" t="s">
         <v>50</v>
       </c>
       <c r="D496" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E496" t="s">
         <v>54</v>
@@ -39230,7 +39230,7 @@
         <v>57</v>
       </c>
       <c r="G496">
-        <v>11516</v>
+        <v>6892</v>
       </c>
       <c r="H496">
         <v>0</v>
@@ -39239,7 +39239,7 @@
         <v>59</v>
       </c>
       <c r="J496" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N496" s="1">
         <v>46290</v>
@@ -39251,31 +39251,31 @@
         <v>2026</v>
       </c>
       <c r="R496">
-        <v>18187985</v>
+        <v>18178288</v>
       </c>
       <c r="S496" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="T496" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="U496" t="s">
         <v>223</v>
       </c>
       <c r="V496" s="1">
-        <v>46290.40572291666</v>
+        <v>46290.56969825231</v>
       </c>
       <c r="W496">
         <v>0</v>
       </c>
       <c r="X496" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="AB496">
         <v>0</v>
       </c>
       <c r="AC496" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="AH496" t="s">
         <v>432</v>
@@ -39286,10 +39286,10 @@
     </row>
     <row r="497" spans="1:35">
       <c r="A497">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B497" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C497" t="s">
         <v>50</v>
@@ -39304,7 +39304,7 @@
         <v>57</v>
       </c>
       <c r="G497">
-        <v>11516</v>
+        <v>6892</v>
       </c>
       <c r="H497">
         <v>0</v>
@@ -39313,7 +39313,7 @@
         <v>59</v>
       </c>
       <c r="J497" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N497" s="1">
         <v>46290</v>
@@ -39325,7 +39325,7 @@
         <v>2026</v>
       </c>
       <c r="R497">
-        <v>18241255</v>
+        <v>18187955</v>
       </c>
       <c r="S497" t="s">
         <v>188</v>
@@ -39337,7 +39337,7 @@
         <v>223</v>
       </c>
       <c r="V497" s="1">
-        <v>46290.40597356481</v>
+        <v>46290.481633125</v>
       </c>
       <c r="W497">
         <v>0</v>
@@ -39360,76 +39360,70 @@
     </row>
     <row r="498" spans="1:35">
       <c r="A498">
-        <v>6548</v>
+        <v>6963</v>
       </c>
       <c r="B498" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C498" t="s">
         <v>50</v>
       </c>
       <c r="D498" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E498" t="s">
         <v>54</v>
       </c>
       <c r="F498" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G498">
-        <v>11542</v>
+        <v>6892</v>
       </c>
       <c r="H498">
         <v>0</v>
       </c>
       <c r="I498" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J498" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
       <c r="N498" s="1">
-        <v>46296</v>
-      </c>
-      <c r="O498" t="s">
-        <v>179</v>
+        <v>46290</v>
       </c>
       <c r="P498">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Q498">
         <v>2026</v>
       </c>
       <c r="R498">
-        <v>17222969</v>
+        <v>18187893</v>
       </c>
       <c r="S498" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="T498" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="U498" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="V498" s="1">
-        <v>46290.46651483796</v>
+        <v>46290.48190942129</v>
       </c>
       <c r="W498">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="X498" t="s">
-        <v>224</v>
-      </c>
-      <c r="Y498" t="s">
-        <v>423</v>
+        <v>228</v>
       </c>
       <c r="AB498">
         <v>0</v>
       </c>
       <c r="AC498" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="AH498" t="s">
         <v>432</v>
@@ -39458,58 +39452,52 @@
         <v>56</v>
       </c>
       <c r="G499">
-        <v>11541</v>
+        <v>11516</v>
       </c>
       <c r="H499">
         <v>0</v>
       </c>
       <c r="I499" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J499" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="N499" s="1">
-        <v>46296</v>
-      </c>
-      <c r="O499" t="s">
-        <v>179</v>
+        <v>46290</v>
       </c>
       <c r="P499">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Q499">
         <v>2026</v>
       </c>
       <c r="R499">
-        <v>17222949</v>
+        <v>17968053</v>
       </c>
       <c r="S499" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="T499" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="U499" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="V499" s="1">
-        <v>46290.46660107639</v>
+        <v>46290.564674375</v>
       </c>
       <c r="W499">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="X499" t="s">
         <v>224</v>
       </c>
-      <c r="Y499" t="s">
-        <v>424</v>
-      </c>
       <c r="AB499">
         <v>0</v>
       </c>
       <c r="AC499" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="AH499" t="s">
         <v>432</v>
@@ -39520,41 +39508,38 @@
     </row>
     <row r="500" spans="1:35">
       <c r="A500">
-        <v>6703</v>
+        <v>6627</v>
       </c>
       <c r="B500" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C500" t="s">
         <v>50</v>
       </c>
       <c r="D500" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E500" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F500" t="s">
         <v>56</v>
       </c>
       <c r="G500">
-        <v>11056</v>
+        <v>11516</v>
       </c>
       <c r="H500">
         <v>0</v>
       </c>
       <c r="I500" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="J500" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="N500" s="1">
         <v>46290</v>
       </c>
-      <c r="O500" t="s">
-        <v>179</v>
-      </c>
       <c r="P500">
         <v>8</v>
       </c>
@@ -39562,36 +39547,495 @@
         <v>2026</v>
       </c>
       <c r="R500">
-        <v>18284872</v>
+        <v>17042662</v>
       </c>
       <c r="S500" t="s">
-        <v>210</v>
+        <v>186</v>
+      </c>
+      <c r="T500" t="s">
+        <v>212</v>
       </c>
       <c r="U500" t="s">
         <v>223</v>
       </c>
       <c r="V500" s="1">
+        <v>46290.56113170139</v>
+      </c>
+      <c r="W500">
+        <v>0</v>
+      </c>
+      <c r="X500" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB500">
+        <v>0</v>
+      </c>
+      <c r="AC500" t="s">
+        <v>186</v>
+      </c>
+      <c r="AH500" t="s">
+        <v>432</v>
+      </c>
+      <c r="AI500" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="501" spans="1:35">
+      <c r="A501">
+        <v>6949</v>
+      </c>
+      <c r="B501" t="s">
+        <v>37</v>
+      </c>
+      <c r="C501" t="s">
+        <v>50</v>
+      </c>
+      <c r="D501" t="s">
+        <v>51</v>
+      </c>
+      <c r="E501" t="s">
+        <v>54</v>
+      </c>
+      <c r="F501" t="s">
+        <v>57</v>
+      </c>
+      <c r="G501">
+        <v>11516</v>
+      </c>
+      <c r="H501">
+        <v>0</v>
+      </c>
+      <c r="I501" t="s">
+        <v>59</v>
+      </c>
+      <c r="J501" t="s">
+        <v>140</v>
+      </c>
+      <c r="N501" s="1">
+        <v>46290</v>
+      </c>
+      <c r="P501">
+        <v>8</v>
+      </c>
+      <c r="Q501">
+        <v>2026</v>
+      </c>
+      <c r="R501">
+        <v>18178314</v>
+      </c>
+      <c r="S501" t="s">
+        <v>185</v>
+      </c>
+      <c r="T501" t="s">
+        <v>211</v>
+      </c>
+      <c r="U501" t="s">
+        <v>223</v>
+      </c>
+      <c r="V501" s="1">
+        <v>46290.56957094908</v>
+      </c>
+      <c r="W501">
+        <v>0</v>
+      </c>
+      <c r="X501" t="s">
+        <v>226</v>
+      </c>
+      <c r="AB501">
+        <v>0</v>
+      </c>
+      <c r="AC501" t="s">
+        <v>185</v>
+      </c>
+      <c r="AH501" t="s">
+        <v>432</v>
+      </c>
+      <c r="AI501" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="502" spans="1:35">
+      <c r="A502">
+        <v>6962</v>
+      </c>
+      <c r="B502" t="s">
+        <v>40</v>
+      </c>
+      <c r="C502" t="s">
+        <v>50</v>
+      </c>
+      <c r="D502" t="s">
+        <v>53</v>
+      </c>
+      <c r="E502" t="s">
+        <v>54</v>
+      </c>
+      <c r="F502" t="s">
+        <v>57</v>
+      </c>
+      <c r="G502">
+        <v>11516</v>
+      </c>
+      <c r="H502">
+        <v>0</v>
+      </c>
+      <c r="I502" t="s">
+        <v>59</v>
+      </c>
+      <c r="J502" t="s">
+        <v>140</v>
+      </c>
+      <c r="N502" s="1">
+        <v>46290</v>
+      </c>
+      <c r="P502">
+        <v>8</v>
+      </c>
+      <c r="Q502">
+        <v>2026</v>
+      </c>
+      <c r="R502">
+        <v>18187985</v>
+      </c>
+      <c r="S502" t="s">
+        <v>188</v>
+      </c>
+      <c r="T502" t="s">
+        <v>212</v>
+      </c>
+      <c r="U502" t="s">
+        <v>223</v>
+      </c>
+      <c r="V502" s="1">
+        <v>46290.40572291666</v>
+      </c>
+      <c r="W502">
+        <v>0</v>
+      </c>
+      <c r="X502" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB502">
+        <v>0</v>
+      </c>
+      <c r="AC502" t="s">
+        <v>188</v>
+      </c>
+      <c r="AH502" t="s">
+        <v>432</v>
+      </c>
+      <c r="AI502" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="503" spans="1:35">
+      <c r="A503">
+        <v>6963</v>
+      </c>
+      <c r="B503" t="s">
+        <v>41</v>
+      </c>
+      <c r="C503" t="s">
+        <v>50</v>
+      </c>
+      <c r="D503" t="s">
+        <v>53</v>
+      </c>
+      <c r="E503" t="s">
+        <v>54</v>
+      </c>
+      <c r="F503" t="s">
+        <v>57</v>
+      </c>
+      <c r="G503">
+        <v>11516</v>
+      </c>
+      <c r="H503">
+        <v>0</v>
+      </c>
+      <c r="I503" t="s">
+        <v>59</v>
+      </c>
+      <c r="J503" t="s">
+        <v>140</v>
+      </c>
+      <c r="N503" s="1">
+        <v>46290</v>
+      </c>
+      <c r="P503">
+        <v>8</v>
+      </c>
+      <c r="Q503">
+        <v>2026</v>
+      </c>
+      <c r="R503">
+        <v>18241255</v>
+      </c>
+      <c r="S503" t="s">
+        <v>188</v>
+      </c>
+      <c r="T503" t="s">
+        <v>212</v>
+      </c>
+      <c r="U503" t="s">
+        <v>223</v>
+      </c>
+      <c r="V503" s="1">
+        <v>46290.40597356481</v>
+      </c>
+      <c r="W503">
+        <v>0</v>
+      </c>
+      <c r="X503" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB503">
+        <v>0</v>
+      </c>
+      <c r="AC503" t="s">
+        <v>188</v>
+      </c>
+      <c r="AH503" t="s">
+        <v>432</v>
+      </c>
+      <c r="AI503" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="504" spans="1:35">
+      <c r="A504">
+        <v>6548</v>
+      </c>
+      <c r="B504" t="s">
+        <v>35</v>
+      </c>
+      <c r="C504" t="s">
+        <v>50</v>
+      </c>
+      <c r="D504" t="s">
+        <v>51</v>
+      </c>
+      <c r="E504" t="s">
+        <v>54</v>
+      </c>
+      <c r="F504" t="s">
+        <v>56</v>
+      </c>
+      <c r="G504">
+        <v>11542</v>
+      </c>
+      <c r="H504">
+        <v>0</v>
+      </c>
+      <c r="I504" t="s">
+        <v>61</v>
+      </c>
+      <c r="J504" t="s">
+        <v>79</v>
+      </c>
+      <c r="N504" s="1">
+        <v>46296</v>
+      </c>
+      <c r="O504" t="s">
+        <v>179</v>
+      </c>
+      <c r="P504">
+        <v>10</v>
+      </c>
+      <c r="Q504">
+        <v>2026</v>
+      </c>
+      <c r="R504">
+        <v>17222969</v>
+      </c>
+      <c r="S504" t="s">
+        <v>199</v>
+      </c>
+      <c r="T504" t="s">
+        <v>215</v>
+      </c>
+      <c r="U504" t="s">
+        <v>222</v>
+      </c>
+      <c r="V504" s="1">
+        <v>46290.46651483796</v>
+      </c>
+      <c r="W504">
+        <v>-6</v>
+      </c>
+      <c r="X504" t="s">
+        <v>224</v>
+      </c>
+      <c r="Y504" t="s">
+        <v>423</v>
+      </c>
+      <c r="AB504">
+        <v>0</v>
+      </c>
+      <c r="AC504" t="s">
+        <v>199</v>
+      </c>
+      <c r="AH504" t="s">
+        <v>432</v>
+      </c>
+      <c r="AI504" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="505" spans="1:35">
+      <c r="A505">
+        <v>6548</v>
+      </c>
+      <c r="B505" t="s">
+        <v>35</v>
+      </c>
+      <c r="C505" t="s">
+        <v>50</v>
+      </c>
+      <c r="D505" t="s">
+        <v>51</v>
+      </c>
+      <c r="E505" t="s">
+        <v>54</v>
+      </c>
+      <c r="F505" t="s">
+        <v>56</v>
+      </c>
+      <c r="G505">
+        <v>11541</v>
+      </c>
+      <c r="H505">
+        <v>0</v>
+      </c>
+      <c r="I505" t="s">
+        <v>61</v>
+      </c>
+      <c r="J505" t="s">
+        <v>144</v>
+      </c>
+      <c r="N505" s="1">
+        <v>46296</v>
+      </c>
+      <c r="O505" t="s">
+        <v>179</v>
+      </c>
+      <c r="P505">
+        <v>10</v>
+      </c>
+      <c r="Q505">
+        <v>2026</v>
+      </c>
+      <c r="R505">
+        <v>17222949</v>
+      </c>
+      <c r="S505" t="s">
+        <v>199</v>
+      </c>
+      <c r="T505" t="s">
+        <v>215</v>
+      </c>
+      <c r="U505" t="s">
+        <v>222</v>
+      </c>
+      <c r="V505" s="1">
+        <v>46290.46660107639</v>
+      </c>
+      <c r="W505">
+        <v>-6</v>
+      </c>
+      <c r="X505" t="s">
+        <v>224</v>
+      </c>
+      <c r="Y505" t="s">
+        <v>424</v>
+      </c>
+      <c r="AB505">
+        <v>0</v>
+      </c>
+      <c r="AC505" t="s">
+        <v>199</v>
+      </c>
+      <c r="AH505" t="s">
+        <v>432</v>
+      </c>
+      <c r="AI505" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="506" spans="1:35">
+      <c r="A506">
+        <v>6703</v>
+      </c>
+      <c r="B506" t="s">
+        <v>46</v>
+      </c>
+      <c r="C506" t="s">
+        <v>50</v>
+      </c>
+      <c r="D506" t="s">
+        <v>53</v>
+      </c>
+      <c r="E506" t="s">
+        <v>54</v>
+      </c>
+      <c r="F506" t="s">
+        <v>56</v>
+      </c>
+      <c r="G506">
+        <v>11056</v>
+      </c>
+      <c r="H506">
+        <v>0</v>
+      </c>
+      <c r="I506" t="s">
+        <v>66</v>
+      </c>
+      <c r="J506" t="s">
+        <v>119</v>
+      </c>
+      <c r="N506" s="1">
+        <v>46290</v>
+      </c>
+      <c r="O506" t="s">
+        <v>179</v>
+      </c>
+      <c r="P506">
+        <v>8</v>
+      </c>
+      <c r="Q506">
+        <v>2026</v>
+      </c>
+      <c r="R506">
+        <v>18284872</v>
+      </c>
+      <c r="S506" t="s">
+        <v>210</v>
+      </c>
+      <c r="U506" t="s">
+        <v>223</v>
+      </c>
+      <c r="V506" s="1">
         <v>46290.42450153935</v>
       </c>
-      <c r="W500">
-        <v>0</v>
-      </c>
-      <c r="X500" t="s">
+      <c r="W506">
+        <v>0</v>
+      </c>
+      <c r="X506" t="s">
         <v>233</v>
       </c>
-      <c r="Y500" t="s">
+      <c r="Y506" t="s">
         <v>425</v>
       </c>
-      <c r="AB500">
-        <v>0</v>
-      </c>
-      <c r="AC500" t="s">
+      <c r="AB506">
+        <v>0</v>
+      </c>
+      <c r="AC506" t="s">
         <v>210</v>
       </c>
-      <c r="AH500" t="s">
+      <c r="AH506" t="s">
         <v>430</v>
       </c>
-      <c r="AI500" t="s">
+      <c r="AI506" t="s">
         <v>436</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-28 10:57
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7538" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7552" uniqueCount="447">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1390,6 +1390,9 @@
   </si>
   <si>
     <t>4 Semana</t>
+  </si>
+  <si>
+    <t>5 Semana</t>
   </si>
 </sst>
 </file>
@@ -1725,7 +1728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI516"/>
+  <dimension ref="A1:AI517"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -40059,10 +40062,10 @@
     </row>
     <row r="507" spans="1:35">
       <c r="A507">
-        <v>6548</v>
+        <v>6949</v>
       </c>
       <c r="B507" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C507" t="s">
         <v>50</v>
@@ -40074,10 +40077,10 @@
         <v>54</v>
       </c>
       <c r="F507" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G507">
-        <v>11541</v>
+        <v>11542</v>
       </c>
       <c r="H507">
         <v>0</v>
@@ -40086,14 +40089,11 @@
         <v>61</v>
       </c>
       <c r="J507" t="s">
-        <v>144</v>
+        <v>79</v>
       </c>
       <c r="N507" s="1">
         <v>46296</v>
       </c>
-      <c r="O507" t="s">
-        <v>180</v>
-      </c>
       <c r="P507">
         <v>10</v>
       </c>
@@ -40101,48 +40101,45 @@
         <v>2026</v>
       </c>
       <c r="R507">
-        <v>17222949</v>
+        <v>18190472</v>
       </c>
       <c r="S507" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="T507" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="U507" t="s">
         <v>222</v>
       </c>
       <c r="V507" s="1">
-        <v>46290.46660107639</v>
+        <v>46293.42116989583</v>
       </c>
       <c r="W507">
         <v>-3</v>
       </c>
       <c r="X507" t="s">
-        <v>224</v>
-      </c>
-      <c r="Y507" t="s">
-        <v>424</v>
+        <v>226</v>
       </c>
       <c r="AB507">
         <v>0</v>
       </c>
       <c r="AC507" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="AH507" t="s">
         <v>441</v>
       </c>
       <c r="AI507" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="508" spans="1:35">
       <c r="A508">
-        <v>5417</v>
+        <v>6548</v>
       </c>
       <c r="B508" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C508" t="s">
         <v>50</v>
@@ -40157,58 +40154,61 @@
         <v>56</v>
       </c>
       <c r="G508">
-        <v>953</v>
+        <v>11541</v>
       </c>
       <c r="H508">
         <v>0</v>
       </c>
       <c r="I508" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J508" t="s">
-        <v>163</v>
+        <v>144</v>
       </c>
       <c r="N508" s="1">
-        <v>46290</v>
+        <v>46296</v>
       </c>
       <c r="O508" t="s">
         <v>180</v>
       </c>
       <c r="P508">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q508">
         <v>2026</v>
       </c>
       <c r="R508">
-        <v>17398883</v>
+        <v>17222949</v>
       </c>
       <c r="S508" t="s">
-        <v>208</v>
+        <v>200</v>
+      </c>
+      <c r="T508" t="s">
+        <v>215</v>
       </c>
       <c r="U508" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="V508" s="1">
-        <v>46290.67228501158</v>
+        <v>46290.46660107639</v>
       </c>
       <c r="W508">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="X508" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="Y508" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AB508">
         <v>0</v>
       </c>
       <c r="AC508" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="AH508" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="AI508" t="s">
         <v>445</v>
@@ -40216,16 +40216,16 @@
     </row>
     <row r="509" spans="1:35">
       <c r="A509">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B509" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C509" t="s">
         <v>50</v>
       </c>
       <c r="D509" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E509" t="s">
         <v>54</v>
@@ -40258,7 +40258,7 @@
         <v>2026</v>
       </c>
       <c r="R509">
-        <v>16962107</v>
+        <v>17398883</v>
       </c>
       <c r="S509" t="s">
         <v>208</v>
@@ -40267,16 +40267,16 @@
         <v>223</v>
       </c>
       <c r="V509" s="1">
-        <v>46290.67228836806</v>
+        <v>46290.67228501158</v>
       </c>
       <c r="W509">
         <v>3</v>
       </c>
       <c r="X509" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="Y509" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="AB509">
         <v>0</v>
@@ -40293,19 +40293,19 @@
     </row>
     <row r="510" spans="1:35">
       <c r="A510">
-        <v>6627</v>
+        <v>6404</v>
       </c>
       <c r="B510" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C510" t="s">
         <v>50</v>
       </c>
       <c r="D510" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E510" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F510" t="s">
         <v>56</v>
@@ -40335,7 +40335,7 @@
         <v>2026</v>
       </c>
       <c r="R510">
-        <v>17042317</v>
+        <v>16962107</v>
       </c>
       <c r="S510" t="s">
         <v>208</v>
@@ -40344,16 +40344,16 @@
         <v>223</v>
       </c>
       <c r="V510" s="1">
-        <v>46290.67181398148</v>
+        <v>46290.67228836806</v>
       </c>
       <c r="W510">
         <v>3</v>
       </c>
       <c r="X510" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="Y510" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="AB510">
         <v>0</v>
@@ -40370,19 +40370,19 @@
     </row>
     <row r="511" spans="1:35">
       <c r="A511">
-        <v>6703</v>
+        <v>6627</v>
       </c>
       <c r="B511" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C511" t="s">
         <v>50</v>
       </c>
       <c r="D511" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E511" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F511" t="s">
         <v>56</v>
@@ -40412,7 +40412,7 @@
         <v>2026</v>
       </c>
       <c r="R511">
-        <v>17941166</v>
+        <v>17042317</v>
       </c>
       <c r="S511" t="s">
         <v>208</v>
@@ -40421,16 +40421,16 @@
         <v>223</v>
       </c>
       <c r="V511" s="1">
-        <v>46290.67229670139</v>
+        <v>46290.67181398148</v>
       </c>
       <c r="W511">
         <v>3</v>
       </c>
       <c r="X511" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="Y511" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="AB511">
         <v>0</v>
@@ -40447,16 +40447,16 @@
     </row>
     <row r="512" spans="1:35">
       <c r="A512">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B512" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C512" t="s">
         <v>50</v>
       </c>
       <c r="D512" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E512" t="s">
         <v>54</v>
@@ -40489,7 +40489,7 @@
         <v>2026</v>
       </c>
       <c r="R512">
-        <v>17952362</v>
+        <v>17941166</v>
       </c>
       <c r="S512" t="s">
         <v>208</v>
@@ -40498,16 +40498,16 @@
         <v>223</v>
       </c>
       <c r="V512" s="1">
-        <v>46290.6722980324</v>
+        <v>46290.67229670139</v>
       </c>
       <c r="W512">
         <v>3</v>
       </c>
       <c r="X512" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="Y512" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="AB512">
         <v>0</v>
@@ -40524,10 +40524,10 @@
     </row>
     <row r="513" spans="1:35">
       <c r="A513">
-        <v>6949</v>
+        <v>6704</v>
       </c>
       <c r="B513" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C513" t="s">
         <v>50</v>
@@ -40539,7 +40539,7 @@
         <v>54</v>
       </c>
       <c r="F513" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G513">
         <v>953</v>
@@ -40556,6 +40556,9 @@
       <c r="N513" s="1">
         <v>46290</v>
       </c>
+      <c r="O513" t="s">
+        <v>180</v>
+      </c>
       <c r="P513">
         <v>8</v>
       </c>
@@ -40563,7 +40566,7 @@
         <v>2026</v>
       </c>
       <c r="R513">
-        <v>18178144</v>
+        <v>17952362</v>
       </c>
       <c r="S513" t="s">
         <v>208</v>
@@ -40572,16 +40575,16 @@
         <v>223</v>
       </c>
       <c r="V513" s="1">
-        <v>46290.67230081018</v>
+        <v>46290.6722980324</v>
       </c>
       <c r="W513">
         <v>3</v>
       </c>
       <c r="X513" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="Y513" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="AB513">
         <v>0</v>
@@ -40598,16 +40601,16 @@
     </row>
     <row r="514" spans="1:35">
       <c r="A514">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B514" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C514" t="s">
         <v>50</v>
       </c>
       <c r="D514" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E514" t="s">
         <v>54</v>
@@ -40630,9 +40633,6 @@
       <c r="N514" s="1">
         <v>46290</v>
       </c>
-      <c r="O514" t="s">
-        <v>180</v>
-      </c>
       <c r="P514">
         <v>8</v>
       </c>
@@ -40640,7 +40640,7 @@
         <v>2026</v>
       </c>
       <c r="R514">
-        <v>18188731</v>
+        <v>18178144</v>
       </c>
       <c r="S514" t="s">
         <v>208</v>
@@ -40649,16 +40649,16 @@
         <v>223</v>
       </c>
       <c r="V514" s="1">
-        <v>46290.67230141204</v>
+        <v>46290.67230081018</v>
       </c>
       <c r="W514">
         <v>3</v>
       </c>
       <c r="X514" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="Y514" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="AB514">
         <v>0</v>
@@ -40675,10 +40675,10 @@
     </row>
     <row r="515" spans="1:35">
       <c r="A515">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B515" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C515" t="s">
         <v>50</v>
@@ -40717,7 +40717,7 @@
         <v>2026</v>
       </c>
       <c r="R515">
-        <v>18188637</v>
+        <v>18188731</v>
       </c>
       <c r="S515" t="s">
         <v>208</v>
@@ -40726,7 +40726,7 @@
         <v>223</v>
       </c>
       <c r="V515" s="1">
-        <v>46290.67230202546</v>
+        <v>46290.67230141204</v>
       </c>
       <c r="W515">
         <v>3</v>
@@ -40735,7 +40735,7 @@
         <v>228</v>
       </c>
       <c r="Y515" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="AB515">
         <v>0</v>
@@ -40752,10 +40752,10 @@
     </row>
     <row r="516" spans="1:35">
       <c r="A516">
-        <v>6703</v>
+        <v>6963</v>
       </c>
       <c r="B516" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C516" t="s">
         <v>50</v>
@@ -40767,19 +40767,19 @@
         <v>54</v>
       </c>
       <c r="F516" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G516">
-        <v>11056</v>
+        <v>953</v>
       </c>
       <c r="H516">
         <v>0</v>
       </c>
       <c r="I516" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J516" t="s">
-        <v>119</v>
+        <v>163</v>
       </c>
       <c r="N516" s="1">
         <v>46290</v>
@@ -40794,33 +40794,110 @@
         <v>2026</v>
       </c>
       <c r="R516">
-        <v>18284872</v>
+        <v>18188637</v>
+      </c>
+      <c r="S516" t="s">
+        <v>208</v>
       </c>
       <c r="U516" t="s">
         <v>223</v>
       </c>
       <c r="V516" s="1">
-        <v>46290.42450153935</v>
+        <v>46290.67230202546</v>
       </c>
       <c r="W516">
         <v>3</v>
       </c>
       <c r="X516" t="s">
+        <v>228</v>
+      </c>
+      <c r="Y516" t="s">
+        <v>432</v>
+      </c>
+      <c r="AB516">
+        <v>0</v>
+      </c>
+      <c r="AC516" t="s">
+        <v>208</v>
+      </c>
+      <c r="AH516" t="s">
+        <v>440</v>
+      </c>
+      <c r="AI516" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="517" spans="1:35">
+      <c r="A517">
+        <v>6703</v>
+      </c>
+      <c r="B517" t="s">
+        <v>46</v>
+      </c>
+      <c r="C517" t="s">
+        <v>50</v>
+      </c>
+      <c r="D517" t="s">
+        <v>53</v>
+      </c>
+      <c r="E517" t="s">
+        <v>54</v>
+      </c>
+      <c r="F517" t="s">
+        <v>56</v>
+      </c>
+      <c r="G517">
+        <v>11056</v>
+      </c>
+      <c r="H517">
+        <v>0</v>
+      </c>
+      <c r="I517" t="s">
+        <v>66</v>
+      </c>
+      <c r="J517" t="s">
+        <v>119</v>
+      </c>
+      <c r="N517" s="1">
+        <v>46290</v>
+      </c>
+      <c r="O517" t="s">
+        <v>180</v>
+      </c>
+      <c r="P517">
+        <v>8</v>
+      </c>
+      <c r="Q517">
+        <v>2026</v>
+      </c>
+      <c r="R517">
+        <v>18284872</v>
+      </c>
+      <c r="U517" t="s">
+        <v>223</v>
+      </c>
+      <c r="V517" s="1">
+        <v>46290.42450153935</v>
+      </c>
+      <c r="W517">
+        <v>3</v>
+      </c>
+      <c r="X517" t="s">
         <v>233</v>
       </c>
-      <c r="Y516" t="s">
+      <c r="Y517" t="s">
         <v>433</v>
       </c>
-      <c r="AB516">
-        <v>0</v>
-      </c>
-      <c r="AC516" t="s">
+      <c r="AB517">
+        <v>0</v>
+      </c>
+      <c r="AC517" t="s">
         <v>438</v>
       </c>
-      <c r="AH516" t="s">
+      <c r="AH517" t="s">
         <v>439</v>
       </c>
-      <c r="AI516" t="s">
+      <c r="AI517" t="s">
         <v>445</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-28 18:30
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7655" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7669" uniqueCount="451">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1741,7 +1741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI524"/>
+  <dimension ref="A1:AI525"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -40685,10 +40685,10 @@
     </row>
     <row r="515" spans="1:35">
       <c r="A515">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B515" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C515" t="s">
         <v>50</v>
@@ -40700,78 +40700,75 @@
         <v>54</v>
       </c>
       <c r="F515" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G515">
-        <v>953</v>
+        <v>11541</v>
       </c>
       <c r="H515">
         <v>0</v>
       </c>
       <c r="I515" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J515" t="s">
-        <v>163</v>
+        <v>144</v>
       </c>
       <c r="N515" s="1">
-        <v>46290</v>
-      </c>
-      <c r="O515" t="s">
-        <v>180</v>
+        <v>46296</v>
       </c>
       <c r="P515">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q515">
         <v>2026</v>
       </c>
       <c r="R515">
-        <v>17398883</v>
+        <v>18190466</v>
       </c>
       <c r="S515" t="s">
-        <v>208</v>
+        <v>197</v>
+      </c>
+      <c r="T515" t="s">
+        <v>217</v>
       </c>
       <c r="U515" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="V515" s="1">
-        <v>46290.67228501158</v>
+        <v>46293.73434695602</v>
       </c>
       <c r="W515">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="X515" t="s">
-        <v>231</v>
-      </c>
-      <c r="Y515" t="s">
-        <v>429</v>
+        <v>227</v>
       </c>
       <c r="AB515">
         <v>0</v>
       </c>
       <c r="AC515" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="AH515" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="AI515" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="516" spans="1:35">
       <c r="A516">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B516" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C516" t="s">
         <v>50</v>
       </c>
       <c r="D516" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E516" t="s">
         <v>54</v>
@@ -40804,7 +40801,7 @@
         <v>2026</v>
       </c>
       <c r="R516">
-        <v>16962107</v>
+        <v>17398883</v>
       </c>
       <c r="S516" t="s">
         <v>208</v>
@@ -40813,16 +40810,16 @@
         <v>224</v>
       </c>
       <c r="V516" s="1">
-        <v>46290.67228836806</v>
+        <v>46290.67228501158</v>
       </c>
       <c r="W516">
         <v>3</v>
       </c>
       <c r="X516" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="Y516" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="AB516">
         <v>0</v>
@@ -40839,19 +40836,19 @@
     </row>
     <row r="517" spans="1:35">
       <c r="A517">
-        <v>6627</v>
+        <v>6404</v>
       </c>
       <c r="B517" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C517" t="s">
         <v>50</v>
       </c>
       <c r="D517" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E517" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F517" t="s">
         <v>56</v>
@@ -40881,7 +40878,7 @@
         <v>2026</v>
       </c>
       <c r="R517">
-        <v>17042317</v>
+        <v>16962107</v>
       </c>
       <c r="S517" t="s">
         <v>208</v>
@@ -40890,16 +40887,16 @@
         <v>224</v>
       </c>
       <c r="V517" s="1">
-        <v>46290.67181398148</v>
+        <v>46290.67228836806</v>
       </c>
       <c r="W517">
         <v>3</v>
       </c>
       <c r="X517" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="Y517" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="AB517">
         <v>0</v>
@@ -40916,19 +40913,19 @@
     </row>
     <row r="518" spans="1:35">
       <c r="A518">
-        <v>6703</v>
+        <v>6627</v>
       </c>
       <c r="B518" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C518" t="s">
         <v>50</v>
       </c>
       <c r="D518" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E518" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F518" t="s">
         <v>56</v>
@@ -40958,7 +40955,7 @@
         <v>2026</v>
       </c>
       <c r="R518">
-        <v>17941166</v>
+        <v>17042317</v>
       </c>
       <c r="S518" t="s">
         <v>208</v>
@@ -40967,16 +40964,16 @@
         <v>224</v>
       </c>
       <c r="V518" s="1">
-        <v>46290.67229670139</v>
+        <v>46290.67181398148</v>
       </c>
       <c r="W518">
         <v>3</v>
       </c>
       <c r="X518" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="Y518" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="AB518">
         <v>0</v>
@@ -40993,16 +40990,16 @@
     </row>
     <row r="519" spans="1:35">
       <c r="A519">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B519" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C519" t="s">
         <v>50</v>
       </c>
       <c r="D519" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E519" t="s">
         <v>54</v>
@@ -41035,7 +41032,7 @@
         <v>2026</v>
       </c>
       <c r="R519">
-        <v>17952362</v>
+        <v>17941166</v>
       </c>
       <c r="S519" t="s">
         <v>208</v>
@@ -41044,16 +41041,16 @@
         <v>224</v>
       </c>
       <c r="V519" s="1">
-        <v>46290.6722980324</v>
+        <v>46290.67229670139</v>
       </c>
       <c r="W519">
         <v>3</v>
       </c>
       <c r="X519" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="Y519" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="AB519">
         <v>0</v>
@@ -41070,10 +41067,10 @@
     </row>
     <row r="520" spans="1:35">
       <c r="A520">
-        <v>6949</v>
+        <v>6704</v>
       </c>
       <c r="B520" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C520" t="s">
         <v>50</v>
@@ -41085,7 +41082,7 @@
         <v>54</v>
       </c>
       <c r="F520" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G520">
         <v>953</v>
@@ -41102,6 +41099,9 @@
       <c r="N520" s="1">
         <v>46290</v>
       </c>
+      <c r="O520" t="s">
+        <v>180</v>
+      </c>
       <c r="P520">
         <v>8</v>
       </c>
@@ -41109,7 +41109,7 @@
         <v>2026</v>
       </c>
       <c r="R520">
-        <v>18178144</v>
+        <v>17952362</v>
       </c>
       <c r="S520" t="s">
         <v>208</v>
@@ -41118,16 +41118,16 @@
         <v>224</v>
       </c>
       <c r="V520" s="1">
-        <v>46290.67230081018</v>
+        <v>46290.6722980324</v>
       </c>
       <c r="W520">
         <v>3</v>
       </c>
       <c r="X520" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="Y520" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="AB520">
         <v>0</v>
@@ -41144,16 +41144,16 @@
     </row>
     <row r="521" spans="1:35">
       <c r="A521">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B521" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C521" t="s">
         <v>50</v>
       </c>
       <c r="D521" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E521" t="s">
         <v>54</v>
@@ -41176,9 +41176,6 @@
       <c r="N521" s="1">
         <v>46290</v>
       </c>
-      <c r="O521" t="s">
-        <v>180</v>
-      </c>
       <c r="P521">
         <v>8</v>
       </c>
@@ -41186,7 +41183,7 @@
         <v>2026</v>
       </c>
       <c r="R521">
-        <v>18188731</v>
+        <v>18178144</v>
       </c>
       <c r="S521" t="s">
         <v>208</v>
@@ -41195,16 +41192,16 @@
         <v>224</v>
       </c>
       <c r="V521" s="1">
-        <v>46290.67230141204</v>
+        <v>46290.67230081018</v>
       </c>
       <c r="W521">
         <v>3</v>
       </c>
       <c r="X521" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="Y521" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="AB521">
         <v>0</v>
@@ -41221,10 +41218,10 @@
     </row>
     <row r="522" spans="1:35">
       <c r="A522">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B522" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C522" t="s">
         <v>50</v>
@@ -41263,7 +41260,7 @@
         <v>2026</v>
       </c>
       <c r="R522">
-        <v>18188637</v>
+        <v>18188731</v>
       </c>
       <c r="S522" t="s">
         <v>208</v>
@@ -41272,7 +41269,7 @@
         <v>224</v>
       </c>
       <c r="V522" s="1">
-        <v>46290.67230202546</v>
+        <v>46290.67230141204</v>
       </c>
       <c r="W522">
         <v>3</v>
@@ -41281,7 +41278,7 @@
         <v>229</v>
       </c>
       <c r="Y522" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="AB522">
         <v>0</v>
@@ -41298,10 +41295,10 @@
     </row>
     <row r="523" spans="1:35">
       <c r="A523">
-        <v>6703</v>
+        <v>6963</v>
       </c>
       <c r="B523" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C523" t="s">
         <v>50</v>
@@ -41313,19 +41310,19 @@
         <v>54</v>
       </c>
       <c r="F523" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G523">
-        <v>11056</v>
+        <v>953</v>
       </c>
       <c r="H523">
         <v>0</v>
       </c>
       <c r="I523" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J523" t="s">
-        <v>119</v>
+        <v>163</v>
       </c>
       <c r="N523" s="1">
         <v>46290</v>
@@ -41340,31 +41337,34 @@
         <v>2026</v>
       </c>
       <c r="R523">
-        <v>18284872</v>
+        <v>18188637</v>
+      </c>
+      <c r="S523" t="s">
+        <v>208</v>
       </c>
       <c r="U523" t="s">
         <v>224</v>
       </c>
       <c r="V523" s="1">
-        <v>46290.42450153935</v>
+        <v>46290.67230202546</v>
       </c>
       <c r="W523">
         <v>3</v>
       </c>
       <c r="X523" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="Y523" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AB523">
         <v>0</v>
       </c>
       <c r="AC523" t="s">
-        <v>442</v>
+        <v>208</v>
       </c>
       <c r="AH523" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="AI523" t="s">
         <v>449</v>
@@ -41372,22 +41372,22 @@
     </row>
     <row r="524" spans="1:35">
       <c r="A524">
-        <v>6949</v>
+        <v>6703</v>
       </c>
       <c r="B524" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C524" t="s">
         <v>50</v>
       </c>
       <c r="D524" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E524" t="s">
         <v>54</v>
       </c>
       <c r="F524" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G524">
         <v>11056</v>
@@ -41402,10 +41402,10 @@
         <v>119</v>
       </c>
       <c r="N524" s="1">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="O524" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="P524">
         <v>8</v>
@@ -41414,36 +41414,110 @@
         <v>2026</v>
       </c>
       <c r="R524">
-        <v>18279142</v>
-      </c>
-      <c r="S524" t="s">
-        <v>211</v>
+        <v>18284872</v>
       </c>
       <c r="U524" t="s">
         <v>224</v>
       </c>
       <c r="V524" s="1">
-        <v>46293.62664548611</v>
+        <v>46290.42450153935</v>
       </c>
       <c r="W524">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X524" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="Y524" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="AB524">
         <v>0</v>
       </c>
       <c r="AC524" t="s">
-        <v>211</v>
+        <v>442</v>
       </c>
       <c r="AH524" t="s">
         <v>443</v>
       </c>
       <c r="AI524" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="525" spans="1:35">
+      <c r="A525">
+        <v>6949</v>
+      </c>
+      <c r="B525" t="s">
+        <v>37</v>
+      </c>
+      <c r="C525" t="s">
+        <v>50</v>
+      </c>
+      <c r="D525" t="s">
+        <v>51</v>
+      </c>
+      <c r="E525" t="s">
+        <v>54</v>
+      </c>
+      <c r="F525" t="s">
+        <v>57</v>
+      </c>
+      <c r="G525">
+        <v>11056</v>
+      </c>
+      <c r="H525">
+        <v>0</v>
+      </c>
+      <c r="I525" t="s">
+        <v>66</v>
+      </c>
+      <c r="J525" t="s">
+        <v>119</v>
+      </c>
+      <c r="N525" s="1">
+        <v>46293</v>
+      </c>
+      <c r="O525" t="s">
+        <v>177</v>
+      </c>
+      <c r="P525">
+        <v>8</v>
+      </c>
+      <c r="Q525">
+        <v>2026</v>
+      </c>
+      <c r="R525">
+        <v>18279142</v>
+      </c>
+      <c r="S525" t="s">
+        <v>211</v>
+      </c>
+      <c r="U525" t="s">
+        <v>224</v>
+      </c>
+      <c r="V525" s="1">
+        <v>46293.62664548611</v>
+      </c>
+      <c r="W525">
+        <v>0</v>
+      </c>
+      <c r="X525" t="s">
+        <v>227</v>
+      </c>
+      <c r="Y525" t="s">
+        <v>438</v>
+      </c>
+      <c r="AB525">
+        <v>0</v>
+      </c>
+      <c r="AC525" t="s">
+        <v>211</v>
+      </c>
+      <c r="AH525" t="s">
+        <v>443</v>
+      </c>
+      <c r="AI525" t="s">
         <v>450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-29 08:44
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -1907,7 +1907,7 @@
         <v>46268.63953865741</v>
       </c>
       <c r="W2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X2" t="s">
         <v>225</v>
@@ -1984,7 +1984,7 @@
         <v>46266.57730150463</v>
       </c>
       <c r="W3">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X3" t="s">
         <v>226</v>
@@ -2061,7 +2061,7 @@
         <v>46266.41668148148</v>
       </c>
       <c r="W4">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X4" t="s">
         <v>227</v>
@@ -2138,7 +2138,7 @@
         <v>46267.75233784723</v>
       </c>
       <c r="W5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X5" t="s">
         <v>225</v>
@@ -2212,7 +2212,7 @@
         <v>46267.75233927083</v>
       </c>
       <c r="W6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X6" t="s">
         <v>226</v>
@@ -2286,7 +2286,7 @@
         <v>46267.7523394676</v>
       </c>
       <c r="W7">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X7" t="s">
         <v>226</v>
@@ -2360,7 +2360,7 @@
         <v>46267.75234278935</v>
       </c>
       <c r="W8">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X8" t="s">
         <v>228</v>
@@ -2434,7 +2434,7 @@
         <v>46267.75234309028</v>
       </c>
       <c r="W9">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X9" t="s">
         <v>227</v>
@@ -2508,7 +2508,7 @@
         <v>46267.75234383102</v>
       </c>
       <c r="W10">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X10" t="s">
         <v>229</v>
@@ -2582,7 +2582,7 @@
         <v>46267.75234424769</v>
       </c>
       <c r="W11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X11" t="s">
         <v>229</v>
@@ -2656,7 +2656,7 @@
         <v>46267.47365627315</v>
       </c>
       <c r="W12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X12" t="s">
         <v>230</v>
@@ -2730,7 +2730,7 @@
         <v>46266.47620831019</v>
       </c>
       <c r="W13">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X13" t="s">
         <v>231</v>
@@ -2804,7 +2804,7 @@
         <v>46267.57586420139</v>
       </c>
       <c r="W14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X14" t="s">
         <v>232</v>
@@ -2875,7 +2875,7 @@
         <v>46266.44145744213</v>
       </c>
       <c r="W15">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="X15" t="s">
         <v>233</v>
@@ -2943,7 +2943,7 @@
         <v>46266.44156952546</v>
       </c>
       <c r="W16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X16" t="s">
         <v>233</v>
@@ -3011,7 +3011,7 @@
         <v>46266.44152346065</v>
       </c>
       <c r="W17">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="X17" t="s">
         <v>233</v>
@@ -3085,7 +3085,7 @@
         <v>46269.3962034375</v>
       </c>
       <c r="W18">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X18" t="s">
         <v>234</v>
@@ -3162,7 +3162,7 @@
         <v>46268.54759884259</v>
       </c>
       <c r="W19">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X19" t="s">
         <v>231</v>
@@ -3239,7 +3239,7 @@
         <v>46269.38216940972</v>
       </c>
       <c r="W20">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X20" t="s">
         <v>232</v>
@@ -3316,7 +3316,7 @@
         <v>46269.40844942129</v>
       </c>
       <c r="W21">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X21" t="s">
         <v>230</v>
@@ -3393,7 +3393,7 @@
         <v>46266.37634084491</v>
       </c>
       <c r="W22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X22" t="s">
         <v>235</v>
@@ -3467,7 +3467,7 @@
         <v>46267.47452163194</v>
       </c>
       <c r="W23">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X23" t="s">
         <v>230</v>
@@ -3541,7 +3541,7 @@
         <v>46267.4745221412</v>
       </c>
       <c r="W24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X24" t="s">
         <v>230</v>
@@ -3615,7 +3615,7 @@
         <v>46267.47452299768</v>
       </c>
       <c r="W25">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X25" t="s">
         <v>230</v>
@@ -3689,7 +3689,7 @@
         <v>46267.75231010417</v>
       </c>
       <c r="W26">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X26" t="s">
         <v>231</v>
@@ -3763,7 +3763,7 @@
         <v>46267.75234059028</v>
       </c>
       <c r="W27">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X27" t="s">
         <v>230</v>
@@ -3837,7 +3837,7 @@
         <v>46267.7523409375</v>
       </c>
       <c r="W28">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X28" t="s">
         <v>230</v>
@@ -3911,7 +3911,7 @@
         <v>46267.75234170139</v>
       </c>
       <c r="W29">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X29" t="s">
         <v>230</v>
@@ -3985,7 +3985,7 @@
         <v>46268.58940019676</v>
       </c>
       <c r="W30">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X30" t="s">
         <v>234</v>
@@ -4062,7 +4062,7 @@
         <v>46268.37896984954</v>
       </c>
       <c r="W31">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X31" t="s">
         <v>226</v>
@@ -4139,7 +4139,7 @@
         <v>46269.71652982639</v>
       </c>
       <c r="W32">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X32" t="s">
         <v>228</v>
@@ -4216,7 +4216,7 @@
         <v>46269.71069613426</v>
       </c>
       <c r="W33">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X33" t="s">
         <v>227</v>
@@ -4296,7 +4296,7 @@
         <v>46267.55838734953</v>
       </c>
       <c r="W34">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="X34" t="s">
         <v>231</v>
@@ -4376,7 +4376,7 @@
         <v>46273.59003707176</v>
       </c>
       <c r="W35">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X35" t="s">
         <v>235</v>
@@ -4456,7 +4456,7 @@
         <v>46268.74069754629</v>
       </c>
       <c r="W36">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X36" t="s">
         <v>225</v>
@@ -4536,7 +4536,7 @@
         <v>46273.45940115741</v>
       </c>
       <c r="W37">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X37" t="s">
         <v>234</v>
@@ -4616,7 +4616,7 @@
         <v>46267.66088636574</v>
       </c>
       <c r="W38">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X38" t="s">
         <v>231</v>
@@ -4696,7 +4696,7 @@
         <v>46268.45922827546</v>
       </c>
       <c r="W39">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X39" t="s">
         <v>232</v>
@@ -4776,7 +4776,7 @@
         <v>46269.59248078704</v>
       </c>
       <c r="W40">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X40" t="s">
         <v>226</v>
@@ -4856,7 +4856,7 @@
         <v>46269.59224453704</v>
       </c>
       <c r="W41">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X41" t="s">
         <v>226</v>
@@ -4936,7 +4936,7 @@
         <v>46268.5891771875</v>
       </c>
       <c r="W42">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X42" t="s">
         <v>234</v>
@@ -5016,7 +5016,7 @@
         <v>46267.64795916666</v>
       </c>
       <c r="W43">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X43" t="s">
         <v>230</v>
@@ -5096,7 +5096,7 @@
         <v>46267.4478849537</v>
       </c>
       <c r="W44">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X44" t="s">
         <v>228</v>
@@ -5176,7 +5176,7 @@
         <v>46269.59056300926</v>
       </c>
       <c r="W45">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X45" t="s">
         <v>227</v>
@@ -5253,7 +5253,7 @@
         <v>46273.67026252315</v>
       </c>
       <c r="W46">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X46" t="s">
         <v>231</v>
@@ -5327,7 +5327,7 @@
         <v>46269.677524375</v>
       </c>
       <c r="W47">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X47" t="s">
         <v>232</v>
@@ -5401,7 +5401,7 @@
         <v>46269.677525</v>
       </c>
       <c r="W48">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X48" t="s">
         <v>226</v>
@@ -5475,7 +5475,7 @@
         <v>46269.677525625</v>
       </c>
       <c r="W49">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X49" t="s">
         <v>226</v>
@@ -5549,7 +5549,7 @@
         <v>46268.58906282407</v>
       </c>
       <c r="W50">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X50" t="s">
         <v>234</v>
@@ -5623,7 +5623,7 @@
         <v>46267.64761306713</v>
       </c>
       <c r="W51">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X51" t="s">
         <v>230</v>
@@ -5700,7 +5700,7 @@
         <v>46273.64957155092</v>
       </c>
       <c r="W52">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X52" t="s">
         <v>228</v>
@@ -5777,7 +5777,7 @@
         <v>46273.39871140046</v>
       </c>
       <c r="W53">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X53" t="s">
         <v>227</v>
@@ -5854,7 +5854,7 @@
         <v>46267.35832805555</v>
       </c>
       <c r="W54">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="X54" t="s">
         <v>232</v>
@@ -5934,7 +5934,7 @@
         <v>46268.71229238426</v>
       </c>
       <c r="W55">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="X55" t="s">
         <v>226</v>
@@ -6014,7 +6014,7 @@
         <v>46268.71229297454</v>
       </c>
       <c r="W56">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="X56" t="s">
         <v>226</v>
@@ -6094,7 +6094,7 @@
         <v>46267.74532275463</v>
       </c>
       <c r="W57">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="X57" t="s">
         <v>234</v>
@@ -6174,7 +6174,7 @@
         <v>46269.60160202546</v>
       </c>
       <c r="W58">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X58" t="s">
         <v>231</v>
@@ -6254,7 +6254,7 @@
         <v>46273.64508760416</v>
       </c>
       <c r="W59">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X59" t="s">
         <v>235</v>
@@ -6334,7 +6334,7 @@
         <v>46268.45926839121</v>
       </c>
       <c r="W60">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X60" t="s">
         <v>232</v>
@@ -6414,7 +6414,7 @@
         <v>46269.59250902777</v>
       </c>
       <c r="W61">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X61" t="s">
         <v>226</v>
@@ -6494,7 +6494,7 @@
         <v>46269.5922865625</v>
       </c>
       <c r="W62">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X62" t="s">
         <v>226</v>
@@ -6574,7 +6574,7 @@
         <v>46268.58922707176</v>
       </c>
       <c r="W63">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X63" t="s">
         <v>234</v>
@@ -6654,7 +6654,7 @@
         <v>46267.64800344907</v>
       </c>
       <c r="W64">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X64" t="s">
         <v>230</v>
@@ -6734,7 +6734,7 @@
         <v>46267.44799793982</v>
       </c>
       <c r="W65">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X65" t="s">
         <v>228</v>
@@ -6814,7 +6814,7 @@
         <v>46269.59070487269</v>
       </c>
       <c r="W66">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X66" t="s">
         <v>227</v>
@@ -6894,7 +6894,7 @@
         <v>46269.49635894676</v>
       </c>
       <c r="W67">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X67" t="s">
         <v>232</v>
@@ -6971,7 +6971,7 @@
         <v>46269.63659284722</v>
       </c>
       <c r="W68">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X68" t="s">
         <v>231</v>
@@ -7045,7 +7045,7 @@
         <v>46273.64532122685</v>
       </c>
       <c r="W69">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X69" t="s">
         <v>235</v>
@@ -7119,7 +7119,7 @@
         <v>46268.45929986111</v>
       </c>
       <c r="W70">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X70" t="s">
         <v>232</v>
@@ -7193,7 +7193,7 @@
         <v>46269.5925421875</v>
       </c>
       <c r="W71">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X71" t="s">
         <v>226</v>
@@ -7267,7 +7267,7 @@
         <v>46269.59231454861</v>
       </c>
       <c r="W72">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X72" t="s">
         <v>226</v>
@@ -7341,7 +7341,7 @@
         <v>46268.58932953704</v>
       </c>
       <c r="W73">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X73" t="s">
         <v>234</v>
@@ -7415,7 +7415,7 @@
         <v>46267.648038125</v>
       </c>
       <c r="W74">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X74" t="s">
         <v>230</v>
@@ -7489,7 +7489,7 @@
         <v>46267.44824061343</v>
       </c>
       <c r="W75">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X75" t="s">
         <v>228</v>
@@ -7563,7 +7563,7 @@
         <v>46269.59082328704</v>
       </c>
       <c r="W76">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X76" t="s">
         <v>227</v>
@@ -7634,7 +7634,7 @@
         <v>46273.63629708334</v>
       </c>
       <c r="W77">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X77" t="s">
         <v>227</v>
@@ -7708,7 +7708,7 @@
         <v>46273.64318633102</v>
       </c>
       <c r="W78">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X78" t="s">
         <v>227</v>
@@ -7782,7 +7782,7 @@
         <v>46273.64880981482</v>
       </c>
       <c r="W79">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X79" t="s">
         <v>227</v>
@@ -7859,7 +7859,7 @@
         <v>46267.72055925926</v>
       </c>
       <c r="W80">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X80" t="s">
         <v>225</v>
@@ -7933,7 +7933,7 @@
         <v>46267.79441380787</v>
       </c>
       <c r="W81">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X81" t="s">
         <v>226</v>
@@ -8004,7 +8004,7 @@
         <v>46267.79441215278</v>
       </c>
       <c r="W82">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X82" t="s">
         <v>227</v>
@@ -8078,7 +8078,7 @@
         <v>46267.7205502662</v>
       </c>
       <c r="W83">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X83" t="s">
         <v>225</v>
@@ -8152,7 +8152,7 @@
         <v>46267.79439748843</v>
       </c>
       <c r="W84">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X84" t="s">
         <v>226</v>
@@ -8223,7 +8223,7 @@
         <v>46267.79440011574</v>
       </c>
       <c r="W85">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X85" t="s">
         <v>228</v>
@@ -8294,7 +8294,7 @@
         <v>46267.79439818287</v>
       </c>
       <c r="W86">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X86" t="s">
         <v>227</v>
@@ -8365,7 +8365,7 @@
         <v>46267.7202693287</v>
       </c>
       <c r="W87">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X87" t="s">
         <v>225</v>
@@ -8439,7 +8439,7 @@
         <v>46267.79409846065</v>
       </c>
       <c r="W88">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X88" t="s">
         <v>226</v>
@@ -8513,7 +8513,7 @@
         <v>46267.79409725694</v>
       </c>
       <c r="W89">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X89" t="s">
         <v>226</v>
@@ -8581,7 +8581,7 @@
         <v>46267.79410239583</v>
       </c>
       <c r="W90">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X90" t="s">
         <v>228</v>
@@ -8649,7 +8649,7 @@
         <v>46267.79409934028</v>
       </c>
       <c r="W91">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X91" t="s">
         <v>227</v>
@@ -8720,7 +8720,7 @@
         <v>46267.72033356482</v>
       </c>
       <c r="W92">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X92" t="s">
         <v>225</v>
@@ -8794,7 +8794,7 @@
         <v>46267.79418105324</v>
       </c>
       <c r="W93">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X93" t="s">
         <v>226</v>
@@ -8868,7 +8868,7 @@
         <v>46267.79418005787</v>
       </c>
       <c r="W94">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X94" t="s">
         <v>226</v>
@@ -8936,7 +8936,7 @@
         <v>46267.79418379629</v>
       </c>
       <c r="W95">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X95" t="s">
         <v>228</v>
@@ -9004,7 +9004,7 @@
         <v>46267.79418283565</v>
       </c>
       <c r="W96">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X96" t="s">
         <v>227</v>
@@ -9075,7 +9075,7 @@
         <v>46267.71937662037</v>
       </c>
       <c r="W97">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X97" t="s">
         <v>225</v>
@@ -9149,7 +9149,7 @@
         <v>46267.79259834491</v>
       </c>
       <c r="W98">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X98" t="s">
         <v>226</v>
@@ -9220,7 +9220,7 @@
         <v>46267.79260170139</v>
       </c>
       <c r="W99">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X99" t="s">
         <v>227</v>
@@ -9297,7 +9297,7 @@
         <v>46268.37621265047</v>
       </c>
       <c r="W100">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X100" t="s">
         <v>229</v>
@@ -9374,7 +9374,7 @@
         <v>46267.79440636574</v>
       </c>
       <c r="W101">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X101" t="s">
         <v>228</v>
@@ -9448,7 +9448,7 @@
         <v>46267.72037954861</v>
       </c>
       <c r="W102">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X102" t="s">
         <v>225</v>
@@ -9522,7 +9522,7 @@
         <v>46267.79424664352</v>
       </c>
       <c r="W103">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X103" t="s">
         <v>226</v>
@@ -9596,7 +9596,7 @@
         <v>46267.79424586806</v>
       </c>
       <c r="W104">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X104" t="s">
         <v>226</v>
@@ -9664,7 +9664,7 @@
         <v>46267.79424864583</v>
       </c>
       <c r="W105">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X105" t="s">
         <v>228</v>
@@ -9732,7 +9732,7 @@
         <v>46267.79424725694</v>
       </c>
       <c r="W106">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X106" t="s">
         <v>227</v>
@@ -9803,7 +9803,7 @@
         <v>46267.79425081018</v>
       </c>
       <c r="W107">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X107" t="s">
         <v>229</v>
@@ -9877,7 +9877,7 @@
         <v>46267.71942916667</v>
       </c>
       <c r="W108">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X108" t="s">
         <v>225</v>
@@ -9951,7 +9951,7 @@
         <v>46267.79268530093</v>
       </c>
       <c r="W109">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X109" t="s">
         <v>228</v>
@@ -10022,7 +10022,7 @@
         <v>46267.79268769676</v>
       </c>
       <c r="W110">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X110" t="s">
         <v>227</v>
@@ -10096,7 +10096,7 @@
         <v>46267.79249748842</v>
       </c>
       <c r="W111">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X111" t="s">
         <v>228</v>
@@ -10167,7 +10167,7 @@
         <v>46267.79249788194</v>
       </c>
       <c r="W112">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X112" t="s">
         <v>227</v>
@@ -10241,7 +10241,7 @@
         <v>46267.71927280092</v>
       </c>
       <c r="W113">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X113" t="s">
         <v>225</v>
@@ -10315,7 +10315,7 @@
         <v>46267.79251079861</v>
       </c>
       <c r="W114">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X114" t="s">
         <v>228</v>
@@ -10386,7 +10386,7 @@
         <v>46267.79251038194</v>
       </c>
       <c r="W115">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X115" t="s">
         <v>227</v>
@@ -10460,7 +10460,7 @@
         <v>46267.72044811342</v>
       </c>
       <c r="W116">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X116" t="s">
         <v>225</v>
@@ -10534,7 +10534,7 @@
         <v>46267.79429737268</v>
       </c>
       <c r="W117">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X117" t="s">
         <v>226</v>
@@ -10608,7 +10608,7 @@
         <v>46267.79429603009</v>
       </c>
       <c r="W118">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X118" t="s">
         <v>226</v>
@@ -10676,7 +10676,7 @@
         <v>46267.79429876158</v>
       </c>
       <c r="W119">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X119" t="s">
         <v>228</v>
@@ -10744,7 +10744,7 @@
         <v>46267.79429826389</v>
       </c>
       <c r="W120">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X120" t="s">
         <v>227</v>
@@ -10815,7 +10815,7 @@
         <v>46267.72050385417</v>
       </c>
       <c r="W121">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X121" t="s">
         <v>225</v>
@@ -10889,7 +10889,7 @@
         <v>46267.79434996528</v>
       </c>
       <c r="W122">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X122" t="s">
         <v>226</v>
@@ -10963,7 +10963,7 @@
         <v>46267.79434864583</v>
       </c>
       <c r="W123">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X123" t="s">
         <v>226</v>
@@ -11031,7 +11031,7 @@
         <v>46267.79435208334</v>
       </c>
       <c r="W124">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X124" t="s">
         <v>228</v>
@@ -11099,7 +11099,7 @@
         <v>46267.79435100695</v>
       </c>
       <c r="W125">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X125" t="s">
         <v>227</v>
@@ -11170,7 +11170,7 @@
         <v>46273.6788224074</v>
       </c>
       <c r="W126">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X126" t="s">
         <v>227</v>
@@ -11247,7 +11247,7 @@
         <v>46273.67943539352</v>
       </c>
       <c r="W127">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X127" t="s">
         <v>227</v>
@@ -11324,7 +11324,7 @@
         <v>46266.37636392361</v>
       </c>
       <c r="W128">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X128" t="s">
         <v>231</v>
@@ -11398,7 +11398,7 @@
         <v>46266.37598834491</v>
       </c>
       <c r="W129">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X129" t="s">
         <v>231</v>
@@ -11475,7 +11475,7 @@
         <v>46268.45899988426</v>
       </c>
       <c r="W130">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X130" t="s">
         <v>232</v>
@@ -11552,7 +11552,7 @@
         <v>46266.45957881944</v>
       </c>
       <c r="W131">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X131" t="s">
         <v>230</v>
@@ -11626,7 +11626,7 @@
         <v>46266.37645462963</v>
       </c>
       <c r="W132">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X132" t="s">
         <v>231</v>
@@ -11700,7 +11700,7 @@
         <v>46266.37649475694</v>
       </c>
       <c r="W133">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X133" t="s">
         <v>231</v>
@@ -11774,7 +11774,7 @@
         <v>46266.37591180555</v>
       </c>
       <c r="W134">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X134" t="s">
         <v>231</v>
@@ -11851,7 +11851,7 @@
         <v>46268.45896508102</v>
       </c>
       <c r="W135">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X135" t="s">
         <v>232</v>
@@ -11928,7 +11928,7 @@
         <v>46266.45946195602</v>
       </c>
       <c r="W136">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X136" t="s">
         <v>230</v>
@@ -12002,7 +12002,7 @@
         <v>46266.37538684028</v>
       </c>
       <c r="W137">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X137" t="s">
         <v>231</v>
@@ -12076,7 +12076,7 @@
         <v>46266.37538506944</v>
       </c>
       <c r="W138">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X138" t="s">
         <v>235</v>
@@ -12153,7 +12153,7 @@
         <v>46268.45881820602</v>
       </c>
       <c r="W139">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X139" t="s">
         <v>232</v>
@@ -12230,7 +12230,7 @@
         <v>46266.45895332176</v>
       </c>
       <c r="W140">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X140" t="s">
         <v>234</v>
@@ -12304,7 +12304,7 @@
         <v>46266.45874105324</v>
       </c>
       <c r="W141">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X141" t="s">
         <v>230</v>
@@ -12378,7 +12378,7 @@
         <v>46266.45873584491</v>
       </c>
       <c r="W142">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X142" t="s">
         <v>230</v>
@@ -12452,7 +12452,7 @@
         <v>46273.6799675</v>
       </c>
       <c r="W143">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X143" t="s">
         <v>230</v>
@@ -12526,7 +12526,7 @@
         <v>46273.55254606481</v>
       </c>
       <c r="W144">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X144" t="s">
         <v>231</v>
@@ -12600,7 +12600,7 @@
         <v>46273.55252126158</v>
       </c>
       <c r="W145">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X145" t="s">
         <v>235</v>
@@ -12674,7 +12674,7 @@
         <v>46273.55254163194</v>
       </c>
       <c r="W146">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X146" t="s">
         <v>232</v>
@@ -12748,7 +12748,7 @@
         <v>46273.5525440162</v>
       </c>
       <c r="W147">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X147" t="s">
         <v>234</v>
@@ -12822,7 +12822,7 @@
         <v>46273.84422141204</v>
       </c>
       <c r="W148">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X148" t="s">
         <v>230</v>
@@ -12896,7 +12896,7 @@
         <v>46273.55254652778</v>
       </c>
       <c r="W149">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X149" t="s">
         <v>230</v>
@@ -12973,7 +12973,7 @@
         <v>46268.45898549769</v>
       </c>
       <c r="W150">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X150" t="s">
         <v>232</v>
@@ -13050,7 +13050,7 @@
         <v>46268.45915543981</v>
       </c>
       <c r="W151">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X151" t="s">
         <v>232</v>
@@ -13124,7 +13124,7 @@
         <v>46273.56305208334</v>
       </c>
       <c r="W152">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X152" t="s">
         <v>230</v>
@@ -13198,7 +13198,7 @@
         <v>46267.44505795139</v>
       </c>
       <c r="W153">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X153" t="s">
         <v>230</v>
@@ -13269,7 +13269,7 @@
         <v>46266.25305112269</v>
       </c>
       <c r="W154">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X154" t="s">
         <v>231</v>
@@ -13343,7 +13343,7 @@
         <v>46266.25275173611</v>
       </c>
       <c r="W155">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X155" t="s">
         <v>226</v>
@@ -13417,7 +13417,7 @@
         <v>46266.25364869213</v>
       </c>
       <c r="W156">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X156" t="s">
         <v>230</v>
@@ -13491,7 +13491,7 @@
         <v>46266.25369988426</v>
       </c>
       <c r="W157">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X157" t="s">
         <v>227</v>
@@ -13568,7 +13568,7 @@
         <v>46268.62318445602</v>
       </c>
       <c r="W158">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X158" t="s">
         <v>231</v>
@@ -13645,7 +13645,7 @@
         <v>46268.62319864584</v>
       </c>
       <c r="W159">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X159" t="s">
         <v>235</v>
@@ -13722,7 +13722,7 @@
         <v>46268.62320026621</v>
       </c>
       <c r="W160">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X160" t="s">
         <v>232</v>
@@ -13799,7 +13799,7 @@
         <v>46268.62320177083</v>
       </c>
       <c r="W161">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X161" t="s">
         <v>225</v>
@@ -13876,7 +13876,7 @@
         <v>46268.62320378472</v>
       </c>
       <c r="W162">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X162" t="s">
         <v>226</v>
@@ -13953,7 +13953,7 @@
         <v>46268.62320393518</v>
       </c>
       <c r="W163">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X163" t="s">
         <v>226</v>
@@ -14030,7 +14030,7 @@
         <v>46268.62320697917</v>
       </c>
       <c r="W164">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X164" t="s">
         <v>234</v>
@@ -14107,7 +14107,7 @@
         <v>46268.62320717592</v>
       </c>
       <c r="W165">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X165" t="s">
         <v>230</v>
@@ -14184,7 +14184,7 @@
         <v>46268.62320732639</v>
       </c>
       <c r="W166">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X166" t="s">
         <v>230</v>
@@ -14261,7 +14261,7 @@
         <v>46268.62320810185</v>
       </c>
       <c r="W167">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X167" t="s">
         <v>230</v>
@@ -14338,7 +14338,7 @@
         <v>46268.6232125</v>
       </c>
       <c r="W168">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X168" t="s">
         <v>228</v>
@@ -14415,7 +14415,7 @@
         <v>46268.62321412037</v>
       </c>
       <c r="W169">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X169" t="s">
         <v>227</v>
@@ -14492,7 +14492,7 @@
         <v>46268.6232128125</v>
       </c>
       <c r="W170">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X170" t="s">
         <v>229</v>
@@ -14569,7 +14569,7 @@
         <v>46268.62321296296</v>
       </c>
       <c r="W171">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X171" t="s">
         <v>229</v>
@@ -14643,7 +14643,7 @@
         <v>46269.41908927084</v>
       </c>
       <c r="W172">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X172" t="s">
         <v>231</v>
@@ -14714,7 +14714,7 @@
         <v>46269.41910457176</v>
       </c>
       <c r="W173">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X173" t="s">
         <v>235</v>
@@ -14785,7 +14785,7 @@
         <v>46269.37885223379</v>
       </c>
       <c r="W174">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X174" t="s">
         <v>232</v>
@@ -14856,7 +14856,7 @@
         <v>46269.3782503125</v>
       </c>
       <c r="W175">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X175" t="s">
         <v>225</v>
@@ -14927,7 +14927,7 @@
         <v>46269.41913152778</v>
       </c>
       <c r="W176">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X176" t="s">
         <v>226</v>
@@ -14998,7 +14998,7 @@
         <v>46269.41913775463</v>
       </c>
       <c r="W177">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X177" t="s">
         <v>226</v>
@@ -15069,7 +15069,7 @@
         <v>46268.7596207176</v>
       </c>
       <c r="W178">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X178" t="s">
         <v>231</v>
@@ -15140,7 +15140,7 @@
         <v>46268.75963109954</v>
       </c>
       <c r="W179">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X179" t="s">
         <v>235</v>
@@ -15211,7 +15211,7 @@
         <v>46268.75963225694</v>
       </c>
       <c r="W180">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X180" t="s">
         <v>232</v>
@@ -15282,7 +15282,7 @@
         <v>46268.75963348379</v>
       </c>
       <c r="W181">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X181" t="s">
         <v>225</v>
@@ -15353,7 +15353,7 @@
         <v>46268.75963414352</v>
       </c>
       <c r="W182">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X182" t="s">
         <v>226</v>
@@ -15424,7 +15424,7 @@
         <v>46268.62326365741</v>
       </c>
       <c r="W183">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X183" t="s">
         <v>226</v>
@@ -15495,7 +15495,7 @@
         <v>46268.75963472222</v>
       </c>
       <c r="W184">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X184" t="s">
         <v>234</v>
@@ -15566,7 +15566,7 @@
         <v>46268.75963475694</v>
       </c>
       <c r="W185">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X185" t="s">
         <v>230</v>
@@ -15637,7 +15637,7 @@
         <v>46268.75963506944</v>
       </c>
       <c r="W186">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X186" t="s">
         <v>230</v>
@@ -15708,7 +15708,7 @@
         <v>46268.7596360301</v>
       </c>
       <c r="W187">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X187" t="s">
         <v>230</v>
@@ -15779,7 +15779,7 @@
         <v>46268.62327121528</v>
       </c>
       <c r="W188">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X188" t="s">
         <v>228</v>
@@ -15850,7 +15850,7 @@
         <v>46268.75963931713</v>
       </c>
       <c r="W189">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X189" t="s">
         <v>227</v>
@@ -15921,7 +15921,7 @@
         <v>46268.75963822917</v>
       </c>
       <c r="W190">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X190" t="s">
         <v>229</v>
@@ -15992,7 +15992,7 @@
         <v>46268.75963857639</v>
       </c>
       <c r="W191">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X191" t="s">
         <v>229</v>
@@ -16063,7 +16063,7 @@
         <v>46269.41908901621</v>
       </c>
       <c r="W192">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X192" t="s">
         <v>231</v>
@@ -16134,7 +16134,7 @@
         <v>46269.41910425926</v>
       </c>
       <c r="W193">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X193" t="s">
         <v>235</v>
@@ -16205,7 +16205,7 @@
         <v>46269.37890997685</v>
       </c>
       <c r="W194">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X194" t="s">
         <v>232</v>
@@ -16276,7 +16276,7 @@
         <v>46269.37833320602</v>
       </c>
       <c r="W195">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X195" t="s">
         <v>225</v>
@@ -16347,7 +16347,7 @@
         <v>46269.41913112268</v>
       </c>
       <c r="W196">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X196" t="s">
         <v>226</v>
@@ -16418,7 +16418,7 @@
         <v>46269.41913740741</v>
       </c>
       <c r="W197">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X197" t="s">
         <v>226</v>
@@ -16489,7 +16489,7 @@
         <v>46267.66131466435</v>
       </c>
       <c r="W198">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X198" t="s">
         <v>235</v>
@@ -16563,7 +16563,7 @@
         <v>46266.21595836805</v>
       </c>
       <c r="W199">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="X199" t="s">
         <v>235</v>
@@ -16637,7 +16637,7 @@
         <v>46266.21572962963</v>
       </c>
       <c r="W200">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="X200" t="s">
         <v>231</v>
@@ -16711,7 +16711,7 @@
         <v>46266.21550011574</v>
       </c>
       <c r="W201">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="X201" t="s">
         <v>232</v>
@@ -16785,7 +16785,7 @@
         <v>46266.00006921296</v>
       </c>
       <c r="W202">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="X202" t="s">
         <v>231</v>
@@ -16856,7 +16856,7 @@
         <v>46266.00006921296</v>
       </c>
       <c r="W203">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="X203" t="s">
         <v>235</v>
@@ -16924,7 +16924,7 @@
         <v>46269.57097615741</v>
       </c>
       <c r="W204">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="X204" t="s">
         <v>232</v>
@@ -16992,7 +16992,7 @@
         <v>46266.00006921296</v>
       </c>
       <c r="W205">
-        <v>-28</v>
+        <v>-27</v>
       </c>
       <c r="X205" t="s">
         <v>232</v>
@@ -17060,7 +17060,7 @@
         <v>46269.46753030093</v>
       </c>
       <c r="W206">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X206" t="s">
         <v>228</v>
@@ -17137,7 +17137,7 @@
         <v>46280.37528408565</v>
       </c>
       <c r="W207">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X207" t="s">
         <v>231</v>
@@ -17214,7 +17214,7 @@
         <v>46281.63558861111</v>
       </c>
       <c r="W208">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X208" t="s">
         <v>226</v>
@@ -17294,7 +17294,7 @@
         <v>46281.6358927662</v>
       </c>
       <c r="W209">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X209" t="s">
         <v>226</v>
@@ -17374,7 +17374,7 @@
         <v>46281.47564895833</v>
       </c>
       <c r="W210">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X210" t="s">
         <v>228</v>
@@ -17454,7 +17454,7 @@
         <v>46279.66710767361</v>
       </c>
       <c r="W211">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X211" t="s">
         <v>230</v>
@@ -17534,7 +17534,7 @@
         <v>46281.68877074074</v>
       </c>
       <c r="W212">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X212" t="s">
         <v>232</v>
@@ -17614,7 +17614,7 @@
         <v>46280.57958537037</v>
       </c>
       <c r="W213">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X213" t="s">
         <v>225</v>
@@ -17694,7 +17694,7 @@
         <v>46281.63570936343</v>
       </c>
       <c r="W214">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X214" t="s">
         <v>226</v>
@@ -17774,7 +17774,7 @@
         <v>46281.63595871528</v>
       </c>
       <c r="W215">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X215" t="s">
         <v>226</v>
@@ -17851,7 +17851,7 @@
         <v>46279.62681744213</v>
       </c>
       <c r="W216">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X216" t="s">
         <v>234</v>
@@ -17925,7 +17925,7 @@
         <v>46279.66707821759</v>
       </c>
       <c r="W217">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X217" t="s">
         <v>230</v>
@@ -18002,7 +18002,7 @@
         <v>46281.68880230324</v>
       </c>
       <c r="W218">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X218" t="s">
         <v>232</v>
@@ -18082,7 +18082,7 @@
         <v>46280.57972293982</v>
       </c>
       <c r="W219">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X219" t="s">
         <v>225</v>
@@ -18162,7 +18162,7 @@
         <v>46281.63575075231</v>
       </c>
       <c r="W220">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X220" t="s">
         <v>226</v>
@@ -18242,7 +18242,7 @@
         <v>46281.63599785879</v>
       </c>
       <c r="W221">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X221" t="s">
         <v>226</v>
@@ -18319,7 +18319,7 @@
         <v>46279.6268503125</v>
       </c>
       <c r="W222">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X222" t="s">
         <v>234</v>
@@ -18393,7 +18393,7 @@
         <v>46279.66698128472</v>
       </c>
       <c r="W223">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X223" t="s">
         <v>230</v>
@@ -18467,7 +18467,7 @@
         <v>46279.66929922454</v>
       </c>
       <c r="W224">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X224" t="s">
         <v>231</v>
@@ -18544,7 +18544,7 @@
         <v>46280.61353684028</v>
       </c>
       <c r="W225">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X225" t="s">
         <v>235</v>
@@ -18621,7 +18621,7 @@
         <v>46280.61353920139</v>
       </c>
       <c r="W226">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X226" t="s">
         <v>232</v>
@@ -18698,7 +18698,7 @@
         <v>46279.63250563657</v>
       </c>
       <c r="W227">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X227" t="s">
         <v>225</v>
@@ -18775,7 +18775,7 @@
         <v>46280.61354019676</v>
       </c>
       <c r="W228">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X228" t="s">
         <v>226</v>
@@ -18852,7 +18852,7 @@
         <v>46280.6135403125</v>
       </c>
       <c r="W229">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X229" t="s">
         <v>226</v>
@@ -18932,7 +18932,7 @@
         <v>46281.71218414352</v>
       </c>
       <c r="W230">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X230" t="s">
         <v>234</v>
@@ -19009,7 +19009,7 @@
         <v>46281.41576883102</v>
       </c>
       <c r="W231">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X231" t="s">
         <v>230</v>
@@ -19086,7 +19086,7 @@
         <v>46280.43132989584</v>
       </c>
       <c r="W232">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X232" t="s">
         <v>228</v>
@@ -19163,7 +19163,7 @@
         <v>46280.61367623843</v>
       </c>
       <c r="W233">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X233" t="s">
         <v>227</v>
@@ -19243,7 +19243,7 @@
         <v>46274.60593387731</v>
       </c>
       <c r="W234">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X234" t="s">
         <v>231</v>
@@ -19323,7 +19323,7 @@
         <v>46274.47210818287</v>
       </c>
       <c r="W235">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X235" t="s">
         <v>232</v>
@@ -19403,7 +19403,7 @@
         <v>46276.48975401621</v>
       </c>
       <c r="W236">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X236" t="s">
         <v>226</v>
@@ -19483,7 +19483,7 @@
         <v>46279.38429019676</v>
       </c>
       <c r="W237">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X237" t="s">
         <v>226</v>
@@ -19563,7 +19563,7 @@
         <v>46274.48792050926</v>
       </c>
       <c r="W238">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X238" t="s">
         <v>230</v>
@@ -19643,7 +19643,7 @@
         <v>46274.588374375</v>
       </c>
       <c r="W239">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X239" t="s">
         <v>228</v>
@@ -19720,7 +19720,7 @@
         <v>46274.34198912037</v>
       </c>
       <c r="W240">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X240" t="s">
         <v>227</v>
@@ -19794,7 +19794,7 @@
         <v>46279.6693627662</v>
       </c>
       <c r="W241">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X241" t="s">
         <v>231</v>
@@ -19874,7 +19874,7 @@
         <v>46279.5886965625</v>
       </c>
       <c r="W242">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X242" t="s">
         <v>232</v>
@@ -19951,7 +19951,7 @@
         <v>46279.40189383102</v>
       </c>
       <c r="W243">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X243" t="s">
         <v>225</v>
@@ -20031,7 +20031,7 @@
         <v>46279.58878520833</v>
       </c>
       <c r="W244">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X244" t="s">
         <v>226</v>
@@ -20111,7 +20111,7 @@
         <v>46279.58873577546</v>
       </c>
       <c r="W245">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X245" t="s">
         <v>226</v>
@@ -20188,7 +20188,7 @@
         <v>46279.63255</v>
       </c>
       <c r="W246">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X246" t="s">
         <v>234</v>
@@ -20265,7 +20265,7 @@
         <v>46276.63187557871</v>
       </c>
       <c r="W247">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X247" t="s">
         <v>230</v>
@@ -20342,7 +20342,7 @@
         <v>46279.6265846875</v>
       </c>
       <c r="W248">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X248" t="s">
         <v>228</v>
@@ -20419,7 +20419,7 @@
         <v>46279.63255401621</v>
       </c>
       <c r="W249">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X249" t="s">
         <v>227</v>
@@ -20499,7 +20499,7 @@
         <v>46279.66713805556</v>
       </c>
       <c r="W250">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X250" t="s">
         <v>230</v>
@@ -20573,7 +20573,7 @@
         <v>46281.63317659722</v>
       </c>
       <c r="W251">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X251" t="s">
         <v>232</v>
@@ -20647,7 +20647,7 @@
         <v>46275.39631951389</v>
       </c>
       <c r="W252">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X252" t="s">
         <v>226</v>
@@ -20721,7 +20721,7 @@
         <v>46275.39631994213</v>
       </c>
       <c r="W253">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X253" t="s">
         <v>226</v>
@@ -20801,7 +20801,7 @@
         <v>46280.62789608796</v>
       </c>
       <c r="W254">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X254" t="s">
         <v>229</v>
@@ -20881,7 +20881,7 @@
         <v>46280.63189497685</v>
       </c>
       <c r="W255">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X255" t="s">
         <v>229</v>
@@ -20961,7 +20961,7 @@
         <v>46280.72961366898</v>
       </c>
       <c r="W256">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X256" t="s">
         <v>226</v>
@@ -21038,7 +21038,7 @@
         <v>46276.37795540509</v>
       </c>
       <c r="W257">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X257" t="s">
         <v>228</v>
@@ -21115,7 +21115,7 @@
         <v>46276.66923222222</v>
       </c>
       <c r="W258">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X258" t="s">
         <v>225</v>
@@ -21192,7 +21192,7 @@
         <v>46276.40669469907</v>
       </c>
       <c r="W259">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X259" t="s">
         <v>226</v>
@@ -21269,7 +21269,7 @@
         <v>46276.64773491898</v>
       </c>
       <c r="W260">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X260" t="s">
         <v>226</v>
@@ -21349,7 +21349,7 @@
         <v>46276.39101108797</v>
       </c>
       <c r="W261">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X261" t="s">
         <v>228</v>
@@ -21426,7 +21426,7 @@
         <v>46280.40395534722</v>
       </c>
       <c r="W262">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X262" t="s">
         <v>227</v>
@@ -21503,7 +21503,7 @@
         <v>46279.74982357639</v>
       </c>
       <c r="W263">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X263" t="s">
         <v>229</v>
@@ -21583,7 +21583,7 @@
         <v>46276.66651596065</v>
       </c>
       <c r="W264">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X264" t="s">
         <v>229</v>
@@ -21660,7 +21660,7 @@
         <v>46280.66345891204</v>
       </c>
       <c r="W265">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X265" t="s">
         <v>226</v>
@@ -21737,7 +21737,7 @@
         <v>46274.36843923611</v>
       </c>
       <c r="W266">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X266" t="s">
         <v>226</v>
@@ -21814,7 +21814,7 @@
         <v>46274.66470667824</v>
       </c>
       <c r="W267">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X267" t="s">
         <v>229</v>
@@ -21891,7 +21891,7 @@
         <v>46274.74452168981</v>
       </c>
       <c r="W268">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X268" t="s">
         <v>229</v>
@@ -21971,7 +21971,7 @@
         <v>46274.64801501157</v>
       </c>
       <c r="W269">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X269" t="s">
         <v>225</v>
@@ -22048,7 +22048,7 @@
         <v>46274.36695243056</v>
       </c>
       <c r="W270">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X270" t="s">
         <v>226</v>
@@ -22125,7 +22125,7 @@
         <v>46276.4084265625</v>
       </c>
       <c r="W271">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X271" t="s">
         <v>228</v>
@@ -22202,7 +22202,7 @@
         <v>46274.7274781713</v>
       </c>
       <c r="W272">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X272" t="s">
         <v>229</v>
@@ -22276,7 +22276,7 @@
         <v>46274.74558746528</v>
       </c>
       <c r="W273">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X273" t="s">
         <v>229</v>
@@ -22347,7 +22347,7 @@
         <v>46275.79245582176</v>
       </c>
       <c r="W274">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X274" t="s">
         <v>227</v>
@@ -22424,7 +22424,7 @@
         <v>46280.63707425926</v>
       </c>
       <c r="W275">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X275" t="s">
         <v>226</v>
@@ -22504,7 +22504,7 @@
         <v>46280.38311703704</v>
       </c>
       <c r="W276">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X276" t="s">
         <v>228</v>
@@ -22581,7 +22581,7 @@
         <v>46280.37743127315</v>
       </c>
       <c r="W277">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X277" t="s">
         <v>227</v>
@@ -22661,7 +22661,7 @@
         <v>46280.45035295139</v>
       </c>
       <c r="W278">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X278" t="s">
         <v>232</v>
@@ -22738,7 +22738,7 @@
         <v>46280.59788275463</v>
       </c>
       <c r="W279">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X279" t="s">
         <v>232</v>
@@ -22818,7 +22818,7 @@
         <v>46280.73313407407</v>
       </c>
       <c r="W280">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X280" t="s">
         <v>230</v>
@@ -22895,7 +22895,7 @@
         <v>46276.49596842592</v>
       </c>
       <c r="W281">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X281" t="s">
         <v>231</v>
@@ -22969,7 +22969,7 @@
         <v>46276.53874935185</v>
       </c>
       <c r="W282">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X282" t="s">
         <v>235</v>
@@ -23043,7 +23043,7 @@
         <v>46276.49597027778</v>
       </c>
       <c r="W283">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X283" t="s">
         <v>232</v>
@@ -23117,7 +23117,7 @@
         <v>46276.62604146991</v>
       </c>
       <c r="W284">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X284" t="s">
         <v>234</v>
@@ -23191,7 +23191,7 @@
         <v>46276.68231165509</v>
       </c>
       <c r="W285">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X285" t="s">
         <v>230</v>
@@ -23268,7 +23268,7 @@
         <v>46276.7163278588</v>
       </c>
       <c r="W286">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X286" t="s">
         <v>230</v>
@@ -23345,7 +23345,7 @@
         <v>46276.6823121412</v>
       </c>
       <c r="W287">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X287" t="s">
         <v>230</v>
@@ -23422,7 +23422,7 @@
         <v>46280.69323744213</v>
       </c>
       <c r="W288">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X288" t="s">
         <v>231</v>
@@ -23499,7 +23499,7 @@
         <v>46274.70622837963</v>
       </c>
       <c r="W289">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X289" t="s">
         <v>235</v>
@@ -23573,7 +23573,7 @@
         <v>46275.71996309028</v>
       </c>
       <c r="W290">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X290" t="s">
         <v>234</v>
@@ -23647,7 +23647,7 @@
         <v>46275.54278886574</v>
       </c>
       <c r="W291">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X291" t="s">
         <v>230</v>
@@ -23724,7 +23724,7 @@
         <v>46280.74859975695</v>
       </c>
       <c r="W292">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X292" t="s">
         <v>231</v>
@@ -23801,7 +23801,7 @@
         <v>46275.7000328588</v>
       </c>
       <c r="W293">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X293" t="s">
         <v>235</v>
@@ -23875,7 +23875,7 @@
         <v>46275.72031699074</v>
       </c>
       <c r="W294">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X294" t="s">
         <v>232</v>
@@ -23949,7 +23949,7 @@
         <v>46275.54095912037</v>
       </c>
       <c r="W295">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X295" t="s">
         <v>234</v>
@@ -24023,7 +24023,7 @@
         <v>46275.72225363426</v>
       </c>
       <c r="W296">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X296" t="s">
         <v>230</v>
@@ -24097,7 +24097,7 @@
         <v>46275.7222629051</v>
       </c>
       <c r="W297">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X297" t="s">
         <v>230</v>
@@ -24171,7 +24171,7 @@
         <v>46275.7222709838</v>
       </c>
       <c r="W298">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X298" t="s">
         <v>230</v>
@@ -24248,7 +24248,7 @@
         <v>46274.74837762731</v>
       </c>
       <c r="W299">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X299" t="s">
         <v>231</v>
@@ -24328,7 +24328,7 @@
         <v>46274.74838096065</v>
       </c>
       <c r="W300">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X300" t="s">
         <v>234</v>
@@ -24408,7 +24408,7 @@
         <v>46280.56274502315</v>
       </c>
       <c r="W301">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X301" t="s">
         <v>230</v>
@@ -24485,7 +24485,7 @@
         <v>46274.42878043981</v>
       </c>
       <c r="W302">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X302" t="s">
         <v>231</v>
@@ -24562,7 +24562,7 @@
         <v>46275.40196778935</v>
       </c>
       <c r="W303">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X303" t="s">
         <v>232</v>
@@ -24639,7 +24639,7 @@
         <v>46276.52399603009</v>
       </c>
       <c r="W304">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X304" t="s">
         <v>234</v>
@@ -24716,7 +24716,7 @@
         <v>46276.5240703125</v>
       </c>
       <c r="W305">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X305" t="s">
         <v>230</v>
@@ -24790,7 +24790,7 @@
         <v>46275.4100730787</v>
       </c>
       <c r="W306">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X306" t="s">
         <v>227</v>
@@ -24864,7 +24864,7 @@
         <v>46275.40964188657</v>
       </c>
       <c r="W307">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X307" t="s">
         <v>229</v>
@@ -24938,7 +24938,7 @@
         <v>46275.40964245371</v>
       </c>
       <c r="W308">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X308" t="s">
         <v>229</v>
@@ -25012,7 +25012,7 @@
         <v>46275.45011145833</v>
       </c>
       <c r="W309">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X309" t="s">
         <v>225</v>
@@ -25086,7 +25086,7 @@
         <v>46275.44901016204</v>
       </c>
       <c r="W310">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X310" t="s">
         <v>226</v>
@@ -25160,7 +25160,7 @@
         <v>46276.71732053241</v>
       </c>
       <c r="W311">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X311" t="s">
         <v>234</v>
@@ -25237,7 +25237,7 @@
         <v>46276.71697232639</v>
       </c>
       <c r="W312">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X312" t="s">
         <v>230</v>
@@ -25314,7 +25314,7 @@
         <v>46276.7175884838</v>
       </c>
       <c r="W313">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X313" t="s">
         <v>230</v>
@@ -25391,7 +25391,7 @@
         <v>46276.7175895949</v>
       </c>
       <c r="W314">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X314" t="s">
         <v>230</v>
@@ -25468,7 +25468,7 @@
         <v>46276.71759461806</v>
       </c>
       <c r="W315">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X315" t="s">
         <v>228</v>
@@ -25542,7 +25542,7 @@
         <v>46275.44975668981</v>
       </c>
       <c r="W316">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X316" t="s">
         <v>227</v>
@@ -25616,7 +25616,7 @@
         <v>46275.44933692129</v>
       </c>
       <c r="W317">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X317" t="s">
         <v>229</v>
@@ -25690,7 +25690,7 @@
         <v>46275.44933814815</v>
       </c>
       <c r="W318">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X318" t="s">
         <v>229</v>
@@ -25764,7 +25764,7 @@
         <v>46274.41771849537</v>
       </c>
       <c r="W319">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X319" t="s">
         <v>234</v>
@@ -25835,7 +25835,7 @@
         <v>46274.41775447917</v>
       </c>
       <c r="W320">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X320" t="s">
         <v>230</v>
@@ -25906,7 +25906,7 @@
         <v>46274.41777533565</v>
       </c>
       <c r="W321">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X321" t="s">
         <v>230</v>
@@ -25977,7 +25977,7 @@
         <v>46274.41799166667</v>
       </c>
       <c r="W322">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X322" t="s">
         <v>228</v>
@@ -26048,7 +26048,7 @@
         <v>46274.41800114583</v>
       </c>
       <c r="W323">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X323" t="s">
         <v>227</v>
@@ -26119,7 +26119,7 @@
         <v>46274.41772148148</v>
       </c>
       <c r="W324">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X324" t="s">
         <v>234</v>
@@ -26190,7 +26190,7 @@
         <v>46274.41773631945</v>
       </c>
       <c r="W325">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X325" t="s">
         <v>230</v>
@@ -26261,7 +26261,7 @@
         <v>46274.41777481481</v>
       </c>
       <c r="W326">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X326" t="s">
         <v>230</v>
@@ -26332,7 +26332,7 @@
         <v>46274.41799332176</v>
       </c>
       <c r="W327">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X327" t="s">
         <v>228</v>
@@ -26403,7 +26403,7 @@
         <v>46274.41800085648</v>
       </c>
       <c r="W328">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X328" t="s">
         <v>227</v>
@@ -26474,7 +26474,7 @@
         <v>46275.31737530093</v>
       </c>
       <c r="W329">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X329" t="s">
         <v>231</v>
@@ -26545,7 +26545,7 @@
         <v>46275.31747032407</v>
       </c>
       <c r="W330">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X330" t="s">
         <v>235</v>
@@ -26616,7 +26616,7 @@
         <v>46275.31747981482</v>
       </c>
       <c r="W331">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X331" t="s">
         <v>232</v>
@@ -26687,7 +26687,7 @@
         <v>46275.31748724537</v>
       </c>
       <c r="W332">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X332" t="s">
         <v>225</v>
@@ -26758,7 +26758,7 @@
         <v>46275.31749535879</v>
       </c>
       <c r="W333">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X333" t="s">
         <v>226</v>
@@ -26829,7 +26829,7 @@
         <v>46275.31750491898</v>
       </c>
       <c r="W334">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X334" t="s">
         <v>234</v>
@@ -26900,7 +26900,7 @@
         <v>46275.31750555555</v>
       </c>
       <c r="W335">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X335" t="s">
         <v>230</v>
@@ -26971,7 +26971,7 @@
         <v>46275.31750599537</v>
       </c>
       <c r="W336">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X336" t="s">
         <v>230</v>
@@ -27042,7 +27042,7 @@
         <v>46275.5810894676</v>
       </c>
       <c r="W337">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X337" t="s">
         <v>231</v>
@@ -27116,7 +27116,7 @@
         <v>46275.58158541666</v>
       </c>
       <c r="W338">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X338" t="s">
         <v>232</v>
@@ -27190,7 +27190,7 @@
         <v>46276.41675075232</v>
       </c>
       <c r="W339">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X339" t="s">
         <v>226</v>
@@ -27270,7 +27270,7 @@
         <v>46288.76065641204</v>
       </c>
       <c r="W340">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X340" t="s">
         <v>226</v>
@@ -27350,7 +27350,7 @@
         <v>46288.7606568287</v>
       </c>
       <c r="W341">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X341" t="s">
         <v>226</v>
@@ -27430,7 +27430,7 @@
         <v>46288.76066791666</v>
       </c>
       <c r="W342">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X342" t="s">
         <v>227</v>
@@ -27507,7 +27507,7 @@
         <v>46289.64172979166</v>
       </c>
       <c r="W343">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X343" t="s">
         <v>226</v>
@@ -27584,7 +27584,7 @@
         <v>46289.56480809028</v>
       </c>
       <c r="W344">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X344" t="s">
         <v>228</v>
@@ -27661,7 +27661,7 @@
         <v>46288.43167056713</v>
       </c>
       <c r="W345">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X345" t="s">
         <v>228</v>
@@ -27738,7 +27738,7 @@
         <v>46282.62254486111</v>
       </c>
       <c r="W346">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X346" t="s">
         <v>225</v>
@@ -27815,7 +27815,7 @@
         <v>46286.64173940972</v>
       </c>
       <c r="W347">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X347" t="s">
         <v>226</v>
@@ -27892,7 +27892,7 @@
         <v>46283.44840582176</v>
       </c>
       <c r="W348">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X348" t="s">
         <v>227</v>
@@ -27969,7 +27969,7 @@
         <v>46287.48052434028</v>
       </c>
       <c r="W349">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X349" t="s">
         <v>231</v>
@@ -28049,7 +28049,7 @@
         <v>46289.41381568287</v>
       </c>
       <c r="W350">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X350" t="s">
         <v>235</v>
@@ -28126,7 +28126,7 @@
         <v>46289.44878592592</v>
       </c>
       <c r="W351">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X351" t="s">
         <v>232</v>
@@ -28200,7 +28200,7 @@
         <v>46289.44878644676</v>
       </c>
       <c r="W352">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X352" t="s">
         <v>234</v>
@@ -28274,7 +28274,7 @@
         <v>46289.64049288195</v>
       </c>
       <c r="W353">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X353" t="s">
         <v>230</v>
@@ -28348,7 +28348,7 @@
         <v>46289.64073386574</v>
       </c>
       <c r="W354">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X354" t="s">
         <v>230</v>
@@ -28425,7 +28425,7 @@
         <v>46287.48083141204</v>
       </c>
       <c r="W355">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X355" t="s">
         <v>231</v>
@@ -28505,7 +28505,7 @@
         <v>46289.40860091435</v>
       </c>
       <c r="W356">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X356" t="s">
         <v>235</v>
@@ -28582,7 +28582,7 @@
         <v>46289.44826453704</v>
       </c>
       <c r="W357">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X357" t="s">
         <v>232</v>
@@ -28656,7 +28656,7 @@
         <v>46289.4482663426</v>
       </c>
       <c r="W358">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X358" t="s">
         <v>234</v>
@@ -28730,7 +28730,7 @@
         <v>46289.57045818287</v>
       </c>
       <c r="W359">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X359" t="s">
         <v>231</v>
@@ -28807,7 +28807,7 @@
         <v>46282.42251184028</v>
       </c>
       <c r="W360">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X360" t="s">
         <v>234</v>
@@ -28881,7 +28881,7 @@
         <v>46282.47420876157</v>
       </c>
       <c r="W361">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X361" t="s">
         <v>231</v>
@@ -28958,7 +28958,7 @@
         <v>46286.7220354051</v>
       </c>
       <c r="W362">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X362" t="s">
         <v>228</v>
@@ -29038,7 +29038,7 @@
         <v>46288.73877236111</v>
       </c>
       <c r="W363">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X363" t="s">
         <v>227</v>
@@ -29115,7 +29115,7 @@
         <v>46282.47437324074</v>
       </c>
       <c r="W364">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X364" t="s">
         <v>231</v>
@@ -29192,7 +29192,7 @@
         <v>46286.7221544213</v>
       </c>
       <c r="W365">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X365" t="s">
         <v>228</v>
@@ -29272,7 +29272,7 @@
         <v>46288.73927210648</v>
       </c>
       <c r="W366">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X366" t="s">
         <v>227</v>
@@ -29349,7 +29349,7 @@
         <v>46288.65462493055</v>
       </c>
       <c r="W367">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X367" t="s">
         <v>231</v>
@@ -29426,7 +29426,7 @@
         <v>46287.66751398148</v>
       </c>
       <c r="W368">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X368" t="s">
         <v>232</v>
@@ -29506,7 +29506,7 @@
         <v>46287.46969533565</v>
       </c>
       <c r="W369">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X369" t="s">
         <v>234</v>
@@ -29586,7 +29586,7 @@
         <v>46286.71510853009</v>
       </c>
       <c r="W370">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X370" t="s">
         <v>231</v>
@@ -29666,7 +29666,7 @@
         <v>46283.59424842593</v>
       </c>
       <c r="W371">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X371" t="s">
         <v>232</v>
@@ -29746,7 +29746,7 @@
         <v>46283.68435655093</v>
       </c>
       <c r="W372">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X372" t="s">
         <v>225</v>
@@ -29826,7 +29826,7 @@
         <v>46283.5942487037</v>
       </c>
       <c r="W373">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X373" t="s">
         <v>226</v>
@@ -29906,7 +29906,7 @@
         <v>46283.59424924768</v>
       </c>
       <c r="W374">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X374" t="s">
         <v>226</v>
@@ -29986,7 +29986,7 @@
         <v>46283.68161918982</v>
       </c>
       <c r="W375">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X375" t="s">
         <v>234</v>
@@ -30066,7 +30066,7 @@
         <v>46286.6489187037</v>
       </c>
       <c r="W376">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X376" t="s">
         <v>230</v>
@@ -30146,7 +30146,7 @@
         <v>46288.38004474537</v>
       </c>
       <c r="W377">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X377" t="s">
         <v>228</v>
@@ -30226,7 +30226,7 @@
         <v>46282.42048836806</v>
       </c>
       <c r="W378">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X378" t="s">
         <v>235</v>
@@ -30303,7 +30303,7 @@
         <v>46282.42138976852</v>
       </c>
       <c r="W379">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X379" t="s">
         <v>235</v>
@@ -30377,7 +30377,7 @@
         <v>46288.65112511574</v>
       </c>
       <c r="W380">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X380" t="s">
         <v>231</v>
@@ -30454,7 +30454,7 @@
         <v>46287.66967658565</v>
       </c>
       <c r="W381">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X381" t="s">
         <v>232</v>
@@ -30534,7 +30534,7 @@
         <v>46287.47257043982</v>
       </c>
       <c r="W382">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X382" t="s">
         <v>234</v>
@@ -30608,7 +30608,7 @@
         <v>46288.72977305556</v>
       </c>
       <c r="W383">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X383" t="s">
         <v>228</v>
@@ -30682,7 +30682,7 @@
         <v>46286.6987844213</v>
       </c>
       <c r="W384">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X384" t="s">
         <v>226</v>
@@ -30756,7 +30756,7 @@
         <v>46289.40156327546</v>
       </c>
       <c r="W385">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X385" t="s">
         <v>226</v>
@@ -30830,7 +30830,7 @@
         <v>46289.40156390046</v>
       </c>
       <c r="W386">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X386" t="s">
         <v>226</v>
@@ -30907,7 +30907,7 @@
         <v>46289.4053630787</v>
       </c>
       <c r="W387">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="X387" t="s">
         <v>235</v>
@@ -30981,7 +30981,7 @@
         <v>46289.40503480324</v>
       </c>
       <c r="W388">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="X388" t="s">
         <v>235</v>
@@ -31052,7 +31052,7 @@
         <v>46287.45807677083</v>
       </c>
       <c r="W389">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X389" t="s">
         <v>231</v>
@@ -31132,7 +31132,7 @@
         <v>46286.74096042824</v>
       </c>
       <c r="W390">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X390" t="s">
         <v>227</v>
@@ -31209,7 +31209,7 @@
         <v>46283.3939177662</v>
       </c>
       <c r="W391">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X391" t="s">
         <v>225</v>
@@ -31286,7 +31286,7 @@
         <v>46286.64017539352</v>
       </c>
       <c r="W392">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X392" t="s">
         <v>226</v>
@@ -31363,7 +31363,7 @@
         <v>46286.7204416551</v>
       </c>
       <c r="W393">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X393" t="s">
         <v>227</v>
@@ -31440,7 +31440,7 @@
         <v>46283.66538607639</v>
       </c>
       <c r="W394">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X394" t="s">
         <v>225</v>
@@ -31517,7 +31517,7 @@
         <v>46286.43482986111</v>
       </c>
       <c r="W395">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X395" t="s">
         <v>226</v>
@@ -31591,7 +31591,7 @@
         <v>46286.74368133102</v>
       </c>
       <c r="W396">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X396" t="s">
         <v>227</v>
@@ -31668,7 +31668,7 @@
         <v>46283.41459880787</v>
       </c>
       <c r="W397">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X397" t="s">
         <v>226</v>
@@ -31745,7 +31745,7 @@
         <v>46283.73838344908</v>
       </c>
       <c r="W398">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X398" t="s">
         <v>228</v>
@@ -31822,7 +31822,7 @@
         <v>46286.76327152778</v>
       </c>
       <c r="W399">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X399" t="s">
         <v>229</v>
@@ -31899,7 +31899,7 @@
         <v>46286.76330447917</v>
       </c>
       <c r="W400">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X400" t="s">
         <v>229</v>
@@ -31979,7 +31979,7 @@
         <v>46287.42040790509</v>
       </c>
       <c r="W401">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X401" t="s">
         <v>225</v>
@@ -32056,7 +32056,7 @@
         <v>46283.75381304398</v>
       </c>
       <c r="W402">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X402" t="s">
         <v>226</v>
@@ -32130,7 +32130,7 @@
         <v>46289.70979120371</v>
       </c>
       <c r="W403">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X403" t="s">
         <v>227</v>
@@ -32210,7 +32210,7 @@
         <v>46287.67534456019</v>
       </c>
       <c r="W404">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X404" t="s">
         <v>225</v>
@@ -32287,7 +32287,7 @@
         <v>46289.49194748842</v>
       </c>
       <c r="W405">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X405" t="s">
         <v>226</v>
@@ -32364,7 +32364,7 @@
         <v>46283.39413969908</v>
       </c>
       <c r="W406">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X406" t="s">
         <v>225</v>
@@ -32438,7 +32438,7 @@
         <v>46286.72051887732</v>
       </c>
       <c r="W407">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X407" t="s">
         <v>227</v>
@@ -32518,7 +32518,7 @@
         <v>46283.54620269676</v>
       </c>
       <c r="W408">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X408" t="s">
         <v>231</v>
@@ -32595,7 +32595,7 @@
         <v>46288.58542337963</v>
       </c>
       <c r="W409">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X409" t="s">
         <v>232</v>
@@ -32675,7 +32675,7 @@
         <v>46289.35188425926</v>
       </c>
       <c r="W410">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X410" t="s">
         <v>230</v>
@@ -32755,7 +32755,7 @@
         <v>46287.46001957176</v>
       </c>
       <c r="W411">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X411" t="s">
         <v>231</v>
@@ -32835,7 +32835,7 @@
         <v>46287.46001266204</v>
       </c>
       <c r="W412">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X412" t="s">
         <v>235</v>
@@ -32915,7 +32915,7 @@
         <v>46286.72594498843</v>
       </c>
       <c r="W413">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X413" t="s">
         <v>232</v>
@@ -32995,7 +32995,7 @@
         <v>46282.70138376157</v>
       </c>
       <c r="W414">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X414" t="s">
         <v>230</v>
@@ -33075,7 +33075,7 @@
         <v>46282.7013840625</v>
       </c>
       <c r="W415">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X415" t="s">
         <v>230</v>
@@ -33152,7 +33152,7 @@
         <v>46283.75077045139</v>
       </c>
       <c r="W416">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X416" t="s">
         <v>234</v>
@@ -33232,7 +33232,7 @@
         <v>46286.36164050926</v>
       </c>
       <c r="W417">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X417" t="s">
         <v>230</v>
@@ -33312,7 +33312,7 @@
         <v>46286.36164494213</v>
       </c>
       <c r="W418">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X418" t="s">
         <v>231</v>
@@ -33392,7 +33392,7 @@
         <v>46286.36164826389</v>
       </c>
       <c r="W419">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X419" t="s">
         <v>235</v>
@@ -33469,7 +33469,7 @@
         <v>46283.35452896991</v>
       </c>
       <c r="W420">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X420" t="s">
         <v>230</v>
@@ -33546,7 +33546,7 @@
         <v>46283.35453171296</v>
       </c>
       <c r="W421">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X421" t="s">
         <v>230</v>
@@ -33626,7 +33626,7 @@
         <v>46287.36782538195</v>
       </c>
       <c r="W422">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X422" t="s">
         <v>234</v>
@@ -33706,7 +33706,7 @@
         <v>46287.42044105324</v>
       </c>
       <c r="W423">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X423" t="s">
         <v>235</v>
@@ -33786,7 +33786,7 @@
         <v>46288.49685543981</v>
       </c>
       <c r="W424">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X424" t="s">
         <v>234</v>
@@ -33866,7 +33866,7 @@
         <v>46287.75597989583</v>
       </c>
       <c r="W425">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X425" t="s">
         <v>231</v>
@@ -33946,7 +33946,7 @@
         <v>46288.76876331019</v>
       </c>
       <c r="W426">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X426" t="s">
         <v>230</v>
@@ -34023,7 +34023,7 @@
         <v>46283.38367943287</v>
       </c>
       <c r="W427">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X427" t="s">
         <v>231</v>
@@ -34100,7 +34100,7 @@
         <v>46282.54038741898</v>
       </c>
       <c r="W428">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X428" t="s">
         <v>235</v>
@@ -34177,7 +34177,7 @@
         <v>46283.64213659722</v>
       </c>
       <c r="W429">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X429" t="s">
         <v>226</v>
@@ -34254,7 +34254,7 @@
         <v>46283.65291121528</v>
       </c>
       <c r="W430">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X430" t="s">
         <v>230</v>
@@ -34331,7 +34331,7 @@
         <v>46283.65291194445</v>
       </c>
       <c r="W431">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X431" t="s">
         <v>230</v>
@@ -34408,7 +34408,7 @@
         <v>46286.39955256944</v>
       </c>
       <c r="W432">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X432" t="s">
         <v>228</v>
@@ -34482,7 +34482,7 @@
         <v>46286.42397924769</v>
       </c>
       <c r="W433">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X433" t="s">
         <v>231</v>
@@ -34556,7 +34556,7 @@
         <v>46286.42389136574</v>
       </c>
       <c r="W434">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X434" t="s">
         <v>235</v>
@@ -34633,7 +34633,7 @@
         <v>46283.67999300926</v>
       </c>
       <c r="W435">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X435" t="s">
         <v>226</v>
@@ -34710,7 +34710,7 @@
         <v>46286.42398471065</v>
       </c>
       <c r="W436">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X436" t="s">
         <v>234</v>
@@ -34784,7 +34784,7 @@
         <v>46286.42398568287</v>
       </c>
       <c r="W437">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X437" t="s">
         <v>230</v>
@@ -34861,7 +34861,7 @@
         <v>46283.67625043981</v>
       </c>
       <c r="W438">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X438" t="s">
         <v>228</v>
@@ -34938,7 +34938,7 @@
         <v>46283.38329579861</v>
       </c>
       <c r="W439">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X439" t="s">
         <v>230</v>
@@ -35015,7 +35015,7 @@
         <v>46282.36440621527</v>
       </c>
       <c r="W440">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X440" t="s">
         <v>231</v>
@@ -35092,7 +35092,7 @@
         <v>46282.36462596065</v>
       </c>
       <c r="W441">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X441" t="s">
         <v>235</v>
@@ -35169,7 +35169,7 @@
         <v>46282.36464421296</v>
       </c>
       <c r="W442">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X442" t="s">
         <v>232</v>
@@ -35246,7 +35246,7 @@
         <v>46282.36467337963</v>
       </c>
       <c r="W443">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X443" t="s">
         <v>225</v>
@@ -35323,7 +35323,7 @@
         <v>46282.36469679398</v>
       </c>
       <c r="W444">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X444" t="s">
         <v>226</v>
@@ -35400,7 +35400,7 @@
         <v>46282.36469869213</v>
       </c>
       <c r="W445">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X445" t="s">
         <v>226</v>
@@ -35477,7 +35477,7 @@
         <v>46282.36473159722</v>
       </c>
       <c r="W446">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X446" t="s">
         <v>234</v>
@@ -35554,7 +35554,7 @@
         <v>46282.36473394676</v>
       </c>
       <c r="W447">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X447" t="s">
         <v>230</v>
@@ -35631,7 +35631,7 @@
         <v>46282.36473579861</v>
       </c>
       <c r="W448">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X448" t="s">
         <v>230</v>
@@ -35708,7 +35708,7 @@
         <v>46282.36475297454</v>
       </c>
       <c r="W449">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X449" t="s">
         <v>230</v>
@@ -35785,7 +35785,7 @@
         <v>46282.36486408565</v>
       </c>
       <c r="W450">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X450" t="s">
         <v>228</v>
@@ -35862,7 +35862,7 @@
         <v>46282.36487561343</v>
       </c>
       <c r="W451">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X451" t="s">
         <v>227</v>
@@ -35939,7 +35939,7 @@
         <v>46282.36486778935</v>
       </c>
       <c r="W452">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X452" t="s">
         <v>229</v>
@@ -36016,7 +36016,7 @@
         <v>46282.36486851852</v>
       </c>
       <c r="W453">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X453" t="s">
         <v>229</v>
@@ -36093,7 +36093,7 @@
         <v>46286.45925082176</v>
       </c>
       <c r="W454">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X454" t="s">
         <v>231</v>
@@ -36170,7 +36170,7 @@
         <v>46282.79619427084</v>
       </c>
       <c r="W455">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X455" t="s">
         <v>235</v>
@@ -36247,7 +36247,7 @@
         <v>46282.79620872685</v>
       </c>
       <c r="W456">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X456" t="s">
         <v>232</v>
@@ -36324,7 +36324,7 @@
         <v>46282.79623825232</v>
       </c>
       <c r="W457">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X457" t="s">
         <v>225</v>
@@ -36401,7 +36401,7 @@
         <v>46282.7962541551</v>
       </c>
       <c r="W458">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X458" t="s">
         <v>226</v>
@@ -36478,7 +36478,7 @@
         <v>46282.7962703125</v>
       </c>
       <c r="W459">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X459" t="s">
         <v>226</v>
@@ -36555,7 +36555,7 @@
         <v>46282.79628381944</v>
       </c>
       <c r="W460">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X460" t="s">
         <v>234</v>
@@ -36632,7 +36632,7 @@
         <v>46282.79630119213</v>
       </c>
       <c r="W461">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X461" t="s">
         <v>230</v>
@@ -36709,7 +36709,7 @@
         <v>46282.79631224537</v>
       </c>
       <c r="W462">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X462" t="s">
         <v>230</v>
@@ -36786,7 +36786,7 @@
         <v>46282.79637734954</v>
       </c>
       <c r="W463">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X463" t="s">
         <v>228</v>
@@ -36863,7 +36863,7 @@
         <v>46282.79638922454</v>
       </c>
       <c r="W464">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X464" t="s">
         <v>227</v>
@@ -36940,7 +36940,7 @@
         <v>46282.3651903588</v>
       </c>
       <c r="W465">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X465" t="s">
         <v>231</v>
@@ -37017,7 +37017,7 @@
         <v>46282.36525856482</v>
       </c>
       <c r="W466">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X466" t="s">
         <v>235</v>
@@ -37094,7 +37094,7 @@
         <v>46282.36526855324</v>
       </c>
       <c r="W467">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X467" t="s">
         <v>232</v>
@@ -37171,7 +37171,7 @@
         <v>46282.36527959491</v>
       </c>
       <c r="W468">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X468" t="s">
         <v>225</v>
@@ -37248,7 +37248,7 @@
         <v>46282.36528526621</v>
       </c>
       <c r="W469">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X469" t="s">
         <v>226</v>
@@ -37325,7 +37325,7 @@
         <v>46282.36528619213</v>
       </c>
       <c r="W470">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X470" t="s">
         <v>226</v>
@@ -37402,7 +37402,7 @@
         <v>46282.36529351852</v>
       </c>
       <c r="W471">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X471" t="s">
         <v>234</v>
@@ -37479,7 +37479,7 @@
         <v>46282.36529424768</v>
       </c>
       <c r="W472">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X472" t="s">
         <v>230</v>
@@ -37556,7 +37556,7 @@
         <v>46282.36529490741</v>
       </c>
       <c r="W473">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X473" t="s">
         <v>230</v>
@@ -37633,7 +37633,7 @@
         <v>46282.36529869213</v>
       </c>
       <c r="W474">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X474" t="s">
         <v>230</v>
@@ -37710,7 +37710,7 @@
         <v>46282.36531149306</v>
       </c>
       <c r="W475">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X475" t="s">
         <v>228</v>
@@ -37787,7 +37787,7 @@
         <v>46282.36531554398</v>
       </c>
       <c r="W476">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X476" t="s">
         <v>227</v>
@@ -37864,7 +37864,7 @@
         <v>46282.36531253472</v>
       </c>
       <c r="W477">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X477" t="s">
         <v>229</v>
@@ -37941,7 +37941,7 @@
         <v>46282.36531288194</v>
       </c>
       <c r="W478">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X478" t="s">
         <v>229</v>
@@ -38018,7 +38018,7 @@
         <v>46286.45925106481</v>
       </c>
       <c r="W479">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X479" t="s">
         <v>231</v>
@@ -38095,7 +38095,7 @@
         <v>46282.79619331018</v>
       </c>
       <c r="W480">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X480" t="s">
         <v>235</v>
@@ -38172,7 +38172,7 @@
         <v>46282.79620888889</v>
       </c>
       <c r="W481">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X481" t="s">
         <v>232</v>
@@ -38249,7 +38249,7 @@
         <v>46282.79623803241</v>
       </c>
       <c r="W482">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X482" t="s">
         <v>225</v>
@@ -38326,7 +38326,7 @@
         <v>46282.79625384259</v>
       </c>
       <c r="W483">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X483" t="s">
         <v>226</v>
@@ -38403,7 +38403,7 @@
         <v>46282.79626969907</v>
       </c>
       <c r="W484">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X484" t="s">
         <v>226</v>
@@ -38480,7 +38480,7 @@
         <v>46282.79628394676</v>
       </c>
       <c r="W485">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X485" t="s">
         <v>234</v>
@@ -38557,7 +38557,7 @@
         <v>46282.79630097222</v>
       </c>
       <c r="W486">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X486" t="s">
         <v>230</v>
@@ -38634,7 +38634,7 @@
         <v>46282.79631204861</v>
       </c>
       <c r="W487">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X487" t="s">
         <v>230</v>
@@ -38711,7 +38711,7 @@
         <v>46282.79637748843</v>
       </c>
       <c r="W488">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X488" t="s">
         <v>228</v>
@@ -38788,7 +38788,7 @@
         <v>46282.79638901621</v>
       </c>
       <c r="W489">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X489" t="s">
         <v>227</v>
@@ -38862,7 +38862,7 @@
         <v>46283.39832862269</v>
       </c>
       <c r="W490">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X490" t="s">
         <v>231</v>
@@ -38936,7 +38936,7 @@
         <v>46282.64018086805</v>
       </c>
       <c r="W491">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X491" t="s">
         <v>235</v>
@@ -39010,7 +39010,7 @@
         <v>46287.492834375</v>
       </c>
       <c r="W492">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X492" t="s">
         <v>231</v>
@@ -39084,7 +39084,7 @@
         <v>46287.49337789352</v>
       </c>
       <c r="W493">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X493" t="s">
         <v>229</v>
@@ -39161,7 +39161,7 @@
         <v>46290.56449253472</v>
       </c>
       <c r="W494">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X494" t="s">
         <v>225</v>
@@ -39235,7 +39235,7 @@
         <v>46290.56093913194</v>
       </c>
       <c r="W495">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X495" t="s">
         <v>226</v>
@@ -39309,7 +39309,7 @@
         <v>46290.56969825231</v>
       </c>
       <c r="W496">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X496" t="s">
         <v>227</v>
@@ -39383,7 +39383,7 @@
         <v>46290.481633125</v>
       </c>
       <c r="W497">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X497" t="s">
         <v>229</v>
@@ -39457,7 +39457,7 @@
         <v>46290.48190942129</v>
       </c>
       <c r="W498">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X498" t="s">
         <v>229</v>
@@ -39531,7 +39531,7 @@
         <v>46290.564674375</v>
       </c>
       <c r="W499">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X499" t="s">
         <v>225</v>
@@ -39605,7 +39605,7 @@
         <v>46290.56113170139</v>
       </c>
       <c r="W500">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X500" t="s">
         <v>226</v>
@@ -39679,7 +39679,7 @@
         <v>46290.56957094908</v>
       </c>
       <c r="W501">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X501" t="s">
         <v>227</v>
@@ -39753,7 +39753,7 @@
         <v>46290.40572291666</v>
       </c>
       <c r="W502">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X502" t="s">
         <v>229</v>
@@ -39827,7 +39827,7 @@
         <v>46290.40597356481</v>
       </c>
       <c r="W503">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X503" t="s">
         <v>229</v>
@@ -39901,7 +39901,7 @@
         <v>46293.54930709491</v>
       </c>
       <c r="W504">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X504" t="s">
         <v>229</v>
@@ -39978,7 +39978,7 @@
         <v>46293.5514684838</v>
       </c>
       <c r="W505">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X505" t="s">
         <v>229</v>
@@ -40055,7 +40055,7 @@
         <v>46293.54923961806</v>
       </c>
       <c r="W506">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X506" t="s">
         <v>229</v>
@@ -40132,7 +40132,7 @@
         <v>46293.5514659375</v>
       </c>
       <c r="W507">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X507" t="s">
         <v>229</v>
@@ -40209,7 +40209,7 @@
         <v>46293.61969709491</v>
       </c>
       <c r="W508">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X508" t="s">
         <v>231</v>
@@ -40283,7 +40283,7 @@
         <v>46293.61789920139</v>
       </c>
       <c r="W509">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X509" t="s">
         <v>232</v>
@@ -40357,7 +40357,7 @@
         <v>46290.67269146991</v>
       </c>
       <c r="W510">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X510" t="s">
         <v>230</v>
@@ -40431,7 +40431,7 @@
         <v>46290.67373011574</v>
       </c>
       <c r="W511">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X511" t="s">
         <v>230</v>
@@ -40508,7 +40508,7 @@
         <v>46290.46651483796</v>
       </c>
       <c r="W512">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X512" t="s">
         <v>225</v>
@@ -40585,7 +40585,7 @@
         <v>46293.42116989583</v>
       </c>
       <c r="W513">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X513" t="s">
         <v>227</v>
@@ -40662,7 +40662,7 @@
         <v>46290.46660107639</v>
       </c>
       <c r="W514">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X514" t="s">
         <v>225</v>
@@ -40739,7 +40739,7 @@
         <v>46293.73434695602</v>
       </c>
       <c r="W515">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="X515" t="s">
         <v>227</v>
@@ -40813,7 +40813,7 @@
         <v>46290.67228501158</v>
       </c>
       <c r="W516">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X516" t="s">
         <v>231</v>
@@ -40890,7 +40890,7 @@
         <v>46290.67228836806</v>
       </c>
       <c r="W517">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X517" t="s">
         <v>235</v>
@@ -40967,7 +40967,7 @@
         <v>46290.67181398148</v>
       </c>
       <c r="W518">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X518" t="s">
         <v>226</v>
@@ -41044,7 +41044,7 @@
         <v>46290.67229670139</v>
       </c>
       <c r="W519">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X519" t="s">
         <v>234</v>
@@ -41121,7 +41121,7 @@
         <v>46290.6722980324</v>
       </c>
       <c r="W520">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X520" t="s">
         <v>230</v>
@@ -41195,7 +41195,7 @@
         <v>46290.67230081018</v>
       </c>
       <c r="W521">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X521" t="s">
         <v>227</v>
@@ -41272,7 +41272,7 @@
         <v>46290.67230141204</v>
       </c>
       <c r="W522">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X522" t="s">
         <v>229</v>
@@ -41349,7 +41349,7 @@
         <v>46290.67230202546</v>
       </c>
       <c r="W523">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X523" t="s">
         <v>229</v>
@@ -41423,7 +41423,7 @@
         <v>46290.42450153935</v>
       </c>
       <c r="W524">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X524" t="s">
         <v>234</v>
@@ -41500,7 +41500,7 @@
         <v>46293.62664548611</v>
       </c>
       <c r="W525">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X525" t="s">
         <v>227</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-30 15:51
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -43739,28 +43739,28 @@
         <v>166</v>
       </c>
       <c r="N555" s="1">
-        <v>46325</v>
+        <v>46295</v>
       </c>
       <c r="P555">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q555">
         <v>2026</v>
       </c>
       <c r="R555">
-        <v>18188711</v>
+        <v>18188710</v>
       </c>
       <c r="S555" t="s">
         <v>212</v>
       </c>
       <c r="U555" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="V555" s="1">
-        <v>46295.35543542824</v>
+        <v>46295.35543454861</v>
       </c>
       <c r="W555">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="X555" t="s">
         <v>233</v>
@@ -43810,28 +43810,28 @@
         <v>166</v>
       </c>
       <c r="N556" s="1">
-        <v>46295</v>
+        <v>46325</v>
       </c>
       <c r="P556">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q556">
         <v>2026</v>
       </c>
       <c r="R556">
-        <v>18188710</v>
+        <v>18188711</v>
       </c>
       <c r="S556" t="s">
         <v>212</v>
       </c>
       <c r="U556" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="V556" s="1">
-        <v>46295.35543454861</v>
+        <v>46295.35543542824</v>
       </c>
       <c r="W556">
-        <v>0</v>
+        <v>-30</v>
       </c>
       <c r="X556" t="s">
         <v>233</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-02 11:05
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1224" uniqueCount="152">
   <si>
     <t>CodCliente</t>
   </si>
@@ -151,10 +151,10 @@
     <t>TECNO COM INFORMATICA LTDA</t>
   </si>
   <si>
+    <t>NARCIZO ALVES CORDEIRO</t>
+  </si>
+  <si>
     <t>PC GAMER GOIANIA LTDA</t>
-  </si>
-  <si>
-    <t>NARCIZO ALVES CORDEIRO</t>
   </si>
   <si>
     <t>GOIAS</t>
@@ -807,7 +807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI82"/>
+  <dimension ref="A1:AI86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -4273,37 +4273,37 @@
     </row>
     <row r="47" spans="1:35">
       <c r="A47">
-        <v>6628</v>
+        <v>6404</v>
       </c>
       <c r="B47" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C47" t="s">
         <v>47</v>
       </c>
       <c r="D47" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E47" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F47" t="s">
         <v>53</v>
       </c>
       <c r="G47">
-        <v>945</v>
+        <v>6233</v>
       </c>
       <c r="H47">
-        <v>0</v>
+        <v>6232</v>
       </c>
       <c r="I47" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J47" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N47" s="1">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="P47">
         <v>9</v>
@@ -4312,34 +4312,34 @@
         <v>2026</v>
       </c>
       <c r="R47">
-        <v>16959939</v>
+        <v>16962295</v>
       </c>
       <c r="S47" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="T47" t="s">
+        <v>108</v>
       </c>
       <c r="U47" t="s">
         <v>109</v>
       </c>
       <c r="V47" s="1">
-        <v>46296.08337256945</v>
+        <v>46297.45869950231</v>
       </c>
       <c r="W47">
-        <v>-18</v>
+        <v>-3</v>
       </c>
       <c r="X47" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y47" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="AB47">
         <v>0</v>
       </c>
       <c r="AC47" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AH47" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AI47" t="s">
         <v>151</v>
@@ -4347,16 +4347,16 @@
     </row>
     <row r="48" spans="1:35">
       <c r="A48">
-        <v>6779</v>
+        <v>6703</v>
       </c>
       <c r="B48" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C48" t="s">
         <v>47</v>
       </c>
       <c r="D48" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E48" t="s">
         <v>51</v>
@@ -4365,19 +4365,19 @@
         <v>53</v>
       </c>
       <c r="G48">
-        <v>945</v>
+        <v>6233</v>
       </c>
       <c r="H48">
-        <v>0</v>
+        <v>6232</v>
       </c>
       <c r="I48" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J48" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N48" s="1">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="P48">
         <v>9</v>
@@ -4386,34 +4386,34 @@
         <v>2026</v>
       </c>
       <c r="R48">
-        <v>18056696</v>
+        <v>17948845</v>
       </c>
       <c r="S48" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="T48" t="s">
+        <v>108</v>
       </c>
       <c r="U48" t="s">
         <v>109</v>
       </c>
       <c r="V48" s="1">
-        <v>46296.0834071412</v>
+        <v>46297.45870309028</v>
       </c>
       <c r="W48">
-        <v>-18</v>
+        <v>-3</v>
       </c>
       <c r="X48" t="s">
-        <v>112</v>
-      </c>
-      <c r="Y48" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="AB48">
         <v>0</v>
       </c>
       <c r="AC48" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AH48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AI48" t="s">
         <v>151</v>
@@ -4421,37 +4421,37 @@
     </row>
     <row r="49" spans="1:35">
       <c r="A49">
-        <v>6945</v>
+        <v>6704</v>
       </c>
       <c r="B49" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C49" t="s">
         <v>47</v>
       </c>
       <c r="D49" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E49" t="s">
         <v>51</v>
       </c>
       <c r="F49" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G49">
-        <v>945</v>
+        <v>6233</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>6232</v>
       </c>
       <c r="I49" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N49" s="1">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="P49">
         <v>9</v>
@@ -4460,34 +4460,34 @@
         <v>2026</v>
       </c>
       <c r="R49">
-        <v>18164488</v>
+        <v>18085265</v>
       </c>
       <c r="S49" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="T49" t="s">
+        <v>108</v>
       </c>
       <c r="U49" t="s">
         <v>109</v>
       </c>
       <c r="V49" s="1">
-        <v>46296.08341825232</v>
+        <v>46297.45870405093</v>
       </c>
       <c r="W49">
-        <v>-18</v>
+        <v>-3</v>
       </c>
       <c r="X49" t="s">
-        <v>117</v>
-      </c>
-      <c r="Y49" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="AB49">
         <v>0</v>
       </c>
       <c r="AC49" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AH49" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AI49" t="s">
         <v>151</v>
@@ -4495,16 +4495,16 @@
     </row>
     <row r="50" spans="1:35">
       <c r="A50">
-        <v>5417</v>
+        <v>6705</v>
       </c>
       <c r="B50" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C50" t="s">
         <v>47</v>
       </c>
       <c r="D50" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E50" t="s">
         <v>51</v>
@@ -4513,19 +4513,19 @@
         <v>53</v>
       </c>
       <c r="G50">
-        <v>946</v>
+        <v>6233</v>
       </c>
       <c r="H50">
-        <v>0</v>
+        <v>6232</v>
       </c>
       <c r="I50" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J50" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="N50" s="1">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="P50">
         <v>9</v>
@@ -4534,34 +4534,34 @@
         <v>2026</v>
       </c>
       <c r="R50">
-        <v>17398870</v>
+        <v>17948990</v>
       </c>
       <c r="S50" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="T50" t="s">
+        <v>108</v>
       </c>
       <c r="U50" t="s">
         <v>109</v>
       </c>
       <c r="V50" s="1">
-        <v>46296.37558109954</v>
+        <v>46297.45870177083</v>
       </c>
       <c r="W50">
-        <v>-18</v>
+        <v>-3</v>
       </c>
       <c r="X50" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y50" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="AB50">
         <v>0</v>
       </c>
       <c r="AC50" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AH50" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AI50" t="s">
         <v>151</v>
@@ -4569,25 +4569,25 @@
     </row>
     <row r="51" spans="1:35">
       <c r="A51">
-        <v>6404</v>
+        <v>6628</v>
       </c>
       <c r="B51" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C51" t="s">
         <v>47</v>
       </c>
       <c r="D51" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E51" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F51" t="s">
         <v>53</v>
       </c>
       <c r="G51">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H51">
         <v>0</v>
@@ -4596,7 +4596,7 @@
         <v>58</v>
       </c>
       <c r="J51" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N51" s="1">
         <v>46315</v>
@@ -4608,7 +4608,7 @@
         <v>2026</v>
       </c>
       <c r="R51">
-        <v>16962094</v>
+        <v>16959939</v>
       </c>
       <c r="S51" t="s">
         <v>104</v>
@@ -4617,16 +4617,16 @@
         <v>109</v>
       </c>
       <c r="V51" s="1">
-        <v>46296.37504012731</v>
+        <v>46296.08337256945</v>
       </c>
       <c r="W51">
         <v>-18</v>
       </c>
       <c r="X51" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Y51" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="AB51">
         <v>0</v>
@@ -4643,16 +4643,16 @@
     </row>
     <row r="52" spans="1:35">
       <c r="A52">
-        <v>6703</v>
+        <v>6779</v>
       </c>
       <c r="B52" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C52" t="s">
         <v>47</v>
       </c>
       <c r="D52" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E52" t="s">
         <v>51</v>
@@ -4661,7 +4661,7 @@
         <v>53</v>
       </c>
       <c r="G52">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H52">
         <v>0</v>
@@ -4670,7 +4670,7 @@
         <v>58</v>
       </c>
       <c r="J52" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N52" s="1">
         <v>46315</v>
@@ -4682,31 +4682,31 @@
         <v>2026</v>
       </c>
       <c r="R52">
-        <v>17941133</v>
+        <v>18056696</v>
       </c>
       <c r="S52" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U52" t="s">
         <v>109</v>
       </c>
       <c r="V52" s="1">
-        <v>46296.3760846412</v>
+        <v>46296.0834071412</v>
       </c>
       <c r="W52">
         <v>-18</v>
       </c>
       <c r="X52" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="Y52" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="AB52">
         <v>0</v>
       </c>
       <c r="AC52" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AH52" t="s">
         <v>150</v>
@@ -4717,25 +4717,25 @@
     </row>
     <row r="53" spans="1:35">
       <c r="A53">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B53" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C53" t="s">
         <v>47</v>
       </c>
       <c r="D53" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E53" t="s">
         <v>51</v>
       </c>
       <c r="F53" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G53">
-        <v>949</v>
+        <v>945</v>
       </c>
       <c r="H53">
         <v>0</v>
@@ -4744,10 +4744,10 @@
         <v>58</v>
       </c>
       <c r="J53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="N53" s="1">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="P53">
         <v>9</v>
@@ -4756,7 +4756,7 @@
         <v>2026</v>
       </c>
       <c r="R53">
-        <v>17398876</v>
+        <v>18164488</v>
       </c>
       <c r="S53" t="s">
         <v>104</v>
@@ -4765,16 +4765,16 @@
         <v>109</v>
       </c>
       <c r="V53" s="1">
-        <v>46296.37648518519</v>
+        <v>46296.08341825232</v>
       </c>
       <c r="W53">
-        <v>-28</v>
+        <v>-18</v>
       </c>
       <c r="X53" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Y53" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="AB53">
         <v>0</v>
@@ -4791,10 +4791,10 @@
     </row>
     <row r="54" spans="1:35">
       <c r="A54">
-        <v>6627</v>
+        <v>5417</v>
       </c>
       <c r="B54" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C54" t="s">
         <v>47</v>
@@ -4803,13 +4803,13 @@
         <v>50</v>
       </c>
       <c r="E54" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F54" t="s">
         <v>53</v>
       </c>
       <c r="G54">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="H54">
         <v>0</v>
@@ -4818,10 +4818,10 @@
         <v>58</v>
       </c>
       <c r="J54" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N54" s="1">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="P54">
         <v>9</v>
@@ -4830,7 +4830,7 @@
         <v>2026</v>
       </c>
       <c r="R54">
-        <v>17042296</v>
+        <v>17398870</v>
       </c>
       <c r="S54" t="s">
         <v>104</v>
@@ -4839,16 +4839,16 @@
         <v>109</v>
       </c>
       <c r="V54" s="1">
-        <v>46296.37615983796</v>
+        <v>46296.37558109954</v>
       </c>
       <c r="W54">
-        <v>-28</v>
+        <v>-18</v>
       </c>
       <c r="X54" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="Y54" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="AB54">
         <v>0</v>
@@ -4865,16 +4865,16 @@
     </row>
     <row r="55" spans="1:35">
       <c r="A55">
-        <v>6704</v>
+        <v>6404</v>
       </c>
       <c r="B55" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C55" t="s">
         <v>47</v>
       </c>
       <c r="D55" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E55" t="s">
         <v>51</v>
@@ -4883,7 +4883,7 @@
         <v>53</v>
       </c>
       <c r="G55">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="H55">
         <v>0</v>
@@ -4892,10 +4892,10 @@
         <v>58</v>
       </c>
       <c r="J55" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N55" s="1">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="P55">
         <v>9</v>
@@ -4904,7 +4904,7 @@
         <v>2026</v>
       </c>
       <c r="R55">
-        <v>17952332</v>
+        <v>16962094</v>
       </c>
       <c r="S55" t="s">
         <v>104</v>
@@ -4913,16 +4913,16 @@
         <v>109</v>
       </c>
       <c r="V55" s="1">
-        <v>46296.37684290509</v>
+        <v>46296.37504012731</v>
       </c>
       <c r="W55">
-        <v>-28</v>
+        <v>-18</v>
       </c>
       <c r="X55" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Y55" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="AB55">
         <v>0</v>
@@ -4939,10 +4939,10 @@
     </row>
     <row r="56" spans="1:35">
       <c r="A56">
-        <v>6404</v>
+        <v>6703</v>
       </c>
       <c r="B56" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C56" t="s">
         <v>47</v>
@@ -4957,7 +4957,7 @@
         <v>53</v>
       </c>
       <c r="G56">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="H56">
         <v>0</v>
@@ -4966,10 +4966,10 @@
         <v>58</v>
       </c>
       <c r="J56" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="N56" s="1">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="P56">
         <v>9</v>
@@ -4978,31 +4978,31 @@
         <v>2026</v>
       </c>
       <c r="R56">
-        <v>16962100</v>
+        <v>17941133</v>
       </c>
       <c r="S56" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U56" t="s">
         <v>109</v>
       </c>
       <c r="V56" s="1">
-        <v>46296.37609667824</v>
+        <v>46296.3760846412</v>
       </c>
       <c r="W56">
-        <v>-28</v>
+        <v>-18</v>
       </c>
       <c r="X56" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="Y56" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="AB56">
         <v>0</v>
       </c>
       <c r="AC56" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH56" t="s">
         <v>150</v>
@@ -5013,16 +5013,16 @@
     </row>
     <row r="57" spans="1:35">
       <c r="A57">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B57" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C57" t="s">
         <v>47</v>
       </c>
       <c r="D57" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E57" t="s">
         <v>51</v>
@@ -5031,7 +5031,7 @@
         <v>53</v>
       </c>
       <c r="G57">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="H57">
         <v>0</v>
@@ -5040,7 +5040,7 @@
         <v>58</v>
       </c>
       <c r="J57" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N57" s="1">
         <v>46325</v>
@@ -5052,31 +5052,31 @@
         <v>2026</v>
       </c>
       <c r="R57">
-        <v>17941139</v>
+        <v>17398876</v>
       </c>
       <c r="S57" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U57" t="s">
         <v>109</v>
       </c>
       <c r="V57" s="1">
-        <v>46296.37683961805</v>
+        <v>46296.37648518519</v>
       </c>
       <c r="W57">
         <v>-28</v>
       </c>
       <c r="X57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="Y57" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="AB57">
         <v>0</v>
       </c>
       <c r="AC57" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AH57" t="s">
         <v>150</v>
@@ -5087,25 +5087,25 @@
     </row>
     <row r="58" spans="1:35">
       <c r="A58">
-        <v>6703</v>
+        <v>6627</v>
       </c>
       <c r="B58" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C58" t="s">
         <v>47</v>
       </c>
       <c r="D58" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E58" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F58" t="s">
         <v>53</v>
       </c>
       <c r="G58">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="H58">
         <v>0</v>
@@ -5114,10 +5114,10 @@
         <v>58</v>
       </c>
       <c r="J58" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N58" s="1">
-        <v>46304</v>
+        <v>46325</v>
       </c>
       <c r="P58">
         <v>9</v>
@@ -5126,31 +5126,31 @@
         <v>2026</v>
       </c>
       <c r="R58">
-        <v>17941147</v>
+        <v>17042296</v>
       </c>
       <c r="S58" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U58" t="s">
         <v>109</v>
       </c>
       <c r="V58" s="1">
-        <v>46296.37684039352</v>
+        <v>46296.37615983796</v>
       </c>
       <c r="W58">
-        <v>-7</v>
+        <v>-28</v>
       </c>
       <c r="X58" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="Y58" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="AB58">
         <v>0</v>
       </c>
       <c r="AC58" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AH58" t="s">
         <v>150</v>
@@ -5161,10 +5161,10 @@
     </row>
     <row r="59" spans="1:35">
       <c r="A59">
-        <v>6949</v>
+        <v>6704</v>
       </c>
       <c r="B59" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C59" t="s">
         <v>47</v>
@@ -5176,10 +5176,10 @@
         <v>51</v>
       </c>
       <c r="F59" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G59">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="H59">
         <v>0</v>
@@ -5188,10 +5188,10 @@
         <v>58</v>
       </c>
       <c r="J59" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N59" s="1">
-        <v>46304</v>
+        <v>46325</v>
       </c>
       <c r="P59">
         <v>9</v>
@@ -5200,7 +5200,7 @@
         <v>2026</v>
       </c>
       <c r="R59">
-        <v>18178133</v>
+        <v>17952332</v>
       </c>
       <c r="S59" t="s">
         <v>104</v>
@@ -5209,16 +5209,16 @@
         <v>109</v>
       </c>
       <c r="V59" s="1">
-        <v>46296.37697557871</v>
+        <v>46296.37684290509</v>
       </c>
       <c r="W59">
-        <v>-7</v>
+        <v>-28</v>
       </c>
       <c r="X59" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="Y59" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="AB59">
         <v>0</v>
@@ -5235,16 +5235,16 @@
     </row>
     <row r="60" spans="1:35">
       <c r="A60">
-        <v>6548</v>
+        <v>6404</v>
       </c>
       <c r="B60" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C60" t="s">
         <v>47</v>
       </c>
       <c r="D60" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E60" t="s">
         <v>51</v>
@@ -5253,7 +5253,7 @@
         <v>53</v>
       </c>
       <c r="G60">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="H60">
         <v>0</v>
@@ -5262,10 +5262,10 @@
         <v>58</v>
       </c>
       <c r="J60" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N60" s="1">
-        <v>46304</v>
+        <v>46325</v>
       </c>
       <c r="P60">
         <v>9</v>
@@ -5274,7 +5274,7 @@
         <v>2026</v>
       </c>
       <c r="R60">
-        <v>17222406</v>
+        <v>16962100</v>
       </c>
       <c r="S60" t="s">
         <v>104</v>
@@ -5283,16 +5283,16 @@
         <v>109</v>
       </c>
       <c r="V60" s="1">
-        <v>46296.37726273148</v>
+        <v>46296.37609667824</v>
       </c>
       <c r="W60">
-        <v>-7</v>
+        <v>-28</v>
       </c>
       <c r="X60" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="Y60" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="AB60">
         <v>0</v>
@@ -5327,7 +5327,7 @@
         <v>53</v>
       </c>
       <c r="G61">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="H61">
         <v>0</v>
@@ -5336,10 +5336,10 @@
         <v>58</v>
       </c>
       <c r="J61" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N61" s="1">
-        <v>46304</v>
+        <v>46325</v>
       </c>
       <c r="P61">
         <v>9</v>
@@ -5348,7 +5348,7 @@
         <v>2026</v>
       </c>
       <c r="R61">
-        <v>17941157</v>
+        <v>17941139</v>
       </c>
       <c r="S61" t="s">
         <v>105</v>
@@ -5357,16 +5357,16 @@
         <v>109</v>
       </c>
       <c r="V61" s="1">
-        <v>46296.37814100694</v>
+        <v>46296.37683961805</v>
       </c>
       <c r="W61">
-        <v>-7</v>
+        <v>-28</v>
       </c>
       <c r="X61" t="s">
         <v>119</v>
       </c>
       <c r="Y61" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="AB61">
         <v>0</v>
@@ -5383,16 +5383,16 @@
     </row>
     <row r="62" spans="1:35">
       <c r="A62">
-        <v>6779</v>
+        <v>6703</v>
       </c>
       <c r="B62" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C62" t="s">
         <v>47</v>
       </c>
       <c r="D62" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E62" t="s">
         <v>51</v>
@@ -5401,7 +5401,7 @@
         <v>53</v>
       </c>
       <c r="G62">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H62">
         <v>0</v>
@@ -5410,7 +5410,7 @@
         <v>58</v>
       </c>
       <c r="J62" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N62" s="1">
         <v>46304</v>
@@ -5422,31 +5422,31 @@
         <v>2026</v>
       </c>
       <c r="R62">
-        <v>18056706</v>
+        <v>17941147</v>
       </c>
       <c r="S62" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U62" t="s">
         <v>109</v>
       </c>
       <c r="V62" s="1">
-        <v>46296.37816597222</v>
+        <v>46296.37684039352</v>
       </c>
       <c r="W62">
         <v>-7</v>
       </c>
       <c r="X62" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="Y62" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="AB62">
         <v>0</v>
       </c>
       <c r="AC62" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH62" t="s">
         <v>150</v>
@@ -5457,16 +5457,16 @@
     </row>
     <row r="63" spans="1:35">
       <c r="A63">
-        <v>6945</v>
+        <v>6949</v>
       </c>
       <c r="B63" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C63" t="s">
         <v>47</v>
       </c>
       <c r="D63" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E63" t="s">
         <v>51</v>
@@ -5475,7 +5475,7 @@
         <v>54</v>
       </c>
       <c r="G63">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H63">
         <v>0</v>
@@ -5484,7 +5484,7 @@
         <v>58</v>
       </c>
       <c r="J63" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N63" s="1">
         <v>46304</v>
@@ -5496,7 +5496,7 @@
         <v>2026</v>
       </c>
       <c r="R63">
-        <v>18164502</v>
+        <v>18178133</v>
       </c>
       <c r="S63" t="s">
         <v>104</v>
@@ -5505,16 +5505,16 @@
         <v>109</v>
       </c>
       <c r="V63" s="1">
-        <v>46296.3782184838</v>
+        <v>46296.37697557871</v>
       </c>
       <c r="W63">
         <v>-7</v>
       </c>
       <c r="X63" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="Y63" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="AB63">
         <v>0</v>
@@ -5531,10 +5531,10 @@
     </row>
     <row r="64" spans="1:35">
       <c r="A64">
-        <v>6949</v>
+        <v>6548</v>
       </c>
       <c r="B64" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C64" t="s">
         <v>47</v>
@@ -5546,7 +5546,7 @@
         <v>51</v>
       </c>
       <c r="F64" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G64">
         <v>951</v>
@@ -5570,7 +5570,7 @@
         <v>2026</v>
       </c>
       <c r="R64">
-        <v>18178139</v>
+        <v>17222406</v>
       </c>
       <c r="S64" t="s">
         <v>104</v>
@@ -5579,16 +5579,16 @@
         <v>109</v>
       </c>
       <c r="V64" s="1">
-        <v>46296.37822091435</v>
+        <v>46296.37726273148</v>
       </c>
       <c r="W64">
         <v>-7</v>
       </c>
       <c r="X64" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="Y64" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AB64">
         <v>0</v>
@@ -5605,16 +5605,16 @@
     </row>
     <row r="65" spans="1:35">
       <c r="A65">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B65" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C65" t="s">
         <v>47</v>
       </c>
       <c r="D65" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E65" t="s">
         <v>51</v>
@@ -5623,7 +5623,7 @@
         <v>53</v>
       </c>
       <c r="G65">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="H65">
         <v>0</v>
@@ -5632,10 +5632,10 @@
         <v>58</v>
       </c>
       <c r="J65" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N65" s="1">
-        <v>46318</v>
+        <v>46304</v>
       </c>
       <c r="P65">
         <v>9</v>
@@ -5644,31 +5644,31 @@
         <v>2026</v>
       </c>
       <c r="R65">
-        <v>17398884</v>
+        <v>17941157</v>
       </c>
       <c r="S65" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U65" t="s">
         <v>109</v>
       </c>
       <c r="V65" s="1">
-        <v>46296.37748545139</v>
+        <v>46296.37814100694</v>
       </c>
       <c r="W65">
-        <v>-21</v>
+        <v>-7</v>
       </c>
       <c r="X65" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="Y65" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AB65">
         <v>0</v>
       </c>
       <c r="AC65" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH65" t="s">
         <v>150</v>
@@ -5679,16 +5679,16 @@
     </row>
     <row r="66" spans="1:35">
       <c r="A66">
-        <v>6404</v>
+        <v>6779</v>
       </c>
       <c r="B66" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C66" t="s">
         <v>47</v>
       </c>
       <c r="D66" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E66" t="s">
         <v>51</v>
@@ -5697,7 +5697,7 @@
         <v>53</v>
       </c>
       <c r="G66">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="H66">
         <v>0</v>
@@ -5706,10 +5706,10 @@
         <v>58</v>
       </c>
       <c r="J66" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N66" s="1">
-        <v>46318</v>
+        <v>46304</v>
       </c>
       <c r="P66">
         <v>9</v>
@@ -5718,7 +5718,7 @@
         <v>2026</v>
       </c>
       <c r="R66">
-        <v>16962108</v>
+        <v>18056706</v>
       </c>
       <c r="S66" t="s">
         <v>104</v>
@@ -5727,16 +5727,16 @@
         <v>109</v>
       </c>
       <c r="V66" s="1">
-        <v>46296.37705413195</v>
+        <v>46296.37816597222</v>
       </c>
       <c r="W66">
-        <v>-21</v>
+        <v>-7</v>
       </c>
       <c r="X66" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="Y66" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="AB66">
         <v>0</v>
@@ -5753,25 +5753,25 @@
     </row>
     <row r="67" spans="1:35">
       <c r="A67">
-        <v>6627</v>
+        <v>6945</v>
       </c>
       <c r="B67" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C67" t="s">
         <v>47</v>
       </c>
       <c r="D67" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E67" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F67" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G67">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="H67">
         <v>0</v>
@@ -5780,10 +5780,10 @@
         <v>58</v>
       </c>
       <c r="J67" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N67" s="1">
-        <v>46318</v>
+        <v>46304</v>
       </c>
       <c r="P67">
         <v>9</v>
@@ -5792,7 +5792,7 @@
         <v>2026</v>
       </c>
       <c r="R67">
-        <v>17042320</v>
+        <v>18164502</v>
       </c>
       <c r="S67" t="s">
         <v>104</v>
@@ -5801,16 +5801,16 @@
         <v>109</v>
       </c>
       <c r="V67" s="1">
-        <v>46296.37710454861</v>
+        <v>46296.3782184838</v>
       </c>
       <c r="W67">
-        <v>-21</v>
+        <v>-7</v>
       </c>
       <c r="X67" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="Y67" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="AB67">
         <v>0</v>
@@ -5827,25 +5827,25 @@
     </row>
     <row r="68" spans="1:35">
       <c r="A68">
-        <v>6703</v>
+        <v>6949</v>
       </c>
       <c r="B68" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C68" t="s">
         <v>47</v>
       </c>
       <c r="D68" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E68" t="s">
         <v>51</v>
       </c>
       <c r="F68" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G68">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="H68">
         <v>0</v>
@@ -5854,10 +5854,10 @@
         <v>58</v>
       </c>
       <c r="J68" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N68" s="1">
-        <v>46318</v>
+        <v>46304</v>
       </c>
       <c r="P68">
         <v>9</v>
@@ -5866,31 +5866,31 @@
         <v>2026</v>
       </c>
       <c r="R68">
-        <v>17941167</v>
+        <v>18178139</v>
       </c>
       <c r="S68" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U68" t="s">
         <v>109</v>
       </c>
       <c r="V68" s="1">
-        <v>46296.37814163195</v>
+        <v>46296.37822091435</v>
       </c>
       <c r="W68">
-        <v>-21</v>
+        <v>-7</v>
       </c>
       <c r="X68" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="Y68" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="AB68">
         <v>0</v>
       </c>
       <c r="AC68" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AH68" t="s">
         <v>150</v>
@@ -5901,10 +5901,10 @@
     </row>
     <row r="69" spans="1:35">
       <c r="A69">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B69" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C69" t="s">
         <v>47</v>
@@ -5916,7 +5916,7 @@
         <v>51</v>
       </c>
       <c r="F69" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G69">
         <v>953</v>
@@ -5940,7 +5940,7 @@
         <v>2026</v>
       </c>
       <c r="R69">
-        <v>18178145</v>
+        <v>17398884</v>
       </c>
       <c r="S69" t="s">
         <v>104</v>
@@ -5949,16 +5949,16 @@
         <v>109</v>
       </c>
       <c r="V69" s="1">
-        <v>46296.37822175926</v>
+        <v>46296.37748545139</v>
       </c>
       <c r="W69">
         <v>-21</v>
       </c>
       <c r="X69" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="Y69" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="AB69">
         <v>0</v>
@@ -5975,16 +5975,16 @@
     </row>
     <row r="70" spans="1:35">
       <c r="A70">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B70" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C70" t="s">
         <v>47</v>
       </c>
       <c r="D70" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E70" t="s">
         <v>51</v>
@@ -5993,7 +5993,7 @@
         <v>53</v>
       </c>
       <c r="G70">
-        <v>941</v>
+        <v>953</v>
       </c>
       <c r="H70">
         <v>0</v>
@@ -6002,10 +6002,10 @@
         <v>58</v>
       </c>
       <c r="J70" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N70" s="1">
-        <v>46297</v>
+        <v>46318</v>
       </c>
       <c r="P70">
         <v>9</v>
@@ -6014,22 +6014,25 @@
         <v>2026</v>
       </c>
       <c r="R70">
-        <v>17398850</v>
+        <v>16962108</v>
       </c>
       <c r="S70" t="s">
         <v>104</v>
       </c>
       <c r="U70" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="V70" s="1">
-        <v>46297.34991217592</v>
+        <v>46296.37705413195</v>
       </c>
       <c r="W70">
-        <v>0</v>
+        <v>-21</v>
       </c>
       <c r="X70" t="s">
-        <v>118</v>
+        <v>113</v>
+      </c>
+      <c r="Y70" t="s">
+        <v>139</v>
       </c>
       <c r="AB70">
         <v>0</v>
@@ -6038,7 +6041,7 @@
         <v>104</v>
       </c>
       <c r="AH70" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AI70" t="s">
         <v>151</v>
@@ -6046,25 +6049,25 @@
     </row>
     <row r="71" spans="1:35">
       <c r="A71">
-        <v>6404</v>
+        <v>6627</v>
       </c>
       <c r="B71" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C71" t="s">
         <v>47</v>
       </c>
       <c r="D71" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E71" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F71" t="s">
         <v>53</v>
       </c>
       <c r="G71">
-        <v>941</v>
+        <v>953</v>
       </c>
       <c r="H71">
         <v>0</v>
@@ -6073,10 +6076,10 @@
         <v>58</v>
       </c>
       <c r="J71" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N71" s="1">
-        <v>46297</v>
+        <v>46318</v>
       </c>
       <c r="P71">
         <v>9</v>
@@ -6085,22 +6088,25 @@
         <v>2026</v>
       </c>
       <c r="R71">
-        <v>16962084</v>
+        <v>17042320</v>
       </c>
       <c r="S71" t="s">
         <v>104</v>
       </c>
       <c r="U71" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="V71" s="1">
-        <v>46297.3499325</v>
+        <v>46296.37710454861</v>
       </c>
       <c r="W71">
-        <v>0</v>
+        <v>-21</v>
       </c>
       <c r="X71" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="Y71" t="s">
+        <v>140</v>
       </c>
       <c r="AB71">
         <v>0</v>
@@ -6109,7 +6115,7 @@
         <v>104</v>
       </c>
       <c r="AH71" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AI71" t="s">
         <v>151</v>
@@ -6117,16 +6123,16 @@
     </row>
     <row r="72" spans="1:35">
       <c r="A72">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B72" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C72" t="s">
         <v>47</v>
       </c>
       <c r="D72" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E72" t="s">
         <v>51</v>
@@ -6135,7 +6141,7 @@
         <v>53</v>
       </c>
       <c r="G72">
-        <v>941</v>
+        <v>953</v>
       </c>
       <c r="H72">
         <v>0</v>
@@ -6144,10 +6150,10 @@
         <v>58</v>
       </c>
       <c r="J72" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N72" s="1">
-        <v>46297</v>
+        <v>46318</v>
       </c>
       <c r="P72">
         <v>9</v>
@@ -6156,31 +6162,34 @@
         <v>2026</v>
       </c>
       <c r="R72">
-        <v>16975881</v>
+        <v>17941167</v>
       </c>
       <c r="S72" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U72" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="V72" s="1">
-        <v>46297.34994254629</v>
+        <v>46296.37814163195</v>
       </c>
       <c r="W72">
-        <v>0</v>
+        <v>-21</v>
       </c>
       <c r="X72" t="s">
-        <v>120</v>
+        <v>119</v>
+      </c>
+      <c r="Y72" t="s">
+        <v>141</v>
       </c>
       <c r="AB72">
         <v>0</v>
       </c>
       <c r="AC72" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH72" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AI72" t="s">
         <v>151</v>
@@ -6188,10 +6197,10 @@
     </row>
     <row r="73" spans="1:35">
       <c r="A73">
-        <v>6627</v>
+        <v>6949</v>
       </c>
       <c r="B73" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C73" t="s">
         <v>47</v>
@@ -6200,13 +6209,13 @@
         <v>50</v>
       </c>
       <c r="E73" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F73" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G73">
-        <v>941</v>
+        <v>953</v>
       </c>
       <c r="H73">
         <v>0</v>
@@ -6215,10 +6224,10 @@
         <v>58</v>
       </c>
       <c r="J73" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N73" s="1">
-        <v>46297</v>
+        <v>46318</v>
       </c>
       <c r="P73">
         <v>9</v>
@@ -6227,22 +6236,25 @@
         <v>2026</v>
       </c>
       <c r="R73">
-        <v>17042242</v>
+        <v>18178145</v>
       </c>
       <c r="S73" t="s">
         <v>104</v>
       </c>
       <c r="U73" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="V73" s="1">
-        <v>46297.34994771991</v>
+        <v>46296.37822175926</v>
       </c>
       <c r="W73">
-        <v>0</v>
+        <v>-21</v>
       </c>
       <c r="X73" t="s">
-        <v>114</v>
+        <v>116</v>
+      </c>
+      <c r="Y73" t="s">
+        <v>142</v>
       </c>
       <c r="AB73">
         <v>0</v>
@@ -6251,7 +6263,7 @@
         <v>104</v>
       </c>
       <c r="AH73" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AI73" t="s">
         <v>151</v>
@@ -6259,10 +6271,10 @@
     </row>
     <row r="74" spans="1:35">
       <c r="A74">
-        <v>6704</v>
+        <v>5417</v>
       </c>
       <c r="B74" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C74" t="s">
         <v>47</v>
@@ -6298,7 +6310,7 @@
         <v>2026</v>
       </c>
       <c r="R74">
-        <v>17952303</v>
+        <v>17398850</v>
       </c>
       <c r="S74" t="s">
         <v>104</v>
@@ -6307,13 +6319,13 @@
         <v>111</v>
       </c>
       <c r="V74" s="1">
-        <v>46297.34994974537</v>
+        <v>46297.34991217592</v>
       </c>
       <c r="W74">
         <v>0</v>
       </c>
       <c r="X74" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="AB74">
         <v>0</v>
@@ -6330,16 +6342,16 @@
     </row>
     <row r="75" spans="1:35">
       <c r="A75">
-        <v>6705</v>
+        <v>6404</v>
       </c>
       <c r="B75" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C75" t="s">
         <v>47</v>
       </c>
       <c r="D75" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E75" t="s">
         <v>51</v>
@@ -6369,7 +6381,7 @@
         <v>2026</v>
       </c>
       <c r="R75">
-        <v>17952502</v>
+        <v>16962084</v>
       </c>
       <c r="S75" t="s">
         <v>104</v>
@@ -6378,13 +6390,13 @@
         <v>111</v>
       </c>
       <c r="V75" s="1">
-        <v>46297.34995063658</v>
+        <v>46297.3499325</v>
       </c>
       <c r="W75">
         <v>0</v>
       </c>
       <c r="X75" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AB75">
         <v>0</v>
@@ -6401,22 +6413,22 @@
     </row>
     <row r="76" spans="1:35">
       <c r="A76">
-        <v>6945</v>
+        <v>6486</v>
       </c>
       <c r="B76" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C76" t="s">
         <v>47</v>
       </c>
       <c r="D76" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E76" t="s">
         <v>51</v>
       </c>
       <c r="F76" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G76">
         <v>941</v>
@@ -6440,7 +6452,7 @@
         <v>2026</v>
       </c>
       <c r="R76">
-        <v>18164480</v>
+        <v>16975881</v>
       </c>
       <c r="S76" t="s">
         <v>104</v>
@@ -6449,13 +6461,13 @@
         <v>111</v>
       </c>
       <c r="V76" s="1">
-        <v>46297.34996266204</v>
+        <v>46297.34994254629</v>
       </c>
       <c r="W76">
         <v>0</v>
       </c>
       <c r="X76" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AB76">
         <v>0</v>
@@ -6472,70 +6484,67 @@
     </row>
     <row r="77" spans="1:35">
       <c r="A77">
-        <v>6404</v>
+        <v>6627</v>
       </c>
       <c r="B77" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C77" t="s">
         <v>47</v>
       </c>
       <c r="D77" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E77" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F77" t="s">
         <v>53</v>
       </c>
       <c r="G77">
-        <v>11001</v>
+        <v>941</v>
       </c>
       <c r="H77">
         <v>0</v>
       </c>
       <c r="I77" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J77" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N77" s="1">
-        <v>46351</v>
+        <v>46297</v>
       </c>
       <c r="P77">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q77">
         <v>2026</v>
       </c>
       <c r="R77">
-        <v>16962456</v>
+        <v>17042242</v>
       </c>
       <c r="S77" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="U77" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="V77" s="1">
-        <v>46296.34114513889</v>
+        <v>46297.34994771991</v>
       </c>
       <c r="W77">
-        <v>-54</v>
+        <v>0</v>
       </c>
       <c r="X77" t="s">
-        <v>113</v>
-      </c>
-      <c r="Y77" t="s">
-        <v>143</v>
+        <v>114</v>
       </c>
       <c r="AB77">
         <v>0</v>
       </c>
       <c r="AC77" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="AH77" t="s">
         <v>149</v>
@@ -6546,10 +6555,10 @@
     </row>
     <row r="78" spans="1:35">
       <c r="A78">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B78" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C78" t="s">
         <v>47</v>
@@ -6564,52 +6573,49 @@
         <v>53</v>
       </c>
       <c r="G78">
-        <v>7877</v>
+        <v>941</v>
       </c>
       <c r="H78">
         <v>0</v>
       </c>
       <c r="I78" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J78" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="N78" s="1">
-        <v>46351</v>
+        <v>46297</v>
       </c>
       <c r="P78">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q78">
         <v>2026</v>
       </c>
       <c r="R78">
-        <v>17399332</v>
+        <v>17952303</v>
       </c>
       <c r="S78" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="U78" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="V78" s="1">
-        <v>46296.34050315972</v>
+        <v>46297.34994974537</v>
       </c>
       <c r="W78">
-        <v>-54</v>
+        <v>0</v>
       </c>
       <c r="X78" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y78" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="AB78">
         <v>0</v>
       </c>
       <c r="AC78" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="AH78" t="s">
         <v>149</v>
@@ -6620,7 +6626,7 @@
     </row>
     <row r="79" spans="1:35">
       <c r="A79">
-        <v>6486</v>
+        <v>6705</v>
       </c>
       <c r="B79" t="s">
         <v>45</v>
@@ -6629,7 +6635,7 @@
         <v>47</v>
       </c>
       <c r="D79" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E79" t="s">
         <v>51</v>
@@ -6638,52 +6644,49 @@
         <v>53</v>
       </c>
       <c r="G79">
-        <v>9774</v>
+        <v>941</v>
       </c>
       <c r="H79">
         <v>0</v>
       </c>
       <c r="I79" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J79" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="N79" s="1">
-        <v>46290</v>
+        <v>46297</v>
       </c>
       <c r="P79">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q79">
         <v>2026</v>
       </c>
       <c r="R79">
-        <v>16976321</v>
+        <v>17952502</v>
       </c>
       <c r="S79" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="U79" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="V79" s="1">
-        <v>46296.39309459491</v>
+        <v>46297.34995063658</v>
       </c>
       <c r="W79">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="X79" t="s">
-        <v>120</v>
-      </c>
-      <c r="Y79" t="s">
-        <v>145</v>
+        <v>112</v>
       </c>
       <c r="AB79">
         <v>0</v>
       </c>
       <c r="AC79" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="AH79" t="s">
         <v>149</v>
@@ -6694,70 +6697,67 @@
     </row>
     <row r="80" spans="1:35">
       <c r="A80">
-        <v>6486</v>
+        <v>6945</v>
       </c>
       <c r="B80" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C80" t="s">
         <v>47</v>
       </c>
       <c r="D80" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E80" t="s">
         <v>51</v>
       </c>
       <c r="F80" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G80">
-        <v>9774</v>
+        <v>941</v>
       </c>
       <c r="H80">
         <v>0</v>
       </c>
       <c r="I80" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J80" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="N80" s="1">
-        <v>46351</v>
+        <v>46297</v>
       </c>
       <c r="P80">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q80">
         <v>2026</v>
       </c>
       <c r="R80">
-        <v>16976323</v>
+        <v>18164480</v>
       </c>
       <c r="S80" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="U80" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="V80" s="1">
-        <v>46296.3409153125</v>
+        <v>46297.34996266204</v>
       </c>
       <c r="W80">
-        <v>-54</v>
+        <v>0</v>
       </c>
       <c r="X80" t="s">
-        <v>120</v>
-      </c>
-      <c r="Y80" t="s">
-        <v>146</v>
+        <v>117</v>
       </c>
       <c r="AB80">
         <v>0</v>
       </c>
       <c r="AC80" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="AH80" t="s">
         <v>149</v>
@@ -6768,16 +6768,16 @@
     </row>
     <row r="81" spans="1:35">
       <c r="A81">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B81" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C81" t="s">
         <v>47</v>
       </c>
       <c r="D81" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E81" t="s">
         <v>51</v>
@@ -6786,7 +6786,7 @@
         <v>53</v>
       </c>
       <c r="G81">
-        <v>7027</v>
+        <v>11001</v>
       </c>
       <c r="H81">
         <v>0</v>
@@ -6795,10 +6795,10 @@
         <v>59</v>
       </c>
       <c r="J81" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="N81" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="P81">
         <v>10</v>
@@ -6807,7 +6807,7 @@
         <v>2026</v>
       </c>
       <c r="R81">
-        <v>17399292</v>
+        <v>16962456</v>
       </c>
       <c r="S81" t="s">
         <v>51</v>
@@ -6816,13 +6816,16 @@
         <v>109</v>
       </c>
       <c r="V81" s="1">
-        <v>46296.0420403125</v>
+        <v>46296.34114513889</v>
       </c>
       <c r="W81">
-        <v>-53</v>
+        <v>-54</v>
       </c>
       <c r="X81" t="s">
-        <v>118</v>
+        <v>113</v>
+      </c>
+      <c r="Y81" t="s">
+        <v>143</v>
       </c>
       <c r="AB81">
         <v>0</v>
@@ -6839,16 +6842,16 @@
     </row>
     <row r="82" spans="1:35">
       <c r="A82">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B82" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C82" t="s">
         <v>47</v>
       </c>
       <c r="D82" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E82" t="s">
         <v>51</v>
@@ -6857,7 +6860,7 @@
         <v>53</v>
       </c>
       <c r="G82">
-        <v>7027</v>
+        <v>7877</v>
       </c>
       <c r="H82">
         <v>0</v>
@@ -6866,10 +6869,10 @@
         <v>59</v>
       </c>
       <c r="J82" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="N82" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="P82">
         <v>10</v>
@@ -6878,7 +6881,7 @@
         <v>2026</v>
       </c>
       <c r="R82">
-        <v>16962350</v>
+        <v>17399332</v>
       </c>
       <c r="S82" t="s">
         <v>51</v>
@@ -6887,13 +6890,16 @@
         <v>109</v>
       </c>
       <c r="V82" s="1">
-        <v>46296.0420403125</v>
+        <v>46296.34050315972</v>
       </c>
       <c r="W82">
-        <v>-53</v>
+        <v>-54</v>
       </c>
       <c r="X82" t="s">
-        <v>113</v>
+        <v>118</v>
+      </c>
+      <c r="Y82" t="s">
+        <v>144</v>
       </c>
       <c r="AB82">
         <v>0</v>
@@ -6905,6 +6911,296 @@
         <v>149</v>
       </c>
       <c r="AI82" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="83" spans="1:35">
+      <c r="A83">
+        <v>6486</v>
+      </c>
+      <c r="B83" t="s">
+        <v>46</v>
+      </c>
+      <c r="C83" t="s">
+        <v>47</v>
+      </c>
+      <c r="D83" t="s">
+        <v>50</v>
+      </c>
+      <c r="E83" t="s">
+        <v>51</v>
+      </c>
+      <c r="F83" t="s">
+        <v>53</v>
+      </c>
+      <c r="G83">
+        <v>9774</v>
+      </c>
+      <c r="H83">
+        <v>0</v>
+      </c>
+      <c r="I83" t="s">
+        <v>59</v>
+      </c>
+      <c r="J83" t="s">
+        <v>94</v>
+      </c>
+      <c r="N83" s="1">
+        <v>46290</v>
+      </c>
+      <c r="P83">
+        <v>8</v>
+      </c>
+      <c r="Q83">
+        <v>2026</v>
+      </c>
+      <c r="R83">
+        <v>16976321</v>
+      </c>
+      <c r="S83" t="s">
+        <v>51</v>
+      </c>
+      <c r="U83" t="s">
+        <v>110</v>
+      </c>
+      <c r="V83" s="1">
+        <v>46296.39309459491</v>
+      </c>
+      <c r="W83">
+        <v>7</v>
+      </c>
+      <c r="X83" t="s">
+        <v>120</v>
+      </c>
+      <c r="Y83" t="s">
+        <v>145</v>
+      </c>
+      <c r="AB83">
+        <v>0</v>
+      </c>
+      <c r="AC83" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH83" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI83" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="84" spans="1:35">
+      <c r="A84">
+        <v>6486</v>
+      </c>
+      <c r="B84" t="s">
+        <v>46</v>
+      </c>
+      <c r="C84" t="s">
+        <v>47</v>
+      </c>
+      <c r="D84" t="s">
+        <v>50</v>
+      </c>
+      <c r="E84" t="s">
+        <v>51</v>
+      </c>
+      <c r="F84" t="s">
+        <v>53</v>
+      </c>
+      <c r="G84">
+        <v>9774</v>
+      </c>
+      <c r="H84">
+        <v>0</v>
+      </c>
+      <c r="I84" t="s">
+        <v>59</v>
+      </c>
+      <c r="J84" t="s">
+        <v>94</v>
+      </c>
+      <c r="N84" s="1">
+        <v>46351</v>
+      </c>
+      <c r="P84">
+        <v>10</v>
+      </c>
+      <c r="Q84">
+        <v>2026</v>
+      </c>
+      <c r="R84">
+        <v>16976323</v>
+      </c>
+      <c r="S84" t="s">
+        <v>51</v>
+      </c>
+      <c r="U84" t="s">
+        <v>109</v>
+      </c>
+      <c r="V84" s="1">
+        <v>46296.3409153125</v>
+      </c>
+      <c r="W84">
+        <v>-54</v>
+      </c>
+      <c r="X84" t="s">
+        <v>120</v>
+      </c>
+      <c r="Y84" t="s">
+        <v>146</v>
+      </c>
+      <c r="AB84">
+        <v>0</v>
+      </c>
+      <c r="AC84" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH84" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI84" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="85" spans="1:35">
+      <c r="A85">
+        <v>5417</v>
+      </c>
+      <c r="B85" t="s">
+        <v>42</v>
+      </c>
+      <c r="C85" t="s">
+        <v>47</v>
+      </c>
+      <c r="D85" t="s">
+        <v>50</v>
+      </c>
+      <c r="E85" t="s">
+        <v>51</v>
+      </c>
+      <c r="F85" t="s">
+        <v>53</v>
+      </c>
+      <c r="G85">
+        <v>7027</v>
+      </c>
+      <c r="H85">
+        <v>0</v>
+      </c>
+      <c r="I85" t="s">
+        <v>59</v>
+      </c>
+      <c r="J85" t="s">
+        <v>95</v>
+      </c>
+      <c r="N85" s="1">
+        <v>46350</v>
+      </c>
+      <c r="P85">
+        <v>10</v>
+      </c>
+      <c r="Q85">
+        <v>2026</v>
+      </c>
+      <c r="R85">
+        <v>17399292</v>
+      </c>
+      <c r="S85" t="s">
+        <v>51</v>
+      </c>
+      <c r="U85" t="s">
+        <v>109</v>
+      </c>
+      <c r="V85" s="1">
+        <v>46296.0420403125</v>
+      </c>
+      <c r="W85">
+        <v>-53</v>
+      </c>
+      <c r="X85" t="s">
+        <v>118</v>
+      </c>
+      <c r="AB85">
+        <v>0</v>
+      </c>
+      <c r="AC85" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH85" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI85" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="86" spans="1:35">
+      <c r="A86">
+        <v>6404</v>
+      </c>
+      <c r="B86" t="s">
+        <v>36</v>
+      </c>
+      <c r="C86" t="s">
+        <v>47</v>
+      </c>
+      <c r="D86" t="s">
+        <v>49</v>
+      </c>
+      <c r="E86" t="s">
+        <v>51</v>
+      </c>
+      <c r="F86" t="s">
+        <v>53</v>
+      </c>
+      <c r="G86">
+        <v>7027</v>
+      </c>
+      <c r="H86">
+        <v>0</v>
+      </c>
+      <c r="I86" t="s">
+        <v>59</v>
+      </c>
+      <c r="J86" t="s">
+        <v>95</v>
+      </c>
+      <c r="N86" s="1">
+        <v>46350</v>
+      </c>
+      <c r="P86">
+        <v>10</v>
+      </c>
+      <c r="Q86">
+        <v>2026</v>
+      </c>
+      <c r="R86">
+        <v>16962350</v>
+      </c>
+      <c r="S86" t="s">
+        <v>51</v>
+      </c>
+      <c r="U86" t="s">
+        <v>109</v>
+      </c>
+      <c r="V86" s="1">
+        <v>46296.0420403125</v>
+      </c>
+      <c r="W86">
+        <v>-53</v>
+      </c>
+      <c r="X86" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB86">
+        <v>0</v>
+      </c>
+      <c r="AC86" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH86" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI86" t="s">
         <v>151</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-02 11:45
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1224" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="152">
   <si>
     <t>CodCliente</t>
   </si>
@@ -145,10 +145,10 @@
     <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
   </si>
   <si>
+    <t>TECNO COM INFORMATICA LTDA</t>
+  </si>
+  <si>
     <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
-  </si>
-  <si>
-    <t>TECNO COM INFORMATICA LTDA</t>
   </si>
   <si>
     <t>NARCIZO ALVES CORDEIRO</t>
@@ -807,7 +807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI86"/>
+  <dimension ref="A1:AI88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -3977,10 +3977,10 @@
     </row>
     <row r="43" spans="1:35">
       <c r="A43">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C43" t="s">
         <v>47</v>
@@ -3995,7 +3995,7 @@
         <v>53</v>
       </c>
       <c r="G43">
-        <v>6802</v>
+        <v>1836</v>
       </c>
       <c r="H43">
         <v>1788</v>
@@ -4004,7 +4004,7 @@
         <v>57</v>
       </c>
       <c r="J43" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N43" s="1">
         <v>46300</v>
@@ -4016,7 +4016,7 @@
         <v>2026</v>
       </c>
       <c r="R43">
-        <v>17399221</v>
+        <v>18085221</v>
       </c>
       <c r="S43" t="s">
         <v>103</v>
@@ -4028,13 +4028,13 @@
         <v>109</v>
       </c>
       <c r="V43" s="1">
-        <v>46297.37681010416</v>
+        <v>46297.45935385417</v>
       </c>
       <c r="W43">
         <v>-3</v>
       </c>
       <c r="X43" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="AB43">
         <v>0</v>
@@ -4069,16 +4069,16 @@
         <v>53</v>
       </c>
       <c r="G44">
-        <v>6801</v>
+        <v>6802</v>
       </c>
       <c r="H44">
-        <v>1796</v>
+        <v>1788</v>
       </c>
       <c r="I44" t="s">
         <v>57</v>
       </c>
       <c r="J44" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="N44" s="1">
         <v>46300</v>
@@ -4090,7 +4090,7 @@
         <v>2026</v>
       </c>
       <c r="R44">
-        <v>17399211</v>
+        <v>17399221</v>
       </c>
       <c r="S44" t="s">
         <v>103</v>
@@ -4102,7 +4102,7 @@
         <v>109</v>
       </c>
       <c r="V44" s="1">
-        <v>46297.37686377315</v>
+        <v>46297.37681010416</v>
       </c>
       <c r="W44">
         <v>-3</v>
@@ -4143,16 +4143,16 @@
         <v>53</v>
       </c>
       <c r="G45">
-        <v>6014</v>
+        <v>6801</v>
       </c>
       <c r="H45">
-        <v>1788</v>
+        <v>1796</v>
       </c>
       <c r="I45" t="s">
         <v>57</v>
       </c>
       <c r="J45" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N45" s="1">
         <v>46300</v>
@@ -4164,7 +4164,7 @@
         <v>2026</v>
       </c>
       <c r="R45">
-        <v>17399137</v>
+        <v>17399211</v>
       </c>
       <c r="S45" t="s">
         <v>103</v>
@@ -4176,7 +4176,7 @@
         <v>109</v>
       </c>
       <c r="V45" s="1">
-        <v>46297.37606362269</v>
+        <v>46297.37686377315</v>
       </c>
       <c r="W45">
         <v>-3</v>
@@ -4217,16 +4217,16 @@
         <v>53</v>
       </c>
       <c r="G46">
-        <v>6233</v>
+        <v>6014</v>
       </c>
       <c r="H46">
-        <v>6232</v>
+        <v>1788</v>
       </c>
       <c r="I46" t="s">
         <v>57</v>
       </c>
       <c r="J46" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N46" s="1">
         <v>46300</v>
@@ -4238,7 +4238,7 @@
         <v>2026</v>
       </c>
       <c r="R46">
-        <v>17399177</v>
+        <v>17399137</v>
       </c>
       <c r="S46" t="s">
         <v>103</v>
@@ -4250,7 +4250,7 @@
         <v>109</v>
       </c>
       <c r="V46" s="1">
-        <v>46297.37537966435</v>
+        <v>46297.37606362269</v>
       </c>
       <c r="W46">
         <v>-3</v>
@@ -4273,16 +4273,16 @@
     </row>
     <row r="47" spans="1:35">
       <c r="A47">
-        <v>6404</v>
+        <v>6704</v>
       </c>
       <c r="B47" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C47" t="s">
         <v>47</v>
       </c>
       <c r="D47" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E47" t="s">
         <v>51</v>
@@ -4291,16 +4291,16 @@
         <v>53</v>
       </c>
       <c r="G47">
-        <v>6233</v>
+        <v>6014</v>
       </c>
       <c r="H47">
-        <v>6232</v>
+        <v>1788</v>
       </c>
       <c r="I47" t="s">
         <v>57</v>
       </c>
       <c r="J47" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N47" s="1">
         <v>46300</v>
@@ -4312,7 +4312,7 @@
         <v>2026</v>
       </c>
       <c r="R47">
-        <v>16962295</v>
+        <v>18085232</v>
       </c>
       <c r="S47" t="s">
         <v>103</v>
@@ -4324,13 +4324,13 @@
         <v>109</v>
       </c>
       <c r="V47" s="1">
-        <v>46297.45869950231</v>
+        <v>46297.45929016203</v>
       </c>
       <c r="W47">
         <v>-3</v>
       </c>
       <c r="X47" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AB47">
         <v>0</v>
@@ -4347,16 +4347,16 @@
     </row>
     <row r="48" spans="1:35">
       <c r="A48">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C48" t="s">
         <v>47</v>
       </c>
       <c r="D48" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E48" t="s">
         <v>51</v>
@@ -4386,7 +4386,7 @@
         <v>2026</v>
       </c>
       <c r="R48">
-        <v>17948845</v>
+        <v>17399177</v>
       </c>
       <c r="S48" t="s">
         <v>103</v>
@@ -4398,13 +4398,13 @@
         <v>109</v>
       </c>
       <c r="V48" s="1">
-        <v>46297.45870309028</v>
+        <v>46297.37537966435</v>
       </c>
       <c r="W48">
         <v>-3</v>
       </c>
       <c r="X48" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AB48">
         <v>0</v>
@@ -4421,16 +4421,16 @@
     </row>
     <row r="49" spans="1:35">
       <c r="A49">
-        <v>6704</v>
+        <v>6404</v>
       </c>
       <c r="B49" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C49" t="s">
         <v>47</v>
       </c>
       <c r="D49" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E49" t="s">
         <v>51</v>
@@ -4460,7 +4460,7 @@
         <v>2026</v>
       </c>
       <c r="R49">
-        <v>18085265</v>
+        <v>16962295</v>
       </c>
       <c r="S49" t="s">
         <v>103</v>
@@ -4472,13 +4472,13 @@
         <v>109</v>
       </c>
       <c r="V49" s="1">
-        <v>46297.45870405093</v>
+        <v>46297.45869950231</v>
       </c>
       <c r="W49">
         <v>-3</v>
       </c>
       <c r="X49" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AB49">
         <v>0</v>
@@ -4495,16 +4495,16 @@
     </row>
     <row r="50" spans="1:35">
       <c r="A50">
-        <v>6705</v>
+        <v>6703</v>
       </c>
       <c r="B50" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C50" t="s">
         <v>47</v>
       </c>
       <c r="D50" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E50" t="s">
         <v>51</v>
@@ -4534,7 +4534,7 @@
         <v>2026</v>
       </c>
       <c r="R50">
-        <v>17948990</v>
+        <v>17948845</v>
       </c>
       <c r="S50" t="s">
         <v>103</v>
@@ -4546,13 +4546,13 @@
         <v>109</v>
       </c>
       <c r="V50" s="1">
-        <v>46297.45870177083</v>
+        <v>46297.45870309028</v>
       </c>
       <c r="W50">
         <v>-3</v>
       </c>
       <c r="X50" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="AB50">
         <v>0</v>
@@ -4569,37 +4569,37 @@
     </row>
     <row r="51" spans="1:35">
       <c r="A51">
-        <v>6628</v>
+        <v>6704</v>
       </c>
       <c r="B51" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C51" t="s">
         <v>47</v>
       </c>
       <c r="D51" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F51" t="s">
         <v>53</v>
       </c>
       <c r="G51">
-        <v>945</v>
+        <v>6233</v>
       </c>
       <c r="H51">
-        <v>0</v>
+        <v>6232</v>
       </c>
       <c r="I51" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J51" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N51" s="1">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="P51">
         <v>9</v>
@@ -4608,34 +4608,34 @@
         <v>2026</v>
       </c>
       <c r="R51">
-        <v>16959939</v>
+        <v>18085265</v>
       </c>
       <c r="S51" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="T51" t="s">
+        <v>108</v>
       </c>
       <c r="U51" t="s">
         <v>109</v>
       </c>
       <c r="V51" s="1">
-        <v>46296.08337256945</v>
+        <v>46297.45870405093</v>
       </c>
       <c r="W51">
-        <v>-18</v>
+        <v>-3</v>
       </c>
       <c r="X51" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y51" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="AB51">
         <v>0</v>
       </c>
       <c r="AC51" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AH51" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AI51" t="s">
         <v>151</v>
@@ -4643,10 +4643,10 @@
     </row>
     <row r="52" spans="1:35">
       <c r="A52">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B52" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C52" t="s">
         <v>47</v>
@@ -4661,19 +4661,19 @@
         <v>53</v>
       </c>
       <c r="G52">
-        <v>945</v>
+        <v>6233</v>
       </c>
       <c r="H52">
-        <v>0</v>
+        <v>6232</v>
       </c>
       <c r="I52" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J52" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N52" s="1">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="P52">
         <v>9</v>
@@ -4682,34 +4682,34 @@
         <v>2026</v>
       </c>
       <c r="R52">
-        <v>18056696</v>
+        <v>17948990</v>
       </c>
       <c r="S52" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="T52" t="s">
+        <v>108</v>
       </c>
       <c r="U52" t="s">
         <v>109</v>
       </c>
       <c r="V52" s="1">
-        <v>46296.0834071412</v>
+        <v>46297.45870177083</v>
       </c>
       <c r="W52">
-        <v>-18</v>
+        <v>-3</v>
       </c>
       <c r="X52" t="s">
         <v>112</v>
       </c>
-      <c r="Y52" t="s">
-        <v>125</v>
-      </c>
       <c r="AB52">
         <v>0</v>
       </c>
       <c r="AC52" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AH52" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AI52" t="s">
         <v>151</v>
@@ -4717,10 +4717,10 @@
     </row>
     <row r="53" spans="1:35">
       <c r="A53">
-        <v>6945</v>
+        <v>6628</v>
       </c>
       <c r="B53" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C53" t="s">
         <v>47</v>
@@ -4729,10 +4729,10 @@
         <v>48</v>
       </c>
       <c r="E53" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F53" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G53">
         <v>945</v>
@@ -4756,7 +4756,7 @@
         <v>2026</v>
       </c>
       <c r="R53">
-        <v>18164488</v>
+        <v>16959939</v>
       </c>
       <c r="S53" t="s">
         <v>104</v>
@@ -4765,13 +4765,13 @@
         <v>109</v>
       </c>
       <c r="V53" s="1">
-        <v>46296.08341825232</v>
+        <v>46296.08337256945</v>
       </c>
       <c r="W53">
         <v>-18</v>
       </c>
       <c r="X53" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="Y53" t="s">
         <v>124</v>
@@ -4791,16 +4791,16 @@
     </row>
     <row r="54" spans="1:35">
       <c r="A54">
-        <v>5417</v>
+        <v>6779</v>
       </c>
       <c r="B54" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C54" t="s">
         <v>47</v>
       </c>
       <c r="D54" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E54" t="s">
         <v>51</v>
@@ -4809,7 +4809,7 @@
         <v>53</v>
       </c>
       <c r="G54">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H54">
         <v>0</v>
@@ -4818,7 +4818,7 @@
         <v>58</v>
       </c>
       <c r="J54" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N54" s="1">
         <v>46315</v>
@@ -4830,7 +4830,7 @@
         <v>2026</v>
       </c>
       <c r="R54">
-        <v>17398870</v>
+        <v>18056696</v>
       </c>
       <c r="S54" t="s">
         <v>104</v>
@@ -4839,16 +4839,16 @@
         <v>109</v>
       </c>
       <c r="V54" s="1">
-        <v>46296.37558109954</v>
+        <v>46296.0834071412</v>
       </c>
       <c r="W54">
         <v>-18</v>
       </c>
       <c r="X54" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="Y54" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AB54">
         <v>0</v>
@@ -4865,25 +4865,25 @@
     </row>
     <row r="55" spans="1:35">
       <c r="A55">
-        <v>6404</v>
+        <v>6945</v>
       </c>
       <c r="B55" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C55" t="s">
         <v>47</v>
       </c>
       <c r="D55" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E55" t="s">
         <v>51</v>
       </c>
       <c r="F55" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G55">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H55">
         <v>0</v>
@@ -4892,7 +4892,7 @@
         <v>58</v>
       </c>
       <c r="J55" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="N55" s="1">
         <v>46315</v>
@@ -4904,7 +4904,7 @@
         <v>2026</v>
       </c>
       <c r="R55">
-        <v>16962094</v>
+        <v>18164488</v>
       </c>
       <c r="S55" t="s">
         <v>104</v>
@@ -4913,16 +4913,16 @@
         <v>109</v>
       </c>
       <c r="V55" s="1">
-        <v>46296.37504012731</v>
+        <v>46296.08341825232</v>
       </c>
       <c r="W55">
         <v>-18</v>
       </c>
       <c r="X55" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="Y55" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="AB55">
         <v>0</v>
@@ -4939,16 +4939,16 @@
     </row>
     <row r="56" spans="1:35">
       <c r="A56">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B56" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C56" t="s">
         <v>47</v>
       </c>
       <c r="D56" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E56" t="s">
         <v>51</v>
@@ -4978,31 +4978,31 @@
         <v>2026</v>
       </c>
       <c r="R56">
-        <v>17941133</v>
+        <v>17398870</v>
       </c>
       <c r="S56" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U56" t="s">
         <v>109</v>
       </c>
       <c r="V56" s="1">
-        <v>46296.3760846412</v>
+        <v>46296.37558109954</v>
       </c>
       <c r="W56">
         <v>-18</v>
       </c>
       <c r="X56" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="Y56" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AB56">
         <v>0</v>
       </c>
       <c r="AC56" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AH56" t="s">
         <v>150</v>
@@ -5013,16 +5013,16 @@
     </row>
     <row r="57" spans="1:35">
       <c r="A57">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B57" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C57" t="s">
         <v>47</v>
       </c>
       <c r="D57" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E57" t="s">
         <v>51</v>
@@ -5031,7 +5031,7 @@
         <v>53</v>
       </c>
       <c r="G57">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="H57">
         <v>0</v>
@@ -5040,10 +5040,10 @@
         <v>58</v>
       </c>
       <c r="J57" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N57" s="1">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="P57">
         <v>9</v>
@@ -5052,7 +5052,7 @@
         <v>2026</v>
       </c>
       <c r="R57">
-        <v>17398876</v>
+        <v>16962094</v>
       </c>
       <c r="S57" t="s">
         <v>104</v>
@@ -5061,16 +5061,16 @@
         <v>109</v>
       </c>
       <c r="V57" s="1">
-        <v>46296.37648518519</v>
+        <v>46296.37504012731</v>
       </c>
       <c r="W57">
-        <v>-28</v>
+        <v>-18</v>
       </c>
       <c r="X57" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="Y57" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="AB57">
         <v>0</v>
@@ -5087,25 +5087,25 @@
     </row>
     <row r="58" spans="1:35">
       <c r="A58">
-        <v>6627</v>
+        <v>6703</v>
       </c>
       <c r="B58" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C58" t="s">
         <v>47</v>
       </c>
       <c r="D58" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E58" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F58" t="s">
         <v>53</v>
       </c>
       <c r="G58">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="H58">
         <v>0</v>
@@ -5114,10 +5114,10 @@
         <v>58</v>
       </c>
       <c r="J58" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N58" s="1">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="P58">
         <v>9</v>
@@ -5126,31 +5126,31 @@
         <v>2026</v>
       </c>
       <c r="R58">
-        <v>17042296</v>
+        <v>17941133</v>
       </c>
       <c r="S58" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U58" t="s">
         <v>109</v>
       </c>
       <c r="V58" s="1">
-        <v>46296.37615983796</v>
+        <v>46296.3760846412</v>
       </c>
       <c r="W58">
-        <v>-28</v>
+        <v>-18</v>
       </c>
       <c r="X58" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="Y58" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="AB58">
         <v>0</v>
       </c>
       <c r="AC58" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH58" t="s">
         <v>150</v>
@@ -5161,10 +5161,10 @@
     </row>
     <row r="59" spans="1:35">
       <c r="A59">
-        <v>6704</v>
+        <v>5417</v>
       </c>
       <c r="B59" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C59" t="s">
         <v>47</v>
@@ -5200,7 +5200,7 @@
         <v>2026</v>
       </c>
       <c r="R59">
-        <v>17952332</v>
+        <v>17398876</v>
       </c>
       <c r="S59" t="s">
         <v>104</v>
@@ -5209,13 +5209,13 @@
         <v>109</v>
       </c>
       <c r="V59" s="1">
-        <v>46296.37684290509</v>
+        <v>46296.37648518519</v>
       </c>
       <c r="W59">
         <v>-28</v>
       </c>
       <c r="X59" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="Y59" t="s">
         <v>129</v>
@@ -5235,25 +5235,25 @@
     </row>
     <row r="60" spans="1:35">
       <c r="A60">
-        <v>6404</v>
+        <v>6627</v>
       </c>
       <c r="B60" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C60" t="s">
         <v>47</v>
       </c>
       <c r="D60" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E60" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F60" t="s">
         <v>53</v>
       </c>
       <c r="G60">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="H60">
         <v>0</v>
@@ -5262,7 +5262,7 @@
         <v>58</v>
       </c>
       <c r="J60" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N60" s="1">
         <v>46325</v>
@@ -5274,7 +5274,7 @@
         <v>2026</v>
       </c>
       <c r="R60">
-        <v>16962100</v>
+        <v>17042296</v>
       </c>
       <c r="S60" t="s">
         <v>104</v>
@@ -5283,16 +5283,16 @@
         <v>109</v>
       </c>
       <c r="V60" s="1">
-        <v>46296.37609667824</v>
+        <v>46296.37615983796</v>
       </c>
       <c r="W60">
         <v>-28</v>
       </c>
       <c r="X60" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Y60" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AB60">
         <v>0</v>
@@ -5309,7 +5309,7 @@
     </row>
     <row r="61" spans="1:35">
       <c r="A61">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B61" t="s">
         <v>43</v>
@@ -5318,7 +5318,7 @@
         <v>47</v>
       </c>
       <c r="D61" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E61" t="s">
         <v>51</v>
@@ -5327,7 +5327,7 @@
         <v>53</v>
       </c>
       <c r="G61">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="H61">
         <v>0</v>
@@ -5336,7 +5336,7 @@
         <v>58</v>
       </c>
       <c r="J61" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N61" s="1">
         <v>46325</v>
@@ -5348,31 +5348,31 @@
         <v>2026</v>
       </c>
       <c r="R61">
-        <v>17941139</v>
+        <v>17952332</v>
       </c>
       <c r="S61" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U61" t="s">
         <v>109</v>
       </c>
       <c r="V61" s="1">
-        <v>46296.37683961805</v>
+        <v>46296.37684290509</v>
       </c>
       <c r="W61">
         <v>-28</v>
       </c>
       <c r="X61" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="Y61" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="AB61">
         <v>0</v>
       </c>
       <c r="AC61" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AH61" t="s">
         <v>150</v>
@@ -5383,10 +5383,10 @@
     </row>
     <row r="62" spans="1:35">
       <c r="A62">
-        <v>6703</v>
+        <v>6404</v>
       </c>
       <c r="B62" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C62" t="s">
         <v>47</v>
@@ -5401,7 +5401,7 @@
         <v>53</v>
       </c>
       <c r="G62">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="H62">
         <v>0</v>
@@ -5410,10 +5410,10 @@
         <v>58</v>
       </c>
       <c r="J62" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="N62" s="1">
-        <v>46304</v>
+        <v>46325</v>
       </c>
       <c r="P62">
         <v>9</v>
@@ -5422,31 +5422,31 @@
         <v>2026</v>
       </c>
       <c r="R62">
-        <v>17941147</v>
+        <v>16962100</v>
       </c>
       <c r="S62" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U62" t="s">
         <v>109</v>
       </c>
       <c r="V62" s="1">
-        <v>46296.37684039352</v>
+        <v>46296.37609667824</v>
       </c>
       <c r="W62">
-        <v>-7</v>
+        <v>-28</v>
       </c>
       <c r="X62" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="Y62" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="AB62">
         <v>0</v>
       </c>
       <c r="AC62" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AH62" t="s">
         <v>150</v>
@@ -5457,25 +5457,25 @@
     </row>
     <row r="63" spans="1:35">
       <c r="A63">
-        <v>6949</v>
+        <v>6703</v>
       </c>
       <c r="B63" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C63" t="s">
         <v>47</v>
       </c>
       <c r="D63" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E63" t="s">
         <v>51</v>
       </c>
       <c r="F63" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G63">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="H63">
         <v>0</v>
@@ -5484,10 +5484,10 @@
         <v>58</v>
       </c>
       <c r="J63" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="N63" s="1">
-        <v>46304</v>
+        <v>46325</v>
       </c>
       <c r="P63">
         <v>9</v>
@@ -5496,31 +5496,31 @@
         <v>2026</v>
       </c>
       <c r="R63">
-        <v>18178133</v>
+        <v>17941139</v>
       </c>
       <c r="S63" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U63" t="s">
         <v>109</v>
       </c>
       <c r="V63" s="1">
-        <v>46296.37697557871</v>
+        <v>46296.37683961805</v>
       </c>
       <c r="W63">
-        <v>-7</v>
+        <v>-28</v>
       </c>
       <c r="X63" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="Y63" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="AB63">
         <v>0</v>
       </c>
       <c r="AC63" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH63" t="s">
         <v>150</v>
@@ -5531,16 +5531,16 @@
     </row>
     <row r="64" spans="1:35">
       <c r="A64">
-        <v>6548</v>
+        <v>6703</v>
       </c>
       <c r="B64" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C64" t="s">
         <v>47</v>
       </c>
       <c r="D64" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E64" t="s">
         <v>51</v>
@@ -5549,7 +5549,7 @@
         <v>53</v>
       </c>
       <c r="G64">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H64">
         <v>0</v>
@@ -5558,7 +5558,7 @@
         <v>58</v>
       </c>
       <c r="J64" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N64" s="1">
         <v>46304</v>
@@ -5570,31 +5570,31 @@
         <v>2026</v>
       </c>
       <c r="R64">
-        <v>17222406</v>
+        <v>17941147</v>
       </c>
       <c r="S64" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U64" t="s">
         <v>109</v>
       </c>
       <c r="V64" s="1">
-        <v>46296.37726273148</v>
+        <v>46296.37684039352</v>
       </c>
       <c r="W64">
         <v>-7</v>
       </c>
       <c r="X64" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="Y64" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="AB64">
         <v>0</v>
       </c>
       <c r="AC64" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH64" t="s">
         <v>150</v>
@@ -5605,25 +5605,25 @@
     </row>
     <row r="65" spans="1:35">
       <c r="A65">
-        <v>6703</v>
+        <v>6949</v>
       </c>
       <c r="B65" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C65" t="s">
         <v>47</v>
       </c>
       <c r="D65" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E65" t="s">
         <v>51</v>
       </c>
       <c r="F65" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G65">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H65">
         <v>0</v>
@@ -5632,7 +5632,7 @@
         <v>58</v>
       </c>
       <c r="J65" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N65" s="1">
         <v>46304</v>
@@ -5644,31 +5644,31 @@
         <v>2026</v>
       </c>
       <c r="R65">
-        <v>17941157</v>
+        <v>18178133</v>
       </c>
       <c r="S65" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U65" t="s">
         <v>109</v>
       </c>
       <c r="V65" s="1">
-        <v>46296.37814100694</v>
+        <v>46296.37697557871</v>
       </c>
       <c r="W65">
         <v>-7</v>
       </c>
       <c r="X65" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="Y65" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AB65">
         <v>0</v>
       </c>
       <c r="AC65" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AH65" t="s">
         <v>150</v>
@@ -5679,16 +5679,16 @@
     </row>
     <row r="66" spans="1:35">
       <c r="A66">
-        <v>6779</v>
+        <v>6548</v>
       </c>
       <c r="B66" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C66" t="s">
         <v>47</v>
       </c>
       <c r="D66" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E66" t="s">
         <v>51</v>
@@ -5718,7 +5718,7 @@
         <v>2026</v>
       </c>
       <c r="R66">
-        <v>18056706</v>
+        <v>17222406</v>
       </c>
       <c r="S66" t="s">
         <v>104</v>
@@ -5727,16 +5727,16 @@
         <v>109</v>
       </c>
       <c r="V66" s="1">
-        <v>46296.37816597222</v>
+        <v>46296.37726273148</v>
       </c>
       <c r="W66">
         <v>-7</v>
       </c>
       <c r="X66" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="Y66" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AB66">
         <v>0</v>
@@ -5753,22 +5753,22 @@
     </row>
     <row r="67" spans="1:35">
       <c r="A67">
-        <v>6945</v>
+        <v>6703</v>
       </c>
       <c r="B67" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C67" t="s">
         <v>47</v>
       </c>
       <c r="D67" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E67" t="s">
         <v>51</v>
       </c>
       <c r="F67" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G67">
         <v>951</v>
@@ -5792,31 +5792,31 @@
         <v>2026</v>
       </c>
       <c r="R67">
-        <v>18164502</v>
+        <v>17941157</v>
       </c>
       <c r="S67" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U67" t="s">
         <v>109</v>
       </c>
       <c r="V67" s="1">
-        <v>46296.3782184838</v>
+        <v>46296.37814100694</v>
       </c>
       <c r="W67">
         <v>-7</v>
       </c>
       <c r="X67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="Y67" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AB67">
         <v>0</v>
       </c>
       <c r="AC67" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH67" t="s">
         <v>150</v>
@@ -5827,22 +5827,22 @@
     </row>
     <row r="68" spans="1:35">
       <c r="A68">
-        <v>6949</v>
+        <v>6779</v>
       </c>
       <c r="B68" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C68" t="s">
         <v>47</v>
       </c>
       <c r="D68" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E68" t="s">
         <v>51</v>
       </c>
       <c r="F68" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G68">
         <v>951</v>
@@ -5866,7 +5866,7 @@
         <v>2026</v>
       </c>
       <c r="R68">
-        <v>18178139</v>
+        <v>18056706</v>
       </c>
       <c r="S68" t="s">
         <v>104</v>
@@ -5875,16 +5875,16 @@
         <v>109</v>
       </c>
       <c r="V68" s="1">
-        <v>46296.37822091435</v>
+        <v>46296.37816597222</v>
       </c>
       <c r="W68">
         <v>-7</v>
       </c>
       <c r="X68" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="Y68" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AB68">
         <v>0</v>
@@ -5901,25 +5901,25 @@
     </row>
     <row r="69" spans="1:35">
       <c r="A69">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B69" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C69" t="s">
         <v>47</v>
       </c>
       <c r="D69" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E69" t="s">
         <v>51</v>
       </c>
       <c r="F69" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G69">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="H69">
         <v>0</v>
@@ -5928,10 +5928,10 @@
         <v>58</v>
       </c>
       <c r="J69" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N69" s="1">
-        <v>46318</v>
+        <v>46304</v>
       </c>
       <c r="P69">
         <v>9</v>
@@ -5940,7 +5940,7 @@
         <v>2026</v>
       </c>
       <c r="R69">
-        <v>17398884</v>
+        <v>18164502</v>
       </c>
       <c r="S69" t="s">
         <v>104</v>
@@ -5949,16 +5949,16 @@
         <v>109</v>
       </c>
       <c r="V69" s="1">
-        <v>46296.37748545139</v>
+        <v>46296.3782184838</v>
       </c>
       <c r="W69">
-        <v>-21</v>
+        <v>-7</v>
       </c>
       <c r="X69" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Y69" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AB69">
         <v>0</v>
@@ -5975,25 +5975,25 @@
     </row>
     <row r="70" spans="1:35">
       <c r="A70">
-        <v>6404</v>
+        <v>6949</v>
       </c>
       <c r="B70" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C70" t="s">
         <v>47</v>
       </c>
       <c r="D70" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E70" t="s">
         <v>51</v>
       </c>
       <c r="F70" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G70">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="H70">
         <v>0</v>
@@ -6002,10 +6002,10 @@
         <v>58</v>
       </c>
       <c r="J70" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N70" s="1">
-        <v>46318</v>
+        <v>46304</v>
       </c>
       <c r="P70">
         <v>9</v>
@@ -6014,7 +6014,7 @@
         <v>2026</v>
       </c>
       <c r="R70">
-        <v>16962108</v>
+        <v>18178139</v>
       </c>
       <c r="S70" t="s">
         <v>104</v>
@@ -6023,16 +6023,16 @@
         <v>109</v>
       </c>
       <c r="V70" s="1">
-        <v>46296.37705413195</v>
+        <v>46296.37822091435</v>
       </c>
       <c r="W70">
-        <v>-21</v>
+        <v>-7</v>
       </c>
       <c r="X70" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="Y70" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="AB70">
         <v>0</v>
@@ -6049,10 +6049,10 @@
     </row>
     <row r="71" spans="1:35">
       <c r="A71">
-        <v>6627</v>
+        <v>5417</v>
       </c>
       <c r="B71" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C71" t="s">
         <v>47</v>
@@ -6061,7 +6061,7 @@
         <v>50</v>
       </c>
       <c r="E71" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F71" t="s">
         <v>53</v>
@@ -6088,7 +6088,7 @@
         <v>2026</v>
       </c>
       <c r="R71">
-        <v>17042320</v>
+        <v>17398884</v>
       </c>
       <c r="S71" t="s">
         <v>104</v>
@@ -6097,16 +6097,16 @@
         <v>109</v>
       </c>
       <c r="V71" s="1">
-        <v>46296.37710454861</v>
+        <v>46296.37748545139</v>
       </c>
       <c r="W71">
         <v>-21</v>
       </c>
       <c r="X71" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="Y71" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="AB71">
         <v>0</v>
@@ -6123,10 +6123,10 @@
     </row>
     <row r="72" spans="1:35">
       <c r="A72">
-        <v>6703</v>
+        <v>6404</v>
       </c>
       <c r="B72" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C72" t="s">
         <v>47</v>
@@ -6162,31 +6162,31 @@
         <v>2026</v>
       </c>
       <c r="R72">
-        <v>17941167</v>
+        <v>16962108</v>
       </c>
       <c r="S72" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="U72" t="s">
         <v>109</v>
       </c>
       <c r="V72" s="1">
-        <v>46296.37814163195</v>
+        <v>46296.37705413195</v>
       </c>
       <c r="W72">
         <v>-21</v>
       </c>
       <c r="X72" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="Y72" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="AB72">
         <v>0</v>
       </c>
       <c r="AC72" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AH72" t="s">
         <v>150</v>
@@ -6197,10 +6197,10 @@
     </row>
     <row r="73" spans="1:35">
       <c r="A73">
-        <v>6949</v>
+        <v>6627</v>
       </c>
       <c r="B73" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C73" t="s">
         <v>47</v>
@@ -6209,10 +6209,10 @@
         <v>50</v>
       </c>
       <c r="E73" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F73" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G73">
         <v>953</v>
@@ -6236,7 +6236,7 @@
         <v>2026</v>
       </c>
       <c r="R73">
-        <v>18178145</v>
+        <v>17042320</v>
       </c>
       <c r="S73" t="s">
         <v>104</v>
@@ -6245,16 +6245,16 @@
         <v>109</v>
       </c>
       <c r="V73" s="1">
-        <v>46296.37822175926</v>
+        <v>46296.37710454861</v>
       </c>
       <c r="W73">
         <v>-21</v>
       </c>
       <c r="X73" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="Y73" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="AB73">
         <v>0</v>
@@ -6271,16 +6271,16 @@
     </row>
     <row r="74" spans="1:35">
       <c r="A74">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B74" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C74" t="s">
         <v>47</v>
       </c>
       <c r="D74" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E74" t="s">
         <v>51</v>
@@ -6289,7 +6289,7 @@
         <v>53</v>
       </c>
       <c r="G74">
-        <v>941</v>
+        <v>953</v>
       </c>
       <c r="H74">
         <v>0</v>
@@ -6298,10 +6298,10 @@
         <v>58</v>
       </c>
       <c r="J74" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N74" s="1">
-        <v>46297</v>
+        <v>46318</v>
       </c>
       <c r="P74">
         <v>9</v>
@@ -6310,31 +6310,34 @@
         <v>2026</v>
       </c>
       <c r="R74">
-        <v>17398850</v>
+        <v>17941167</v>
       </c>
       <c r="S74" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="U74" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="V74" s="1">
-        <v>46297.34991217592</v>
+        <v>46296.37814163195</v>
       </c>
       <c r="W74">
-        <v>0</v>
+        <v>-21</v>
       </c>
       <c r="X74" t="s">
-        <v>118</v>
+        <v>119</v>
+      </c>
+      <c r="Y74" t="s">
+        <v>141</v>
       </c>
       <c r="AB74">
         <v>0</v>
       </c>
       <c r="AC74" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH74" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AI74" t="s">
         <v>151</v>
@@ -6342,25 +6345,25 @@
     </row>
     <row r="75" spans="1:35">
       <c r="A75">
-        <v>6404</v>
+        <v>6949</v>
       </c>
       <c r="B75" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C75" t="s">
         <v>47</v>
       </c>
       <c r="D75" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E75" t="s">
         <v>51</v>
       </c>
       <c r="F75" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G75">
-        <v>941</v>
+        <v>953</v>
       </c>
       <c r="H75">
         <v>0</v>
@@ -6369,10 +6372,10 @@
         <v>58</v>
       </c>
       <c r="J75" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N75" s="1">
-        <v>46297</v>
+        <v>46318</v>
       </c>
       <c r="P75">
         <v>9</v>
@@ -6381,22 +6384,25 @@
         <v>2026</v>
       </c>
       <c r="R75">
-        <v>16962084</v>
+        <v>18178145</v>
       </c>
       <c r="S75" t="s">
         <v>104</v>
       </c>
       <c r="U75" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="V75" s="1">
-        <v>46297.3499325</v>
+        <v>46296.37822175926</v>
       </c>
       <c r="W75">
-        <v>0</v>
+        <v>-21</v>
       </c>
       <c r="X75" t="s">
-        <v>113</v>
+        <v>116</v>
+      </c>
+      <c r="Y75" t="s">
+        <v>142</v>
       </c>
       <c r="AB75">
         <v>0</v>
@@ -6405,7 +6411,7 @@
         <v>104</v>
       </c>
       <c r="AH75" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AI75" t="s">
         <v>151</v>
@@ -6413,10 +6419,10 @@
     </row>
     <row r="76" spans="1:35">
       <c r="A76">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B76" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C76" t="s">
         <v>47</v>
@@ -6452,7 +6458,7 @@
         <v>2026</v>
       </c>
       <c r="R76">
-        <v>16975881</v>
+        <v>17398850</v>
       </c>
       <c r="S76" t="s">
         <v>104</v>
@@ -6461,13 +6467,13 @@
         <v>111</v>
       </c>
       <c r="V76" s="1">
-        <v>46297.34994254629</v>
+        <v>46297.34991217592</v>
       </c>
       <c r="W76">
         <v>0</v>
       </c>
       <c r="X76" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AB76">
         <v>0</v>
@@ -6484,19 +6490,19 @@
     </row>
     <row r="77" spans="1:35">
       <c r="A77">
-        <v>6627</v>
+        <v>6404</v>
       </c>
       <c r="B77" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C77" t="s">
         <v>47</v>
       </c>
       <c r="D77" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E77" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F77" t="s">
         <v>53</v>
@@ -6523,7 +6529,7 @@
         <v>2026</v>
       </c>
       <c r="R77">
-        <v>17042242</v>
+        <v>16962084</v>
       </c>
       <c r="S77" t="s">
         <v>104</v>
@@ -6532,13 +6538,13 @@
         <v>111</v>
       </c>
       <c r="V77" s="1">
-        <v>46297.34994771991</v>
+        <v>46297.3499325</v>
       </c>
       <c r="W77">
         <v>0</v>
       </c>
       <c r="X77" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="AB77">
         <v>0</v>
@@ -6555,10 +6561,10 @@
     </row>
     <row r="78" spans="1:35">
       <c r="A78">
-        <v>6704</v>
+        <v>6486</v>
       </c>
       <c r="B78" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C78" t="s">
         <v>47</v>
@@ -6594,7 +6600,7 @@
         <v>2026</v>
       </c>
       <c r="R78">
-        <v>17952303</v>
+        <v>16975881</v>
       </c>
       <c r="S78" t="s">
         <v>104</v>
@@ -6603,13 +6609,13 @@
         <v>111</v>
       </c>
       <c r="V78" s="1">
-        <v>46297.34994974537</v>
+        <v>46297.34994254629</v>
       </c>
       <c r="W78">
         <v>0</v>
       </c>
       <c r="X78" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="AB78">
         <v>0</v>
@@ -6626,19 +6632,19 @@
     </row>
     <row r="79" spans="1:35">
       <c r="A79">
-        <v>6705</v>
+        <v>6627</v>
       </c>
       <c r="B79" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C79" t="s">
         <v>47</v>
       </c>
       <c r="D79" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E79" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F79" t="s">
         <v>53</v>
@@ -6665,7 +6671,7 @@
         <v>2026</v>
       </c>
       <c r="R79">
-        <v>17952502</v>
+        <v>17042242</v>
       </c>
       <c r="S79" t="s">
         <v>104</v>
@@ -6674,13 +6680,13 @@
         <v>111</v>
       </c>
       <c r="V79" s="1">
-        <v>46297.34995063658</v>
+        <v>46297.34994771991</v>
       </c>
       <c r="W79">
         <v>0</v>
       </c>
       <c r="X79" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="AB79">
         <v>0</v>
@@ -6697,22 +6703,22 @@
     </row>
     <row r="80" spans="1:35">
       <c r="A80">
-        <v>6945</v>
+        <v>6704</v>
       </c>
       <c r="B80" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C80" t="s">
         <v>47</v>
       </c>
       <c r="D80" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E80" t="s">
         <v>51</v>
       </c>
       <c r="F80" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G80">
         <v>941</v>
@@ -6736,7 +6742,7 @@
         <v>2026</v>
       </c>
       <c r="R80">
-        <v>18164480</v>
+        <v>17952303</v>
       </c>
       <c r="S80" t="s">
         <v>104</v>
@@ -6745,13 +6751,13 @@
         <v>111</v>
       </c>
       <c r="V80" s="1">
-        <v>46297.34996266204</v>
+        <v>46297.34994974537</v>
       </c>
       <c r="W80">
         <v>0</v>
       </c>
       <c r="X80" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="AB80">
         <v>0</v>
@@ -6768,16 +6774,16 @@
     </row>
     <row r="81" spans="1:35">
       <c r="A81">
-        <v>6404</v>
+        <v>6705</v>
       </c>
       <c r="B81" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C81" t="s">
         <v>47</v>
       </c>
       <c r="D81" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E81" t="s">
         <v>51</v>
@@ -6786,52 +6792,49 @@
         <v>53</v>
       </c>
       <c r="G81">
-        <v>11001</v>
+        <v>941</v>
       </c>
       <c r="H81">
         <v>0</v>
       </c>
       <c r="I81" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J81" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N81" s="1">
-        <v>46351</v>
+        <v>46297</v>
       </c>
       <c r="P81">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q81">
         <v>2026</v>
       </c>
       <c r="R81">
-        <v>16962456</v>
+        <v>17952502</v>
       </c>
       <c r="S81" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="U81" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="V81" s="1">
-        <v>46296.34114513889</v>
+        <v>46297.34995063658</v>
       </c>
       <c r="W81">
-        <v>-54</v>
+        <v>0</v>
       </c>
       <c r="X81" t="s">
-        <v>113</v>
-      </c>
-      <c r="Y81" t="s">
-        <v>143</v>
+        <v>112</v>
       </c>
       <c r="AB81">
         <v>0</v>
       </c>
       <c r="AC81" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="AH81" t="s">
         <v>149</v>
@@ -6842,70 +6845,67 @@
     </row>
     <row r="82" spans="1:35">
       <c r="A82">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B82" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C82" t="s">
         <v>47</v>
       </c>
       <c r="D82" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E82" t="s">
         <v>51</v>
       </c>
       <c r="F82" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G82">
-        <v>7877</v>
+        <v>941</v>
       </c>
       <c r="H82">
         <v>0</v>
       </c>
       <c r="I82" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J82" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="N82" s="1">
-        <v>46351</v>
+        <v>46297</v>
       </c>
       <c r="P82">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q82">
         <v>2026</v>
       </c>
       <c r="R82">
-        <v>17399332</v>
+        <v>18164480</v>
       </c>
       <c r="S82" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="U82" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="V82" s="1">
-        <v>46296.34050315972</v>
+        <v>46297.34996266204</v>
       </c>
       <c r="W82">
-        <v>-54</v>
+        <v>0</v>
       </c>
       <c r="X82" t="s">
-        <v>118</v>
-      </c>
-      <c r="Y82" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
       <c r="AB82">
         <v>0</v>
       </c>
       <c r="AC82" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="AH82" t="s">
         <v>149</v>
@@ -6916,16 +6916,16 @@
     </row>
     <row r="83" spans="1:35">
       <c r="A83">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B83" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C83" t="s">
         <v>47</v>
       </c>
       <c r="D83" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E83" t="s">
         <v>51</v>
@@ -6934,7 +6934,7 @@
         <v>53</v>
       </c>
       <c r="G83">
-        <v>9774</v>
+        <v>11001</v>
       </c>
       <c r="H83">
         <v>0</v>
@@ -6943,37 +6943,37 @@
         <v>59</v>
       </c>
       <c r="J83" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="N83" s="1">
-        <v>46290</v>
+        <v>46351</v>
       </c>
       <c r="P83">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q83">
         <v>2026</v>
       </c>
       <c r="R83">
-        <v>16976321</v>
+        <v>16962456</v>
       </c>
       <c r="S83" t="s">
         <v>51</v>
       </c>
       <c r="U83" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="V83" s="1">
-        <v>46296.39309459491</v>
+        <v>46296.34114513889</v>
       </c>
       <c r="W83">
-        <v>7</v>
+        <v>-54</v>
       </c>
       <c r="X83" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="Y83" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="AB83">
         <v>0</v>
@@ -6990,10 +6990,10 @@
     </row>
     <row r="84" spans="1:35">
       <c r="A84">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B84" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C84" t="s">
         <v>47</v>
@@ -7008,7 +7008,7 @@
         <v>53</v>
       </c>
       <c r="G84">
-        <v>9774</v>
+        <v>7877</v>
       </c>
       <c r="H84">
         <v>0</v>
@@ -7017,7 +7017,7 @@
         <v>59</v>
       </c>
       <c r="J84" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N84" s="1">
         <v>46351</v>
@@ -7029,7 +7029,7 @@
         <v>2026</v>
       </c>
       <c r="R84">
-        <v>16976323</v>
+        <v>17399332</v>
       </c>
       <c r="S84" t="s">
         <v>51</v>
@@ -7038,16 +7038,16 @@
         <v>109</v>
       </c>
       <c r="V84" s="1">
-        <v>46296.3409153125</v>
+        <v>46296.34050315972</v>
       </c>
       <c r="W84">
         <v>-54</v>
       </c>
       <c r="X84" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Y84" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AB84">
         <v>0</v>
@@ -7064,10 +7064,10 @@
     </row>
     <row r="85" spans="1:35">
       <c r="A85">
-        <v>5417</v>
+        <v>6486</v>
       </c>
       <c r="B85" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C85" t="s">
         <v>47</v>
@@ -7082,7 +7082,7 @@
         <v>53</v>
       </c>
       <c r="G85">
-        <v>7027</v>
+        <v>9774</v>
       </c>
       <c r="H85">
         <v>0</v>
@@ -7091,34 +7091,37 @@
         <v>59</v>
       </c>
       <c r="J85" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="N85" s="1">
-        <v>46350</v>
+        <v>46290</v>
       </c>
       <c r="P85">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Q85">
         <v>2026</v>
       </c>
       <c r="R85">
-        <v>17399292</v>
+        <v>16976321</v>
       </c>
       <c r="S85" t="s">
         <v>51</v>
       </c>
       <c r="U85" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="V85" s="1">
-        <v>46296.0420403125</v>
+        <v>46296.39309459491</v>
       </c>
       <c r="W85">
-        <v>-53</v>
+        <v>7</v>
       </c>
       <c r="X85" t="s">
-        <v>118</v>
+        <v>120</v>
+      </c>
+      <c r="Y85" t="s">
+        <v>145</v>
       </c>
       <c r="AB85">
         <v>0</v>
@@ -7135,16 +7138,16 @@
     </row>
     <row r="86" spans="1:35">
       <c r="A86">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B86" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="C86" t="s">
         <v>47</v>
       </c>
       <c r="D86" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E86" t="s">
         <v>51</v>
@@ -7153,7 +7156,7 @@
         <v>53</v>
       </c>
       <c r="G86">
-        <v>7027</v>
+        <v>9774</v>
       </c>
       <c r="H86">
         <v>0</v>
@@ -7162,10 +7165,10 @@
         <v>59</v>
       </c>
       <c r="J86" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="N86" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="P86">
         <v>10</v>
@@ -7174,7 +7177,7 @@
         <v>2026</v>
       </c>
       <c r="R86">
-        <v>16962350</v>
+        <v>16976323</v>
       </c>
       <c r="S86" t="s">
         <v>51</v>
@@ -7183,13 +7186,16 @@
         <v>109</v>
       </c>
       <c r="V86" s="1">
-        <v>46296.0420403125</v>
+        <v>46296.3409153125</v>
       </c>
       <c r="W86">
-        <v>-53</v>
+        <v>-54</v>
       </c>
       <c r="X86" t="s">
-        <v>113</v>
+        <v>120</v>
+      </c>
+      <c r="Y86" t="s">
+        <v>146</v>
       </c>
       <c r="AB86">
         <v>0</v>
@@ -7201,6 +7207,148 @@
         <v>149</v>
       </c>
       <c r="AI86" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="87" spans="1:35">
+      <c r="A87">
+        <v>5417</v>
+      </c>
+      <c r="B87" t="s">
+        <v>42</v>
+      </c>
+      <c r="C87" t="s">
+        <v>47</v>
+      </c>
+      <c r="D87" t="s">
+        <v>50</v>
+      </c>
+      <c r="E87" t="s">
+        <v>51</v>
+      </c>
+      <c r="F87" t="s">
+        <v>53</v>
+      </c>
+      <c r="G87">
+        <v>7027</v>
+      </c>
+      <c r="H87">
+        <v>0</v>
+      </c>
+      <c r="I87" t="s">
+        <v>59</v>
+      </c>
+      <c r="J87" t="s">
+        <v>95</v>
+      </c>
+      <c r="N87" s="1">
+        <v>46350</v>
+      </c>
+      <c r="P87">
+        <v>10</v>
+      </c>
+      <c r="Q87">
+        <v>2026</v>
+      </c>
+      <c r="R87">
+        <v>17399292</v>
+      </c>
+      <c r="S87" t="s">
+        <v>51</v>
+      </c>
+      <c r="U87" t="s">
+        <v>109</v>
+      </c>
+      <c r="V87" s="1">
+        <v>46296.0420403125</v>
+      </c>
+      <c r="W87">
+        <v>-53</v>
+      </c>
+      <c r="X87" t="s">
+        <v>118</v>
+      </c>
+      <c r="AB87">
+        <v>0</v>
+      </c>
+      <c r="AC87" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH87" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI87" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="88" spans="1:35">
+      <c r="A88">
+        <v>6404</v>
+      </c>
+      <c r="B88" t="s">
+        <v>36</v>
+      </c>
+      <c r="C88" t="s">
+        <v>47</v>
+      </c>
+      <c r="D88" t="s">
+        <v>49</v>
+      </c>
+      <c r="E88" t="s">
+        <v>51</v>
+      </c>
+      <c r="F88" t="s">
+        <v>53</v>
+      </c>
+      <c r="G88">
+        <v>7027</v>
+      </c>
+      <c r="H88">
+        <v>0</v>
+      </c>
+      <c r="I88" t="s">
+        <v>59</v>
+      </c>
+      <c r="J88" t="s">
+        <v>95</v>
+      </c>
+      <c r="N88" s="1">
+        <v>46350</v>
+      </c>
+      <c r="P88">
+        <v>10</v>
+      </c>
+      <c r="Q88">
+        <v>2026</v>
+      </c>
+      <c r="R88">
+        <v>16962350</v>
+      </c>
+      <c r="S88" t="s">
+        <v>51</v>
+      </c>
+      <c r="U88" t="s">
+        <v>109</v>
+      </c>
+      <c r="V88" s="1">
+        <v>46296.0420403125</v>
+      </c>
+      <c r="W88">
+        <v>-53</v>
+      </c>
+      <c r="X88" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB88">
+        <v>0</v>
+      </c>
+      <c r="AC88" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH88" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI88" t="s">
         <v>151</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-06 15:35
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2990" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="238">
   <si>
     <t>CodCliente</t>
   </si>
@@ -644,6 +644,9 @@
   </si>
   <si>
     <t>Imposto enviado via SCI Report - Data Comentário: 06/10/2026 12:39</t>
+  </si>
+  <si>
+    <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 06/10/2026 - Data Comentário: 05/10/2026 16:53</t>
   </si>
   <si>
     <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1879]. - Data Comentário: 01/10/2026 01:58</t>
@@ -1258,10 +1261,10 @@
         <v>124</v>
       </c>
       <c r="AH2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:35">
@@ -1335,10 +1338,10 @@
         <v>124</v>
       </c>
       <c r="AH3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:35">
@@ -1409,10 +1412,10 @@
         <v>125</v>
       </c>
       <c r="AH4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:35">
@@ -1483,10 +1486,10 @@
         <v>124</v>
       </c>
       <c r="AH5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:35">
@@ -1557,10 +1560,10 @@
         <v>124</v>
       </c>
       <c r="AH6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" spans="1:35">
@@ -1631,10 +1634,10 @@
         <v>126</v>
       </c>
       <c r="AH7" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" spans="1:35">
@@ -1705,10 +1708,10 @@
         <v>125</v>
       </c>
       <c r="AH8" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="1:35">
@@ -1779,10 +1782,10 @@
         <v>127</v>
       </c>
       <c r="AH9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" spans="1:35">
@@ -1853,10 +1856,10 @@
         <v>127</v>
       </c>
       <c r="AH10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:35">
@@ -1930,10 +1933,10 @@
         <v>128</v>
       </c>
       <c r="AH11" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI11" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12" spans="1:35">
@@ -2004,10 +2007,10 @@
         <v>128</v>
       </c>
       <c r="AH12" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="13" spans="1:35">
@@ -2078,10 +2081,10 @@
         <v>129</v>
       </c>
       <c r="AH13" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="14" spans="1:35">
@@ -2152,10 +2155,10 @@
         <v>130</v>
       </c>
       <c r="AH14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI14" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:35">
@@ -2226,10 +2229,10 @@
         <v>130</v>
       </c>
       <c r="AH15" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:35">
@@ -2300,10 +2303,10 @@
         <v>130</v>
       </c>
       <c r="AH16" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI16" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="17" spans="1:35">
@@ -2374,10 +2377,10 @@
         <v>132</v>
       </c>
       <c r="AH17" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="18" spans="1:35">
@@ -2448,10 +2451,10 @@
         <v>132</v>
       </c>
       <c r="AH18" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" spans="1:35">
@@ -2522,10 +2525,10 @@
         <v>131</v>
       </c>
       <c r="AH19" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI19" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" spans="1:35">
@@ -2602,10 +2605,10 @@
         <v>132</v>
       </c>
       <c r="AH20" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI20" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="21" spans="1:35">
@@ -2682,10 +2685,10 @@
         <v>133</v>
       </c>
       <c r="AH21" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI21" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="22" spans="1:35">
@@ -2762,10 +2765,10 @@
         <v>134</v>
       </c>
       <c r="AH22" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI22" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="23" spans="1:35">
@@ -2836,10 +2839,10 @@
         <v>135</v>
       </c>
       <c r="AH23" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI23" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" spans="1:35">
@@ -2916,10 +2919,10 @@
         <v>132</v>
       </c>
       <c r="AH24" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI24" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="25" spans="1:35">
@@ -2996,10 +2999,10 @@
         <v>136</v>
       </c>
       <c r="AH25" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI25" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" spans="1:35">
@@ -3076,10 +3079,10 @@
         <v>132</v>
       </c>
       <c r="AH26" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI26" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="27" spans="1:35">
@@ -3156,10 +3159,10 @@
         <v>132</v>
       </c>
       <c r="AH27" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI27" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="28" spans="1:35">
@@ -3236,10 +3239,10 @@
         <v>132</v>
       </c>
       <c r="AH28" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI28" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="29" spans="1:35">
@@ -3316,10 +3319,10 @@
         <v>131</v>
       </c>
       <c r="AH29" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI29" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="30" spans="1:35">
@@ -3396,10 +3399,10 @@
         <v>137</v>
       </c>
       <c r="AH30" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI30" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="31" spans="1:35">
@@ -3476,10 +3479,10 @@
         <v>133</v>
       </c>
       <c r="AH31" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI31" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="32" spans="1:35">
@@ -3556,10 +3559,10 @@
         <v>134</v>
       </c>
       <c r="AH32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI32" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="33" spans="1:35">
@@ -3636,10 +3639,10 @@
         <v>132</v>
       </c>
       <c r="AH33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI33" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" spans="1:35">
@@ -3716,10 +3719,10 @@
         <v>132</v>
       </c>
       <c r="AH34" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI34" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="35" spans="1:35">
@@ -3796,10 +3799,10 @@
         <v>132</v>
       </c>
       <c r="AH35" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI35" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="36" spans="1:35">
@@ -3870,10 +3873,10 @@
         <v>131</v>
       </c>
       <c r="AH36" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI36" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="37" spans="1:35">
@@ -3944,10 +3947,10 @@
         <v>137</v>
       </c>
       <c r="AH37" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI37" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="38" spans="1:35">
@@ -4018,10 +4021,10 @@
         <v>133</v>
       </c>
       <c r="AH38" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI38" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="39" spans="1:35">
@@ -4092,10 +4095,10 @@
         <v>134</v>
       </c>
       <c r="AH39" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI39" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="40" spans="1:35">
@@ -4166,10 +4169,10 @@
         <v>135</v>
       </c>
       <c r="AH40" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI40" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="41" spans="1:35">
@@ -4246,10 +4249,10 @@
         <v>132</v>
       </c>
       <c r="AH41" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI41" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="42" spans="1:35">
@@ -4326,10 +4329,10 @@
         <v>132</v>
       </c>
       <c r="AH42" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI42" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="43" spans="1:35">
@@ -4406,10 +4409,10 @@
         <v>132</v>
       </c>
       <c r="AH43" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI43" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="44" spans="1:35">
@@ -4486,10 +4489,10 @@
         <v>131</v>
       </c>
       <c r="AH44" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI44" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="45" spans="1:35">
@@ -4566,10 +4569,10 @@
         <v>136</v>
       </c>
       <c r="AH45" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI45" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="46" spans="1:35">
@@ -4646,10 +4649,10 @@
         <v>137</v>
       </c>
       <c r="AH46" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI46" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="47" spans="1:35">
@@ -4726,10 +4729,10 @@
         <v>136</v>
       </c>
       <c r="AH47" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI47" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="48" spans="1:35">
@@ -4806,10 +4809,10 @@
         <v>132</v>
       </c>
       <c r="AH48" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI48" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="49" spans="1:35">
@@ -4886,10 +4889,10 @@
         <v>132</v>
       </c>
       <c r="AH49" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI49" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="50" spans="1:35">
@@ -4966,10 +4969,10 @@
         <v>132</v>
       </c>
       <c r="AH50" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI50" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="51" spans="1:35">
@@ -5040,10 +5043,10 @@
         <v>131</v>
       </c>
       <c r="AH51" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI51" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="52" spans="1:35">
@@ -5120,10 +5123,10 @@
         <v>137</v>
       </c>
       <c r="AH52" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI52" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="53" spans="1:35">
@@ -5200,10 +5203,10 @@
         <v>133</v>
       </c>
       <c r="AH53" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI53" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="54" spans="1:35">
@@ -5280,10 +5283,10 @@
         <v>134</v>
       </c>
       <c r="AH54" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI54" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="55" spans="1:35">
@@ -5360,10 +5363,10 @@
         <v>132</v>
       </c>
       <c r="AH55" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI55" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="56" spans="1:35">
@@ -5440,10 +5443,10 @@
         <v>136</v>
       </c>
       <c r="AH56" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI56" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="57" spans="1:35">
@@ -5520,10 +5523,10 @@
         <v>132</v>
       </c>
       <c r="AH57" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI57" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="58" spans="1:35">
@@ -5600,10 +5603,10 @@
         <v>132</v>
       </c>
       <c r="AH58" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI58" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="59" spans="1:35">
@@ -5680,10 +5683,10 @@
         <v>132</v>
       </c>
       <c r="AH59" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI59" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="60" spans="1:35">
@@ -5754,10 +5757,10 @@
         <v>131</v>
       </c>
       <c r="AH60" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI60" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="61" spans="1:35">
@@ -5834,10 +5837,10 @@
         <v>137</v>
       </c>
       <c r="AH61" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI61" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="62" spans="1:35">
@@ -5914,10 +5917,10 @@
         <v>133</v>
       </c>
       <c r="AH62" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI62" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="63" spans="1:35">
@@ -5994,10 +5997,10 @@
         <v>134</v>
       </c>
       <c r="AH63" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI63" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="64" spans="1:35">
@@ -6068,10 +6071,10 @@
         <v>132</v>
       </c>
       <c r="AH64" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI64" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="65" spans="1:35">
@@ -6142,10 +6145,10 @@
         <v>138</v>
       </c>
       <c r="AH65" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI65" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="66" spans="1:35">
@@ -6216,10 +6219,10 @@
         <v>139</v>
       </c>
       <c r="AH66" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI66" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="67" spans="1:35">
@@ -6290,10 +6293,10 @@
         <v>139</v>
       </c>
       <c r="AH67" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI67" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="68" spans="1:35">
@@ -6364,10 +6367,10 @@
         <v>138</v>
       </c>
       <c r="AH68" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI68" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="69" spans="1:35">
@@ -6438,10 +6441,10 @@
         <v>139</v>
       </c>
       <c r="AH69" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI69" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="70" spans="1:35">
@@ -6512,10 +6515,10 @@
         <v>138</v>
       </c>
       <c r="AH70" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI70" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="71" spans="1:35">
@@ -6586,10 +6589,10 @@
         <v>139</v>
       </c>
       <c r="AH71" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI71" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="72" spans="1:35">
@@ -6660,10 +6663,10 @@
         <v>140</v>
       </c>
       <c r="AH72" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI72" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="73" spans="1:35">
@@ -6734,10 +6737,10 @@
         <v>138</v>
       </c>
       <c r="AH73" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI73" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="74" spans="1:35">
@@ -6808,10 +6811,10 @@
         <v>139</v>
       </c>
       <c r="AH74" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI74" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="75" spans="1:35">
@@ -6882,10 +6885,10 @@
         <v>140</v>
       </c>
       <c r="AH75" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI75" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="76" spans="1:35">
@@ -6956,10 +6959,10 @@
         <v>138</v>
       </c>
       <c r="AH76" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI76" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="77" spans="1:35">
@@ -7030,10 +7033,10 @@
         <v>139</v>
       </c>
       <c r="AH77" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI77" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="78" spans="1:35">
@@ -7104,10 +7107,10 @@
         <v>139</v>
       </c>
       <c r="AH78" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI78" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="79" spans="1:35">
@@ -7178,10 +7181,10 @@
         <v>155</v>
       </c>
       <c r="AH79" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI79" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="80" spans="1:35">
@@ -7252,10 +7255,10 @@
         <v>139</v>
       </c>
       <c r="AH80" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI80" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="81" spans="1:35">
@@ -7326,10 +7329,10 @@
         <v>138</v>
       </c>
       <c r="AH81" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI81" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="82" spans="1:35">
@@ -7400,10 +7403,10 @@
         <v>139</v>
       </c>
       <c r="AH82" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI82" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="83" spans="1:35">
@@ -7474,10 +7477,10 @@
         <v>140</v>
       </c>
       <c r="AH83" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI83" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="84" spans="1:35">
@@ -7548,10 +7551,10 @@
         <v>155</v>
       </c>
       <c r="AH84" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI84" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="85" spans="1:35">
@@ -7622,10 +7625,10 @@
         <v>138</v>
       </c>
       <c r="AH85" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI85" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="86" spans="1:35">
@@ -7696,10 +7699,10 @@
         <v>139</v>
       </c>
       <c r="AH86" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI86" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="87" spans="1:35">
@@ -7770,10 +7773,10 @@
         <v>139</v>
       </c>
       <c r="AH87" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI87" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="88" spans="1:35">
@@ -7844,10 +7847,10 @@
         <v>139</v>
       </c>
       <c r="AH88" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI88" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="89" spans="1:35">
@@ -7918,10 +7921,10 @@
         <v>139</v>
       </c>
       <c r="AH89" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI89" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="90" spans="1:35">
@@ -7992,10 +7995,10 @@
         <v>138</v>
       </c>
       <c r="AH90" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI90" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="91" spans="1:35">
@@ -8066,10 +8069,10 @@
         <v>139</v>
       </c>
       <c r="AH91" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI91" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="92" spans="1:35">
@@ -8140,10 +8143,10 @@
         <v>139</v>
       </c>
       <c r="AH92" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI92" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="93" spans="1:35">
@@ -8214,10 +8217,10 @@
         <v>138</v>
       </c>
       <c r="AH93" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI93" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="94" spans="1:35">
@@ -8288,10 +8291,10 @@
         <v>139</v>
       </c>
       <c r="AH94" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI94" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="95" spans="1:35">
@@ -8362,10 +8365,10 @@
         <v>140</v>
       </c>
       <c r="AH95" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI95" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="96" spans="1:35">
@@ -8436,10 +8439,10 @@
         <v>138</v>
       </c>
       <c r="AH96" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI96" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="97" spans="1:35">
@@ -8510,10 +8513,10 @@
         <v>139</v>
       </c>
       <c r="AH97" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI97" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="98" spans="1:35">
@@ -8584,10 +8587,10 @@
         <v>140</v>
       </c>
       <c r="AH98" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI98" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="99" spans="1:35">
@@ -8664,10 +8667,10 @@
         <v>139</v>
       </c>
       <c r="AH99" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI99" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="100" spans="1:35">
@@ -8741,45 +8744,48 @@
         <v>139</v>
       </c>
       <c r="AH100" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI100" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="101" spans="1:35">
       <c r="A101">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B101" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C101" t="s">
         <v>49</v>
       </c>
       <c r="D101" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E101" t="s">
         <v>54</v>
       </c>
       <c r="F101" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G101">
-        <v>6883</v>
+        <v>1867</v>
       </c>
       <c r="H101">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I101" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J101" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="N101" s="1">
-        <v>46308</v>
+        <v>46304</v>
+      </c>
+      <c r="O101" t="s">
+        <v>121</v>
       </c>
       <c r="P101">
         <v>9</v>
@@ -8788,34 +8794,37 @@
         <v>2026</v>
       </c>
       <c r="R101">
-        <v>17399251</v>
+        <v>18220183</v>
       </c>
       <c r="S101" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="T101" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="U101" t="s">
         <v>158</v>
       </c>
       <c r="V101" s="1">
-        <v>46297.37673402778</v>
+        <v>46301.61803621528</v>
       </c>
       <c r="W101">
-        <v>-7</v>
+        <v>-3</v>
       </c>
       <c r="X101" t="s">
-        <v>166</v>
+        <v>162</v>
+      </c>
+      <c r="Y101" t="s">
+        <v>205</v>
       </c>
       <c r="AB101">
         <v>0</v>
       </c>
       <c r="AC101" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="AH101" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="AI101" t="s">
         <v>236</v>
@@ -8841,7 +8850,7 @@
         <v>55</v>
       </c>
       <c r="G102">
-        <v>1836</v>
+        <v>6883</v>
       </c>
       <c r="H102">
         <v>1788</v>
@@ -8850,10 +8859,10 @@
         <v>61</v>
       </c>
       <c r="J102" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="N102" s="1">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="P102">
         <v>9</v>
@@ -8862,7 +8871,7 @@
         <v>2026</v>
       </c>
       <c r="R102">
-        <v>17398976</v>
+        <v>17399251</v>
       </c>
       <c r="S102" t="s">
         <v>143</v>
@@ -8874,10 +8883,10 @@
         <v>158</v>
       </c>
       <c r="V102" s="1">
-        <v>46297.37618915509</v>
+        <v>46297.37673402778</v>
       </c>
       <c r="W102">
-        <v>1</v>
+        <v>-7</v>
       </c>
       <c r="X102" t="s">
         <v>166</v>
@@ -8889,18 +8898,18 @@
         <v>143</v>
       </c>
       <c r="AH102" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI102" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="103" spans="1:35">
       <c r="A103">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B103" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C103" t="s">
         <v>49</v>
@@ -8936,7 +8945,7 @@
         <v>2026</v>
       </c>
       <c r="R103">
-        <v>18155319</v>
+        <v>17398976</v>
       </c>
       <c r="S103" t="s">
         <v>143</v>
@@ -8948,13 +8957,13 @@
         <v>158</v>
       </c>
       <c r="V103" s="1">
-        <v>46297.66736068287</v>
+        <v>46297.37618915509</v>
       </c>
       <c r="W103">
         <v>1</v>
       </c>
       <c r="X103" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="AB103">
         <v>0</v>
@@ -8963,18 +8972,18 @@
         <v>143</v>
       </c>
       <c r="AH103" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI103" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="104" spans="1:35">
       <c r="A104">
-        <v>6704</v>
+        <v>6486</v>
       </c>
       <c r="B104" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C104" t="s">
         <v>49</v>
@@ -9010,7 +9019,7 @@
         <v>2026</v>
       </c>
       <c r="R104">
-        <v>18085221</v>
+        <v>18155319</v>
       </c>
       <c r="S104" t="s">
         <v>143</v>
@@ -9022,13 +9031,13 @@
         <v>158</v>
       </c>
       <c r="V104" s="1">
-        <v>46297.45935385417</v>
+        <v>46297.66736068287</v>
       </c>
       <c r="W104">
         <v>1</v>
       </c>
       <c r="X104" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AB104">
         <v>0</v>
@@ -9037,18 +9046,18 @@
         <v>143</v>
       </c>
       <c r="AH104" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI104" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="105" spans="1:35">
       <c r="A105">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B105" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C105" t="s">
         <v>49</v>
@@ -9063,7 +9072,7 @@
         <v>55</v>
       </c>
       <c r="G105">
-        <v>6802</v>
+        <v>1836</v>
       </c>
       <c r="H105">
         <v>1788</v>
@@ -9072,7 +9081,7 @@
         <v>61</v>
       </c>
       <c r="J105" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N105" s="1">
         <v>46300</v>
@@ -9084,7 +9093,7 @@
         <v>2026</v>
       </c>
       <c r="R105">
-        <v>17399221</v>
+        <v>18085221</v>
       </c>
       <c r="S105" t="s">
         <v>143</v>
@@ -9096,13 +9105,13 @@
         <v>158</v>
       </c>
       <c r="V105" s="1">
-        <v>46297.37681010416</v>
+        <v>46297.45935385417</v>
       </c>
       <c r="W105">
         <v>1</v>
       </c>
       <c r="X105" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AB105">
         <v>0</v>
@@ -9111,10 +9120,10 @@
         <v>143</v>
       </c>
       <c r="AH105" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI105" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="106" spans="1:35">
@@ -9137,16 +9146,16 @@
         <v>55</v>
       </c>
       <c r="G106">
-        <v>6801</v>
+        <v>6802</v>
       </c>
       <c r="H106">
-        <v>1796</v>
+        <v>1788</v>
       </c>
       <c r="I106" t="s">
         <v>61</v>
       </c>
       <c r="J106" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="N106" s="1">
         <v>46300</v>
@@ -9158,7 +9167,7 @@
         <v>2026</v>
       </c>
       <c r="R106">
-        <v>17399211</v>
+        <v>17399221</v>
       </c>
       <c r="S106" t="s">
         <v>143</v>
@@ -9170,7 +9179,7 @@
         <v>158</v>
       </c>
       <c r="V106" s="1">
-        <v>46297.37686377315</v>
+        <v>46297.37681010416</v>
       </c>
       <c r="W106">
         <v>1</v>
@@ -9185,10 +9194,10 @@
         <v>143</v>
       </c>
       <c r="AH106" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI106" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="107" spans="1:35">
@@ -9211,16 +9220,16 @@
         <v>55</v>
       </c>
       <c r="G107">
-        <v>6014</v>
+        <v>6801</v>
       </c>
       <c r="H107">
-        <v>1788</v>
+        <v>1796</v>
       </c>
       <c r="I107" t="s">
         <v>61</v>
       </c>
       <c r="J107" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="N107" s="1">
         <v>46300</v>
@@ -9232,7 +9241,7 @@
         <v>2026</v>
       </c>
       <c r="R107">
-        <v>17399137</v>
+        <v>17399211</v>
       </c>
       <c r="S107" t="s">
         <v>143</v>
@@ -9244,7 +9253,7 @@
         <v>158</v>
       </c>
       <c r="V107" s="1">
-        <v>46297.37606362269</v>
+        <v>46297.37686377315</v>
       </c>
       <c r="W107">
         <v>1</v>
@@ -9259,18 +9268,18 @@
         <v>143</v>
       </c>
       <c r="AH107" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI107" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="108" spans="1:35">
       <c r="A108">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B108" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C108" t="s">
         <v>49</v>
@@ -9306,7 +9315,7 @@
         <v>2026</v>
       </c>
       <c r="R108">
-        <v>18155328</v>
+        <v>17399137</v>
       </c>
       <c r="S108" t="s">
         <v>143</v>
@@ -9318,13 +9327,13 @@
         <v>158</v>
       </c>
       <c r="V108" s="1">
-        <v>46297.66734447917</v>
+        <v>46297.37606362269</v>
       </c>
       <c r="W108">
         <v>1</v>
       </c>
       <c r="X108" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="AB108">
         <v>0</v>
@@ -9333,18 +9342,18 @@
         <v>143</v>
       </c>
       <c r="AH108" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI108" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="109" spans="1:35">
       <c r="A109">
-        <v>6704</v>
+        <v>6486</v>
       </c>
       <c r="B109" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C109" t="s">
         <v>49</v>
@@ -9380,7 +9389,7 @@
         <v>2026</v>
       </c>
       <c r="R109">
-        <v>18085232</v>
+        <v>18155328</v>
       </c>
       <c r="S109" t="s">
         <v>143</v>
@@ -9392,13 +9401,13 @@
         <v>158</v>
       </c>
       <c r="V109" s="1">
-        <v>46297.45929016203</v>
+        <v>46297.66734447917</v>
       </c>
       <c r="W109">
         <v>1</v>
       </c>
       <c r="X109" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AB109">
         <v>0</v>
@@ -9407,18 +9416,18 @@
         <v>143</v>
       </c>
       <c r="AH109" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI109" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="110" spans="1:35">
       <c r="A110">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B110" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C110" t="s">
         <v>49</v>
@@ -9433,16 +9442,16 @@
         <v>55</v>
       </c>
       <c r="G110">
-        <v>6233</v>
+        <v>6014</v>
       </c>
       <c r="H110">
-        <v>6232</v>
+        <v>1788</v>
       </c>
       <c r="I110" t="s">
         <v>61</v>
       </c>
       <c r="J110" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N110" s="1">
         <v>46300</v>
@@ -9454,7 +9463,7 @@
         <v>2026</v>
       </c>
       <c r="R110">
-        <v>17399177</v>
+        <v>18085232</v>
       </c>
       <c r="S110" t="s">
         <v>143</v>
@@ -9466,13 +9475,13 @@
         <v>158</v>
       </c>
       <c r="V110" s="1">
-        <v>46297.37537966435</v>
+        <v>46297.45929016203</v>
       </c>
       <c r="W110">
         <v>1</v>
       </c>
       <c r="X110" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AB110">
         <v>0</v>
@@ -9481,24 +9490,24 @@
         <v>143</v>
       </c>
       <c r="AH110" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI110" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="111" spans="1:35">
       <c r="A111">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B111" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C111" t="s">
         <v>49</v>
       </c>
       <c r="D111" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E111" t="s">
         <v>54</v>
@@ -9528,7 +9537,7 @@
         <v>2026</v>
       </c>
       <c r="R111">
-        <v>16962295</v>
+        <v>17399177</v>
       </c>
       <c r="S111" t="s">
         <v>143</v>
@@ -9540,13 +9549,13 @@
         <v>158</v>
       </c>
       <c r="V111" s="1">
-        <v>46297.45869950231</v>
+        <v>46297.37537966435</v>
       </c>
       <c r="W111">
         <v>1</v>
       </c>
       <c r="X111" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AB111">
         <v>0</v>
@@ -9555,24 +9564,24 @@
         <v>143</v>
       </c>
       <c r="AH111" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI111" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="112" spans="1:35">
       <c r="A112">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B112" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C112" t="s">
         <v>49</v>
       </c>
       <c r="D112" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E112" t="s">
         <v>54</v>
@@ -9602,7 +9611,7 @@
         <v>2026</v>
       </c>
       <c r="R112">
-        <v>16976157</v>
+        <v>16962295</v>
       </c>
       <c r="S112" t="s">
         <v>143</v>
@@ -9611,16 +9620,16 @@
         <v>156</v>
       </c>
       <c r="U112" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="V112" s="1">
-        <v>46300.66721489583</v>
+        <v>46297.45869950231</v>
       </c>
       <c r="W112">
         <v>1</v>
       </c>
       <c r="X112" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AB112">
         <v>0</v>
@@ -9629,24 +9638,24 @@
         <v>143</v>
       </c>
       <c r="AH112" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI112" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="113" spans="1:35">
       <c r="A113">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B113" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C113" t="s">
         <v>49</v>
       </c>
       <c r="D113" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E113" t="s">
         <v>54</v>
@@ -9676,7 +9685,7 @@
         <v>2026</v>
       </c>
       <c r="R113">
-        <v>17948845</v>
+        <v>16976157</v>
       </c>
       <c r="S113" t="s">
         <v>143</v>
@@ -9685,16 +9694,16 @@
         <v>156</v>
       </c>
       <c r="U113" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="V113" s="1">
-        <v>46297.45870309028</v>
+        <v>46300.66721489583</v>
       </c>
       <c r="W113">
         <v>1</v>
       </c>
       <c r="X113" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AB113">
         <v>0</v>
@@ -9703,7 +9712,7 @@
         <v>143</v>
       </c>
       <c r="AH113" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI113" t="s">
         <v>236</v>
@@ -9711,16 +9720,16 @@
     </row>
     <row r="114" spans="1:35">
       <c r="A114">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B114" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C114" t="s">
         <v>49</v>
       </c>
       <c r="D114" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E114" t="s">
         <v>54</v>
@@ -9750,7 +9759,7 @@
         <v>2026</v>
       </c>
       <c r="R114">
-        <v>18085265</v>
+        <v>17948845</v>
       </c>
       <c r="S114" t="s">
         <v>143</v>
@@ -9762,13 +9771,13 @@
         <v>158</v>
       </c>
       <c r="V114" s="1">
-        <v>46297.45870405093</v>
+        <v>46297.45870309028</v>
       </c>
       <c r="W114">
         <v>1</v>
       </c>
       <c r="X114" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="AB114">
         <v>0</v>
@@ -9777,24 +9786,24 @@
         <v>143</v>
       </c>
       <c r="AH114" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI114" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="115" spans="1:35">
       <c r="A115">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B115" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C115" t="s">
         <v>49</v>
       </c>
       <c r="D115" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E115" t="s">
         <v>54</v>
@@ -9824,7 +9833,7 @@
         <v>2026</v>
       </c>
       <c r="R115">
-        <v>17948990</v>
+        <v>18085265</v>
       </c>
       <c r="S115" t="s">
         <v>143</v>
@@ -9836,7 +9845,7 @@
         <v>158</v>
       </c>
       <c r="V115" s="1">
-        <v>46297.45870177083</v>
+        <v>46297.45870405093</v>
       </c>
       <c r="W115">
         <v>1</v>
@@ -9851,24 +9860,24 @@
         <v>143</v>
       </c>
       <c r="AH115" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI115" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="116" spans="1:35">
       <c r="A116">
-        <v>5417</v>
+        <v>6705</v>
       </c>
       <c r="B116" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C116" t="s">
         <v>49</v>
       </c>
       <c r="D116" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E116" t="s">
         <v>54</v>
@@ -9877,16 +9886,16 @@
         <v>55</v>
       </c>
       <c r="G116">
-        <v>6230</v>
+        <v>6233</v>
       </c>
       <c r="H116">
-        <v>9114</v>
+        <v>6232</v>
       </c>
       <c r="I116" t="s">
         <v>61</v>
       </c>
       <c r="J116" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="N116" s="1">
         <v>46300</v>
@@ -9898,7 +9907,7 @@
         <v>2026</v>
       </c>
       <c r="R116">
-        <v>17399157</v>
+        <v>17948990</v>
       </c>
       <c r="S116" t="s">
         <v>143</v>
@@ -9907,16 +9916,16 @@
         <v>156</v>
       </c>
       <c r="U116" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="V116" s="1">
-        <v>46300.65013206018</v>
+        <v>46297.45870177083</v>
       </c>
       <c r="W116">
         <v>1</v>
       </c>
       <c r="X116" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AB116">
         <v>0</v>
@@ -9925,24 +9934,24 @@
         <v>143</v>
       </c>
       <c r="AH116" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI116" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="117" spans="1:35">
       <c r="A117">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B117" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C117" t="s">
         <v>49</v>
       </c>
       <c r="D117" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E117" t="s">
         <v>54</v>
@@ -9972,7 +9981,7 @@
         <v>2026</v>
       </c>
       <c r="R117">
-        <v>16962275</v>
+        <v>17399157</v>
       </c>
       <c r="S117" t="s">
         <v>143</v>
@@ -9984,13 +9993,13 @@
         <v>159</v>
       </c>
       <c r="V117" s="1">
-        <v>46300.65011049769</v>
+        <v>46300.65013206018</v>
       </c>
       <c r="W117">
         <v>1</v>
       </c>
       <c r="X117" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AB117">
         <v>0</v>
@@ -9999,24 +10008,24 @@
         <v>143</v>
       </c>
       <c r="AH117" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI117" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="118" spans="1:35">
       <c r="A118">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B118" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C118" t="s">
         <v>49</v>
       </c>
       <c r="D118" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E118" t="s">
         <v>54</v>
@@ -10046,7 +10055,7 @@
         <v>2026</v>
       </c>
       <c r="R118">
-        <v>16976137</v>
+        <v>16962275</v>
       </c>
       <c r="S118" t="s">
         <v>143</v>
@@ -10058,13 +10067,13 @@
         <v>159</v>
       </c>
       <c r="V118" s="1">
-        <v>46300.66713765046</v>
+        <v>46300.65011049769</v>
       </c>
       <c r="W118">
         <v>1</v>
       </c>
       <c r="X118" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AB118">
         <v>0</v>
@@ -10073,24 +10082,24 @@
         <v>143</v>
       </c>
       <c r="AH118" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI118" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="119" spans="1:35">
       <c r="A119">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B119" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C119" t="s">
         <v>49</v>
       </c>
       <c r="D119" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E119" t="s">
         <v>54</v>
@@ -10120,7 +10129,7 @@
         <v>2026</v>
       </c>
       <c r="R119">
-        <v>17948825</v>
+        <v>16976137</v>
       </c>
       <c r="S119" t="s">
         <v>143</v>
@@ -10132,13 +10141,13 @@
         <v>159</v>
       </c>
       <c r="V119" s="1">
-        <v>46300.66713784722</v>
+        <v>46300.66713765046</v>
       </c>
       <c r="W119">
         <v>1</v>
       </c>
       <c r="X119" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AB119">
         <v>0</v>
@@ -10147,24 +10156,24 @@
         <v>143</v>
       </c>
       <c r="AH119" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI119" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="120" spans="1:35">
       <c r="A120">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B120" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C120" t="s">
         <v>49</v>
       </c>
       <c r="D120" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E120" t="s">
         <v>54</v>
@@ -10194,7 +10203,7 @@
         <v>2026</v>
       </c>
       <c r="R120">
-        <v>18085243</v>
+        <v>17948825</v>
       </c>
       <c r="S120" t="s">
         <v>143</v>
@@ -10206,13 +10215,13 @@
         <v>159</v>
       </c>
       <c r="V120" s="1">
-        <v>46300.66713822917</v>
+        <v>46300.66713784722</v>
       </c>
       <c r="W120">
         <v>1</v>
       </c>
       <c r="X120" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="AB120">
         <v>0</v>
@@ -10221,24 +10230,24 @@
         <v>143</v>
       </c>
       <c r="AH120" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI120" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="121" spans="1:35">
       <c r="A121">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B121" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C121" t="s">
         <v>49</v>
       </c>
       <c r="D121" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E121" t="s">
         <v>54</v>
@@ -10268,7 +10277,7 @@
         <v>2026</v>
       </c>
       <c r="R121">
-        <v>17948970</v>
+        <v>18085243</v>
       </c>
       <c r="S121" t="s">
         <v>143</v>
@@ -10280,7 +10289,7 @@
         <v>159</v>
       </c>
       <c r="V121" s="1">
-        <v>46300.75530894676</v>
+        <v>46300.66713822917</v>
       </c>
       <c r="W121">
         <v>1</v>
@@ -10295,24 +10304,24 @@
         <v>143</v>
       </c>
       <c r="AH121" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI121" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="122" spans="1:35">
       <c r="A122">
-        <v>6486</v>
+        <v>6705</v>
       </c>
       <c r="B122" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C122" t="s">
         <v>49</v>
       </c>
       <c r="D122" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E122" t="s">
         <v>54</v>
@@ -10321,19 +10330,19 @@
         <v>55</v>
       </c>
       <c r="G122">
-        <v>11359</v>
+        <v>6230</v>
       </c>
       <c r="H122">
-        <v>0</v>
+        <v>9114</v>
       </c>
       <c r="I122" t="s">
         <v>61</v>
       </c>
       <c r="J122" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="N122" s="1">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="P122">
         <v>9</v>
@@ -10342,7 +10351,7 @@
         <v>2026</v>
       </c>
       <c r="R122">
-        <v>18155346</v>
+        <v>17948970</v>
       </c>
       <c r="S122" t="s">
         <v>143</v>
@@ -10354,13 +10363,13 @@
         <v>159</v>
       </c>
       <c r="V122" s="1">
-        <v>46297.66734765047</v>
+        <v>46300.75530894676</v>
       </c>
       <c r="W122">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X122" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AB122">
         <v>0</v>
@@ -10369,7 +10378,7 @@
         <v>143</v>
       </c>
       <c r="AH122" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI122" t="s">
         <v>236</v>
@@ -10377,37 +10386,37 @@
     </row>
     <row r="123" spans="1:35">
       <c r="A123">
-        <v>6628</v>
+        <v>6486</v>
       </c>
       <c r="B123" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C123" t="s">
         <v>49</v>
       </c>
       <c r="D123" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E123" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F123" t="s">
         <v>55</v>
       </c>
       <c r="G123">
-        <v>945</v>
+        <v>11359</v>
       </c>
       <c r="H123">
         <v>0</v>
       </c>
       <c r="I123" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J123" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N123" s="1">
-        <v>46315</v>
+        <v>46297</v>
       </c>
       <c r="P123">
         <v>9</v>
@@ -10416,45 +10425,45 @@
         <v>2026</v>
       </c>
       <c r="R123">
-        <v>16959939</v>
+        <v>18155346</v>
       </c>
       <c r="S123" t="s">
-        <v>144</v>
+        <v>143</v>
+      </c>
+      <c r="T123" t="s">
+        <v>156</v>
       </c>
       <c r="U123" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="V123" s="1">
-        <v>46296.08337256945</v>
+        <v>46297.66734765047</v>
       </c>
       <c r="W123">
-        <v>-14</v>
+        <v>4</v>
       </c>
       <c r="X123" t="s">
-        <v>160</v>
-      </c>
-      <c r="Y123" t="s">
-        <v>205</v>
+        <v>168</v>
       </c>
       <c r="AB123">
         <v>0</v>
       </c>
       <c r="AC123" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AH123" t="s">
         <v>233</v>
       </c>
       <c r="AI123" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="124" spans="1:35">
       <c r="A124">
-        <v>6779</v>
+        <v>6628</v>
       </c>
       <c r="B124" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C124" t="s">
         <v>49</v>
@@ -10463,7 +10472,7 @@
         <v>51</v>
       </c>
       <c r="E124" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F124" t="s">
         <v>55</v>
@@ -10490,7 +10499,7 @@
         <v>2026</v>
       </c>
       <c r="R124">
-        <v>18056696</v>
+        <v>16959939</v>
       </c>
       <c r="S124" t="s">
         <v>144</v>
@@ -10499,13 +10508,13 @@
         <v>158</v>
       </c>
       <c r="V124" s="1">
-        <v>46296.0834071412</v>
+        <v>46296.08337256945</v>
       </c>
       <c r="W124">
         <v>-14</v>
       </c>
       <c r="X124" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="Y124" t="s">
         <v>206</v>
@@ -10517,18 +10526,18 @@
         <v>144</v>
       </c>
       <c r="AH124" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI124" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="125" spans="1:35">
       <c r="A125">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B125" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C125" t="s">
         <v>49</v>
@@ -10540,7 +10549,7 @@
         <v>54</v>
       </c>
       <c r="F125" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G125">
         <v>945</v>
@@ -10564,7 +10573,7 @@
         <v>2026</v>
       </c>
       <c r="R125">
-        <v>18164488</v>
+        <v>18056696</v>
       </c>
       <c r="S125" t="s">
         <v>144</v>
@@ -10573,16 +10582,16 @@
         <v>158</v>
       </c>
       <c r="V125" s="1">
-        <v>46296.08341825232</v>
+        <v>46296.0834071412</v>
       </c>
       <c r="W125">
         <v>-14</v>
       </c>
       <c r="X125" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="Y125" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="AB125">
         <v>0</v>
@@ -10591,33 +10600,33 @@
         <v>144</v>
       </c>
       <c r="AH125" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI125" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="126" spans="1:35">
       <c r="A126">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B126" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C126" t="s">
         <v>49</v>
       </c>
       <c r="D126" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E126" t="s">
         <v>54</v>
       </c>
       <c r="F126" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G126">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H126">
         <v>0</v>
@@ -10626,7 +10635,7 @@
         <v>62</v>
       </c>
       <c r="J126" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="N126" s="1">
         <v>46315</v>
@@ -10638,7 +10647,7 @@
         <v>2026</v>
       </c>
       <c r="R126">
-        <v>17398870</v>
+        <v>18164488</v>
       </c>
       <c r="S126" t="s">
         <v>144</v>
@@ -10647,16 +10656,16 @@
         <v>158</v>
       </c>
       <c r="V126" s="1">
-        <v>46296.37558109954</v>
+        <v>46296.08341825232</v>
       </c>
       <c r="W126">
         <v>-14</v>
       </c>
       <c r="X126" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="Y126" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AB126">
         <v>0</v>
@@ -10665,24 +10674,24 @@
         <v>144</v>
       </c>
       <c r="AH126" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI126" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="127" spans="1:35">
       <c r="A127">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B127" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C127" t="s">
         <v>49</v>
       </c>
       <c r="D127" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E127" t="s">
         <v>54</v>
@@ -10712,7 +10721,7 @@
         <v>2026</v>
       </c>
       <c r="R127">
-        <v>16962094</v>
+        <v>17398870</v>
       </c>
       <c r="S127" t="s">
         <v>144</v>
@@ -10721,13 +10730,13 @@
         <v>158</v>
       </c>
       <c r="V127" s="1">
-        <v>46296.37504012731</v>
+        <v>46296.37558109954</v>
       </c>
       <c r="W127">
         <v>-14</v>
       </c>
       <c r="X127" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="Y127" t="s">
         <v>208</v>
@@ -10739,18 +10748,18 @@
         <v>144</v>
       </c>
       <c r="AH127" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI127" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="128" spans="1:35">
       <c r="A128">
-        <v>6703</v>
+        <v>6404</v>
       </c>
       <c r="B128" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C128" t="s">
         <v>49</v>
@@ -10786,22 +10795,22 @@
         <v>2026</v>
       </c>
       <c r="R128">
-        <v>17941133</v>
+        <v>16962094</v>
       </c>
       <c r="S128" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="U128" t="s">
         <v>158</v>
       </c>
       <c r="V128" s="1">
-        <v>46296.3760846412</v>
+        <v>46296.37504012731</v>
       </c>
       <c r="W128">
         <v>-14</v>
       </c>
       <c r="X128" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Y128" t="s">
         <v>209</v>
@@ -10810,27 +10819,27 @@
         <v>0</v>
       </c>
       <c r="AC128" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AH128" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI128" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="129" spans="1:35">
       <c r="A129">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B129" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C129" t="s">
         <v>49</v>
       </c>
       <c r="D129" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E129" t="s">
         <v>54</v>
@@ -10839,7 +10848,7 @@
         <v>55</v>
       </c>
       <c r="G129">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="H129">
         <v>0</v>
@@ -10848,10 +10857,10 @@
         <v>62</v>
       </c>
       <c r="J129" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="N129" s="1">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="P129">
         <v>9</v>
@@ -10860,22 +10869,22 @@
         <v>2026</v>
       </c>
       <c r="R129">
-        <v>17398876</v>
+        <v>17941133</v>
       </c>
       <c r="S129" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="U129" t="s">
         <v>158</v>
       </c>
       <c r="V129" s="1">
-        <v>46296.37648518519</v>
+        <v>46296.3760846412</v>
       </c>
       <c r="W129">
-        <v>-24</v>
+        <v>-14</v>
       </c>
       <c r="X129" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="Y129" t="s">
         <v>210</v>
@@ -10884,21 +10893,21 @@
         <v>0</v>
       </c>
       <c r="AC129" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AH129" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI129" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="130" spans="1:35">
       <c r="A130">
-        <v>6627</v>
+        <v>5417</v>
       </c>
       <c r="B130" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C130" t="s">
         <v>49</v>
@@ -10907,7 +10916,7 @@
         <v>50</v>
       </c>
       <c r="E130" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F130" t="s">
         <v>55</v>
@@ -10934,7 +10943,7 @@
         <v>2026</v>
       </c>
       <c r="R130">
-        <v>17042296</v>
+        <v>17398876</v>
       </c>
       <c r="S130" t="s">
         <v>144</v>
@@ -10943,13 +10952,13 @@
         <v>158</v>
       </c>
       <c r="V130" s="1">
-        <v>46296.37615983796</v>
+        <v>46296.37648518519</v>
       </c>
       <c r="W130">
         <v>-24</v>
       </c>
       <c r="X130" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="Y130" t="s">
         <v>211</v>
@@ -10961,18 +10970,18 @@
         <v>144</v>
       </c>
       <c r="AH130" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI130" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="131" spans="1:35">
       <c r="A131">
-        <v>6704</v>
+        <v>6627</v>
       </c>
       <c r="B131" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C131" t="s">
         <v>49</v>
@@ -10981,7 +10990,7 @@
         <v>50</v>
       </c>
       <c r="E131" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F131" t="s">
         <v>55</v>
@@ -11008,7 +11017,7 @@
         <v>2026</v>
       </c>
       <c r="R131">
-        <v>17952332</v>
+        <v>17042296</v>
       </c>
       <c r="S131" t="s">
         <v>144</v>
@@ -11017,16 +11026,16 @@
         <v>158</v>
       </c>
       <c r="V131" s="1">
-        <v>46296.37684290509</v>
+        <v>46296.37615983796</v>
       </c>
       <c r="W131">
         <v>-24</v>
       </c>
       <c r="X131" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="Y131" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="AB131">
         <v>0</v>
@@ -11035,24 +11044,24 @@
         <v>144</v>
       </c>
       <c r="AH131" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI131" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="132" spans="1:35">
       <c r="A132">
-        <v>6404</v>
+        <v>6704</v>
       </c>
       <c r="B132" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C132" t="s">
         <v>49</v>
       </c>
       <c r="D132" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E132" t="s">
         <v>54</v>
@@ -11061,7 +11070,7 @@
         <v>55</v>
       </c>
       <c r="G132">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="H132">
         <v>0</v>
@@ -11070,7 +11079,7 @@
         <v>62</v>
       </c>
       <c r="J132" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N132" s="1">
         <v>46325</v>
@@ -11082,7 +11091,7 @@
         <v>2026</v>
       </c>
       <c r="R132">
-        <v>16962100</v>
+        <v>17952332</v>
       </c>
       <c r="S132" t="s">
         <v>144</v>
@@ -11091,16 +11100,16 @@
         <v>158</v>
       </c>
       <c r="V132" s="1">
-        <v>46296.37609667824</v>
+        <v>46296.37684290509</v>
       </c>
       <c r="W132">
         <v>-24</v>
       </c>
       <c r="X132" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="Y132" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AB132">
         <v>0</v>
@@ -11109,18 +11118,18 @@
         <v>144</v>
       </c>
       <c r="AH132" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI132" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="133" spans="1:35">
       <c r="A133">
-        <v>6703</v>
+        <v>6404</v>
       </c>
       <c r="B133" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C133" t="s">
         <v>49</v>
@@ -11156,22 +11165,22 @@
         <v>2026</v>
       </c>
       <c r="R133">
-        <v>17941139</v>
+        <v>16962100</v>
       </c>
       <c r="S133" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="U133" t="s">
         <v>158</v>
       </c>
       <c r="V133" s="1">
-        <v>46296.37683961805</v>
+        <v>46296.37609667824</v>
       </c>
       <c r="W133">
         <v>-24</v>
       </c>
       <c r="X133" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Y133" t="s">
         <v>213</v>
@@ -11180,13 +11189,13 @@
         <v>0</v>
       </c>
       <c r="AC133" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AH133" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI133" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="134" spans="1:35">
@@ -11209,7 +11218,7 @@
         <v>55</v>
       </c>
       <c r="G134">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="H134">
         <v>0</v>
@@ -11218,10 +11227,10 @@
         <v>62</v>
       </c>
       <c r="J134" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N134" s="1">
-        <v>46304</v>
+        <v>46325</v>
       </c>
       <c r="P134">
         <v>9</v>
@@ -11230,7 +11239,7 @@
         <v>2026</v>
       </c>
       <c r="R134">
-        <v>17941147</v>
+        <v>17941139</v>
       </c>
       <c r="S134" t="s">
         <v>145</v>
@@ -11239,10 +11248,10 @@
         <v>158</v>
       </c>
       <c r="V134" s="1">
-        <v>46296.37684039352</v>
+        <v>46296.37683961805</v>
       </c>
       <c r="W134">
-        <v>-3</v>
+        <v>-24</v>
       </c>
       <c r="X134" t="s">
         <v>169</v>
@@ -11257,30 +11266,30 @@
         <v>145</v>
       </c>
       <c r="AH134" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI134" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="135" spans="1:35">
       <c r="A135">
-        <v>6949</v>
+        <v>6703</v>
       </c>
       <c r="B135" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C135" t="s">
         <v>49</v>
       </c>
       <c r="D135" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E135" t="s">
         <v>54</v>
       </c>
       <c r="F135" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G135">
         <v>950</v>
@@ -11304,22 +11313,22 @@
         <v>2026</v>
       </c>
       <c r="R135">
-        <v>18178133</v>
+        <v>17941147</v>
       </c>
       <c r="S135" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="U135" t="s">
         <v>158</v>
       </c>
       <c r="V135" s="1">
-        <v>46296.37697557871</v>
+        <v>46296.37684039352</v>
       </c>
       <c r="W135">
         <v>-3</v>
       </c>
       <c r="X135" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="Y135" t="s">
         <v>215</v>
@@ -11328,21 +11337,21 @@
         <v>0</v>
       </c>
       <c r="AC135" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AH135" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI135" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="136" spans="1:35">
       <c r="A136">
-        <v>6548</v>
+        <v>6949</v>
       </c>
       <c r="B136" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C136" t="s">
         <v>49</v>
@@ -11354,10 +11363,10 @@
         <v>54</v>
       </c>
       <c r="F136" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G136">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H136">
         <v>0</v>
@@ -11366,7 +11375,7 @@
         <v>62</v>
       </c>
       <c r="J136" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N136" s="1">
         <v>46304</v>
@@ -11378,7 +11387,7 @@
         <v>2026</v>
       </c>
       <c r="R136">
-        <v>17222406</v>
+        <v>18178133</v>
       </c>
       <c r="S136" t="s">
         <v>144</v>
@@ -11387,13 +11396,13 @@
         <v>158</v>
       </c>
       <c r="V136" s="1">
-        <v>46296.37726273148</v>
+        <v>46296.37697557871</v>
       </c>
       <c r="W136">
         <v>-3</v>
       </c>
       <c r="X136" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="Y136" t="s">
         <v>216</v>
@@ -11405,24 +11414,24 @@
         <v>144</v>
       </c>
       <c r="AH136" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI136" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="137" spans="1:35">
       <c r="A137">
-        <v>6703</v>
+        <v>6548</v>
       </c>
       <c r="B137" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C137" t="s">
         <v>49</v>
       </c>
       <c r="D137" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E137" t="s">
         <v>54</v>
@@ -11452,22 +11461,22 @@
         <v>2026</v>
       </c>
       <c r="R137">
-        <v>17941157</v>
+        <v>17222406</v>
       </c>
       <c r="S137" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="U137" t="s">
         <v>158</v>
       </c>
       <c r="V137" s="1">
-        <v>46296.37814100694</v>
+        <v>46296.37726273148</v>
       </c>
       <c r="W137">
         <v>-3</v>
       </c>
       <c r="X137" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="Y137" t="s">
         <v>217</v>
@@ -11476,27 +11485,27 @@
         <v>0</v>
       </c>
       <c r="AC137" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AH137" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI137" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="138" spans="1:35">
       <c r="A138">
-        <v>6779</v>
+        <v>6703</v>
       </c>
       <c r="B138" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C138" t="s">
         <v>49</v>
       </c>
       <c r="D138" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E138" t="s">
         <v>54</v>
@@ -11526,45 +11535,45 @@
         <v>2026</v>
       </c>
       <c r="R138">
-        <v>18056706</v>
+        <v>17941157</v>
       </c>
       <c r="S138" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="U138" t="s">
         <v>158</v>
       </c>
       <c r="V138" s="1">
-        <v>46296.37816597222</v>
+        <v>46296.37814100694</v>
       </c>
       <c r="W138">
         <v>-3</v>
       </c>
       <c r="X138" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="Y138" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB138">
         <v>0</v>
       </c>
       <c r="AC138" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AH138" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI138" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="139" spans="1:35">
       <c r="A139">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B139" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C139" t="s">
         <v>49</v>
@@ -11576,7 +11585,7 @@
         <v>54</v>
       </c>
       <c r="F139" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G139">
         <v>951</v>
@@ -11600,7 +11609,7 @@
         <v>2026</v>
       </c>
       <c r="R139">
-        <v>18164502</v>
+        <v>18056706</v>
       </c>
       <c r="S139" t="s">
         <v>144</v>
@@ -11609,13 +11618,13 @@
         <v>158</v>
       </c>
       <c r="V139" s="1">
-        <v>46296.3782184838</v>
+        <v>46296.37816597222</v>
       </c>
       <c r="W139">
         <v>-3</v>
       </c>
       <c r="X139" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="Y139" t="s">
         <v>218</v>
@@ -11627,10 +11636,10 @@
         <v>144</v>
       </c>
       <c r="AH139" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI139" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="140" spans="1:35">
@@ -11692,7 +11701,7 @@
         <v>163</v>
       </c>
       <c r="Y140" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AB140">
         <v>0</v>
@@ -11701,10 +11710,10 @@
         <v>144</v>
       </c>
       <c r="AH140" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI140" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="141" spans="1:35">
@@ -11766,7 +11775,7 @@
         <v>166</v>
       </c>
       <c r="Y141" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AB141">
         <v>0</v>
@@ -11775,10 +11784,10 @@
         <v>144</v>
       </c>
       <c r="AH141" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI141" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="142" spans="1:35">
@@ -11840,7 +11849,7 @@
         <v>165</v>
       </c>
       <c r="Y142" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AB142">
         <v>0</v>
@@ -11849,10 +11858,10 @@
         <v>144</v>
       </c>
       <c r="AH142" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI142" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="143" spans="1:35">
@@ -11914,7 +11923,7 @@
         <v>160</v>
       </c>
       <c r="Y143" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AB143">
         <v>0</v>
@@ -11923,10 +11932,10 @@
         <v>144</v>
       </c>
       <c r="AH143" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI143" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="144" spans="1:35">
@@ -11988,7 +11997,7 @@
         <v>169</v>
       </c>
       <c r="Y144" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AB144">
         <v>0</v>
@@ -11997,10 +12006,10 @@
         <v>145</v>
       </c>
       <c r="AH144" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI144" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="145" spans="1:35">
@@ -12062,7 +12071,7 @@
         <v>163</v>
       </c>
       <c r="Y145" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AB145">
         <v>0</v>
@@ -12071,10 +12080,10 @@
         <v>144</v>
       </c>
       <c r="AH145" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI145" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="146" spans="1:35">
@@ -12142,10 +12151,10 @@
         <v>144</v>
       </c>
       <c r="AH146" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI146" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="147" spans="1:35">
@@ -12213,10 +12222,10 @@
         <v>144</v>
       </c>
       <c r="AH147" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI147" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="148" spans="1:35">
@@ -12284,10 +12293,10 @@
         <v>144</v>
       </c>
       <c r="AH148" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI148" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="149" spans="1:35">
@@ -12355,10 +12364,10 @@
         <v>144</v>
       </c>
       <c r="AH149" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI149" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="150" spans="1:35">
@@ -12426,10 +12435,10 @@
         <v>144</v>
       </c>
       <c r="AH150" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI150" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="151" spans="1:35">
@@ -12497,10 +12506,10 @@
         <v>144</v>
       </c>
       <c r="AH151" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI151" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="152" spans="1:35">
@@ -12568,10 +12577,10 @@
         <v>145</v>
       </c>
       <c r="AH152" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI152" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="153" spans="1:35">
@@ -12639,10 +12648,10 @@
         <v>144</v>
       </c>
       <c r="AH153" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI153" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="154" spans="1:35">
@@ -12710,10 +12719,10 @@
         <v>144</v>
       </c>
       <c r="AH154" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI154" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="155" spans="1:35">
@@ -12781,10 +12790,10 @@
         <v>144</v>
       </c>
       <c r="AH155" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI155" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="156" spans="1:35">
@@ -12852,10 +12861,10 @@
         <v>144</v>
       </c>
       <c r="AH156" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI156" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="157" spans="1:35">
@@ -12923,10 +12932,10 @@
         <v>144</v>
       </c>
       <c r="AH157" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI157" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="158" spans="1:35">
@@ -12994,10 +13003,10 @@
         <v>144</v>
       </c>
       <c r="AH158" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI158" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="159" spans="1:35">
@@ -13065,10 +13074,10 @@
         <v>144</v>
       </c>
       <c r="AH159" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI159" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="160" spans="1:35">
@@ -13133,7 +13142,7 @@
         <v>166</v>
       </c>
       <c r="Y160" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB160">
         <v>0</v>
@@ -13142,10 +13151,10 @@
         <v>144</v>
       </c>
       <c r="AH160" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI160" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="161" spans="1:35">
@@ -13210,7 +13219,7 @@
         <v>165</v>
       </c>
       <c r="Y161" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB161">
         <v>0</v>
@@ -13219,10 +13228,10 @@
         <v>144</v>
       </c>
       <c r="AH161" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI161" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="162" spans="1:35">
@@ -13287,7 +13296,7 @@
         <v>168</v>
       </c>
       <c r="Y162" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB162">
         <v>0</v>
@@ -13296,10 +13305,10 @@
         <v>144</v>
       </c>
       <c r="AH162" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI162" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="163" spans="1:35">
@@ -13364,7 +13373,7 @@
         <v>161</v>
       </c>
       <c r="Y163" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB163">
         <v>0</v>
@@ -13373,10 +13382,10 @@
         <v>144</v>
       </c>
       <c r="AH163" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI163" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="164" spans="1:35">
@@ -13441,7 +13450,7 @@
         <v>160</v>
       </c>
       <c r="Y164" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB164">
         <v>0</v>
@@ -13450,10 +13459,10 @@
         <v>144</v>
       </c>
       <c r="AH164" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI164" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="165" spans="1:35">
@@ -13518,7 +13527,7 @@
         <v>160</v>
       </c>
       <c r="Y165" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB165">
         <v>0</v>
@@ -13527,10 +13536,10 @@
         <v>144</v>
       </c>
       <c r="AH165" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI165" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="166" spans="1:35">
@@ -13595,7 +13604,7 @@
         <v>169</v>
       </c>
       <c r="Y166" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB166">
         <v>0</v>
@@ -13604,10 +13613,10 @@
         <v>145</v>
       </c>
       <c r="AH166" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI166" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="167" spans="1:35">
@@ -13672,7 +13681,7 @@
         <v>167</v>
       </c>
       <c r="Y167" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AB167">
         <v>0</v>
@@ -13681,10 +13690,10 @@
         <v>144</v>
       </c>
       <c r="AH167" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI167" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="168" spans="1:35">
@@ -13749,7 +13758,7 @@
         <v>167</v>
       </c>
       <c r="Y168" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB168">
         <v>0</v>
@@ -13758,10 +13767,10 @@
         <v>144</v>
       </c>
       <c r="AH168" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI168" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="169" spans="1:35">
@@ -13826,7 +13835,7 @@
         <v>162</v>
       </c>
       <c r="Y169" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB169">
         <v>0</v>
@@ -13835,10 +13844,10 @@
         <v>144</v>
       </c>
       <c r="AH169" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI169" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="170" spans="1:35">
@@ -13903,7 +13912,7 @@
         <v>163</v>
       </c>
       <c r="Y170" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AB170">
         <v>0</v>
@@ -13912,10 +13921,10 @@
         <v>144</v>
       </c>
       <c r="AH170" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI170" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="171" spans="1:35">
@@ -13983,10 +13992,10 @@
         <v>144</v>
       </c>
       <c r="AH171" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI171" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="172" spans="1:35">
@@ -14054,10 +14063,10 @@
         <v>144</v>
       </c>
       <c r="AH172" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI172" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="173" spans="1:35">
@@ -14125,10 +14134,10 @@
         <v>144</v>
       </c>
       <c r="AH173" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI173" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="174" spans="1:35">
@@ -14196,10 +14205,10 @@
         <v>144</v>
       </c>
       <c r="AH174" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI174" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="175" spans="1:35">
@@ -14267,10 +14276,10 @@
         <v>144</v>
       </c>
       <c r="AH175" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI175" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="176" spans="1:35">
@@ -14338,10 +14347,10 @@
         <v>144</v>
       </c>
       <c r="AH176" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI176" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="177" spans="1:35">
@@ -14409,10 +14418,10 @@
         <v>144</v>
       </c>
       <c r="AH177" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI177" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="178" spans="1:35">
@@ -14480,10 +14489,10 @@
         <v>54</v>
       </c>
       <c r="AH178" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI178" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="179" spans="1:35">
@@ -14551,10 +14560,10 @@
         <v>54</v>
       </c>
       <c r="AH179" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI179" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="180" spans="1:35">
@@ -14622,10 +14631,10 @@
         <v>54</v>
       </c>
       <c r="AH180" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI180" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="181" spans="1:35">
@@ -14693,10 +14702,10 @@
         <v>54</v>
       </c>
       <c r="AH181" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI181" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="182" spans="1:35">
@@ -14764,10 +14773,10 @@
         <v>53</v>
       </c>
       <c r="AH182" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI182" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="183" spans="1:35">
@@ -14835,10 +14844,10 @@
         <v>53</v>
       </c>
       <c r="AH183" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI183" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="184" spans="1:35">
@@ -14906,10 +14915,10 @@
         <v>54</v>
       </c>
       <c r="AH184" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI184" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="185" spans="1:35">
@@ -14977,10 +14986,10 @@
         <v>54</v>
       </c>
       <c r="AH185" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI185" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="186" spans="1:35">
@@ -15048,10 +15057,10 @@
         <v>54</v>
       </c>
       <c r="AH186" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI186" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="187" spans="1:35">
@@ -15119,10 +15128,10 @@
         <v>146</v>
       </c>
       <c r="AH187" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI187" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="188" spans="1:35">
@@ -15190,10 +15199,10 @@
         <v>54</v>
       </c>
       <c r="AH188" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI188" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="189" spans="1:35">
@@ -15261,10 +15270,10 @@
         <v>54</v>
       </c>
       <c r="AH189" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI189" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="190" spans="1:35">
@@ -15332,10 +15341,10 @@
         <v>54</v>
       </c>
       <c r="AH190" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI190" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="191" spans="1:35">
@@ -15403,10 +15412,10 @@
         <v>54</v>
       </c>
       <c r="AH191" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI191" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="192" spans="1:35">
@@ -15474,10 +15483,10 @@
         <v>54</v>
       </c>
       <c r="AH192" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI192" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="193" spans="1:35">
@@ -15545,10 +15554,10 @@
         <v>54</v>
       </c>
       <c r="AH193" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI193" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="194" spans="1:35">
@@ -15616,10 +15625,10 @@
         <v>54</v>
       </c>
       <c r="AH194" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI194" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="195" spans="1:35">
@@ -15687,10 +15696,10 @@
         <v>54</v>
       </c>
       <c r="AH195" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI195" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="196" spans="1:35">
@@ -15758,10 +15767,10 @@
         <v>53</v>
       </c>
       <c r="AH196" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI196" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="197" spans="1:35">
@@ -15829,10 +15838,10 @@
         <v>53</v>
       </c>
       <c r="AH197" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI197" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="198" spans="1:35">
@@ -15900,10 +15909,10 @@
         <v>54</v>
       </c>
       <c r="AH198" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI198" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="199" spans="1:35">
@@ -15971,10 +15980,10 @@
         <v>54</v>
       </c>
       <c r="AH199" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI199" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="200" spans="1:35">
@@ -16042,10 +16051,10 @@
         <v>54</v>
       </c>
       <c r="AH200" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI200" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="201" spans="1:35">
@@ -16113,10 +16122,10 @@
         <v>54</v>
       </c>
       <c r="AH201" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AI201" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="202" spans="1:35">
@@ -16178,7 +16187,7 @@
         <v>165</v>
       </c>
       <c r="Y202" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AB202">
         <v>0</v>
@@ -16187,10 +16196,10 @@
         <v>54</v>
       </c>
       <c r="AH202" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI202" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="203" spans="1:35">
@@ -16252,7 +16261,7 @@
         <v>166</v>
       </c>
       <c r="Y203" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AB203">
         <v>0</v>
@@ -16261,10 +16270,10 @@
         <v>54</v>
       </c>
       <c r="AH203" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI203" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="204" spans="1:35">
@@ -16326,7 +16335,7 @@
         <v>168</v>
       </c>
       <c r="Y204" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AB204">
         <v>0</v>
@@ -16335,10 +16344,10 @@
         <v>54</v>
       </c>
       <c r="AH204" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI204" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="205" spans="1:35">
@@ -16400,7 +16409,7 @@
         <v>168</v>
       </c>
       <c r="Y205" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AB205">
         <v>0</v>
@@ -16409,10 +16418,10 @@
         <v>54</v>
       </c>
       <c r="AH205" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI205" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="206" spans="1:35">
@@ -16480,10 +16489,10 @@
         <v>54</v>
       </c>
       <c r="AH206" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI206" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="207" spans="1:35">
@@ -16551,10 +16560,10 @@
         <v>54</v>
       </c>
       <c r="AH207" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI207" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="208" spans="1:35">
@@ -16619,7 +16628,7 @@
         <v>165</v>
       </c>
       <c r="Y208" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AB208">
         <v>0</v>
@@ -16628,10 +16637,10 @@
         <v>147</v>
       </c>
       <c r="AH208" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI208" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="209" spans="1:35">
@@ -16693,7 +16702,7 @@
         <v>163</v>
       </c>
       <c r="Y209" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AB209">
         <v>0</v>
@@ -16702,10 +16711,10 @@
         <v>147</v>
       </c>
       <c r="AH209" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AI209" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-06 16:38
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2992" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2993" uniqueCount="238">
   <si>
     <t>CodCliente</t>
   </si>
@@ -649,6 +649,9 @@
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 06/10/2026 - Data Comentário: 05/10/2026 16:53</t>
   </si>
   <si>
+    <t>Imposto enviado via SCI Report - Data Comentário: 06/10/2026 16:25</t>
+  </si>
+  <si>
     <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1879]. - Data Comentário: 01/10/2026 01:58</t>
   </si>
   <si>
@@ -686,9 +689,6 @@
   </si>
   <si>
     <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1793]. - Data Comentário: 01/10/2026 09:02</t>
-  </si>
-  <si>
-    <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1867]. - Data Comentário: 01/10/2026 09:02</t>
   </si>
   <si>
     <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1808]. - Data Comentário: 01/10/2026 09:01</t>
@@ -8832,10 +8832,10 @@
     </row>
     <row r="102" spans="1:35">
       <c r="A102">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B102" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C102" t="s">
         <v>49</v>
@@ -8847,22 +8847,22 @@
         <v>54</v>
       </c>
       <c r="F102" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G102">
-        <v>6883</v>
+        <v>1867</v>
       </c>
       <c r="H102">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I102" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J102" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="N102" s="1">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="P102">
         <v>9</v>
@@ -8871,37 +8871,40 @@
         <v>2026</v>
       </c>
       <c r="R102">
-        <v>17399251</v>
+        <v>18214860</v>
       </c>
       <c r="S102" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="T102" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="U102" t="s">
         <v>158</v>
       </c>
       <c r="V102" s="1">
-        <v>46297.37673402778</v>
+        <v>46301.68910333333</v>
       </c>
       <c r="W102">
-        <v>-7</v>
+        <v>-3</v>
       </c>
       <c r="X102" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+      <c r="Y102" t="s">
+        <v>206</v>
       </c>
       <c r="AB102">
         <v>0</v>
       </c>
       <c r="AC102" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="AH102" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AI102" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="103" spans="1:35">
@@ -8924,7 +8927,7 @@
         <v>55</v>
       </c>
       <c r="G103">
-        <v>1836</v>
+        <v>6883</v>
       </c>
       <c r="H103">
         <v>1788</v>
@@ -8933,10 +8936,10 @@
         <v>61</v>
       </c>
       <c r="J103" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="N103" s="1">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="P103">
         <v>9</v>
@@ -8945,7 +8948,7 @@
         <v>2026</v>
       </c>
       <c r="R103">
-        <v>17398976</v>
+        <v>17399251</v>
       </c>
       <c r="S103" t="s">
         <v>143</v>
@@ -8957,10 +8960,10 @@
         <v>158</v>
       </c>
       <c r="V103" s="1">
-        <v>46297.37618915509</v>
+        <v>46297.37673402778</v>
       </c>
       <c r="W103">
-        <v>1</v>
+        <v>-7</v>
       </c>
       <c r="X103" t="s">
         <v>166</v>
@@ -8980,10 +8983,10 @@
     </row>
     <row r="104" spans="1:35">
       <c r="A104">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B104" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C104" t="s">
         <v>49</v>
@@ -9019,7 +9022,7 @@
         <v>2026</v>
       </c>
       <c r="R104">
-        <v>18155319</v>
+        <v>17398976</v>
       </c>
       <c r="S104" t="s">
         <v>143</v>
@@ -9031,13 +9034,13 @@
         <v>158</v>
       </c>
       <c r="V104" s="1">
-        <v>46297.66736068287</v>
+        <v>46297.37618915509</v>
       </c>
       <c r="W104">
         <v>1</v>
       </c>
       <c r="X104" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="AB104">
         <v>0</v>
@@ -9054,10 +9057,10 @@
     </row>
     <row r="105" spans="1:35">
       <c r="A105">
-        <v>6704</v>
+        <v>6486</v>
       </c>
       <c r="B105" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C105" t="s">
         <v>49</v>
@@ -9093,7 +9096,7 @@
         <v>2026</v>
       </c>
       <c r="R105">
-        <v>18085221</v>
+        <v>18155319</v>
       </c>
       <c r="S105" t="s">
         <v>143</v>
@@ -9105,13 +9108,13 @@
         <v>158</v>
       </c>
       <c r="V105" s="1">
-        <v>46297.45935385417</v>
+        <v>46297.66736068287</v>
       </c>
       <c r="W105">
         <v>1</v>
       </c>
       <c r="X105" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AB105">
         <v>0</v>
@@ -9128,10 +9131,10 @@
     </row>
     <row r="106" spans="1:35">
       <c r="A106">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B106" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C106" t="s">
         <v>49</v>
@@ -9146,7 +9149,7 @@
         <v>55</v>
       </c>
       <c r="G106">
-        <v>6802</v>
+        <v>1836</v>
       </c>
       <c r="H106">
         <v>1788</v>
@@ -9155,7 +9158,7 @@
         <v>61</v>
       </c>
       <c r="J106" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N106" s="1">
         <v>46300</v>
@@ -9167,7 +9170,7 @@
         <v>2026</v>
       </c>
       <c r="R106">
-        <v>17399221</v>
+        <v>18085221</v>
       </c>
       <c r="S106" t="s">
         <v>143</v>
@@ -9179,13 +9182,13 @@
         <v>158</v>
       </c>
       <c r="V106" s="1">
-        <v>46297.37681010416</v>
+        <v>46297.45935385417</v>
       </c>
       <c r="W106">
         <v>1</v>
       </c>
       <c r="X106" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AB106">
         <v>0</v>
@@ -9220,16 +9223,16 @@
         <v>55</v>
       </c>
       <c r="G107">
-        <v>6801</v>
+        <v>6802</v>
       </c>
       <c r="H107">
-        <v>1796</v>
+        <v>1788</v>
       </c>
       <c r="I107" t="s">
         <v>61</v>
       </c>
       <c r="J107" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="N107" s="1">
         <v>46300</v>
@@ -9241,7 +9244,7 @@
         <v>2026</v>
       </c>
       <c r="R107">
-        <v>17399211</v>
+        <v>17399221</v>
       </c>
       <c r="S107" t="s">
         <v>143</v>
@@ -9253,7 +9256,7 @@
         <v>158</v>
       </c>
       <c r="V107" s="1">
-        <v>46297.37686377315</v>
+        <v>46297.37681010416</v>
       </c>
       <c r="W107">
         <v>1</v>
@@ -9294,16 +9297,16 @@
         <v>55</v>
       </c>
       <c r="G108">
-        <v>6014</v>
+        <v>6801</v>
       </c>
       <c r="H108">
-        <v>1788</v>
+        <v>1796</v>
       </c>
       <c r="I108" t="s">
         <v>61</v>
       </c>
       <c r="J108" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="N108" s="1">
         <v>46300</v>
@@ -9315,7 +9318,7 @@
         <v>2026</v>
       </c>
       <c r="R108">
-        <v>17399137</v>
+        <v>17399211</v>
       </c>
       <c r="S108" t="s">
         <v>143</v>
@@ -9327,7 +9330,7 @@
         <v>158</v>
       </c>
       <c r="V108" s="1">
-        <v>46297.37606362269</v>
+        <v>46297.37686377315</v>
       </c>
       <c r="W108">
         <v>1</v>
@@ -9350,10 +9353,10 @@
     </row>
     <row r="109" spans="1:35">
       <c r="A109">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B109" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C109" t="s">
         <v>49</v>
@@ -9389,7 +9392,7 @@
         <v>2026</v>
       </c>
       <c r="R109">
-        <v>18155328</v>
+        <v>17399137</v>
       </c>
       <c r="S109" t="s">
         <v>143</v>
@@ -9401,13 +9404,13 @@
         <v>158</v>
       </c>
       <c r="V109" s="1">
-        <v>46297.66734447917</v>
+        <v>46297.37606362269</v>
       </c>
       <c r="W109">
         <v>1</v>
       </c>
       <c r="X109" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="AB109">
         <v>0</v>
@@ -9424,10 +9427,10 @@
     </row>
     <row r="110" spans="1:35">
       <c r="A110">
-        <v>6704</v>
+        <v>6486</v>
       </c>
       <c r="B110" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C110" t="s">
         <v>49</v>
@@ -9463,7 +9466,7 @@
         <v>2026</v>
       </c>
       <c r="R110">
-        <v>18085232</v>
+        <v>18155328</v>
       </c>
       <c r="S110" t="s">
         <v>143</v>
@@ -9475,13 +9478,13 @@
         <v>158</v>
       </c>
       <c r="V110" s="1">
-        <v>46297.45929016203</v>
+        <v>46297.66734447917</v>
       </c>
       <c r="W110">
         <v>1</v>
       </c>
       <c r="X110" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AB110">
         <v>0</v>
@@ -9498,10 +9501,10 @@
     </row>
     <row r="111" spans="1:35">
       <c r="A111">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B111" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C111" t="s">
         <v>49</v>
@@ -9516,16 +9519,16 @@
         <v>55</v>
       </c>
       <c r="G111">
-        <v>6233</v>
+        <v>6014</v>
       </c>
       <c r="H111">
-        <v>6232</v>
+        <v>1788</v>
       </c>
       <c r="I111" t="s">
         <v>61</v>
       </c>
       <c r="J111" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N111" s="1">
         <v>46300</v>
@@ -9537,7 +9540,7 @@
         <v>2026</v>
       </c>
       <c r="R111">
-        <v>17399177</v>
+        <v>18085232</v>
       </c>
       <c r="S111" t="s">
         <v>143</v>
@@ -9549,13 +9552,13 @@
         <v>158</v>
       </c>
       <c r="V111" s="1">
-        <v>46297.37537966435</v>
+        <v>46297.45929016203</v>
       </c>
       <c r="W111">
         <v>1</v>
       </c>
       <c r="X111" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AB111">
         <v>0</v>
@@ -9572,16 +9575,16 @@
     </row>
     <row r="112" spans="1:35">
       <c r="A112">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B112" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C112" t="s">
         <v>49</v>
       </c>
       <c r="D112" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E112" t="s">
         <v>54</v>
@@ -9611,7 +9614,7 @@
         <v>2026</v>
       </c>
       <c r="R112">
-        <v>16962295</v>
+        <v>17399177</v>
       </c>
       <c r="S112" t="s">
         <v>143</v>
@@ -9623,13 +9626,13 @@
         <v>158</v>
       </c>
       <c r="V112" s="1">
-        <v>46297.45869950231</v>
+        <v>46297.37537966435</v>
       </c>
       <c r="W112">
         <v>1</v>
       </c>
       <c r="X112" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AB112">
         <v>0</v>
@@ -9646,16 +9649,16 @@
     </row>
     <row r="113" spans="1:35">
       <c r="A113">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B113" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C113" t="s">
         <v>49</v>
       </c>
       <c r="D113" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E113" t="s">
         <v>54</v>
@@ -9685,7 +9688,7 @@
         <v>2026</v>
       </c>
       <c r="R113">
-        <v>16976157</v>
+        <v>16962295</v>
       </c>
       <c r="S113" t="s">
         <v>143</v>
@@ -9694,16 +9697,16 @@
         <v>156</v>
       </c>
       <c r="U113" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="V113" s="1">
-        <v>46300.66721489583</v>
+        <v>46297.45869950231</v>
       </c>
       <c r="W113">
         <v>1</v>
       </c>
       <c r="X113" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AB113">
         <v>0</v>
@@ -9715,21 +9718,21 @@
         <v>233</v>
       </c>
       <c r="AI113" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="114" spans="1:35">
       <c r="A114">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B114" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C114" t="s">
         <v>49</v>
       </c>
       <c r="D114" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E114" t="s">
         <v>54</v>
@@ -9759,7 +9762,7 @@
         <v>2026</v>
       </c>
       <c r="R114">
-        <v>17948845</v>
+        <v>16976157</v>
       </c>
       <c r="S114" t="s">
         <v>143</v>
@@ -9768,16 +9771,16 @@
         <v>156</v>
       </c>
       <c r="U114" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="V114" s="1">
-        <v>46297.45870309028</v>
+        <v>46300.66721489583</v>
       </c>
       <c r="W114">
         <v>1</v>
       </c>
       <c r="X114" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AB114">
         <v>0</v>
@@ -9789,21 +9792,21 @@
         <v>233</v>
       </c>
       <c r="AI114" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="115" spans="1:35">
       <c r="A115">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B115" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C115" t="s">
         <v>49</v>
       </c>
       <c r="D115" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E115" t="s">
         <v>54</v>
@@ -9833,7 +9836,7 @@
         <v>2026</v>
       </c>
       <c r="R115">
-        <v>18085265</v>
+        <v>17948845</v>
       </c>
       <c r="S115" t="s">
         <v>143</v>
@@ -9845,13 +9848,13 @@
         <v>158</v>
       </c>
       <c r="V115" s="1">
-        <v>46297.45870405093</v>
+        <v>46297.45870309028</v>
       </c>
       <c r="W115">
         <v>1</v>
       </c>
       <c r="X115" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="AB115">
         <v>0</v>
@@ -9868,16 +9871,16 @@
     </row>
     <row r="116" spans="1:35">
       <c r="A116">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B116" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C116" t="s">
         <v>49</v>
       </c>
       <c r="D116" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E116" t="s">
         <v>54</v>
@@ -9907,7 +9910,7 @@
         <v>2026</v>
       </c>
       <c r="R116">
-        <v>17948990</v>
+        <v>18085265</v>
       </c>
       <c r="S116" t="s">
         <v>143</v>
@@ -9919,7 +9922,7 @@
         <v>158</v>
       </c>
       <c r="V116" s="1">
-        <v>46297.45870177083</v>
+        <v>46297.45870405093</v>
       </c>
       <c r="W116">
         <v>1</v>
@@ -9942,16 +9945,16 @@
     </row>
     <row r="117" spans="1:35">
       <c r="A117">
-        <v>5417</v>
+        <v>6705</v>
       </c>
       <c r="B117" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C117" t="s">
         <v>49</v>
       </c>
       <c r="D117" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E117" t="s">
         <v>54</v>
@@ -9960,16 +9963,16 @@
         <v>55</v>
       </c>
       <c r="G117">
-        <v>6230</v>
+        <v>6233</v>
       </c>
       <c r="H117">
-        <v>9114</v>
+        <v>6232</v>
       </c>
       <c r="I117" t="s">
         <v>61</v>
       </c>
       <c r="J117" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="N117" s="1">
         <v>46300</v>
@@ -9981,7 +9984,7 @@
         <v>2026</v>
       </c>
       <c r="R117">
-        <v>17399157</v>
+        <v>17948990</v>
       </c>
       <c r="S117" t="s">
         <v>143</v>
@@ -9990,16 +9993,16 @@
         <v>156</v>
       </c>
       <c r="U117" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="V117" s="1">
-        <v>46300.65013206018</v>
+        <v>46297.45870177083</v>
       </c>
       <c r="W117">
         <v>1</v>
       </c>
       <c r="X117" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AB117">
         <v>0</v>
@@ -10011,21 +10014,21 @@
         <v>233</v>
       </c>
       <c r="AI117" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="118" spans="1:35">
       <c r="A118">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B118" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C118" t="s">
         <v>49</v>
       </c>
       <c r="D118" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E118" t="s">
         <v>54</v>
@@ -10055,7 +10058,7 @@
         <v>2026</v>
       </c>
       <c r="R118">
-        <v>16962275</v>
+        <v>17399157</v>
       </c>
       <c r="S118" t="s">
         <v>143</v>
@@ -10067,13 +10070,13 @@
         <v>159</v>
       </c>
       <c r="V118" s="1">
-        <v>46300.65011049769</v>
+        <v>46300.65013206018</v>
       </c>
       <c r="W118">
         <v>1</v>
       </c>
       <c r="X118" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AB118">
         <v>0</v>
@@ -10090,16 +10093,16 @@
     </row>
     <row r="119" spans="1:35">
       <c r="A119">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B119" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C119" t="s">
         <v>49</v>
       </c>
       <c r="D119" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E119" t="s">
         <v>54</v>
@@ -10129,7 +10132,7 @@
         <v>2026</v>
       </c>
       <c r="R119">
-        <v>16976137</v>
+        <v>16962275</v>
       </c>
       <c r="S119" t="s">
         <v>143</v>
@@ -10141,13 +10144,13 @@
         <v>159</v>
       </c>
       <c r="V119" s="1">
-        <v>46300.66713765046</v>
+        <v>46300.65011049769</v>
       </c>
       <c r="W119">
         <v>1</v>
       </c>
       <c r="X119" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AB119">
         <v>0</v>
@@ -10164,16 +10167,16 @@
     </row>
     <row r="120" spans="1:35">
       <c r="A120">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B120" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C120" t="s">
         <v>49</v>
       </c>
       <c r="D120" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E120" t="s">
         <v>54</v>
@@ -10203,7 +10206,7 @@
         <v>2026</v>
       </c>
       <c r="R120">
-        <v>17948825</v>
+        <v>16976137</v>
       </c>
       <c r="S120" t="s">
         <v>143</v>
@@ -10215,13 +10218,13 @@
         <v>159</v>
       </c>
       <c r="V120" s="1">
-        <v>46300.66713784722</v>
+        <v>46300.66713765046</v>
       </c>
       <c r="W120">
         <v>1</v>
       </c>
       <c r="X120" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AB120">
         <v>0</v>
@@ -10238,16 +10241,16 @@
     </row>
     <row r="121" spans="1:35">
       <c r="A121">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B121" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C121" t="s">
         <v>49</v>
       </c>
       <c r="D121" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E121" t="s">
         <v>54</v>
@@ -10277,7 +10280,7 @@
         <v>2026</v>
       </c>
       <c r="R121">
-        <v>18085243</v>
+        <v>17948825</v>
       </c>
       <c r="S121" t="s">
         <v>143</v>
@@ -10289,13 +10292,13 @@
         <v>159</v>
       </c>
       <c r="V121" s="1">
-        <v>46300.66713822917</v>
+        <v>46300.66713784722</v>
       </c>
       <c r="W121">
         <v>1</v>
       </c>
       <c r="X121" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="AB121">
         <v>0</v>
@@ -10312,16 +10315,16 @@
     </row>
     <row r="122" spans="1:35">
       <c r="A122">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B122" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C122" t="s">
         <v>49</v>
       </c>
       <c r="D122" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E122" t="s">
         <v>54</v>
@@ -10351,7 +10354,7 @@
         <v>2026</v>
       </c>
       <c r="R122">
-        <v>17948970</v>
+        <v>18085243</v>
       </c>
       <c r="S122" t="s">
         <v>143</v>
@@ -10363,7 +10366,7 @@
         <v>159</v>
       </c>
       <c r="V122" s="1">
-        <v>46300.75530894676</v>
+        <v>46300.66713822917</v>
       </c>
       <c r="W122">
         <v>1</v>
@@ -10386,16 +10389,16 @@
     </row>
     <row r="123" spans="1:35">
       <c r="A123">
-        <v>6486</v>
+        <v>6705</v>
       </c>
       <c r="B123" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C123" t="s">
         <v>49</v>
       </c>
       <c r="D123" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E123" t="s">
         <v>54</v>
@@ -10404,19 +10407,19 @@
         <v>55</v>
       </c>
       <c r="G123">
-        <v>11359</v>
+        <v>6230</v>
       </c>
       <c r="H123">
-        <v>0</v>
+        <v>9114</v>
       </c>
       <c r="I123" t="s">
         <v>61</v>
       </c>
       <c r="J123" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="N123" s="1">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="P123">
         <v>9</v>
@@ -10425,7 +10428,7 @@
         <v>2026</v>
       </c>
       <c r="R123">
-        <v>18155346</v>
+        <v>17948970</v>
       </c>
       <c r="S123" t="s">
         <v>143</v>
@@ -10437,13 +10440,13 @@
         <v>159</v>
       </c>
       <c r="V123" s="1">
-        <v>46297.66734765047</v>
+        <v>46300.75530894676</v>
       </c>
       <c r="W123">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X123" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="AB123">
         <v>0</v>
@@ -10455,42 +10458,42 @@
         <v>233</v>
       </c>
       <c r="AI123" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="124" spans="1:35">
       <c r="A124">
-        <v>6628</v>
+        <v>6486</v>
       </c>
       <c r="B124" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C124" t="s">
         <v>49</v>
       </c>
       <c r="D124" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E124" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F124" t="s">
         <v>55</v>
       </c>
       <c r="G124">
-        <v>945</v>
+        <v>11359</v>
       </c>
       <c r="H124">
         <v>0</v>
       </c>
       <c r="I124" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J124" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N124" s="1">
-        <v>46315</v>
+        <v>46297</v>
       </c>
       <c r="P124">
         <v>9</v>
@@ -10499,34 +10502,34 @@
         <v>2026</v>
       </c>
       <c r="R124">
-        <v>16959939</v>
+        <v>18155346</v>
       </c>
       <c r="S124" t="s">
-        <v>144</v>
+        <v>143</v>
+      </c>
+      <c r="T124" t="s">
+        <v>156</v>
       </c>
       <c r="U124" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="V124" s="1">
-        <v>46296.08337256945</v>
+        <v>46297.66734765047</v>
       </c>
       <c r="W124">
-        <v>-14</v>
+        <v>4</v>
       </c>
       <c r="X124" t="s">
-        <v>160</v>
-      </c>
-      <c r="Y124" t="s">
-        <v>206</v>
+        <v>168</v>
       </c>
       <c r="AB124">
         <v>0</v>
       </c>
       <c r="AC124" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AH124" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AI124" t="s">
         <v>237</v>
@@ -10534,10 +10537,10 @@
     </row>
     <row r="125" spans="1:35">
       <c r="A125">
-        <v>6779</v>
+        <v>6628</v>
       </c>
       <c r="B125" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C125" t="s">
         <v>49</v>
@@ -10546,7 +10549,7 @@
         <v>51</v>
       </c>
       <c r="E125" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F125" t="s">
         <v>55</v>
@@ -10573,7 +10576,7 @@
         <v>2026</v>
       </c>
       <c r="R125">
-        <v>18056696</v>
+        <v>16959939</v>
       </c>
       <c r="S125" t="s">
         <v>144</v>
@@ -10582,13 +10585,13 @@
         <v>158</v>
       </c>
       <c r="V125" s="1">
-        <v>46296.0834071412</v>
+        <v>46296.08337256945</v>
       </c>
       <c r="W125">
         <v>-14</v>
       </c>
       <c r="X125" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="Y125" t="s">
         <v>207</v>
@@ -10608,10 +10611,10 @@
     </row>
     <row r="126" spans="1:35">
       <c r="A126">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B126" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C126" t="s">
         <v>49</v>
@@ -10623,7 +10626,7 @@
         <v>54</v>
       </c>
       <c r="F126" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G126">
         <v>945</v>
@@ -10647,7 +10650,7 @@
         <v>2026</v>
       </c>
       <c r="R126">
-        <v>18164488</v>
+        <v>18056696</v>
       </c>
       <c r="S126" t="s">
         <v>144</v>
@@ -10656,16 +10659,16 @@
         <v>158</v>
       </c>
       <c r="V126" s="1">
-        <v>46296.08341825232</v>
+        <v>46296.0834071412</v>
       </c>
       <c r="W126">
         <v>-14</v>
       </c>
       <c r="X126" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="Y126" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="AB126">
         <v>0</v>
@@ -10682,25 +10685,25 @@
     </row>
     <row r="127" spans="1:35">
       <c r="A127">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B127" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C127" t="s">
         <v>49</v>
       </c>
       <c r="D127" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E127" t="s">
         <v>54</v>
       </c>
       <c r="F127" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G127">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H127">
         <v>0</v>
@@ -10709,7 +10712,7 @@
         <v>62</v>
       </c>
       <c r="J127" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="N127" s="1">
         <v>46315</v>
@@ -10721,7 +10724,7 @@
         <v>2026</v>
       </c>
       <c r="R127">
-        <v>17398870</v>
+        <v>18164488</v>
       </c>
       <c r="S127" t="s">
         <v>144</v>
@@ -10730,16 +10733,16 @@
         <v>158</v>
       </c>
       <c r="V127" s="1">
-        <v>46296.37558109954</v>
+        <v>46296.08341825232</v>
       </c>
       <c r="W127">
         <v>-14</v>
       </c>
       <c r="X127" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="Y127" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AB127">
         <v>0</v>
@@ -10756,16 +10759,16 @@
     </row>
     <row r="128" spans="1:35">
       <c r="A128">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B128" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C128" t="s">
         <v>49</v>
       </c>
       <c r="D128" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E128" t="s">
         <v>54</v>
@@ -10795,7 +10798,7 @@
         <v>2026</v>
       </c>
       <c r="R128">
-        <v>16962094</v>
+        <v>17398870</v>
       </c>
       <c r="S128" t="s">
         <v>144</v>
@@ -10804,13 +10807,13 @@
         <v>158</v>
       </c>
       <c r="V128" s="1">
-        <v>46296.37504012731</v>
+        <v>46296.37558109954</v>
       </c>
       <c r="W128">
         <v>-14</v>
       </c>
       <c r="X128" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="Y128" t="s">
         <v>209</v>
@@ -10830,10 +10833,10 @@
     </row>
     <row r="129" spans="1:35">
       <c r="A129">
-        <v>6703</v>
+        <v>6404</v>
       </c>
       <c r="B129" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C129" t="s">
         <v>49</v>
@@ -10869,22 +10872,22 @@
         <v>2026</v>
       </c>
       <c r="R129">
-        <v>17941133</v>
+        <v>16962094</v>
       </c>
       <c r="S129" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="U129" t="s">
         <v>158</v>
       </c>
       <c r="V129" s="1">
-        <v>46296.3760846412</v>
+        <v>46296.37504012731</v>
       </c>
       <c r="W129">
         <v>-14</v>
       </c>
       <c r="X129" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Y129" t="s">
         <v>210</v>
@@ -10893,7 +10896,7 @@
         <v>0</v>
       </c>
       <c r="AC129" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AH129" t="s">
         <v>234</v>
@@ -10904,16 +10907,16 @@
     </row>
     <row r="130" spans="1:35">
       <c r="A130">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B130" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C130" t="s">
         <v>49</v>
       </c>
       <c r="D130" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E130" t="s">
         <v>54</v>
@@ -10922,7 +10925,7 @@
         <v>55</v>
       </c>
       <c r="G130">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="H130">
         <v>0</v>
@@ -10931,10 +10934,10 @@
         <v>62</v>
       </c>
       <c r="J130" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="N130" s="1">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="P130">
         <v>9</v>
@@ -10943,22 +10946,22 @@
         <v>2026</v>
       </c>
       <c r="R130">
-        <v>17398876</v>
+        <v>17941133</v>
       </c>
       <c r="S130" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="U130" t="s">
         <v>158</v>
       </c>
       <c r="V130" s="1">
-        <v>46296.37648518519</v>
+        <v>46296.3760846412</v>
       </c>
       <c r="W130">
-        <v>-24</v>
+        <v>-14</v>
       </c>
       <c r="X130" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="Y130" t="s">
         <v>211</v>
@@ -10967,7 +10970,7 @@
         <v>0</v>
       </c>
       <c r="AC130" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AH130" t="s">
         <v>234</v>
@@ -10978,10 +10981,10 @@
     </row>
     <row r="131" spans="1:35">
       <c r="A131">
-        <v>6627</v>
+        <v>5417</v>
       </c>
       <c r="B131" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C131" t="s">
         <v>49</v>
@@ -10990,7 +10993,7 @@
         <v>50</v>
       </c>
       <c r="E131" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F131" t="s">
         <v>55</v>
@@ -11017,7 +11020,7 @@
         <v>2026</v>
       </c>
       <c r="R131">
-        <v>17042296</v>
+        <v>17398876</v>
       </c>
       <c r="S131" t="s">
         <v>144</v>
@@ -11026,13 +11029,13 @@
         <v>158</v>
       </c>
       <c r="V131" s="1">
-        <v>46296.37615983796</v>
+        <v>46296.37648518519</v>
       </c>
       <c r="W131">
         <v>-24</v>
       </c>
       <c r="X131" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="Y131" t="s">
         <v>212</v>
@@ -11052,10 +11055,10 @@
     </row>
     <row r="132" spans="1:35">
       <c r="A132">
-        <v>6704</v>
+        <v>6627</v>
       </c>
       <c r="B132" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C132" t="s">
         <v>49</v>
@@ -11064,7 +11067,7 @@
         <v>50</v>
       </c>
       <c r="E132" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F132" t="s">
         <v>55</v>
@@ -11091,7 +11094,7 @@
         <v>2026</v>
       </c>
       <c r="R132">
-        <v>17952332</v>
+        <v>17042296</v>
       </c>
       <c r="S132" t="s">
         <v>144</v>
@@ -11100,16 +11103,16 @@
         <v>158</v>
       </c>
       <c r="V132" s="1">
-        <v>46296.37684290509</v>
+        <v>46296.37615983796</v>
       </c>
       <c r="W132">
         <v>-24</v>
       </c>
       <c r="X132" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="Y132" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="AB132">
         <v>0</v>
@@ -11126,16 +11129,16 @@
     </row>
     <row r="133" spans="1:35">
       <c r="A133">
-        <v>6404</v>
+        <v>6704</v>
       </c>
       <c r="B133" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C133" t="s">
         <v>49</v>
       </c>
       <c r="D133" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E133" t="s">
         <v>54</v>
@@ -11144,7 +11147,7 @@
         <v>55</v>
       </c>
       <c r="G133">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="H133">
         <v>0</v>
@@ -11153,7 +11156,7 @@
         <v>62</v>
       </c>
       <c r="J133" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N133" s="1">
         <v>46325</v>
@@ -11165,7 +11168,7 @@
         <v>2026</v>
       </c>
       <c r="R133">
-        <v>16962100</v>
+        <v>17952332</v>
       </c>
       <c r="S133" t="s">
         <v>144</v>
@@ -11174,16 +11177,16 @@
         <v>158</v>
       </c>
       <c r="V133" s="1">
-        <v>46296.37609667824</v>
+        <v>46296.37684290509</v>
       </c>
       <c r="W133">
         <v>-24</v>
       </c>
       <c r="X133" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="Y133" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AB133">
         <v>0</v>
@@ -11200,10 +11203,10 @@
     </row>
     <row r="134" spans="1:35">
       <c r="A134">
-        <v>6703</v>
+        <v>6404</v>
       </c>
       <c r="B134" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C134" t="s">
         <v>49</v>
@@ -11239,22 +11242,22 @@
         <v>2026</v>
       </c>
       <c r="R134">
-        <v>17941139</v>
+        <v>16962100</v>
       </c>
       <c r="S134" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="U134" t="s">
         <v>158</v>
       </c>
       <c r="V134" s="1">
-        <v>46296.37683961805</v>
+        <v>46296.37609667824</v>
       </c>
       <c r="W134">
         <v>-24</v>
       </c>
       <c r="X134" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Y134" t="s">
         <v>214</v>
@@ -11263,7 +11266,7 @@
         <v>0</v>
       </c>
       <c r="AC134" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AH134" t="s">
         <v>234</v>
@@ -11292,7 +11295,7 @@
         <v>55</v>
       </c>
       <c r="G135">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="H135">
         <v>0</v>
@@ -11301,10 +11304,10 @@
         <v>62</v>
       </c>
       <c r="J135" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N135" s="1">
-        <v>46304</v>
+        <v>46325</v>
       </c>
       <c r="P135">
         <v>9</v>
@@ -11313,7 +11316,7 @@
         <v>2026</v>
       </c>
       <c r="R135">
-        <v>17941147</v>
+        <v>17941139</v>
       </c>
       <c r="S135" t="s">
         <v>145</v>
@@ -11322,10 +11325,10 @@
         <v>158</v>
       </c>
       <c r="V135" s="1">
-        <v>46296.37684039352</v>
+        <v>46296.37683961805</v>
       </c>
       <c r="W135">
-        <v>-3</v>
+        <v>-24</v>
       </c>
       <c r="X135" t="s">
         <v>169</v>
@@ -11348,22 +11351,22 @@
     </row>
     <row r="136" spans="1:35">
       <c r="A136">
-        <v>6949</v>
+        <v>6703</v>
       </c>
       <c r="B136" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C136" t="s">
         <v>49</v>
       </c>
       <c r="D136" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E136" t="s">
         <v>54</v>
       </c>
       <c r="F136" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G136">
         <v>950</v>
@@ -11387,22 +11390,22 @@
         <v>2026</v>
       </c>
       <c r="R136">
-        <v>18178133</v>
+        <v>17941147</v>
       </c>
       <c r="S136" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="U136" t="s">
         <v>158</v>
       </c>
       <c r="V136" s="1">
-        <v>46296.37697557871</v>
+        <v>46296.37684039352</v>
       </c>
       <c r="W136">
         <v>-3</v>
       </c>
       <c r="X136" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="Y136" t="s">
         <v>216</v>
@@ -11411,7 +11414,7 @@
         <v>0</v>
       </c>
       <c r="AC136" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AH136" t="s">
         <v>234</v>
@@ -11422,10 +11425,10 @@
     </row>
     <row r="137" spans="1:35">
       <c r="A137">
-        <v>6548</v>
+        <v>6949</v>
       </c>
       <c r="B137" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C137" t="s">
         <v>49</v>
@@ -11437,10 +11440,10 @@
         <v>54</v>
       </c>
       <c r="F137" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G137">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H137">
         <v>0</v>
@@ -11449,7 +11452,7 @@
         <v>62</v>
       </c>
       <c r="J137" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N137" s="1">
         <v>46304</v>
@@ -11461,7 +11464,7 @@
         <v>2026</v>
       </c>
       <c r="R137">
-        <v>17222406</v>
+        <v>18178133</v>
       </c>
       <c r="S137" t="s">
         <v>144</v>
@@ -11470,13 +11473,13 @@
         <v>158</v>
       </c>
       <c r="V137" s="1">
-        <v>46296.37726273148</v>
+        <v>46296.37697557871</v>
       </c>
       <c r="W137">
         <v>-3</v>
       </c>
       <c r="X137" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="Y137" t="s">
         <v>217</v>
@@ -11496,16 +11499,16 @@
     </row>
     <row r="138" spans="1:35">
       <c r="A138">
-        <v>6703</v>
+        <v>6548</v>
       </c>
       <c r="B138" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C138" t="s">
         <v>49</v>
       </c>
       <c r="D138" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E138" t="s">
         <v>54</v>
@@ -11535,22 +11538,22 @@
         <v>2026</v>
       </c>
       <c r="R138">
-        <v>17941157</v>
+        <v>17222406</v>
       </c>
       <c r="S138" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="U138" t="s">
         <v>158</v>
       </c>
       <c r="V138" s="1">
-        <v>46296.37814100694</v>
+        <v>46296.37726273148</v>
       </c>
       <c r="W138">
         <v>-3</v>
       </c>
       <c r="X138" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="Y138" t="s">
         <v>218</v>
@@ -11559,7 +11562,7 @@
         <v>0</v>
       </c>
       <c r="AC138" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AH138" t="s">
         <v>234</v>
@@ -11570,16 +11573,16 @@
     </row>
     <row r="139" spans="1:35">
       <c r="A139">
-        <v>6779</v>
+        <v>6703</v>
       </c>
       <c r="B139" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C139" t="s">
         <v>49</v>
       </c>
       <c r="D139" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E139" t="s">
         <v>54</v>
@@ -11609,31 +11612,31 @@
         <v>2026</v>
       </c>
       <c r="R139">
-        <v>18056706</v>
+        <v>17941157</v>
       </c>
       <c r="S139" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="U139" t="s">
         <v>158</v>
       </c>
       <c r="V139" s="1">
-        <v>46296.37816597222</v>
+        <v>46296.37814100694</v>
       </c>
       <c r="W139">
         <v>-3</v>
       </c>
       <c r="X139" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="Y139" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AB139">
         <v>0</v>
       </c>
       <c r="AC139" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="AH139" t="s">
         <v>234</v>
@@ -11644,22 +11647,22 @@
     </row>
     <row r="140" spans="1:35">
       <c r="A140">
-        <v>6949</v>
+        <v>6779</v>
       </c>
       <c r="B140" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C140" t="s">
         <v>49</v>
       </c>
       <c r="D140" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E140" t="s">
         <v>54</v>
       </c>
       <c r="F140" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G140">
         <v>951</v>
@@ -11683,7 +11686,7 @@
         <v>2026</v>
       </c>
       <c r="R140">
-        <v>18178139</v>
+        <v>18056706</v>
       </c>
       <c r="S140" t="s">
         <v>144</v>
@@ -11692,13 +11695,13 @@
         <v>158</v>
       </c>
       <c r="V140" s="1">
-        <v>46296.37822091435</v>
+        <v>46296.37816597222</v>
       </c>
       <c r="W140">
         <v>-3</v>
       </c>
       <c r="X140" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="Y140" t="s">
         <v>219</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-07 12:36
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3109" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3124" uniqueCount="246">
   <si>
     <t>CodCliente</t>
   </si>
@@ -729,6 +729,9 @@
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 06/10/2026 - Data Comentário: 05/10/2026 18:36</t>
+  </si>
+  <si>
+    <t>Comentário Colaborador + Previsão De Conclusão   Previsto para conclusão dia 06/10/2026. - Data Comentário: 06/10/2026 18:20</t>
   </si>
   <si>
     <t>Baixado via rotina MGC x Analise Balanço em 01/10/2026 08:11:14. - Data Comentário: 01/10/2026 08:09</t>
@@ -1102,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI217"/>
+  <dimension ref="A1:AI218"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -1283,10 +1286,10 @@
         <v>128</v>
       </c>
       <c r="AH2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:35">
@@ -1360,10 +1363,10 @@
         <v>128</v>
       </c>
       <c r="AH3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:35">
@@ -1434,10 +1437,10 @@
         <v>129</v>
       </c>
       <c r="AH4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" spans="1:35">
@@ -1508,10 +1511,10 @@
         <v>128</v>
       </c>
       <c r="AH5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6" spans="1:35">
@@ -1582,10 +1585,10 @@
         <v>128</v>
       </c>
       <c r="AH6" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI6" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" spans="1:35">
@@ -1656,10 +1659,10 @@
         <v>130</v>
       </c>
       <c r="AH7" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI7" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" spans="1:35">
@@ -1730,10 +1733,10 @@
         <v>129</v>
       </c>
       <c r="AH8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="9" spans="1:35">
@@ -1804,10 +1807,10 @@
         <v>131</v>
       </c>
       <c r="AH9" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10" spans="1:35">
@@ -1878,10 +1881,10 @@
         <v>131</v>
       </c>
       <c r="AH10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:35">
@@ -1952,10 +1955,10 @@
         <v>132</v>
       </c>
       <c r="AH11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" spans="1:35">
@@ -2029,10 +2032,10 @@
         <v>132</v>
       </c>
       <c r="AH12" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI12" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:35">
@@ -2103,10 +2106,10 @@
         <v>132</v>
       </c>
       <c r="AH13" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI13" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="14" spans="1:35">
@@ -2177,10 +2180,10 @@
         <v>132</v>
       </c>
       <c r="AH14" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="15" spans="1:35">
@@ -2251,10 +2254,10 @@
         <v>133</v>
       </c>
       <c r="AH15" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI15" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" spans="1:35">
@@ -2325,10 +2328,10 @@
         <v>134</v>
       </c>
       <c r="AH16" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI16" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17" spans="1:35">
@@ -2399,10 +2402,10 @@
         <v>134</v>
       </c>
       <c r="AH17" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI17" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="18" spans="1:35">
@@ -2473,10 +2476,10 @@
         <v>134</v>
       </c>
       <c r="AH18" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI18" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="19" spans="1:35">
@@ -2547,10 +2550,10 @@
         <v>136</v>
       </c>
       <c r="AH19" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI19" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="20" spans="1:35">
@@ -2621,10 +2624,10 @@
         <v>136</v>
       </c>
       <c r="AH20" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI20" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="21" spans="1:35">
@@ -2695,10 +2698,10 @@
         <v>135</v>
       </c>
       <c r="AH21" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI21" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="22" spans="1:35">
@@ -2775,10 +2778,10 @@
         <v>136</v>
       </c>
       <c r="AH22" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI22" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="23" spans="1:35">
@@ -2855,10 +2858,10 @@
         <v>137</v>
       </c>
       <c r="AH23" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI23" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="24" spans="1:35">
@@ -2935,10 +2938,10 @@
         <v>138</v>
       </c>
       <c r="AH24" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI24" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="25" spans="1:35">
@@ -3009,10 +3012,10 @@
         <v>139</v>
       </c>
       <c r="AH25" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI25" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="26" spans="1:35">
@@ -3089,10 +3092,10 @@
         <v>136</v>
       </c>
       <c r="AH26" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI26" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="27" spans="1:35">
@@ -3163,10 +3166,10 @@
         <v>137</v>
       </c>
       <c r="AH27" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI27" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="28" spans="1:35">
@@ -3243,10 +3246,10 @@
         <v>140</v>
       </c>
       <c r="AH28" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI28" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="29" spans="1:35">
@@ -3323,10 +3326,10 @@
         <v>136</v>
       </c>
       <c r="AH29" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI29" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="30" spans="1:35">
@@ -3403,10 +3406,10 @@
         <v>136</v>
       </c>
       <c r="AH30" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI30" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="31" spans="1:35">
@@ -3483,10 +3486,10 @@
         <v>136</v>
       </c>
       <c r="AH31" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI31" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="32" spans="1:35">
@@ -3563,10 +3566,10 @@
         <v>135</v>
       </c>
       <c r="AH32" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI32" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="33" spans="1:35">
@@ -3643,10 +3646,10 @@
         <v>141</v>
       </c>
       <c r="AH33" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="34" spans="1:35">
@@ -3723,10 +3726,10 @@
         <v>137</v>
       </c>
       <c r="AH34" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI34" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="35" spans="1:35">
@@ -3803,10 +3806,10 @@
         <v>138</v>
       </c>
       <c r="AH35" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI35" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="36" spans="1:35">
@@ -3883,10 +3886,10 @@
         <v>140</v>
       </c>
       <c r="AH36" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI36" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="37" spans="1:35">
@@ -3963,10 +3966,10 @@
         <v>136</v>
       </c>
       <c r="AH37" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI37" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="38" spans="1:35">
@@ -4043,10 +4046,10 @@
         <v>136</v>
       </c>
       <c r="AH38" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI38" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="39" spans="1:35">
@@ -4123,10 +4126,10 @@
         <v>136</v>
       </c>
       <c r="AH39" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI39" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="40" spans="1:35">
@@ -4197,10 +4200,10 @@
         <v>135</v>
       </c>
       <c r="AH40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="41" spans="1:35">
@@ -4271,10 +4274,10 @@
         <v>141</v>
       </c>
       <c r="AH41" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI41" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="42" spans="1:35">
@@ -4345,10 +4348,10 @@
         <v>137</v>
       </c>
       <c r="AH42" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI42" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="43" spans="1:35">
@@ -4419,10 +4422,10 @@
         <v>138</v>
       </c>
       <c r="AH43" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI43" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="44" spans="1:35">
@@ -4493,10 +4496,10 @@
         <v>139</v>
       </c>
       <c r="AH44" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI44" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="45" spans="1:35">
@@ -4573,10 +4576,10 @@
         <v>136</v>
       </c>
       <c r="AH45" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI45" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="46" spans="1:35">
@@ -4653,10 +4656,10 @@
         <v>136</v>
       </c>
       <c r="AH46" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI46" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="47" spans="1:35">
@@ -4733,10 +4736,10 @@
         <v>136</v>
       </c>
       <c r="AH47" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI47" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="48" spans="1:35">
@@ -4813,10 +4816,10 @@
         <v>135</v>
       </c>
       <c r="AH48" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI48" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="49" spans="1:35">
@@ -4893,10 +4896,10 @@
         <v>140</v>
       </c>
       <c r="AH49" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="50" spans="1:35">
@@ -4973,10 +4976,10 @@
         <v>141</v>
       </c>
       <c r="AH50" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI50" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="51" spans="1:35">
@@ -5053,10 +5056,10 @@
         <v>140</v>
       </c>
       <c r="AH51" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI51" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="52" spans="1:35">
@@ -5133,10 +5136,10 @@
         <v>136</v>
       </c>
       <c r="AH52" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI52" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="53" spans="1:35">
@@ -5213,10 +5216,10 @@
         <v>136</v>
       </c>
       <c r="AH53" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI53" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="54" spans="1:35">
@@ -5293,10 +5296,10 @@
         <v>136</v>
       </c>
       <c r="AH54" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI54" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="55" spans="1:35">
@@ -5367,10 +5370,10 @@
         <v>135</v>
       </c>
       <c r="AH55" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI55" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="56" spans="1:35">
@@ -5447,10 +5450,10 @@
         <v>141</v>
       </c>
       <c r="AH56" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI56" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57" spans="1:35">
@@ -5527,10 +5530,10 @@
         <v>137</v>
       </c>
       <c r="AH57" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI57" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="58" spans="1:35">
@@ -5607,10 +5610,10 @@
         <v>138</v>
       </c>
       <c r="AH58" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI58" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="59" spans="1:35">
@@ -5687,10 +5690,10 @@
         <v>136</v>
       </c>
       <c r="AH59" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI59" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="60" spans="1:35">
@@ -5767,10 +5770,10 @@
         <v>140</v>
       </c>
       <c r="AH60" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI60" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="61" spans="1:35">
@@ -5847,10 +5850,10 @@
         <v>136</v>
       </c>
       <c r="AH61" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI61" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="62" spans="1:35">
@@ -5927,10 +5930,10 @@
         <v>136</v>
       </c>
       <c r="AH62" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI62" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="63" spans="1:35">
@@ -6007,10 +6010,10 @@
         <v>136</v>
       </c>
       <c r="AH63" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI63" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="64" spans="1:35">
@@ -6081,10 +6084,10 @@
         <v>135</v>
       </c>
       <c r="AH64" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI64" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="65" spans="1:35">
@@ -6161,10 +6164,10 @@
         <v>141</v>
       </c>
       <c r="AH65" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI65" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="66" spans="1:35">
@@ -6241,10 +6244,10 @@
         <v>137</v>
       </c>
       <c r="AH66" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI66" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="67" spans="1:35">
@@ -6321,10 +6324,10 @@
         <v>138</v>
       </c>
       <c r="AH67" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI67" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="68" spans="1:35">
@@ -6395,10 +6398,10 @@
         <v>136</v>
       </c>
       <c r="AH68" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI68" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="69" spans="1:35">
@@ -6469,10 +6472,10 @@
         <v>142</v>
       </c>
       <c r="AH69" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI69" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="70" spans="1:35">
@@ -6543,10 +6546,10 @@
         <v>143</v>
       </c>
       <c r="AH70" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI70" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="71" spans="1:35">
@@ -6617,10 +6620,10 @@
         <v>143</v>
       </c>
       <c r="AH71" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI71" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="72" spans="1:35">
@@ -6691,10 +6694,10 @@
         <v>142</v>
       </c>
       <c r="AH72" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI72" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="73" spans="1:35">
@@ -6765,10 +6768,10 @@
         <v>143</v>
       </c>
       <c r="AH73" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI73" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="74" spans="1:35">
@@ -6839,10 +6842,10 @@
         <v>142</v>
       </c>
       <c r="AH74" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI74" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="75" spans="1:35">
@@ -6913,10 +6916,10 @@
         <v>143</v>
       </c>
       <c r="AH75" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI75" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="76" spans="1:35">
@@ -6987,10 +6990,10 @@
         <v>144</v>
       </c>
       <c r="AH76" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI76" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="77" spans="1:35">
@@ -7061,10 +7064,10 @@
         <v>142</v>
       </c>
       <c r="AH77" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI77" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="78" spans="1:35">
@@ -7135,10 +7138,10 @@
         <v>143</v>
       </c>
       <c r="AH78" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI78" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="79" spans="1:35">
@@ -7209,10 +7212,10 @@
         <v>144</v>
       </c>
       <c r="AH79" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI79" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="80" spans="1:35">
@@ -7283,10 +7286,10 @@
         <v>142</v>
       </c>
       <c r="AH80" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI80" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="81" spans="1:35">
@@ -7357,10 +7360,10 @@
         <v>143</v>
       </c>
       <c r="AH81" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI81" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="82" spans="1:35">
@@ -7431,10 +7434,10 @@
         <v>143</v>
       </c>
       <c r="AH82" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI82" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="83" spans="1:35">
@@ -7505,10 +7508,10 @@
         <v>158</v>
       </c>
       <c r="AH83" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI83" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="84" spans="1:35">
@@ -7579,10 +7582,10 @@
         <v>143</v>
       </c>
       <c r="AH84" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI84" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="85" spans="1:35">
@@ -7653,10 +7656,10 @@
         <v>142</v>
       </c>
       <c r="AH85" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI85" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="86" spans="1:35">
@@ -7727,10 +7730,10 @@
         <v>143</v>
       </c>
       <c r="AH86" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI86" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="87" spans="1:35">
@@ -7801,10 +7804,10 @@
         <v>144</v>
       </c>
       <c r="AH87" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI87" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="88" spans="1:35">
@@ -7875,10 +7878,10 @@
         <v>158</v>
       </c>
       <c r="AH88" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI88" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="89" spans="1:35">
@@ -7949,10 +7952,10 @@
         <v>142</v>
       </c>
       <c r="AH89" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI89" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="90" spans="1:35">
@@ -8023,10 +8026,10 @@
         <v>143</v>
       </c>
       <c r="AH90" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI90" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="91" spans="1:35">
@@ -8097,10 +8100,10 @@
         <v>143</v>
       </c>
       <c r="AH91" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI91" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="92" spans="1:35">
@@ -8171,10 +8174,10 @@
         <v>143</v>
       </c>
       <c r="AH92" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI92" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="93" spans="1:35">
@@ -8245,10 +8248,10 @@
         <v>143</v>
       </c>
       <c r="AH93" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI93" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="94" spans="1:35">
@@ -8319,10 +8322,10 @@
         <v>142</v>
       </c>
       <c r="AH94" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI94" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="95" spans="1:35">
@@ -8393,10 +8396,10 @@
         <v>143</v>
       </c>
       <c r="AH95" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI95" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="96" spans="1:35">
@@ -8467,10 +8470,10 @@
         <v>143</v>
       </c>
       <c r="AH96" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI96" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="97" spans="1:35">
@@ -8541,10 +8544,10 @@
         <v>142</v>
       </c>
       <c r="AH97" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI97" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="98" spans="1:35">
@@ -8615,10 +8618,10 @@
         <v>143</v>
       </c>
       <c r="AH98" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI98" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="99" spans="1:35">
@@ -8689,10 +8692,10 @@
         <v>144</v>
       </c>
       <c r="AH99" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI99" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="100" spans="1:35">
@@ -8763,10 +8766,10 @@
         <v>142</v>
       </c>
       <c r="AH100" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI100" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="101" spans="1:35">
@@ -8837,10 +8840,10 @@
         <v>143</v>
       </c>
       <c r="AH101" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI101" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="102" spans="1:35">
@@ -8911,10 +8914,10 @@
         <v>144</v>
       </c>
       <c r="AH102" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI102" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="103" spans="1:35">
@@ -8991,10 +8994,10 @@
         <v>143</v>
       </c>
       <c r="AH103" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI103" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="104" spans="1:35">
@@ -9068,10 +9071,10 @@
         <v>143</v>
       </c>
       <c r="AH104" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI104" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="105" spans="1:35">
@@ -9145,10 +9148,10 @@
         <v>145</v>
       </c>
       <c r="AH105" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI105" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="106" spans="1:35">
@@ -9222,10 +9225,10 @@
         <v>143</v>
       </c>
       <c r="AH106" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI106" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="107" spans="1:35">
@@ -9302,10 +9305,10 @@
         <v>143</v>
       </c>
       <c r="AH107" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI107" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="108" spans="1:35">
@@ -9379,10 +9382,10 @@
         <v>143</v>
       </c>
       <c r="AH108" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI108" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="109" spans="1:35">
@@ -9456,10 +9459,10 @@
         <v>145</v>
       </c>
       <c r="AH109" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI109" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="110" spans="1:35">
@@ -9530,10 +9533,10 @@
         <v>147</v>
       </c>
       <c r="AH110" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI110" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="111" spans="1:35">
@@ -9604,10 +9607,10 @@
         <v>147</v>
       </c>
       <c r="AH111" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI111" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="112" spans="1:35">
@@ -9678,10 +9681,10 @@
         <v>147</v>
       </c>
       <c r="AH112" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI112" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="113" spans="1:35">
@@ -9752,10 +9755,10 @@
         <v>147</v>
       </c>
       <c r="AH113" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI113" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="114" spans="1:35">
@@ -9826,10 +9829,10 @@
         <v>147</v>
       </c>
       <c r="AH114" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI114" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="115" spans="1:35">
@@ -9900,10 +9903,10 @@
         <v>147</v>
       </c>
       <c r="AH115" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI115" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="116" spans="1:35">
@@ -9974,10 +9977,10 @@
         <v>147</v>
       </c>
       <c r="AH116" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI116" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="117" spans="1:35">
@@ -10048,10 +10051,10 @@
         <v>147</v>
       </c>
       <c r="AH117" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI117" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="118" spans="1:35">
@@ -10122,10 +10125,10 @@
         <v>147</v>
       </c>
       <c r="AH118" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI118" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="119" spans="1:35">
@@ -10196,10 +10199,10 @@
         <v>147</v>
       </c>
       <c r="AH119" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI119" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="120" spans="1:35">
@@ -10270,10 +10273,10 @@
         <v>147</v>
       </c>
       <c r="AH120" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI120" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="121" spans="1:35">
@@ -10344,10 +10347,10 @@
         <v>147</v>
       </c>
       <c r="AH121" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI121" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="122" spans="1:35">
@@ -10418,10 +10421,10 @@
         <v>147</v>
       </c>
       <c r="AH122" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI122" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="123" spans="1:35">
@@ -10492,10 +10495,10 @@
         <v>147</v>
       </c>
       <c r="AH123" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI123" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="124" spans="1:35">
@@ -10566,10 +10569,10 @@
         <v>147</v>
       </c>
       <c r="AH124" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI124" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="125" spans="1:35">
@@ -10640,10 +10643,10 @@
         <v>147</v>
       </c>
       <c r="AH125" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI125" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="126" spans="1:35">
@@ -10714,10 +10717,10 @@
         <v>147</v>
       </c>
       <c r="AH126" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI126" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="127" spans="1:35">
@@ -10788,10 +10791,10 @@
         <v>147</v>
       </c>
       <c r="AH127" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI127" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="128" spans="1:35">
@@ -10862,10 +10865,10 @@
         <v>147</v>
       </c>
       <c r="AH128" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI128" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="129" spans="1:35">
@@ -10936,10 +10939,10 @@
         <v>147</v>
       </c>
       <c r="AH129" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI129" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="130" spans="1:35">
@@ -11010,10 +11013,10 @@
         <v>147</v>
       </c>
       <c r="AH130" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI130" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="131" spans="1:35">
@@ -11084,10 +11087,10 @@
         <v>147</v>
       </c>
       <c r="AH131" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI131" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="132" spans="1:35">
@@ -11158,10 +11161,10 @@
         <v>147</v>
       </c>
       <c r="AH132" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI132" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="133" spans="1:35">
@@ -11232,10 +11235,10 @@
         <v>147</v>
       </c>
       <c r="AH133" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI133" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="134" spans="1:35">
@@ -11306,10 +11309,10 @@
         <v>148</v>
       </c>
       <c r="AH134" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI134" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="135" spans="1:35">
@@ -11380,10 +11383,10 @@
         <v>148</v>
       </c>
       <c r="AH135" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI135" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="136" spans="1:35">
@@ -11454,10 +11457,10 @@
         <v>148</v>
       </c>
       <c r="AH136" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI136" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="137" spans="1:35">
@@ -11528,10 +11531,10 @@
         <v>148</v>
       </c>
       <c r="AH137" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI137" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="138" spans="1:35">
@@ -11602,10 +11605,10 @@
         <v>148</v>
       </c>
       <c r="AH138" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI138" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="139" spans="1:35">
@@ -11676,10 +11679,10 @@
         <v>149</v>
       </c>
       <c r="AH139" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI139" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="140" spans="1:35">
@@ -11750,10 +11753,10 @@
         <v>148</v>
       </c>
       <c r="AH140" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI140" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="141" spans="1:35">
@@ -11824,10 +11827,10 @@
         <v>148</v>
       </c>
       <c r="AH141" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI141" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="142" spans="1:35">
@@ -11898,10 +11901,10 @@
         <v>148</v>
       </c>
       <c r="AH142" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI142" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="143" spans="1:35">
@@ -11972,10 +11975,10 @@
         <v>148</v>
       </c>
       <c r="AH143" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI143" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="144" spans="1:35">
@@ -12046,10 +12049,10 @@
         <v>149</v>
       </c>
       <c r="AH144" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI144" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="145" spans="1:35">
@@ -12120,10 +12123,10 @@
         <v>149</v>
       </c>
       <c r="AH145" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI145" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="146" spans="1:35">
@@ -12194,10 +12197,10 @@
         <v>148</v>
       </c>
       <c r="AH146" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI146" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="147" spans="1:35">
@@ -12268,10 +12271,10 @@
         <v>149</v>
       </c>
       <c r="AH147" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI147" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="148" spans="1:35">
@@ -12342,10 +12345,10 @@
         <v>148</v>
       </c>
       <c r="AH148" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI148" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="149" spans="1:35">
@@ -12416,10 +12419,10 @@
         <v>148</v>
       </c>
       <c r="AH149" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI149" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="150" spans="1:35">
@@ -12490,10 +12493,10 @@
         <v>148</v>
       </c>
       <c r="AH150" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI150" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="151" spans="1:35">
@@ -12564,10 +12567,10 @@
         <v>148</v>
       </c>
       <c r="AH151" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI151" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="152" spans="1:35">
@@ -12638,10 +12641,10 @@
         <v>149</v>
       </c>
       <c r="AH152" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI152" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="153" spans="1:35">
@@ -12712,10 +12715,10 @@
         <v>148</v>
       </c>
       <c r="AH153" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI153" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="154" spans="1:35">
@@ -12783,10 +12786,10 @@
         <v>148</v>
       </c>
       <c r="AH154" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI154" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="155" spans="1:35">
@@ -12854,10 +12857,10 @@
         <v>148</v>
       </c>
       <c r="AH155" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI155" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="156" spans="1:35">
@@ -12925,10 +12928,10 @@
         <v>148</v>
       </c>
       <c r="AH156" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI156" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="157" spans="1:35">
@@ -12996,10 +12999,10 @@
         <v>148</v>
       </c>
       <c r="AH157" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI157" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="158" spans="1:35">
@@ -13067,10 +13070,10 @@
         <v>148</v>
       </c>
       <c r="AH158" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI158" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="159" spans="1:35">
@@ -13138,10 +13141,10 @@
         <v>148</v>
       </c>
       <c r="AH159" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI159" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="160" spans="1:35">
@@ -13209,10 +13212,10 @@
         <v>149</v>
       </c>
       <c r="AH160" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI160" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="161" spans="1:35">
@@ -13280,10 +13283,10 @@
         <v>148</v>
       </c>
       <c r="AH161" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI161" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="162" spans="1:35">
@@ -13351,10 +13354,10 @@
         <v>148</v>
       </c>
       <c r="AH162" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI162" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="163" spans="1:35">
@@ -13422,10 +13425,10 @@
         <v>148</v>
       </c>
       <c r="AH163" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI163" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="164" spans="1:35">
@@ -13493,10 +13496,10 @@
         <v>148</v>
       </c>
       <c r="AH164" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI164" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="165" spans="1:35">
@@ -13564,10 +13567,10 @@
         <v>148</v>
       </c>
       <c r="AH165" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI165" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="166" spans="1:35">
@@ -13635,10 +13638,10 @@
         <v>148</v>
       </c>
       <c r="AH166" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI166" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="167" spans="1:35">
@@ -13706,10 +13709,10 @@
         <v>148</v>
       </c>
       <c r="AH167" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI167" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="168" spans="1:35">
@@ -13783,10 +13786,10 @@
         <v>148</v>
       </c>
       <c r="AH168" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI168" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="169" spans="1:35">
@@ -13860,10 +13863,10 @@
         <v>148</v>
       </c>
       <c r="AH169" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI169" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="170" spans="1:35">
@@ -13937,10 +13940,10 @@
         <v>148</v>
       </c>
       <c r="AH170" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI170" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="171" spans="1:35">
@@ -14014,10 +14017,10 @@
         <v>148</v>
       </c>
       <c r="AH171" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI171" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="172" spans="1:35">
@@ -14091,10 +14094,10 @@
         <v>148</v>
       </c>
       <c r="AH172" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI172" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="173" spans="1:35">
@@ -14168,10 +14171,10 @@
         <v>148</v>
       </c>
       <c r="AH173" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI173" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="174" spans="1:35">
@@ -14245,10 +14248,10 @@
         <v>149</v>
       </c>
       <c r="AH174" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI174" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="175" spans="1:35">
@@ -14322,10 +14325,10 @@
         <v>148</v>
       </c>
       <c r="AH175" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI175" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="176" spans="1:35">
@@ -14399,10 +14402,10 @@
         <v>148</v>
       </c>
       <c r="AH176" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI176" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="177" spans="1:35">
@@ -14476,10 +14479,10 @@
         <v>148</v>
       </c>
       <c r="AH177" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI177" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="178" spans="1:35">
@@ -14553,10 +14556,10 @@
         <v>148</v>
       </c>
       <c r="AH178" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI178" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="179" spans="1:35">
@@ -14624,10 +14627,10 @@
         <v>148</v>
       </c>
       <c r="AH179" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI179" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="180" spans="1:35">
@@ -14695,10 +14698,10 @@
         <v>148</v>
       </c>
       <c r="AH180" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI180" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="181" spans="1:35">
@@ -14766,10 +14769,10 @@
         <v>148</v>
       </c>
       <c r="AH181" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI181" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="182" spans="1:35">
@@ -14837,10 +14840,10 @@
         <v>148</v>
       </c>
       <c r="AH182" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI182" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="183" spans="1:35">
@@ -14908,10 +14911,10 @@
         <v>148</v>
       </c>
       <c r="AH183" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI183" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="184" spans="1:35">
@@ -14979,10 +14982,10 @@
         <v>148</v>
       </c>
       <c r="AH184" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI184" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="185" spans="1:35">
@@ -15050,10 +15053,10 @@
         <v>148</v>
       </c>
       <c r="AH185" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI185" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="186" spans="1:35">
@@ -15121,10 +15124,10 @@
         <v>54</v>
       </c>
       <c r="AH186" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI186" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="187" spans="1:35">
@@ -15192,10 +15195,10 @@
         <v>54</v>
       </c>
       <c r="AH187" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI187" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="188" spans="1:35">
@@ -15263,10 +15266,10 @@
         <v>54</v>
       </c>
       <c r="AH188" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI188" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="189" spans="1:35">
@@ -15334,10 +15337,10 @@
         <v>54</v>
       </c>
       <c r="AH189" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI189" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="190" spans="1:35">
@@ -15405,10 +15408,10 @@
         <v>53</v>
       </c>
       <c r="AH190" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI190" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="191" spans="1:35">
@@ -15476,10 +15479,10 @@
         <v>53</v>
       </c>
       <c r="AH191" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI191" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="192" spans="1:35">
@@ -15547,10 +15550,10 @@
         <v>54</v>
       </c>
       <c r="AH192" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI192" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="193" spans="1:35">
@@ -15618,10 +15621,10 @@
         <v>54</v>
       </c>
       <c r="AH193" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI193" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="194" spans="1:35">
@@ -15689,10 +15692,10 @@
         <v>54</v>
       </c>
       <c r="AH194" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI194" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="195" spans="1:35">
@@ -15760,10 +15763,10 @@
         <v>150</v>
       </c>
       <c r="AH195" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI195" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="196" spans="1:35">
@@ -15831,10 +15834,10 @@
         <v>54</v>
       </c>
       <c r="AH196" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI196" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="197" spans="1:35">
@@ -15902,10 +15905,10 @@
         <v>54</v>
       </c>
       <c r="AH197" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI197" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="198" spans="1:35">
@@ -15973,10 +15976,10 @@
         <v>54</v>
       </c>
       <c r="AH198" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI198" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="199" spans="1:35">
@@ -16044,10 +16047,10 @@
         <v>54</v>
       </c>
       <c r="AH199" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI199" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="200" spans="1:35">
@@ -16115,10 +16118,10 @@
         <v>54</v>
       </c>
       <c r="AH200" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI200" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="201" spans="1:35">
@@ -16186,10 +16189,10 @@
         <v>54</v>
       </c>
       <c r="AH201" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI201" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="202" spans="1:35">
@@ -16257,10 +16260,10 @@
         <v>54</v>
       </c>
       <c r="AH202" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI202" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="203" spans="1:35">
@@ -16328,10 +16331,10 @@
         <v>54</v>
       </c>
       <c r="AH203" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI203" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="204" spans="1:35">
@@ -16399,10 +16402,10 @@
         <v>53</v>
       </c>
       <c r="AH204" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI204" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="205" spans="1:35">
@@ -16470,10 +16473,10 @@
         <v>53</v>
       </c>
       <c r="AH205" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI205" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="206" spans="1:35">
@@ -16541,24 +16544,24 @@
         <v>54</v>
       </c>
       <c r="AH206" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI206" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="207" spans="1:35">
       <c r="A207">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B207" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C207" t="s">
         <v>49</v>
       </c>
       <c r="D207" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E207" t="s">
         <v>54</v>
@@ -16581,6 +16584,9 @@
       <c r="N207" s="1">
         <v>46300</v>
       </c>
+      <c r="O207" t="s">
+        <v>126</v>
+      </c>
       <c r="P207">
         <v>10</v>
       </c>
@@ -16588,16 +16594,16 @@
         <v>2026</v>
       </c>
       <c r="R207">
-        <v>17952581</v>
+        <v>17952401</v>
       </c>
       <c r="S207" t="s">
         <v>54</v>
       </c>
       <c r="U207" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="V207" s="1">
-        <v>46300.6768006713</v>
+        <v>46302.51963612268</v>
       </c>
       <c r="W207">
         <v>2</v>
@@ -16605,25 +16611,28 @@
       <c r="X207" t="s">
         <v>170</v>
       </c>
+      <c r="Y207" t="s">
+        <v>233</v>
+      </c>
       <c r="AB207">
         <v>0</v>
       </c>
       <c r="AC207" t="s">
-        <v>54</v>
+        <v>150</v>
       </c>
       <c r="AH207" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI207" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="208" spans="1:35">
       <c r="A208">
-        <v>6945</v>
+        <v>6705</v>
       </c>
       <c r="B208" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C208" t="s">
         <v>49</v>
@@ -16635,7 +16644,7 @@
         <v>54</v>
       </c>
       <c r="F208" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G208">
         <v>6215</v>
@@ -16659,7 +16668,7 @@
         <v>2026</v>
       </c>
       <c r="R208">
-        <v>18164524</v>
+        <v>17952581</v>
       </c>
       <c r="S208" t="s">
         <v>54</v>
@@ -16668,13 +16677,13 @@
         <v>162</v>
       </c>
       <c r="V208" s="1">
-        <v>46300.6769528125</v>
+        <v>46300.6768006713</v>
       </c>
       <c r="W208">
         <v>2</v>
       </c>
       <c r="X208" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="AB208">
         <v>0</v>
@@ -16683,24 +16692,24 @@
         <v>54</v>
       </c>
       <c r="AH208" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI208" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="209" spans="1:35">
       <c r="A209">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B209" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C209" t="s">
         <v>49</v>
       </c>
       <c r="D209" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E209" t="s">
         <v>54</v>
@@ -16730,7 +16739,7 @@
         <v>2026</v>
       </c>
       <c r="R209">
-        <v>18178164</v>
+        <v>18164524</v>
       </c>
       <c r="S209" t="s">
         <v>54</v>
@@ -16739,13 +16748,13 @@
         <v>162</v>
       </c>
       <c r="V209" s="1">
-        <v>46300.67696615741</v>
+        <v>46300.6769528125</v>
       </c>
       <c r="W209">
         <v>2</v>
       </c>
       <c r="X209" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AB209">
         <v>0</v>
@@ -16754,33 +16763,33 @@
         <v>54</v>
       </c>
       <c r="AH209" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AI209" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="210" spans="1:35">
       <c r="A210">
-        <v>6404</v>
+        <v>6949</v>
       </c>
       <c r="B210" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C210" t="s">
         <v>49</v>
       </c>
       <c r="D210" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E210" t="s">
         <v>54</v>
       </c>
       <c r="F210" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G210">
-        <v>11001</v>
+        <v>6215</v>
       </c>
       <c r="H210">
         <v>0</v>
@@ -16789,10 +16798,10 @@
         <v>63</v>
       </c>
       <c r="J210" t="s">
-        <v>69</v>
+        <v>119</v>
       </c>
       <c r="N210" s="1">
-        <v>46351</v>
+        <v>46300</v>
       </c>
       <c r="P210">
         <v>10</v>
@@ -16801,25 +16810,22 @@
         <v>2026</v>
       </c>
       <c r="R210">
-        <v>16962456</v>
+        <v>18178164</v>
       </c>
       <c r="S210" t="s">
         <v>54</v>
       </c>
       <c r="U210" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="V210" s="1">
-        <v>46296.34114513889</v>
+        <v>46300.67696615741</v>
       </c>
       <c r="W210">
-        <v>-49</v>
+        <v>2</v>
       </c>
       <c r="X210" t="s">
-        <v>168</v>
-      </c>
-      <c r="Y210" t="s">
-        <v>233</v>
+        <v>166</v>
       </c>
       <c r="AB210">
         <v>0</v>
@@ -16828,7 +16834,7 @@
         <v>54</v>
       </c>
       <c r="AH210" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="AI210" t="s">
         <v>244</v>
@@ -16836,16 +16842,16 @@
     </row>
     <row r="211" spans="1:35">
       <c r="A211">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B211" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C211" t="s">
         <v>49</v>
       </c>
       <c r="D211" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E211" t="s">
         <v>54</v>
@@ -16854,7 +16860,7 @@
         <v>55</v>
       </c>
       <c r="G211">
-        <v>7877</v>
+        <v>11001</v>
       </c>
       <c r="H211">
         <v>0</v>
@@ -16863,7 +16869,7 @@
         <v>63</v>
       </c>
       <c r="J211" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="N211" s="1">
         <v>46351</v>
@@ -16875,7 +16881,7 @@
         <v>2026</v>
       </c>
       <c r="R211">
-        <v>17399332</v>
+        <v>16962456</v>
       </c>
       <c r="S211" t="s">
         <v>54</v>
@@ -16884,13 +16890,13 @@
         <v>161</v>
       </c>
       <c r="V211" s="1">
-        <v>46296.34050315972</v>
+        <v>46296.34114513889</v>
       </c>
       <c r="W211">
         <v>-49</v>
       </c>
       <c r="X211" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Y211" t="s">
         <v>234</v>
@@ -16902,18 +16908,18 @@
         <v>54</v>
       </c>
       <c r="AH211" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI211" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="212" spans="1:35">
       <c r="A212">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B212" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C212" t="s">
         <v>49</v>
@@ -16928,7 +16934,7 @@
         <v>55</v>
       </c>
       <c r="G212">
-        <v>9774</v>
+        <v>7877</v>
       </c>
       <c r="H212">
         <v>0</v>
@@ -16937,34 +16943,34 @@
         <v>63</v>
       </c>
       <c r="J212" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="N212" s="1">
-        <v>46290</v>
+        <v>46351</v>
       </c>
       <c r="P212">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q212">
         <v>2026</v>
       </c>
       <c r="R212">
-        <v>16976321</v>
+        <v>17399332</v>
       </c>
       <c r="S212" t="s">
         <v>54</v>
       </c>
       <c r="U212" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="V212" s="1">
-        <v>46296.39309459491</v>
+        <v>46296.34050315972</v>
       </c>
       <c r="W212">
-        <v>12</v>
+        <v>-49</v>
       </c>
       <c r="X212" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="Y212" t="s">
         <v>235</v>
@@ -16976,10 +16982,10 @@
         <v>54</v>
       </c>
       <c r="AH212" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI212" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="213" spans="1:35">
@@ -17014,28 +17020,28 @@
         <v>66</v>
       </c>
       <c r="N213" s="1">
-        <v>46351</v>
+        <v>46290</v>
       </c>
       <c r="P213">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Q213">
         <v>2026</v>
       </c>
       <c r="R213">
-        <v>16976323</v>
+        <v>16976321</v>
       </c>
       <c r="S213" t="s">
         <v>54</v>
       </c>
       <c r="U213" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="V213" s="1">
-        <v>46296.3409153125</v>
+        <v>46296.39309459491</v>
       </c>
       <c r="W213">
-        <v>-49</v>
+        <v>12</v>
       </c>
       <c r="X213" t="s">
         <v>171</v>
@@ -17050,18 +17056,18 @@
         <v>54</v>
       </c>
       <c r="AH213" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI213" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="214" spans="1:35">
       <c r="A214">
-        <v>5417</v>
+        <v>6486</v>
       </c>
       <c r="B214" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C214" t="s">
         <v>49</v>
@@ -17076,7 +17082,7 @@
         <v>55</v>
       </c>
       <c r="G214">
-        <v>7027</v>
+        <v>9774</v>
       </c>
       <c r="H214">
         <v>0</v>
@@ -17085,10 +17091,10 @@
         <v>63</v>
       </c>
       <c r="J214" t="s">
-        <v>120</v>
+        <v>66</v>
       </c>
       <c r="N214" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="P214">
         <v>10</v>
@@ -17097,7 +17103,7 @@
         <v>2026</v>
       </c>
       <c r="R214">
-        <v>17399292</v>
+        <v>16976323</v>
       </c>
       <c r="S214" t="s">
         <v>54</v>
@@ -17106,13 +17112,16 @@
         <v>161</v>
       </c>
       <c r="V214" s="1">
-        <v>46296.0420403125</v>
+        <v>46296.3409153125</v>
       </c>
       <c r="W214">
-        <v>-48</v>
+        <v>-49</v>
       </c>
       <c r="X214" t="s">
-        <v>169</v>
+        <v>171</v>
+      </c>
+      <c r="Y214" t="s">
+        <v>237</v>
       </c>
       <c r="AB214">
         <v>0</v>
@@ -17121,24 +17130,24 @@
         <v>54</v>
       </c>
       <c r="AH214" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI214" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="215" spans="1:35">
       <c r="A215">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B215" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C215" t="s">
         <v>49</v>
       </c>
       <c r="D215" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E215" t="s">
         <v>54</v>
@@ -17168,7 +17177,7 @@
         <v>2026</v>
       </c>
       <c r="R215">
-        <v>16962350</v>
+        <v>17399292</v>
       </c>
       <c r="S215" t="s">
         <v>54</v>
@@ -17183,7 +17192,7 @@
         <v>-48</v>
       </c>
       <c r="X215" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="AB215">
         <v>0</v>
@@ -17192,10 +17201,10 @@
         <v>54</v>
       </c>
       <c r="AH215" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI215" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="216" spans="1:35">
@@ -17218,78 +17227,75 @@
         <v>55</v>
       </c>
       <c r="G216">
-        <v>11056</v>
+        <v>7027</v>
       </c>
       <c r="H216">
         <v>0</v>
       </c>
       <c r="I216" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J216" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="N216" s="1">
-        <v>46301</v>
-      </c>
-      <c r="O216" t="s">
-        <v>124</v>
+        <v>46350</v>
       </c>
       <c r="P216">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q216">
         <v>2026</v>
       </c>
       <c r="R216">
-        <v>18288551</v>
+        <v>16962350</v>
+      </c>
+      <c r="S216" t="s">
+        <v>54</v>
       </c>
       <c r="U216" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="V216" s="1">
-        <v>46301.49091145834</v>
+        <v>46296.0420403125</v>
       </c>
       <c r="W216">
-        <v>1</v>
+        <v>-48</v>
       </c>
       <c r="X216" t="s">
         <v>168</v>
       </c>
-      <c r="Y216" t="s">
-        <v>237</v>
-      </c>
       <c r="AB216">
         <v>0</v>
       </c>
       <c r="AC216" t="s">
-        <v>239</v>
+        <v>54</v>
       </c>
       <c r="AH216" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI216" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="217" spans="1:35">
       <c r="A217">
-        <v>6949</v>
+        <v>6404</v>
       </c>
       <c r="B217" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C217" t="s">
         <v>49</v>
       </c>
       <c r="D217" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E217" t="s">
         <v>54</v>
       </c>
       <c r="F217" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G217">
         <v>11056</v>
@@ -17304,10 +17310,10 @@
         <v>121</v>
       </c>
       <c r="N217" s="1">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="O217" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P217">
         <v>9</v>
@@ -17316,19 +17322,19 @@
         <v>2026</v>
       </c>
       <c r="R217">
-        <v>18286473</v>
+        <v>18288551</v>
       </c>
       <c r="U217" t="s">
         <v>162</v>
       </c>
       <c r="V217" s="1">
-        <v>46297.49393364583</v>
+        <v>46301.49091145834</v>
       </c>
       <c r="W217">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="X217" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="Y217" t="s">
         <v>238</v>
@@ -17337,13 +17343,87 @@
         <v>0</v>
       </c>
       <c r="AC217" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="AH217" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AI217" t="s">
         <v>244</v>
+      </c>
+    </row>
+    <row r="218" spans="1:35">
+      <c r="A218">
+        <v>6949</v>
+      </c>
+      <c r="B218" t="s">
+        <v>39</v>
+      </c>
+      <c r="C218" t="s">
+        <v>49</v>
+      </c>
+      <c r="D218" t="s">
+        <v>50</v>
+      </c>
+      <c r="E218" t="s">
+        <v>54</v>
+      </c>
+      <c r="F218" t="s">
+        <v>56</v>
+      </c>
+      <c r="G218">
+        <v>11056</v>
+      </c>
+      <c r="H218">
+        <v>0</v>
+      </c>
+      <c r="I218" t="s">
+        <v>64</v>
+      </c>
+      <c r="J218" t="s">
+        <v>121</v>
+      </c>
+      <c r="N218" s="1">
+        <v>46297</v>
+      </c>
+      <c r="O218" t="s">
+        <v>123</v>
+      </c>
+      <c r="P218">
+        <v>9</v>
+      </c>
+      <c r="Q218">
+        <v>2026</v>
+      </c>
+      <c r="R218">
+        <v>18286473</v>
+      </c>
+      <c r="U218" t="s">
+        <v>162</v>
+      </c>
+      <c r="V218" s="1">
+        <v>46297.49393364583</v>
+      </c>
+      <c r="W218">
+        <v>5</v>
+      </c>
+      <c r="X218" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y218" t="s">
+        <v>239</v>
+      </c>
+      <c r="AB218">
+        <v>0</v>
+      </c>
+      <c r="AC218" t="s">
+        <v>240</v>
+      </c>
+      <c r="AH218" t="s">
+        <v>241</v>
+      </c>
+      <c r="AI218" t="s">
+        <v>245</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-08 08:41
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -1274,7 +1274,7 @@
         <v>46300.43100663194</v>
       </c>
       <c r="W2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X2" t="s">
         <v>163</v>
@@ -1351,7 +1351,7 @@
         <v>46300.3901340625</v>
       </c>
       <c r="W3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X3" t="s">
         <v>163</v>
@@ -1428,7 +1428,7 @@
         <v>46297.71198460648</v>
       </c>
       <c r="W4">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X4" t="s">
         <v>164</v>
@@ -1502,7 +1502,7 @@
         <v>46297.7119869213</v>
       </c>
       <c r="W5">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X5" t="s">
         <v>163</v>
@@ -1576,7 +1576,7 @@
         <v>46297.71198738426</v>
       </c>
       <c r="W6">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X6" t="s">
         <v>163</v>
@@ -1650,7 +1650,7 @@
         <v>46297.71199320602</v>
       </c>
       <c r="W7">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X7" t="s">
         <v>165</v>
@@ -1724,7 +1724,7 @@
         <v>46297.71199371527</v>
       </c>
       <c r="W8">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X8" t="s">
         <v>166</v>
@@ -1798,7 +1798,7 @@
         <v>46297.71199424769</v>
       </c>
       <c r="W9">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X9" t="s">
         <v>167</v>
@@ -1872,7 +1872,7 @@
         <v>46297.71199479167</v>
       </c>
       <c r="W10">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X10" t="s">
         <v>167</v>
@@ -1946,7 +1946,7 @@
         <v>46302.37134707176</v>
       </c>
       <c r="W11">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="X11" t="s">
         <v>168</v>
@@ -2020,7 +2020,7 @@
         <v>46297.69881809028</v>
       </c>
       <c r="W12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X12" t="s">
         <v>168</v>
@@ -2097,7 +2097,7 @@
         <v>46300.38749403935</v>
       </c>
       <c r="W13">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X13" t="s">
         <v>168</v>
@@ -2171,7 +2171,7 @@
         <v>46302.3710765625</v>
       </c>
       <c r="W14">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X14" t="s">
         <v>168</v>
@@ -2245,7 +2245,7 @@
         <v>46297.71197056713</v>
       </c>
       <c r="W15">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X15" t="s">
         <v>169</v>
@@ -2319,7 +2319,7 @@
         <v>46297.71198896991</v>
       </c>
       <c r="W16">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X16" t="s">
         <v>170</v>
@@ -2393,7 +2393,7 @@
         <v>46297.71198950231</v>
       </c>
       <c r="W17">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X17" t="s">
         <v>170</v>
@@ -2467,7 +2467,7 @@
         <v>46297.71199112268</v>
       </c>
       <c r="W18">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X18" t="s">
         <v>170</v>
@@ -2538,7 +2538,7 @@
         <v>46297.68986506944</v>
       </c>
       <c r="W19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X19" t="s">
         <v>171</v>
@@ -2612,7 +2612,7 @@
         <v>46297.68986576389</v>
       </c>
       <c r="W20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X20" t="s">
         <v>163</v>
@@ -2689,7 +2689,7 @@
         <v>46300.68237630787</v>
       </c>
       <c r="W21">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="X21" t="s">
         <v>172</v>
@@ -2766,7 +2766,7 @@
         <v>46300.57769349537</v>
       </c>
       <c r="W22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X22" t="s">
         <v>163</v>
@@ -2846,7 +2846,7 @@
         <v>46300.56213424769</v>
       </c>
       <c r="W23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X23" t="s">
         <v>165</v>
@@ -2926,7 +2926,7 @@
         <v>46301.46998128472</v>
       </c>
       <c r="W24">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X24" t="s">
         <v>166</v>
@@ -3003,7 +3003,7 @@
         <v>46300.75766230324</v>
       </c>
       <c r="W25">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X25" t="s">
         <v>168</v>
@@ -3080,7 +3080,7 @@
         <v>46300.7473044213</v>
       </c>
       <c r="W26">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X26" t="s">
         <v>171</v>
@@ -3160,7 +3160,7 @@
         <v>46302.56370974537</v>
       </c>
       <c r="W27">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X27" t="s">
         <v>163</v>
@@ -3237,7 +3237,7 @@
         <v>46301.75716237268</v>
       </c>
       <c r="W28">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X28" t="s">
         <v>165</v>
@@ -3314,7 +3314,7 @@
         <v>46300.4280221412</v>
       </c>
       <c r="W29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X29" t="s">
         <v>169</v>
@@ -3394,7 +3394,7 @@
         <v>46300.57060454861</v>
       </c>
       <c r="W30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X30" t="s">
         <v>171</v>
@@ -3474,7 +3474,7 @@
         <v>46301.60203489583</v>
       </c>
       <c r="W31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X31" t="s">
         <v>163</v>
@@ -3554,7 +3554,7 @@
         <v>46301.60118045139</v>
       </c>
       <c r="W32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X32" t="s">
         <v>163</v>
@@ -3634,7 +3634,7 @@
         <v>46300.67849611111</v>
       </c>
       <c r="W33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X33" t="s">
         <v>172</v>
@@ -3714,7 +3714,7 @@
         <v>46296.64258336806</v>
       </c>
       <c r="W34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X34" t="s">
         <v>170</v>
@@ -3794,7 +3794,7 @@
         <v>46300.44301378472</v>
       </c>
       <c r="W35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X35" t="s">
         <v>165</v>
@@ -3874,7 +3874,7 @@
         <v>46301.46967876158</v>
       </c>
       <c r="W36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X36" t="s">
         <v>166</v>
@@ -3954,7 +3954,7 @@
         <v>46302.40341663195</v>
       </c>
       <c r="W37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X37" t="s">
         <v>169</v>
@@ -4034,7 +4034,7 @@
         <v>46300.57039657408</v>
       </c>
       <c r="W38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X38" t="s">
         <v>171</v>
@@ -4114,7 +4114,7 @@
         <v>46301.60196542824</v>
       </c>
       <c r="W39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X39" t="s">
         <v>163</v>
@@ -4194,7 +4194,7 @@
         <v>46301.60178498842</v>
       </c>
       <c r="W40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X40" t="s">
         <v>163</v>
@@ -4271,7 +4271,7 @@
         <v>46300.67840927083</v>
       </c>
       <c r="W41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X41" t="s">
         <v>172</v>
@@ -4345,7 +4345,7 @@
         <v>46296.64250469908</v>
       </c>
       <c r="W42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X42" t="s">
         <v>170</v>
@@ -4419,7 +4419,7 @@
         <v>46300.44324319444</v>
       </c>
       <c r="W43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X43" t="s">
         <v>165</v>
@@ -4493,7 +4493,7 @@
         <v>46301.46964587963</v>
       </c>
       <c r="W44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X44" t="s">
         <v>166</v>
@@ -4567,7 +4567,7 @@
         <v>46296.01593988426</v>
       </c>
       <c r="W45">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X45" t="s">
         <v>168</v>
@@ -4644,7 +4644,7 @@
         <v>46300.3863081713</v>
       </c>
       <c r="W46">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X46" t="s">
         <v>171</v>
@@ -4724,7 +4724,7 @@
         <v>46300.38630890047</v>
       </c>
       <c r="W47">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X47" t="s">
         <v>163</v>
@@ -4804,7 +4804,7 @@
         <v>46300.38631003472</v>
       </c>
       <c r="W48">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X48" t="s">
         <v>163</v>
@@ -4884,7 +4884,7 @@
         <v>46300.67853358796</v>
       </c>
       <c r="W49">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X49" t="s">
         <v>172</v>
@@ -4964,7 +4964,7 @@
         <v>46297.71954039352</v>
       </c>
       <c r="W50">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X50" t="s">
         <v>169</v>
@@ -5044,7 +5044,7 @@
         <v>46296.48787840278</v>
       </c>
       <c r="W51">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X51" t="s">
         <v>170</v>
@@ -5124,7 +5124,7 @@
         <v>46300.42827539352</v>
       </c>
       <c r="W52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X52" t="s">
         <v>169</v>
@@ -5204,7 +5204,7 @@
         <v>46300.57064887731</v>
       </c>
       <c r="W53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X53" t="s">
         <v>171</v>
@@ -5284,7 +5284,7 @@
         <v>46301.60206459491</v>
       </c>
       <c r="W54">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X54" t="s">
         <v>163</v>
@@ -5364,7 +5364,7 @@
         <v>46301.60121219907</v>
       </c>
       <c r="W55">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X55" t="s">
         <v>163</v>
@@ -5441,7 +5441,7 @@
         <v>46300.67857046297</v>
       </c>
       <c r="W56">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X56" t="s">
         <v>172</v>
@@ -5518,7 +5518,7 @@
         <v>46296.64261186343</v>
       </c>
       <c r="W57">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X57" t="s">
         <v>170</v>
@@ -5598,7 +5598,7 @@
         <v>46300.44350421296</v>
       </c>
       <c r="W58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X58" t="s">
         <v>165</v>
@@ -5678,7 +5678,7 @@
         <v>46301.46971603009</v>
       </c>
       <c r="W59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X59" t="s">
         <v>166</v>
@@ -5758,7 +5758,7 @@
         <v>46300.57801363426</v>
       </c>
       <c r="W60">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X60" t="s">
         <v>171</v>
@@ -5838,7 +5838,7 @@
         <v>46300.42855335648</v>
       </c>
       <c r="W61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X61" t="s">
         <v>169</v>
@@ -5918,7 +5918,7 @@
         <v>46300.57068319445</v>
       </c>
       <c r="W62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X62" t="s">
         <v>171</v>
@@ -5998,7 +5998,7 @@
         <v>46301.60209734954</v>
       </c>
       <c r="W63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X63" t="s">
         <v>163</v>
@@ -6078,7 +6078,7 @@
         <v>46301.60124362269</v>
       </c>
       <c r="W64">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X64" t="s">
         <v>163</v>
@@ -6155,7 +6155,7 @@
         <v>46300.67860491898</v>
       </c>
       <c r="W65">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X65" t="s">
         <v>172</v>
@@ -6232,7 +6232,7 @@
         <v>46296.64263715278</v>
       </c>
       <c r="W66">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X66" t="s">
         <v>170</v>
@@ -6312,7 +6312,7 @@
         <v>46300.44361263889</v>
       </c>
       <c r="W67">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X67" t="s">
         <v>165</v>
@@ -6392,7 +6392,7 @@
         <v>46301.46975131945</v>
       </c>
       <c r="W68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X68" t="s">
         <v>166</v>
@@ -6466,7 +6466,7 @@
         <v>46296.71263638889</v>
       </c>
       <c r="W69">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X69" t="s">
         <v>163</v>
@@ -6546,7 +6546,7 @@
         <v>46302.74648497685</v>
       </c>
       <c r="W70">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X70" t="s">
         <v>166</v>
@@ -6623,7 +6623,7 @@
         <v>46296.37884409722</v>
       </c>
       <c r="W71">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X71" t="s">
         <v>164</v>
@@ -6697,7 +6697,7 @@
         <v>46296.37884371528</v>
       </c>
       <c r="W72">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X72" t="s">
         <v>163</v>
@@ -6771,7 +6771,7 @@
         <v>46296.46064649305</v>
       </c>
       <c r="W73">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X73" t="s">
         <v>166</v>
@@ -6845,7 +6845,7 @@
         <v>46296.3788346875</v>
       </c>
       <c r="W74">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X74" t="s">
         <v>164</v>
@@ -6919,7 +6919,7 @@
         <v>46296.37883295139</v>
       </c>
       <c r="W75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X75" t="s">
         <v>163</v>
@@ -6993,7 +6993,7 @@
         <v>46296.37860081019</v>
       </c>
       <c r="W76">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X76" t="s">
         <v>164</v>
@@ -7067,7 +7067,7 @@
         <v>46296.37859760417</v>
       </c>
       <c r="W77">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X77" t="s">
         <v>163</v>
@@ -7141,7 +7141,7 @@
         <v>46296.79357893518</v>
       </c>
       <c r="W78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X78" t="s">
         <v>163</v>
@@ -7215,7 +7215,7 @@
         <v>46296.37868082176</v>
       </c>
       <c r="W79">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X79" t="s">
         <v>164</v>
@@ -7289,7 +7289,7 @@
         <v>46296.37867766204</v>
       </c>
       <c r="W80">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X80" t="s">
         <v>163</v>
@@ -7363,7 +7363,7 @@
         <v>46296.7936246875</v>
       </c>
       <c r="W81">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X81" t="s">
         <v>163</v>
@@ -7437,7 +7437,7 @@
         <v>46296.37638978009</v>
       </c>
       <c r="W82">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X82" t="s">
         <v>164</v>
@@ -7511,7 +7511,7 @@
         <v>46296.37638726852</v>
       </c>
       <c r="W83">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X83" t="s">
         <v>163</v>
@@ -7585,7 +7585,7 @@
         <v>46296.45920883102</v>
       </c>
       <c r="W84">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X84" t="s">
         <v>166</v>
@@ -7659,7 +7659,7 @@
         <v>46300.37640358796</v>
       </c>
       <c r="W85">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X85" t="s">
         <v>167</v>
@@ -7733,7 +7733,7 @@
         <v>46296.37883935186</v>
       </c>
       <c r="W86">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X86" t="s">
         <v>165</v>
@@ -7807,7 +7807,7 @@
         <v>46296.37873302084</v>
       </c>
       <c r="W87">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X87" t="s">
         <v>164</v>
@@ -7881,7 +7881,7 @@
         <v>46296.37872700232</v>
       </c>
       <c r="W88">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X88" t="s">
         <v>163</v>
@@ -7955,7 +7955,7 @@
         <v>46296.79365752315</v>
       </c>
       <c r="W89">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X89" t="s">
         <v>163</v>
@@ -8029,7 +8029,7 @@
         <v>46297.71059528935</v>
       </c>
       <c r="W90">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X90" t="s">
         <v>167</v>
@@ -8103,7 +8103,7 @@
         <v>46296.37648703704</v>
       </c>
       <c r="W91">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X91" t="s">
         <v>164</v>
@@ -8177,7 +8177,7 @@
         <v>46296.37648807871</v>
       </c>
       <c r="W92">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X92" t="s">
         <v>165</v>
@@ -8251,7 +8251,7 @@
         <v>46296.45925008102</v>
       </c>
       <c r="W93">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X93" t="s">
         <v>166</v>
@@ -8325,7 +8325,7 @@
         <v>46296.37619637731</v>
       </c>
       <c r="W94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X94" t="s">
         <v>165</v>
@@ -8399,7 +8399,7 @@
         <v>46296.45913734954</v>
       </c>
       <c r="W95">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X95" t="s">
         <v>166</v>
@@ -8473,7 +8473,7 @@
         <v>46296.37620748843</v>
       </c>
       <c r="W96">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X96" t="s">
         <v>164</v>
@@ -8547,7 +8547,7 @@
         <v>46296.37620686342</v>
       </c>
       <c r="W97">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X97" t="s">
         <v>165</v>
@@ -8621,7 +8621,7 @@
         <v>46296.45914429398</v>
       </c>
       <c r="W98">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X98" t="s">
         <v>166</v>
@@ -8695,7 +8695,7 @@
         <v>46296.37877858796</v>
       </c>
       <c r="W99">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X99" t="s">
         <v>164</v>
@@ -8769,7 +8769,7 @@
         <v>46296.37877496528</v>
       </c>
       <c r="W100">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X100" t="s">
         <v>163</v>
@@ -8843,7 +8843,7 @@
         <v>46296.79368927083</v>
       </c>
       <c r="W101">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X101" t="s">
         <v>163</v>
@@ -8917,7 +8917,7 @@
         <v>46296.37881099537</v>
       </c>
       <c r="W102">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X102" t="s">
         <v>164</v>
@@ -8991,7 +8991,7 @@
         <v>46296.37880798611</v>
       </c>
       <c r="W103">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X103" t="s">
         <v>163</v>
@@ -9065,7 +9065,7 @@
         <v>46296.79371550926</v>
       </c>
       <c r="W104">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X104" t="s">
         <v>163</v>
@@ -9142,7 +9142,7 @@
         <v>46301.53076038195</v>
       </c>
       <c r="W105">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X105" t="s">
         <v>163</v>
@@ -9219,7 +9219,7 @@
         <v>46301.77168440972</v>
       </c>
       <c r="W106">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X106" t="s">
         <v>166</v>
@@ -9296,7 +9296,7 @@
         <v>46302.45135077546</v>
       </c>
       <c r="W107">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X107" t="s">
         <v>167</v>
@@ -9373,7 +9373,7 @@
         <v>46301.53482881944</v>
       </c>
       <c r="W108">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X108" t="s">
         <v>163</v>
@@ -9453,7 +9453,7 @@
         <v>46301.61803621528</v>
       </c>
       <c r="W109">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X109" t="s">
         <v>165</v>
@@ -9530,7 +9530,7 @@
         <v>46301.68910333333</v>
       </c>
       <c r="W110">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X110" t="s">
         <v>166</v>
@@ -9607,7 +9607,7 @@
         <v>46302.40335295139</v>
       </c>
       <c r="W111">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X111" t="s">
         <v>167</v>
@@ -9684,7 +9684,7 @@
         <v>46297.37673402778</v>
       </c>
       <c r="W112">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X112" t="s">
         <v>169</v>
@@ -9758,7 +9758,7 @@
         <v>46297.37618915509</v>
       </c>
       <c r="W113">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X113" t="s">
         <v>169</v>
@@ -9832,7 +9832,7 @@
         <v>46297.66736068287</v>
       </c>
       <c r="W114">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X114" t="s">
         <v>171</v>
@@ -9906,7 +9906,7 @@
         <v>46297.45935385417</v>
       </c>
       <c r="W115">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X115" t="s">
         <v>170</v>
@@ -9980,7 +9980,7 @@
         <v>46297.37681010416</v>
       </c>
       <c r="W116">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X116" t="s">
         <v>169</v>
@@ -10054,7 +10054,7 @@
         <v>46297.37686377315</v>
       </c>
       <c r="W117">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X117" t="s">
         <v>169</v>
@@ -10128,7 +10128,7 @@
         <v>46297.37606362269</v>
       </c>
       <c r="W118">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X118" t="s">
         <v>169</v>
@@ -10202,7 +10202,7 @@
         <v>46297.66734447917</v>
       </c>
       <c r="W119">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X119" t="s">
         <v>171</v>
@@ -10276,7 +10276,7 @@
         <v>46297.45929016203</v>
       </c>
       <c r="W120">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X120" t="s">
         <v>170</v>
@@ -10350,7 +10350,7 @@
         <v>46297.37537966435</v>
       </c>
       <c r="W121">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X121" t="s">
         <v>169</v>
@@ -10424,7 +10424,7 @@
         <v>46297.45869950231</v>
       </c>
       <c r="W122">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X122" t="s">
         <v>168</v>
@@ -10498,7 +10498,7 @@
         <v>46300.66721489583</v>
       </c>
       <c r="W123">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X123" t="s">
         <v>171</v>
@@ -10572,7 +10572,7 @@
         <v>46297.45870309028</v>
       </c>
       <c r="W124">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X124" t="s">
         <v>172</v>
@@ -10646,7 +10646,7 @@
         <v>46297.45870405093</v>
       </c>
       <c r="W125">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X125" t="s">
         <v>170</v>
@@ -10720,7 +10720,7 @@
         <v>46297.45870177083</v>
       </c>
       <c r="W126">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X126" t="s">
         <v>170</v>
@@ -10794,7 +10794,7 @@
         <v>46300.65013206018</v>
       </c>
       <c r="W127">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X127" t="s">
         <v>169</v>
@@ -10868,7 +10868,7 @@
         <v>46300.65011049769</v>
       </c>
       <c r="W128">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X128" t="s">
         <v>168</v>
@@ -10942,7 +10942,7 @@
         <v>46300.66713765046</v>
       </c>
       <c r="W129">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X129" t="s">
         <v>171</v>
@@ -11016,7 +11016,7 @@
         <v>46300.66713784722</v>
       </c>
       <c r="W130">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X130" t="s">
         <v>172</v>
@@ -11090,7 +11090,7 @@
         <v>46300.66713822917</v>
       </c>
       <c r="W131">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X131" t="s">
         <v>170</v>
@@ -11164,7 +11164,7 @@
         <v>46300.75530894676</v>
       </c>
       <c r="W132">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X132" t="s">
         <v>170</v>
@@ -11238,7 +11238,7 @@
         <v>46297.66734765047</v>
       </c>
       <c r="W133">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X133" t="s">
         <v>171</v>
@@ -11312,7 +11312,7 @@
         <v>46301.70844945602</v>
       </c>
       <c r="W134">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X134" t="s">
         <v>169</v>
@@ -11386,7 +11386,7 @@
         <v>46301.70847283565</v>
       </c>
       <c r="W135">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="X135" t="s">
         <v>170</v>
@@ -11457,7 +11457,7 @@
         <v>46296.08337256945</v>
       </c>
       <c r="W136">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X136" t="s">
         <v>163</v>
@@ -11531,7 +11531,7 @@
         <v>46296.0834071412</v>
       </c>
       <c r="W137">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X137" t="s">
         <v>170</v>
@@ -11605,7 +11605,7 @@
         <v>46296.08341825232</v>
       </c>
       <c r="W138">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X138" t="s">
         <v>165</v>
@@ -11679,7 +11679,7 @@
         <v>46296.37558109954</v>
       </c>
       <c r="W139">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X139" t="s">
         <v>169</v>
@@ -11753,7 +11753,7 @@
         <v>46296.37504012731</v>
       </c>
       <c r="W140">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X140" t="s">
         <v>168</v>
@@ -11827,7 +11827,7 @@
         <v>46296.3760846412</v>
       </c>
       <c r="W141">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="X141" t="s">
         <v>172</v>
@@ -11901,7 +11901,7 @@
         <v>46296.37648518519</v>
       </c>
       <c r="W142">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="X142" t="s">
         <v>169</v>
@@ -11975,7 +11975,7 @@
         <v>46296.37615983796</v>
       </c>
       <c r="W143">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="X143" t="s">
         <v>163</v>
@@ -12049,7 +12049,7 @@
         <v>46296.37684290509</v>
       </c>
       <c r="W144">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="X144" t="s">
         <v>170</v>
@@ -12123,7 +12123,7 @@
         <v>46296.37609667824</v>
       </c>
       <c r="W145">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="X145" t="s">
         <v>168</v>
@@ -12197,7 +12197,7 @@
         <v>46296.37683961805</v>
       </c>
       <c r="W146">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="X146" t="s">
         <v>172</v>
@@ -12271,7 +12271,7 @@
         <v>46296.37684039352</v>
       </c>
       <c r="W147">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X147" t="s">
         <v>172</v>
@@ -12345,7 +12345,7 @@
         <v>46296.37726273148</v>
       </c>
       <c r="W148">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X148" t="s">
         <v>164</v>
@@ -12419,7 +12419,7 @@
         <v>46296.37814100694</v>
       </c>
       <c r="W149">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X149" t="s">
         <v>172</v>
@@ -12493,7 +12493,7 @@
         <v>46296.37816597222</v>
       </c>
       <c r="W150">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="X150" t="s">
         <v>170</v>
@@ -12567,7 +12567,7 @@
         <v>46296.37748545139</v>
       </c>
       <c r="W151">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="X151" t="s">
         <v>169</v>
@@ -12641,7 +12641,7 @@
         <v>46296.37705413195</v>
       </c>
       <c r="W152">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="X152" t="s">
         <v>168</v>
@@ -12715,7 +12715,7 @@
         <v>46296.37710454861</v>
       </c>
       <c r="W153">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="X153" t="s">
         <v>163</v>
@@ -12789,7 +12789,7 @@
         <v>46296.37814163195</v>
       </c>
       <c r="W154">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="X154" t="s">
         <v>172</v>
@@ -12863,7 +12863,7 @@
         <v>46296.37822175926</v>
       </c>
       <c r="W155">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="X155" t="s">
         <v>166</v>
@@ -12937,7 +12937,7 @@
         <v>46297.67728344908</v>
       </c>
       <c r="W156">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X156" t="s">
         <v>169</v>
@@ -13008,7 +13008,7 @@
         <v>46297.67730740741</v>
       </c>
       <c r="W157">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X157" t="s">
         <v>168</v>
@@ -13079,7 +13079,7 @@
         <v>46297.67730972222</v>
       </c>
       <c r="W158">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X158" t="s">
         <v>171</v>
@@ -13150,7 +13150,7 @@
         <v>46297.67731253472</v>
       </c>
       <c r="W159">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X159" t="s">
         <v>164</v>
@@ -13221,7 +13221,7 @@
         <v>46297.67731608796</v>
       </c>
       <c r="W160">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X160" t="s">
         <v>163</v>
@@ -13292,7 +13292,7 @@
         <v>46297.6773164699</v>
       </c>
       <c r="W161">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X161" t="s">
         <v>163</v>
@@ -13363,7 +13363,7 @@
         <v>46297.67732225695</v>
       </c>
       <c r="W162">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X162" t="s">
         <v>172</v>
@@ -13434,7 +13434,7 @@
         <v>46297.67732283565</v>
       </c>
       <c r="W163">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X163" t="s">
         <v>170</v>
@@ -13505,7 +13505,7 @@
         <v>46297.67732337963</v>
       </c>
       <c r="W164">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X164" t="s">
         <v>170</v>
@@ -13576,7 +13576,7 @@
         <v>46297.6773253125</v>
       </c>
       <c r="W165">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X165" t="s">
         <v>170</v>
@@ -13647,7 +13647,7 @@
         <v>46297.67733796296</v>
       </c>
       <c r="W166">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X166" t="s">
         <v>165</v>
@@ -13718,7 +13718,7 @@
         <v>46297.67733896991</v>
       </c>
       <c r="W167">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X167" t="s">
         <v>166</v>
@@ -13789,7 +13789,7 @@
         <v>46297.67734047454</v>
       </c>
       <c r="W168">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X168" t="s">
         <v>167</v>
@@ -13860,7 +13860,7 @@
         <v>46297.67734097222</v>
       </c>
       <c r="W169">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X169" t="s">
         <v>167</v>
@@ -13934,7 +13934,7 @@
         <v>46300.67560568287</v>
       </c>
       <c r="W170">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X170" t="s">
         <v>169</v>
@@ -14011,7 +14011,7 @@
         <v>46300.67612549769</v>
       </c>
       <c r="W171">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X171" t="s">
         <v>168</v>
@@ -14088,7 +14088,7 @@
         <v>46300.67620415509</v>
       </c>
       <c r="W172">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X172" t="s">
         <v>171</v>
@@ -14165,7 +14165,7 @@
         <v>46300.67631252314</v>
       </c>
       <c r="W173">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X173" t="s">
         <v>164</v>
@@ -14242,7 +14242,7 @@
         <v>46300.6765974537</v>
       </c>
       <c r="W174">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X174" t="s">
         <v>163</v>
@@ -14319,7 +14319,7 @@
         <v>46300.67662010417</v>
       </c>
       <c r="W175">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X175" t="s">
         <v>163</v>
@@ -14396,7 +14396,7 @@
         <v>46300.67678489583</v>
       </c>
       <c r="W176">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X176" t="s">
         <v>172</v>
@@ -14473,7 +14473,7 @@
         <v>46301.34827806713</v>
       </c>
       <c r="W177">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X177" t="s">
         <v>170</v>
@@ -14550,7 +14550,7 @@
         <v>46300.67680096065</v>
       </c>
       <c r="W178">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X178" t="s">
         <v>170</v>
@@ -14627,7 +14627,7 @@
         <v>46300.6769524537</v>
       </c>
       <c r="W179">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X179" t="s">
         <v>165</v>
@@ -14704,7 +14704,7 @@
         <v>46300.67696659722</v>
       </c>
       <c r="W180">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X180" t="s">
         <v>166</v>
@@ -14778,7 +14778,7 @@
         <v>46297.34991217592</v>
       </c>
       <c r="W181">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X181" t="s">
         <v>169</v>
@@ -14849,7 +14849,7 @@
         <v>46297.3499325</v>
       </c>
       <c r="W182">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X182" t="s">
         <v>168</v>
@@ -14920,7 +14920,7 @@
         <v>46297.34994254629</v>
       </c>
       <c r="W183">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X183" t="s">
         <v>171</v>
@@ -14991,7 +14991,7 @@
         <v>46297.34994771991</v>
       </c>
       <c r="W184">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X184" t="s">
         <v>163</v>
@@ -15062,7 +15062,7 @@
         <v>46297.34994974537</v>
       </c>
       <c r="W185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X185" t="s">
         <v>170</v>
@@ -15133,7 +15133,7 @@
         <v>46297.34995063658</v>
       </c>
       <c r="W186">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X186" t="s">
         <v>170</v>
@@ -15204,7 +15204,7 @@
         <v>46297.34996266204</v>
       </c>
       <c r="W187">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X187" t="s">
         <v>165</v>
@@ -15275,7 +15275,7 @@
         <v>46297.68732318287</v>
       </c>
       <c r="W188">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X188" t="s">
         <v>169</v>
@@ -15346,7 +15346,7 @@
         <v>46297.68735216435</v>
       </c>
       <c r="W189">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X189" t="s">
         <v>168</v>
@@ -15417,7 +15417,7 @@
         <v>46297.68735517361</v>
       </c>
       <c r="W190">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X190" t="s">
         <v>171</v>
@@ -15488,7 +15488,7 @@
         <v>46297.68735752315</v>
       </c>
       <c r="W191">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X191" t="s">
         <v>164</v>
@@ -15559,7 +15559,7 @@
         <v>46297.68736119213</v>
       </c>
       <c r="W192">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X192" t="s">
         <v>163</v>
@@ -15630,7 +15630,7 @@
         <v>46297.68736145833</v>
       </c>
       <c r="W193">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X193" t="s">
         <v>163</v>
@@ -15701,7 +15701,7 @@
         <v>46297.68736666667</v>
       </c>
       <c r="W194">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X194" t="s">
         <v>172</v>
@@ -15772,7 +15772,7 @@
         <v>46297.68736686343</v>
       </c>
       <c r="W195">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X195" t="s">
         <v>170</v>
@@ -15843,7 +15843,7 @@
         <v>46297.68736712963</v>
       </c>
       <c r="W196">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X196" t="s">
         <v>170</v>
@@ -15914,7 +15914,7 @@
         <v>46297.68736878473</v>
       </c>
       <c r="W197">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X197" t="s">
         <v>170</v>
@@ -15985,7 +15985,7 @@
         <v>46297.6873764699</v>
       </c>
       <c r="W198">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X198" t="s">
         <v>165</v>
@@ -16056,7 +16056,7 @@
         <v>46297.68737700232</v>
       </c>
       <c r="W199">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X199" t="s">
         <v>166</v>
@@ -16127,7 +16127,7 @@
         <v>46297.68737777778</v>
       </c>
       <c r="W200">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X200" t="s">
         <v>167</v>
@@ -16198,7 +16198,7 @@
         <v>46297.68737800926</v>
       </c>
       <c r="W201">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X201" t="s">
         <v>167</v>
@@ -16269,7 +16269,7 @@
         <v>46300.67560523148</v>
       </c>
       <c r="W202">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X202" t="s">
         <v>169</v>
@@ -16340,7 +16340,7 @@
         <v>46300.67612488426</v>
       </c>
       <c r="W203">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X203" t="s">
         <v>168</v>
@@ -16411,7 +16411,7 @@
         <v>46300.67620471065</v>
       </c>
       <c r="W204">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X204" t="s">
         <v>171</v>
@@ -16482,7 +16482,7 @@
         <v>46300.67631207176</v>
       </c>
       <c r="W205">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X205" t="s">
         <v>164</v>
@@ -16553,7 +16553,7 @@
         <v>46300.67659613426</v>
       </c>
       <c r="W206">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X206" t="s">
         <v>163</v>
@@ -16624,7 +16624,7 @@
         <v>46300.67661899306</v>
       </c>
       <c r="W207">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X207" t="s">
         <v>163</v>
@@ -16695,7 +16695,7 @@
         <v>46300.67678520834</v>
       </c>
       <c r="W208">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X208" t="s">
         <v>172</v>
@@ -16769,7 +16769,7 @@
         <v>46302.51963612268</v>
       </c>
       <c r="W209">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X209" t="s">
         <v>170</v>
@@ -16843,7 +16843,7 @@
         <v>46300.6768006713</v>
       </c>
       <c r="W210">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X210" t="s">
         <v>170</v>
@@ -16914,7 +16914,7 @@
         <v>46300.6769528125</v>
       </c>
       <c r="W211">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X211" t="s">
         <v>165</v>
@@ -16985,7 +16985,7 @@
         <v>46300.67696615741</v>
       </c>
       <c r="W212">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X212" t="s">
         <v>166</v>
@@ -17056,7 +17056,7 @@
         <v>46296.34114513889</v>
       </c>
       <c r="W213">
-        <v>-49</v>
+        <v>-48</v>
       </c>
       <c r="X213" t="s">
         <v>168</v>
@@ -17130,7 +17130,7 @@
         <v>46296.34050315972</v>
       </c>
       <c r="W214">
-        <v>-49</v>
+        <v>-48</v>
       </c>
       <c r="X214" t="s">
         <v>169</v>
@@ -17204,7 +17204,7 @@
         <v>46296.39309459491</v>
       </c>
       <c r="W215">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X215" t="s">
         <v>171</v>
@@ -17278,7 +17278,7 @@
         <v>46296.3409153125</v>
       </c>
       <c r="W216">
-        <v>-49</v>
+        <v>-48</v>
       </c>
       <c r="X216" t="s">
         <v>171</v>
@@ -17352,7 +17352,7 @@
         <v>46296.0420403125</v>
       </c>
       <c r="W217">
-        <v>-48</v>
+        <v>-47</v>
       </c>
       <c r="X217" t="s">
         <v>169</v>
@@ -17423,7 +17423,7 @@
         <v>46296.0420403125</v>
       </c>
       <c r="W218">
-        <v>-48</v>
+        <v>-47</v>
       </c>
       <c r="X218" t="s">
         <v>168</v>
@@ -17494,7 +17494,7 @@
         <v>46301.49091145834</v>
       </c>
       <c r="W219">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X219" t="s">
         <v>168</v>
@@ -17568,7 +17568,7 @@
         <v>46297.49393364583</v>
       </c>
       <c r="W220">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X220" t="s">
         <v>166</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-08 11:40
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -747,10 +747,10 @@
     <t>Baixado via rotina MGC x Analise Balanço em 01/10/2026 08:10:19. - Data Comentário: 01/10/2026 08:08</t>
   </si>
   <si>
+    <t>Baixado via API integração MGC x Analise Balanço em 01/10/2026 09:29:38. - Data Comentário: 01/10/2026 09:24</t>
+  </si>
+  <si>
     <t>Baixado via rotina MGC x Analise Balanço em 01/10/2026 08:10:55. - Data Comentário: 01/10/2026 08:09</t>
-  </si>
-  <si>
-    <t>Baixado via API integração MGC x Analise Balanço em 01/10/2026 09:29:38. - Data Comentário: 01/10/2026 09:24</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 06/10/2026 
@@ -17267,28 +17267,28 @@
         <v>66</v>
       </c>
       <c r="N216" s="1">
-        <v>46351</v>
+        <v>46290</v>
       </c>
       <c r="P216">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Q216">
         <v>2026</v>
       </c>
       <c r="R216">
-        <v>16976323</v>
+        <v>16976321</v>
       </c>
       <c r="S216" t="s">
         <v>54</v>
       </c>
       <c r="U216" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="V216" s="1">
-        <v>46296.3409153125</v>
+        <v>46296.39309459491</v>
       </c>
       <c r="W216">
-        <v>-48</v>
+        <v>13</v>
       </c>
       <c r="X216" t="s">
         <v>172</v>
@@ -17341,28 +17341,28 @@
         <v>66</v>
       </c>
       <c r="N217" s="1">
-        <v>46290</v>
+        <v>46351</v>
       </c>
       <c r="P217">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q217">
         <v>2026</v>
       </c>
       <c r="R217">
-        <v>16976321</v>
+        <v>16976323</v>
       </c>
       <c r="S217" t="s">
         <v>54</v>
       </c>
       <c r="U217" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="V217" s="1">
-        <v>46296.39309459491</v>
+        <v>46296.3409153125</v>
       </c>
       <c r="W217">
-        <v>13</v>
+        <v>-48</v>
       </c>
       <c r="X217" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-09 16:43
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3579" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3664" uniqueCount="276">
   <si>
     <t>CodCliente</t>
   </si>
@@ -795,6 +795,9 @@
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 09/10/2026 - Data Comentário: 06/10/2026 10:53</t>
   </si>
   <si>
+    <t>Imposto enviado via SCI Report - Data Comentário: 09/10/2026 15:17</t>
+  </si>
+  <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 09/10/2026 - Data Comentário: 09/10/2026 09:00</t>
   </si>
   <si>
@@ -813,6 +816,12 @@
     <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1866] sendo a ultima baixa feita [1866]-07/10/2026 10:49:56.. - Data Comentário: 07/10/2026 10:44</t>
   </si>
   <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-08/10/2026 08:54:54.. - Data Comentário: 08/10/2026 08:49</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-09/10/2026 15:05:38.. - Data Comentário: 09/10/2026 15:00</t>
+  </si>
+  <si>
     <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-09/10/2026 15:05:39.. - Data Comentário: 09/10/2026 15:00</t>
   </si>
   <si>
@@ -820,6 +829,15 @@
   </si>
   <si>
     <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-06/10/2026 14:49:58.. - Data Comentário: 06/10/2026 14:44</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-06/10/2026 16:32:18.. - Data Comentário: 06/10/2026 16:27</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-09/10/2026 15:24:52.. - Data Comentário: 09/10/2026 15:19</t>
+  </si>
+  <si>
+    <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-07/10/2026 09:40:49.. - Data Comentário: 07/10/2026 09:35</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 09/10/2026 
@@ -1180,7 +1198,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI250"/>
+  <dimension ref="A1:AI256"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -1361,10 +1379,10 @@
         <v>135</v>
       </c>
       <c r="AH2" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI2" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:35">
@@ -1438,10 +1456,10 @@
         <v>135</v>
       </c>
       <c r="AH3" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI3" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" spans="1:35">
@@ -1512,10 +1530,10 @@
         <v>136</v>
       </c>
       <c r="AH4" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI4" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:35">
@@ -1586,10 +1604,10 @@
         <v>135</v>
       </c>
       <c r="AH5" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" spans="1:35">
@@ -1660,10 +1678,10 @@
         <v>135</v>
       </c>
       <c r="AH6" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI6" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:35">
@@ -1734,10 +1752,10 @@
         <v>137</v>
       </c>
       <c r="AH7" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI7" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:35">
@@ -1808,10 +1826,10 @@
         <v>136</v>
       </c>
       <c r="AH8" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI8" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:35">
@@ -1882,10 +1900,10 @@
         <v>138</v>
       </c>
       <c r="AH9" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI9" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" spans="1:35">
@@ -1956,10 +1974,10 @@
         <v>138</v>
       </c>
       <c r="AH10" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI10" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:35">
@@ -2030,10 +2048,10 @@
         <v>139</v>
       </c>
       <c r="AH11" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI11" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:35">
@@ -2107,10 +2125,10 @@
         <v>139</v>
       </c>
       <c r="AH12" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI12" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" spans="1:35">
@@ -2181,10 +2199,10 @@
         <v>139</v>
       </c>
       <c r="AH13" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI13" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14" spans="1:35">
@@ -2255,10 +2273,10 @@
         <v>139</v>
       </c>
       <c r="AH14" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI14" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:35">
@@ -2329,10 +2347,10 @@
         <v>140</v>
       </c>
       <c r="AH15" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI15" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="16" spans="1:35">
@@ -2403,10 +2421,10 @@
         <v>141</v>
       </c>
       <c r="AH16" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI16" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="17" spans="1:35">
@@ -2477,10 +2495,10 @@
         <v>141</v>
       </c>
       <c r="AH17" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI17" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="18" spans="1:35">
@@ -2551,10 +2569,10 @@
         <v>141</v>
       </c>
       <c r="AH18" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI18" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="19" spans="1:35">
@@ -2625,10 +2643,10 @@
         <v>149</v>
       </c>
       <c r="AH19" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI19" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="20" spans="1:35">
@@ -2699,10 +2717,10 @@
         <v>149</v>
       </c>
       <c r="AH20" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI20" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="21" spans="1:35">
@@ -2773,10 +2791,10 @@
         <v>142</v>
       </c>
       <c r="AH21" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI21" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="22" spans="1:35">
@@ -2850,10 +2868,10 @@
         <v>149</v>
       </c>
       <c r="AH22" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI22" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23" spans="1:35">
@@ -2930,10 +2948,10 @@
         <v>144</v>
       </c>
       <c r="AH23" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI23" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="24" spans="1:35">
@@ -3010,10 +3028,10 @@
         <v>145</v>
       </c>
       <c r="AH24" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI24" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" spans="1:35">
@@ -3084,10 +3102,10 @@
         <v>146</v>
       </c>
       <c r="AH25" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI25" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="26" spans="1:35">
@@ -3158,10 +3176,10 @@
         <v>147</v>
       </c>
       <c r="AH26" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI26" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27" spans="1:35">
@@ -3235,10 +3253,10 @@
         <v>149</v>
       </c>
       <c r="AH27" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI27" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="28" spans="1:35">
@@ -3312,10 +3330,10 @@
         <v>149</v>
       </c>
       <c r="AH28" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI28" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="29" spans="1:35">
@@ -3386,10 +3404,10 @@
         <v>144</v>
       </c>
       <c r="AH29" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI29" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="30" spans="1:35">
@@ -3460,10 +3478,10 @@
         <v>145</v>
       </c>
       <c r="AH30" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI30" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="31" spans="1:35">
@@ -3540,10 +3558,10 @@
         <v>146</v>
       </c>
       <c r="AH31" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI31" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="32" spans="1:35">
@@ -3617,10 +3635,10 @@
         <v>149</v>
       </c>
       <c r="AH32" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI32" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="33" spans="1:35">
@@ -3694,10 +3712,10 @@
         <v>149</v>
       </c>
       <c r="AH33" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI33" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="34" spans="1:35">
@@ -3771,10 +3789,10 @@
         <v>149</v>
       </c>
       <c r="AH34" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI34" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="35" spans="1:35">
@@ -3851,10 +3869,10 @@
         <v>142</v>
       </c>
       <c r="AH35" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI35" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="36" spans="1:35">
@@ -3931,10 +3949,10 @@
         <v>148</v>
       </c>
       <c r="AH36" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI36" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="37" spans="1:35">
@@ -4011,10 +4029,10 @@
         <v>144</v>
       </c>
       <c r="AH37" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI37" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="38" spans="1:35">
@@ -4091,10 +4109,10 @@
         <v>145</v>
       </c>
       <c r="AH38" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI38" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="39" spans="1:35">
@@ -4171,10 +4189,10 @@
         <v>146</v>
       </c>
       <c r="AH39" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI39" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="40" spans="1:35">
@@ -4248,10 +4266,10 @@
         <v>149</v>
       </c>
       <c r="AH40" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI40" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="41" spans="1:35">
@@ -4325,10 +4343,10 @@
         <v>149</v>
       </c>
       <c r="AH41" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI41" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="42" spans="1:35">
@@ -4402,10 +4420,10 @@
         <v>149</v>
       </c>
       <c r="AH42" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI42" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="43" spans="1:35">
@@ -4476,10 +4494,10 @@
         <v>142</v>
       </c>
       <c r="AH43" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI43" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="44" spans="1:35">
@@ -4550,10 +4568,10 @@
         <v>148</v>
       </c>
       <c r="AH44" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI44" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="45" spans="1:35">
@@ -4624,10 +4642,10 @@
         <v>144</v>
       </c>
       <c r="AH45" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI45" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="46" spans="1:35">
@@ -4698,10 +4716,10 @@
         <v>145</v>
       </c>
       <c r="AH46" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI46" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="47" spans="1:35">
@@ -4772,10 +4790,10 @@
         <v>147</v>
       </c>
       <c r="AH47" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI47" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="48" spans="1:35">
@@ -4846,10 +4864,10 @@
         <v>148</v>
       </c>
       <c r="AH48" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI48" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="49" spans="1:35">
@@ -4926,10 +4944,10 @@
         <v>148</v>
       </c>
       <c r="AH49" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI49" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="50" spans="1:35">
@@ -5003,10 +5021,10 @@
         <v>149</v>
       </c>
       <c r="AH50" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI50" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="51" spans="1:35">
@@ -5080,10 +5098,10 @@
         <v>149</v>
       </c>
       <c r="AH51" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI51" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="52" spans="1:35">
@@ -5157,10 +5175,10 @@
         <v>149</v>
       </c>
       <c r="AH52" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI52" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="53" spans="1:35">
@@ -5237,10 +5255,10 @@
         <v>142</v>
       </c>
       <c r="AH53" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI53" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="54" spans="1:35">
@@ -5317,10 +5335,10 @@
         <v>146</v>
       </c>
       <c r="AH54" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI54" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="55" spans="1:35">
@@ -5397,10 +5415,10 @@
         <v>148</v>
       </c>
       <c r="AH55" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI55" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="56" spans="1:35">
@@ -5477,10 +5495,10 @@
         <v>146</v>
       </c>
       <c r="AH56" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI56" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="57" spans="1:35">
@@ -5554,10 +5572,10 @@
         <v>149</v>
       </c>
       <c r="AH57" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI57" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="58" spans="1:35">
@@ -5631,10 +5649,10 @@
         <v>149</v>
       </c>
       <c r="AH58" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI58" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="59" spans="1:35">
@@ -5708,10 +5726,10 @@
         <v>149</v>
       </c>
       <c r="AH59" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI59" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="60" spans="1:35">
@@ -5782,10 +5800,10 @@
         <v>142</v>
       </c>
       <c r="AH60" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI60" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="61" spans="1:35">
@@ -5862,10 +5880,10 @@
         <v>148</v>
       </c>
       <c r="AH61" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI61" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="62" spans="1:35">
@@ -5942,10 +5960,10 @@
         <v>144</v>
       </c>
       <c r="AH62" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI62" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="63" spans="1:35">
@@ -6022,10 +6040,10 @@
         <v>145</v>
       </c>
       <c r="AH63" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI63" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="64" spans="1:35">
@@ -6102,10 +6120,10 @@
         <v>149</v>
       </c>
       <c r="AH64" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI64" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="65" spans="1:35">
@@ -6182,10 +6200,10 @@
         <v>146</v>
       </c>
       <c r="AH65" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI65" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="66" spans="1:35">
@@ -6259,10 +6277,10 @@
         <v>149</v>
       </c>
       <c r="AH66" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI66" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="67" spans="1:35">
@@ -6336,10 +6354,10 @@
         <v>149</v>
       </c>
       <c r="AH67" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI67" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="68" spans="1:35">
@@ -6413,10 +6431,10 @@
         <v>149</v>
       </c>
       <c r="AH68" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI68" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="69" spans="1:35">
@@ -6487,10 +6505,10 @@
         <v>142</v>
       </c>
       <c r="AH69" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI69" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="70" spans="1:35">
@@ -6567,10 +6585,10 @@
         <v>148</v>
       </c>
       <c r="AH70" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI70" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="71" spans="1:35">
@@ -6647,10 +6665,10 @@
         <v>144</v>
       </c>
       <c r="AH71" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI71" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="72" spans="1:35">
@@ -6727,10 +6745,10 @@
         <v>145</v>
       </c>
       <c r="AH72" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI72" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="73" spans="1:35">
@@ -6801,10 +6819,10 @@
         <v>149</v>
       </c>
       <c r="AH73" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI73" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="74" spans="1:35">
@@ -6881,10 +6899,10 @@
         <v>145</v>
       </c>
       <c r="AH74" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI74" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="75" spans="1:35">
@@ -6961,10 +6979,10 @@
         <v>145</v>
       </c>
       <c r="AH75" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI75" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="76" spans="1:35">
@@ -7035,10 +7053,10 @@
         <v>150</v>
       </c>
       <c r="AH76" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI76" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="77" spans="1:35">
@@ -7109,10 +7127,10 @@
         <v>151</v>
       </c>
       <c r="AH77" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI77" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="78" spans="1:35">
@@ -7183,10 +7201,10 @@
         <v>151</v>
       </c>
       <c r="AH78" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI78" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="79" spans="1:35">
@@ -7257,10 +7275,10 @@
         <v>150</v>
       </c>
       <c r="AH79" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI79" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="80" spans="1:35">
@@ -7331,10 +7349,10 @@
         <v>151</v>
       </c>
       <c r="AH80" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI80" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="81" spans="1:35">
@@ -7405,10 +7423,10 @@
         <v>150</v>
       </c>
       <c r="AH81" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI81" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="82" spans="1:35">
@@ -7479,10 +7497,10 @@
         <v>151</v>
       </c>
       <c r="AH82" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI82" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="83" spans="1:35">
@@ -7553,10 +7571,10 @@
         <v>152</v>
       </c>
       <c r="AH83" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI83" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="84" spans="1:35">
@@ -7627,10 +7645,10 @@
         <v>150</v>
       </c>
       <c r="AH84" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI84" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="85" spans="1:35">
@@ -7701,10 +7719,10 @@
         <v>151</v>
       </c>
       <c r="AH85" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI85" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="86" spans="1:35">
@@ -7775,10 +7793,10 @@
         <v>152</v>
       </c>
       <c r="AH86" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI86" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="87" spans="1:35">
@@ -7849,10 +7867,10 @@
         <v>150</v>
       </c>
       <c r="AH87" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI87" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="88" spans="1:35">
@@ -7923,10 +7941,10 @@
         <v>151</v>
       </c>
       <c r="AH88" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI88" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="89" spans="1:35">
@@ -7997,10 +8015,10 @@
         <v>151</v>
       </c>
       <c r="AH89" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI89" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="90" spans="1:35">
@@ -8071,10 +8089,10 @@
         <v>167</v>
       </c>
       <c r="AH90" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI90" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="91" spans="1:35">
@@ -8145,10 +8163,10 @@
         <v>151</v>
       </c>
       <c r="AH91" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI91" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="92" spans="1:35">
@@ -8219,10 +8237,10 @@
         <v>150</v>
       </c>
       <c r="AH92" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI92" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="93" spans="1:35">
@@ -8293,10 +8311,10 @@
         <v>151</v>
       </c>
       <c r="AH93" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI93" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="94" spans="1:35">
@@ -8367,10 +8385,10 @@
         <v>152</v>
       </c>
       <c r="AH94" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI94" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="95" spans="1:35">
@@ -8441,10 +8459,10 @@
         <v>167</v>
       </c>
       <c r="AH95" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI95" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="96" spans="1:35">
@@ -8515,10 +8533,10 @@
         <v>150</v>
       </c>
       <c r="AH96" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI96" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="97" spans="1:35">
@@ -8589,10 +8607,10 @@
         <v>151</v>
       </c>
       <c r="AH97" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI97" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="98" spans="1:35">
@@ -8663,10 +8681,10 @@
         <v>151</v>
       </c>
       <c r="AH98" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI98" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="99" spans="1:35">
@@ -8737,10 +8755,10 @@
         <v>151</v>
       </c>
       <c r="AH99" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI99" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="100" spans="1:35">
@@ -8811,10 +8829,10 @@
         <v>151</v>
       </c>
       <c r="AH100" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI100" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="101" spans="1:35">
@@ -8885,10 +8903,10 @@
         <v>150</v>
       </c>
       <c r="AH101" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI101" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="102" spans="1:35">
@@ -8959,10 +8977,10 @@
         <v>151</v>
       </c>
       <c r="AH102" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI102" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="103" spans="1:35">
@@ -9033,10 +9051,10 @@
         <v>151</v>
       </c>
       <c r="AH103" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI103" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="104" spans="1:35">
@@ -9107,10 +9125,10 @@
         <v>150</v>
       </c>
       <c r="AH104" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI104" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="105" spans="1:35">
@@ -9181,10 +9199,10 @@
         <v>151</v>
       </c>
       <c r="AH105" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI105" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="106" spans="1:35">
@@ -9255,10 +9273,10 @@
         <v>152</v>
       </c>
       <c r="AH106" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI106" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="107" spans="1:35">
@@ -9329,10 +9347,10 @@
         <v>150</v>
       </c>
       <c r="AH107" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI107" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="108" spans="1:35">
@@ -9403,10 +9421,10 @@
         <v>151</v>
       </c>
       <c r="AH108" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI108" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="109" spans="1:35">
@@ -9477,10 +9495,10 @@
         <v>152</v>
       </c>
       <c r="AH109" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI109" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="110" spans="1:35">
@@ -9551,10 +9569,10 @@
         <v>151</v>
       </c>
       <c r="AH110" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI110" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="111" spans="1:35">
@@ -9631,10 +9649,10 @@
         <v>151</v>
       </c>
       <c r="AH111" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI111" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="112" spans="1:35">
@@ -9708,10 +9726,10 @@
         <v>151</v>
       </c>
       <c r="AH112" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI112" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="113" spans="1:35">
@@ -9785,10 +9803,10 @@
         <v>153</v>
       </c>
       <c r="AH113" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI113" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="114" spans="1:35">
@@ -9865,10 +9883,10 @@
         <v>150</v>
       </c>
       <c r="AH114" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI114" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="115" spans="1:35">
@@ -9942,10 +9960,10 @@
         <v>151</v>
       </c>
       <c r="AH115" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI115" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="116" spans="1:35">
@@ -10022,10 +10040,10 @@
         <v>151</v>
       </c>
       <c r="AH116" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI116" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="117" spans="1:35">
@@ -10099,10 +10117,10 @@
         <v>151</v>
       </c>
       <c r="AH117" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI117" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="118" spans="1:35">
@@ -10176,10 +10194,10 @@
         <v>153</v>
       </c>
       <c r="AH118" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI118" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="119" spans="1:35">
@@ -10250,10 +10268,10 @@
         <v>154</v>
       </c>
       <c r="AH119" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI119" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="120" spans="1:35">
@@ -10324,10 +10342,10 @@
         <v>154</v>
       </c>
       <c r="AH120" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI120" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="121" spans="1:35">
@@ -10398,10 +10416,10 @@
         <v>154</v>
       </c>
       <c r="AH121" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI121" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="122" spans="1:35">
@@ -10472,10 +10490,10 @@
         <v>154</v>
       </c>
       <c r="AH122" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI122" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="123" spans="1:35">
@@ -10546,10 +10564,10 @@
         <v>154</v>
       </c>
       <c r="AH123" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI123" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="124" spans="1:35">
@@ -10620,10 +10638,10 @@
         <v>154</v>
       </c>
       <c r="AH124" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI124" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="125" spans="1:35">
@@ -10694,10 +10712,10 @@
         <v>154</v>
       </c>
       <c r="AH125" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI125" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="126" spans="1:35">
@@ -10768,10 +10786,10 @@
         <v>154</v>
       </c>
       <c r="AH126" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI126" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="127" spans="1:35">
@@ -10842,10 +10860,10 @@
         <v>154</v>
       </c>
       <c r="AH127" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI127" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="128" spans="1:35">
@@ -10916,10 +10934,10 @@
         <v>154</v>
       </c>
       <c r="AH128" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI128" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="129" spans="1:35">
@@ -10990,10 +11008,10 @@
         <v>154</v>
       </c>
       <c r="AH129" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI129" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="130" spans="1:35">
@@ -11064,10 +11082,10 @@
         <v>154</v>
       </c>
       <c r="AH130" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI130" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="131" spans="1:35">
@@ -11138,10 +11156,10 @@
         <v>154</v>
       </c>
       <c r="AH131" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI131" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="132" spans="1:35">
@@ -11212,10 +11230,10 @@
         <v>154</v>
       </c>
       <c r="AH132" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI132" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="133" spans="1:35">
@@ -11286,10 +11304,10 @@
         <v>154</v>
       </c>
       <c r="AH133" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI133" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="134" spans="1:35">
@@ -11360,10 +11378,10 @@
         <v>154</v>
       </c>
       <c r="AH134" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI134" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="135" spans="1:35">
@@ -11434,10 +11452,10 @@
         <v>154</v>
       </c>
       <c r="AH135" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI135" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="136" spans="1:35">
@@ -11508,10 +11526,10 @@
         <v>154</v>
       </c>
       <c r="AH136" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI136" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="137" spans="1:35">
@@ -11582,10 +11600,10 @@
         <v>154</v>
       </c>
       <c r="AH137" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI137" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="138" spans="1:35">
@@ -11656,10 +11674,10 @@
         <v>154</v>
       </c>
       <c r="AH138" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI138" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="139" spans="1:35">
@@ -11730,10 +11748,10 @@
         <v>154</v>
       </c>
       <c r="AH139" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI139" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="140" spans="1:35">
@@ -11804,10 +11822,10 @@
         <v>154</v>
       </c>
       <c r="AH140" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI140" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="141" spans="1:35">
@@ -11878,10 +11896,10 @@
         <v>154</v>
       </c>
       <c r="AH141" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI141" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="142" spans="1:35">
@@ -11958,10 +11976,10 @@
         <v>154</v>
       </c>
       <c r="AH142" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI142" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="143" spans="1:35">
@@ -12038,10 +12056,10 @@
         <v>154</v>
       </c>
       <c r="AH143" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI143" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="144" spans="1:35">
@@ -12112,10 +12130,10 @@
         <v>154</v>
       </c>
       <c r="AH144" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI144" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="145" spans="1:35">
@@ -12186,10 +12204,10 @@
         <v>154</v>
       </c>
       <c r="AH145" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI145" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="146" spans="1:35">
@@ -12260,10 +12278,10 @@
         <v>155</v>
       </c>
       <c r="AH146" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI146" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="147" spans="1:35">
@@ -12334,10 +12352,10 @@
         <v>155</v>
       </c>
       <c r="AH147" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI147" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="148" spans="1:35">
@@ -12408,10 +12426,10 @@
         <v>155</v>
       </c>
       <c r="AH148" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI148" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="149" spans="1:35">
@@ -12482,10 +12500,10 @@
         <v>155</v>
       </c>
       <c r="AH149" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI149" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="150" spans="1:35">
@@ -12556,10 +12574,10 @@
         <v>155</v>
       </c>
       <c r="AH150" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI150" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="151" spans="1:35">
@@ -12630,10 +12648,10 @@
         <v>156</v>
       </c>
       <c r="AH151" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI151" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="152" spans="1:35">
@@ -12704,10 +12722,10 @@
         <v>155</v>
       </c>
       <c r="AH152" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI152" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="153" spans="1:35">
@@ -12778,10 +12796,10 @@
         <v>155</v>
       </c>
       <c r="AH153" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI153" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="154" spans="1:35">
@@ -12852,10 +12870,10 @@
         <v>155</v>
       </c>
       <c r="AH154" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI154" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="155" spans="1:35">
@@ -12926,10 +12944,10 @@
         <v>155</v>
       </c>
       <c r="AH155" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI155" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="156" spans="1:35">
@@ -13000,10 +13018,10 @@
         <v>156</v>
       </c>
       <c r="AH156" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI156" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="157" spans="1:35">
@@ -13074,10 +13092,10 @@
         <v>155</v>
       </c>
       <c r="AH157" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI157" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="158" spans="1:35">
@@ -13148,10 +13166,10 @@
         <v>155</v>
       </c>
       <c r="AH158" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI158" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="159" spans="1:35">
@@ -13222,10 +13240,10 @@
         <v>155</v>
       </c>
       <c r="AH159" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI159" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="160" spans="1:35">
@@ -13296,10 +13314,10 @@
         <v>156</v>
       </c>
       <c r="AH160" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI160" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="161" spans="1:35">
@@ -13370,10 +13388,10 @@
         <v>155</v>
       </c>
       <c r="AH161" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI161" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="162" spans="1:35">
@@ -13441,10 +13459,10 @@
         <v>155</v>
       </c>
       <c r="AH162" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI162" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="163" spans="1:35">
@@ -13512,10 +13530,10 @@
         <v>155</v>
       </c>
       <c r="AH163" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI163" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="164" spans="1:35">
@@ -13583,10 +13601,10 @@
         <v>155</v>
       </c>
       <c r="AH164" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI164" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="165" spans="1:35">
@@ -13654,10 +13672,10 @@
         <v>155</v>
       </c>
       <c r="AH165" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI165" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="166" spans="1:35">
@@ -13725,10 +13743,10 @@
         <v>155</v>
       </c>
       <c r="AH166" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI166" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="167" spans="1:35">
@@ -13796,10 +13814,10 @@
         <v>155</v>
       </c>
       <c r="AH167" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI167" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="168" spans="1:35">
@@ -13867,10 +13885,10 @@
         <v>156</v>
       </c>
       <c r="AH168" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI168" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="169" spans="1:35">
@@ -13938,10 +13956,10 @@
         <v>155</v>
       </c>
       <c r="AH169" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI169" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="170" spans="1:35">
@@ -14009,10 +14027,10 @@
         <v>155</v>
       </c>
       <c r="AH170" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI170" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="171" spans="1:35">
@@ -14080,10 +14098,10 @@
         <v>155</v>
       </c>
       <c r="AH171" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI171" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="172" spans="1:35">
@@ -14151,10 +14169,10 @@
         <v>155</v>
       </c>
       <c r="AH172" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI172" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="173" spans="1:35">
@@ -14222,10 +14240,10 @@
         <v>155</v>
       </c>
       <c r="AH173" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI173" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="174" spans="1:35">
@@ -14293,10 +14311,10 @@
         <v>155</v>
       </c>
       <c r="AH174" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI174" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="175" spans="1:35">
@@ -14364,10 +14382,10 @@
         <v>155</v>
       </c>
       <c r="AH175" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI175" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="176" spans="1:35">
@@ -14441,10 +14459,10 @@
         <v>155</v>
       </c>
       <c r="AH176" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI176" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="177" spans="1:35">
@@ -14518,10 +14536,10 @@
         <v>155</v>
       </c>
       <c r="AH177" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI177" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="178" spans="1:35">
@@ -14595,10 +14613,10 @@
         <v>155</v>
       </c>
       <c r="AH178" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI178" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="179" spans="1:35">
@@ -14672,10 +14690,10 @@
         <v>155</v>
       </c>
       <c r="AH179" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI179" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="180" spans="1:35">
@@ -14749,10 +14767,10 @@
         <v>155</v>
       </c>
       <c r="AH180" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI180" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="181" spans="1:35">
@@ -14826,10 +14844,10 @@
         <v>155</v>
       </c>
       <c r="AH181" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI181" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="182" spans="1:35">
@@ -14903,10 +14921,10 @@
         <v>156</v>
       </c>
       <c r="AH182" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI182" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="183" spans="1:35">
@@ -14980,10 +14998,10 @@
         <v>155</v>
       </c>
       <c r="AH183" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI183" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="184" spans="1:35">
@@ -15057,10 +15075,10 @@
         <v>155</v>
       </c>
       <c r="AH184" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI184" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="185" spans="1:35">
@@ -15134,10 +15152,10 @@
         <v>155</v>
       </c>
       <c r="AH185" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI185" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="186" spans="1:35">
@@ -15211,10 +15229,10 @@
         <v>155</v>
       </c>
       <c r="AH186" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI186" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="187" spans="1:35">
@@ -15282,10 +15300,10 @@
         <v>155</v>
       </c>
       <c r="AH187" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI187" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="188" spans="1:35">
@@ -15353,10 +15371,10 @@
         <v>155</v>
       </c>
       <c r="AH188" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI188" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="189" spans="1:35">
@@ -15424,10 +15442,10 @@
         <v>155</v>
       </c>
       <c r="AH189" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI189" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="190" spans="1:35">
@@ -15495,10 +15513,10 @@
         <v>155</v>
       </c>
       <c r="AH190" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI190" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="191" spans="1:35">
@@ -15566,10 +15584,10 @@
         <v>155</v>
       </c>
       <c r="AH191" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI191" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="192" spans="1:35">
@@ -15637,10 +15655,10 @@
         <v>155</v>
       </c>
       <c r="AH192" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI192" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="193" spans="1:35">
@@ -15708,10 +15726,10 @@
         <v>155</v>
       </c>
       <c r="AH193" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI193" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="194" spans="1:35">
@@ -15779,10 +15797,10 @@
         <v>54</v>
       </c>
       <c r="AH194" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI194" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="195" spans="1:35">
@@ -15850,10 +15868,10 @@
         <v>54</v>
       </c>
       <c r="AH195" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI195" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="196" spans="1:35">
@@ -15921,10 +15939,10 @@
         <v>54</v>
       </c>
       <c r="AH196" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI196" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="197" spans="1:35">
@@ -15992,10 +16010,10 @@
         <v>54</v>
       </c>
       <c r="AH197" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI197" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="198" spans="1:35">
@@ -16063,10 +16081,10 @@
         <v>53</v>
       </c>
       <c r="AH198" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI198" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="199" spans="1:35">
@@ -16134,10 +16152,10 @@
         <v>53</v>
       </c>
       <c r="AH199" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI199" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="200" spans="1:35">
@@ -16205,10 +16223,10 @@
         <v>54</v>
       </c>
       <c r="AH200" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI200" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="201" spans="1:35">
@@ -16276,10 +16294,10 @@
         <v>54</v>
       </c>
       <c r="AH201" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI201" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="202" spans="1:35">
@@ -16347,10 +16365,10 @@
         <v>54</v>
       </c>
       <c r="AH202" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI202" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="203" spans="1:35">
@@ -16418,10 +16436,10 @@
         <v>157</v>
       </c>
       <c r="AH203" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI203" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="204" spans="1:35">
@@ -16489,10 +16507,10 @@
         <v>54</v>
       </c>
       <c r="AH204" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI204" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="205" spans="1:35">
@@ -16560,10 +16578,10 @@
         <v>54</v>
       </c>
       <c r="AH205" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI205" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="206" spans="1:35">
@@ -16631,10 +16649,10 @@
         <v>54</v>
       </c>
       <c r="AH206" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI206" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="207" spans="1:35">
@@ -16702,10 +16720,10 @@
         <v>54</v>
       </c>
       <c r="AH207" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI207" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="208" spans="1:35">
@@ -16773,10 +16791,10 @@
         <v>54</v>
       </c>
       <c r="AH208" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI208" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="209" spans="1:35">
@@ -16844,10 +16862,10 @@
         <v>54</v>
       </c>
       <c r="AH209" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI209" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="210" spans="1:35">
@@ -16915,10 +16933,10 @@
         <v>54</v>
       </c>
       <c r="AH210" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI210" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="211" spans="1:35">
@@ -16986,10 +17004,10 @@
         <v>54</v>
       </c>
       <c r="AH211" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI211" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="212" spans="1:35">
@@ -17057,10 +17075,10 @@
         <v>53</v>
       </c>
       <c r="AH212" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI212" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="213" spans="1:35">
@@ -17128,10 +17146,10 @@
         <v>53</v>
       </c>
       <c r="AH213" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI213" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="214" spans="1:35">
@@ -17199,10 +17217,10 @@
         <v>54</v>
       </c>
       <c r="AH214" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI214" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="215" spans="1:35">
@@ -17276,10 +17294,10 @@
         <v>157</v>
       </c>
       <c r="AH215" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI215" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="216" spans="1:35">
@@ -17347,10 +17365,10 @@
         <v>54</v>
       </c>
       <c r="AH216" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI216" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="217" spans="1:35">
@@ -17418,10 +17436,10 @@
         <v>54</v>
       </c>
       <c r="AH217" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI217" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="218" spans="1:35">
@@ -17489,10 +17507,10 @@
         <v>54</v>
       </c>
       <c r="AH218" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI218" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="219" spans="1:35">
@@ -17563,10 +17581,10 @@
         <v>54</v>
       </c>
       <c r="AH219" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI219" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="220" spans="1:35">
@@ -17637,10 +17655,10 @@
         <v>54</v>
       </c>
       <c r="AH220" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI220" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="221" spans="1:35">
@@ -17711,10 +17729,10 @@
         <v>54</v>
       </c>
       <c r="AH221" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI221" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="222" spans="1:35">
@@ -17785,10 +17803,10 @@
         <v>54</v>
       </c>
       <c r="AH222" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI222" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="223" spans="1:35">
@@ -17856,10 +17874,10 @@
         <v>54</v>
       </c>
       <c r="AH223" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI223" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="224" spans="1:35">
@@ -17927,10 +17945,10 @@
         <v>54</v>
       </c>
       <c r="AH224" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI224" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="225" spans="1:35">
@@ -17998,13 +18016,13 @@
         <v>0</v>
       </c>
       <c r="AC225" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="AH225" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI225" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="226" spans="1:35">
@@ -18072,13 +18090,13 @@
         <v>0</v>
       </c>
       <c r="AC226" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="AH226" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI226" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="227" spans="1:35">
@@ -18149,10 +18167,10 @@
         <v>163</v>
       </c>
       <c r="AH227" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI227" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="228" spans="1:35">
@@ -18229,10 +18247,10 @@
         <v>159</v>
       </c>
       <c r="AH228" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI228" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="229" spans="1:35">
@@ -18309,10 +18327,10 @@
         <v>142</v>
       </c>
       <c r="AH229" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI229" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="230" spans="1:35">
@@ -18383,10 +18401,10 @@
         <v>150</v>
       </c>
       <c r="AH230" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI230" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="231" spans="1:35">
@@ -18457,10 +18475,10 @@
         <v>151</v>
       </c>
       <c r="AH231" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI231" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="232" spans="1:35">
@@ -18531,10 +18549,10 @@
         <v>151</v>
       </c>
       <c r="AH232" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="AI232" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="233" spans="1:35">
@@ -18557,7 +18575,7 @@
         <v>56</v>
       </c>
       <c r="G233">
-        <v>1867</v>
+        <v>1866</v>
       </c>
       <c r="H233">
         <v>0</v>
@@ -18566,14 +18584,11 @@
         <v>60</v>
       </c>
       <c r="J233" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N233" s="1">
         <v>46304</v>
       </c>
-      <c r="O233" t="s">
-        <v>131</v>
-      </c>
       <c r="P233">
         <v>9</v>
       </c>
@@ -18581,7 +18596,7 @@
         <v>2026</v>
       </c>
       <c r="R233">
-        <v>18186954</v>
+        <v>18186947</v>
       </c>
       <c r="S233" t="s">
         <v>153</v>
@@ -18593,7 +18608,7 @@
         <v>171</v>
       </c>
       <c r="V233" s="1">
-        <v>46304.64227313657</v>
+        <v>46304.67984788195</v>
       </c>
       <c r="W233">
         <v>0</v>
@@ -18608,21 +18623,21 @@
         <v>0</v>
       </c>
       <c r="AC233" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="AH233" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI233" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="234" spans="1:35">
       <c r="A234">
-        <v>6703</v>
+        <v>6962</v>
       </c>
       <c r="B234" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C234" t="s">
         <v>49</v>
@@ -18634,19 +18649,19 @@
         <v>54</v>
       </c>
       <c r="F234" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G234">
-        <v>1792</v>
+        <v>1867</v>
       </c>
       <c r="H234">
         <v>0</v>
       </c>
       <c r="I234" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J234" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N234" s="1">
         <v>46304</v>
@@ -18661,25 +18676,25 @@
         <v>2026</v>
       </c>
       <c r="R234">
-        <v>17948757</v>
+        <v>18186954</v>
       </c>
       <c r="S234" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="T234" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="U234" t="s">
         <v>171</v>
       </c>
       <c r="V234" s="1">
-        <v>46304.56084105324</v>
+        <v>46304.64227313657</v>
       </c>
       <c r="W234">
         <v>0</v>
       </c>
       <c r="X234" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="Y234" t="s">
         <v>254</v>
@@ -18688,27 +18703,27 @@
         <v>0</v>
       </c>
       <c r="AC234" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="AH234" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI234" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="235" spans="1:35">
       <c r="A235">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B235" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C235" t="s">
         <v>49</v>
       </c>
       <c r="D235" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E235" t="s">
         <v>54</v>
@@ -18717,7 +18732,7 @@
         <v>55</v>
       </c>
       <c r="G235">
-        <v>1793</v>
+        <v>1792</v>
       </c>
       <c r="H235">
         <v>0</v>
@@ -18726,10 +18741,13 @@
         <v>61</v>
       </c>
       <c r="J235" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N235" s="1">
-        <v>46311</v>
+        <v>46304</v>
+      </c>
+      <c r="O235" t="s">
+        <v>131</v>
       </c>
       <c r="P235">
         <v>9</v>
@@ -18738,7 +18756,7 @@
         <v>2026</v>
       </c>
       <c r="R235">
-        <v>17398946</v>
+        <v>17948757</v>
       </c>
       <c r="S235" t="s">
         <v>154</v>
@@ -18747,16 +18765,19 @@
         <v>168</v>
       </c>
       <c r="U235" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="V235" s="1">
-        <v>46304.56110010417</v>
+        <v>46304.56084105324</v>
       </c>
       <c r="W235">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="X235" t="s">
-        <v>178</v>
+        <v>181</v>
+      </c>
+      <c r="Y235" t="s">
+        <v>255</v>
       </c>
       <c r="AB235">
         <v>0</v>
@@ -18765,24 +18786,24 @@
         <v>154</v>
       </c>
       <c r="AH235" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI235" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="236" spans="1:35">
       <c r="A236">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B236" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C236" t="s">
         <v>49</v>
       </c>
       <c r="D236" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E236" t="s">
         <v>54</v>
@@ -18803,7 +18824,7 @@
         <v>102</v>
       </c>
       <c r="N236" s="1">
-        <v>46304</v>
+        <v>46311</v>
       </c>
       <c r="P236">
         <v>9</v>
@@ -18812,7 +18833,7 @@
         <v>2026</v>
       </c>
       <c r="R236">
-        <v>16962162</v>
+        <v>17398946</v>
       </c>
       <c r="S236" t="s">
         <v>154</v>
@@ -18821,16 +18842,16 @@
         <v>168</v>
       </c>
       <c r="U236" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="V236" s="1">
-        <v>46304.62889446759</v>
+        <v>46304.56110010417</v>
       </c>
       <c r="W236">
-        <v>0</v>
+        <v>-7</v>
       </c>
       <c r="X236" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AB236">
         <v>0</v>
@@ -18839,24 +18860,24 @@
         <v>154</v>
       </c>
       <c r="AH236" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI236" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="237" spans="1:35">
       <c r="A237">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B237" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C237" t="s">
         <v>49</v>
       </c>
       <c r="D237" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E237" t="s">
         <v>54</v>
@@ -18886,7 +18907,7 @@
         <v>2026</v>
       </c>
       <c r="R237">
-        <v>16975953</v>
+        <v>16962162</v>
       </c>
       <c r="S237" t="s">
         <v>154</v>
@@ -18898,13 +18919,13 @@
         <v>171</v>
       </c>
       <c r="V237" s="1">
-        <v>46304.62889520833</v>
+        <v>46304.62889446759</v>
       </c>
       <c r="W237">
         <v>0</v>
       </c>
       <c r="X237" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="AB237">
         <v>0</v>
@@ -18913,24 +18934,24 @@
         <v>154</v>
       </c>
       <c r="AH237" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI237" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="238" spans="1:35">
       <c r="A238">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B238" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C238" t="s">
         <v>49</v>
       </c>
       <c r="D238" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E238" t="s">
         <v>54</v>
@@ -18960,7 +18981,7 @@
         <v>2026</v>
       </c>
       <c r="R238">
-        <v>17948767</v>
+        <v>16975953</v>
       </c>
       <c r="S238" t="s">
         <v>154</v>
@@ -18972,13 +18993,13 @@
         <v>171</v>
       </c>
       <c r="V238" s="1">
-        <v>46304.62891434028</v>
+        <v>46304.62889520833</v>
       </c>
       <c r="W238">
         <v>0</v>
       </c>
       <c r="X238" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AB238">
         <v>0</v>
@@ -18987,24 +19008,24 @@
         <v>154</v>
       </c>
       <c r="AH238" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI238" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="239" spans="1:35">
       <c r="A239">
-        <v>6705</v>
+        <v>6703</v>
       </c>
       <c r="B239" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C239" t="s">
         <v>49</v>
       </c>
       <c r="D239" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E239" t="s">
         <v>54</v>
@@ -19034,7 +19055,7 @@
         <v>2026</v>
       </c>
       <c r="R239">
-        <v>17948929</v>
+        <v>17948767</v>
       </c>
       <c r="S239" t="s">
         <v>154</v>
@@ -19046,13 +19067,13 @@
         <v>171</v>
       </c>
       <c r="V239" s="1">
-        <v>46304.62892777778</v>
+        <v>46304.62891434028</v>
       </c>
       <c r="W239">
         <v>0</v>
       </c>
       <c r="X239" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AB239">
         <v>0</v>
@@ -19061,18 +19082,18 @@
         <v>154</v>
       </c>
       <c r="AH239" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI239" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="240" spans="1:35">
       <c r="A240">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B240" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C240" t="s">
         <v>49</v>
@@ -19108,7 +19129,7 @@
         <v>2026</v>
       </c>
       <c r="R240">
-        <v>18084956</v>
+        <v>17948929</v>
       </c>
       <c r="S240" t="s">
         <v>154</v>
@@ -19120,7 +19141,7 @@
         <v>171</v>
       </c>
       <c r="V240" s="1">
-        <v>46304.62893950231</v>
+        <v>46304.62892777778</v>
       </c>
       <c r="W240">
         <v>0</v>
@@ -19135,24 +19156,24 @@
         <v>154</v>
       </c>
       <c r="AH240" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI240" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="241" spans="1:35">
       <c r="A241">
-        <v>5417</v>
+        <v>6779</v>
       </c>
       <c r="B241" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C241" t="s">
         <v>49</v>
       </c>
       <c r="D241" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E241" t="s">
         <v>54</v>
@@ -19161,7 +19182,7 @@
         <v>55</v>
       </c>
       <c r="G241">
-        <v>1796</v>
+        <v>1793</v>
       </c>
       <c r="H241">
         <v>0</v>
@@ -19170,13 +19191,10 @@
         <v>61</v>
       </c>
       <c r="J241" t="s">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="N241" s="1">
-        <v>46303</v>
-      </c>
-      <c r="O241" t="s">
-        <v>131</v>
+        <v>46304</v>
       </c>
       <c r="P241">
         <v>9</v>
@@ -19185,7 +19203,7 @@
         <v>2026</v>
       </c>
       <c r="R241">
-        <v>17398956</v>
+        <v>18084956</v>
       </c>
       <c r="S241" t="s">
         <v>154</v>
@@ -19194,19 +19212,16 @@
         <v>168</v>
       </c>
       <c r="U241" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="V241" s="1">
-        <v>46304.49370603009</v>
+        <v>46304.62893950231</v>
       </c>
       <c r="W241">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X241" t="s">
-        <v>178</v>
-      </c>
-      <c r="Y241" t="s">
-        <v>255</v>
+        <v>179</v>
       </c>
       <c r="AB241">
         <v>0</v>
@@ -19215,24 +19230,24 @@
         <v>154</v>
       </c>
       <c r="AH241" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="AI241" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="242" spans="1:35">
       <c r="A242">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B242" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C242" t="s">
         <v>49</v>
       </c>
       <c r="D242" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E242" t="s">
         <v>54</v>
@@ -19265,7 +19280,7 @@
         <v>2026</v>
       </c>
       <c r="R242">
-        <v>18073099</v>
+        <v>17398956</v>
       </c>
       <c r="S242" t="s">
         <v>154</v>
@@ -19277,16 +19292,16 @@
         <v>169</v>
       </c>
       <c r="V242" s="1">
-        <v>46304.50006596064</v>
+        <v>46304.49370603009</v>
       </c>
       <c r="W242">
         <v>1</v>
       </c>
       <c r="X242" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="Y242" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AB242">
         <v>0</v>
@@ -19295,10 +19310,10 @@
         <v>154</v>
       </c>
       <c r="AH242" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="AI242" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="243" spans="1:35">
@@ -19321,19 +19336,22 @@
         <v>55</v>
       </c>
       <c r="G243">
-        <v>950</v>
+        <v>1796</v>
       </c>
       <c r="H243">
         <v>0</v>
       </c>
       <c r="I243" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J243" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N243" s="1">
-        <v>46304</v>
+        <v>46303</v>
+      </c>
+      <c r="O243" t="s">
+        <v>131</v>
       </c>
       <c r="P243">
         <v>9</v>
@@ -19342,19 +19360,22 @@
         <v>2026</v>
       </c>
       <c r="R243">
-        <v>17941147</v>
+        <v>18073099</v>
       </c>
       <c r="S243" t="s">
-        <v>156</v>
+        <v>154</v>
+      </c>
+      <c r="T243" t="s">
+        <v>168</v>
       </c>
       <c r="U243" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="V243" s="1">
-        <v>46304.66642386574</v>
+        <v>46304.50006596064</v>
       </c>
       <c r="W243">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X243" t="s">
         <v>181</v>
@@ -19366,33 +19387,33 @@
         <v>0</v>
       </c>
       <c r="AC243" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="AH243" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="AI243" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="244" spans="1:35">
       <c r="A244">
-        <v>6949</v>
+        <v>6703</v>
       </c>
       <c r="B244" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C244" t="s">
         <v>49</v>
       </c>
       <c r="D244" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E244" t="s">
         <v>54</v>
       </c>
       <c r="F244" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G244">
         <v>950</v>
@@ -19416,22 +19437,22 @@
         <v>2026</v>
       </c>
       <c r="R244">
-        <v>18178133</v>
+        <v>17941147</v>
       </c>
       <c r="S244" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="U244" t="s">
         <v>171</v>
       </c>
       <c r="V244" s="1">
-        <v>46304.65366649305</v>
+        <v>46304.66642386574</v>
       </c>
       <c r="W244">
         <v>0</v>
       </c>
       <c r="X244" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="Y244" t="s">
         <v>257</v>
@@ -19440,27 +19461,27 @@
         <v>0</v>
       </c>
       <c r="AC244" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="AH244" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI244" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="245" spans="1:35">
       <c r="A245">
-        <v>6963</v>
+        <v>6949</v>
       </c>
       <c r="B245" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C245" t="s">
         <v>49</v>
       </c>
       <c r="D245" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E245" t="s">
         <v>54</v>
@@ -19490,7 +19511,7 @@
         <v>2026</v>
       </c>
       <c r="R245">
-        <v>18188624</v>
+        <v>18178133</v>
       </c>
       <c r="S245" t="s">
         <v>155</v>
@@ -19499,13 +19520,13 @@
         <v>171</v>
       </c>
       <c r="V245" s="1">
-        <v>46304.65441696759</v>
+        <v>46304.65366649305</v>
       </c>
       <c r="W245">
         <v>0</v>
       </c>
       <c r="X245" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Y245" t="s">
         <v>258</v>
@@ -19517,33 +19538,33 @@
         <v>155</v>
       </c>
       <c r="AH245" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI245" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="246" spans="1:35">
       <c r="A246">
-        <v>6628</v>
+        <v>6963</v>
       </c>
       <c r="B246" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C246" t="s">
         <v>49</v>
       </c>
       <c r="D246" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E246" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F246" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G246">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H246">
         <v>0</v>
@@ -19552,7 +19573,7 @@
         <v>62</v>
       </c>
       <c r="J246" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="N246" s="1">
         <v>46304</v>
@@ -19564,7 +19585,7 @@
         <v>2026</v>
       </c>
       <c r="R246">
-        <v>16959951</v>
+        <v>18188624</v>
       </c>
       <c r="S246" t="s">
         <v>155</v>
@@ -19573,13 +19594,16 @@
         <v>171</v>
       </c>
       <c r="V246" s="1">
-        <v>46304.66202476852</v>
+        <v>46304.65441696759</v>
       </c>
       <c r="W246">
         <v>0</v>
       </c>
       <c r="X246" t="s">
-        <v>172</v>
+        <v>176</v>
+      </c>
+      <c r="Y246" t="s">
+        <v>259</v>
       </c>
       <c r="AB246">
         <v>0</v>
@@ -19588,24 +19612,24 @@
         <v>155</v>
       </c>
       <c r="AH246" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI246" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="247" spans="1:35">
       <c r="A247">
-        <v>6705</v>
+        <v>6548</v>
       </c>
       <c r="B247" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="C247" t="s">
         <v>49</v>
       </c>
       <c r="D247" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E247" t="s">
         <v>54</v>
@@ -19635,7 +19659,7 @@
         <v>2026</v>
       </c>
       <c r="R247">
-        <v>17952536</v>
+        <v>17222406</v>
       </c>
       <c r="S247" t="s">
         <v>155</v>
@@ -19644,16 +19668,16 @@
         <v>171</v>
       </c>
       <c r="V247" s="1">
-        <v>46304.66202549769</v>
+        <v>46304.67485967593</v>
       </c>
       <c r="W247">
         <v>0</v>
       </c>
       <c r="X247" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="Y247" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AB247">
         <v>0</v>
@@ -19662,18 +19686,18 @@
         <v>155</v>
       </c>
       <c r="AH247" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI247" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="248" spans="1:35">
       <c r="A248">
-        <v>6779</v>
+        <v>6628</v>
       </c>
       <c r="B248" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C248" t="s">
         <v>49</v>
@@ -19682,7 +19706,7 @@
         <v>51</v>
       </c>
       <c r="E248" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F248" t="s">
         <v>55</v>
@@ -19709,7 +19733,7 @@
         <v>2026</v>
       </c>
       <c r="R248">
-        <v>18056706</v>
+        <v>16959951</v>
       </c>
       <c r="S248" t="s">
         <v>155</v>
@@ -19718,16 +19742,13 @@
         <v>171</v>
       </c>
       <c r="V248" s="1">
-        <v>46304.66202701389</v>
+        <v>46304.66202476852</v>
       </c>
       <c r="W248">
         <v>0</v>
       </c>
       <c r="X248" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y248" t="s">
-        <v>260</v>
+        <v>172</v>
       </c>
       <c r="AB248">
         <v>0</v>
@@ -19736,30 +19757,30 @@
         <v>155</v>
       </c>
       <c r="AH248" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI248" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="249" spans="1:35">
       <c r="A249">
-        <v>6945</v>
+        <v>6703</v>
       </c>
       <c r="B249" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C249" t="s">
         <v>49</v>
       </c>
       <c r="D249" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E249" t="s">
         <v>54</v>
       </c>
       <c r="F249" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G249">
         <v>951</v>
@@ -19783,22 +19804,22 @@
         <v>2026</v>
       </c>
       <c r="R249">
-        <v>18164502</v>
+        <v>17941157</v>
       </c>
       <c r="S249" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="U249" t="s">
         <v>171</v>
       </c>
       <c r="V249" s="1">
-        <v>46304.66203011574</v>
+        <v>46304.68831197917</v>
       </c>
       <c r="W249">
         <v>0</v>
       </c>
       <c r="X249" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="Y249" t="s">
         <v>261</v>
@@ -19807,52 +19828,49 @@
         <v>0</v>
       </c>
       <c r="AC249" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="AH249" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AI249" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="250" spans="1:35">
       <c r="A250">
-        <v>6949</v>
+        <v>6705</v>
       </c>
       <c r="B250" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C250" t="s">
         <v>49</v>
       </c>
       <c r="D250" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E250" t="s">
         <v>54</v>
       </c>
       <c r="F250" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G250">
-        <v>11056</v>
+        <v>951</v>
       </c>
       <c r="H250">
         <v>0</v>
       </c>
       <c r="I250" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="J250" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="N250" s="1">
         <v>46304</v>
       </c>
-      <c r="O250" t="s">
-        <v>131</v>
-      </c>
       <c r="P250">
         <v>9</v>
       </c>
@@ -19860,19 +19878,22 @@
         <v>2026</v>
       </c>
       <c r="R250">
-        <v>18293645</v>
+        <v>17952536</v>
+      </c>
+      <c r="S250" t="s">
+        <v>155</v>
       </c>
       <c r="U250" t="s">
         <v>171</v>
       </c>
       <c r="V250" s="1">
-        <v>46304.42026608796</v>
+        <v>46304.66202549769</v>
       </c>
       <c r="W250">
         <v>0</v>
       </c>
       <c r="X250" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="Y250" t="s">
         <v>262</v>
@@ -19881,13 +19902,457 @@
         <v>0</v>
       </c>
       <c r="AC250" t="s">
+        <v>155</v>
+      </c>
+      <c r="AH250" t="s">
+        <v>272</v>
+      </c>
+      <c r="AI250" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="251" spans="1:35">
+      <c r="A251">
+        <v>6779</v>
+      </c>
+      <c r="B251" t="s">
+        <v>46</v>
+      </c>
+      <c r="C251" t="s">
+        <v>49</v>
+      </c>
+      <c r="D251" t="s">
+        <v>51</v>
+      </c>
+      <c r="E251" t="s">
+        <v>54</v>
+      </c>
+      <c r="F251" t="s">
+        <v>55</v>
+      </c>
+      <c r="G251">
+        <v>951</v>
+      </c>
+      <c r="H251">
+        <v>0</v>
+      </c>
+      <c r="I251" t="s">
+        <v>62</v>
+      </c>
+      <c r="J251" t="s">
+        <v>127</v>
+      </c>
+      <c r="N251" s="1">
+        <v>46304</v>
+      </c>
+      <c r="P251">
+        <v>9</v>
+      </c>
+      <c r="Q251">
+        <v>2026</v>
+      </c>
+      <c r="R251">
+        <v>18056706</v>
+      </c>
+      <c r="S251" t="s">
+        <v>155</v>
+      </c>
+      <c r="U251" t="s">
+        <v>171</v>
+      </c>
+      <c r="V251" s="1">
+        <v>46304.66202701389</v>
+      </c>
+      <c r="W251">
+        <v>0</v>
+      </c>
+      <c r="X251" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y251" t="s">
+        <v>263</v>
+      </c>
+      <c r="AB251">
+        <v>0</v>
+      </c>
+      <c r="AC251" t="s">
+        <v>155</v>
+      </c>
+      <c r="AH251" t="s">
+        <v>272</v>
+      </c>
+      <c r="AI251" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="252" spans="1:35">
+      <c r="A252">
+        <v>6945</v>
+      </c>
+      <c r="B252" t="s">
+        <v>38</v>
+      </c>
+      <c r="C252" t="s">
+        <v>49</v>
+      </c>
+      <c r="D252" t="s">
+        <v>50</v>
+      </c>
+      <c r="E252" t="s">
+        <v>54</v>
+      </c>
+      <c r="F252" t="s">
+        <v>56</v>
+      </c>
+      <c r="G252">
+        <v>951</v>
+      </c>
+      <c r="H252">
+        <v>0</v>
+      </c>
+      <c r="I252" t="s">
+        <v>62</v>
+      </c>
+      <c r="J252" t="s">
+        <v>127</v>
+      </c>
+      <c r="N252" s="1">
+        <v>46304</v>
+      </c>
+      <c r="P252">
+        <v>9</v>
+      </c>
+      <c r="Q252">
+        <v>2026</v>
+      </c>
+      <c r="R252">
+        <v>18164502</v>
+      </c>
+      <c r="S252" t="s">
+        <v>155</v>
+      </c>
+      <c r="U252" t="s">
+        <v>171</v>
+      </c>
+      <c r="V252" s="1">
+        <v>46304.66203011574</v>
+      </c>
+      <c r="W252">
+        <v>0</v>
+      </c>
+      <c r="X252" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y252" t="s">
         <v>264</v>
       </c>
-      <c r="AH250" t="s">
+      <c r="AB252">
+        <v>0</v>
+      </c>
+      <c r="AC252" t="s">
+        <v>155</v>
+      </c>
+      <c r="AH252" t="s">
+        <v>272</v>
+      </c>
+      <c r="AI252" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="253" spans="1:35">
+      <c r="A253">
+        <v>6949</v>
+      </c>
+      <c r="B253" t="s">
+        <v>39</v>
+      </c>
+      <c r="C253" t="s">
+        <v>49</v>
+      </c>
+      <c r="D253" t="s">
+        <v>50</v>
+      </c>
+      <c r="E253" t="s">
+        <v>54</v>
+      </c>
+      <c r="F253" t="s">
+        <v>56</v>
+      </c>
+      <c r="G253">
+        <v>951</v>
+      </c>
+      <c r="H253">
+        <v>0</v>
+      </c>
+      <c r="I253" t="s">
+        <v>62</v>
+      </c>
+      <c r="J253" t="s">
+        <v>127</v>
+      </c>
+      <c r="N253" s="1">
+        <v>46304</v>
+      </c>
+      <c r="P253">
+        <v>9</v>
+      </c>
+      <c r="Q253">
+        <v>2026</v>
+      </c>
+      <c r="R253">
+        <v>18178139</v>
+      </c>
+      <c r="S253" t="s">
+        <v>155</v>
+      </c>
+      <c r="U253" t="s">
+        <v>171</v>
+      </c>
+      <c r="V253" s="1">
+        <v>46304.69242271991</v>
+      </c>
+      <c r="W253">
+        <v>0</v>
+      </c>
+      <c r="X253" t="s">
+        <v>175</v>
+      </c>
+      <c r="Y253" t="s">
         <v>265</v>
       </c>
-      <c r="AI250" t="s">
+      <c r="AB253">
+        <v>0</v>
+      </c>
+      <c r="AC253" t="s">
+        <v>155</v>
+      </c>
+      <c r="AH253" t="s">
+        <v>272</v>
+      </c>
+      <c r="AI253" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="254" spans="1:35">
+      <c r="A254">
+        <v>6962</v>
+      </c>
+      <c r="B254" t="s">
+        <v>40</v>
+      </c>
+      <c r="C254" t="s">
+        <v>49</v>
+      </c>
+      <c r="D254" t="s">
+        <v>52</v>
+      </c>
+      <c r="E254" t="s">
+        <v>54</v>
+      </c>
+      <c r="F254" t="s">
+        <v>56</v>
+      </c>
+      <c r="G254">
+        <v>951</v>
+      </c>
+      <c r="H254">
+        <v>0</v>
+      </c>
+      <c r="I254" t="s">
+        <v>62</v>
+      </c>
+      <c r="J254" t="s">
+        <v>127</v>
+      </c>
+      <c r="N254" s="1">
+        <v>46304</v>
+      </c>
+      <c r="P254">
+        <v>9</v>
+      </c>
+      <c r="Q254">
+        <v>2026</v>
+      </c>
+      <c r="R254">
+        <v>18188725</v>
+      </c>
+      <c r="S254" t="s">
+        <v>155</v>
+      </c>
+      <c r="U254" t="s">
+        <v>171</v>
+      </c>
+      <c r="V254" s="1">
+        <v>46304.69295292824</v>
+      </c>
+      <c r="W254">
+        <v>0</v>
+      </c>
+      <c r="X254" t="s">
+        <v>176</v>
+      </c>
+      <c r="Y254" t="s">
+        <v>266</v>
+      </c>
+      <c r="AB254">
+        <v>0</v>
+      </c>
+      <c r="AC254" t="s">
+        <v>155</v>
+      </c>
+      <c r="AH254" t="s">
+        <v>272</v>
+      </c>
+      <c r="AI254" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="255" spans="1:35">
+      <c r="A255">
+        <v>6963</v>
+      </c>
+      <c r="B255" t="s">
+        <v>41</v>
+      </c>
+      <c r="C255" t="s">
+        <v>49</v>
+      </c>
+      <c r="D255" t="s">
+        <v>52</v>
+      </c>
+      <c r="E255" t="s">
+        <v>54</v>
+      </c>
+      <c r="F255" t="s">
+        <v>56</v>
+      </c>
+      <c r="G255">
+        <v>951</v>
+      </c>
+      <c r="H255">
+        <v>0</v>
+      </c>
+      <c r="I255" t="s">
+        <v>62</v>
+      </c>
+      <c r="J255" t="s">
+        <v>127</v>
+      </c>
+      <c r="N255" s="1">
+        <v>46304</v>
+      </c>
+      <c r="P255">
+        <v>9</v>
+      </c>
+      <c r="Q255">
+        <v>2026</v>
+      </c>
+      <c r="R255">
+        <v>18188631</v>
+      </c>
+      <c r="S255" t="s">
+        <v>155</v>
+      </c>
+      <c r="U255" t="s">
+        <v>171</v>
+      </c>
+      <c r="V255" s="1">
+        <v>46304.69368494213</v>
+      </c>
+      <c r="W255">
+        <v>0</v>
+      </c>
+      <c r="X255" t="s">
+        <v>176</v>
+      </c>
+      <c r="Y255" t="s">
+        <v>267</v>
+      </c>
+      <c r="AB255">
+        <v>0</v>
+      </c>
+      <c r="AC255" t="s">
+        <v>155</v>
+      </c>
+      <c r="AH255" t="s">
+        <v>272</v>
+      </c>
+      <c r="AI255" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="256" spans="1:35">
+      <c r="A256">
+        <v>6949</v>
+      </c>
+      <c r="B256" t="s">
+        <v>39</v>
+      </c>
+      <c r="C256" t="s">
+        <v>49</v>
+      </c>
+      <c r="D256" t="s">
+        <v>50</v>
+      </c>
+      <c r="E256" t="s">
+        <v>54</v>
+      </c>
+      <c r="F256" t="s">
+        <v>56</v>
+      </c>
+      <c r="G256">
+        <v>11056</v>
+      </c>
+      <c r="H256">
+        <v>0</v>
+      </c>
+      <c r="I256" t="s">
+        <v>64</v>
+      </c>
+      <c r="J256" t="s">
+        <v>123</v>
+      </c>
+      <c r="N256" s="1">
+        <v>46304</v>
+      </c>
+      <c r="O256" t="s">
+        <v>131</v>
+      </c>
+      <c r="P256">
+        <v>9</v>
+      </c>
+      <c r="Q256">
+        <v>2026</v>
+      </c>
+      <c r="R256">
+        <v>18293645</v>
+      </c>
+      <c r="U256" t="s">
+        <v>171</v>
+      </c>
+      <c r="V256" s="1">
+        <v>46304.42026608796</v>
+      </c>
+      <c r="W256">
+        <v>0</v>
+      </c>
+      <c r="X256" t="s">
+        <v>175</v>
+      </c>
+      <c r="Y256" t="s">
         <v>268</v>
+      </c>
+      <c r="AB256">
+        <v>0</v>
+      </c>
+      <c r="AC256" t="s">
+        <v>270</v>
+      </c>
+      <c r="AH256" t="s">
+        <v>271</v>
+      </c>
+      <c r="AI256" t="s">
+        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-13 11:18
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3721" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3735" uniqueCount="280">
   <si>
     <t>CodCliente</t>
   </si>
@@ -844,6 +844,9 @@
   </si>
   <si>
     <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-07/10/2026 09:40:49.. - Data Comentário: 07/10/2026 09:35</t>
+  </si>
+  <si>
+    <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 13/10/2026 10:58:54. - Data Comentário: 13/10/2026 10:53</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 09/10/2026 
@@ -1207,7 +1210,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI260"/>
+  <dimension ref="A1:AI261"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -1388,10 +1391,10 @@
         <v>135</v>
       </c>
       <c r="AH2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:35">
@@ -1465,10 +1468,10 @@
         <v>135</v>
       </c>
       <c r="AH3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:35">
@@ -1539,10 +1542,10 @@
         <v>136</v>
       </c>
       <c r="AH4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:35">
@@ -1613,10 +1616,10 @@
         <v>135</v>
       </c>
       <c r="AH5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="1:35">
@@ -1687,10 +1690,10 @@
         <v>135</v>
       </c>
       <c r="AH6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" spans="1:35">
@@ -1761,10 +1764,10 @@
         <v>137</v>
       </c>
       <c r="AH7" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:35">
@@ -1835,10 +1838,10 @@
         <v>136</v>
       </c>
       <c r="AH8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:35">
@@ -1909,10 +1912,10 @@
         <v>138</v>
       </c>
       <c r="AH9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI9" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:35">
@@ -1983,10 +1986,10 @@
         <v>138</v>
       </c>
       <c r="AH10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:35">
@@ -2057,10 +2060,10 @@
         <v>139</v>
       </c>
       <c r="AH11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI11" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:35">
@@ -2134,10 +2137,10 @@
         <v>139</v>
       </c>
       <c r="AH12" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI12" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:35">
@@ -2208,10 +2211,10 @@
         <v>139</v>
       </c>
       <c r="AH13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI13" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" spans="1:35">
@@ -2282,10 +2285,10 @@
         <v>139</v>
       </c>
       <c r="AH14" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" spans="1:35">
@@ -2356,10 +2359,10 @@
         <v>140</v>
       </c>
       <c r="AH15" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI15" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" spans="1:35">
@@ -2430,10 +2433,10 @@
         <v>141</v>
       </c>
       <c r="AH16" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI16" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="17" spans="1:35">
@@ -2504,10 +2507,10 @@
         <v>141</v>
       </c>
       <c r="AH17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI17" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" spans="1:35">
@@ -2578,10 +2581,10 @@
         <v>141</v>
       </c>
       <c r="AH18" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI18" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="19" spans="1:35">
@@ -2652,10 +2655,10 @@
         <v>149</v>
       </c>
       <c r="AH19" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI19" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="20" spans="1:35">
@@ -2726,10 +2729,10 @@
         <v>149</v>
       </c>
       <c r="AH20" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI20" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="21" spans="1:35">
@@ -2800,10 +2803,10 @@
         <v>142</v>
       </c>
       <c r="AH21" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI21" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="22" spans="1:35">
@@ -2877,10 +2880,10 @@
         <v>149</v>
       </c>
       <c r="AH22" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI22" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="23" spans="1:35">
@@ -2957,10 +2960,10 @@
         <v>144</v>
       </c>
       <c r="AH23" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI23" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="24" spans="1:35">
@@ -3037,10 +3040,10 @@
         <v>145</v>
       </c>
       <c r="AH24" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI24" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="25" spans="1:35">
@@ -3111,10 +3114,10 @@
         <v>146</v>
       </c>
       <c r="AH25" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI25" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="26" spans="1:35">
@@ -3185,10 +3188,10 @@
         <v>147</v>
       </c>
       <c r="AH26" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI26" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27" spans="1:35">
@@ -3262,10 +3265,10 @@
         <v>149</v>
       </c>
       <c r="AH27" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI27" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" spans="1:35">
@@ -3339,10 +3342,10 @@
         <v>149</v>
       </c>
       <c r="AH28" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI28" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="29" spans="1:35">
@@ -3413,10 +3416,10 @@
         <v>144</v>
       </c>
       <c r="AH29" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI29" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30" spans="1:35">
@@ -3487,10 +3490,10 @@
         <v>145</v>
       </c>
       <c r="AH30" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI30" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" spans="1:35">
@@ -3567,10 +3570,10 @@
         <v>146</v>
       </c>
       <c r="AH31" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI31" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="32" spans="1:35">
@@ -3644,10 +3647,10 @@
         <v>149</v>
       </c>
       <c r="AH32" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI32" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="33" spans="1:35">
@@ -3721,10 +3724,10 @@
         <v>149</v>
       </c>
       <c r="AH33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" spans="1:35">
@@ -3798,10 +3801,10 @@
         <v>149</v>
       </c>
       <c r="AH34" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI34" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="35" spans="1:35">
@@ -3878,10 +3881,10 @@
         <v>142</v>
       </c>
       <c r="AH35" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI35" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="36" spans="1:35">
@@ -3958,10 +3961,10 @@
         <v>148</v>
       </c>
       <c r="AH36" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI36" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="37" spans="1:35">
@@ -4038,10 +4041,10 @@
         <v>144</v>
       </c>
       <c r="AH37" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI37" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="38" spans="1:35">
@@ -4118,10 +4121,10 @@
         <v>145</v>
       </c>
       <c r="AH38" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI38" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="39" spans="1:35">
@@ -4198,10 +4201,10 @@
         <v>146</v>
       </c>
       <c r="AH39" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI39" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="40" spans="1:35">
@@ -4275,10 +4278,10 @@
         <v>149</v>
       </c>
       <c r="AH40" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI40" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41" spans="1:35">
@@ -4352,10 +4355,10 @@
         <v>149</v>
       </c>
       <c r="AH41" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI41" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="42" spans="1:35">
@@ -4429,10 +4432,10 @@
         <v>149</v>
       </c>
       <c r="AH42" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI42" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="43" spans="1:35">
@@ -4503,10 +4506,10 @@
         <v>142</v>
       </c>
       <c r="AH43" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI43" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="44" spans="1:35">
@@ -4577,10 +4580,10 @@
         <v>148</v>
       </c>
       <c r="AH44" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI44" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="45" spans="1:35">
@@ -4651,10 +4654,10 @@
         <v>144</v>
       </c>
       <c r="AH45" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI45" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="46" spans="1:35">
@@ -4725,10 +4728,10 @@
         <v>145</v>
       </c>
       <c r="AH46" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI46" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="47" spans="1:35">
@@ -4799,10 +4802,10 @@
         <v>147</v>
       </c>
       <c r="AH47" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI47" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="48" spans="1:35">
@@ -4873,10 +4876,10 @@
         <v>148</v>
       </c>
       <c r="AH48" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI48" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="49" spans="1:35">
@@ -4953,10 +4956,10 @@
         <v>148</v>
       </c>
       <c r="AH49" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI49" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="50" spans="1:35">
@@ -5030,10 +5033,10 @@
         <v>149</v>
       </c>
       <c r="AH50" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI50" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="51" spans="1:35">
@@ -5107,10 +5110,10 @@
         <v>149</v>
       </c>
       <c r="AH51" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI51" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="52" spans="1:35">
@@ -5184,10 +5187,10 @@
         <v>149</v>
       </c>
       <c r="AH52" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI52" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="53" spans="1:35">
@@ -5264,10 +5267,10 @@
         <v>142</v>
       </c>
       <c r="AH53" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI53" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="54" spans="1:35">
@@ -5344,10 +5347,10 @@
         <v>146</v>
       </c>
       <c r="AH54" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI54" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="55" spans="1:35">
@@ -5424,10 +5427,10 @@
         <v>148</v>
       </c>
       <c r="AH55" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI55" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="56" spans="1:35">
@@ -5504,10 +5507,10 @@
         <v>146</v>
       </c>
       <c r="AH56" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI56" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="57" spans="1:35">
@@ -5581,10 +5584,10 @@
         <v>149</v>
       </c>
       <c r="AH57" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI57" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="58" spans="1:35">
@@ -5658,10 +5661,10 @@
         <v>149</v>
       </c>
       <c r="AH58" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI58" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="59" spans="1:35">
@@ -5735,10 +5738,10 @@
         <v>149</v>
       </c>
       <c r="AH59" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI59" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="60" spans="1:35">
@@ -5809,10 +5812,10 @@
         <v>142</v>
       </c>
       <c r="AH60" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI60" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="61" spans="1:35">
@@ -5889,10 +5892,10 @@
         <v>148</v>
       </c>
       <c r="AH61" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI61" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="62" spans="1:35">
@@ -5969,10 +5972,10 @@
         <v>144</v>
       </c>
       <c r="AH62" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI62" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="63" spans="1:35">
@@ -6049,10 +6052,10 @@
         <v>145</v>
       </c>
       <c r="AH63" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI63" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="64" spans="1:35">
@@ -6129,10 +6132,10 @@
         <v>149</v>
       </c>
       <c r="AH64" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI64" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="65" spans="1:35">
@@ -6209,10 +6212,10 @@
         <v>146</v>
       </c>
       <c r="AH65" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI65" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="66" spans="1:35">
@@ -6286,10 +6289,10 @@
         <v>149</v>
       </c>
       <c r="AH66" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI66" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="67" spans="1:35">
@@ -6363,10 +6366,10 @@
         <v>149</v>
       </c>
       <c r="AH67" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI67" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="68" spans="1:35">
@@ -6440,10 +6443,10 @@
         <v>149</v>
       </c>
       <c r="AH68" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI68" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="69" spans="1:35">
@@ -6514,10 +6517,10 @@
         <v>142</v>
       </c>
       <c r="AH69" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI69" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="70" spans="1:35">
@@ -6594,10 +6597,10 @@
         <v>148</v>
       </c>
       <c r="AH70" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI70" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="71" spans="1:35">
@@ -6674,10 +6677,10 @@
         <v>144</v>
       </c>
       <c r="AH71" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI71" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="72" spans="1:35">
@@ -6754,10 +6757,10 @@
         <v>145</v>
       </c>
       <c r="AH72" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI72" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="73" spans="1:35">
@@ -6828,10 +6831,10 @@
         <v>149</v>
       </c>
       <c r="AH73" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI73" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="74" spans="1:35">
@@ -6908,10 +6911,10 @@
         <v>145</v>
       </c>
       <c r="AH74" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI74" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="75" spans="1:35">
@@ -6988,10 +6991,10 @@
         <v>145</v>
       </c>
       <c r="AH75" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI75" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="76" spans="1:35">
@@ -7062,10 +7065,10 @@
         <v>150</v>
       </c>
       <c r="AH76" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI76" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="77" spans="1:35">
@@ -7136,10 +7139,10 @@
         <v>151</v>
       </c>
       <c r="AH77" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI77" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="78" spans="1:35">
@@ -7210,10 +7213,10 @@
         <v>151</v>
       </c>
       <c r="AH78" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI78" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="79" spans="1:35">
@@ -7284,10 +7287,10 @@
         <v>150</v>
       </c>
       <c r="AH79" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI79" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="80" spans="1:35">
@@ -7358,10 +7361,10 @@
         <v>151</v>
       </c>
       <c r="AH80" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI80" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="81" spans="1:35">
@@ -7432,10 +7435,10 @@
         <v>150</v>
       </c>
       <c r="AH81" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI81" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="82" spans="1:35">
@@ -7506,10 +7509,10 @@
         <v>151</v>
       </c>
       <c r="AH82" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI82" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="83" spans="1:35">
@@ -7580,10 +7583,10 @@
         <v>152</v>
       </c>
       <c r="AH83" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI83" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="84" spans="1:35">
@@ -7654,10 +7657,10 @@
         <v>150</v>
       </c>
       <c r="AH84" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI84" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="85" spans="1:35">
@@ -7728,10 +7731,10 @@
         <v>151</v>
       </c>
       <c r="AH85" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI85" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="86" spans="1:35">
@@ -7802,10 +7805,10 @@
         <v>152</v>
       </c>
       <c r="AH86" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI86" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="87" spans="1:35">
@@ -7876,10 +7879,10 @@
         <v>150</v>
       </c>
       <c r="AH87" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI87" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="88" spans="1:35">
@@ -7950,10 +7953,10 @@
         <v>151</v>
       </c>
       <c r="AH88" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI88" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="89" spans="1:35">
@@ -8024,10 +8027,10 @@
         <v>151</v>
       </c>
       <c r="AH89" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI89" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="90" spans="1:35">
@@ -8098,10 +8101,10 @@
         <v>167</v>
       </c>
       <c r="AH90" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI90" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="91" spans="1:35">
@@ -8172,10 +8175,10 @@
         <v>151</v>
       </c>
       <c r="AH91" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI91" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="92" spans="1:35">
@@ -8246,10 +8249,10 @@
         <v>150</v>
       </c>
       <c r="AH92" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI92" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="93" spans="1:35">
@@ -8320,10 +8323,10 @@
         <v>151</v>
       </c>
       <c r="AH93" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI93" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="94" spans="1:35">
@@ -8394,10 +8397,10 @@
         <v>152</v>
       </c>
       <c r="AH94" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI94" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="95" spans="1:35">
@@ -8468,10 +8471,10 @@
         <v>167</v>
       </c>
       <c r="AH95" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI95" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="96" spans="1:35">
@@ -8542,10 +8545,10 @@
         <v>150</v>
       </c>
       <c r="AH96" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI96" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="97" spans="1:35">
@@ -8616,10 +8619,10 @@
         <v>151</v>
       </c>
       <c r="AH97" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI97" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="98" spans="1:35">
@@ -8690,10 +8693,10 @@
         <v>151</v>
       </c>
       <c r="AH98" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI98" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="99" spans="1:35">
@@ -8764,10 +8767,10 @@
         <v>151</v>
       </c>
       <c r="AH99" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI99" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="100" spans="1:35">
@@ -8838,10 +8841,10 @@
         <v>151</v>
       </c>
       <c r="AH100" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI100" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="101" spans="1:35">
@@ -8912,10 +8915,10 @@
         <v>150</v>
       </c>
       <c r="AH101" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI101" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="102" spans="1:35">
@@ -8986,10 +8989,10 @@
         <v>151</v>
       </c>
       <c r="AH102" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI102" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="103" spans="1:35">
@@ -9060,10 +9063,10 @@
         <v>151</v>
       </c>
       <c r="AH103" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI103" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="104" spans="1:35">
@@ -9134,10 +9137,10 @@
         <v>150</v>
       </c>
       <c r="AH104" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI104" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="105" spans="1:35">
@@ -9208,10 +9211,10 @@
         <v>151</v>
       </c>
       <c r="AH105" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI105" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="106" spans="1:35">
@@ -9282,10 +9285,10 @@
         <v>152</v>
       </c>
       <c r="AH106" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI106" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="107" spans="1:35">
@@ -9356,10 +9359,10 @@
         <v>150</v>
       </c>
       <c r="AH107" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI107" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="108" spans="1:35">
@@ -9430,10 +9433,10 @@
         <v>151</v>
       </c>
       <c r="AH108" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI108" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="109" spans="1:35">
@@ -9504,10 +9507,10 @@
         <v>152</v>
       </c>
       <c r="AH109" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI109" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="110" spans="1:35">
@@ -9578,10 +9581,10 @@
         <v>151</v>
       </c>
       <c r="AH110" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI110" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="111" spans="1:35">
@@ -9658,10 +9661,10 @@
         <v>151</v>
       </c>
       <c r="AH111" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI111" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="112" spans="1:35">
@@ -9735,10 +9738,10 @@
         <v>151</v>
       </c>
       <c r="AH112" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI112" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="113" spans="1:35">
@@ -9812,10 +9815,10 @@
         <v>153</v>
       </c>
       <c r="AH113" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI113" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="114" spans="1:35">
@@ -9892,10 +9895,10 @@
         <v>150</v>
       </c>
       <c r="AH114" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI114" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="115" spans="1:35">
@@ -9969,10 +9972,10 @@
         <v>151</v>
       </c>
       <c r="AH115" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI115" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="116" spans="1:35">
@@ -10049,10 +10052,10 @@
         <v>151</v>
       </c>
       <c r="AH116" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI116" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="117" spans="1:35">
@@ -10126,10 +10129,10 @@
         <v>151</v>
       </c>
       <c r="AH117" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI117" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="118" spans="1:35">
@@ -10203,10 +10206,10 @@
         <v>153</v>
       </c>
       <c r="AH118" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI118" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="119" spans="1:35">
@@ -10277,10 +10280,10 @@
         <v>154</v>
       </c>
       <c r="AH119" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI119" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="120" spans="1:35">
@@ -10351,10 +10354,10 @@
         <v>154</v>
       </c>
       <c r="AH120" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI120" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="121" spans="1:35">
@@ -10425,10 +10428,10 @@
         <v>154</v>
       </c>
       <c r="AH121" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI121" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="122" spans="1:35">
@@ -10499,10 +10502,10 @@
         <v>154</v>
       </c>
       <c r="AH122" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI122" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="123" spans="1:35">
@@ -10573,10 +10576,10 @@
         <v>154</v>
       </c>
       <c r="AH123" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI123" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="124" spans="1:35">
@@ -10647,10 +10650,10 @@
         <v>154</v>
       </c>
       <c r="AH124" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI124" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="125" spans="1:35">
@@ -10721,10 +10724,10 @@
         <v>154</v>
       </c>
       <c r="AH125" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI125" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="126" spans="1:35">
@@ -10795,10 +10798,10 @@
         <v>154</v>
       </c>
       <c r="AH126" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI126" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="127" spans="1:35">
@@ -10869,10 +10872,10 @@
         <v>154</v>
       </c>
       <c r="AH127" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI127" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="128" spans="1:35">
@@ -10943,10 +10946,10 @@
         <v>154</v>
       </c>
       <c r="AH128" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI128" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="129" spans="1:35">
@@ -11017,10 +11020,10 @@
         <v>154</v>
       </c>
       <c r="AH129" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI129" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="130" spans="1:35">
@@ -11091,10 +11094,10 @@
         <v>154</v>
       </c>
       <c r="AH130" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI130" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="131" spans="1:35">
@@ -11165,10 +11168,10 @@
         <v>154</v>
       </c>
       <c r="AH131" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI131" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="132" spans="1:35">
@@ -11239,10 +11242,10 @@
         <v>154</v>
       </c>
       <c r="AH132" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI132" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="133" spans="1:35">
@@ -11313,10 +11316,10 @@
         <v>154</v>
       </c>
       <c r="AH133" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI133" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="134" spans="1:35">
@@ -11387,10 +11390,10 @@
         <v>154</v>
       </c>
       <c r="AH134" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI134" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="135" spans="1:35">
@@ -11461,10 +11464,10 @@
         <v>154</v>
       </c>
       <c r="AH135" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI135" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="136" spans="1:35">
@@ -11535,10 +11538,10 @@
         <v>154</v>
       </c>
       <c r="AH136" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI136" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="137" spans="1:35">
@@ -11609,10 +11612,10 @@
         <v>154</v>
       </c>
       <c r="AH137" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI137" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="138" spans="1:35">
@@ -11683,10 +11686,10 @@
         <v>154</v>
       </c>
       <c r="AH138" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI138" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="139" spans="1:35">
@@ -11757,10 +11760,10 @@
         <v>154</v>
       </c>
       <c r="AH139" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI139" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="140" spans="1:35">
@@ -11831,10 +11834,10 @@
         <v>154</v>
       </c>
       <c r="AH140" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI140" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="141" spans="1:35">
@@ -11905,10 +11908,10 @@
         <v>154</v>
       </c>
       <c r="AH141" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI141" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="142" spans="1:35">
@@ -11985,10 +11988,10 @@
         <v>154</v>
       </c>
       <c r="AH142" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI142" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="143" spans="1:35">
@@ -12065,10 +12068,10 @@
         <v>154</v>
       </c>
       <c r="AH143" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI143" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="144" spans="1:35">
@@ -12139,10 +12142,10 @@
         <v>154</v>
       </c>
       <c r="AH144" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI144" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="145" spans="1:35">
@@ -12213,10 +12216,10 @@
         <v>154</v>
       </c>
       <c r="AH145" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI145" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="146" spans="1:35">
@@ -12287,10 +12290,10 @@
         <v>155</v>
       </c>
       <c r="AH146" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI146" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="147" spans="1:35">
@@ -12361,10 +12364,10 @@
         <v>155</v>
       </c>
       <c r="AH147" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI147" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="148" spans="1:35">
@@ -12435,10 +12438,10 @@
         <v>155</v>
       </c>
       <c r="AH148" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI148" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="149" spans="1:35">
@@ -12509,10 +12512,10 @@
         <v>155</v>
       </c>
       <c r="AH149" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI149" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="150" spans="1:35">
@@ -12583,10 +12586,10 @@
         <v>155</v>
       </c>
       <c r="AH150" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI150" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="151" spans="1:35">
@@ -12657,10 +12660,10 @@
         <v>156</v>
       </c>
       <c r="AH151" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI151" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="152" spans="1:35">
@@ -12731,10 +12734,10 @@
         <v>155</v>
       </c>
       <c r="AH152" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI152" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="153" spans="1:35">
@@ -12805,10 +12808,10 @@
         <v>155</v>
       </c>
       <c r="AH153" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI153" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="154" spans="1:35">
@@ -12879,10 +12882,10 @@
         <v>155</v>
       </c>
       <c r="AH154" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI154" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="155" spans="1:35">
@@ -12953,10 +12956,10 @@
         <v>155</v>
       </c>
       <c r="AH155" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI155" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="156" spans="1:35">
@@ -13027,10 +13030,10 @@
         <v>156</v>
       </c>
       <c r="AH156" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI156" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="157" spans="1:35">
@@ -13101,10 +13104,10 @@
         <v>155</v>
       </c>
       <c r="AH157" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI157" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="158" spans="1:35">
@@ -13175,10 +13178,10 @@
         <v>155</v>
       </c>
       <c r="AH158" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI158" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="159" spans="1:35">
@@ -13249,10 +13252,10 @@
         <v>155</v>
       </c>
       <c r="AH159" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI159" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="160" spans="1:35">
@@ -13323,10 +13326,10 @@
         <v>156</v>
       </c>
       <c r="AH160" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI160" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="161" spans="1:35">
@@ -13397,10 +13400,10 @@
         <v>155</v>
       </c>
       <c r="AH161" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI161" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="162" spans="1:35">
@@ -13468,10 +13471,10 @@
         <v>155</v>
       </c>
       <c r="AH162" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI162" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="163" spans="1:35">
@@ -13539,10 +13542,10 @@
         <v>155</v>
       </c>
       <c r="AH163" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI163" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="164" spans="1:35">
@@ -13610,10 +13613,10 @@
         <v>155</v>
       </c>
       <c r="AH164" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI164" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="165" spans="1:35">
@@ -13681,10 +13684,10 @@
         <v>155</v>
       </c>
       <c r="AH165" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI165" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="166" spans="1:35">
@@ -13752,10 +13755,10 @@
         <v>155</v>
       </c>
       <c r="AH166" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI166" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="167" spans="1:35">
@@ -13823,10 +13826,10 @@
         <v>155</v>
       </c>
       <c r="AH167" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI167" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="168" spans="1:35">
@@ -13894,10 +13897,10 @@
         <v>156</v>
       </c>
       <c r="AH168" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI168" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="169" spans="1:35">
@@ -13965,10 +13968,10 @@
         <v>155</v>
       </c>
       <c r="AH169" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI169" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="170" spans="1:35">
@@ -14036,10 +14039,10 @@
         <v>155</v>
       </c>
       <c r="AH170" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI170" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="171" spans="1:35">
@@ -14107,10 +14110,10 @@
         <v>155</v>
       </c>
       <c r="AH171" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI171" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="172" spans="1:35">
@@ -14178,10 +14181,10 @@
         <v>155</v>
       </c>
       <c r="AH172" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI172" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="173" spans="1:35">
@@ -14249,10 +14252,10 @@
         <v>155</v>
       </c>
       <c r="AH173" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI173" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="174" spans="1:35">
@@ -14320,10 +14323,10 @@
         <v>155</v>
       </c>
       <c r="AH174" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI174" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="175" spans="1:35">
@@ -14391,10 +14394,10 @@
         <v>155</v>
       </c>
       <c r="AH175" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI175" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="176" spans="1:35">
@@ -14468,10 +14471,10 @@
         <v>155</v>
       </c>
       <c r="AH176" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI176" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="177" spans="1:35">
@@ -14545,10 +14548,10 @@
         <v>155</v>
       </c>
       <c r="AH177" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI177" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="178" spans="1:35">
@@ -14622,10 +14625,10 @@
         <v>155</v>
       </c>
       <c r="AH178" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI178" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="179" spans="1:35">
@@ -14699,10 +14702,10 @@
         <v>155</v>
       </c>
       <c r="AH179" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI179" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="180" spans="1:35">
@@ -14776,10 +14779,10 @@
         <v>155</v>
       </c>
       <c r="AH180" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI180" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="181" spans="1:35">
@@ -14853,10 +14856,10 @@
         <v>155</v>
       </c>
       <c r="AH181" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI181" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="182" spans="1:35">
@@ -14930,10 +14933,10 @@
         <v>156</v>
       </c>
       <c r="AH182" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI182" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="183" spans="1:35">
@@ -15007,10 +15010,10 @@
         <v>155</v>
       </c>
       <c r="AH183" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI183" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="184" spans="1:35">
@@ -15084,10 +15087,10 @@
         <v>155</v>
       </c>
       <c r="AH184" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI184" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="185" spans="1:35">
@@ -15161,10 +15164,10 @@
         <v>155</v>
       </c>
       <c r="AH185" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI185" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="186" spans="1:35">
@@ -15238,10 +15241,10 @@
         <v>155</v>
       </c>
       <c r="AH186" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI186" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="187" spans="1:35">
@@ -15309,10 +15312,10 @@
         <v>155</v>
       </c>
       <c r="AH187" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI187" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="188" spans="1:35">
@@ -15380,10 +15383,10 @@
         <v>155</v>
       </c>
       <c r="AH188" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI188" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="189" spans="1:35">
@@ -15451,10 +15454,10 @@
         <v>155</v>
       </c>
       <c r="AH189" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI189" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="190" spans="1:35">
@@ -15522,10 +15525,10 @@
         <v>155</v>
       </c>
       <c r="AH190" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI190" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="191" spans="1:35">
@@ -15593,10 +15596,10 @@
         <v>155</v>
       </c>
       <c r="AH191" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI191" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="192" spans="1:35">
@@ -15664,10 +15667,10 @@
         <v>155</v>
       </c>
       <c r="AH192" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI192" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="193" spans="1:35">
@@ -15735,10 +15738,10 @@
         <v>155</v>
       </c>
       <c r="AH193" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI193" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="194" spans="1:35">
@@ -15806,10 +15809,10 @@
         <v>54</v>
       </c>
       <c r="AH194" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI194" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="195" spans="1:35">
@@ -15877,10 +15880,10 @@
         <v>54</v>
       </c>
       <c r="AH195" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI195" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="196" spans="1:35">
@@ -15948,10 +15951,10 @@
         <v>54</v>
       </c>
       <c r="AH196" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI196" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="197" spans="1:35">
@@ -16019,10 +16022,10 @@
         <v>54</v>
       </c>
       <c r="AH197" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI197" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="198" spans="1:35">
@@ -16090,10 +16093,10 @@
         <v>53</v>
       </c>
       <c r="AH198" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI198" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="199" spans="1:35">
@@ -16161,10 +16164,10 @@
         <v>53</v>
       </c>
       <c r="AH199" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI199" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="200" spans="1:35">
@@ -16232,10 +16235,10 @@
         <v>54</v>
       </c>
       <c r="AH200" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI200" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="201" spans="1:35">
@@ -16303,10 +16306,10 @@
         <v>54</v>
       </c>
       <c r="AH201" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI201" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="202" spans="1:35">
@@ -16374,10 +16377,10 @@
         <v>54</v>
       </c>
       <c r="AH202" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI202" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="203" spans="1:35">
@@ -16445,10 +16448,10 @@
         <v>157</v>
       </c>
       <c r="AH203" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI203" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="204" spans="1:35">
@@ -16516,10 +16519,10 @@
         <v>54</v>
       </c>
       <c r="AH204" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI204" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="205" spans="1:35">
@@ -16587,10 +16590,10 @@
         <v>54</v>
       </c>
       <c r="AH205" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI205" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="206" spans="1:35">
@@ -16658,10 +16661,10 @@
         <v>54</v>
       </c>
       <c r="AH206" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI206" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="207" spans="1:35">
@@ -16729,10 +16732,10 @@
         <v>54</v>
       </c>
       <c r="AH207" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI207" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="208" spans="1:35">
@@ -16800,10 +16803,10 @@
         <v>54</v>
       </c>
       <c r="AH208" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI208" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="209" spans="1:35">
@@ -16871,10 +16874,10 @@
         <v>54</v>
       </c>
       <c r="AH209" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI209" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="210" spans="1:35">
@@ -16942,10 +16945,10 @@
         <v>54</v>
       </c>
       <c r="AH210" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI210" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="211" spans="1:35">
@@ -17013,10 +17016,10 @@
         <v>54</v>
       </c>
       <c r="AH211" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI211" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="212" spans="1:35">
@@ -17084,10 +17087,10 @@
         <v>53</v>
       </c>
       <c r="AH212" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI212" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="213" spans="1:35">
@@ -17155,10 +17158,10 @@
         <v>53</v>
       </c>
       <c r="AH213" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI213" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="214" spans="1:35">
@@ -17226,10 +17229,10 @@
         <v>54</v>
       </c>
       <c r="AH214" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI214" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="215" spans="1:35">
@@ -17303,10 +17306,10 @@
         <v>157</v>
       </c>
       <c r="AH215" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI215" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="216" spans="1:35">
@@ -17374,10 +17377,10 @@
         <v>54</v>
       </c>
       <c r="AH216" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI216" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="217" spans="1:35">
@@ -17445,10 +17448,10 @@
         <v>54</v>
       </c>
       <c r="AH217" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI217" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="218" spans="1:35">
@@ -17516,10 +17519,10 @@
         <v>54</v>
       </c>
       <c r="AH218" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI218" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="219" spans="1:35">
@@ -17590,10 +17593,10 @@
         <v>54</v>
       </c>
       <c r="AH219" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI219" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="220" spans="1:35">
@@ -17664,10 +17667,10 @@
         <v>54</v>
       </c>
       <c r="AH220" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI220" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="221" spans="1:35">
@@ -17738,10 +17741,10 @@
         <v>54</v>
       </c>
       <c r="AH221" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI221" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="222" spans="1:35">
@@ -17812,10 +17815,10 @@
         <v>54</v>
       </c>
       <c r="AH222" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI222" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="223" spans="1:35">
@@ -17883,10 +17886,10 @@
         <v>54</v>
       </c>
       <c r="AH223" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI223" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="224" spans="1:35">
@@ -17954,10 +17957,10 @@
         <v>54</v>
       </c>
       <c r="AH224" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI224" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="225" spans="1:35">
@@ -18025,13 +18028,13 @@
         <v>0</v>
       </c>
       <c r="AC225" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AH225" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI225" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="226" spans="1:35">
@@ -18099,13 +18102,13 @@
         <v>0</v>
       </c>
       <c r="AC226" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AH226" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI226" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="227" spans="1:35">
@@ -18176,10 +18179,10 @@
         <v>140</v>
       </c>
       <c r="AH227" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI227" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="228" spans="1:35">
@@ -18250,10 +18253,10 @@
         <v>163</v>
       </c>
       <c r="AH228" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI228" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="229" spans="1:35">
@@ -18330,10 +18333,10 @@
         <v>159</v>
       </c>
       <c r="AH229" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI229" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="230" spans="1:35">
@@ -18410,10 +18413,10 @@
         <v>142</v>
       </c>
       <c r="AH230" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI230" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="231" spans="1:35">
@@ -18484,10 +18487,10 @@
         <v>150</v>
       </c>
       <c r="AH231" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI231" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="232" spans="1:35">
@@ -18558,10 +18561,10 @@
         <v>152</v>
       </c>
       <c r="AH232" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI232" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="233" spans="1:35">
@@ -18632,10 +18635,10 @@
         <v>151</v>
       </c>
       <c r="AH233" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI233" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="234" spans="1:35">
@@ -18706,10 +18709,10 @@
         <v>151</v>
       </c>
       <c r="AH234" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AI234" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="235" spans="1:35">
@@ -18783,10 +18786,10 @@
         <v>153</v>
       </c>
       <c r="AH235" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI235" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="236" spans="1:35">
@@ -18863,10 +18866,10 @@
         <v>167</v>
       </c>
       <c r="AH236" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI236" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="237" spans="1:35">
@@ -18940,10 +18943,10 @@
         <v>154</v>
       </c>
       <c r="AH237" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI237" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="238" spans="1:35">
@@ -19020,10 +19023,10 @@
         <v>154</v>
       </c>
       <c r="AH238" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI238" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="239" spans="1:35">
@@ -19094,10 +19097,10 @@
         <v>154</v>
       </c>
       <c r="AH239" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI239" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="240" spans="1:35">
@@ -19168,10 +19171,10 @@
         <v>154</v>
       </c>
       <c r="AH240" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI240" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="241" spans="1:35">
@@ -19242,10 +19245,10 @@
         <v>154</v>
       </c>
       <c r="AH241" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI241" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="242" spans="1:35">
@@ -19316,10 +19319,10 @@
         <v>154</v>
       </c>
       <c r="AH242" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI242" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="243" spans="1:35">
@@ -19390,10 +19393,10 @@
         <v>154</v>
       </c>
       <c r="AH243" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI243" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="244" spans="1:35">
@@ -19464,10 +19467,10 @@
         <v>154</v>
       </c>
       <c r="AH244" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI244" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="245" spans="1:35">
@@ -19544,10 +19547,10 @@
         <v>154</v>
       </c>
       <c r="AH245" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI245" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="246" spans="1:35">
@@ -19624,10 +19627,10 @@
         <v>154</v>
       </c>
       <c r="AH246" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AI246" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="247" spans="1:35">
@@ -19698,10 +19701,10 @@
         <v>156</v>
       </c>
       <c r="AH247" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI247" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="248" spans="1:35">
@@ -19772,10 +19775,10 @@
         <v>155</v>
       </c>
       <c r="AH248" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI248" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="249" spans="1:35">
@@ -19846,10 +19849,10 @@
         <v>155</v>
       </c>
       <c r="AH249" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI249" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="250" spans="1:35">
@@ -19920,10 +19923,10 @@
         <v>155</v>
       </c>
       <c r="AH250" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI250" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="251" spans="1:35">
@@ -19994,10 +19997,10 @@
         <v>155</v>
       </c>
       <c r="AH251" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI251" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="252" spans="1:35">
@@ -20065,10 +20068,10 @@
         <v>155</v>
       </c>
       <c r="AH252" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI252" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="253" spans="1:35">
@@ -20139,10 +20142,10 @@
         <v>156</v>
       </c>
       <c r="AH253" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI253" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="254" spans="1:35">
@@ -20213,10 +20216,10 @@
         <v>155</v>
       </c>
       <c r="AH254" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI254" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="255" spans="1:35">
@@ -20287,10 +20290,10 @@
         <v>155</v>
       </c>
       <c r="AH255" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI255" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="256" spans="1:35">
@@ -20361,10 +20364,10 @@
         <v>155</v>
       </c>
       <c r="AH256" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI256" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="257" spans="1:35">
@@ -20435,10 +20438,10 @@
         <v>155</v>
       </c>
       <c r="AH257" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI257" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="258" spans="1:35">
@@ -20509,10 +20512,10 @@
         <v>155</v>
       </c>
       <c r="AH258" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI258" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="259" spans="1:35">
@@ -20583,18 +20586,18 @@
         <v>155</v>
       </c>
       <c r="AH259" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AI259" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="260" spans="1:35">
       <c r="A260">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B260" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C260" t="s">
         <v>49</v>
@@ -20606,25 +20609,22 @@
         <v>54</v>
       </c>
       <c r="F260" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G260">
-        <v>11056</v>
+        <v>7027</v>
       </c>
       <c r="H260">
         <v>0</v>
       </c>
       <c r="I260" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J260" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N260" s="1">
-        <v>46304</v>
-      </c>
-      <c r="O260" t="s">
-        <v>131</v>
+        <v>46321</v>
       </c>
       <c r="P260">
         <v>9</v>
@@ -20633,19 +20633,22 @@
         <v>2026</v>
       </c>
       <c r="R260">
-        <v>18293645</v>
+        <v>17399291</v>
+      </c>
+      <c r="S260" t="s">
+        <v>54</v>
       </c>
       <c r="U260" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="V260" s="1">
-        <v>46304.42026608796</v>
+        <v>46308.4550522338</v>
       </c>
       <c r="W260">
-        <v>4</v>
+        <v>-13</v>
       </c>
       <c r="X260" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="Y260" t="s">
         <v>270</v>
@@ -20654,13 +20657,87 @@
         <v>0</v>
       </c>
       <c r="AC260" t="s">
-        <v>272</v>
+        <v>54</v>
       </c>
       <c r="AH260" t="s">
+        <v>274</v>
+      </c>
+      <c r="AI260" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="261" spans="1:35">
+      <c r="A261">
+        <v>6949</v>
+      </c>
+      <c r="B261" t="s">
+        <v>39</v>
+      </c>
+      <c r="C261" t="s">
+        <v>49</v>
+      </c>
+      <c r="D261" t="s">
+        <v>50</v>
+      </c>
+      <c r="E261" t="s">
+        <v>54</v>
+      </c>
+      <c r="F261" t="s">
+        <v>56</v>
+      </c>
+      <c r="G261">
+        <v>11056</v>
+      </c>
+      <c r="H261">
+        <v>0</v>
+      </c>
+      <c r="I261" t="s">
+        <v>64</v>
+      </c>
+      <c r="J261" t="s">
+        <v>123</v>
+      </c>
+      <c r="N261" s="1">
+        <v>46304</v>
+      </c>
+      <c r="O261" t="s">
+        <v>131</v>
+      </c>
+      <c r="P261">
+        <v>9</v>
+      </c>
+      <c r="Q261">
+        <v>2026</v>
+      </c>
+      <c r="R261">
+        <v>18293645</v>
+      </c>
+      <c r="U261" t="s">
+        <v>171</v>
+      </c>
+      <c r="V261" s="1">
+        <v>46304.42026608796</v>
+      </c>
+      <c r="W261">
+        <v>4</v>
+      </c>
+      <c r="X261" t="s">
+        <v>175</v>
+      </c>
+      <c r="Y261" t="s">
+        <v>271</v>
+      </c>
+      <c r="AB261">
+        <v>0</v>
+      </c>
+      <c r="AC261" t="s">
         <v>273</v>
       </c>
-      <c r="AI260" t="s">
-        <v>276</v>
+      <c r="AH261" t="s">
+        <v>274</v>
+      </c>
+      <c r="AI261" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-15 09:36
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4270" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4318" uniqueCount="311">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1307,7 +1307,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI297"/>
+  <dimension ref="A1:AI300"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -20668,10 +20668,10 @@
     </row>
     <row r="259" spans="1:35">
       <c r="A259">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B259" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C259" t="s">
         <v>49</v>
@@ -20686,7 +20686,7 @@
         <v>55</v>
       </c>
       <c r="G259">
-        <v>7025</v>
+        <v>6806</v>
       </c>
       <c r="H259">
         <v>0</v>
@@ -20695,10 +20695,13 @@
         <v>61</v>
       </c>
       <c r="J259" t="s">
-        <v>122</v>
+        <v>100</v>
       </c>
       <c r="N259" s="1">
-        <v>46318</v>
+        <v>46308</v>
+      </c>
+      <c r="O259" t="s">
+        <v>140</v>
       </c>
       <c r="P259">
         <v>9</v>
@@ -20707,7 +20710,7 @@
         <v>2026</v>
       </c>
       <c r="R259">
-        <v>17399281</v>
+        <v>18085298</v>
       </c>
       <c r="S259" t="s">
         <v>162</v>
@@ -20716,19 +20719,19 @@
         <v>176</v>
       </c>
       <c r="U259" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="V259" s="1">
-        <v>46308.41418804398</v>
+        <v>46310.39575521991</v>
       </c>
       <c r="W259">
-        <v>-8</v>
+        <v>2</v>
       </c>
       <c r="X259" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="Y259" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="AB259">
         <v>0</v>
@@ -20737,7 +20740,7 @@
         <v>162</v>
       </c>
       <c r="AH259" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="AI259" t="s">
         <v>310</v>
@@ -20745,16 +20748,16 @@
     </row>
     <row r="260" spans="1:35">
       <c r="A260">
-        <v>6703</v>
+        <v>6705</v>
       </c>
       <c r="B260" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C260" t="s">
         <v>49</v>
       </c>
       <c r="D260" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E260" t="s">
         <v>54</v>
@@ -20763,7 +20766,7 @@
         <v>55</v>
       </c>
       <c r="G260">
-        <v>1792</v>
+        <v>6806</v>
       </c>
       <c r="H260">
         <v>0</v>
@@ -20772,13 +20775,13 @@
         <v>61</v>
       </c>
       <c r="J260" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="N260" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O260" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="P260">
         <v>9</v>
@@ -20787,7 +20790,7 @@
         <v>2026</v>
       </c>
       <c r="R260">
-        <v>17948757</v>
+        <v>17949030</v>
       </c>
       <c r="S260" t="s">
         <v>162</v>
@@ -20796,19 +20799,19 @@
         <v>176</v>
       </c>
       <c r="U260" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="V260" s="1">
-        <v>46304.56084105324</v>
+        <v>46310.39575559027</v>
       </c>
       <c r="W260">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="X260" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="Y260" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="AB260">
         <v>0</v>
@@ -20817,24 +20820,24 @@
         <v>162</v>
       </c>
       <c r="AH260" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="AI260" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="261" spans="1:35">
       <c r="A261">
-        <v>6704</v>
+        <v>6779</v>
       </c>
       <c r="B261" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C261" t="s">
         <v>49</v>
       </c>
       <c r="D261" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E261" t="s">
         <v>54</v>
@@ -20843,7 +20846,7 @@
         <v>55</v>
       </c>
       <c r="G261">
-        <v>1792</v>
+        <v>6806</v>
       </c>
       <c r="H261">
         <v>0</v>
@@ -20852,13 +20855,13 @@
         <v>61</v>
       </c>
       <c r="J261" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="N261" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O261" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="P261">
         <v>9</v>
@@ -20867,7 +20870,7 @@
         <v>2026</v>
       </c>
       <c r="R261">
-        <v>18085144</v>
+        <v>18085067</v>
       </c>
       <c r="S261" t="s">
         <v>162</v>
@@ -20879,16 +20882,16 @@
         <v>177</v>
       </c>
       <c r="V261" s="1">
-        <v>46309.65179342592</v>
+        <v>46310.39575600695</v>
       </c>
       <c r="W261">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="X261" t="s">
         <v>187</v>
       </c>
       <c r="Y261" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="AB261">
         <v>0</v>
@@ -20897,7 +20900,7 @@
         <v>162</v>
       </c>
       <c r="AH261" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="AI261" t="s">
         <v>310</v>
@@ -20923,7 +20926,7 @@
         <v>55</v>
       </c>
       <c r="G262">
-        <v>1793</v>
+        <v>7025</v>
       </c>
       <c r="H262">
         <v>0</v>
@@ -20932,10 +20935,10 @@
         <v>61</v>
       </c>
       <c r="J262" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="N262" s="1">
-        <v>46311</v>
+        <v>46318</v>
       </c>
       <c r="P262">
         <v>9</v>
@@ -20944,7 +20947,7 @@
         <v>2026</v>
       </c>
       <c r="R262">
-        <v>17398946</v>
+        <v>17399281</v>
       </c>
       <c r="S262" t="s">
         <v>162</v>
@@ -20956,14 +20959,17 @@
         <v>178</v>
       </c>
       <c r="V262" s="1">
-        <v>46304.56110010417</v>
+        <v>46308.41418804398</v>
       </c>
       <c r="W262">
-        <v>-1</v>
+        <v>-8</v>
       </c>
       <c r="X262" t="s">
         <v>186</v>
       </c>
+      <c r="Y262" t="s">
+        <v>280</v>
+      </c>
       <c r="AB262">
         <v>0</v>
       </c>
@@ -20971,18 +20977,18 @@
         <v>162</v>
       </c>
       <c r="AH262" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AI262" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="263" spans="1:35">
       <c r="A263">
-        <v>6404</v>
+        <v>6703</v>
       </c>
       <c r="B263" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C263" t="s">
         <v>49</v>
@@ -20997,7 +21003,7 @@
         <v>55</v>
       </c>
       <c r="G263">
-        <v>1793</v>
+        <v>1792</v>
       </c>
       <c r="H263">
         <v>0</v>
@@ -21006,11 +21012,14 @@
         <v>61</v>
       </c>
       <c r="J263" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N263" s="1">
         <v>46304</v>
       </c>
+      <c r="O263" t="s">
+        <v>136</v>
+      </c>
       <c r="P263">
         <v>9</v>
       </c>
@@ -21018,7 +21027,7 @@
         <v>2026</v>
       </c>
       <c r="R263">
-        <v>16962162</v>
+        <v>17948757</v>
       </c>
       <c r="S263" t="s">
         <v>162</v>
@@ -21030,13 +21039,16 @@
         <v>179</v>
       </c>
       <c r="V263" s="1">
-        <v>46304.62889446759</v>
+        <v>46304.56084105324</v>
       </c>
       <c r="W263">
         <v>6</v>
       </c>
       <c r="X263" t="s">
-        <v>185</v>
+        <v>189</v>
+      </c>
+      <c r="Y263" t="s">
+        <v>281</v>
       </c>
       <c r="AB263">
         <v>0</v>
@@ -21053,10 +21065,10 @@
     </row>
     <row r="264" spans="1:35">
       <c r="A264">
-        <v>6486</v>
+        <v>6704</v>
       </c>
       <c r="B264" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C264" t="s">
         <v>49</v>
@@ -21071,7 +21083,7 @@
         <v>55</v>
       </c>
       <c r="G264">
-        <v>1793</v>
+        <v>1792</v>
       </c>
       <c r="H264">
         <v>0</v>
@@ -21080,11 +21092,14 @@
         <v>61</v>
       </c>
       <c r="J264" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N264" s="1">
         <v>46304</v>
       </c>
+      <c r="O264" t="s">
+        <v>142</v>
+      </c>
       <c r="P264">
         <v>9</v>
       </c>
@@ -21092,7 +21107,7 @@
         <v>2026</v>
       </c>
       <c r="R264">
-        <v>16975953</v>
+        <v>18085144</v>
       </c>
       <c r="S264" t="s">
         <v>162</v>
@@ -21101,16 +21116,19 @@
         <v>176</v>
       </c>
       <c r="U264" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="V264" s="1">
-        <v>46304.62889520833</v>
+        <v>46309.65179342592</v>
       </c>
       <c r="W264">
         <v>6</v>
       </c>
       <c r="X264" t="s">
-        <v>188</v>
+        <v>187</v>
+      </c>
+      <c r="Y264" t="s">
+        <v>282</v>
       </c>
       <c r="AB264">
         <v>0</v>
@@ -21122,21 +21140,21 @@
         <v>306</v>
       </c>
       <c r="AI264" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="265" spans="1:35">
       <c r="A265">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B265" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C265" t="s">
         <v>49</v>
       </c>
       <c r="D265" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E265" t="s">
         <v>54</v>
@@ -21157,7 +21175,7 @@
         <v>102</v>
       </c>
       <c r="N265" s="1">
-        <v>46304</v>
+        <v>46311</v>
       </c>
       <c r="P265">
         <v>9</v>
@@ -21166,7 +21184,7 @@
         <v>2026</v>
       </c>
       <c r="R265">
-        <v>17948767</v>
+        <v>17398946</v>
       </c>
       <c r="S265" t="s">
         <v>162</v>
@@ -21175,16 +21193,16 @@
         <v>176</v>
       </c>
       <c r="U265" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="V265" s="1">
-        <v>46304.62891434028</v>
+        <v>46304.56110010417</v>
       </c>
       <c r="W265">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="X265" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AB265">
         <v>0</v>
@@ -21201,16 +21219,16 @@
     </row>
     <row r="266" spans="1:35">
       <c r="A266">
-        <v>6705</v>
+        <v>6404</v>
       </c>
       <c r="B266" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C266" t="s">
         <v>49</v>
       </c>
       <c r="D266" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E266" t="s">
         <v>54</v>
@@ -21240,7 +21258,7 @@
         <v>2026</v>
       </c>
       <c r="R266">
-        <v>17948929</v>
+        <v>16962162</v>
       </c>
       <c r="S266" t="s">
         <v>162</v>
@@ -21252,13 +21270,13 @@
         <v>179</v>
       </c>
       <c r="V266" s="1">
-        <v>46304.62892777778</v>
+        <v>46304.62889446759</v>
       </c>
       <c r="W266">
         <v>6</v>
       </c>
       <c r="X266" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="AB266">
         <v>0</v>
@@ -21275,16 +21293,16 @@
     </row>
     <row r="267" spans="1:35">
       <c r="A267">
-        <v>6779</v>
+        <v>6486</v>
       </c>
       <c r="B267" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C267" t="s">
         <v>49</v>
       </c>
       <c r="D267" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E267" t="s">
         <v>54</v>
@@ -21314,7 +21332,7 @@
         <v>2026</v>
       </c>
       <c r="R267">
-        <v>18084956</v>
+        <v>16975953</v>
       </c>
       <c r="S267" t="s">
         <v>162</v>
@@ -21326,13 +21344,13 @@
         <v>179</v>
       </c>
       <c r="V267" s="1">
-        <v>46304.62893950231</v>
+        <v>46304.62889520833</v>
       </c>
       <c r="W267">
         <v>6</v>
       </c>
       <c r="X267" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AB267">
         <v>0</v>
@@ -21349,16 +21367,16 @@
     </row>
     <row r="268" spans="1:35">
       <c r="A268">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B268" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C268" t="s">
         <v>49</v>
       </c>
       <c r="D268" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E268" t="s">
         <v>54</v>
@@ -21367,7 +21385,7 @@
         <v>55</v>
       </c>
       <c r="G268">
-        <v>1796</v>
+        <v>1793</v>
       </c>
       <c r="H268">
         <v>0</v>
@@ -21376,13 +21394,10 @@
         <v>61</v>
       </c>
       <c r="J268" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="N268" s="1">
-        <v>46303</v>
-      </c>
-      <c r="O268" t="s">
-        <v>136</v>
+        <v>46304</v>
       </c>
       <c r="P268">
         <v>9</v>
@@ -21391,7 +21406,7 @@
         <v>2026</v>
       </c>
       <c r="R268">
-        <v>17398956</v>
+        <v>17948767</v>
       </c>
       <c r="S268" t="s">
         <v>162</v>
@@ -21400,19 +21415,16 @@
         <v>176</v>
       </c>
       <c r="U268" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="V268" s="1">
-        <v>46304.49370603009</v>
+        <v>46304.62891434028</v>
       </c>
       <c r="W268">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X268" t="s">
-        <v>186</v>
-      </c>
-      <c r="Y268" t="s">
-        <v>283</v>
+        <v>189</v>
       </c>
       <c r="AB268">
         <v>0</v>
@@ -21421,7 +21433,7 @@
         <v>162</v>
       </c>
       <c r="AH268" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="AI268" t="s">
         <v>308</v>
@@ -21429,16 +21441,16 @@
     </row>
     <row r="269" spans="1:35">
       <c r="A269">
-        <v>6703</v>
+        <v>6705</v>
       </c>
       <c r="B269" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C269" t="s">
         <v>49</v>
       </c>
       <c r="D269" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E269" t="s">
         <v>54</v>
@@ -21447,7 +21459,7 @@
         <v>55</v>
       </c>
       <c r="G269">
-        <v>1796</v>
+        <v>1793</v>
       </c>
       <c r="H269">
         <v>0</v>
@@ -21456,13 +21468,10 @@
         <v>61</v>
       </c>
       <c r="J269" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="N269" s="1">
-        <v>46303</v>
-      </c>
-      <c r="O269" t="s">
-        <v>136</v>
+        <v>46304</v>
       </c>
       <c r="P269">
         <v>9</v>
@@ -21471,7 +21480,7 @@
         <v>2026</v>
       </c>
       <c r="R269">
-        <v>18073099</v>
+        <v>17948929</v>
       </c>
       <c r="S269" t="s">
         <v>162</v>
@@ -21480,19 +21489,16 @@
         <v>176</v>
       </c>
       <c r="U269" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="V269" s="1">
-        <v>46304.50006596064</v>
+        <v>46304.62892777778</v>
       </c>
       <c r="W269">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X269" t="s">
-        <v>189</v>
-      </c>
-      <c r="Y269" t="s">
-        <v>283</v>
+        <v>187</v>
       </c>
       <c r="AB269">
         <v>0</v>
@@ -21501,7 +21507,7 @@
         <v>162</v>
       </c>
       <c r="AH269" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="AI269" t="s">
         <v>308</v>
@@ -21509,10 +21515,10 @@
     </row>
     <row r="270" spans="1:35">
       <c r="A270">
-        <v>6705</v>
+        <v>6779</v>
       </c>
       <c r="B270" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C270" t="s">
         <v>49</v>
@@ -21527,19 +21533,19 @@
         <v>55</v>
       </c>
       <c r="G270">
-        <v>6294</v>
+        <v>1793</v>
       </c>
       <c r="H270">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I270" t="s">
         <v>61</v>
       </c>
       <c r="J270" t="s">
-        <v>129</v>
+        <v>102</v>
       </c>
       <c r="N270" s="1">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="P270">
         <v>9</v>
@@ -21548,7 +21554,7 @@
         <v>2026</v>
       </c>
       <c r="R270">
-        <v>17949000</v>
+        <v>18084956</v>
       </c>
       <c r="S270" t="s">
         <v>162</v>
@@ -21560,10 +21566,10 @@
         <v>179</v>
       </c>
       <c r="V270" s="1">
-        <v>46308.56276559028</v>
+        <v>46304.62893950231</v>
       </c>
       <c r="W270">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="X270" t="s">
         <v>187</v>
@@ -21575,24 +21581,24 @@
         <v>162</v>
       </c>
       <c r="AH270" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="AI270" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="271" spans="1:35">
       <c r="A271">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B271" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C271" t="s">
         <v>49</v>
       </c>
       <c r="D271" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E271" t="s">
         <v>54</v>
@@ -21601,19 +21607,22 @@
         <v>55</v>
       </c>
       <c r="G271">
-        <v>950</v>
+        <v>1796</v>
       </c>
       <c r="H271">
         <v>0</v>
       </c>
       <c r="I271" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J271" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="N271" s="1">
-        <v>46304</v>
+        <v>46303</v>
+      </c>
+      <c r="O271" t="s">
+        <v>136</v>
       </c>
       <c r="P271">
         <v>9</v>
@@ -21622,34 +21631,37 @@
         <v>2026</v>
       </c>
       <c r="R271">
-        <v>17941147</v>
+        <v>17398956</v>
       </c>
       <c r="S271" t="s">
-        <v>164</v>
+        <v>162</v>
+      </c>
+      <c r="T271" t="s">
+        <v>176</v>
       </c>
       <c r="U271" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="V271" s="1">
-        <v>46304.66642386574</v>
+        <v>46304.49370603009</v>
       </c>
       <c r="W271">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X271" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="Y271" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="AB271">
         <v>0</v>
       </c>
       <c r="AC271" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="AH271" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AI271" t="s">
         <v>308</v>
@@ -21657,16 +21669,16 @@
     </row>
     <row r="272" spans="1:35">
       <c r="A272">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B272" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C272" t="s">
         <v>49</v>
       </c>
       <c r="D272" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E272" t="s">
         <v>54</v>
@@ -21675,22 +21687,22 @@
         <v>55</v>
       </c>
       <c r="G272">
-        <v>950</v>
+        <v>1796</v>
       </c>
       <c r="H272">
         <v>0</v>
       </c>
       <c r="I272" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J272" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="N272" s="1">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="O272" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="P272">
         <v>9</v>
@@ -21699,72 +21711,75 @@
         <v>2026</v>
       </c>
       <c r="R272">
-        <v>17952341</v>
+        <v>18073099</v>
       </c>
       <c r="S272" t="s">
-        <v>163</v>
+        <v>162</v>
+      </c>
+      <c r="T272" t="s">
+        <v>176</v>
       </c>
       <c r="U272" t="s">
         <v>177</v>
       </c>
       <c r="V272" s="1">
-        <v>46309.68758141204</v>
+        <v>46304.50006596064</v>
       </c>
       <c r="W272">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X272" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="Y272" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="AB272">
         <v>0</v>
       </c>
       <c r="AC272" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AH272" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AI272" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="273" spans="1:35">
       <c r="A273">
-        <v>6949</v>
+        <v>6705</v>
       </c>
       <c r="B273" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C273" t="s">
         <v>49</v>
       </c>
       <c r="D273" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E273" t="s">
         <v>54</v>
       </c>
       <c r="F273" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G273">
-        <v>950</v>
+        <v>6294</v>
       </c>
       <c r="H273">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I273" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J273" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N273" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="P273">
         <v>9</v>
@@ -21773,45 +21788,45 @@
         <v>2026</v>
       </c>
       <c r="R273">
-        <v>18178133</v>
+        <v>17949000</v>
       </c>
       <c r="S273" t="s">
-        <v>163</v>
+        <v>162</v>
+      </c>
+      <c r="T273" t="s">
+        <v>176</v>
       </c>
       <c r="U273" t="s">
         <v>179</v>
       </c>
       <c r="V273" s="1">
-        <v>46304.65366649305</v>
+        <v>46308.56276559028</v>
       </c>
       <c r="W273">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="X273" t="s">
-        <v>183</v>
-      </c>
-      <c r="Y273" t="s">
-        <v>286</v>
+        <v>187</v>
       </c>
       <c r="AB273">
         <v>0</v>
       </c>
       <c r="AC273" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AH273" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AI273" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="274" spans="1:35">
       <c r="A274">
-        <v>6962</v>
+        <v>6703</v>
       </c>
       <c r="B274" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C274" t="s">
         <v>49</v>
@@ -21823,7 +21838,7 @@
         <v>54</v>
       </c>
       <c r="F274" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G274">
         <v>950</v>
@@ -21847,31 +21862,31 @@
         <v>2026</v>
       </c>
       <c r="R274">
-        <v>18188718</v>
+        <v>17941147</v>
       </c>
       <c r="S274" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="U274" t="s">
         <v>179</v>
       </c>
       <c r="V274" s="1">
-        <v>46304.71076834491</v>
+        <v>46304.66642386574</v>
       </c>
       <c r="W274">
         <v>6</v>
       </c>
       <c r="X274" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="Y274" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="AB274">
         <v>0</v>
       </c>
       <c r="AC274" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AH274" t="s">
         <v>306</v>
@@ -21882,22 +21897,22 @@
     </row>
     <row r="275" spans="1:35">
       <c r="A275">
-        <v>6963</v>
+        <v>6704</v>
       </c>
       <c r="B275" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C275" t="s">
         <v>49</v>
       </c>
       <c r="D275" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E275" t="s">
         <v>54</v>
       </c>
       <c r="F275" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G275">
         <v>950</v>
@@ -21914,6 +21929,9 @@
       <c r="N275" s="1">
         <v>46304</v>
       </c>
+      <c r="O275" t="s">
+        <v>142</v>
+      </c>
       <c r="P275">
         <v>9</v>
       </c>
@@ -21921,25 +21939,25 @@
         <v>2026</v>
       </c>
       <c r="R275">
-        <v>18188624</v>
+        <v>17952341</v>
       </c>
       <c r="S275" t="s">
         <v>163</v>
       </c>
       <c r="U275" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="V275" s="1">
-        <v>46304.65441696759</v>
+        <v>46309.68758141204</v>
       </c>
       <c r="W275">
         <v>6</v>
       </c>
       <c r="X275" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="Y275" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="AB275">
         <v>0</v>
@@ -21951,15 +21969,15 @@
         <v>306</v>
       </c>
       <c r="AI275" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="276" spans="1:35">
       <c r="A276">
-        <v>6548</v>
+        <v>6949</v>
       </c>
       <c r="B276" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C276" t="s">
         <v>49</v>
@@ -21971,10 +21989,10 @@
         <v>54</v>
       </c>
       <c r="F276" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G276">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H276">
         <v>0</v>
@@ -21983,7 +22001,7 @@
         <v>62</v>
       </c>
       <c r="J276" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N276" s="1">
         <v>46304</v>
@@ -21995,7 +22013,7 @@
         <v>2026</v>
       </c>
       <c r="R276">
-        <v>17222406</v>
+        <v>18178133</v>
       </c>
       <c r="S276" t="s">
         <v>163</v>
@@ -22004,16 +22022,16 @@
         <v>179</v>
       </c>
       <c r="V276" s="1">
-        <v>46304.67485967593</v>
+        <v>46304.65366649305</v>
       </c>
       <c r="W276">
         <v>6</v>
       </c>
       <c r="X276" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="Y276" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="AB276">
         <v>0</v>
@@ -22030,25 +22048,25 @@
     </row>
     <row r="277" spans="1:35">
       <c r="A277">
-        <v>6628</v>
+        <v>6962</v>
       </c>
       <c r="B277" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C277" t="s">
         <v>49</v>
       </c>
       <c r="D277" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E277" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F277" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G277">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H277">
         <v>0</v>
@@ -22057,7 +22075,7 @@
         <v>62</v>
       </c>
       <c r="J277" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N277" s="1">
         <v>46304</v>
@@ -22069,7 +22087,7 @@
         <v>2026</v>
       </c>
       <c r="R277">
-        <v>16959951</v>
+        <v>18188718</v>
       </c>
       <c r="S277" t="s">
         <v>163</v>
@@ -22078,13 +22096,16 @@
         <v>179</v>
       </c>
       <c r="V277" s="1">
-        <v>46304.66202476852</v>
+        <v>46304.71076834491</v>
       </c>
       <c r="W277">
         <v>6</v>
       </c>
       <c r="X277" t="s">
-        <v>180</v>
+        <v>184</v>
+      </c>
+      <c r="Y277" t="s">
+        <v>287</v>
       </c>
       <c r="AB277">
         <v>0</v>
@@ -22101,10 +22122,10 @@
     </row>
     <row r="278" spans="1:35">
       <c r="A278">
-        <v>6703</v>
+        <v>6963</v>
       </c>
       <c r="B278" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C278" t="s">
         <v>49</v>
@@ -22116,10 +22137,10 @@
         <v>54</v>
       </c>
       <c r="F278" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G278">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H278">
         <v>0</v>
@@ -22128,7 +22149,7 @@
         <v>62</v>
       </c>
       <c r="J278" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N278" s="1">
         <v>46304</v>
@@ -22140,31 +22161,31 @@
         <v>2026</v>
       </c>
       <c r="R278">
-        <v>17941157</v>
+        <v>18188624</v>
       </c>
       <c r="S278" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="U278" t="s">
         <v>179</v>
       </c>
       <c r="V278" s="1">
-        <v>46304.68831197917</v>
+        <v>46304.65441696759</v>
       </c>
       <c r="W278">
         <v>6</v>
       </c>
       <c r="X278" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="Y278" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="AB278">
         <v>0</v>
       </c>
       <c r="AC278" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AH278" t="s">
         <v>306</v>
@@ -22175,16 +22196,16 @@
     </row>
     <row r="279" spans="1:35">
       <c r="A279">
-        <v>6705</v>
+        <v>6548</v>
       </c>
       <c r="B279" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="C279" t="s">
         <v>49</v>
       </c>
       <c r="D279" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E279" t="s">
         <v>54</v>
@@ -22214,7 +22235,7 @@
         <v>2026</v>
       </c>
       <c r="R279">
-        <v>17952536</v>
+        <v>17222406</v>
       </c>
       <c r="S279" t="s">
         <v>163</v>
@@ -22223,16 +22244,16 @@
         <v>179</v>
       </c>
       <c r="V279" s="1">
-        <v>46304.66202549769</v>
+        <v>46304.67485967593</v>
       </c>
       <c r="W279">
         <v>6</v>
       </c>
       <c r="X279" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="Y279" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="AB279">
         <v>0</v>
@@ -22249,10 +22270,10 @@
     </row>
     <row r="280" spans="1:35">
       <c r="A280">
-        <v>6779</v>
+        <v>6628</v>
       </c>
       <c r="B280" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C280" t="s">
         <v>49</v>
@@ -22261,7 +22282,7 @@
         <v>51</v>
       </c>
       <c r="E280" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F280" t="s">
         <v>55</v>
@@ -22288,7 +22309,7 @@
         <v>2026</v>
       </c>
       <c r="R280">
-        <v>18056706</v>
+        <v>16959951</v>
       </c>
       <c r="S280" t="s">
         <v>163</v>
@@ -22297,16 +22318,13 @@
         <v>179</v>
       </c>
       <c r="V280" s="1">
-        <v>46304.66202701389</v>
+        <v>46304.66202476852</v>
       </c>
       <c r="W280">
         <v>6</v>
       </c>
       <c r="X280" t="s">
-        <v>187</v>
-      </c>
-      <c r="Y280" t="s">
-        <v>292</v>
+        <v>180</v>
       </c>
       <c r="AB280">
         <v>0</v>
@@ -22323,22 +22341,22 @@
     </row>
     <row r="281" spans="1:35">
       <c r="A281">
-        <v>6945</v>
+        <v>6703</v>
       </c>
       <c r="B281" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C281" t="s">
         <v>49</v>
       </c>
       <c r="D281" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E281" t="s">
         <v>54</v>
       </c>
       <c r="F281" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G281">
         <v>951</v>
@@ -22362,31 +22380,31 @@
         <v>2026</v>
       </c>
       <c r="R281">
-        <v>18164502</v>
+        <v>17941157</v>
       </c>
       <c r="S281" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="U281" t="s">
         <v>179</v>
       </c>
       <c r="V281" s="1">
-        <v>46304.66203011574</v>
+        <v>46304.68831197917</v>
       </c>
       <c r="W281">
         <v>6</v>
       </c>
       <c r="X281" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="Y281" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="AB281">
         <v>0</v>
       </c>
       <c r="AC281" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AH281" t="s">
         <v>306</v>
@@ -22397,22 +22415,22 @@
     </row>
     <row r="282" spans="1:35">
       <c r="A282">
-        <v>6949</v>
+        <v>6705</v>
       </c>
       <c r="B282" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C282" t="s">
         <v>49</v>
       </c>
       <c r="D282" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E282" t="s">
         <v>54</v>
       </c>
       <c r="F282" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G282">
         <v>951</v>
@@ -22436,7 +22454,7 @@
         <v>2026</v>
       </c>
       <c r="R282">
-        <v>18178139</v>
+        <v>17952536</v>
       </c>
       <c r="S282" t="s">
         <v>163</v>
@@ -22445,16 +22463,16 @@
         <v>179</v>
       </c>
       <c r="V282" s="1">
-        <v>46304.69242271991</v>
+        <v>46304.66202549769</v>
       </c>
       <c r="W282">
         <v>6</v>
       </c>
       <c r="X282" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="Y282" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="AB282">
         <v>0</v>
@@ -22471,22 +22489,22 @@
     </row>
     <row r="283" spans="1:35">
       <c r="A283">
-        <v>6962</v>
+        <v>6779</v>
       </c>
       <c r="B283" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="C283" t="s">
         <v>49</v>
       </c>
       <c r="D283" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E283" t="s">
         <v>54</v>
       </c>
       <c r="F283" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G283">
         <v>951</v>
@@ -22510,7 +22528,7 @@
         <v>2026</v>
       </c>
       <c r="R283">
-        <v>18188725</v>
+        <v>18056706</v>
       </c>
       <c r="S283" t="s">
         <v>163</v>
@@ -22519,16 +22537,16 @@
         <v>179</v>
       </c>
       <c r="V283" s="1">
-        <v>46304.69295292824</v>
+        <v>46304.66202701389</v>
       </c>
       <c r="W283">
         <v>6</v>
       </c>
       <c r="X283" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="Y283" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="AB283">
         <v>0</v>
@@ -22545,16 +22563,16 @@
     </row>
     <row r="284" spans="1:35">
       <c r="A284">
-        <v>6963</v>
+        <v>6945</v>
       </c>
       <c r="B284" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C284" t="s">
         <v>49</v>
       </c>
       <c r="D284" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E284" t="s">
         <v>54</v>
@@ -22584,7 +22602,7 @@
         <v>2026</v>
       </c>
       <c r="R284">
-        <v>18188631</v>
+        <v>18164502</v>
       </c>
       <c r="S284" t="s">
         <v>163</v>
@@ -22593,16 +22611,16 @@
         <v>179</v>
       </c>
       <c r="V284" s="1">
-        <v>46304.69368494213</v>
+        <v>46304.66203011574</v>
       </c>
       <c r="W284">
         <v>6</v>
       </c>
       <c r="X284" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="Y284" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="AB284">
         <v>0</v>
@@ -22619,10 +22637,10 @@
     </row>
     <row r="285" spans="1:35">
       <c r="A285">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B285" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C285" t="s">
         <v>49</v>
@@ -22634,25 +22652,22 @@
         <v>54</v>
       </c>
       <c r="F285" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G285">
-        <v>11746</v>
+        <v>951</v>
       </c>
       <c r="H285">
         <v>0</v>
       </c>
       <c r="I285" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J285" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="N285" s="1">
-        <v>46308</v>
-      </c>
-      <c r="O285" t="s">
-        <v>142</v>
+        <v>46304</v>
       </c>
       <c r="P285">
         <v>9</v>
@@ -22661,45 +22676,45 @@
         <v>2026</v>
       </c>
       <c r="R285">
-        <v>17994312</v>
+        <v>18178139</v>
       </c>
       <c r="S285" t="s">
-        <v>54</v>
+        <v>163</v>
       </c>
       <c r="U285" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="V285" s="1">
-        <v>46309.40991104166</v>
+        <v>46304.69242271991</v>
       </c>
       <c r="W285">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="X285" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="Y285" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="AB285">
         <v>0</v>
       </c>
       <c r="AC285" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="AH285" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="AI285" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="286" spans="1:35">
       <c r="A286">
-        <v>6404</v>
+        <v>6962</v>
       </c>
       <c r="B286" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C286" t="s">
         <v>49</v>
@@ -22711,25 +22726,22 @@
         <v>54</v>
       </c>
       <c r="F286" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G286">
-        <v>11746</v>
+        <v>951</v>
       </c>
       <c r="H286">
         <v>0</v>
       </c>
       <c r="I286" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J286" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="N286" s="1">
-        <v>46308</v>
-      </c>
-      <c r="O286" t="s">
-        <v>142</v>
+        <v>46304</v>
       </c>
       <c r="P286">
         <v>9</v>
@@ -22738,75 +22750,72 @@
         <v>2026</v>
       </c>
       <c r="R286">
-        <v>17994676</v>
+        <v>18188725</v>
       </c>
       <c r="S286" t="s">
-        <v>54</v>
+        <v>163</v>
       </c>
       <c r="U286" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="V286" s="1">
-        <v>46309.41020521991</v>
+        <v>46304.69295292824</v>
       </c>
       <c r="W286">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="X286" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Y286" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="AB286">
         <v>0</v>
       </c>
       <c r="AC286" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="AH286" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="AI286" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="287" spans="1:35">
       <c r="A287">
-        <v>6486</v>
+        <v>6963</v>
       </c>
       <c r="B287" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C287" t="s">
         <v>49</v>
       </c>
       <c r="D287" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E287" t="s">
         <v>54</v>
       </c>
       <c r="F287" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G287">
-        <v>11746</v>
+        <v>951</v>
       </c>
       <c r="H287">
         <v>0</v>
       </c>
       <c r="I287" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J287" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="N287" s="1">
-        <v>46308</v>
-      </c>
-      <c r="O287" t="s">
-        <v>142</v>
+        <v>46304</v>
       </c>
       <c r="P287">
         <v>9</v>
@@ -22815,45 +22824,45 @@
         <v>2026</v>
       </c>
       <c r="R287">
-        <v>17994810</v>
+        <v>18188631</v>
       </c>
       <c r="S287" t="s">
-        <v>54</v>
+        <v>163</v>
       </c>
       <c r="U287" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="V287" s="1">
-        <v>46309.41022715278</v>
+        <v>46304.69368494213</v>
       </c>
       <c r="W287">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="X287" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="Y287" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="AB287">
         <v>0</v>
       </c>
       <c r="AC287" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="AH287" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="AI287" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="288" spans="1:35">
       <c r="A288">
-        <v>6548</v>
+        <v>5417</v>
       </c>
       <c r="B288" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C288" t="s">
         <v>49</v>
@@ -22892,7 +22901,7 @@
         <v>2026</v>
       </c>
       <c r="R288">
-        <v>18006052</v>
+        <v>17994312</v>
       </c>
       <c r="S288" t="s">
         <v>54</v>
@@ -22901,13 +22910,13 @@
         <v>177</v>
       </c>
       <c r="V288" s="1">
-        <v>46309.41024563657</v>
+        <v>46309.40991104166</v>
       </c>
       <c r="W288">
         <v>2</v>
       </c>
       <c r="X288" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="Y288" t="s">
         <v>297</v>
@@ -22927,19 +22936,19 @@
     </row>
     <row r="289" spans="1:35">
       <c r="A289">
-        <v>6628</v>
+        <v>6404</v>
       </c>
       <c r="B289" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C289" t="s">
         <v>49</v>
       </c>
       <c r="D289" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E289" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F289" t="s">
         <v>55</v>
@@ -22969,22 +22978,22 @@
         <v>2026</v>
       </c>
       <c r="R289">
-        <v>18003257</v>
+        <v>17994676</v>
       </c>
       <c r="S289" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="U289" t="s">
         <v>177</v>
       </c>
       <c r="V289" s="1">
-        <v>46309.41025899306</v>
+        <v>46309.41020521991</v>
       </c>
       <c r="W289">
         <v>2</v>
       </c>
       <c r="X289" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="Y289" t="s">
         <v>297</v>
@@ -23004,16 +23013,16 @@
     </row>
     <row r="290" spans="1:35">
       <c r="A290">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B290" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C290" t="s">
         <v>49</v>
       </c>
       <c r="D290" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E290" t="s">
         <v>54</v>
@@ -23046,7 +23055,7 @@
         <v>2026</v>
       </c>
       <c r="R290">
-        <v>18004018</v>
+        <v>17994810</v>
       </c>
       <c r="S290" t="s">
         <v>54</v>
@@ -23055,13 +23064,13 @@
         <v>177</v>
       </c>
       <c r="V290" s="1">
-        <v>46309.41028034722</v>
+        <v>46309.41022715278</v>
       </c>
       <c r="W290">
         <v>2</v>
       </c>
       <c r="X290" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="Y290" t="s">
         <v>297</v>
@@ -23081,10 +23090,10 @@
     </row>
     <row r="291" spans="1:35">
       <c r="A291">
-        <v>6704</v>
+        <v>6548</v>
       </c>
       <c r="B291" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C291" t="s">
         <v>49</v>
@@ -23123,7 +23132,7 @@
         <v>2026</v>
       </c>
       <c r="R291">
-        <v>17995165</v>
+        <v>18006052</v>
       </c>
       <c r="S291" t="s">
         <v>54</v>
@@ -23132,13 +23141,13 @@
         <v>177</v>
       </c>
       <c r="V291" s="1">
-        <v>46309.41028116898</v>
+        <v>46309.41024563657</v>
       </c>
       <c r="W291">
         <v>2</v>
       </c>
       <c r="X291" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="Y291" t="s">
         <v>297</v>
@@ -23158,10 +23167,10 @@
     </row>
     <row r="292" spans="1:35">
       <c r="A292">
-        <v>6705</v>
+        <v>6628</v>
       </c>
       <c r="B292" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C292" t="s">
         <v>49</v>
@@ -23170,7 +23179,7 @@
         <v>51</v>
       </c>
       <c r="E292" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F292" t="s">
         <v>55</v>
@@ -23200,22 +23209,22 @@
         <v>2026</v>
       </c>
       <c r="R292">
-        <v>18004029</v>
+        <v>18003257</v>
       </c>
       <c r="S292" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="U292" t="s">
         <v>177</v>
       </c>
       <c r="V292" s="1">
-        <v>46309.41028195602</v>
+        <v>46309.41025899306</v>
       </c>
       <c r="W292">
         <v>2</v>
       </c>
       <c r="X292" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="Y292" t="s">
         <v>297</v>
@@ -23235,16 +23244,16 @@
     </row>
     <row r="293" spans="1:35">
       <c r="A293">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B293" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C293" t="s">
         <v>49</v>
       </c>
       <c r="D293" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E293" t="s">
         <v>54</v>
@@ -23253,7 +23262,7 @@
         <v>55</v>
       </c>
       <c r="G293">
-        <v>7027</v>
+        <v>11746</v>
       </c>
       <c r="H293">
         <v>0</v>
@@ -23262,10 +23271,13 @@
         <v>63</v>
       </c>
       <c r="J293" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="N293" s="1">
-        <v>46321</v>
+        <v>46308</v>
+      </c>
+      <c r="O293" t="s">
+        <v>142</v>
       </c>
       <c r="P293">
         <v>9</v>
@@ -23274,31 +23286,31 @@
         <v>2026</v>
       </c>
       <c r="R293">
-        <v>17399291</v>
+        <v>18004018</v>
       </c>
       <c r="S293" t="s">
         <v>54</v>
       </c>
       <c r="U293" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="V293" s="1">
-        <v>46308.4550522338</v>
+        <v>46309.41028034722</v>
       </c>
       <c r="W293">
-        <v>-11</v>
+        <v>2</v>
       </c>
       <c r="X293" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="Y293" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="AB293">
         <v>0</v>
       </c>
       <c r="AC293" t="s">
-        <v>54</v>
+        <v>165</v>
       </c>
       <c r="AH293" t="s">
         <v>305</v>
@@ -23309,10 +23321,10 @@
     </row>
     <row r="294" spans="1:35">
       <c r="A294">
-        <v>6945</v>
+        <v>6704</v>
       </c>
       <c r="B294" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C294" t="s">
         <v>49</v>
@@ -23324,22 +23336,25 @@
         <v>54</v>
       </c>
       <c r="F294" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G294">
-        <v>11056</v>
+        <v>11746</v>
       </c>
       <c r="H294">
         <v>0</v>
       </c>
       <c r="I294" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J294" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="N294" s="1">
-        <v>46316</v>
+        <v>46308</v>
+      </c>
+      <c r="O294" t="s">
+        <v>142</v>
       </c>
       <c r="P294">
         <v>9</v>
@@ -23348,28 +23363,31 @@
         <v>2026</v>
       </c>
       <c r="R294">
-        <v>18300939</v>
+        <v>17995165</v>
+      </c>
+      <c r="S294" t="s">
+        <v>54</v>
       </c>
       <c r="U294" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="V294" s="1">
-        <v>46309.68971350694</v>
+        <v>46309.41028116898</v>
       </c>
       <c r="W294">
-        <v>-6</v>
+        <v>2</v>
       </c>
       <c r="X294" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="Y294" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="AB294">
         <v>0</v>
       </c>
       <c r="AC294" t="s">
-        <v>303</v>
+        <v>165</v>
       </c>
       <c r="AH294" t="s">
         <v>305</v>
@@ -23380,40 +23398,40 @@
     </row>
     <row r="295" spans="1:35">
       <c r="A295">
-        <v>6949</v>
+        <v>6705</v>
       </c>
       <c r="B295" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C295" t="s">
         <v>49</v>
       </c>
       <c r="D295" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E295" t="s">
         <v>54</v>
       </c>
       <c r="F295" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G295">
-        <v>11056</v>
+        <v>11746</v>
       </c>
       <c r="H295">
         <v>0</v>
       </c>
       <c r="I295" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J295" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="N295" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O295" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="P295">
         <v>9</v>
@@ -23422,42 +23440,45 @@
         <v>2026</v>
       </c>
       <c r="R295">
-        <v>18293645</v>
+        <v>18004029</v>
+      </c>
+      <c r="S295" t="s">
+        <v>54</v>
       </c>
       <c r="U295" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="V295" s="1">
-        <v>46304.42026608796</v>
+        <v>46309.41028195602</v>
       </c>
       <c r="W295">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="X295" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="Y295" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="AB295">
         <v>0</v>
       </c>
       <c r="AC295" t="s">
-        <v>304</v>
+        <v>165</v>
       </c>
       <c r="AH295" t="s">
         <v>305</v>
       </c>
       <c r="AI295" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="296" spans="1:35">
       <c r="A296">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B296" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C296" t="s">
         <v>49</v>
@@ -23469,22 +23490,22 @@
         <v>54</v>
       </c>
       <c r="F296" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G296">
-        <v>11056</v>
+        <v>7027</v>
       </c>
       <c r="H296">
         <v>0</v>
       </c>
       <c r="I296" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J296" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N296" s="1">
-        <v>46316</v>
+        <v>46321</v>
       </c>
       <c r="P296">
         <v>9</v>
@@ -23493,28 +23514,31 @@
         <v>2026</v>
       </c>
       <c r="R296">
-        <v>18300938</v>
+        <v>17399291</v>
+      </c>
+      <c r="S296" t="s">
+        <v>54</v>
       </c>
       <c r="U296" t="s">
         <v>178</v>
       </c>
       <c r="V296" s="1">
-        <v>46309.68950355324</v>
+        <v>46308.4550522338</v>
       </c>
       <c r="W296">
-        <v>-6</v>
+        <v>-11</v>
       </c>
       <c r="X296" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="Y296" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="AB296">
         <v>0</v>
       </c>
       <c r="AC296" t="s">
-        <v>303</v>
+        <v>54</v>
       </c>
       <c r="AH296" t="s">
         <v>305</v>
@@ -23525,16 +23549,16 @@
     </row>
     <row r="297" spans="1:35">
       <c r="A297">
-        <v>6962</v>
+        <v>6945</v>
       </c>
       <c r="B297" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C297" t="s">
         <v>49</v>
       </c>
       <c r="D297" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E297" t="s">
         <v>54</v>
@@ -23555,7 +23579,7 @@
         <v>123</v>
       </c>
       <c r="N297" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="P297">
         <v>9</v>
@@ -23564,22 +23588,22 @@
         <v>2026</v>
       </c>
       <c r="R297">
-        <v>18300934</v>
+        <v>18300939</v>
       </c>
       <c r="U297" t="s">
         <v>178</v>
       </c>
       <c r="V297" s="1">
-        <v>46309.68881501158</v>
+        <v>46309.68971350694</v>
       </c>
       <c r="W297">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="X297" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="Y297" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="AB297">
         <v>0</v>
@@ -23591,6 +23615,222 @@
         <v>305</v>
       </c>
       <c r="AI297" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="298" spans="1:35">
+      <c r="A298">
+        <v>6949</v>
+      </c>
+      <c r="B298" t="s">
+        <v>39</v>
+      </c>
+      <c r="C298" t="s">
+        <v>49</v>
+      </c>
+      <c r="D298" t="s">
+        <v>50</v>
+      </c>
+      <c r="E298" t="s">
+        <v>54</v>
+      </c>
+      <c r="F298" t="s">
+        <v>56</v>
+      </c>
+      <c r="G298">
+        <v>11056</v>
+      </c>
+      <c r="H298">
+        <v>0</v>
+      </c>
+      <c r="I298" t="s">
+        <v>64</v>
+      </c>
+      <c r="J298" t="s">
+        <v>123</v>
+      </c>
+      <c r="N298" s="1">
+        <v>46304</v>
+      </c>
+      <c r="O298" t="s">
+        <v>136</v>
+      </c>
+      <c r="P298">
+        <v>9</v>
+      </c>
+      <c r="Q298">
+        <v>2026</v>
+      </c>
+      <c r="R298">
+        <v>18293645</v>
+      </c>
+      <c r="U298" t="s">
+        <v>179</v>
+      </c>
+      <c r="V298" s="1">
+        <v>46304.42026608796</v>
+      </c>
+      <c r="W298">
+        <v>6</v>
+      </c>
+      <c r="X298" t="s">
+        <v>183</v>
+      </c>
+      <c r="Y298" t="s">
+        <v>300</v>
+      </c>
+      <c r="AB298">
+        <v>0</v>
+      </c>
+      <c r="AC298" t="s">
+        <v>304</v>
+      </c>
+      <c r="AH298" t="s">
+        <v>305</v>
+      </c>
+      <c r="AI298" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="299" spans="1:35">
+      <c r="A299">
+        <v>6949</v>
+      </c>
+      <c r="B299" t="s">
+        <v>39</v>
+      </c>
+      <c r="C299" t="s">
+        <v>49</v>
+      </c>
+      <c r="D299" t="s">
+        <v>50</v>
+      </c>
+      <c r="E299" t="s">
+        <v>54</v>
+      </c>
+      <c r="F299" t="s">
+        <v>56</v>
+      </c>
+      <c r="G299">
+        <v>11056</v>
+      </c>
+      <c r="H299">
+        <v>0</v>
+      </c>
+      <c r="I299" t="s">
+        <v>64</v>
+      </c>
+      <c r="J299" t="s">
+        <v>123</v>
+      </c>
+      <c r="N299" s="1">
+        <v>46316</v>
+      </c>
+      <c r="P299">
+        <v>9</v>
+      </c>
+      <c r="Q299">
+        <v>2026</v>
+      </c>
+      <c r="R299">
+        <v>18300938</v>
+      </c>
+      <c r="U299" t="s">
+        <v>178</v>
+      </c>
+      <c r="V299" s="1">
+        <v>46309.68950355324</v>
+      </c>
+      <c r="W299">
+        <v>-6</v>
+      </c>
+      <c r="X299" t="s">
+        <v>183</v>
+      </c>
+      <c r="Y299" t="s">
+        <v>301</v>
+      </c>
+      <c r="AB299">
+        <v>0</v>
+      </c>
+      <c r="AC299" t="s">
+        <v>303</v>
+      </c>
+      <c r="AH299" t="s">
+        <v>305</v>
+      </c>
+      <c r="AI299" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="300" spans="1:35">
+      <c r="A300">
+        <v>6962</v>
+      </c>
+      <c r="B300" t="s">
+        <v>40</v>
+      </c>
+      <c r="C300" t="s">
+        <v>49</v>
+      </c>
+      <c r="D300" t="s">
+        <v>52</v>
+      </c>
+      <c r="E300" t="s">
+        <v>54</v>
+      </c>
+      <c r="F300" t="s">
+        <v>56</v>
+      </c>
+      <c r="G300">
+        <v>11056</v>
+      </c>
+      <c r="H300">
+        <v>0</v>
+      </c>
+      <c r="I300" t="s">
+        <v>64</v>
+      </c>
+      <c r="J300" t="s">
+        <v>123</v>
+      </c>
+      <c r="N300" s="1">
+        <v>46315</v>
+      </c>
+      <c r="P300">
+        <v>9</v>
+      </c>
+      <c r="Q300">
+        <v>2026</v>
+      </c>
+      <c r="R300">
+        <v>18300934</v>
+      </c>
+      <c r="U300" t="s">
+        <v>178</v>
+      </c>
+      <c r="V300" s="1">
+        <v>46309.68881501158</v>
+      </c>
+      <c r="W300">
+        <v>-5</v>
+      </c>
+      <c r="X300" t="s">
+        <v>184</v>
+      </c>
+      <c r="Y300" t="s">
+        <v>302</v>
+      </c>
+      <c r="AB300">
+        <v>0</v>
+      </c>
+      <c r="AC300" t="s">
+        <v>303</v>
+      </c>
+      <c r="AH300" t="s">
+        <v>305</v>
+      </c>
+      <c r="AI300" t="s">
         <v>310</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-20 11:28
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6215" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6229" uniqueCount="386">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1535,7 +1535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI435"/>
+  <dimension ref="A1:AI436"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -28256,73 +28256,70 @@
     </row>
     <row r="357" spans="1:35">
       <c r="A357">
-        <v>6703</v>
+        <v>6949</v>
       </c>
       <c r="B357" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C357" t="s">
         <v>49</v>
       </c>
       <c r="D357" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E357" t="s">
         <v>54</v>
       </c>
       <c r="F357" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G357">
-        <v>10988</v>
+        <v>1697</v>
       </c>
       <c r="H357">
-        <v>0</v>
+        <v>1650</v>
       </c>
       <c r="I357" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J357" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N357" s="1">
-        <v>46295</v>
+        <v>46315</v>
       </c>
       <c r="P357">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q357">
         <v>2026</v>
       </c>
       <c r="R357">
-        <v>18112918</v>
+        <v>18178281</v>
       </c>
       <c r="S357" t="s">
-        <v>193</v>
+        <v>172</v>
       </c>
       <c r="T357" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="U357" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="V357" s="1">
-        <v>46315.37095327547</v>
+        <v>46315.43829979167</v>
       </c>
       <c r="W357">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="X357" t="s">
-        <v>216</v>
-      </c>
-      <c r="Y357" t="s">
-        <v>348</v>
+        <v>210</v>
       </c>
       <c r="AB357">
         <v>0</v>
       </c>
       <c r="AC357" t="s">
-        <v>193</v>
+        <v>172</v>
       </c>
       <c r="AH357" t="s">
         <v>379</v>
@@ -28351,28 +28348,28 @@
         <v>55</v>
       </c>
       <c r="G358">
-        <v>1628</v>
+        <v>10988</v>
       </c>
       <c r="H358">
-        <v>1581</v>
+        <v>0</v>
       </c>
       <c r="I358" t="s">
         <v>58</v>
       </c>
       <c r="J358" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N358" s="1">
-        <v>46315</v>
+        <v>46295</v>
       </c>
       <c r="P358">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q358">
         <v>2026</v>
       </c>
       <c r="R358">
-        <v>17955177</v>
+        <v>18112918</v>
       </c>
       <c r="S358" t="s">
         <v>193</v>
@@ -28381,16 +28378,19 @@
         <v>198</v>
       </c>
       <c r="U358" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="V358" s="1">
-        <v>46314.43610068287</v>
+        <v>46315.37095327547</v>
       </c>
       <c r="W358">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="X358" t="s">
         <v>216</v>
+      </c>
+      <c r="Y358" t="s">
+        <v>348</v>
       </c>
       <c r="AB358">
         <v>0</v>
@@ -28425,16 +28425,16 @@
         <v>55</v>
       </c>
       <c r="G359">
-        <v>1607</v>
+        <v>1628</v>
       </c>
       <c r="H359">
-        <v>0</v>
+        <v>1581</v>
       </c>
       <c r="I359" t="s">
         <v>58</v>
       </c>
       <c r="J359" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N359" s="1">
         <v>46315</v>
@@ -28446,7 +28446,7 @@
         <v>2026</v>
       </c>
       <c r="R359">
-        <v>17955169</v>
+        <v>17955177</v>
       </c>
       <c r="S359" t="s">
         <v>193</v>
@@ -28458,7 +28458,7 @@
         <v>205</v>
       </c>
       <c r="V359" s="1">
-        <v>46314.70899030093</v>
+        <v>46314.43610068287</v>
       </c>
       <c r="W359">
         <v>0</v>
@@ -28481,16 +28481,16 @@
     </row>
     <row r="360" spans="1:35">
       <c r="A360">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B360" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C360" t="s">
         <v>49</v>
       </c>
       <c r="D360" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E360" t="s">
         <v>54</v>
@@ -28499,58 +28499,52 @@
         <v>55</v>
       </c>
       <c r="G360">
-        <v>5883</v>
+        <v>1607</v>
       </c>
       <c r="H360">
-        <v>5792</v>
+        <v>0</v>
       </c>
       <c r="I360" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J360" t="s">
-        <v>124</v>
+        <v>71</v>
       </c>
       <c r="N360" s="1">
         <v>46315</v>
       </c>
-      <c r="O360" t="s">
-        <v>167</v>
-      </c>
       <c r="P360">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q360">
         <v>2026</v>
       </c>
       <c r="R360">
-        <v>17399068</v>
+        <v>17955169</v>
       </c>
       <c r="S360" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="T360" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="U360" t="s">
         <v>205</v>
       </c>
       <c r="V360" s="1">
-        <v>46314.58550305555</v>
+        <v>46314.70899030093</v>
       </c>
       <c r="W360">
         <v>0</v>
       </c>
       <c r="X360" t="s">
-        <v>213</v>
-      </c>
-      <c r="Y360" t="s">
-        <v>349</v>
+        <v>216</v>
       </c>
       <c r="AB360">
         <v>0</v>
       </c>
       <c r="AC360" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="AH360" t="s">
         <v>379</v>
@@ -28561,10 +28555,10 @@
     </row>
     <row r="361" spans="1:35">
       <c r="A361">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B361" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C361" t="s">
         <v>49</v>
@@ -28593,6 +28587,9 @@
       <c r="N361" s="1">
         <v>46315</v>
       </c>
+      <c r="O361" t="s">
+        <v>167</v>
+      </c>
       <c r="P361">
         <v>10</v>
       </c>
@@ -28600,28 +28597,34 @@
         <v>2026</v>
       </c>
       <c r="R361">
-        <v>16976068</v>
+        <v>17399068</v>
       </c>
       <c r="S361" t="s">
-        <v>179</v>
+        <v>182</v>
+      </c>
+      <c r="T361" t="s">
+        <v>201</v>
       </c>
       <c r="U361" t="s">
         <v>205</v>
       </c>
       <c r="V361" s="1">
-        <v>46314.42976884259</v>
+        <v>46314.58550305555</v>
       </c>
       <c r="W361">
         <v>0</v>
       </c>
       <c r="X361" t="s">
-        <v>215</v>
+        <v>213</v>
+      </c>
+      <c r="Y361" t="s">
+        <v>349</v>
       </c>
       <c r="AB361">
         <v>0</v>
       </c>
       <c r="AC361" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="AH361" t="s">
         <v>379</v>
@@ -28632,10 +28635,10 @@
     </row>
     <row r="362" spans="1:35">
       <c r="A362">
-        <v>6627</v>
+        <v>6486</v>
       </c>
       <c r="B362" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="C362" t="s">
         <v>49</v>
@@ -28644,7 +28647,7 @@
         <v>50</v>
       </c>
       <c r="E362" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F362" t="s">
         <v>55</v>
@@ -28671,7 +28674,7 @@
         <v>2026</v>
       </c>
       <c r="R362">
-        <v>18068545</v>
+        <v>16976068</v>
       </c>
       <c r="S362" t="s">
         <v>179</v>
@@ -28680,13 +28683,13 @@
         <v>205</v>
       </c>
       <c r="V362" s="1">
-        <v>46314.40348229167</v>
+        <v>46314.42976884259</v>
       </c>
       <c r="W362">
         <v>0</v>
       </c>
       <c r="X362" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="AB362">
         <v>0</v>
@@ -28703,16 +28706,16 @@
     </row>
     <row r="363" spans="1:35">
       <c r="A363">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B363" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C363" t="s">
         <v>49</v>
       </c>
       <c r="D363" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E363" t="s">
         <v>53</v>
@@ -28742,7 +28745,7 @@
         <v>2026</v>
       </c>
       <c r="R363">
-        <v>18052464</v>
+        <v>18068545</v>
       </c>
       <c r="S363" t="s">
         <v>179</v>
@@ -28751,7 +28754,7 @@
         <v>205</v>
       </c>
       <c r="V363" s="1">
-        <v>46314.42774210648</v>
+        <v>46314.40348229167</v>
       </c>
       <c r="W363">
         <v>0</v>
@@ -28774,19 +28777,19 @@
     </row>
     <row r="364" spans="1:35">
       <c r="A364">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B364" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C364" t="s">
         <v>49</v>
       </c>
       <c r="D364" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E364" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F364" t="s">
         <v>55</v>
@@ -28806,9 +28809,6 @@
       <c r="N364" s="1">
         <v>46315</v>
       </c>
-      <c r="O364" t="s">
-        <v>167</v>
-      </c>
       <c r="P364">
         <v>10</v>
       </c>
@@ -28816,34 +28816,28 @@
         <v>2026</v>
       </c>
       <c r="R364">
-        <v>18077113</v>
+        <v>18052464</v>
       </c>
       <c r="S364" t="s">
-        <v>178</v>
-      </c>
-      <c r="T364" t="s">
-        <v>199</v>
+        <v>179</v>
       </c>
       <c r="U364" t="s">
         <v>205</v>
       </c>
       <c r="V364" s="1">
-        <v>46314.60497207176</v>
+        <v>46314.42774210648</v>
       </c>
       <c r="W364">
         <v>0</v>
       </c>
       <c r="X364" t="s">
-        <v>216</v>
-      </c>
-      <c r="Y364" t="s">
-        <v>350</v>
+        <v>207</v>
       </c>
       <c r="AB364">
         <v>0</v>
       </c>
       <c r="AC364" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AH364" t="s">
         <v>379</v>
@@ -28854,22 +28848,22 @@
     </row>
     <row r="365" spans="1:35">
       <c r="A365">
-        <v>6949</v>
+        <v>6703</v>
       </c>
       <c r="B365" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C365" t="s">
         <v>49</v>
       </c>
       <c r="D365" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E365" t="s">
         <v>54</v>
       </c>
       <c r="F365" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G365">
         <v>5883</v>
@@ -28886,6 +28880,9 @@
       <c r="N365" s="1">
         <v>46315</v>
       </c>
+      <c r="O365" t="s">
+        <v>167</v>
+      </c>
       <c r="P365">
         <v>10</v>
       </c>
@@ -28893,31 +28890,34 @@
         <v>2026</v>
       </c>
       <c r="R365">
-        <v>18190421</v>
+        <v>18077113</v>
       </c>
       <c r="S365" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="T365" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="U365" t="s">
         <v>205</v>
       </c>
       <c r="V365" s="1">
-        <v>46314.7029991088</v>
+        <v>46314.60497207176</v>
       </c>
       <c r="W365">
         <v>0</v>
       </c>
       <c r="X365" t="s">
-        <v>210</v>
+        <v>216</v>
+      </c>
+      <c r="Y365" t="s">
+        <v>350</v>
       </c>
       <c r="AB365">
         <v>0</v>
       </c>
       <c r="AC365" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="AH365" t="s">
         <v>379</v>
@@ -28928,10 +28928,10 @@
     </row>
     <row r="366" spans="1:35">
       <c r="A366">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B366" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C366" t="s">
         <v>49</v>
@@ -28943,10 +28943,10 @@
         <v>54</v>
       </c>
       <c r="F366" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G366">
-        <v>5884</v>
+        <v>5883</v>
       </c>
       <c r="H366">
         <v>5792</v>
@@ -28955,14 +28955,11 @@
         <v>59</v>
       </c>
       <c r="J366" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="N366" s="1">
         <v>46315</v>
       </c>
-      <c r="O366" t="s">
-        <v>168</v>
-      </c>
       <c r="P366">
         <v>10</v>
       </c>
@@ -28970,34 +28967,31 @@
         <v>2026</v>
       </c>
       <c r="R366">
-        <v>17399078</v>
+        <v>18190421</v>
       </c>
       <c r="S366" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="T366" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="U366" t="s">
         <v>205</v>
       </c>
       <c r="V366" s="1">
-        <v>46314.58562635416</v>
+        <v>46314.7029991088</v>
       </c>
       <c r="W366">
         <v>0</v>
       </c>
       <c r="X366" t="s">
-        <v>213</v>
-      </c>
-      <c r="Y366" t="s">
-        <v>351</v>
+        <v>210</v>
       </c>
       <c r="AB366">
         <v>0</v>
       </c>
       <c r="AC366" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AH366" t="s">
         <v>379</v>
@@ -29008,10 +29002,10 @@
     </row>
     <row r="367" spans="1:35">
       <c r="A367">
-        <v>6486</v>
+        <v>5417</v>
       </c>
       <c r="B367" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C367" t="s">
         <v>49</v>
@@ -29040,6 +29034,9 @@
       <c r="N367" s="1">
         <v>46315</v>
       </c>
+      <c r="O367" t="s">
+        <v>168</v>
+      </c>
       <c r="P367">
         <v>10</v>
       </c>
@@ -29047,28 +29044,34 @@
         <v>2026</v>
       </c>
       <c r="R367">
-        <v>16976078</v>
+        <v>17399078</v>
       </c>
       <c r="S367" t="s">
-        <v>179</v>
+        <v>182</v>
+      </c>
+      <c r="T367" t="s">
+        <v>201</v>
       </c>
       <c r="U367" t="s">
         <v>205</v>
       </c>
       <c r="V367" s="1">
-        <v>46314.42981640046</v>
+        <v>46314.58562635416</v>
       </c>
       <c r="W367">
         <v>0</v>
       </c>
       <c r="X367" t="s">
-        <v>215</v>
+        <v>213</v>
+      </c>
+      <c r="Y367" t="s">
+        <v>351</v>
       </c>
       <c r="AB367">
         <v>0</v>
       </c>
       <c r="AC367" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="AH367" t="s">
         <v>379</v>
@@ -29079,10 +29082,10 @@
     </row>
     <row r="368" spans="1:35">
       <c r="A368">
-        <v>6627</v>
+        <v>6486</v>
       </c>
       <c r="B368" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="C368" t="s">
         <v>49</v>
@@ -29091,7 +29094,7 @@
         <v>50</v>
       </c>
       <c r="E368" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F368" t="s">
         <v>55</v>
@@ -29118,7 +29121,7 @@
         <v>2026</v>
       </c>
       <c r="R368">
-        <v>18068556</v>
+        <v>16976078</v>
       </c>
       <c r="S368" t="s">
         <v>179</v>
@@ -29127,13 +29130,13 @@
         <v>205</v>
       </c>
       <c r="V368" s="1">
-        <v>46314.41026230324</v>
+        <v>46314.42981640046</v>
       </c>
       <c r="W368">
         <v>0</v>
       </c>
       <c r="X368" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="AB368">
         <v>0</v>
@@ -29150,16 +29153,16 @@
     </row>
     <row r="369" spans="1:35">
       <c r="A369">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B369" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C369" t="s">
         <v>49</v>
       </c>
       <c r="D369" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E369" t="s">
         <v>53</v>
@@ -29189,7 +29192,7 @@
         <v>2026</v>
       </c>
       <c r="R369">
-        <v>18052475</v>
+        <v>18068556</v>
       </c>
       <c r="S369" t="s">
         <v>179</v>
@@ -29198,7 +29201,7 @@
         <v>205</v>
       </c>
       <c r="V369" s="1">
-        <v>46314.42900954861</v>
+        <v>46314.41026230324</v>
       </c>
       <c r="W369">
         <v>0</v>
@@ -29221,19 +29224,19 @@
     </row>
     <row r="370" spans="1:35">
       <c r="A370">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B370" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C370" t="s">
         <v>49</v>
       </c>
       <c r="D370" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E370" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F370" t="s">
         <v>55</v>
@@ -29253,9 +29256,6 @@
       <c r="N370" s="1">
         <v>46315</v>
       </c>
-      <c r="O370" t="s">
-        <v>167</v>
-      </c>
       <c r="P370">
         <v>10</v>
       </c>
@@ -29263,34 +29263,28 @@
         <v>2026</v>
       </c>
       <c r="R370">
-        <v>18077123</v>
+        <v>18052475</v>
       </c>
       <c r="S370" t="s">
-        <v>178</v>
-      </c>
-      <c r="T370" t="s">
-        <v>199</v>
+        <v>179</v>
       </c>
       <c r="U370" t="s">
         <v>205</v>
       </c>
       <c r="V370" s="1">
-        <v>46314.60515678241</v>
+        <v>46314.42900954861</v>
       </c>
       <c r="W370">
         <v>0</v>
       </c>
       <c r="X370" t="s">
-        <v>216</v>
-      </c>
-      <c r="Y370" t="s">
-        <v>352</v>
+        <v>207</v>
       </c>
       <c r="AB370">
         <v>0</v>
       </c>
       <c r="AC370" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AH370" t="s">
         <v>379</v>
@@ -29301,22 +29295,22 @@
     </row>
     <row r="371" spans="1:35">
       <c r="A371">
-        <v>6949</v>
+        <v>6703</v>
       </c>
       <c r="B371" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C371" t="s">
         <v>49</v>
       </c>
       <c r="D371" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E371" t="s">
         <v>54</v>
       </c>
       <c r="F371" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G371">
         <v>5884</v>
@@ -29333,6 +29327,9 @@
       <c r="N371" s="1">
         <v>46315</v>
       </c>
+      <c r="O371" t="s">
+        <v>167</v>
+      </c>
       <c r="P371">
         <v>10</v>
       </c>
@@ -29340,31 +29337,34 @@
         <v>2026</v>
       </c>
       <c r="R371">
-        <v>18190427</v>
+        <v>18077123</v>
       </c>
       <c r="S371" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="T371" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="U371" t="s">
         <v>205</v>
       </c>
       <c r="V371" s="1">
-        <v>46314.70295032408</v>
+        <v>46314.60515678241</v>
       </c>
       <c r="W371">
         <v>0</v>
       </c>
       <c r="X371" t="s">
-        <v>210</v>
+        <v>216</v>
+      </c>
+      <c r="Y371" t="s">
+        <v>352</v>
       </c>
       <c r="AB371">
         <v>0</v>
       </c>
       <c r="AC371" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="AH371" t="s">
         <v>379</v>
@@ -29375,10 +29375,10 @@
     </row>
     <row r="372" spans="1:35">
       <c r="A372">
-        <v>6486</v>
+        <v>6949</v>
       </c>
       <c r="B372" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C372" t="s">
         <v>49</v>
@@ -29390,19 +29390,19 @@
         <v>54</v>
       </c>
       <c r="F372" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G372">
-        <v>5836</v>
+        <v>5884</v>
       </c>
       <c r="H372">
-        <v>5784</v>
+        <v>5792</v>
       </c>
       <c r="I372" t="s">
         <v>59</v>
       </c>
       <c r="J372" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="N372" s="1">
         <v>46315</v>
@@ -29414,28 +29414,31 @@
         <v>2026</v>
       </c>
       <c r="R372">
-        <v>16976038</v>
+        <v>18190427</v>
       </c>
       <c r="S372" t="s">
-        <v>179</v>
+        <v>181</v>
+      </c>
+      <c r="T372" t="s">
+        <v>200</v>
       </c>
       <c r="U372" t="s">
         <v>205</v>
       </c>
       <c r="V372" s="1">
-        <v>46314.57059383102</v>
+        <v>46314.70295032408</v>
       </c>
       <c r="W372">
         <v>0</v>
       </c>
       <c r="X372" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="AB372">
         <v>0</v>
       </c>
       <c r="AC372" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AH372" t="s">
         <v>379</v>
@@ -29446,10 +29449,10 @@
     </row>
     <row r="373" spans="1:35">
       <c r="A373">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B373" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C373" t="s">
         <v>49</v>
@@ -29478,9 +29481,6 @@
       <c r="N373" s="1">
         <v>46315</v>
       </c>
-      <c r="O373" t="s">
-        <v>168</v>
-      </c>
       <c r="P373">
         <v>10</v>
       </c>
@@ -29488,34 +29488,28 @@
         <v>2026</v>
       </c>
       <c r="R373">
-        <v>17222580</v>
+        <v>16976038</v>
       </c>
       <c r="S373" t="s">
-        <v>194</v>
-      </c>
-      <c r="T373" t="s">
-        <v>199</v>
+        <v>179</v>
       </c>
       <c r="U373" t="s">
         <v>205</v>
       </c>
       <c r="V373" s="1">
-        <v>46314.73644534723</v>
+        <v>46314.57059383102</v>
       </c>
       <c r="W373">
         <v>0</v>
       </c>
       <c r="X373" t="s">
-        <v>208</v>
-      </c>
-      <c r="Y373" t="s">
-        <v>353</v>
+        <v>215</v>
       </c>
       <c r="AB373">
         <v>0</v>
       </c>
       <c r="AC373" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="AH373" t="s">
         <v>379</v>
@@ -29526,10 +29520,10 @@
     </row>
     <row r="374" spans="1:35">
       <c r="A374">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B374" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C374" t="s">
         <v>49</v>
@@ -29538,7 +29532,7 @@
         <v>50</v>
       </c>
       <c r="E374" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F374" t="s">
         <v>55</v>
@@ -29558,6 +29552,9 @@
       <c r="N374" s="1">
         <v>46315</v>
       </c>
+      <c r="O374" t="s">
+        <v>168</v>
+      </c>
       <c r="P374">
         <v>10</v>
       </c>
@@ -29565,28 +29562,34 @@
         <v>2026</v>
       </c>
       <c r="R374">
-        <v>18068501</v>
+        <v>17222580</v>
       </c>
       <c r="S374" t="s">
-        <v>179</v>
+        <v>194</v>
+      </c>
+      <c r="T374" t="s">
+        <v>199</v>
       </c>
       <c r="U374" t="s">
         <v>205</v>
       </c>
       <c r="V374" s="1">
-        <v>46314.56284280093</v>
+        <v>46314.73644534723</v>
       </c>
       <c r="W374">
         <v>0</v>
       </c>
       <c r="X374" t="s">
-        <v>207</v>
+        <v>208</v>
+      </c>
+      <c r="Y374" t="s">
+        <v>353</v>
       </c>
       <c r="AB374">
         <v>0</v>
       </c>
       <c r="AC374" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="AH374" t="s">
         <v>379</v>
@@ -29597,16 +29600,16 @@
     </row>
     <row r="375" spans="1:35">
       <c r="A375">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B375" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C375" t="s">
         <v>49</v>
       </c>
       <c r="D375" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E375" t="s">
         <v>53</v>
@@ -29636,7 +29639,7 @@
         <v>2026</v>
       </c>
       <c r="R375">
-        <v>18052420</v>
+        <v>18068501</v>
       </c>
       <c r="S375" t="s">
         <v>179</v>
@@ -29645,7 +29648,7 @@
         <v>205</v>
       </c>
       <c r="V375" s="1">
-        <v>46314.56304628473</v>
+        <v>46314.56284280093</v>
       </c>
       <c r="W375">
         <v>0</v>
@@ -29668,41 +29671,38 @@
     </row>
     <row r="376" spans="1:35">
       <c r="A376">
-        <v>6404</v>
+        <v>6628</v>
       </c>
       <c r="B376" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C376" t="s">
         <v>49</v>
       </c>
       <c r="D376" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E376" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F376" t="s">
         <v>55</v>
       </c>
       <c r="G376">
-        <v>5903</v>
+        <v>5836</v>
       </c>
       <c r="H376">
-        <v>5830</v>
+        <v>5784</v>
       </c>
       <c r="I376" t="s">
         <v>59</v>
       </c>
       <c r="J376" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N376" s="1">
         <v>46315</v>
       </c>
-      <c r="O376" t="s">
-        <v>167</v>
-      </c>
       <c r="P376">
         <v>10</v>
       </c>
@@ -29710,34 +29710,28 @@
         <v>2026</v>
       </c>
       <c r="R376">
-        <v>16962222</v>
+        <v>18052420</v>
       </c>
       <c r="S376" t="s">
-        <v>183</v>
-      </c>
-      <c r="T376" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="U376" t="s">
         <v>205</v>
       </c>
       <c r="V376" s="1">
-        <v>46314.39188924769</v>
+        <v>46314.56304628473</v>
       </c>
       <c r="W376">
         <v>0</v>
       </c>
       <c r="X376" t="s">
-        <v>212</v>
-      </c>
-      <c r="Y376" t="s">
-        <v>354</v>
+        <v>207</v>
       </c>
       <c r="AB376">
         <v>0</v>
       </c>
       <c r="AC376" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="AH376" t="s">
         <v>379</v>
@@ -29766,20 +29760,23 @@
         <v>55</v>
       </c>
       <c r="G377">
+        <v>5903</v>
+      </c>
+      <c r="H377">
         <v>5830</v>
-      </c>
-      <c r="H377">
-        <v>5784</v>
       </c>
       <c r="I377" t="s">
         <v>59</v>
       </c>
       <c r="J377" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="N377" s="1">
         <v>46315</v>
       </c>
+      <c r="O377" t="s">
+        <v>167</v>
+      </c>
       <c r="P377">
         <v>10</v>
       </c>
@@ -29787,7 +29784,7 @@
         <v>2026</v>
       </c>
       <c r="R377">
-        <v>16962212</v>
+        <v>16962222</v>
       </c>
       <c r="S377" t="s">
         <v>183</v>
@@ -29799,7 +29796,7 @@
         <v>205</v>
       </c>
       <c r="V377" s="1">
-        <v>46314.44518351852</v>
+        <v>46314.39188924769</v>
       </c>
       <c r="W377">
         <v>0</v>
@@ -29807,6 +29804,9 @@
       <c r="X377" t="s">
         <v>212</v>
       </c>
+      <c r="Y377" t="s">
+        <v>354</v>
+      </c>
       <c r="AB377">
         <v>0</v>
       </c>
@@ -29822,16 +29822,16 @@
     </row>
     <row r="378" spans="1:35">
       <c r="A378">
-        <v>6548</v>
+        <v>6404</v>
       </c>
       <c r="B378" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C378" t="s">
         <v>49</v>
       </c>
       <c r="D378" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E378" t="s">
         <v>54</v>
@@ -29840,7 +29840,7 @@
         <v>55</v>
       </c>
       <c r="G378">
-        <v>5839</v>
+        <v>5830</v>
       </c>
       <c r="H378">
         <v>5784</v>
@@ -29849,10 +29849,10 @@
         <v>59</v>
       </c>
       <c r="J378" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N378" s="1">
-        <v>46329</v>
+        <v>46315</v>
       </c>
       <c r="P378">
         <v>10</v>
@@ -29861,31 +29861,31 @@
         <v>2026</v>
       </c>
       <c r="R378">
-        <v>18158845</v>
+        <v>16962212</v>
       </c>
       <c r="S378" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="T378" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="U378" t="s">
         <v>205</v>
       </c>
       <c r="V378" s="1">
-        <v>46314.73711247685</v>
+        <v>46314.44518351852</v>
       </c>
       <c r="W378">
-        <v>-14</v>
+        <v>0</v>
       </c>
       <c r="X378" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="AB378">
         <v>0</v>
       </c>
       <c r="AC378" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="AH378" t="s">
         <v>379</v>
@@ -29896,10 +29896,10 @@
     </row>
     <row r="379" spans="1:35">
       <c r="A379">
-        <v>5417</v>
+        <v>6548</v>
       </c>
       <c r="B379" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C379" t="s">
         <v>49</v>
@@ -29914,22 +29914,19 @@
         <v>55</v>
       </c>
       <c r="G379">
-        <v>6348</v>
+        <v>5839</v>
       </c>
       <c r="H379">
-        <v>0</v>
+        <v>5784</v>
       </c>
       <c r="I379" t="s">
         <v>59</v>
       </c>
       <c r="J379" t="s">
-        <v>87</v>
+        <v>145</v>
       </c>
       <c r="N379" s="1">
-        <v>46317</v>
-      </c>
-      <c r="O379" t="s">
-        <v>169</v>
+        <v>46329</v>
       </c>
       <c r="P379">
         <v>10</v>
@@ -29938,31 +29935,34 @@
         <v>2026</v>
       </c>
       <c r="R379">
-        <v>18301415</v>
+        <v>18158845</v>
+      </c>
+      <c r="S379" t="s">
+        <v>194</v>
+      </c>
+      <c r="T379" t="s">
+        <v>199</v>
       </c>
       <c r="U379" t="s">
         <v>205</v>
       </c>
       <c r="V379" s="1">
-        <v>46314.56177552084</v>
+        <v>46314.73711247685</v>
       </c>
       <c r="W379">
-        <v>-2</v>
+        <v>-14</v>
       </c>
       <c r="X379" t="s">
-        <v>213</v>
-      </c>
-      <c r="Y379" t="s">
-        <v>355</v>
+        <v>208</v>
       </c>
       <c r="AB379">
         <v>0</v>
       </c>
       <c r="AC379" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="AH379" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AI379" t="s">
         <v>385</v>
@@ -29970,10 +29970,10 @@
     </row>
     <row r="380" spans="1:35">
       <c r="A380">
-        <v>6548</v>
+        <v>5417</v>
       </c>
       <c r="B380" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C380" t="s">
         <v>49</v>
@@ -29988,55 +29988,55 @@
         <v>55</v>
       </c>
       <c r="G380">
-        <v>1913</v>
+        <v>6348</v>
       </c>
       <c r="H380">
-        <v>1862</v>
+        <v>0</v>
       </c>
       <c r="I380" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J380" t="s">
-        <v>146</v>
+        <v>87</v>
       </c>
       <c r="N380" s="1">
-        <v>46316</v>
+        <v>46317</v>
+      </c>
+      <c r="O380" t="s">
+        <v>169</v>
       </c>
       <c r="P380">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q380">
         <v>2026</v>
       </c>
       <c r="R380">
-        <v>17988580</v>
-      </c>
-      <c r="S380" t="s">
-        <v>186</v>
-      </c>
-      <c r="T380" t="s">
-        <v>202</v>
+        <v>18301415</v>
       </c>
       <c r="U380" t="s">
         <v>205</v>
       </c>
       <c r="V380" s="1">
-        <v>46314.51585246528</v>
+        <v>46314.56177552084</v>
       </c>
       <c r="W380">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="X380" t="s">
-        <v>208</v>
+        <v>213</v>
+      </c>
+      <c r="Y380" t="s">
+        <v>355</v>
       </c>
       <c r="AB380">
         <v>0</v>
       </c>
       <c r="AC380" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="AH380" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AI380" t="s">
         <v>385</v>
@@ -30062,19 +30062,19 @@
         <v>55</v>
       </c>
       <c r="G381">
-        <v>1876</v>
+        <v>1913</v>
       </c>
       <c r="H381">
-        <v>0</v>
+        <v>1862</v>
       </c>
       <c r="I381" t="s">
         <v>60</v>
       </c>
       <c r="J381" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="N381" s="1">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="P381">
         <v>9</v>
@@ -30083,7 +30083,7 @@
         <v>2026</v>
       </c>
       <c r="R381">
-        <v>17988556</v>
+        <v>17988580</v>
       </c>
       <c r="S381" t="s">
         <v>186</v>
@@ -30092,20 +30092,17 @@
         <v>202</v>
       </c>
       <c r="U381" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="V381" s="1">
-        <v>46314.7779269676</v>
+        <v>46314.51585246528</v>
       </c>
       <c r="W381">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="X381" t="s">
         <v>208</v>
       </c>
-      <c r="Y381" t="s">
-        <v>356</v>
-      </c>
       <c r="AB381">
         <v>0</v>
       </c>
@@ -30113,7 +30110,7 @@
         <v>186</v>
       </c>
       <c r="AH381" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AI381" t="s">
         <v>385</v>
@@ -30121,10 +30118,10 @@
     </row>
     <row r="382" spans="1:35">
       <c r="A382">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B382" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C382" t="s">
         <v>49</v>
@@ -30133,13 +30130,13 @@
         <v>50</v>
       </c>
       <c r="E382" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F382" t="s">
         <v>55</v>
       </c>
       <c r="G382">
-        <v>11411</v>
+        <v>1876</v>
       </c>
       <c r="H382">
         <v>0</v>
@@ -30148,14 +30145,11 @@
         <v>60</v>
       </c>
       <c r="J382" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="N382" s="1">
         <v>46311</v>
       </c>
-      <c r="O382" t="s">
-        <v>168</v>
-      </c>
       <c r="P382">
         <v>9</v>
       </c>
@@ -30163,10 +30157,10 @@
         <v>2026</v>
       </c>
       <c r="R382">
-        <v>18048484</v>
+        <v>17988556</v>
       </c>
       <c r="S382" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="T382" t="s">
         <v>202</v>
@@ -30175,22 +30169,22 @@
         <v>204</v>
       </c>
       <c r="V382" s="1">
-        <v>46314.41760023148</v>
+        <v>46314.7779269676</v>
       </c>
       <c r="W382">
         <v>4</v>
       </c>
       <c r="X382" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Y382" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="AB382">
         <v>0</v>
       </c>
       <c r="AC382" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AH382" t="s">
         <v>380</v>
@@ -30201,16 +30195,16 @@
     </row>
     <row r="383" spans="1:35">
       <c r="A383">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B383" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C383" t="s">
         <v>49</v>
       </c>
       <c r="D383" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E383" t="s">
         <v>53</v>
@@ -30219,7 +30213,7 @@
         <v>55</v>
       </c>
       <c r="G383">
-        <v>1879</v>
+        <v>11411</v>
       </c>
       <c r="H383">
         <v>0</v>
@@ -30228,13 +30222,13 @@
         <v>60</v>
       </c>
       <c r="J383" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="N383" s="1">
         <v>46311</v>
       </c>
       <c r="O383" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="P383">
         <v>9</v>
@@ -30243,10 +30237,10 @@
         <v>2026</v>
       </c>
       <c r="R383">
-        <v>17988685</v>
+        <v>18048484</v>
       </c>
       <c r="S383" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="T383" t="s">
         <v>202</v>
@@ -30255,7 +30249,7 @@
         <v>204</v>
       </c>
       <c r="V383" s="1">
-        <v>46314.38417774306</v>
+        <v>46314.41760023148</v>
       </c>
       <c r="W383">
         <v>4</v>
@@ -30264,13 +30258,13 @@
         <v>207</v>
       </c>
       <c r="Y383" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="AB383">
         <v>0</v>
       </c>
       <c r="AC383" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AH383" t="s">
         <v>380</v>
@@ -30281,22 +30275,22 @@
     </row>
     <row r="384" spans="1:35">
       <c r="A384">
-        <v>6945</v>
+        <v>6628</v>
       </c>
       <c r="B384" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C384" t="s">
         <v>49</v>
       </c>
       <c r="D384" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E384" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F384" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G384">
         <v>1879</v>
@@ -30314,7 +30308,7 @@
         <v>46311</v>
       </c>
       <c r="O384" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="P384">
         <v>9</v>
@@ -30323,10 +30317,10 @@
         <v>2026</v>
       </c>
       <c r="R384">
-        <v>18220195</v>
+        <v>17988685</v>
       </c>
       <c r="S384" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="T384" t="s">
         <v>202</v>
@@ -30335,22 +30329,22 @@
         <v>204</v>
       </c>
       <c r="V384" s="1">
-        <v>46314.4276216088</v>
+        <v>46314.38417774306</v>
       </c>
       <c r="W384">
         <v>4</v>
       </c>
       <c r="X384" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="Y384" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="AB384">
         <v>0</v>
       </c>
       <c r="AC384" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AH384" t="s">
         <v>380</v>
@@ -30361,10 +30355,10 @@
     </row>
     <row r="385" spans="1:35">
       <c r="A385">
-        <v>6548</v>
+        <v>6945</v>
       </c>
       <c r="B385" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C385" t="s">
         <v>49</v>
@@ -30376,22 +30370,25 @@
         <v>54</v>
       </c>
       <c r="F385" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G385">
-        <v>1914</v>
+        <v>1879</v>
       </c>
       <c r="H385">
-        <v>1862</v>
+        <v>0</v>
       </c>
       <c r="I385" t="s">
         <v>60</v>
       </c>
       <c r="J385" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="N385" s="1">
-        <v>46316</v>
+        <v>46311</v>
+      </c>
+      <c r="O385" t="s">
+        <v>168</v>
       </c>
       <c r="P385">
         <v>9</v>
@@ -30400,34 +30397,37 @@
         <v>2026</v>
       </c>
       <c r="R385">
-        <v>17988592</v>
+        <v>18220195</v>
       </c>
       <c r="S385" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="T385" t="s">
         <v>202</v>
       </c>
       <c r="U385" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="V385" s="1">
-        <v>46314.51604481482</v>
+        <v>46314.4276216088</v>
       </c>
       <c r="W385">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="X385" t="s">
-        <v>208</v>
+        <v>209</v>
+      </c>
+      <c r="Y385" t="s">
+        <v>359</v>
       </c>
       <c r="AB385">
         <v>0</v>
       </c>
       <c r="AC385" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AH385" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AI385" t="s">
         <v>385</v>
@@ -30435,10 +30435,10 @@
     </row>
     <row r="386" spans="1:35">
       <c r="A386">
-        <v>6486</v>
+        <v>6548</v>
       </c>
       <c r="B386" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C386" t="s">
         <v>49</v>
@@ -30453,22 +30453,19 @@
         <v>55</v>
       </c>
       <c r="G386">
-        <v>1837</v>
+        <v>1914</v>
       </c>
       <c r="H386">
-        <v>1788</v>
+        <v>1862</v>
       </c>
       <c r="I386" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J386" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="N386" s="1">
-        <v>46310</v>
-      </c>
-      <c r="O386" t="s">
-        <v>168</v>
+        <v>46316</v>
       </c>
       <c r="P386">
         <v>9</v>
@@ -30477,48 +30474,45 @@
         <v>2026</v>
       </c>
       <c r="R386">
-        <v>16975984</v>
+        <v>17988592</v>
       </c>
       <c r="S386" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="T386" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="U386" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="V386" s="1">
-        <v>46313.46956228009</v>
+        <v>46314.51604481482</v>
       </c>
       <c r="W386">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="X386" t="s">
-        <v>215</v>
-      </c>
-      <c r="Y386" t="s">
-        <v>360</v>
+        <v>208</v>
       </c>
       <c r="AB386">
         <v>0</v>
       </c>
       <c r="AC386" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="AH386" t="s">
         <v>379</v>
       </c>
       <c r="AI386" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="387" spans="1:35">
       <c r="A387">
-        <v>6704</v>
+        <v>6486</v>
       </c>
       <c r="B387" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C387" t="s">
         <v>49</v>
@@ -30533,22 +30527,22 @@
         <v>55</v>
       </c>
       <c r="G387">
-        <v>11874</v>
+        <v>1837</v>
       </c>
       <c r="H387">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I387" t="s">
         <v>61</v>
       </c>
       <c r="J387" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="N387" s="1">
-        <v>46314</v>
+        <v>46310</v>
       </c>
       <c r="O387" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="P387">
         <v>9</v>
@@ -30557,7 +30551,7 @@
         <v>2026</v>
       </c>
       <c r="R387">
-        <v>18273590</v>
+        <v>16975984</v>
       </c>
       <c r="S387" t="s">
         <v>190</v>
@@ -30566,19 +30560,19 @@
         <v>203</v>
       </c>
       <c r="U387" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="V387" s="1">
-        <v>46314.38488630787</v>
+        <v>46313.46956228009</v>
       </c>
       <c r="W387">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="X387" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Y387" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="AB387">
         <v>0</v>
@@ -30587,24 +30581,24 @@
         <v>190</v>
       </c>
       <c r="AH387" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AI387" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="388" spans="1:35">
       <c r="A388">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B388" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C388" t="s">
         <v>49</v>
       </c>
       <c r="D388" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E388" t="s">
         <v>54</v>
@@ -30613,7 +30607,7 @@
         <v>55</v>
       </c>
       <c r="G388">
-        <v>1802</v>
+        <v>11874</v>
       </c>
       <c r="H388">
         <v>0</v>
@@ -30622,13 +30616,13 @@
         <v>61</v>
       </c>
       <c r="J388" t="s">
-        <v>147</v>
+        <v>126</v>
       </c>
       <c r="N388" s="1">
         <v>46314</v>
       </c>
       <c r="O388" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="P388">
         <v>9</v>
@@ -30637,7 +30631,7 @@
         <v>2026</v>
       </c>
       <c r="R388">
-        <v>17948797</v>
+        <v>18273590</v>
       </c>
       <c r="S388" t="s">
         <v>190</v>
@@ -30649,16 +30643,16 @@
         <v>206</v>
       </c>
       <c r="V388" s="1">
-        <v>46314.78502430556</v>
+        <v>46314.38488630787</v>
       </c>
       <c r="W388">
         <v>1</v>
       </c>
       <c r="X388" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="Y388" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="AB388">
         <v>0</v>
@@ -30675,16 +30669,16 @@
     </row>
     <row r="389" spans="1:35">
       <c r="A389">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B389" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C389" t="s">
         <v>49</v>
       </c>
       <c r="D389" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E389" t="s">
         <v>54</v>
@@ -30693,7 +30687,7 @@
         <v>55</v>
       </c>
       <c r="G389">
-        <v>11286</v>
+        <v>1802</v>
       </c>
       <c r="H389">
         <v>0</v>
@@ -30702,7 +30696,7 @@
         <v>61</v>
       </c>
       <c r="J389" t="s">
-        <v>129</v>
+        <v>147</v>
       </c>
       <c r="N389" s="1">
         <v>46314</v>
@@ -30717,7 +30711,7 @@
         <v>2026</v>
       </c>
       <c r="R389">
-        <v>17399435</v>
+        <v>17948797</v>
       </c>
       <c r="S389" t="s">
         <v>190</v>
@@ -30729,16 +30723,16 @@
         <v>206</v>
       </c>
       <c r="V389" s="1">
-        <v>46314.38564537037</v>
+        <v>46314.78502430556</v>
       </c>
       <c r="W389">
         <v>1</v>
       </c>
       <c r="X389" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="Y389" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AB389">
         <v>0</v>
@@ -30755,16 +30749,16 @@
     </row>
     <row r="390" spans="1:35">
       <c r="A390">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B390" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C390" t="s">
         <v>49</v>
       </c>
       <c r="D390" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E390" t="s">
         <v>54</v>
@@ -30797,7 +30791,7 @@
         <v>2026</v>
       </c>
       <c r="R390">
-        <v>16962465</v>
+        <v>17399435</v>
       </c>
       <c r="S390" t="s">
         <v>190</v>
@@ -30809,16 +30803,16 @@
         <v>206</v>
       </c>
       <c r="V390" s="1">
-        <v>46314.38565289352</v>
+        <v>46314.38564537037</v>
       </c>
       <c r="W390">
         <v>1</v>
       </c>
       <c r="X390" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="Y390" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AB390">
         <v>0</v>
@@ -30835,16 +30829,16 @@
     </row>
     <row r="391" spans="1:35">
       <c r="A391">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B391" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C391" t="s">
         <v>49</v>
       </c>
       <c r="D391" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E391" t="s">
         <v>54</v>
@@ -30867,6 +30861,9 @@
       <c r="N391" s="1">
         <v>46314</v>
       </c>
+      <c r="O391" t="s">
+        <v>168</v>
+      </c>
       <c r="P391">
         <v>9</v>
       </c>
@@ -30874,7 +30871,7 @@
         <v>2026</v>
       </c>
       <c r="R391">
-        <v>18155337</v>
+        <v>16962465</v>
       </c>
       <c r="S391" t="s">
         <v>190</v>
@@ -30886,16 +30883,16 @@
         <v>206</v>
       </c>
       <c r="V391" s="1">
-        <v>46314.37977384259</v>
+        <v>46314.38565289352</v>
       </c>
       <c r="W391">
         <v>1</v>
       </c>
       <c r="X391" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="Y391" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AB391">
         <v>0</v>
@@ -30912,37 +30909,37 @@
     </row>
     <row r="392" spans="1:35">
       <c r="A392">
-        <v>6628</v>
+        <v>6486</v>
       </c>
       <c r="B392" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C392" t="s">
         <v>49</v>
       </c>
       <c r="D392" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E392" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F392" t="s">
         <v>55</v>
       </c>
       <c r="G392">
-        <v>945</v>
+        <v>11286</v>
       </c>
       <c r="H392">
         <v>0</v>
       </c>
       <c r="I392" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J392" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="N392" s="1">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="P392">
         <v>9</v>
@@ -30951,31 +30948,34 @@
         <v>2026</v>
       </c>
       <c r="R392">
-        <v>16959939</v>
+        <v>18155337</v>
       </c>
       <c r="S392" t="s">
-        <v>191</v>
+        <v>190</v>
+      </c>
+      <c r="T392" t="s">
+        <v>203</v>
       </c>
       <c r="U392" t="s">
         <v>206</v>
       </c>
       <c r="V392" s="1">
-        <v>46315.43458024305</v>
+        <v>46314.37977384259</v>
       </c>
       <c r="W392">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X392" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="Y392" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AB392">
         <v>0</v>
       </c>
       <c r="AC392" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AH392" t="s">
         <v>380</v>
@@ -30986,10 +30986,10 @@
     </row>
     <row r="393" spans="1:35">
       <c r="A393">
-        <v>6705</v>
+        <v>6628</v>
       </c>
       <c r="B393" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C393" t="s">
         <v>49</v>
@@ -30998,7 +30998,7 @@
         <v>51</v>
       </c>
       <c r="E393" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F393" t="s">
         <v>55</v>
@@ -31025,7 +31025,7 @@
         <v>2026</v>
       </c>
       <c r="R393">
-        <v>17952525</v>
+        <v>16959939</v>
       </c>
       <c r="S393" t="s">
         <v>191</v>
@@ -31034,16 +31034,16 @@
         <v>206</v>
       </c>
       <c r="V393" s="1">
-        <v>46315.4345809375</v>
+        <v>46315.43458024305</v>
       </c>
       <c r="W393">
         <v>0</v>
       </c>
       <c r="X393" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="Y393" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AB393">
         <v>0</v>
@@ -31060,10 +31060,10 @@
     </row>
     <row r="394" spans="1:35">
       <c r="A394">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B394" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C394" t="s">
         <v>49</v>
@@ -31099,7 +31099,7 @@
         <v>2026</v>
       </c>
       <c r="R394">
-        <v>18056696</v>
+        <v>17952525</v>
       </c>
       <c r="S394" t="s">
         <v>191</v>
@@ -31108,7 +31108,7 @@
         <v>206</v>
       </c>
       <c r="V394" s="1">
-        <v>46315.43458121528</v>
+        <v>46315.4345809375</v>
       </c>
       <c r="W394">
         <v>0</v>
@@ -31117,7 +31117,7 @@
         <v>214</v>
       </c>
       <c r="Y394" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AB394">
         <v>0</v>
@@ -31134,22 +31134,22 @@
     </row>
     <row r="395" spans="1:35">
       <c r="A395">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B395" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C395" t="s">
         <v>49</v>
       </c>
       <c r="D395" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E395" t="s">
         <v>54</v>
       </c>
       <c r="F395" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G395">
         <v>945</v>
@@ -31173,7 +31173,7 @@
         <v>2026</v>
       </c>
       <c r="R395">
-        <v>18164488</v>
+        <v>18056696</v>
       </c>
       <c r="S395" t="s">
         <v>191</v>
@@ -31182,16 +31182,16 @@
         <v>206</v>
       </c>
       <c r="V395" s="1">
-        <v>46315.43458645833</v>
+        <v>46315.43458121528</v>
       </c>
       <c r="W395">
         <v>0</v>
       </c>
       <c r="X395" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="Y395" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="AB395">
         <v>0</v>
@@ -31208,10 +31208,10 @@
     </row>
     <row r="396" spans="1:35">
       <c r="A396">
-        <v>6627</v>
+        <v>6945</v>
       </c>
       <c r="B396" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C396" t="s">
         <v>49</v>
@@ -31220,13 +31220,13 @@
         <v>50</v>
       </c>
       <c r="E396" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F396" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G396">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H396">
         <v>0</v>
@@ -31235,7 +31235,7 @@
         <v>62</v>
       </c>
       <c r="J396" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="N396" s="1">
         <v>46315</v>
@@ -31247,7 +31247,7 @@
         <v>2026</v>
       </c>
       <c r="R396">
-        <v>17042280</v>
+        <v>18164488</v>
       </c>
       <c r="S396" t="s">
         <v>191</v>
@@ -31256,13 +31256,16 @@
         <v>206</v>
       </c>
       <c r="V396" s="1">
-        <v>46315.43472936343</v>
+        <v>46315.43458645833</v>
       </c>
       <c r="W396">
         <v>0</v>
       </c>
       <c r="X396" t="s">
-        <v>207</v>
+        <v>209</v>
+      </c>
+      <c r="Y396" t="s">
+        <v>369</v>
       </c>
       <c r="AB396">
         <v>0</v>
@@ -31279,19 +31282,19 @@
     </row>
     <row r="397" spans="1:35">
       <c r="A397">
-        <v>6703</v>
+        <v>6627</v>
       </c>
       <c r="B397" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="C397" t="s">
         <v>49</v>
       </c>
       <c r="D397" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E397" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F397" t="s">
         <v>55</v>
@@ -31318,7 +31321,7 @@
         <v>2026</v>
       </c>
       <c r="R397">
-        <v>17941133</v>
+        <v>17042280</v>
       </c>
       <c r="S397" t="s">
         <v>191</v>
@@ -31327,16 +31330,13 @@
         <v>206</v>
       </c>
       <c r="V397" s="1">
-        <v>46315.43473040509</v>
+        <v>46315.43472936343</v>
       </c>
       <c r="W397">
         <v>0</v>
       </c>
       <c r="X397" t="s">
-        <v>216</v>
-      </c>
-      <c r="Y397" t="s">
-        <v>370</v>
+        <v>207</v>
       </c>
       <c r="AB397">
         <v>0</v>
@@ -31353,16 +31353,16 @@
     </row>
     <row r="398" spans="1:35">
       <c r="A398">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B398" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C398" t="s">
         <v>49</v>
       </c>
       <c r="D398" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E398" t="s">
         <v>54</v>
@@ -31371,7 +31371,7 @@
         <v>55</v>
       </c>
       <c r="G398">
-        <v>7022</v>
+        <v>946</v>
       </c>
       <c r="H398">
         <v>0</v>
@@ -31380,7 +31380,7 @@
         <v>62</v>
       </c>
       <c r="J398" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="N398" s="1">
         <v>46315</v>
@@ -31392,7 +31392,7 @@
         <v>2026</v>
       </c>
       <c r="R398">
-        <v>17399271</v>
+        <v>17941133</v>
       </c>
       <c r="S398" t="s">
         <v>191</v>
@@ -31401,13 +31401,16 @@
         <v>206</v>
       </c>
       <c r="V398" s="1">
-        <v>46315.43446484954</v>
+        <v>46315.43473040509</v>
       </c>
       <c r="W398">
         <v>0</v>
       </c>
       <c r="X398" t="s">
-        <v>213</v>
+        <v>216</v>
+      </c>
+      <c r="Y398" t="s">
+        <v>370</v>
       </c>
       <c r="AB398">
         <v>0</v>
@@ -31424,10 +31427,10 @@
     </row>
     <row r="399" spans="1:35">
       <c r="A399">
-        <v>6627</v>
+        <v>5417</v>
       </c>
       <c r="B399" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C399" t="s">
         <v>49</v>
@@ -31436,7 +31439,7 @@
         <v>50</v>
       </c>
       <c r="E399" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F399" t="s">
         <v>55</v>
@@ -31463,7 +31466,7 @@
         <v>2026</v>
       </c>
       <c r="R399">
-        <v>17042506</v>
+        <v>17399271</v>
       </c>
       <c r="S399" t="s">
         <v>191</v>
@@ -31472,13 +31475,13 @@
         <v>206</v>
       </c>
       <c r="V399" s="1">
-        <v>46315.43447334491</v>
+        <v>46315.43446484954</v>
       </c>
       <c r="W399">
         <v>0</v>
       </c>
       <c r="X399" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="AB399">
         <v>0</v>
@@ -31495,10 +31498,10 @@
     </row>
     <row r="400" spans="1:35">
       <c r="A400">
-        <v>6704</v>
+        <v>6627</v>
       </c>
       <c r="B400" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C400" t="s">
         <v>49</v>
@@ -31507,7 +31510,7 @@
         <v>50</v>
       </c>
       <c r="E400" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F400" t="s">
         <v>55</v>
@@ -31534,7 +31537,7 @@
         <v>2026</v>
       </c>
       <c r="R400">
-        <v>17952422</v>
+        <v>17042506</v>
       </c>
       <c r="S400" t="s">
         <v>191</v>
@@ -31543,13 +31546,13 @@
         <v>206</v>
       </c>
       <c r="V400" s="1">
-        <v>46315.43447511574</v>
+        <v>46315.43447334491</v>
       </c>
       <c r="W400">
         <v>0</v>
       </c>
       <c r="X400" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="AB400">
         <v>0</v>
@@ -31566,10 +31569,10 @@
     </row>
     <row r="401" spans="1:35">
       <c r="A401">
-        <v>6949</v>
+        <v>6704</v>
       </c>
       <c r="B401" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C401" t="s">
         <v>49</v>
@@ -31581,7 +31584,7 @@
         <v>54</v>
       </c>
       <c r="F401" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G401">
         <v>7022</v>
@@ -31605,7 +31608,7 @@
         <v>2026</v>
       </c>
       <c r="R401">
-        <v>18178175</v>
+        <v>17952422</v>
       </c>
       <c r="S401" t="s">
         <v>191</v>
@@ -31614,13 +31617,13 @@
         <v>206</v>
       </c>
       <c r="V401" s="1">
-        <v>46315.4344778588</v>
+        <v>46315.43447511574</v>
       </c>
       <c r="W401">
         <v>0</v>
       </c>
       <c r="X401" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="AB401">
         <v>0</v>
@@ -31637,10 +31640,10 @@
     </row>
     <row r="402" spans="1:35">
       <c r="A402">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B402" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C402" t="s">
         <v>49</v>
@@ -31652,10 +31655,10 @@
         <v>54</v>
       </c>
       <c r="F402" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G402">
-        <v>9086</v>
+        <v>7022</v>
       </c>
       <c r="H402">
         <v>0</v>
@@ -31664,19 +31667,19 @@
         <v>62</v>
       </c>
       <c r="J402" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="N402" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="P402">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q402">
         <v>2026</v>
       </c>
       <c r="R402">
-        <v>17399364</v>
+        <v>18178175</v>
       </c>
       <c r="S402" t="s">
         <v>191</v>
@@ -31685,13 +31688,13 @@
         <v>206</v>
       </c>
       <c r="V402" s="1">
-        <v>46314.51296478009</v>
+        <v>46315.4344778588</v>
       </c>
       <c r="W402">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X402" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="AB402">
         <v>0</v>
@@ -31700,7 +31703,7 @@
         <v>191</v>
       </c>
       <c r="AH402" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AI402" t="s">
         <v>385</v>
@@ -31708,16 +31711,16 @@
     </row>
     <row r="403" spans="1:35">
       <c r="A403">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B403" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C403" t="s">
         <v>49</v>
       </c>
       <c r="D403" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E403" t="s">
         <v>54</v>
@@ -31747,7 +31750,7 @@
         <v>2026</v>
       </c>
       <c r="R403">
-        <v>16962381</v>
+        <v>17399364</v>
       </c>
       <c r="S403" t="s">
         <v>191</v>
@@ -31756,13 +31759,13 @@
         <v>206</v>
       </c>
       <c r="V403" s="1">
-        <v>46314.5130255787</v>
+        <v>46314.51296478009</v>
       </c>
       <c r="W403">
         <v>1</v>
       </c>
       <c r="X403" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AB403">
         <v>0</v>
@@ -31779,16 +31782,16 @@
     </row>
     <row r="404" spans="1:35">
       <c r="A404">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B404" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C404" t="s">
         <v>49</v>
       </c>
       <c r="D404" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E404" t="s">
         <v>54</v>
@@ -31818,7 +31821,7 @@
         <v>2026</v>
       </c>
       <c r="R404">
-        <v>16976271</v>
+        <v>16962381</v>
       </c>
       <c r="S404" t="s">
         <v>191</v>
@@ -31827,13 +31830,13 @@
         <v>206</v>
       </c>
       <c r="V404" s="1">
-        <v>46314.51303561343</v>
+        <v>46314.5130255787</v>
       </c>
       <c r="W404">
         <v>1</v>
       </c>
       <c r="X404" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="AB404">
         <v>0</v>
@@ -31850,10 +31853,10 @@
     </row>
     <row r="405" spans="1:35">
       <c r="A405">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B405" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C405" t="s">
         <v>49</v>
@@ -31889,7 +31892,7 @@
         <v>2026</v>
       </c>
       <c r="R405">
-        <v>17222866</v>
+        <v>16976271</v>
       </c>
       <c r="S405" t="s">
         <v>191</v>
@@ -31898,13 +31901,13 @@
         <v>206</v>
       </c>
       <c r="V405" s="1">
-        <v>46314.51303834491</v>
+        <v>46314.51303561343</v>
       </c>
       <c r="W405">
         <v>1</v>
       </c>
       <c r="X405" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="AB405">
         <v>0</v>
@@ -31921,10 +31924,10 @@
     </row>
     <row r="406" spans="1:35">
       <c r="A406">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B406" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C406" t="s">
         <v>49</v>
@@ -31933,7 +31936,7 @@
         <v>50</v>
       </c>
       <c r="E406" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F406" t="s">
         <v>55</v>
@@ -31960,7 +31963,7 @@
         <v>2026</v>
       </c>
       <c r="R406">
-        <v>17042588</v>
+        <v>17222866</v>
       </c>
       <c r="S406" t="s">
         <v>191</v>
@@ -31969,13 +31972,13 @@
         <v>206</v>
       </c>
       <c r="V406" s="1">
-        <v>46314.51304019676</v>
+        <v>46314.51303834491</v>
       </c>
       <c r="W406">
         <v>1</v>
       </c>
       <c r="X406" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AB406">
         <v>0</v>
@@ -31992,16 +31995,16 @@
     </row>
     <row r="407" spans="1:35">
       <c r="A407">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B407" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C407" t="s">
         <v>49</v>
       </c>
       <c r="D407" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E407" t="s">
         <v>53</v>
@@ -32031,7 +32034,7 @@
         <v>2026</v>
       </c>
       <c r="R407">
-        <v>16960075</v>
+        <v>17042588</v>
       </c>
       <c r="S407" t="s">
         <v>191</v>
@@ -32063,19 +32066,19 @@
     </row>
     <row r="408" spans="1:35">
       <c r="A408">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B408" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C408" t="s">
         <v>49</v>
       </c>
       <c r="D408" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E408" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F408" t="s">
         <v>55</v>
@@ -32102,7 +32105,7 @@
         <v>2026</v>
       </c>
       <c r="R408">
-        <v>17941218</v>
+        <v>16960075</v>
       </c>
       <c r="S408" t="s">
         <v>191</v>
@@ -32111,13 +32114,13 @@
         <v>206</v>
       </c>
       <c r="V408" s="1">
-        <v>46314.51304733796</v>
+        <v>46314.51304019676</v>
       </c>
       <c r="W408">
         <v>1</v>
       </c>
       <c r="X408" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="AB408">
         <v>0</v>
@@ -32134,16 +32137,16 @@
     </row>
     <row r="409" spans="1:35">
       <c r="A409">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B409" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C409" t="s">
         <v>49</v>
       </c>
       <c r="D409" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E409" t="s">
         <v>54</v>
@@ -32173,7 +32176,7 @@
         <v>2026</v>
       </c>
       <c r="R409">
-        <v>17952445</v>
+        <v>17941218</v>
       </c>
       <c r="S409" t="s">
         <v>191</v>
@@ -32182,13 +32185,13 @@
         <v>206</v>
       </c>
       <c r="V409" s="1">
-        <v>46314.51304903935</v>
+        <v>46314.51304733796</v>
       </c>
       <c r="W409">
         <v>1</v>
       </c>
       <c r="X409" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="AB409">
         <v>0</v>
@@ -32205,16 +32208,16 @@
     </row>
     <row r="410" spans="1:35">
       <c r="A410">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B410" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C410" t="s">
         <v>49</v>
       </c>
       <c r="D410" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E410" t="s">
         <v>54</v>
@@ -32244,7 +32247,7 @@
         <v>2026</v>
       </c>
       <c r="R410">
-        <v>17952625</v>
+        <v>17952445</v>
       </c>
       <c r="S410" t="s">
         <v>191</v>
@@ -32253,7 +32256,7 @@
         <v>206</v>
       </c>
       <c r="V410" s="1">
-        <v>46314.51305077547</v>
+        <v>46314.51304903935</v>
       </c>
       <c r="W410">
         <v>1</v>
@@ -32276,10 +32279,10 @@
     </row>
     <row r="411" spans="1:35">
       <c r="A411">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B411" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C411" t="s">
         <v>49</v>
@@ -32315,7 +32318,7 @@
         <v>2026</v>
       </c>
       <c r="R411">
-        <v>18056802</v>
+        <v>17952625</v>
       </c>
       <c r="S411" t="s">
         <v>191</v>
@@ -32324,7 +32327,7 @@
         <v>206</v>
       </c>
       <c r="V411" s="1">
-        <v>46314.51305917824</v>
+        <v>46314.51305077547</v>
       </c>
       <c r="W411">
         <v>1</v>
@@ -32347,22 +32350,22 @@
     </row>
     <row r="412" spans="1:35">
       <c r="A412">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B412" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C412" t="s">
         <v>49</v>
       </c>
       <c r="D412" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E412" t="s">
         <v>54</v>
       </c>
       <c r="F412" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G412">
         <v>9086</v>
@@ -32386,7 +32389,7 @@
         <v>2026</v>
       </c>
       <c r="R412">
-        <v>18164552</v>
+        <v>18056802</v>
       </c>
       <c r="S412" t="s">
         <v>191</v>
@@ -32395,13 +32398,13 @@
         <v>206</v>
       </c>
       <c r="V412" s="1">
-        <v>46314.51306744213</v>
+        <v>46314.51305917824</v>
       </c>
       <c r="W412">
         <v>1</v>
       </c>
       <c r="X412" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="AB412">
         <v>0</v>
@@ -32418,10 +32421,10 @@
     </row>
     <row r="413" spans="1:35">
       <c r="A413">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B413" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C413" t="s">
         <v>49</v>
@@ -32457,7 +32460,7 @@
         <v>2026</v>
       </c>
       <c r="R413">
-        <v>18178188</v>
+        <v>18164552</v>
       </c>
       <c r="S413" t="s">
         <v>191</v>
@@ -32466,13 +32469,13 @@
         <v>206</v>
       </c>
       <c r="V413" s="1">
-        <v>46314.51306767361</v>
+        <v>46314.51306744213</v>
       </c>
       <c r="W413">
         <v>1</v>
       </c>
       <c r="X413" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AB413">
         <v>0</v>
@@ -32489,16 +32492,16 @@
     </row>
     <row r="414" spans="1:35">
       <c r="A414">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B414" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C414" t="s">
         <v>49</v>
       </c>
       <c r="D414" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E414" t="s">
         <v>54</v>
@@ -32528,7 +32531,7 @@
         <v>2026</v>
       </c>
       <c r="R414">
-        <v>18188775</v>
+        <v>18178188</v>
       </c>
       <c r="S414" t="s">
         <v>191</v>
@@ -32537,13 +32540,13 @@
         <v>206</v>
       </c>
       <c r="V414" s="1">
-        <v>46314.5130681713</v>
+        <v>46314.51306767361</v>
       </c>
       <c r="W414">
         <v>1</v>
       </c>
       <c r="X414" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AB414">
         <v>0</v>
@@ -32560,10 +32563,10 @@
     </row>
     <row r="415" spans="1:35">
       <c r="A415">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B415" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C415" t="s">
         <v>49</v>
@@ -32599,7 +32602,7 @@
         <v>2026</v>
       </c>
       <c r="R415">
-        <v>18188681</v>
+        <v>18188775</v>
       </c>
       <c r="S415" t="s">
         <v>191</v>
@@ -32608,7 +32611,7 @@
         <v>206</v>
       </c>
       <c r="V415" s="1">
-        <v>46314.51306832176</v>
+        <v>46314.5130681713</v>
       </c>
       <c r="W415">
         <v>1</v>
@@ -32631,25 +32634,25 @@
     </row>
     <row r="416" spans="1:35">
       <c r="A416">
-        <v>6627</v>
+        <v>6963</v>
       </c>
       <c r="B416" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C416" t="s">
         <v>49</v>
       </c>
       <c r="D416" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E416" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F416" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G416">
-        <v>940</v>
+        <v>9086</v>
       </c>
       <c r="H416">
         <v>0</v>
@@ -32658,13 +32661,10 @@
         <v>62</v>
       </c>
       <c r="J416" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="N416" s="1">
-        <v>46311</v>
-      </c>
-      <c r="O416" t="s">
-        <v>168</v>
+        <v>46314</v>
       </c>
       <c r="P416">
         <v>10</v>
@@ -32673,25 +32673,22 @@
         <v>2026</v>
       </c>
       <c r="R416">
-        <v>17042222</v>
+        <v>18188681</v>
       </c>
       <c r="S416" t="s">
         <v>191</v>
       </c>
       <c r="U416" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="V416" s="1">
-        <v>46314.42010680556</v>
+        <v>46314.51306832176</v>
       </c>
       <c r="W416">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X416" t="s">
-        <v>207</v>
-      </c>
-      <c r="Y416" t="s">
-        <v>371</v>
+        <v>211</v>
       </c>
       <c r="AB416">
         <v>0</v>
@@ -32708,19 +32705,19 @@
     </row>
     <row r="417" spans="1:35">
       <c r="A417">
-        <v>6703</v>
+        <v>6627</v>
       </c>
       <c r="B417" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="C417" t="s">
         <v>49</v>
       </c>
       <c r="D417" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E417" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F417" t="s">
         <v>55</v>
@@ -32741,7 +32738,7 @@
         <v>46311</v>
       </c>
       <c r="O417" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="P417">
         <v>10</v>
@@ -32750,7 +32747,7 @@
         <v>2026</v>
       </c>
       <c r="R417">
-        <v>17941113</v>
+        <v>17042222</v>
       </c>
       <c r="S417" t="s">
         <v>191</v>
@@ -32759,16 +32756,16 @@
         <v>204</v>
       </c>
       <c r="V417" s="1">
-        <v>46314.78063420139</v>
+        <v>46314.42010680556</v>
       </c>
       <c r="W417">
         <v>4</v>
       </c>
       <c r="X417" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="Y417" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AB417">
         <v>0</v>
@@ -32785,16 +32782,16 @@
     </row>
     <row r="418" spans="1:35">
       <c r="A418">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B418" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C418" t="s">
         <v>49</v>
       </c>
       <c r="D418" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E418" t="s">
         <v>54</v>
@@ -32803,19 +32800,22 @@
         <v>55</v>
       </c>
       <c r="G418">
-        <v>9088</v>
+        <v>940</v>
       </c>
       <c r="H418">
         <v>0</v>
       </c>
       <c r="I418" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J418" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="N418" s="1">
-        <v>46315</v>
+        <v>46311</v>
+      </c>
+      <c r="O418" t="s">
+        <v>167</v>
       </c>
       <c r="P418">
         <v>10</v>
@@ -32824,28 +32824,31 @@
         <v>2026</v>
       </c>
       <c r="R418">
-        <v>17399384</v>
+        <v>17941113</v>
       </c>
       <c r="S418" t="s">
-        <v>54</v>
+        <v>191</v>
       </c>
       <c r="U418" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="V418" s="1">
-        <v>46314.51310813658</v>
+        <v>46314.78063420139</v>
       </c>
       <c r="W418">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X418" t="s">
-        <v>213</v>
+        <v>216</v>
+      </c>
+      <c r="Y418" t="s">
+        <v>372</v>
       </c>
       <c r="AB418">
         <v>0</v>
       </c>
       <c r="AC418" t="s">
-        <v>54</v>
+        <v>191</v>
       </c>
       <c r="AH418" t="s">
         <v>381</v>
@@ -32856,16 +32859,16 @@
     </row>
     <row r="419" spans="1:35">
       <c r="A419">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B419" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C419" t="s">
         <v>49</v>
       </c>
       <c r="D419" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E419" t="s">
         <v>54</v>
@@ -32895,7 +32898,7 @@
         <v>2026</v>
       </c>
       <c r="R419">
-        <v>16962401</v>
+        <v>17399384</v>
       </c>
       <c r="S419" t="s">
         <v>54</v>
@@ -32904,13 +32907,13 @@
         <v>205</v>
       </c>
       <c r="V419" s="1">
-        <v>46314.51312306713</v>
+        <v>46314.51310813658</v>
       </c>
       <c r="W419">
         <v>0</v>
       </c>
       <c r="X419" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AB419">
         <v>0</v>
@@ -32927,16 +32930,16 @@
     </row>
     <row r="420" spans="1:35">
       <c r="A420">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B420" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C420" t="s">
         <v>49</v>
       </c>
       <c r="D420" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E420" t="s">
         <v>54</v>
@@ -32966,7 +32969,7 @@
         <v>2026</v>
       </c>
       <c r="R420">
-        <v>16976291</v>
+        <v>16962401</v>
       </c>
       <c r="S420" t="s">
         <v>54</v>
@@ -32975,13 +32978,13 @@
         <v>205</v>
       </c>
       <c r="V420" s="1">
-        <v>46314.51312457176</v>
+        <v>46314.51312306713</v>
       </c>
       <c r="W420">
         <v>0</v>
       </c>
       <c r="X420" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="AB420">
         <v>0</v>
@@ -32998,10 +33001,10 @@
     </row>
     <row r="421" spans="1:35">
       <c r="A421">
-        <v>6548</v>
+        <v>6486</v>
       </c>
       <c r="B421" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C421" t="s">
         <v>49</v>
@@ -33037,7 +33040,7 @@
         <v>2026</v>
       </c>
       <c r="R421">
-        <v>17222901</v>
+        <v>16976291</v>
       </c>
       <c r="S421" t="s">
         <v>54</v>
@@ -33046,13 +33049,13 @@
         <v>205</v>
       </c>
       <c r="V421" s="1">
-        <v>46314.51312600695</v>
+        <v>46314.51312457176</v>
       </c>
       <c r="W421">
         <v>0</v>
       </c>
       <c r="X421" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="AB421">
         <v>0</v>
@@ -33069,10 +33072,10 @@
     </row>
     <row r="422" spans="1:35">
       <c r="A422">
-        <v>6627</v>
+        <v>6548</v>
       </c>
       <c r="B422" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C422" t="s">
         <v>49</v>
@@ -33081,7 +33084,7 @@
         <v>50</v>
       </c>
       <c r="E422" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F422" t="s">
         <v>55</v>
@@ -33108,28 +33111,28 @@
         <v>2026</v>
       </c>
       <c r="R422">
-        <v>17042628</v>
+        <v>17222901</v>
       </c>
       <c r="S422" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="U422" t="s">
         <v>205</v>
       </c>
       <c r="V422" s="1">
-        <v>46314.51312769676</v>
+        <v>46314.51312600695</v>
       </c>
       <c r="W422">
         <v>0</v>
       </c>
       <c r="X422" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AB422">
         <v>0</v>
       </c>
       <c r="AC422" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AH422" t="s">
         <v>381</v>
@@ -33140,16 +33143,16 @@
     </row>
     <row r="423" spans="1:35">
       <c r="A423">
-        <v>6628</v>
+        <v>6627</v>
       </c>
       <c r="B423" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C423" t="s">
         <v>49</v>
       </c>
       <c r="D423" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E423" t="s">
         <v>53</v>
@@ -33179,7 +33182,7 @@
         <v>2026</v>
       </c>
       <c r="R423">
-        <v>16960099</v>
+        <v>17042628</v>
       </c>
       <c r="S423" t="s">
         <v>53</v>
@@ -33188,7 +33191,7 @@
         <v>205</v>
       </c>
       <c r="V423" s="1">
-        <v>46314.5131278125</v>
+        <v>46314.51312769676</v>
       </c>
       <c r="W423">
         <v>0</v>
@@ -33211,19 +33214,19 @@
     </row>
     <row r="424" spans="1:35">
       <c r="A424">
-        <v>6703</v>
+        <v>6628</v>
       </c>
       <c r="B424" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C424" t="s">
         <v>49</v>
       </c>
       <c r="D424" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E424" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F424" t="s">
         <v>55</v>
@@ -33250,28 +33253,28 @@
         <v>2026</v>
       </c>
       <c r="R424">
-        <v>17941238</v>
+        <v>16960099</v>
       </c>
       <c r="S424" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="U424" t="s">
         <v>205</v>
       </c>
       <c r="V424" s="1">
-        <v>46314.51313017361</v>
+        <v>46314.5131278125</v>
       </c>
       <c r="W424">
         <v>0</v>
       </c>
       <c r="X424" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="AB424">
         <v>0</v>
       </c>
       <c r="AC424" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AH424" t="s">
         <v>381</v>
@@ -33282,16 +33285,16 @@
     </row>
     <row r="425" spans="1:35">
       <c r="A425">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B425" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C425" t="s">
         <v>49</v>
       </c>
       <c r="D425" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E425" t="s">
         <v>54</v>
@@ -33321,7 +33324,7 @@
         <v>2026</v>
       </c>
       <c r="R425">
-        <v>17952467</v>
+        <v>17941238</v>
       </c>
       <c r="S425" t="s">
         <v>54</v>
@@ -33330,13 +33333,13 @@
         <v>205</v>
       </c>
       <c r="V425" s="1">
-        <v>46314.5131303588</v>
+        <v>46314.51313017361</v>
       </c>
       <c r="W425">
         <v>0</v>
       </c>
       <c r="X425" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="AB425">
         <v>0</v>
@@ -33353,16 +33356,16 @@
     </row>
     <row r="426" spans="1:35">
       <c r="A426">
-        <v>6705</v>
+        <v>6704</v>
       </c>
       <c r="B426" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C426" t="s">
         <v>49</v>
       </c>
       <c r="D426" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E426" t="s">
         <v>54</v>
@@ -33392,7 +33395,7 @@
         <v>2026</v>
       </c>
       <c r="R426">
-        <v>17952647</v>
+        <v>17952467</v>
       </c>
       <c r="S426" t="s">
         <v>54</v>
@@ -33401,7 +33404,7 @@
         <v>205</v>
       </c>
       <c r="V426" s="1">
-        <v>46314.51313075231</v>
+        <v>46314.5131303588</v>
       </c>
       <c r="W426">
         <v>0</v>
@@ -33424,10 +33427,10 @@
     </row>
     <row r="427" spans="1:35">
       <c r="A427">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B427" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C427" t="s">
         <v>49</v>
@@ -33463,16 +33466,16 @@
         <v>2026</v>
       </c>
       <c r="R427">
-        <v>18056822</v>
+        <v>17952647</v>
       </c>
       <c r="S427" t="s">
-        <v>192</v>
+        <v>54</v>
       </c>
       <c r="U427" t="s">
         <v>205</v>
       </c>
       <c r="V427" s="1">
-        <v>46314.5131318287</v>
+        <v>46314.51313075231</v>
       </c>
       <c r="W427">
         <v>0</v>
@@ -33484,7 +33487,7 @@
         <v>0</v>
       </c>
       <c r="AC427" t="s">
-        <v>192</v>
+        <v>54</v>
       </c>
       <c r="AH427" t="s">
         <v>381</v>
@@ -33495,22 +33498,22 @@
     </row>
     <row r="428" spans="1:35">
       <c r="A428">
-        <v>6945</v>
+        <v>6779</v>
       </c>
       <c r="B428" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C428" t="s">
         <v>49</v>
       </c>
       <c r="D428" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E428" t="s">
         <v>54</v>
       </c>
       <c r="F428" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G428">
         <v>9088</v>
@@ -33534,28 +33537,28 @@
         <v>2026</v>
       </c>
       <c r="R428">
-        <v>18164566</v>
+        <v>18056822</v>
       </c>
       <c r="S428" t="s">
-        <v>54</v>
+        <v>192</v>
       </c>
       <c r="U428" t="s">
         <v>205</v>
       </c>
       <c r="V428" s="1">
-        <v>46314.51313622685</v>
+        <v>46314.5131318287</v>
       </c>
       <c r="W428">
         <v>0</v>
       </c>
       <c r="X428" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="AB428">
         <v>0</v>
       </c>
       <c r="AC428" t="s">
-        <v>54</v>
+        <v>192</v>
       </c>
       <c r="AH428" t="s">
         <v>381</v>
@@ -33566,10 +33569,10 @@
     </row>
     <row r="429" spans="1:35">
       <c r="A429">
-        <v>6949</v>
+        <v>6945</v>
       </c>
       <c r="B429" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C429" t="s">
         <v>49</v>
@@ -33605,7 +33608,7 @@
         <v>2026</v>
       </c>
       <c r="R429">
-        <v>18178200</v>
+        <v>18164566</v>
       </c>
       <c r="S429" t="s">
         <v>54</v>
@@ -33614,13 +33617,13 @@
         <v>205</v>
       </c>
       <c r="V429" s="1">
-        <v>46314.51313657407</v>
+        <v>46314.51313622685</v>
       </c>
       <c r="W429">
         <v>0</v>
       </c>
       <c r="X429" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AB429">
         <v>0</v>
@@ -33637,16 +33640,16 @@
     </row>
     <row r="430" spans="1:35">
       <c r="A430">
-        <v>6962</v>
+        <v>6949</v>
       </c>
       <c r="B430" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C430" t="s">
         <v>49</v>
       </c>
       <c r="D430" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E430" t="s">
         <v>54</v>
@@ -33676,7 +33679,7 @@
         <v>2026</v>
       </c>
       <c r="R430">
-        <v>18188789</v>
+        <v>18178200</v>
       </c>
       <c r="S430" t="s">
         <v>54</v>
@@ -33685,13 +33688,13 @@
         <v>205</v>
       </c>
       <c r="V430" s="1">
-        <v>46314.51313734954</v>
+        <v>46314.51313657407</v>
       </c>
       <c r="W430">
         <v>0</v>
       </c>
       <c r="X430" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AB430">
         <v>0</v>
@@ -33708,10 +33711,10 @@
     </row>
     <row r="431" spans="1:35">
       <c r="A431">
-        <v>6963</v>
+        <v>6962</v>
       </c>
       <c r="B431" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C431" t="s">
         <v>49</v>
@@ -33747,7 +33750,7 @@
         <v>2026</v>
       </c>
       <c r="R431">
-        <v>18188695</v>
+        <v>18188789</v>
       </c>
       <c r="S431" t="s">
         <v>54</v>
@@ -33756,7 +33759,7 @@
         <v>205</v>
       </c>
       <c r="V431" s="1">
-        <v>46314.51313761574</v>
+        <v>46314.51313734954</v>
       </c>
       <c r="W431">
         <v>0</v>
@@ -33779,25 +33782,25 @@
     </row>
     <row r="432" spans="1:35">
       <c r="A432">
-        <v>6627</v>
+        <v>6963</v>
       </c>
       <c r="B432" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C432" t="s">
         <v>49</v>
       </c>
       <c r="D432" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E432" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F432" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G432">
-        <v>6813</v>
+        <v>9088</v>
       </c>
       <c r="H432">
         <v>0</v>
@@ -33806,10 +33809,10 @@
         <v>63</v>
       </c>
       <c r="J432" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="N432" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="P432">
         <v>10</v>
@@ -33818,28 +33821,28 @@
         <v>2026</v>
       </c>
       <c r="R432">
-        <v>17042471</v>
+        <v>18188695</v>
       </c>
       <c r="S432" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="U432" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="V432" s="1">
-        <v>46314.42010591435</v>
+        <v>46314.51313761574</v>
       </c>
       <c r="W432">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X432" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="AB432">
         <v>0</v>
       </c>
       <c r="AC432" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AH432" t="s">
         <v>381</v>
@@ -33850,19 +33853,19 @@
     </row>
     <row r="433" spans="1:35">
       <c r="A433">
-        <v>6703</v>
+        <v>6627</v>
       </c>
       <c r="B433" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="C433" t="s">
         <v>49</v>
       </c>
       <c r="D433" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E433" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F433" t="s">
         <v>55</v>
@@ -33882,9 +33885,6 @@
       <c r="N433" s="1">
         <v>46314</v>
       </c>
-      <c r="O433" t="s">
-        <v>167</v>
-      </c>
       <c r="P433">
         <v>10</v>
       </c>
@@ -33892,31 +33892,28 @@
         <v>2026</v>
       </c>
       <c r="R433">
-        <v>17941198</v>
+        <v>17042471</v>
       </c>
       <c r="S433" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="U433" t="s">
         <v>206</v>
       </c>
       <c r="V433" s="1">
-        <v>46314.78063710648</v>
+        <v>46314.42010591435</v>
       </c>
       <c r="W433">
         <v>1</v>
       </c>
       <c r="X433" t="s">
-        <v>216</v>
-      </c>
-      <c r="Y433" t="s">
-        <v>373</v>
+        <v>207</v>
       </c>
       <c r="AB433">
         <v>0</v>
       </c>
       <c r="AC433" t="s">
-        <v>191</v>
+        <v>53</v>
       </c>
       <c r="AH433" t="s">
         <v>381</v>
@@ -33927,10 +33924,10 @@
     </row>
     <row r="434" spans="1:35">
       <c r="A434">
-        <v>6404</v>
+        <v>6703</v>
       </c>
       <c r="B434" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C434" t="s">
         <v>49</v>
@@ -33945,7 +33942,7 @@
         <v>55</v>
       </c>
       <c r="G434">
-        <v>11001</v>
+        <v>6813</v>
       </c>
       <c r="H434">
         <v>0</v>
@@ -33954,46 +33951,49 @@
         <v>63</v>
       </c>
       <c r="J434" t="s">
-        <v>69</v>
+        <v>140</v>
       </c>
       <c r="N434" s="1">
-        <v>46290</v>
+        <v>46314</v>
+      </c>
+      <c r="O434" t="s">
+        <v>167</v>
       </c>
       <c r="P434">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q434">
         <v>2026</v>
       </c>
       <c r="R434">
-        <v>16962454</v>
+        <v>17941198</v>
       </c>
       <c r="S434" t="s">
         <v>54</v>
       </c>
       <c r="U434" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="V434" s="1">
-        <v>46314.6513366088</v>
+        <v>46314.78063710648</v>
       </c>
       <c r="W434">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="X434" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="Y434" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="AB434">
         <v>0</v>
       </c>
       <c r="AC434" t="s">
-        <v>54</v>
+        <v>191</v>
       </c>
       <c r="AH434" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="AI434" t="s">
         <v>385</v>
@@ -34001,16 +34001,16 @@
     </row>
     <row r="435" spans="1:35">
       <c r="A435">
-        <v>5417</v>
+        <v>6404</v>
       </c>
       <c r="B435" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C435" t="s">
         <v>49</v>
       </c>
       <c r="D435" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E435" t="s">
         <v>54</v>
@@ -34019,7 +34019,7 @@
         <v>55</v>
       </c>
       <c r="G435">
-        <v>7877</v>
+        <v>11001</v>
       </c>
       <c r="H435">
         <v>0</v>
@@ -34028,7 +34028,7 @@
         <v>63</v>
       </c>
       <c r="J435" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="N435" s="1">
         <v>46290</v>
@@ -34040,7 +34040,7 @@
         <v>2026</v>
       </c>
       <c r="R435">
-        <v>17399330</v>
+        <v>16962454</v>
       </c>
       <c r="S435" t="s">
         <v>54</v>
@@ -34049,16 +34049,16 @@
         <v>204</v>
       </c>
       <c r="V435" s="1">
-        <v>46314.64967491898</v>
+        <v>46314.6513366088</v>
       </c>
       <c r="W435">
         <v>25</v>
       </c>
       <c r="X435" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Y435" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="AB435">
         <v>0</v>
@@ -34070,6 +34070,80 @@
         <v>379</v>
       </c>
       <c r="AI435" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="436" spans="1:35">
+      <c r="A436">
+        <v>5417</v>
+      </c>
+      <c r="B436" t="s">
+        <v>43</v>
+      </c>
+      <c r="C436" t="s">
+        <v>49</v>
+      </c>
+      <c r="D436" t="s">
+        <v>50</v>
+      </c>
+      <c r="E436" t="s">
+        <v>54</v>
+      </c>
+      <c r="F436" t="s">
+        <v>55</v>
+      </c>
+      <c r="G436">
+        <v>7877</v>
+      </c>
+      <c r="H436">
+        <v>0</v>
+      </c>
+      <c r="I436" t="s">
+        <v>63</v>
+      </c>
+      <c r="J436" t="s">
+        <v>65</v>
+      </c>
+      <c r="N436" s="1">
+        <v>46290</v>
+      </c>
+      <c r="P436">
+        <v>8</v>
+      </c>
+      <c r="Q436">
+        <v>2026</v>
+      </c>
+      <c r="R436">
+        <v>17399330</v>
+      </c>
+      <c r="S436" t="s">
+        <v>54</v>
+      </c>
+      <c r="U436" t="s">
+        <v>204</v>
+      </c>
+      <c r="V436" s="1">
+        <v>46314.64967491898</v>
+      </c>
+      <c r="W436">
+        <v>25</v>
+      </c>
+      <c r="X436" t="s">
+        <v>213</v>
+      </c>
+      <c r="Y436" t="s">
+        <v>375</v>
+      </c>
+      <c r="AB436">
+        <v>0</v>
+      </c>
+      <c r="AC436" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH436" t="s">
+        <v>379</v>
+      </c>
+      <c r="AI436" t="s">
         <v>385</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-21 18:18
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6693" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6729" uniqueCount="414">
   <si>
     <t>CodCliente</t>
   </si>
@@ -3275,6 +3275,9 @@
       <c r="S22" t="s">
         <v>187</v>
       </c>
+      <c r="T22" t="s">
+        <v>207</v>
+      </c>
       <c r="U22" t="s">
         <v>214</v>
       </c>
@@ -3660,6 +3663,9 @@
       <c r="S27" t="s">
         <v>187</v>
       </c>
+      <c r="T27" t="s">
+        <v>207</v>
+      </c>
       <c r="U27" t="s">
         <v>213</v>
       </c>
@@ -3737,6 +3743,9 @@
       <c r="S28" t="s">
         <v>187</v>
       </c>
+      <c r="T28" t="s">
+        <v>207</v>
+      </c>
       <c r="U28" t="s">
         <v>213</v>
       </c>
@@ -4042,6 +4051,9 @@
       <c r="S32" t="s">
         <v>187</v>
       </c>
+      <c r="T32" t="s">
+        <v>207</v>
+      </c>
       <c r="U32" t="s">
         <v>214</v>
       </c>
@@ -4119,6 +4131,9 @@
       <c r="S33" t="s">
         <v>187</v>
       </c>
+      <c r="T33" t="s">
+        <v>207</v>
+      </c>
       <c r="U33" t="s">
         <v>212</v>
       </c>
@@ -4196,6 +4211,9 @@
       <c r="S34" t="s">
         <v>187</v>
       </c>
+      <c r="T34" t="s">
+        <v>207</v>
+      </c>
       <c r="U34" t="s">
         <v>212</v>
       </c>
@@ -4673,6 +4691,9 @@
       <c r="S40" t="s">
         <v>187</v>
       </c>
+      <c r="T40" t="s">
+        <v>207</v>
+      </c>
       <c r="U40" t="s">
         <v>213</v>
       </c>
@@ -4750,6 +4771,9 @@
       <c r="S41" t="s">
         <v>187</v>
       </c>
+      <c r="T41" t="s">
+        <v>207</v>
+      </c>
       <c r="U41" t="s">
         <v>213</v>
       </c>
@@ -4827,6 +4851,9 @@
       <c r="S42" t="s">
         <v>187</v>
       </c>
+      <c r="T42" t="s">
+        <v>207</v>
+      </c>
       <c r="U42" t="s">
         <v>213</v>
       </c>
@@ -5428,6 +5455,9 @@
       <c r="S50" t="s">
         <v>187</v>
       </c>
+      <c r="T50" t="s">
+        <v>207</v>
+      </c>
       <c r="U50" t="s">
         <v>212</v>
       </c>
@@ -5505,6 +5535,9 @@
       <c r="S51" t="s">
         <v>187</v>
       </c>
+      <c r="T51" t="s">
+        <v>207</v>
+      </c>
       <c r="U51" t="s">
         <v>212</v>
       </c>
@@ -5582,6 +5615,9 @@
       <c r="S52" t="s">
         <v>187</v>
       </c>
+      <c r="T52" t="s">
+        <v>207</v>
+      </c>
       <c r="U52" t="s">
         <v>212</v>
       </c>
@@ -5979,6 +6015,9 @@
       <c r="S57" t="s">
         <v>187</v>
       </c>
+      <c r="T57" t="s">
+        <v>207</v>
+      </c>
       <c r="U57" t="s">
         <v>214</v>
       </c>
@@ -6056,6 +6095,9 @@
       <c r="S58" t="s">
         <v>187</v>
       </c>
+      <c r="T58" t="s">
+        <v>207</v>
+      </c>
       <c r="U58" t="s">
         <v>212</v>
       </c>
@@ -6133,6 +6175,9 @@
       <c r="S59" t="s">
         <v>187</v>
       </c>
+      <c r="T59" t="s">
+        <v>207</v>
+      </c>
       <c r="U59" t="s">
         <v>212</v>
       </c>
@@ -6684,6 +6729,9 @@
       <c r="S66" t="s">
         <v>187</v>
       </c>
+      <c r="T66" t="s">
+        <v>207</v>
+      </c>
       <c r="U66" t="s">
         <v>214</v>
       </c>
@@ -6761,6 +6809,9 @@
       <c r="S67" t="s">
         <v>187</v>
       </c>
+      <c r="T67" t="s">
+        <v>207</v>
+      </c>
       <c r="U67" t="s">
         <v>212</v>
       </c>
@@ -6838,6 +6889,9 @@
       <c r="S68" t="s">
         <v>187</v>
       </c>
+      <c r="T68" t="s">
+        <v>207</v>
+      </c>
       <c r="U68" t="s">
         <v>212</v>
       </c>
@@ -18429,6 +18483,9 @@
       <c r="S225" t="s">
         <v>187</v>
       </c>
+      <c r="T225" t="s">
+        <v>207</v>
+      </c>
       <c r="U225" t="s">
         <v>214</v>
       </c>
@@ -18500,6 +18557,9 @@
       <c r="S226" t="s">
         <v>187</v>
       </c>
+      <c r="T226" t="s">
+        <v>207</v>
+      </c>
       <c r="U226" t="s">
         <v>214</v>
       </c>
@@ -19101,6 +19161,9 @@
       <c r="S234" t="s">
         <v>187</v>
       </c>
+      <c r="T234" t="s">
+        <v>207</v>
+      </c>
       <c r="U234" t="s">
         <v>213</v>
       </c>
@@ -19252,6 +19315,9 @@
       <c r="S236" t="s">
         <v>187</v>
       </c>
+      <c r="T236" t="s">
+        <v>207</v>
+      </c>
       <c r="U236" t="s">
         <v>213</v>
       </c>
@@ -19326,6 +19392,9 @@
       <c r="S237" t="s">
         <v>187</v>
       </c>
+      <c r="T237" t="s">
+        <v>207</v>
+      </c>
       <c r="U237" t="s">
         <v>213</v>
       </c>
@@ -19797,6 +19866,9 @@
       <c r="S243" t="s">
         <v>187</v>
       </c>
+      <c r="T243" t="s">
+        <v>207</v>
+      </c>
       <c r="U243" t="s">
         <v>212</v>
       </c>
@@ -20108,6 +20180,9 @@
       <c r="S247" t="s">
         <v>187</v>
       </c>
+      <c r="T247" t="s">
+        <v>207</v>
+      </c>
       <c r="U247" t="s">
         <v>213</v>
       </c>
@@ -20259,6 +20334,9 @@
       <c r="S249" t="s">
         <v>187</v>
       </c>
+      <c r="T249" t="s">
+        <v>207</v>
+      </c>
       <c r="U249" t="s">
         <v>213</v>
       </c>
@@ -20333,6 +20411,9 @@
       <c r="S250" t="s">
         <v>187</v>
       </c>
+      <c r="T250" t="s">
+        <v>207</v>
+      </c>
       <c r="U250" t="s">
         <v>213</v>
       </c>
@@ -28703,6 +28784,9 @@
       <c r="S361" t="s">
         <v>187</v>
       </c>
+      <c r="T361" t="s">
+        <v>207</v>
+      </c>
       <c r="U361" t="s">
         <v>213</v>
       </c>
@@ -28774,6 +28858,9 @@
       <c r="S362" t="s">
         <v>187</v>
       </c>
+      <c r="T362" t="s">
+        <v>207</v>
+      </c>
       <c r="U362" t="s">
         <v>213</v>
       </c>
@@ -28845,6 +28932,9 @@
       <c r="S363" t="s">
         <v>187</v>
       </c>
+      <c r="T363" t="s">
+        <v>207</v>
+      </c>
       <c r="U363" t="s">
         <v>213</v>
       </c>
@@ -29230,6 +29320,9 @@
       <c r="S368" t="s">
         <v>187</v>
       </c>
+      <c r="T368" t="s">
+        <v>207</v>
+      </c>
       <c r="U368" t="s">
         <v>213</v>
       </c>
@@ -29301,6 +29394,9 @@
       <c r="S369" t="s">
         <v>187</v>
       </c>
+      <c r="T369" t="s">
+        <v>207</v>
+      </c>
       <c r="U369" t="s">
         <v>213</v>
       </c>
@@ -29372,6 +29468,9 @@
       <c r="S370" t="s">
         <v>187</v>
       </c>
+      <c r="T370" t="s">
+        <v>207</v>
+      </c>
       <c r="U370" t="s">
         <v>213</v>
       </c>
@@ -29757,6 +29856,9 @@
       <c r="S375" t="s">
         <v>187</v>
       </c>
+      <c r="T375" t="s">
+        <v>207</v>
+      </c>
       <c r="U375" t="s">
         <v>213</v>
       </c>
@@ -29908,6 +30010,9 @@
       <c r="S377" t="s">
         <v>187</v>
       </c>
+      <c r="T377" t="s">
+        <v>207</v>
+      </c>
       <c r="U377" t="s">
         <v>213</v>
       </c>
@@ -29978,6 +30083,9 @@
       </c>
       <c r="S378" t="s">
         <v>187</v>
+      </c>
+      <c r="T378" t="s">
+        <v>207</v>
       </c>
       <c r="U378" t="s">
         <v>213</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-26 16:15
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7443" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7499" uniqueCount="456">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1761,7 +1761,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI514"/>
+  <dimension ref="A1:AI518"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -40291,10 +40291,10 @@
     </row>
     <row r="512" spans="1:35">
       <c r="A512">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B512" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C512" t="s">
         <v>49</v>
@@ -40306,10 +40306,10 @@
         <v>54</v>
       </c>
       <c r="F512" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G512">
-        <v>11541</v>
+        <v>11542</v>
       </c>
       <c r="H512">
         <v>0</v>
@@ -40318,7 +40318,7 @@
         <v>59</v>
       </c>
       <c r="J512" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="N512" s="1">
         <v>46325</v>
@@ -40330,31 +40330,31 @@
         <v>2026</v>
       </c>
       <c r="R512">
-        <v>18248553</v>
+        <v>18307831</v>
       </c>
       <c r="S512" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="T512" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="U512" t="s">
         <v>226</v>
       </c>
       <c r="V512" s="1">
-        <v>46321.59424188657</v>
+        <v>46321.66110923611</v>
       </c>
       <c r="W512">
         <v>-4</v>
       </c>
       <c r="X512" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="AB512">
         <v>0</v>
       </c>
       <c r="AC512" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="AH512" t="s">
         <v>450</v>
@@ -40365,73 +40365,73 @@
     </row>
     <row r="513" spans="1:35">
       <c r="A513">
-        <v>6962</v>
+        <v>5417</v>
       </c>
       <c r="B513" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C513" t="s">
         <v>49</v>
       </c>
       <c r="D513" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E513" t="s">
         <v>54</v>
       </c>
       <c r="F513" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G513">
-        <v>5984</v>
+        <v>11541</v>
       </c>
       <c r="H513">
-        <v>1884</v>
+        <v>0</v>
       </c>
       <c r="I513" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J513" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="N513" s="1">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="P513">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q513">
         <v>2026</v>
       </c>
       <c r="R513">
-        <v>18260053</v>
+        <v>18248553</v>
       </c>
       <c r="S513" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="T513" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="U513" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V513" s="1">
-        <v>46321.39266284723</v>
+        <v>46321.59424188657</v>
       </c>
       <c r="W513">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="X513" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="AB513">
         <v>0</v>
       </c>
       <c r="AC513" t="s">
-        <v>223</v>
+        <v>203</v>
       </c>
       <c r="AH513" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="AI513" t="s">
         <v>455</v>
@@ -40439,16 +40439,16 @@
     </row>
     <row r="514" spans="1:35">
       <c r="A514">
-        <v>6963</v>
+        <v>6945</v>
       </c>
       <c r="B514" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C514" t="s">
         <v>49</v>
       </c>
       <c r="D514" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E514" t="s">
         <v>54</v>
@@ -40457,57 +40457,353 @@
         <v>56</v>
       </c>
       <c r="G514">
+        <v>11541</v>
+      </c>
+      <c r="H514">
+        <v>0</v>
+      </c>
+      <c r="I514" t="s">
+        <v>59</v>
+      </c>
+      <c r="J514" t="s">
+        <v>169</v>
+      </c>
+      <c r="N514" s="1">
+        <v>46325</v>
+      </c>
+      <c r="P514">
+        <v>11</v>
+      </c>
+      <c r="Q514">
+        <v>2026</v>
+      </c>
+      <c r="R514">
+        <v>18307829</v>
+      </c>
+      <c r="S514" t="s">
+        <v>201</v>
+      </c>
+      <c r="T514" t="s">
+        <v>220</v>
+      </c>
+      <c r="U514" t="s">
+        <v>226</v>
+      </c>
+      <c r="V514" s="1">
+        <v>46321.6622389699</v>
+      </c>
+      <c r="W514">
+        <v>-4</v>
+      </c>
+      <c r="X514" t="s">
+        <v>230</v>
+      </c>
+      <c r="AB514">
+        <v>0</v>
+      </c>
+      <c r="AC514" t="s">
+        <v>201</v>
+      </c>
+      <c r="AH514" t="s">
+        <v>450</v>
+      </c>
+      <c r="AI514" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="515" spans="1:35">
+      <c r="A515">
+        <v>6962</v>
+      </c>
+      <c r="B515" t="s">
+        <v>40</v>
+      </c>
+      <c r="C515" t="s">
+        <v>49</v>
+      </c>
+      <c r="D515" t="s">
+        <v>52</v>
+      </c>
+      <c r="E515" t="s">
+        <v>54</v>
+      </c>
+      <c r="F515" t="s">
+        <v>56</v>
+      </c>
+      <c r="G515">
         <v>5984</v>
       </c>
-      <c r="H514">
+      <c r="H515">
         <v>1884</v>
       </c>
-      <c r="I514" t="s">
+      <c r="I515" t="s">
         <v>60</v>
       </c>
-      <c r="J514" t="s">
+      <c r="J515" t="s">
         <v>170</v>
       </c>
-      <c r="N514" s="1">
+      <c r="N515" s="1">
         <v>46321</v>
       </c>
-      <c r="P514">
+      <c r="P515">
         <v>9</v>
       </c>
-      <c r="Q514">
-        <v>2026</v>
-      </c>
-      <c r="R514">
+      <c r="Q515">
+        <v>2026</v>
+      </c>
+      <c r="R515">
+        <v>18260053</v>
+      </c>
+      <c r="S515" t="s">
+        <v>210</v>
+      </c>
+      <c r="T515" t="s">
+        <v>223</v>
+      </c>
+      <c r="U515" t="s">
+        <v>227</v>
+      </c>
+      <c r="V515" s="1">
+        <v>46321.39266284723</v>
+      </c>
+      <c r="W515">
+        <v>0</v>
+      </c>
+      <c r="X515" t="s">
+        <v>232</v>
+      </c>
+      <c r="AB515">
+        <v>0</v>
+      </c>
+      <c r="AC515" t="s">
+        <v>223</v>
+      </c>
+      <c r="AH515" t="s">
+        <v>448</v>
+      </c>
+      <c r="AI515" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="516" spans="1:35">
+      <c r="A516">
+        <v>6963</v>
+      </c>
+      <c r="B516" t="s">
+        <v>41</v>
+      </c>
+      <c r="C516" t="s">
+        <v>49</v>
+      </c>
+      <c r="D516" t="s">
+        <v>52</v>
+      </c>
+      <c r="E516" t="s">
+        <v>54</v>
+      </c>
+      <c r="F516" t="s">
+        <v>56</v>
+      </c>
+      <c r="G516">
+        <v>5984</v>
+      </c>
+      <c r="H516">
+        <v>1884</v>
+      </c>
+      <c r="I516" t="s">
+        <v>60</v>
+      </c>
+      <c r="J516" t="s">
+        <v>170</v>
+      </c>
+      <c r="N516" s="1">
+        <v>46321</v>
+      </c>
+      <c r="P516">
+        <v>9</v>
+      </c>
+      <c r="Q516">
+        <v>2026</v>
+      </c>
+      <c r="R516">
         <v>18260186</v>
       </c>
-      <c r="S514" t="s">
+      <c r="S516" t="s">
         <v>210</v>
       </c>
-      <c r="T514" t="s">
+      <c r="T516" t="s">
         <v>223</v>
       </c>
-      <c r="U514" t="s">
+      <c r="U516" t="s">
         <v>227</v>
       </c>
-      <c r="V514" s="1">
+      <c r="V516" s="1">
         <v>46321.39266328704</v>
       </c>
-      <c r="W514">
-        <v>0</v>
-      </c>
-      <c r="X514" t="s">
+      <c r="W516">
+        <v>0</v>
+      </c>
+      <c r="X516" t="s">
         <v>232</v>
       </c>
-      <c r="AB514">
-        <v>0</v>
-      </c>
-      <c r="AC514" t="s">
+      <c r="AB516">
+        <v>0</v>
+      </c>
+      <c r="AC516" t="s">
         <v>223</v>
       </c>
-      <c r="AH514" t="s">
+      <c r="AH516" t="s">
         <v>448</v>
       </c>
-      <c r="AI514" t="s">
+      <c r="AI516" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="517" spans="1:35">
+      <c r="A517">
+        <v>5417</v>
+      </c>
+      <c r="B517" t="s">
+        <v>43</v>
+      </c>
+      <c r="C517" t="s">
+        <v>49</v>
+      </c>
+      <c r="D517" t="s">
+        <v>50</v>
+      </c>
+      <c r="E517" t="s">
+        <v>54</v>
+      </c>
+      <c r="F517" t="s">
+        <v>55</v>
+      </c>
+      <c r="G517">
+        <v>6759</v>
+      </c>
+      <c r="H517">
+        <v>1788</v>
+      </c>
+      <c r="I517" t="s">
+        <v>61</v>
+      </c>
+      <c r="J517" t="s">
+        <v>160</v>
+      </c>
+      <c r="N517" s="1">
+        <v>46321</v>
+      </c>
+      <c r="P517">
+        <v>9</v>
+      </c>
+      <c r="Q517">
+        <v>2026</v>
+      </c>
+      <c r="R517">
+        <v>17399191</v>
+      </c>
+      <c r="S517" t="s">
+        <v>211</v>
+      </c>
+      <c r="T517" t="s">
+        <v>224</v>
+      </c>
+      <c r="U517" t="s">
+        <v>227</v>
+      </c>
+      <c r="V517" s="1">
+        <v>46321.66995337963</v>
+      </c>
+      <c r="W517">
+        <v>0</v>
+      </c>
+      <c r="X517" t="s">
+        <v>234</v>
+      </c>
+      <c r="AB517">
+        <v>0</v>
+      </c>
+      <c r="AC517" t="s">
+        <v>211</v>
+      </c>
+      <c r="AH517" t="s">
+        <v>448</v>
+      </c>
+      <c r="AI517" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="518" spans="1:35">
+      <c r="A518">
+        <v>6705</v>
+      </c>
+      <c r="B518" t="s">
+        <v>45</v>
+      </c>
+      <c r="C518" t="s">
+        <v>49</v>
+      </c>
+      <c r="D518" t="s">
+        <v>51</v>
+      </c>
+      <c r="E518" t="s">
+        <v>54</v>
+      </c>
+      <c r="F518" t="s">
+        <v>55</v>
+      </c>
+      <c r="G518">
+        <v>6759</v>
+      </c>
+      <c r="H518">
+        <v>1788</v>
+      </c>
+      <c r="I518" t="s">
+        <v>61</v>
+      </c>
+      <c r="J518" t="s">
+        <v>160</v>
+      </c>
+      <c r="N518" s="1">
+        <v>46321</v>
+      </c>
+      <c r="P518">
+        <v>9</v>
+      </c>
+      <c r="Q518">
+        <v>2026</v>
+      </c>
+      <c r="R518">
+        <v>17949020</v>
+      </c>
+      <c r="S518" t="s">
+        <v>211</v>
+      </c>
+      <c r="T518" t="s">
+        <v>224</v>
+      </c>
+      <c r="U518" t="s">
+        <v>227</v>
+      </c>
+      <c r="V518" s="1">
+        <v>46321.6685106713</v>
+      </c>
+      <c r="W518">
+        <v>0</v>
+      </c>
+      <c r="X518" t="s">
+        <v>235</v>
+      </c>
+      <c r="AB518">
+        <v>0</v>
+      </c>
+      <c r="AC518" t="s">
+        <v>211</v>
+      </c>
+      <c r="AH518" t="s">
+        <v>448</v>
+      </c>
+      <c r="AI518" t="s">
         <v>455</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-26 16:46
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7499" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7527" uniqueCount="456">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1761,7 +1761,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI518"/>
+  <dimension ref="A1:AI520"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -28205,7 +28205,7 @@
         <v>54</v>
       </c>
       <c r="F352" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G352">
         <v>7869</v>
@@ -28504,7 +28504,7 @@
         <v>54</v>
       </c>
       <c r="F356" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G356">
         <v>1697</v>
@@ -29881,7 +29881,7 @@
         <v>54</v>
       </c>
       <c r="F374" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G374">
         <v>5883</v>
@@ -30417,7 +30417,7 @@
         <v>54</v>
       </c>
       <c r="F381" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G381">
         <v>5884</v>
@@ -31753,7 +31753,7 @@
         <v>54</v>
       </c>
       <c r="F398" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G398">
         <v>5823</v>
@@ -32523,7 +32523,7 @@
         <v>54</v>
       </c>
       <c r="F408" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G408">
         <v>1913</v>
@@ -33388,7 +33388,7 @@
         <v>54</v>
       </c>
       <c r="F419" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G419">
         <v>1882</v>
@@ -33702,7 +33702,7 @@
         <v>54</v>
       </c>
       <c r="F423" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G423">
         <v>1914</v>
@@ -36018,7 +36018,7 @@
         <v>54</v>
       </c>
       <c r="F453" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G453">
         <v>953</v>
@@ -36533,7 +36533,7 @@
         <v>54</v>
       </c>
       <c r="F460" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G460">
         <v>7022</v>
@@ -37385,7 +37385,7 @@
         <v>54</v>
       </c>
       <c r="F472" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G472">
         <v>9086</v>
@@ -38533,7 +38533,7 @@
         <v>54</v>
       </c>
       <c r="F488" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G488">
         <v>9088</v>
@@ -39560,7 +39560,7 @@
         <v>54</v>
       </c>
       <c r="F502" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G502">
         <v>11056</v>
@@ -40217,16 +40217,16 @@
     </row>
     <row r="511" spans="1:35">
       <c r="A511">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B511" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C511" t="s">
         <v>49</v>
       </c>
       <c r="D511" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E511" t="s">
         <v>54</v>
@@ -40256,10 +40256,10 @@
         <v>2026</v>
       </c>
       <c r="R511">
-        <v>18077187</v>
+        <v>16976374</v>
       </c>
       <c r="S511" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="T511" t="s">
         <v>220</v>
@@ -40268,19 +40268,19 @@
         <v>226</v>
       </c>
       <c r="V511" s="1">
-        <v>46321.36862734954</v>
+        <v>46321.69687025463</v>
       </c>
       <c r="W511">
         <v>-4</v>
       </c>
       <c r="X511" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AB511">
         <v>0</v>
       </c>
       <c r="AC511" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="AH511" t="s">
         <v>450</v>
@@ -40291,22 +40291,22 @@
     </row>
     <row r="512" spans="1:35">
       <c r="A512">
-        <v>6945</v>
+        <v>6703</v>
       </c>
       <c r="B512" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C512" t="s">
         <v>49</v>
       </c>
       <c r="D512" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E512" t="s">
         <v>54</v>
       </c>
       <c r="F512" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G512">
         <v>11542</v>
@@ -40330,10 +40330,10 @@
         <v>2026</v>
       </c>
       <c r="R512">
-        <v>18307831</v>
+        <v>18077187</v>
       </c>
       <c r="S512" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="T512" t="s">
         <v>220</v>
@@ -40342,19 +40342,19 @@
         <v>226</v>
       </c>
       <c r="V512" s="1">
-        <v>46321.66110923611</v>
+        <v>46321.36862734954</v>
       </c>
       <c r="W512">
         <v>-4</v>
       </c>
       <c r="X512" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="AB512">
         <v>0</v>
       </c>
       <c r="AC512" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="AH512" t="s">
         <v>450</v>
@@ -40365,10 +40365,10 @@
     </row>
     <row r="513" spans="1:35">
       <c r="A513">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B513" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C513" t="s">
         <v>49</v>
@@ -40380,10 +40380,10 @@
         <v>54</v>
       </c>
       <c r="F513" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G513">
-        <v>11541</v>
+        <v>11542</v>
       </c>
       <c r="H513">
         <v>0</v>
@@ -40392,7 +40392,7 @@
         <v>59</v>
       </c>
       <c r="J513" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="N513" s="1">
         <v>46325</v>
@@ -40404,31 +40404,31 @@
         <v>2026</v>
       </c>
       <c r="R513">
-        <v>18248553</v>
+        <v>18307831</v>
       </c>
       <c r="S513" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="T513" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="U513" t="s">
         <v>226</v>
       </c>
       <c r="V513" s="1">
-        <v>46321.59424188657</v>
+        <v>46321.66110923611</v>
       </c>
       <c r="W513">
         <v>-4</v>
       </c>
       <c r="X513" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="AB513">
         <v>0</v>
       </c>
       <c r="AC513" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="AH513" t="s">
         <v>450</v>
@@ -40439,10 +40439,10 @@
     </row>
     <row r="514" spans="1:35">
       <c r="A514">
-        <v>6945</v>
+        <v>5417</v>
       </c>
       <c r="B514" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C514" t="s">
         <v>49</v>
@@ -40454,7 +40454,7 @@
         <v>54</v>
       </c>
       <c r="F514" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G514">
         <v>11541</v>
@@ -40478,31 +40478,31 @@
         <v>2026</v>
       </c>
       <c r="R514">
-        <v>18307829</v>
+        <v>18248553</v>
       </c>
       <c r="S514" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="T514" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="U514" t="s">
         <v>226</v>
       </c>
       <c r="V514" s="1">
-        <v>46321.6622389699</v>
+        <v>46321.59424188657</v>
       </c>
       <c r="W514">
         <v>-4</v>
       </c>
       <c r="X514" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="AB514">
         <v>0</v>
       </c>
       <c r="AC514" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="AH514" t="s">
         <v>450</v>
@@ -40513,73 +40513,73 @@
     </row>
     <row r="515" spans="1:35">
       <c r="A515">
-        <v>6962</v>
+        <v>6486</v>
       </c>
       <c r="B515" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C515" t="s">
         <v>49</v>
       </c>
       <c r="D515" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E515" t="s">
         <v>54</v>
       </c>
       <c r="F515" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G515">
-        <v>5984</v>
+        <v>11541</v>
       </c>
       <c r="H515">
-        <v>1884</v>
+        <v>0</v>
       </c>
       <c r="I515" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J515" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="N515" s="1">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="P515">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q515">
         <v>2026</v>
       </c>
       <c r="R515">
-        <v>18260053</v>
+        <v>16976364</v>
       </c>
       <c r="S515" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="T515" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="U515" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V515" s="1">
-        <v>46321.39266284723</v>
+        <v>46321.69699869213</v>
       </c>
       <c r="W515">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="X515" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="AB515">
         <v>0</v>
       </c>
       <c r="AC515" t="s">
-        <v>223</v>
+        <v>200</v>
       </c>
       <c r="AH515" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="AI515" t="s">
         <v>455</v>
@@ -40587,16 +40587,16 @@
     </row>
     <row r="516" spans="1:35">
       <c r="A516">
-        <v>6963</v>
+        <v>6945</v>
       </c>
       <c r="B516" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C516" t="s">
         <v>49</v>
       </c>
       <c r="D516" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E516" t="s">
         <v>54</v>
@@ -40605,55 +40605,55 @@
         <v>56</v>
       </c>
       <c r="G516">
-        <v>5984</v>
+        <v>11541</v>
       </c>
       <c r="H516">
-        <v>1884</v>
+        <v>0</v>
       </c>
       <c r="I516" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J516" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="N516" s="1">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="P516">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q516">
         <v>2026</v>
       </c>
       <c r="R516">
-        <v>18260186</v>
+        <v>18307829</v>
       </c>
       <c r="S516" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="T516" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="U516" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="V516" s="1">
-        <v>46321.39266328704</v>
+        <v>46321.6622389699</v>
       </c>
       <c r="W516">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="X516" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AB516">
         <v>0</v>
       </c>
       <c r="AC516" t="s">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="AH516" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="AI516" t="s">
         <v>455</v>
@@ -40661,16 +40661,16 @@
     </row>
     <row r="517" spans="1:35">
       <c r="A517">
-        <v>5417</v>
+        <v>6962</v>
       </c>
       <c r="B517" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C517" t="s">
         <v>49</v>
       </c>
       <c r="D517" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E517" t="s">
         <v>54</v>
@@ -40679,16 +40679,16 @@
         <v>55</v>
       </c>
       <c r="G517">
-        <v>6759</v>
+        <v>5984</v>
       </c>
       <c r="H517">
-        <v>1788</v>
+        <v>1884</v>
       </c>
       <c r="I517" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J517" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="N517" s="1">
         <v>46321</v>
@@ -40700,31 +40700,31 @@
         <v>2026</v>
       </c>
       <c r="R517">
-        <v>17399191</v>
+        <v>18260053</v>
       </c>
       <c r="S517" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="T517" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="U517" t="s">
         <v>227</v>
       </c>
       <c r="V517" s="1">
-        <v>46321.66995337963</v>
+        <v>46321.39266284723</v>
       </c>
       <c r="W517">
         <v>0</v>
       </c>
       <c r="X517" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="AB517">
         <v>0</v>
       </c>
       <c r="AC517" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="AH517" t="s">
         <v>448</v>
@@ -40735,16 +40735,16 @@
     </row>
     <row r="518" spans="1:35">
       <c r="A518">
-        <v>6705</v>
+        <v>6963</v>
       </c>
       <c r="B518" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C518" t="s">
         <v>49</v>
       </c>
       <c r="D518" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E518" t="s">
         <v>54</v>
@@ -40753,16 +40753,16 @@
         <v>55</v>
       </c>
       <c r="G518">
-        <v>6759</v>
+        <v>5984</v>
       </c>
       <c r="H518">
-        <v>1788</v>
+        <v>1884</v>
       </c>
       <c r="I518" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J518" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="N518" s="1">
         <v>46321</v>
@@ -40774,36 +40774,184 @@
         <v>2026</v>
       </c>
       <c r="R518">
-        <v>17949020</v>
+        <v>18260186</v>
       </c>
       <c r="S518" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="T518" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="U518" t="s">
         <v>227</v>
       </c>
       <c r="V518" s="1">
-        <v>46321.6685106713</v>
+        <v>46321.39266328704</v>
       </c>
       <c r="W518">
         <v>0</v>
       </c>
       <c r="X518" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="AB518">
         <v>0</v>
       </c>
       <c r="AC518" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="AH518" t="s">
         <v>448</v>
       </c>
       <c r="AI518" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="519" spans="1:35">
+      <c r="A519">
+        <v>5417</v>
+      </c>
+      <c r="B519" t="s">
+        <v>43</v>
+      </c>
+      <c r="C519" t="s">
+        <v>49</v>
+      </c>
+      <c r="D519" t="s">
+        <v>50</v>
+      </c>
+      <c r="E519" t="s">
+        <v>54</v>
+      </c>
+      <c r="F519" t="s">
+        <v>55</v>
+      </c>
+      <c r="G519">
+        <v>6759</v>
+      </c>
+      <c r="H519">
+        <v>1788</v>
+      </c>
+      <c r="I519" t="s">
+        <v>61</v>
+      </c>
+      <c r="J519" t="s">
+        <v>160</v>
+      </c>
+      <c r="N519" s="1">
+        <v>46321</v>
+      </c>
+      <c r="P519">
+        <v>9</v>
+      </c>
+      <c r="Q519">
+        <v>2026</v>
+      </c>
+      <c r="R519">
+        <v>17399191</v>
+      </c>
+      <c r="S519" t="s">
+        <v>211</v>
+      </c>
+      <c r="T519" t="s">
+        <v>224</v>
+      </c>
+      <c r="U519" t="s">
+        <v>227</v>
+      </c>
+      <c r="V519" s="1">
+        <v>46321.66995337963</v>
+      </c>
+      <c r="W519">
+        <v>0</v>
+      </c>
+      <c r="X519" t="s">
+        <v>234</v>
+      </c>
+      <c r="AB519">
+        <v>0</v>
+      </c>
+      <c r="AC519" t="s">
+        <v>211</v>
+      </c>
+      <c r="AH519" t="s">
+        <v>448</v>
+      </c>
+      <c r="AI519" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="520" spans="1:35">
+      <c r="A520">
+        <v>6705</v>
+      </c>
+      <c r="B520" t="s">
+        <v>45</v>
+      </c>
+      <c r="C520" t="s">
+        <v>49</v>
+      </c>
+      <c r="D520" t="s">
+        <v>51</v>
+      </c>
+      <c r="E520" t="s">
+        <v>54</v>
+      </c>
+      <c r="F520" t="s">
+        <v>55</v>
+      </c>
+      <c r="G520">
+        <v>6759</v>
+      </c>
+      <c r="H520">
+        <v>1788</v>
+      </c>
+      <c r="I520" t="s">
+        <v>61</v>
+      </c>
+      <c r="J520" t="s">
+        <v>160</v>
+      </c>
+      <c r="N520" s="1">
+        <v>46321</v>
+      </c>
+      <c r="P520">
+        <v>9</v>
+      </c>
+      <c r="Q520">
+        <v>2026</v>
+      </c>
+      <c r="R520">
+        <v>17949020</v>
+      </c>
+      <c r="S520" t="s">
+        <v>211</v>
+      </c>
+      <c r="T520" t="s">
+        <v>224</v>
+      </c>
+      <c r="U520" t="s">
+        <v>227</v>
+      </c>
+      <c r="V520" s="1">
+        <v>46321.6685106713</v>
+      </c>
+      <c r="W520">
+        <v>0</v>
+      </c>
+      <c r="X520" t="s">
+        <v>235</v>
+      </c>
+      <c r="AB520">
+        <v>0</v>
+      </c>
+      <c r="AC520" t="s">
+        <v>211</v>
+      </c>
+      <c r="AH520" t="s">
+        <v>448</v>
+      </c>
+      <c r="AI520" t="s">
         <v>455</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-27 09:05
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -1933,7 +1933,7 @@
         <v>46300.43100663194</v>
       </c>
       <c r="W2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X2" t="s">
         <v>228</v>
@@ -2010,7 +2010,7 @@
         <v>46300.3901340625</v>
       </c>
       <c r="W3">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X3" t="s">
         <v>228</v>
@@ -2087,7 +2087,7 @@
         <v>46297.71198460648</v>
       </c>
       <c r="W4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X4" t="s">
         <v>229</v>
@@ -2161,7 +2161,7 @@
         <v>46297.7119869213</v>
       </c>
       <c r="W5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X5" t="s">
         <v>228</v>
@@ -2235,7 +2235,7 @@
         <v>46297.71198738426</v>
       </c>
       <c r="W6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X6" t="s">
         <v>228</v>
@@ -2309,7 +2309,7 @@
         <v>46297.71199320602</v>
       </c>
       <c r="W7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X7" t="s">
         <v>230</v>
@@ -2383,7 +2383,7 @@
         <v>46297.71199371527</v>
       </c>
       <c r="W8">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X8" t="s">
         <v>231</v>
@@ -2457,7 +2457,7 @@
         <v>46297.71199424769</v>
       </c>
       <c r="W9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X9" t="s">
         <v>232</v>
@@ -2531,7 +2531,7 @@
         <v>46297.71199479167</v>
       </c>
       <c r="W10">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X10" t="s">
         <v>232</v>
@@ -2605,7 +2605,7 @@
         <v>46302.37134707176</v>
       </c>
       <c r="W11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X11" t="s">
         <v>233</v>
@@ -2679,7 +2679,7 @@
         <v>46297.69881809028</v>
       </c>
       <c r="W12">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X12" t="s">
         <v>233</v>
@@ -2756,7 +2756,7 @@
         <v>46300.38749403935</v>
       </c>
       <c r="W13">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X13" t="s">
         <v>233</v>
@@ -2830,7 +2830,7 @@
         <v>46302.3710765625</v>
       </c>
       <c r="W14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X14" t="s">
         <v>233</v>
@@ -2904,7 +2904,7 @@
         <v>46297.71197056713</v>
       </c>
       <c r="W15">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X15" t="s">
         <v>234</v>
@@ -2978,7 +2978,7 @@
         <v>46297.71198896991</v>
       </c>
       <c r="W16">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X16" t="s">
         <v>235</v>
@@ -3052,7 +3052,7 @@
         <v>46297.71198950231</v>
       </c>
       <c r="W17">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X17" t="s">
         <v>235</v>
@@ -3126,7 +3126,7 @@
         <v>46297.71199112268</v>
       </c>
       <c r="W18">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X18" t="s">
         <v>235</v>
@@ -3197,7 +3197,7 @@
         <v>46297.68986506944</v>
       </c>
       <c r="W19">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X19" t="s">
         <v>236</v>
@@ -3271,7 +3271,7 @@
         <v>46297.68986576389</v>
       </c>
       <c r="W20">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X20" t="s">
         <v>228</v>
@@ -3348,7 +3348,7 @@
         <v>46300.68237630787</v>
       </c>
       <c r="W21">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X21" t="s">
         <v>237</v>
@@ -3425,7 +3425,7 @@
         <v>46300.57769349537</v>
       </c>
       <c r="W22">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X22" t="s">
         <v>228</v>
@@ -3505,7 +3505,7 @@
         <v>46300.56213424769</v>
       </c>
       <c r="W23">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X23" t="s">
         <v>230</v>
@@ -3585,7 +3585,7 @@
         <v>46301.46998128472</v>
       </c>
       <c r="W24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X24" t="s">
         <v>231</v>
@@ -3662,7 +3662,7 @@
         <v>46303.69944310185</v>
       </c>
       <c r="W25">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X25" t="s">
         <v>234</v>
@@ -3736,7 +3736,7 @@
         <v>46300.75766230324</v>
       </c>
       <c r="W26">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X26" t="s">
         <v>233</v>
@@ -3813,7 +3813,7 @@
         <v>46300.7473044213</v>
       </c>
       <c r="W27">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X27" t="s">
         <v>236</v>
@@ -3893,7 +3893,7 @@
         <v>46302.56370974537</v>
       </c>
       <c r="W28">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X28" t="s">
         <v>228</v>
@@ -3970,7 +3970,7 @@
         <v>46301.75716237268</v>
       </c>
       <c r="W29">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X29" t="s">
         <v>230</v>
@@ -4044,7 +4044,7 @@
         <v>46303.39799296296</v>
       </c>
       <c r="W30">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X30" t="s">
         <v>231</v>
@@ -4121,7 +4121,7 @@
         <v>46300.4280221412</v>
       </c>
       <c r="W31">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X31" t="s">
         <v>234</v>
@@ -4201,7 +4201,7 @@
         <v>46300.57060454861</v>
       </c>
       <c r="W32">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X32" t="s">
         <v>236</v>
@@ -4281,7 +4281,7 @@
         <v>46301.60203489583</v>
       </c>
       <c r="W33">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X33" t="s">
         <v>228</v>
@@ -4361,7 +4361,7 @@
         <v>46301.60118045139</v>
       </c>
       <c r="W34">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X34" t="s">
         <v>228</v>
@@ -4441,7 +4441,7 @@
         <v>46300.67849611111</v>
       </c>
       <c r="W35">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X35" t="s">
         <v>237</v>
@@ -4521,7 +4521,7 @@
         <v>46296.64258336806</v>
       </c>
       <c r="W36">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X36" t="s">
         <v>235</v>
@@ -4601,7 +4601,7 @@
         <v>46300.44301378472</v>
       </c>
       <c r="W37">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X37" t="s">
         <v>230</v>
@@ -4681,7 +4681,7 @@
         <v>46301.46967876158</v>
       </c>
       <c r="W38">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X38" t="s">
         <v>231</v>
@@ -4761,7 +4761,7 @@
         <v>46302.40341663195</v>
       </c>
       <c r="W39">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X39" t="s">
         <v>234</v>
@@ -4841,7 +4841,7 @@
         <v>46300.57039657408</v>
       </c>
       <c r="W40">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X40" t="s">
         <v>236</v>
@@ -4921,7 +4921,7 @@
         <v>46301.60196542824</v>
       </c>
       <c r="W41">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X41" t="s">
         <v>228</v>
@@ -5001,7 +5001,7 @@
         <v>46301.60178498842</v>
       </c>
       <c r="W42">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X42" t="s">
         <v>228</v>
@@ -5078,7 +5078,7 @@
         <v>46300.67840927083</v>
       </c>
       <c r="W43">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X43" t="s">
         <v>237</v>
@@ -5152,7 +5152,7 @@
         <v>46296.64250469908</v>
       </c>
       <c r="W44">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X44" t="s">
         <v>235</v>
@@ -5226,7 +5226,7 @@
         <v>46300.44324319444</v>
       </c>
       <c r="W45">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X45" t="s">
         <v>230</v>
@@ -5300,7 +5300,7 @@
         <v>46301.46964587963</v>
       </c>
       <c r="W46">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X46" t="s">
         <v>231</v>
@@ -5374,7 +5374,7 @@
         <v>46296.01593988426</v>
       </c>
       <c r="W47">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X47" t="s">
         <v>233</v>
@@ -5448,7 +5448,7 @@
         <v>46303.69171724537</v>
       </c>
       <c r="W48">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X48" t="s">
         <v>235</v>
@@ -5525,7 +5525,7 @@
         <v>46303.69195155093</v>
       </c>
       <c r="W49">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X49" t="s">
         <v>235</v>
@@ -5605,7 +5605,7 @@
         <v>46300.3863081713</v>
       </c>
       <c r="W50">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X50" t="s">
         <v>236</v>
@@ -5685,7 +5685,7 @@
         <v>46300.38630890047</v>
       </c>
       <c r="W51">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X51" t="s">
         <v>228</v>
@@ -5765,7 +5765,7 @@
         <v>46300.38631003472</v>
       </c>
       <c r="W52">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X52" t="s">
         <v>228</v>
@@ -5845,7 +5845,7 @@
         <v>46300.67853358796</v>
       </c>
       <c r="W53">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X53" t="s">
         <v>237</v>
@@ -5925,7 +5925,7 @@
         <v>46297.71954039352</v>
       </c>
       <c r="W54">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X54" t="s">
         <v>234</v>
@@ -6005,7 +6005,7 @@
         <v>46296.48787840278</v>
       </c>
       <c r="W55">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X55" t="s">
         <v>235</v>
@@ -6085,7 +6085,7 @@
         <v>46300.42827539352</v>
       </c>
       <c r="W56">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X56" t="s">
         <v>234</v>
@@ -6165,7 +6165,7 @@
         <v>46300.57064887731</v>
       </c>
       <c r="W57">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X57" t="s">
         <v>236</v>
@@ -6245,7 +6245,7 @@
         <v>46301.60206459491</v>
       </c>
       <c r="W58">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X58" t="s">
         <v>228</v>
@@ -6325,7 +6325,7 @@
         <v>46301.60121219907</v>
       </c>
       <c r="W59">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X59" t="s">
         <v>228</v>
@@ -6402,7 +6402,7 @@
         <v>46300.67857046297</v>
       </c>
       <c r="W60">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X60" t="s">
         <v>237</v>
@@ -6479,7 +6479,7 @@
         <v>46296.64261186343</v>
       </c>
       <c r="W61">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X61" t="s">
         <v>235</v>
@@ -6559,7 +6559,7 @@
         <v>46300.44350421296</v>
       </c>
       <c r="W62">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X62" t="s">
         <v>230</v>
@@ -6639,7 +6639,7 @@
         <v>46301.46971603009</v>
       </c>
       <c r="W63">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X63" t="s">
         <v>231</v>
@@ -6719,7 +6719,7 @@
         <v>46300.57801363426</v>
       </c>
       <c r="W64">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X64" t="s">
         <v>236</v>
@@ -6799,7 +6799,7 @@
         <v>46300.42855335648</v>
       </c>
       <c r="W65">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X65" t="s">
         <v>234</v>
@@ -6879,7 +6879,7 @@
         <v>46300.57068319445</v>
       </c>
       <c r="W66">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X66" t="s">
         <v>236</v>
@@ -6959,7 +6959,7 @@
         <v>46301.60209734954</v>
       </c>
       <c r="W67">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X67" t="s">
         <v>228</v>
@@ -7039,7 +7039,7 @@
         <v>46301.60124362269</v>
       </c>
       <c r="W68">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X68" t="s">
         <v>228</v>
@@ -7116,7 +7116,7 @@
         <v>46300.67860491898</v>
       </c>
       <c r="W69">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X69" t="s">
         <v>237</v>
@@ -7193,7 +7193,7 @@
         <v>46296.64263715278</v>
       </c>
       <c r="W70">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X70" t="s">
         <v>235</v>
@@ -7273,7 +7273,7 @@
         <v>46300.44361263889</v>
       </c>
       <c r="W71">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X71" t="s">
         <v>230</v>
@@ -7353,7 +7353,7 @@
         <v>46301.46975131945</v>
       </c>
       <c r="W72">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X72" t="s">
         <v>231</v>
@@ -7427,7 +7427,7 @@
         <v>46296.71263638889</v>
       </c>
       <c r="W73">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="X73" t="s">
         <v>228</v>
@@ -7507,7 +7507,7 @@
         <v>46303.73557287037</v>
       </c>
       <c r="W74">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X74" t="s">
         <v>231</v>
@@ -7587,7 +7587,7 @@
         <v>46302.74648497685</v>
       </c>
       <c r="W75">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X75" t="s">
         <v>231</v>
@@ -7664,7 +7664,7 @@
         <v>46296.37884409722</v>
       </c>
       <c r="W76">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X76" t="s">
         <v>229</v>
@@ -7738,7 +7738,7 @@
         <v>46296.37884371528</v>
       </c>
       <c r="W77">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X77" t="s">
         <v>228</v>
@@ -7812,7 +7812,7 @@
         <v>46296.46064649305</v>
       </c>
       <c r="W78">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X78" t="s">
         <v>231</v>
@@ -7886,7 +7886,7 @@
         <v>46296.3788346875</v>
       </c>
       <c r="W79">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X79" t="s">
         <v>229</v>
@@ -7960,7 +7960,7 @@
         <v>46296.37883295139</v>
       </c>
       <c r="W80">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X80" t="s">
         <v>228</v>
@@ -8034,7 +8034,7 @@
         <v>46296.37860081019</v>
       </c>
       <c r="W81">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X81" t="s">
         <v>229</v>
@@ -8108,7 +8108,7 @@
         <v>46296.37859760417</v>
       </c>
       <c r="W82">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X82" t="s">
         <v>228</v>
@@ -8182,7 +8182,7 @@
         <v>46296.79357893518</v>
       </c>
       <c r="W83">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X83" t="s">
         <v>228</v>
@@ -8256,7 +8256,7 @@
         <v>46296.37868082176</v>
       </c>
       <c r="W84">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X84" t="s">
         <v>229</v>
@@ -8330,7 +8330,7 @@
         <v>46296.37867766204</v>
       </c>
       <c r="W85">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X85" t="s">
         <v>228</v>
@@ -8404,7 +8404,7 @@
         <v>46296.7936246875</v>
       </c>
       <c r="W86">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X86" t="s">
         <v>228</v>
@@ -8478,7 +8478,7 @@
         <v>46296.37638978009</v>
       </c>
       <c r="W87">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X87" t="s">
         <v>229</v>
@@ -8552,7 +8552,7 @@
         <v>46296.37638726852</v>
       </c>
       <c r="W88">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X88" t="s">
         <v>228</v>
@@ -8626,7 +8626,7 @@
         <v>46296.45920883102</v>
       </c>
       <c r="W89">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X89" t="s">
         <v>231</v>
@@ -8700,7 +8700,7 @@
         <v>46300.37640358796</v>
       </c>
       <c r="W90">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X90" t="s">
         <v>232</v>
@@ -8774,7 +8774,7 @@
         <v>46296.37883935186</v>
       </c>
       <c r="W91">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X91" t="s">
         <v>230</v>
@@ -8848,7 +8848,7 @@
         <v>46296.37873302084</v>
       </c>
       <c r="W92">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X92" t="s">
         <v>229</v>
@@ -8922,7 +8922,7 @@
         <v>46296.37872700232</v>
       </c>
       <c r="W93">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X93" t="s">
         <v>228</v>
@@ -8996,7 +8996,7 @@
         <v>46296.79365752315</v>
       </c>
       <c r="W94">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X94" t="s">
         <v>228</v>
@@ -9070,7 +9070,7 @@
         <v>46297.71059528935</v>
       </c>
       <c r="W95">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X95" t="s">
         <v>232</v>
@@ -9144,7 +9144,7 @@
         <v>46296.37648703704</v>
       </c>
       <c r="W96">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X96" t="s">
         <v>229</v>
@@ -9218,7 +9218,7 @@
         <v>46296.37648807871</v>
       </c>
       <c r="W97">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X97" t="s">
         <v>230</v>
@@ -9292,7 +9292,7 @@
         <v>46296.45925008102</v>
       </c>
       <c r="W98">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X98" t="s">
         <v>231</v>
@@ -9366,7 +9366,7 @@
         <v>46296.37619637731</v>
       </c>
       <c r="W99">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X99" t="s">
         <v>230</v>
@@ -9440,7 +9440,7 @@
         <v>46296.45913734954</v>
       </c>
       <c r="W100">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X100" t="s">
         <v>231</v>
@@ -9514,7 +9514,7 @@
         <v>46296.37620748843</v>
       </c>
       <c r="W101">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X101" t="s">
         <v>229</v>
@@ -9588,7 +9588,7 @@
         <v>46296.37620686342</v>
       </c>
       <c r="W102">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X102" t="s">
         <v>230</v>
@@ -9662,7 +9662,7 @@
         <v>46296.45914429398</v>
       </c>
       <c r="W103">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X103" t="s">
         <v>231</v>
@@ -9736,7 +9736,7 @@
         <v>46296.37877858796</v>
       </c>
       <c r="W104">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X104" t="s">
         <v>229</v>
@@ -9810,7 +9810,7 @@
         <v>46296.37877496528</v>
       </c>
       <c r="W105">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X105" t="s">
         <v>228</v>
@@ -9884,7 +9884,7 @@
         <v>46296.79368927083</v>
       </c>
       <c r="W106">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X106" t="s">
         <v>228</v>
@@ -9958,7 +9958,7 @@
         <v>46296.37881099537</v>
       </c>
       <c r="W107">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X107" t="s">
         <v>229</v>
@@ -10032,7 +10032,7 @@
         <v>46296.37880798611</v>
       </c>
       <c r="W108">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X108" t="s">
         <v>228</v>
@@ -10106,7 +10106,7 @@
         <v>46296.79371550926</v>
       </c>
       <c r="W109">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X109" t="s">
         <v>228</v>
@@ -10180,7 +10180,7 @@
         <v>46303.6633371875</v>
       </c>
       <c r="W110">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X110" t="s">
         <v>228</v>
@@ -10257,7 +10257,7 @@
         <v>46301.53076038195</v>
       </c>
       <c r="W111">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X111" t="s">
         <v>228</v>
@@ -10334,7 +10334,7 @@
         <v>46301.77168440972</v>
       </c>
       <c r="W112">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X112" t="s">
         <v>231</v>
@@ -10411,7 +10411,7 @@
         <v>46302.45135077546</v>
       </c>
       <c r="W113">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X113" t="s">
         <v>232</v>
@@ -10491,7 +10491,7 @@
         <v>46303.37146987268</v>
       </c>
       <c r="W114">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X114" t="s">
         <v>229</v>
@@ -10568,7 +10568,7 @@
         <v>46301.53482881944</v>
       </c>
       <c r="W115">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X115" t="s">
         <v>228</v>
@@ -10648,7 +10648,7 @@
         <v>46301.61803621528</v>
       </c>
       <c r="W116">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X116" t="s">
         <v>230</v>
@@ -10725,7 +10725,7 @@
         <v>46301.68910333333</v>
       </c>
       <c r="W117">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X117" t="s">
         <v>231</v>
@@ -10802,7 +10802,7 @@
         <v>46302.40335295139</v>
       </c>
       <c r="W118">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X118" t="s">
         <v>232</v>
@@ -10879,7 +10879,7 @@
         <v>46297.37673402778</v>
       </c>
       <c r="W119">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X119" t="s">
         <v>234</v>
@@ -10953,7 +10953,7 @@
         <v>46297.37618915509</v>
       </c>
       <c r="W120">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X120" t="s">
         <v>234</v>
@@ -11027,7 +11027,7 @@
         <v>46297.66736068287</v>
       </c>
       <c r="W121">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X121" t="s">
         <v>236</v>
@@ -11101,7 +11101,7 @@
         <v>46297.45935385417</v>
       </c>
       <c r="W122">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X122" t="s">
         <v>235</v>
@@ -11175,7 +11175,7 @@
         <v>46297.37681010416</v>
       </c>
       <c r="W123">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X123" t="s">
         <v>234</v>
@@ -11249,7 +11249,7 @@
         <v>46297.37686377315</v>
       </c>
       <c r="W124">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X124" t="s">
         <v>234</v>
@@ -11323,7 +11323,7 @@
         <v>46297.37606362269</v>
       </c>
       <c r="W125">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X125" t="s">
         <v>234</v>
@@ -11397,7 +11397,7 @@
         <v>46297.66734447917</v>
       </c>
       <c r="W126">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X126" t="s">
         <v>236</v>
@@ -11471,7 +11471,7 @@
         <v>46297.45929016203</v>
       </c>
       <c r="W127">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X127" t="s">
         <v>235</v>
@@ -11545,7 +11545,7 @@
         <v>46297.37537966435</v>
       </c>
       <c r="W128">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X128" t="s">
         <v>234</v>
@@ -11619,7 +11619,7 @@
         <v>46297.45869950231</v>
       </c>
       <c r="W129">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X129" t="s">
         <v>233</v>
@@ -11693,7 +11693,7 @@
         <v>46300.66721489583</v>
       </c>
       <c r="W130">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X130" t="s">
         <v>236</v>
@@ -11767,7 +11767,7 @@
         <v>46297.45870309028</v>
       </c>
       <c r="W131">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X131" t="s">
         <v>237</v>
@@ -11841,7 +11841,7 @@
         <v>46297.45870405093</v>
       </c>
       <c r="W132">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X132" t="s">
         <v>235</v>
@@ -11915,7 +11915,7 @@
         <v>46297.45870177083</v>
       </c>
       <c r="W133">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X133" t="s">
         <v>235</v>
@@ -11989,7 +11989,7 @@
         <v>46300.65013206018</v>
       </c>
       <c r="W134">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X134" t="s">
         <v>234</v>
@@ -12063,7 +12063,7 @@
         <v>46300.65011049769</v>
       </c>
       <c r="W135">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X135" t="s">
         <v>233</v>
@@ -12137,7 +12137,7 @@
         <v>46300.66713765046</v>
       </c>
       <c r="W136">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X136" t="s">
         <v>236</v>
@@ -12211,7 +12211,7 @@
         <v>46300.66713784722</v>
       </c>
       <c r="W137">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X137" t="s">
         <v>237</v>
@@ -12285,7 +12285,7 @@
         <v>46300.66713822917</v>
       </c>
       <c r="W138">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X138" t="s">
         <v>235</v>
@@ -12359,7 +12359,7 @@
         <v>46300.75530894676</v>
       </c>
       <c r="W139">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X139" t="s">
         <v>235</v>
@@ -12433,7 +12433,7 @@
         <v>46303.68045927084</v>
       </c>
       <c r="W140">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X140" t="s">
         <v>233</v>
@@ -12507,7 +12507,7 @@
         <v>46297.66734765047</v>
       </c>
       <c r="W141">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X141" t="s">
         <v>236</v>
@@ -12584,7 +12584,7 @@
         <v>46303.79348310185</v>
       </c>
       <c r="W142">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X142" t="s">
         <v>236</v>
@@ -12664,7 +12664,7 @@
         <v>46303.79351134259</v>
       </c>
       <c r="W143">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X143" t="s">
         <v>235</v>
@@ -12741,7 +12741,7 @@
         <v>46301.70844945602</v>
       </c>
       <c r="W144">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X144" t="s">
         <v>234</v>
@@ -12815,7 +12815,7 @@
         <v>46301.70847283565</v>
       </c>
       <c r="W145">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X145" t="s">
         <v>235</v>
@@ -12886,7 +12886,7 @@
         <v>46296.37648518519</v>
       </c>
       <c r="W146">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X146" t="s">
         <v>234</v>
@@ -12960,7 +12960,7 @@
         <v>46296.37615983796</v>
       </c>
       <c r="W147">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X147" t="s">
         <v>228</v>
@@ -13034,7 +13034,7 @@
         <v>46296.37684290509</v>
       </c>
       <c r="W148">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X148" t="s">
         <v>235</v>
@@ -13108,7 +13108,7 @@
         <v>46296.37609667824</v>
       </c>
       <c r="W149">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X149" t="s">
         <v>233</v>
@@ -13182,7 +13182,7 @@
         <v>46296.37683961805</v>
       </c>
       <c r="W150">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X150" t="s">
         <v>237</v>
@@ -13256,7 +13256,7 @@
         <v>46297.67728344908</v>
       </c>
       <c r="W151">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X151" t="s">
         <v>234</v>
@@ -13327,7 +13327,7 @@
         <v>46297.67730740741</v>
       </c>
       <c r="W152">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X152" t="s">
         <v>233</v>
@@ -13398,7 +13398,7 @@
         <v>46297.67730972222</v>
       </c>
       <c r="W153">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X153" t="s">
         <v>236</v>
@@ -13469,7 +13469,7 @@
         <v>46297.67731253472</v>
       </c>
       <c r="W154">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X154" t="s">
         <v>229</v>
@@ -13540,7 +13540,7 @@
         <v>46297.67731608796</v>
       </c>
       <c r="W155">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X155" t="s">
         <v>228</v>
@@ -13611,7 +13611,7 @@
         <v>46297.6773164699</v>
       </c>
       <c r="W156">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X156" t="s">
         <v>228</v>
@@ -13682,7 +13682,7 @@
         <v>46297.67732225695</v>
       </c>
       <c r="W157">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X157" t="s">
         <v>237</v>
@@ -13753,7 +13753,7 @@
         <v>46297.67732283565</v>
       </c>
       <c r="W158">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X158" t="s">
         <v>235</v>
@@ -13824,7 +13824,7 @@
         <v>46297.67732337963</v>
       </c>
       <c r="W159">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X159" t="s">
         <v>235</v>
@@ -13895,7 +13895,7 @@
         <v>46297.6773253125</v>
       </c>
       <c r="W160">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X160" t="s">
         <v>235</v>
@@ -13966,7 +13966,7 @@
         <v>46297.67733796296</v>
       </c>
       <c r="W161">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X161" t="s">
         <v>230</v>
@@ -14037,7 +14037,7 @@
         <v>46297.67733896991</v>
       </c>
       <c r="W162">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X162" t="s">
         <v>231</v>
@@ -14108,7 +14108,7 @@
         <v>46297.67734047454</v>
       </c>
       <c r="W163">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X163" t="s">
         <v>232</v>
@@ -14179,7 +14179,7 @@
         <v>46297.67734097222</v>
       </c>
       <c r="W164">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X164" t="s">
         <v>232</v>
@@ -14253,7 +14253,7 @@
         <v>46300.67560568287</v>
       </c>
       <c r="W165">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X165" t="s">
         <v>234</v>
@@ -14330,7 +14330,7 @@
         <v>46300.67612549769</v>
       </c>
       <c r="W166">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X166" t="s">
         <v>233</v>
@@ -14407,7 +14407,7 @@
         <v>46300.67620415509</v>
       </c>
       <c r="W167">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X167" t="s">
         <v>236</v>
@@ -14484,7 +14484,7 @@
         <v>46300.67631252314</v>
       </c>
       <c r="W168">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X168" t="s">
         <v>229</v>
@@ -14561,7 +14561,7 @@
         <v>46300.6765974537</v>
       </c>
       <c r="W169">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X169" t="s">
         <v>228</v>
@@ -14638,7 +14638,7 @@
         <v>46300.67662010417</v>
       </c>
       <c r="W170">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X170" t="s">
         <v>228</v>
@@ -14715,7 +14715,7 @@
         <v>46300.67678489583</v>
       </c>
       <c r="W171">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X171" t="s">
         <v>237</v>
@@ -14792,7 +14792,7 @@
         <v>46301.34827806713</v>
       </c>
       <c r="W172">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X172" t="s">
         <v>235</v>
@@ -14869,7 +14869,7 @@
         <v>46300.67680096065</v>
       </c>
       <c r="W173">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X173" t="s">
         <v>235</v>
@@ -14946,7 +14946,7 @@
         <v>46300.6769524537</v>
       </c>
       <c r="W174">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X174" t="s">
         <v>230</v>
@@ -15023,7 +15023,7 @@
         <v>46300.67696659722</v>
       </c>
       <c r="W175">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X175" t="s">
         <v>231</v>
@@ -15097,7 +15097,7 @@
         <v>46297.34991217592</v>
       </c>
       <c r="W176">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X176" t="s">
         <v>234</v>
@@ -15168,7 +15168,7 @@
         <v>46297.3499325</v>
       </c>
       <c r="W177">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X177" t="s">
         <v>233</v>
@@ -15239,7 +15239,7 @@
         <v>46297.34994254629</v>
       </c>
       <c r="W178">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X178" t="s">
         <v>236</v>
@@ -15310,7 +15310,7 @@
         <v>46297.34994771991</v>
       </c>
       <c r="W179">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X179" t="s">
         <v>228</v>
@@ -15381,7 +15381,7 @@
         <v>46297.34994974537</v>
       </c>
       <c r="W180">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X180" t="s">
         <v>235</v>
@@ -15452,7 +15452,7 @@
         <v>46297.34995063658</v>
       </c>
       <c r="W181">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X181" t="s">
         <v>235</v>
@@ -15523,7 +15523,7 @@
         <v>46297.34996266204</v>
       </c>
       <c r="W182">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X182" t="s">
         <v>230</v>
@@ -15594,7 +15594,7 @@
         <v>46297.68732318287</v>
       </c>
       <c r="W183">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X183" t="s">
         <v>234</v>
@@ -15665,7 +15665,7 @@
         <v>46297.68735216435</v>
       </c>
       <c r="W184">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X184" t="s">
         <v>233</v>
@@ -15736,7 +15736,7 @@
         <v>46297.68735517361</v>
       </c>
       <c r="W185">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X185" t="s">
         <v>236</v>
@@ -15807,7 +15807,7 @@
         <v>46297.68735752315</v>
       </c>
       <c r="W186">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X186" t="s">
         <v>229</v>
@@ -15878,7 +15878,7 @@
         <v>46297.68736119213</v>
       </c>
       <c r="W187">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X187" t="s">
         <v>228</v>
@@ -15949,7 +15949,7 @@
         <v>46297.68736145833</v>
       </c>
       <c r="W188">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X188" t="s">
         <v>228</v>
@@ -16020,7 +16020,7 @@
         <v>46297.68736666667</v>
       </c>
       <c r="W189">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X189" t="s">
         <v>237</v>
@@ -16091,7 +16091,7 @@
         <v>46297.68736686343</v>
       </c>
       <c r="W190">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X190" t="s">
         <v>235</v>
@@ -16162,7 +16162,7 @@
         <v>46297.68736712963</v>
       </c>
       <c r="W191">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X191" t="s">
         <v>235</v>
@@ -16233,7 +16233,7 @@
         <v>46297.68736878473</v>
       </c>
       <c r="W192">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X192" t="s">
         <v>235</v>
@@ -16304,7 +16304,7 @@
         <v>46297.6873764699</v>
       </c>
       <c r="W193">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X193" t="s">
         <v>230</v>
@@ -16375,7 +16375,7 @@
         <v>46297.68737700232</v>
       </c>
       <c r="W194">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X194" t="s">
         <v>231</v>
@@ -16446,7 +16446,7 @@
         <v>46297.68737777778</v>
       </c>
       <c r="W195">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X195" t="s">
         <v>232</v>
@@ -16517,7 +16517,7 @@
         <v>46297.68737800926</v>
       </c>
       <c r="W196">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X196" t="s">
         <v>232</v>
@@ -16588,7 +16588,7 @@
         <v>46300.67560523148</v>
       </c>
       <c r="W197">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X197" t="s">
         <v>234</v>
@@ -16659,7 +16659,7 @@
         <v>46300.67612488426</v>
       </c>
       <c r="W198">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X198" t="s">
         <v>233</v>
@@ -16730,7 +16730,7 @@
         <v>46300.67620471065</v>
       </c>
       <c r="W199">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X199" t="s">
         <v>236</v>
@@ -16801,7 +16801,7 @@
         <v>46300.67631207176</v>
       </c>
       <c r="W200">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X200" t="s">
         <v>229</v>
@@ -16872,7 +16872,7 @@
         <v>46300.67659613426</v>
       </c>
       <c r="W201">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X201" t="s">
         <v>228</v>
@@ -16943,7 +16943,7 @@
         <v>46300.67661899306</v>
       </c>
       <c r="W202">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X202" t="s">
         <v>228</v>
@@ -17014,7 +17014,7 @@
         <v>46300.67678520834</v>
       </c>
       <c r="W203">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X203" t="s">
         <v>237</v>
@@ -17088,7 +17088,7 @@
         <v>46302.51963612268</v>
       </c>
       <c r="W204">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X204" t="s">
         <v>235</v>
@@ -17162,7 +17162,7 @@
         <v>46300.6768006713</v>
       </c>
       <c r="W205">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X205" t="s">
         <v>235</v>
@@ -17233,7 +17233,7 @@
         <v>46300.6769528125</v>
       </c>
       <c r="W206">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X206" t="s">
         <v>230</v>
@@ -17304,7 +17304,7 @@
         <v>46300.67696615741</v>
       </c>
       <c r="W207">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X207" t="s">
         <v>231</v>
@@ -17375,7 +17375,7 @@
         <v>46296.34114513889</v>
       </c>
       <c r="W208">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="X208" t="s">
         <v>233</v>
@@ -17449,7 +17449,7 @@
         <v>46296.34050315972</v>
       </c>
       <c r="W209">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="X209" t="s">
         <v>234</v>
@@ -17523,7 +17523,7 @@
         <v>46296.39309459491</v>
       </c>
       <c r="W210">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="X210" t="s">
         <v>236</v>
@@ -17597,7 +17597,7 @@
         <v>46296.3409153125</v>
       </c>
       <c r="W211">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="X211" t="s">
         <v>236</v>
@@ -17671,7 +17671,7 @@
         <v>46296.0420403125</v>
       </c>
       <c r="W212">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="X212" t="s">
         <v>234</v>
@@ -17742,7 +17742,7 @@
         <v>46296.0420403125</v>
       </c>
       <c r="W213">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="X213" t="s">
         <v>233</v>
@@ -17813,7 +17813,7 @@
         <v>46301.49091145834</v>
       </c>
       <c r="W214">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="X214" t="s">
         <v>233</v>
@@ -17887,7 +17887,7 @@
         <v>46297.49393364583</v>
       </c>
       <c r="W215">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X215" t="s">
         <v>231</v>
@@ -17964,7 +17964,7 @@
         <v>46311.61321276621</v>
       </c>
       <c r="W216">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X216" t="s">
         <v>229</v>
@@ -18038,7 +18038,7 @@
         <v>46308.43011417824</v>
       </c>
       <c r="W217">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X217" t="s">
         <v>234</v>
@@ -18112,7 +18112,7 @@
         <v>46304.6292707176</v>
       </c>
       <c r="W218">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X218" t="s">
         <v>236</v>
@@ -18186,7 +18186,7 @@
         <v>46311.57832534723</v>
       </c>
       <c r="W219">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X219" t="s">
         <v>234</v>
@@ -18263,7 +18263,7 @@
         <v>46309.72495443287</v>
       </c>
       <c r="W220">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X220" t="s">
         <v>234</v>
@@ -18337,7 +18337,7 @@
         <v>46311.37595946759</v>
       </c>
       <c r="W221">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X221" t="s">
         <v>235</v>
@@ -18411,7 +18411,7 @@
         <v>46311.37596002315</v>
       </c>
       <c r="W222">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X222" t="s">
         <v>235</v>
@@ -18485,7 +18485,7 @@
         <v>46311.37596055555</v>
       </c>
       <c r="W223">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X223" t="s">
         <v>235</v>
@@ -18559,7 +18559,7 @@
         <v>46311.64911328704</v>
       </c>
       <c r="W224">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X224" t="s">
         <v>228</v>
@@ -18633,7 +18633,7 @@
         <v>46311.64885200231</v>
       </c>
       <c r="W225">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X225" t="s">
         <v>228</v>
@@ -18710,7 +18710,7 @@
         <v>46310.64891221065</v>
       </c>
       <c r="W226">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X226" t="s">
         <v>230</v>
@@ -18787,7 +18787,7 @@
         <v>46310.65490846064</v>
       </c>
       <c r="W227">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X227" t="s">
         <v>229</v>
@@ -18861,7 +18861,7 @@
         <v>46310.65010393519</v>
       </c>
       <c r="W228">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X228" t="s">
         <v>230</v>
@@ -18935,7 +18935,7 @@
         <v>46310.65496277778</v>
       </c>
       <c r="W229">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X229" t="s">
         <v>229</v>
@@ -19009,7 +19009,7 @@
         <v>46310.65023333333</v>
       </c>
       <c r="W230">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X230" t="s">
         <v>230</v>
@@ -19083,7 +19083,7 @@
         <v>46310.40488353009</v>
       </c>
       <c r="W231">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X231" t="s">
         <v>234</v>
@@ -19160,7 +19160,7 @@
         <v>46310.59350474537</v>
       </c>
       <c r="W232">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X232" t="s">
         <v>233</v>
@@ -19237,7 +19237,7 @@
         <v>46309.73508298611</v>
       </c>
       <c r="W233">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X233" t="s">
         <v>236</v>
@@ -19314,7 +19314,7 @@
         <v>46310.58456605324</v>
       </c>
       <c r="W234">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X234" t="s">
         <v>229</v>
@@ -19391,7 +19391,7 @@
         <v>46309.73508329861</v>
       </c>
       <c r="W235">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X235" t="s">
         <v>228</v>
@@ -19468,7 +19468,7 @@
         <v>46309.73508391203</v>
       </c>
       <c r="W236">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X236" t="s">
         <v>228</v>
@@ -19545,7 +19545,7 @@
         <v>46310.66711284722</v>
       </c>
       <c r="W237">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X237" t="s">
         <v>237</v>
@@ -19625,7 +19625,7 @@
         <v>46311.45926010417</v>
       </c>
       <c r="W238">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X238" t="s">
         <v>235</v>
@@ -19702,7 +19702,7 @@
         <v>46310.58457245371</v>
       </c>
       <c r="W239">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X239" t="s">
         <v>230</v>
@@ -19782,7 +19782,7 @@
         <v>46311.60723116898</v>
       </c>
       <c r="W240">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X240" t="s">
         <v>231</v>
@@ -19862,7 +19862,7 @@
         <v>46304.46463219907</v>
       </c>
       <c r="W241">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X241" t="s">
         <v>229</v>
@@ -19942,7 +19942,7 @@
         <v>46309.76001859954</v>
       </c>
       <c r="W242">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X242" t="s">
         <v>228</v>
@@ -20022,7 +20022,7 @@
         <v>46304.60026121528</v>
       </c>
       <c r="W243">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X243" t="s">
         <v>237</v>
@@ -20102,7 +20102,7 @@
         <v>46308.63474228009</v>
       </c>
       <c r="W244">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X244" t="s">
         <v>235</v>
@@ -20179,7 +20179,7 @@
         <v>46310.40489282407</v>
       </c>
       <c r="W245">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X245" t="s">
         <v>234</v>
@@ -20256,7 +20256,7 @@
         <v>46309.74981408565</v>
       </c>
       <c r="W246">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X246" t="s">
         <v>236</v>
@@ -20333,7 +20333,7 @@
         <v>46309.70497604166</v>
       </c>
       <c r="W247">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X247" t="s">
         <v>229</v>
@@ -20410,7 +20410,7 @@
         <v>46309.73512677084</v>
       </c>
       <c r="W248">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X248" t="s">
         <v>228</v>
@@ -20487,7 +20487,7 @@
         <v>46309.73512769676</v>
       </c>
       <c r="W249">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X249" t="s">
         <v>228</v>
@@ -20567,7 +20567,7 @@
         <v>46311.36172075231</v>
       </c>
       <c r="W250">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X250" t="s">
         <v>237</v>
@@ -20644,7 +20644,7 @@
         <v>46308.76593190972</v>
       </c>
       <c r="W251">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X251" t="s">
         <v>235</v>
@@ -20721,7 +20721,7 @@
         <v>46309.72397658565</v>
       </c>
       <c r="W252">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X252" t="s">
         <v>230</v>
@@ -20801,7 +20801,7 @@
         <v>46310.6671994213</v>
       </c>
       <c r="W253">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X253" t="s">
         <v>231</v>
@@ -20875,7 +20875,7 @@
         <v>46310.63595796296</v>
       </c>
       <c r="W254">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X254" t="s">
         <v>230</v>
@@ -20955,7 +20955,7 @@
         <v>46310.75598100694</v>
       </c>
       <c r="W255">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X255" t="s">
         <v>231</v>
@@ -21032,7 +21032,7 @@
         <v>46311.63215984953</v>
       </c>
       <c r="W256">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X256" t="s">
         <v>232</v>
@@ -21106,7 +21106,7 @@
         <v>46311.63216135417</v>
       </c>
       <c r="W257">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X257" t="s">
         <v>232</v>
@@ -21180,7 +21180,7 @@
         <v>46309.63688255787</v>
       </c>
       <c r="W258">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X258" t="s">
         <v>231</v>
@@ -21257,7 +21257,7 @@
         <v>46310.43009836806</v>
       </c>
       <c r="W259">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X259" t="s">
         <v>228</v>
@@ -21331,7 +21331,7 @@
         <v>46304.34308188657</v>
       </c>
       <c r="W260">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X260" t="s">
         <v>229</v>
@@ -21405,7 +21405,7 @@
         <v>46304.71027804398</v>
       </c>
       <c r="W261">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X261" t="s">
         <v>228</v>
@@ -21479,7 +21479,7 @@
         <v>46304.48249973379</v>
       </c>
       <c r="W262">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X262" t="s">
         <v>230</v>
@@ -21553,7 +21553,7 @@
         <v>46304.48129263889</v>
       </c>
       <c r="W263">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X263" t="s">
         <v>231</v>
@@ -21630,7 +21630,7 @@
         <v>46308.72984224537</v>
       </c>
       <c r="W264">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X264" t="s">
         <v>232</v>
@@ -21710,7 +21710,7 @@
         <v>46308.73013729167</v>
       </c>
       <c r="W265">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X265" t="s">
         <v>232</v>
@@ -21787,7 +21787,7 @@
         <v>46309.7328783912</v>
       </c>
       <c r="W266">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X266" t="s">
         <v>228</v>
@@ -21864,7 +21864,7 @@
         <v>46304.67984788195</v>
       </c>
       <c r="W267">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X267" t="s">
         <v>232</v>
@@ -21944,7 +21944,7 @@
         <v>46304.64227313657</v>
       </c>
       <c r="W268">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X268" t="s">
         <v>232</v>
@@ -22024,7 +22024,7 @@
         <v>46309.37679274305</v>
       </c>
       <c r="W269">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X269" t="s">
         <v>231</v>
@@ -22104,7 +22104,7 @@
         <v>46310.80710414352</v>
       </c>
       <c r="W270">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X270" t="s">
         <v>228</v>
@@ -22184,7 +22184,7 @@
         <v>46310.81041364584</v>
       </c>
       <c r="W271">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X271" t="s">
         <v>230</v>
@@ -22264,7 +22264,7 @@
         <v>46310.8112078125</v>
       </c>
       <c r="W272">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X272" t="s">
         <v>231</v>
@@ -22341,7 +22341,7 @@
         <v>46311.52606443287</v>
       </c>
       <c r="W273">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X273" t="s">
         <v>234</v>
@@ -22415,7 +22415,7 @@
         <v>46311.53678394676</v>
       </c>
       <c r="W274">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X274" t="s">
         <v>233</v>
@@ -22489,7 +22489,7 @@
         <v>46311.53327506944</v>
       </c>
       <c r="W275">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X275" t="s">
         <v>236</v>
@@ -22566,7 +22566,7 @@
         <v>46311.52103310185</v>
       </c>
       <c r="W276">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X276" t="s">
         <v>235</v>
@@ -22646,7 +22646,7 @@
         <v>46311.7195858449</v>
       </c>
       <c r="W277">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X277" t="s">
         <v>235</v>
@@ -22726,7 +22726,7 @@
         <v>46311.71959521991</v>
       </c>
       <c r="W278">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X278" t="s">
         <v>235</v>
@@ -22806,7 +22806,7 @@
         <v>46309.56217365741</v>
       </c>
       <c r="W279">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X279" t="s">
         <v>234</v>
@@ -22886,7 +22886,7 @@
         <v>46309.78174778935</v>
       </c>
       <c r="W280">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X280" t="s">
         <v>233</v>
@@ -22966,7 +22966,7 @@
         <v>46309.78175008102</v>
       </c>
       <c r="W281">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X281" t="s">
         <v>236</v>
@@ -23046,7 +23046,7 @@
         <v>46309.83028228009</v>
       </c>
       <c r="W282">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X282" t="s">
         <v>237</v>
@@ -23126,7 +23126,7 @@
         <v>46310.39575521991</v>
       </c>
       <c r="W283">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X283" t="s">
         <v>235</v>
@@ -23206,7 +23206,7 @@
         <v>46310.39575559027</v>
       </c>
       <c r="W284">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X284" t="s">
         <v>235</v>
@@ -23286,7 +23286,7 @@
         <v>46310.39575600695</v>
       </c>
       <c r="W285">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X285" t="s">
         <v>235</v>
@@ -23366,7 +23366,7 @@
         <v>46311.51453325232</v>
       </c>
       <c r="W286">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X286" t="s">
         <v>234</v>
@@ -23443,7 +23443,7 @@
         <v>46308.41418804398</v>
       </c>
       <c r="W287">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X287" t="s">
         <v>234</v>
@@ -23520,7 +23520,7 @@
         <v>46311.67661959491</v>
       </c>
       <c r="W288">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X288" t="s">
         <v>233</v>
@@ -23600,7 +23600,7 @@
         <v>46304.56084105324</v>
       </c>
       <c r="W289">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X289" t="s">
         <v>237</v>
@@ -23680,7 +23680,7 @@
         <v>46309.65179342592</v>
       </c>
       <c r="W290">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X290" t="s">
         <v>235</v>
@@ -23757,7 +23757,7 @@
         <v>46304.56110010417</v>
       </c>
       <c r="W291">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X291" t="s">
         <v>234</v>
@@ -23831,7 +23831,7 @@
         <v>46304.62889446759</v>
       </c>
       <c r="W292">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X292" t="s">
         <v>233</v>
@@ -23905,7 +23905,7 @@
         <v>46304.62889520833</v>
       </c>
       <c r="W293">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X293" t="s">
         <v>236</v>
@@ -23979,7 +23979,7 @@
         <v>46304.62891434028</v>
       </c>
       <c r="W294">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X294" t="s">
         <v>237</v>
@@ -24056,7 +24056,7 @@
         <v>46311.52127074074</v>
       </c>
       <c r="W295">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X295" t="s">
         <v>235</v>
@@ -24133,7 +24133,7 @@
         <v>46304.62892777778</v>
       </c>
       <c r="W296">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X296" t="s">
         <v>235</v>
@@ -24207,7 +24207,7 @@
         <v>46304.62893950231</v>
       </c>
       <c r="W297">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X297" t="s">
         <v>235</v>
@@ -24284,7 +24284,7 @@
         <v>46304.49370603009</v>
       </c>
       <c r="W298">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X298" t="s">
         <v>234</v>
@@ -24364,7 +24364,7 @@
         <v>46304.50006596064</v>
       </c>
       <c r="W299">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X299" t="s">
         <v>237</v>
@@ -24441,7 +24441,7 @@
         <v>46308.56276559028</v>
       </c>
       <c r="W300">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X300" t="s">
         <v>235</v>
@@ -24515,7 +24515,7 @@
         <v>46310.7258505787</v>
       </c>
       <c r="W301">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X301" t="s">
         <v>236</v>
@@ -24589,7 +24589,7 @@
         <v>46304.66642386574</v>
       </c>
       <c r="W302">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X302" t="s">
         <v>237</v>
@@ -24666,7 +24666,7 @@
         <v>46309.68758141204</v>
       </c>
       <c r="W303">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X303" t="s">
         <v>235</v>
@@ -24740,7 +24740,7 @@
         <v>46304.65366649305</v>
       </c>
       <c r="W304">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X304" t="s">
         <v>231</v>
@@ -24814,7 +24814,7 @@
         <v>46304.71076834491</v>
       </c>
       <c r="W305">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X305" t="s">
         <v>232</v>
@@ -24888,7 +24888,7 @@
         <v>46304.65441696759</v>
       </c>
       <c r="W306">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X306" t="s">
         <v>232</v>
@@ -24962,7 +24962,7 @@
         <v>46304.67485967593</v>
       </c>
       <c r="W307">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X307" t="s">
         <v>229</v>
@@ -25036,7 +25036,7 @@
         <v>46304.66202476852</v>
       </c>
       <c r="W308">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X308" t="s">
         <v>228</v>
@@ -25107,7 +25107,7 @@
         <v>46304.68831197917</v>
       </c>
       <c r="W309">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X309" t="s">
         <v>237</v>
@@ -25181,7 +25181,7 @@
         <v>46311.5913249537</v>
       </c>
       <c r="W310">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X310" t="s">
         <v>235</v>
@@ -25255,7 +25255,7 @@
         <v>46304.66202549769</v>
       </c>
       <c r="W311">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X311" t="s">
         <v>235</v>
@@ -25329,7 +25329,7 @@
         <v>46304.66202701389</v>
       </c>
       <c r="W312">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X312" t="s">
         <v>235</v>
@@ -25403,7 +25403,7 @@
         <v>46304.66203011574</v>
       </c>
       <c r="W313">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X313" t="s">
         <v>230</v>
@@ -25477,7 +25477,7 @@
         <v>46304.69242271991</v>
       </c>
       <c r="W314">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X314" t="s">
         <v>231</v>
@@ -25551,7 +25551,7 @@
         <v>46304.69295292824</v>
       </c>
       <c r="W315">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X315" t="s">
         <v>232</v>
@@ -25625,7 +25625,7 @@
         <v>46304.69368494213</v>
       </c>
       <c r="W316">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X316" t="s">
         <v>232</v>
@@ -25699,7 +25699,7 @@
         <v>46311.55331846065</v>
       </c>
       <c r="W317">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X317" t="s">
         <v>234</v>
@@ -25770,7 +25770,7 @@
         <v>46311.55337682871</v>
       </c>
       <c r="W318">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X318" t="s">
         <v>233</v>
@@ -25841,7 +25841,7 @@
         <v>46311.55342422453</v>
       </c>
       <c r="W319">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X319" t="s">
         <v>236</v>
@@ -25912,7 +25912,7 @@
         <v>46311.5534503588</v>
       </c>
       <c r="W320">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X320" t="s">
         <v>229</v>
@@ -25983,7 +25983,7 @@
         <v>46311.55347895833</v>
       </c>
       <c r="W321">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X321" t="s">
         <v>228</v>
@@ -26054,7 +26054,7 @@
         <v>46311.55351039352</v>
       </c>
       <c r="W322">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X322" t="s">
         <v>235</v>
@@ -26125,7 +26125,7 @@
         <v>46311.55354799768</v>
       </c>
       <c r="W323">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X323" t="s">
         <v>235</v>
@@ -26196,7 +26196,7 @@
         <v>46311.55385321759</v>
       </c>
       <c r="W324">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X324" t="s">
         <v>230</v>
@@ -26267,7 +26267,7 @@
         <v>46311.55389814815</v>
       </c>
       <c r="W325">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X325" t="s">
         <v>231</v>
@@ -26338,7 +26338,7 @@
         <v>46311.55331813658</v>
       </c>
       <c r="W326">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X326" t="s">
         <v>234</v>
@@ -26409,7 +26409,7 @@
         <v>46311.55337631945</v>
       </c>
       <c r="W327">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X327" t="s">
         <v>233</v>
@@ -26480,7 +26480,7 @@
         <v>46311.55342443287</v>
       </c>
       <c r="W328">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X328" t="s">
         <v>236</v>
@@ -26551,7 +26551,7 @@
         <v>46311.55345010417</v>
       </c>
       <c r="W329">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X329" t="s">
         <v>229</v>
@@ -26622,7 +26622,7 @@
         <v>46311.55347851852</v>
       </c>
       <c r="W330">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X330" t="s">
         <v>228</v>
@@ -26693,7 +26693,7 @@
         <v>46311.55350982639</v>
       </c>
       <c r="W331">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X331" t="s">
         <v>235</v>
@@ -26764,7 +26764,7 @@
         <v>46311.55354752314</v>
       </c>
       <c r="W332">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X332" t="s">
         <v>235</v>
@@ -26835,7 +26835,7 @@
         <v>46311.55385335648</v>
       </c>
       <c r="W333">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X333" t="s">
         <v>230</v>
@@ -26906,7 +26906,7 @@
         <v>46311.5538971412</v>
       </c>
       <c r="W334">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X334" t="s">
         <v>231</v>
@@ -26980,7 +26980,7 @@
         <v>46309.40991104166</v>
       </c>
       <c r="W335">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X335" t="s">
         <v>234</v>
@@ -27057,7 +27057,7 @@
         <v>46309.41020521991</v>
       </c>
       <c r="W336">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X336" t="s">
         <v>233</v>
@@ -27134,7 +27134,7 @@
         <v>46309.41022715278</v>
       </c>
       <c r="W337">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X337" t="s">
         <v>236</v>
@@ -27211,7 +27211,7 @@
         <v>46309.41024563657</v>
       </c>
       <c r="W338">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X338" t="s">
         <v>229</v>
@@ -27288,7 +27288,7 @@
         <v>46309.41025899306</v>
       </c>
       <c r="W339">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X339" t="s">
         <v>228</v>
@@ -27365,7 +27365,7 @@
         <v>46309.41028034722</v>
       </c>
       <c r="W340">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X340" t="s">
         <v>237</v>
@@ -27442,7 +27442,7 @@
         <v>46309.41028116898</v>
       </c>
       <c r="W341">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X341" t="s">
         <v>235</v>
@@ -27519,7 +27519,7 @@
         <v>46309.41028195602</v>
       </c>
       <c r="W342">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="X342" t="s">
         <v>235</v>
@@ -27593,7 +27593,7 @@
         <v>46308.4550522338</v>
       </c>
       <c r="W343">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X343" t="s">
         <v>234</v>
@@ -27667,7 +27667,7 @@
         <v>46311.71324008102</v>
       </c>
       <c r="W344">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X344" t="s">
         <v>233</v>
@@ -27738,7 +27738,7 @@
         <v>46310.71018491898</v>
       </c>
       <c r="W345">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X345" t="s">
         <v>229</v>
@@ -27809,7 +27809,7 @@
         <v>46309.68971350694</v>
       </c>
       <c r="W346">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X346" t="s">
         <v>230</v>
@@ -27883,7 +27883,7 @@
         <v>46304.42026608796</v>
       </c>
       <c r="W347">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="X347" t="s">
         <v>231</v>
@@ -27954,7 +27954,7 @@
         <v>46309.68950355324</v>
       </c>
       <c r="W348">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X348" t="s">
         <v>231</v>
@@ -28025,7 +28025,7 @@
         <v>46309.68881501158</v>
       </c>
       <c r="W349">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X349" t="s">
         <v>232</v>
@@ -28102,7 +28102,7 @@
         <v>46317.63681168982</v>
       </c>
       <c r="W350">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X350" t="s">
         <v>228</v>
@@ -28176,7 +28176,7 @@
         <v>46317.63681204861</v>
       </c>
       <c r="W351">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X351" t="s">
         <v>228</v>
@@ -28250,7 +28250,7 @@
         <v>46317.63682094908</v>
       </c>
       <c r="W352">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X352" t="s">
         <v>231</v>
@@ -28324,7 +28324,7 @@
         <v>46318.63617619213</v>
       </c>
       <c r="W353">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X353" t="s">
         <v>228</v>
@@ -28398,7 +28398,7 @@
         <v>46315.41924965278</v>
       </c>
       <c r="W354">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X354" t="s">
         <v>230</v>
@@ -28475,7 +28475,7 @@
         <v>46314.74461128472</v>
       </c>
       <c r="W355">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X355" t="s">
         <v>228</v>
@@ -28549,7 +28549,7 @@
         <v>46315.43829979167</v>
       </c>
       <c r="W356">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X356" t="s">
         <v>231</v>
@@ -28626,7 +28626,7 @@
         <v>46318.65577725694</v>
       </c>
       <c r="W357">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X357" t="s">
         <v>232</v>
@@ -28706,7 +28706,7 @@
         <v>46318.65363291667</v>
       </c>
       <c r="W358">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X358" t="s">
         <v>232</v>
@@ -28783,7 +28783,7 @@
         <v>46318.59088555555</v>
       </c>
       <c r="W359">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X359" t="s">
         <v>235</v>
@@ -28857,7 +28857,7 @@
         <v>46318.59526878472</v>
       </c>
       <c r="W360">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X360" t="s">
         <v>235</v>
@@ -28931,7 +28931,7 @@
         <v>46316.59550709491</v>
       </c>
       <c r="W361">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X361" t="s">
         <v>237</v>
@@ -29005,7 +29005,7 @@
         <v>46316.5955075926</v>
       </c>
       <c r="W362">
-        <v>-88</v>
+        <v>-87</v>
       </c>
       <c r="X362" t="s">
         <v>237</v>
@@ -29079,7 +29079,7 @@
         <v>46315.37095327547</v>
       </c>
       <c r="W363">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X363" t="s">
         <v>237</v>
@@ -29159,7 +29159,7 @@
         <v>46317.42165659722</v>
       </c>
       <c r="W364">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X364" t="s">
         <v>237</v>
@@ -29236,7 +29236,7 @@
         <v>46314.43610068287</v>
       </c>
       <c r="W365">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X365" t="s">
         <v>237</v>
@@ -29310,7 +29310,7 @@
         <v>46314.70899030093</v>
       </c>
       <c r="W366">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X366" t="s">
         <v>237</v>
@@ -29387,7 +29387,7 @@
         <v>46315.60659672454</v>
       </c>
       <c r="W367">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X367" t="s">
         <v>235</v>
@@ -29467,7 +29467,7 @@
         <v>46314.58550305555</v>
       </c>
       <c r="W368">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X368" t="s">
         <v>234</v>
@@ -29544,7 +29544,7 @@
         <v>46314.42976884259</v>
       </c>
       <c r="W369">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X369" t="s">
         <v>236</v>
@@ -29618,7 +29618,7 @@
         <v>46314.40348229167</v>
       </c>
       <c r="W370">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X370" t="s">
         <v>228</v>
@@ -29692,7 +29692,7 @@
         <v>46314.42774210648</v>
       </c>
       <c r="W371">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X371" t="s">
         <v>228</v>
@@ -29769,7 +29769,7 @@
         <v>46314.60497207176</v>
       </c>
       <c r="W372">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X372" t="s">
         <v>237</v>
@@ -29849,7 +29849,7 @@
         <v>46315.60625753472</v>
       </c>
       <c r="W373">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X373" t="s">
         <v>235</v>
@@ -29926,7 +29926,7 @@
         <v>46314.7029991088</v>
       </c>
       <c r="W374">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X374" t="s">
         <v>231</v>
@@ -30003,7 +30003,7 @@
         <v>46314.58562635416</v>
       </c>
       <c r="W375">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X375" t="s">
         <v>234</v>
@@ -30080,7 +30080,7 @@
         <v>46314.42981640046</v>
       </c>
       <c r="W376">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X376" t="s">
         <v>236</v>
@@ -30154,7 +30154,7 @@
         <v>46314.41026230324</v>
       </c>
       <c r="W377">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X377" t="s">
         <v>228</v>
@@ -30228,7 +30228,7 @@
         <v>46314.42900954861</v>
       </c>
       <c r="W378">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X378" t="s">
         <v>228</v>
@@ -30305,7 +30305,7 @@
         <v>46314.60515678241</v>
       </c>
       <c r="W379">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X379" t="s">
         <v>237</v>
@@ -30385,7 +30385,7 @@
         <v>46315.60667663194</v>
       </c>
       <c r="W380">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X380" t="s">
         <v>235</v>
@@ -30462,7 +30462,7 @@
         <v>46314.70295032408</v>
       </c>
       <c r="W381">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X381" t="s">
         <v>231</v>
@@ -30539,7 +30539,7 @@
         <v>46315.62770037037</v>
       </c>
       <c r="W382">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X382" t="s">
         <v>234</v>
@@ -30616,7 +30616,7 @@
         <v>46314.57059383102</v>
       </c>
       <c r="W383">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X383" t="s">
         <v>236</v>
@@ -30693,7 +30693,7 @@
         <v>46314.73644534723</v>
       </c>
       <c r="W384">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X384" t="s">
         <v>229</v>
@@ -30770,7 +30770,7 @@
         <v>46314.56284280093</v>
       </c>
       <c r="W385">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X385" t="s">
         <v>228</v>
@@ -30844,7 +30844,7 @@
         <v>46314.56304628473</v>
       </c>
       <c r="W386">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X386" t="s">
         <v>228</v>
@@ -30921,7 +30921,7 @@
         <v>46315.72720311343</v>
       </c>
       <c r="W387">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X387" t="s">
         <v>237</v>
@@ -31001,7 +31001,7 @@
         <v>46315.58232621528</v>
       </c>
       <c r="W388">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X388" t="s">
         <v>235</v>
@@ -31081,7 +31081,7 @@
         <v>46315.72212693287</v>
       </c>
       <c r="W389">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X389" t="s">
         <v>230</v>
@@ -31161,7 +31161,7 @@
         <v>46318.62068615741</v>
       </c>
       <c r="W390">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X390" t="s">
         <v>234</v>
@@ -31241,7 +31241,7 @@
         <v>46317.35409214121</v>
       </c>
       <c r="W391">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X391" t="s">
         <v>233</v>
@@ -31321,7 +31321,7 @@
         <v>46317.70514107639</v>
       </c>
       <c r="W392">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X392" t="s">
         <v>236</v>
@@ -31401,7 +31401,7 @@
         <v>46316.41266554398</v>
       </c>
       <c r="W393">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X393" t="s">
         <v>229</v>
@@ -31481,7 +31481,7 @@
         <v>46317.70444474537</v>
       </c>
       <c r="W394">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X394" t="s">
         <v>228</v>
@@ -31561,7 +31561,7 @@
         <v>46317.70479641204</v>
       </c>
       <c r="W395">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X395" t="s">
         <v>228</v>
@@ -31641,7 +31641,7 @@
         <v>46318.4163918287</v>
       </c>
       <c r="W396">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X396" t="s">
         <v>237</v>
@@ -31721,7 +31721,7 @@
         <v>46317.70633898148</v>
       </c>
       <c r="W397">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X397" t="s">
         <v>230</v>
@@ -31801,7 +31801,7 @@
         <v>46318.71577450231</v>
       </c>
       <c r="W398">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X398" t="s">
         <v>231</v>
@@ -31881,7 +31881,7 @@
         <v>46314.39188924769</v>
       </c>
       <c r="W399">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X399" t="s">
         <v>233</v>
@@ -31958,7 +31958,7 @@
         <v>46314.44518351852</v>
       </c>
       <c r="W400">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X400" t="s">
         <v>233</v>
@@ -32032,7 +32032,7 @@
         <v>46314.73711247685</v>
       </c>
       <c r="W401">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="X401" t="s">
         <v>229</v>
@@ -32109,7 +32109,7 @@
         <v>46315.60662145833</v>
       </c>
       <c r="W402">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X402" t="s">
         <v>235</v>
@@ -32183,7 +32183,7 @@
         <v>46314.56177552084</v>
       </c>
       <c r="W403">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X403" t="s">
         <v>234</v>
@@ -32263,7 +32263,7 @@
         <v>46318.67778146991</v>
       </c>
       <c r="W404">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X404" t="s">
         <v>230</v>
@@ -32337,7 +32337,7 @@
         <v>46318.69314135417</v>
       </c>
       <c r="W405">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X405" t="s">
         <v>230</v>
@@ -32414,7 +32414,7 @@
         <v>46314.51585246528</v>
       </c>
       <c r="W406">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X406" t="s">
         <v>229</v>
@@ -32491,7 +32491,7 @@
         <v>46316.40514603009</v>
       </c>
       <c r="W407">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X407" t="s">
         <v>228</v>
@@ -32571,7 +32571,7 @@
         <v>46316.40514767361</v>
       </c>
       <c r="W408">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X408" t="s">
         <v>231</v>
@@ -32645,7 +32645,7 @@
         <v>46318.70265150463</v>
       </c>
       <c r="W409">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X409" t="s">
         <v>232</v>
@@ -32719,7 +32719,7 @@
         <v>46318.70292207176</v>
       </c>
       <c r="W410">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X410" t="s">
         <v>232</v>
@@ -32796,7 +32796,7 @@
         <v>46314.7779269676</v>
       </c>
       <c r="W411">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X411" t="s">
         <v>229</v>
@@ -32876,7 +32876,7 @@
         <v>46314.41760023148</v>
       </c>
       <c r="W412">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X412" t="s">
         <v>228</v>
@@ -32956,7 +32956,7 @@
         <v>46314.38417774306</v>
       </c>
       <c r="W413">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X413" t="s">
         <v>228</v>
@@ -33036,7 +33036,7 @@
         <v>46314.4276216088</v>
       </c>
       <c r="W414">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X414" t="s">
         <v>230</v>
@@ -33116,7 +33116,7 @@
         <v>46317.46467885416</v>
       </c>
       <c r="W415">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X415" t="s">
         <v>232</v>
@@ -33196,7 +33196,7 @@
         <v>46316.61403607639</v>
       </c>
       <c r="W416">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X416" t="s">
         <v>232</v>
@@ -33276,7 +33276,7 @@
         <v>46316.62803978009</v>
       </c>
       <c r="W417">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X417" t="s">
         <v>229</v>
@@ -33356,7 +33356,7 @@
         <v>46316.50641068287</v>
       </c>
       <c r="W418">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X418" t="s">
         <v>228</v>
@@ -33436,7 +33436,7 @@
         <v>46317.73924351852</v>
       </c>
       <c r="W419">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X419" t="s">
         <v>231</v>
@@ -33516,7 +33516,7 @@
         <v>46316.53861512731</v>
       </c>
       <c r="W420">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X420" t="s">
         <v>229</v>
@@ -33596,7 +33596,7 @@
         <v>46316.42401107639</v>
       </c>
       <c r="W421">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X421" t="s">
         <v>228</v>
@@ -33673,7 +33673,7 @@
         <v>46314.51604481482</v>
       </c>
       <c r="W422">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X422" t="s">
         <v>229</v>
@@ -33750,7 +33750,7 @@
         <v>46316.40539234954</v>
       </c>
       <c r="W423">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X423" t="s">
         <v>231</v>
@@ -33830,7 +33830,7 @@
         <v>46313.46956228009</v>
       </c>
       <c r="W424">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="X424" t="s">
         <v>236</v>
@@ -33910,7 +33910,7 @@
         <v>46316.40987146991</v>
       </c>
       <c r="W425">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X425" t="s">
         <v>235</v>
@@ -33990,7 +33990,7 @@
         <v>46317.62761559027</v>
       </c>
       <c r="W426">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X426" t="s">
         <v>236</v>
@@ -34070,7 +34070,7 @@
         <v>46314.38488630787</v>
       </c>
       <c r="W427">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X427" t="s">
         <v>235</v>
@@ -34150,7 +34150,7 @@
         <v>46316.42903232639</v>
       </c>
       <c r="W428">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X428" t="s">
         <v>235</v>
@@ -34230,7 +34230,7 @@
         <v>46314.78502430556</v>
       </c>
       <c r="W429">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X429" t="s">
         <v>237</v>
@@ -34310,7 +34310,7 @@
         <v>46315.65595015046</v>
       </c>
       <c r="W430">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X430" t="s">
         <v>235</v>
@@ -34390,7 +34390,7 @@
         <v>46314.38564537037</v>
       </c>
       <c r="W431">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X431" t="s">
         <v>234</v>
@@ -34470,7 +34470,7 @@
         <v>46314.38565289352</v>
       </c>
       <c r="W432">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X432" t="s">
         <v>233</v>
@@ -34547,7 +34547,7 @@
         <v>46314.37977384259</v>
       </c>
       <c r="W433">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X433" t="s">
         <v>236</v>
@@ -34627,7 +34627,7 @@
         <v>46316.50932392361</v>
       </c>
       <c r="W434">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X434" t="s">
         <v>233</v>
@@ -34707,7 +34707,7 @@
         <v>46316.50933533565</v>
       </c>
       <c r="W435">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X435" t="s">
         <v>237</v>
@@ -34787,7 +34787,7 @@
         <v>46316.61414429398</v>
       </c>
       <c r="W436">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X436" t="s">
         <v>234</v>
@@ -34867,7 +34867,7 @@
         <v>46318.67454332176</v>
       </c>
       <c r="W437">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X437" t="s">
         <v>235</v>
@@ -34941,7 +34941,7 @@
         <v>46315.43458024305</v>
       </c>
       <c r="W438">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X438" t="s">
         <v>228</v>
@@ -35015,7 +35015,7 @@
         <v>46315.4345809375</v>
       </c>
       <c r="W439">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X439" t="s">
         <v>235</v>
@@ -35089,7 +35089,7 @@
         <v>46315.43458121528</v>
       </c>
       <c r="W440">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X440" t="s">
         <v>235</v>
@@ -35163,7 +35163,7 @@
         <v>46315.43458645833</v>
       </c>
       <c r="W441">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X441" t="s">
         <v>230</v>
@@ -35237,7 +35237,7 @@
         <v>46315.6810275463</v>
       </c>
       <c r="W442">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X442" t="s">
         <v>234</v>
@@ -35311,7 +35311,7 @@
         <v>46315.68103180556</v>
       </c>
       <c r="W443">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X443" t="s">
         <v>233</v>
@@ -35385,7 +35385,7 @@
         <v>46315.43472936343</v>
       </c>
       <c r="W444">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X444" t="s">
         <v>228</v>
@@ -35456,7 +35456,7 @@
         <v>46315.43473040509</v>
       </c>
       <c r="W445">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X445" t="s">
         <v>237</v>
@@ -35530,7 +35530,7 @@
         <v>46315.68297636574</v>
       </c>
       <c r="W446">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X446" t="s">
         <v>235</v>
@@ -35604,7 +35604,7 @@
         <v>46315.67390174769</v>
       </c>
       <c r="W447">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X447" t="s">
         <v>230</v>
@@ -35678,7 +35678,7 @@
         <v>46318.46352369213</v>
       </c>
       <c r="W448">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X448" t="s">
         <v>234</v>
@@ -35755,7 +35755,7 @@
         <v>46318.46352971065</v>
       </c>
       <c r="W449">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X449" t="s">
         <v>233</v>
@@ -35832,7 +35832,7 @@
         <v>46318.66275958333</v>
       </c>
       <c r="W450">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X450" t="s">
         <v>228</v>
@@ -35909,7 +35909,7 @@
         <v>46318.46353538195</v>
       </c>
       <c r="W451">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X451" t="s">
         <v>237</v>
@@ -35986,7 +35986,7 @@
         <v>46318.68674609953</v>
       </c>
       <c r="W452">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X452" t="s">
         <v>235</v>
@@ -36063,7 +36063,7 @@
         <v>46318.46353634259</v>
       </c>
       <c r="W453">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X453" t="s">
         <v>231</v>
@@ -36140,7 +36140,7 @@
         <v>46318.65573842593</v>
       </c>
       <c r="W454">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X454" t="s">
         <v>232</v>
@@ -36217,7 +36217,7 @@
         <v>46318.46353657408</v>
       </c>
       <c r="W455">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X455" t="s">
         <v>232</v>
@@ -36291,7 +36291,7 @@
         <v>46315.43446484954</v>
       </c>
       <c r="W456">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X456" t="s">
         <v>234</v>
@@ -36362,7 +36362,7 @@
         <v>46315.43447334491</v>
       </c>
       <c r="W457">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X457" t="s">
         <v>228</v>
@@ -36433,7 +36433,7 @@
         <v>46315.43447511574</v>
       </c>
       <c r="W458">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X458" t="s">
         <v>235</v>
@@ -36504,7 +36504,7 @@
         <v>46315.75501361111</v>
       </c>
       <c r="W459">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X459" t="s">
         <v>235</v>
@@ -36575,7 +36575,7 @@
         <v>46315.4344778588</v>
       </c>
       <c r="W460">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X460" t="s">
         <v>231</v>
@@ -36646,7 +36646,7 @@
         <v>46314.51296478009</v>
       </c>
       <c r="W461">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X461" t="s">
         <v>234</v>
@@ -36717,7 +36717,7 @@
         <v>46314.5130255787</v>
       </c>
       <c r="W462">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X462" t="s">
         <v>233</v>
@@ -36788,7 +36788,7 @@
         <v>46314.51303561343</v>
       </c>
       <c r="W463">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X463" t="s">
         <v>236</v>
@@ -36859,7 +36859,7 @@
         <v>46314.51303834491</v>
       </c>
       <c r="W464">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X464" t="s">
         <v>229</v>
@@ -36930,7 +36930,7 @@
         <v>46314.51304019676</v>
       </c>
       <c r="W465">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X465" t="s">
         <v>228</v>
@@ -37001,7 +37001,7 @@
         <v>46314.51304019676</v>
       </c>
       <c r="W466">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X466" t="s">
         <v>228</v>
@@ -37072,7 +37072,7 @@
         <v>46314.51304733796</v>
       </c>
       <c r="W467">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X467" t="s">
         <v>237</v>
@@ -37143,7 +37143,7 @@
         <v>46314.51304903935</v>
       </c>
       <c r="W468">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X468" t="s">
         <v>235</v>
@@ -37214,7 +37214,7 @@
         <v>46314.51305077547</v>
       </c>
       <c r="W469">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X469" t="s">
         <v>235</v>
@@ -37285,7 +37285,7 @@
         <v>46314.51305917824</v>
       </c>
       <c r="W470">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X470" t="s">
         <v>235</v>
@@ -37356,7 +37356,7 @@
         <v>46314.51306744213</v>
       </c>
       <c r="W471">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X471" t="s">
         <v>230</v>
@@ -37427,7 +37427,7 @@
         <v>46314.51306767361</v>
       </c>
       <c r="W472">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X472" t="s">
         <v>231</v>
@@ -37498,7 +37498,7 @@
         <v>46314.5130681713</v>
       </c>
       <c r="W473">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X473" t="s">
         <v>232</v>
@@ -37569,7 +37569,7 @@
         <v>46314.51306832176</v>
       </c>
       <c r="W474">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X474" t="s">
         <v>232</v>
@@ -37643,7 +37643,7 @@
         <v>46314.42010680556</v>
       </c>
       <c r="W475">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X475" t="s">
         <v>228</v>
@@ -37720,7 +37720,7 @@
         <v>46314.78063420139</v>
       </c>
       <c r="W476">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="X476" t="s">
         <v>237</v>
@@ -37794,7 +37794,7 @@
         <v>46314.51310813658</v>
       </c>
       <c r="W477">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X477" t="s">
         <v>234</v>
@@ -37865,7 +37865,7 @@
         <v>46314.51312306713</v>
       </c>
       <c r="W478">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X478" t="s">
         <v>233</v>
@@ -37936,7 +37936,7 @@
         <v>46314.51312457176</v>
       </c>
       <c r="W479">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X479" t="s">
         <v>236</v>
@@ -38007,7 +38007,7 @@
         <v>46314.51312600695</v>
       </c>
       <c r="W480">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X480" t="s">
         <v>229</v>
@@ -38078,7 +38078,7 @@
         <v>46314.51312769676</v>
       </c>
       <c r="W481">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X481" t="s">
         <v>228</v>
@@ -38149,7 +38149,7 @@
         <v>46314.5131278125</v>
       </c>
       <c r="W482">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X482" t="s">
         <v>228</v>
@@ -38220,7 +38220,7 @@
         <v>46314.51313017361</v>
       </c>
       <c r="W483">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X483" t="s">
         <v>237</v>
@@ -38291,7 +38291,7 @@
         <v>46314.5131303588</v>
       </c>
       <c r="W484">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X484" t="s">
         <v>235</v>
@@ -38362,7 +38362,7 @@
         <v>46314.51313075231</v>
       </c>
       <c r="W485">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X485" t="s">
         <v>235</v>
@@ -38433,7 +38433,7 @@
         <v>46314.5131318287</v>
       </c>
       <c r="W486">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X486" t="s">
         <v>235</v>
@@ -38504,7 +38504,7 @@
         <v>46314.51313622685</v>
       </c>
       <c r="W487">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X487" t="s">
         <v>230</v>
@@ -38575,7 +38575,7 @@
         <v>46314.51313657407</v>
       </c>
       <c r="W488">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X488" t="s">
         <v>231</v>
@@ -38646,7 +38646,7 @@
         <v>46314.51313734954</v>
       </c>
       <c r="W489">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X489" t="s">
         <v>232</v>
@@ -38717,7 +38717,7 @@
         <v>46314.51313761574</v>
       </c>
       <c r="W490">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X490" t="s">
         <v>232</v>
@@ -38788,7 +38788,7 @@
         <v>46314.42010591435</v>
       </c>
       <c r="W491">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X491" t="s">
         <v>228</v>
@@ -38862,7 +38862,7 @@
         <v>46314.78063710648</v>
       </c>
       <c r="W492">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X492" t="s">
         <v>237</v>
@@ -38936,7 +38936,7 @@
         <v>46314.6513366088</v>
       </c>
       <c r="W493">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="X493" t="s">
         <v>233</v>
@@ -39010,7 +39010,7 @@
         <v>46314.64967491898</v>
       </c>
       <c r="W494">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="X494" t="s">
         <v>234</v>
@@ -39084,7 +39084,7 @@
         <v>46315.74513215278</v>
       </c>
       <c r="W495">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X495" t="s">
         <v>234</v>
@@ -39158,7 +39158,7 @@
         <v>46315.74771738426</v>
       </c>
       <c r="W496">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X496" t="s">
         <v>233</v>
@@ -39232,7 +39232,7 @@
         <v>46317.4619591088</v>
       </c>
       <c r="W497">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X497" t="s">
         <v>229</v>
@@ -39306,7 +39306,7 @@
         <v>46315.74643540509</v>
       </c>
       <c r="W498">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X498" t="s">
         <v>228</v>
@@ -39380,7 +39380,7 @@
         <v>46317.4583884838</v>
       </c>
       <c r="W499">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X499" t="s">
         <v>237</v>
@@ -39454,7 +39454,7 @@
         <v>46315.74965298611</v>
       </c>
       <c r="W500">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X500" t="s">
         <v>235</v>
@@ -39528,7 +39528,7 @@
         <v>46317.4610706713</v>
       </c>
       <c r="W501">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X501" t="s">
         <v>230</v>
@@ -39602,7 +39602,7 @@
         <v>46317.46036609953</v>
       </c>
       <c r="W502">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X502" t="s">
         <v>231</v>
@@ -39676,7 +39676,7 @@
         <v>46317.46297976852</v>
       </c>
       <c r="W503">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X503" t="s">
         <v>232</v>
@@ -39756,7 +39756,7 @@
         <v>46321.75051832176</v>
       </c>
       <c r="W504">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X504" t="s">
         <v>231</v>
@@ -39836,7 +39836,7 @@
         <v>46321.46183368056</v>
       </c>
       <c r="W505">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X505" t="s">
         <v>228</v>
@@ -39913,7 +39913,7 @@
         <v>46321.3853146412</v>
       </c>
       <c r="W506">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X506" t="s">
         <v>234</v>
@@ -39987,7 +39987,7 @@
         <v>46321.73676908565</v>
       </c>
       <c r="W507">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X507" t="s">
         <v>236</v>
@@ -40061,7 +40061,7 @@
         <v>46321.57058112269</v>
       </c>
       <c r="W508">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X508" t="s">
         <v>235</v>
@@ -40135,7 +40135,7 @@
         <v>46321.72535310185</v>
       </c>
       <c r="W509">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X509" t="s">
         <v>234</v>
@@ -40209,7 +40209,7 @@
         <v>46321.46283237269</v>
       </c>
       <c r="W510">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X510" t="s">
         <v>236</v>
@@ -40283,7 +40283,7 @@
         <v>46321.45487747686</v>
       </c>
       <c r="W511">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X511" t="s">
         <v>237</v>
@@ -40357,7 +40357,7 @@
         <v>46321.72719111111</v>
       </c>
       <c r="W512">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X512" t="s">
         <v>234</v>
@@ -40431,7 +40431,7 @@
         <v>46321.46301969908</v>
       </c>
       <c r="W513">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X513" t="s">
         <v>236</v>
@@ -40505,7 +40505,7 @@
         <v>46321.45513766204</v>
       </c>
       <c r="W514">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X514" t="s">
         <v>237</v>
@@ -40579,7 +40579,7 @@
         <v>46321.69687025463</v>
       </c>
       <c r="W515">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X515" t="s">
         <v>236</v>
@@ -40653,7 +40653,7 @@
         <v>46321.36862734954</v>
       </c>
       <c r="W516">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X516" t="s">
         <v>237</v>
@@ -40727,7 +40727,7 @@
         <v>46321.66110923611</v>
       </c>
       <c r="W517">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X517" t="s">
         <v>230</v>
@@ -40801,7 +40801,7 @@
         <v>46321.59424188657</v>
       </c>
       <c r="W518">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X518" t="s">
         <v>234</v>
@@ -40875,7 +40875,7 @@
         <v>46321.69699869213</v>
       </c>
       <c r="W519">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X519" t="s">
         <v>236</v>
@@ -40949,7 +40949,7 @@
         <v>46321.6622389699</v>
       </c>
       <c r="W520">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="X520" t="s">
         <v>230</v>
@@ -41023,7 +41023,7 @@
         <v>46321.39266284723</v>
       </c>
       <c r="W521">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X521" t="s">
         <v>232</v>
@@ -41097,7 +41097,7 @@
         <v>46321.39266328704</v>
       </c>
       <c r="W522">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X522" t="s">
         <v>232</v>
@@ -41171,7 +41171,7 @@
         <v>46321.66995337963</v>
       </c>
       <c r="W523">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X523" t="s">
         <v>234</v>
@@ -41245,7 +41245,7 @@
         <v>46321.6685106713</v>
       </c>
       <c r="W524">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X524" t="s">
         <v>235</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-28 10:47
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8185" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8215" uniqueCount="469">
   <si>
     <t>CodCliente</t>
   </si>
@@ -1802,7 +1802,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI531"/>
+  <dimension ref="A1:AI533"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:35">
@@ -42850,10 +42850,10 @@
     </row>
     <row r="526" spans="1:35">
       <c r="A526">
-        <v>6962</v>
+        <v>6404</v>
       </c>
       <c r="B526" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C526" t="s">
         <v>49</v>
@@ -42868,58 +42868,58 @@
         <v>55</v>
       </c>
       <c r="G526">
-        <v>5984</v>
+        <v>5906</v>
       </c>
       <c r="H526">
-        <v>1884</v>
+        <v>5784</v>
       </c>
       <c r="I526" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J526" t="s">
-        <v>169</v>
+        <v>84</v>
       </c>
       <c r="L526" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="N526" s="1">
-        <v>46321</v>
+        <v>46331</v>
       </c>
       <c r="P526">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q526">
         <v>2026</v>
       </c>
       <c r="R526">
-        <v>18260053</v>
+        <v>16962232</v>
       </c>
       <c r="S526" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="T526" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U526" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="V526" s="1">
-        <v>46321.39266284723</v>
+        <v>46323.43912737269</v>
       </c>
       <c r="W526">
-        <v>2</v>
+        <v>-8</v>
       </c>
       <c r="X526" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AB526">
         <v>0</v>
       </c>
       <c r="AC526" t="s">
-        <v>227</v>
+        <v>208</v>
       </c>
       <c r="AH526" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="AI526" t="s">
         <v>468</v>
@@ -42927,10 +42927,10 @@
     </row>
     <row r="527" spans="1:35">
       <c r="A527">
-        <v>6963</v>
+        <v>6404</v>
       </c>
       <c r="B527" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C527" t="s">
         <v>49</v>
@@ -42945,55 +42945,55 @@
         <v>55</v>
       </c>
       <c r="G527">
-        <v>5984</v>
+        <v>5907</v>
       </c>
       <c r="H527">
-        <v>1884</v>
+        <v>5784</v>
       </c>
       <c r="I527" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J527" t="s">
-        <v>169</v>
+        <v>86</v>
       </c>
       <c r="L527" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="N527" s="1">
-        <v>46321</v>
+        <v>46331</v>
       </c>
       <c r="P527">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q527">
         <v>2026</v>
       </c>
       <c r="R527">
-        <v>18260186</v>
+        <v>16962242</v>
       </c>
       <c r="S527" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="T527" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="U527" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="V527" s="1">
-        <v>46321.39266328704</v>
+        <v>46323.43942153935</v>
       </c>
       <c r="W527">
-        <v>2</v>
+        <v>-8</v>
       </c>
       <c r="X527" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AB527">
         <v>0</v>
       </c>
       <c r="AC527" t="s">
-        <v>227</v>
+        <v>208</v>
       </c>
       <c r="AH527" t="s">
         <v>461</v>
@@ -43004,16 +43004,16 @@
     </row>
     <row r="528" spans="1:35">
       <c r="A528">
-        <v>5417</v>
+        <v>6962</v>
       </c>
       <c r="B528" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C528" t="s">
         <v>49</v>
       </c>
       <c r="D528" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E528" t="s">
         <v>54</v>
@@ -43022,19 +43022,19 @@
         <v>55</v>
       </c>
       <c r="G528">
-        <v>6759</v>
+        <v>5984</v>
       </c>
       <c r="H528">
-        <v>1788</v>
+        <v>1884</v>
       </c>
       <c r="I528" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J528" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="L528" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="N528" s="1">
         <v>46321</v>
@@ -43046,31 +43046,31 @@
         <v>2026</v>
       </c>
       <c r="R528">
-        <v>17399191</v>
+        <v>18260053</v>
       </c>
       <c r="S528" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="T528" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="U528" t="s">
         <v>231</v>
       </c>
       <c r="V528" s="1">
-        <v>46321.66995337963</v>
+        <v>46321.39266284723</v>
       </c>
       <c r="W528">
         <v>2</v>
       </c>
       <c r="X528" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="AB528">
         <v>0</v>
       </c>
       <c r="AC528" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="AH528" t="s">
         <v>461</v>
@@ -43081,16 +43081,16 @@
     </row>
     <row r="529" spans="1:35">
       <c r="A529">
-        <v>6705</v>
+        <v>6963</v>
       </c>
       <c r="B529" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C529" t="s">
         <v>49</v>
       </c>
       <c r="D529" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E529" t="s">
         <v>54</v>
@@ -43099,19 +43099,19 @@
         <v>55</v>
       </c>
       <c r="G529">
-        <v>6759</v>
+        <v>5984</v>
       </c>
       <c r="H529">
-        <v>1788</v>
+        <v>1884</v>
       </c>
       <c r="I529" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J529" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="L529" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="N529" s="1">
         <v>46321</v>
@@ -43123,31 +43123,31 @@
         <v>2026</v>
       </c>
       <c r="R529">
-        <v>17949020</v>
+        <v>18260186</v>
       </c>
       <c r="S529" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="T529" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="U529" t="s">
         <v>231</v>
       </c>
       <c r="V529" s="1">
-        <v>46321.6685106713</v>
+        <v>46321.39266328704</v>
       </c>
       <c r="W529">
         <v>2</v>
       </c>
       <c r="X529" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="AB529">
         <v>0</v>
       </c>
       <c r="AC529" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="AH529" t="s">
         <v>461</v>
@@ -43158,16 +43158,16 @@
     </row>
     <row r="530" spans="1:35">
       <c r="A530">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B530" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C530" t="s">
         <v>49</v>
       </c>
       <c r="D530" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E530" t="s">
         <v>54</v>
@@ -43176,25 +43176,22 @@
         <v>55</v>
       </c>
       <c r="G530">
-        <v>1810</v>
+        <v>6759</v>
       </c>
       <c r="H530">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I530" t="s">
         <v>61</v>
       </c>
       <c r="J530" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="L530" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="N530" s="1">
-        <v>46322</v>
-      </c>
-      <c r="O530" t="s">
-        <v>195</v>
+        <v>46321</v>
       </c>
       <c r="P530">
         <v>9</v>
@@ -43203,7 +43200,7 @@
         <v>2026</v>
       </c>
       <c r="R530">
-        <v>16962178</v>
+        <v>17399191</v>
       </c>
       <c r="S530" t="s">
         <v>215</v>
@@ -43215,16 +43212,13 @@
         <v>231</v>
       </c>
       <c r="V530" s="1">
-        <v>46322.77760795139</v>
+        <v>46321.66995337963</v>
       </c>
       <c r="W530">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X530" t="s">
-        <v>237</v>
-      </c>
-      <c r="Y530" t="s">
-        <v>453</v>
+        <v>238</v>
       </c>
       <c r="AB530">
         <v>0</v>
@@ -43233,7 +43227,7 @@
         <v>215</v>
       </c>
       <c r="AH530" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="AI530" t="s">
         <v>468</v>
@@ -43241,16 +43235,16 @@
     </row>
     <row r="531" spans="1:35">
       <c r="A531">
-        <v>6703</v>
+        <v>6705</v>
       </c>
       <c r="B531" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C531" t="s">
         <v>49</v>
       </c>
       <c r="D531" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E531" t="s">
         <v>54</v>
@@ -43259,25 +43253,22 @@
         <v>55</v>
       </c>
       <c r="G531">
-        <v>1810</v>
+        <v>6759</v>
       </c>
       <c r="H531">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I531" t="s">
         <v>61</v>
       </c>
       <c r="J531" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="L531" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="N531" s="1">
-        <v>46322</v>
-      </c>
-      <c r="O531" t="s">
-        <v>186</v>
+        <v>46321</v>
       </c>
       <c r="P531">
         <v>9</v>
@@ -43286,7 +43277,7 @@
         <v>2026</v>
       </c>
       <c r="R531">
-        <v>17948813</v>
+        <v>17949020</v>
       </c>
       <c r="S531" t="s">
         <v>215</v>
@@ -43298,16 +43289,13 @@
         <v>231</v>
       </c>
       <c r="V531" s="1">
-        <v>46322.76616149305</v>
+        <v>46321.6685106713</v>
       </c>
       <c r="W531">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X531" t="s">
-        <v>241</v>
-      </c>
-      <c r="Y531" t="s">
-        <v>454</v>
+        <v>239</v>
       </c>
       <c r="AB531">
         <v>0</v>
@@ -43316,9 +43304,175 @@
         <v>215</v>
       </c>
       <c r="AH531" t="s">
+        <v>461</v>
+      </c>
+      <c r="AI531" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="532" spans="1:35">
+      <c r="A532">
+        <v>6404</v>
+      </c>
+      <c r="B532" t="s">
+        <v>42</v>
+      </c>
+      <c r="C532" t="s">
+        <v>49</v>
+      </c>
+      <c r="D532" t="s">
+        <v>52</v>
+      </c>
+      <c r="E532" t="s">
+        <v>54</v>
+      </c>
+      <c r="F532" t="s">
+        <v>55</v>
+      </c>
+      <c r="G532">
+        <v>1810</v>
+      </c>
+      <c r="H532">
+        <v>0</v>
+      </c>
+      <c r="I532" t="s">
+        <v>61</v>
+      </c>
+      <c r="J532" t="s">
+        <v>170</v>
+      </c>
+      <c r="L532" t="s">
+        <v>171</v>
+      </c>
+      <c r="N532" s="1">
+        <v>46322</v>
+      </c>
+      <c r="O532" t="s">
+        <v>195</v>
+      </c>
+      <c r="P532">
+        <v>9</v>
+      </c>
+      <c r="Q532">
+        <v>2026</v>
+      </c>
+      <c r="R532">
+        <v>16962178</v>
+      </c>
+      <c r="S532" t="s">
+        <v>215</v>
+      </c>
+      <c r="T532" t="s">
+        <v>228</v>
+      </c>
+      <c r="U532" t="s">
+        <v>231</v>
+      </c>
+      <c r="V532" s="1">
+        <v>46322.77760795139</v>
+      </c>
+      <c r="W532">
+        <v>1</v>
+      </c>
+      <c r="X532" t="s">
+        <v>237</v>
+      </c>
+      <c r="Y532" t="s">
+        <v>453</v>
+      </c>
+      <c r="AB532">
+        <v>0</v>
+      </c>
+      <c r="AC532" t="s">
+        <v>215</v>
+      </c>
+      <c r="AH532" t="s">
         <v>462</v>
       </c>
-      <c r="AI531" t="s">
+      <c r="AI532" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="533" spans="1:35">
+      <c r="A533">
+        <v>6703</v>
+      </c>
+      <c r="B533" t="s">
+        <v>48</v>
+      </c>
+      <c r="C533" t="s">
+        <v>49</v>
+      </c>
+      <c r="D533" t="s">
+        <v>52</v>
+      </c>
+      <c r="E533" t="s">
+        <v>54</v>
+      </c>
+      <c r="F533" t="s">
+        <v>55</v>
+      </c>
+      <c r="G533">
+        <v>1810</v>
+      </c>
+      <c r="H533">
+        <v>0</v>
+      </c>
+      <c r="I533" t="s">
+        <v>61</v>
+      </c>
+      <c r="J533" t="s">
+        <v>170</v>
+      </c>
+      <c r="L533" t="s">
+        <v>171</v>
+      </c>
+      <c r="N533" s="1">
+        <v>46322</v>
+      </c>
+      <c r="O533" t="s">
+        <v>186</v>
+      </c>
+      <c r="P533">
+        <v>9</v>
+      </c>
+      <c r="Q533">
+        <v>2026</v>
+      </c>
+      <c r="R533">
+        <v>17948813</v>
+      </c>
+      <c r="S533" t="s">
+        <v>215</v>
+      </c>
+      <c r="T533" t="s">
+        <v>228</v>
+      </c>
+      <c r="U533" t="s">
+        <v>231</v>
+      </c>
+      <c r="V533" s="1">
+        <v>46322.76616149305</v>
+      </c>
+      <c r="W533">
+        <v>1</v>
+      </c>
+      <c r="X533" t="s">
+        <v>241</v>
+      </c>
+      <c r="Y533" t="s">
+        <v>454</v>
+      </c>
+      <c r="AB533">
+        <v>0</v>
+      </c>
+      <c r="AC533" t="s">
+        <v>215</v>
+      </c>
+      <c r="AH533" t="s">
+        <v>462</v>
+      </c>
+      <c r="AI533" t="s">
         <v>468</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-30 09:46
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -879,10 +879,10 @@
 Aguardando o envio das informações pela empresa. - Data Comentário: 30/09/2026 09:11</t>
   </si>
   <si>
+    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 07/10/2026 - Data Comentário: 06/10/2026 17:01</t>
+  </si>
+  <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 08/10/2026 - Data Comentário: 07/10/2026 17:07</t>
-  </si>
-  <si>
-    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 07/10/2026 - Data Comentário: 06/10/2026 17:01</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 06/10/2026 - Data Comentário: 05/10/2026 16:52</t>
@@ -7798,10 +7798,10 @@
         <v>175</v>
       </c>
       <c r="N74" s="1">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="O74" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="P74">
         <v>10</v>
@@ -7810,7 +7810,7 @@
         <v>2026</v>
       </c>
       <c r="R74">
-        <v>18272234</v>
+        <v>18290119</v>
       </c>
       <c r="S74" t="s">
         <v>211</v>
@@ -7822,10 +7822,10 @@
         <v>235</v>
       </c>
       <c r="V74" s="1">
-        <v>46303.73557287037</v>
+        <v>46302.74648497685</v>
       </c>
       <c r="W74">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X74" t="s">
         <v>240</v>
@@ -7881,10 +7881,10 @@
         <v>175</v>
       </c>
       <c r="N75" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="O75" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P75">
         <v>10</v>
@@ -7893,7 +7893,7 @@
         <v>2026</v>
       </c>
       <c r="R75">
-        <v>18290119</v>
+        <v>18272234</v>
       </c>
       <c r="S75" t="s">
         <v>211</v>
@@ -7905,10 +7905,10 @@
         <v>235</v>
       </c>
       <c r="V75" s="1">
-        <v>46302.74648497685</v>
+        <v>46303.73557287037</v>
       </c>
       <c r="W75">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="X75" t="s">
         <v>240</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-30 10:24
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -879,10 +879,10 @@
 Aguardando o envio das informações pela empresa. - Data Comentário: 30/09/2026 09:11</t>
   </si>
   <si>
+    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 08/10/2026 - Data Comentário: 07/10/2026 17:07</t>
+  </si>
+  <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 07/10/2026 - Data Comentário: 06/10/2026 17:01</t>
-  </si>
-  <si>
-    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 08/10/2026 - Data Comentário: 07/10/2026 17:07</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 06/10/2026 - Data Comentário: 05/10/2026 16:52</t>
@@ -7798,10 +7798,10 @@
         <v>175</v>
       </c>
       <c r="N74" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="O74" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P74">
         <v>10</v>
@@ -7810,7 +7810,7 @@
         <v>2026</v>
       </c>
       <c r="R74">
-        <v>18290119</v>
+        <v>18272234</v>
       </c>
       <c r="S74" t="s">
         <v>211</v>
@@ -7822,10 +7822,10 @@
         <v>235</v>
       </c>
       <c r="V74" s="1">
-        <v>46302.74648497685</v>
+        <v>46303.73557287037</v>
       </c>
       <c r="W74">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="X74" t="s">
         <v>240</v>
@@ -7881,10 +7881,10 @@
         <v>175</v>
       </c>
       <c r="N75" s="1">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="O75" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="P75">
         <v>10</v>
@@ -7893,7 +7893,7 @@
         <v>2026</v>
       </c>
       <c r="R75">
-        <v>18272234</v>
+        <v>18290119</v>
       </c>
       <c r="S75" t="s">
         <v>211</v>
@@ -7905,10 +7905,10 @@
         <v>235</v>
       </c>
       <c r="V75" s="1">
-        <v>46303.73557287037</v>
+        <v>46302.74648497685</v>
       </c>
       <c r="W75">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X75" t="s">
         <v>240</v>

</xml_diff>

<commit_message>
Atualização automática: 2026-10-30 11:58
</commit_message>
<xml_diff>
--- a/data/base/goias.xlsx
+++ b/data/base/goias.xlsx
@@ -879,10 +879,10 @@
 Aguardando o envio das informações pela empresa. - Data Comentário: 30/09/2026 09:11</t>
   </si>
   <si>
+    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 07/10/2026 - Data Comentário: 06/10/2026 17:01</t>
+  </si>
+  <si>
     <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 08/10/2026 - Data Comentário: 07/10/2026 17:07</t>
-  </si>
-  <si>
-    <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 07/10/2026 - Data Comentário: 06/10/2026 17:01</t>
   </si>
   <si>
     <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 06/10/2026 - Data Comentário: 05/10/2026 16:52</t>
@@ -7801,10 +7801,10 @@
         <v>175</v>
       </c>
       <c r="N74" s="1">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="O74" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="P74">
         <v>10</v>
@@ -7813,7 +7813,7 @@
         <v>2026</v>
       </c>
       <c r="R74">
-        <v>18272234</v>
+        <v>18290119</v>
       </c>
       <c r="S74" t="s">
         <v>211</v>
@@ -7825,10 +7825,10 @@
         <v>235</v>
       </c>
       <c r="V74" s="1">
-        <v>46303.73557287037</v>
+        <v>46302.74648497685</v>
       </c>
       <c r="W74">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X74" t="s">
         <v>240</v>
@@ -7884,10 +7884,10 @@
         <v>175</v>
       </c>
       <c r="N75" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="O75" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P75">
         <v>10</v>
@@ -7896,7 +7896,7 @@
         <v>2026</v>
       </c>
       <c r="R75">
-        <v>18290119</v>
+        <v>18272234</v>
       </c>
       <c r="S75" t="s">
         <v>211</v>
@@ -7908,10 +7908,10 @@
         <v>235</v>
       </c>
       <c r="V75" s="1">
-        <v>46302.74648497685</v>
+        <v>46303.73557287037</v>
       </c>
       <c r="W75">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="X75" t="s">
         <v>240</v>

</xml_diff>